<commit_message>
> sim RTL ysyx_23060246 韩炳晋 Linux archlinux 6.6.60-1-lts #1 SMP PREEMPT_DYNAMIC Fri, 08 Nov 2024 16:03:02 +0000 x86_64 GNU/Linux  13:59:18 up 20:14,  2 users,  load average: 1.66, 1.76, 1.81
</commit_message>
<xml_diff>
--- a/npc/tools/control_gen/control_table.xlsx
+++ b/npc/tools/control_gen/control_table.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="27795" windowHeight="12075"/>
+    <workbookView windowWidth="27795" windowHeight="12735"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="28">
   <si>
     <t>commont</t>
   </si>
@@ -40,40 +40,64 @@
     <t>wb_sel</t>
   </si>
   <si>
+    <t>ld_sel</t>
+  </si>
+  <si>
+    <t>st_sel</t>
+  </si>
+  <si>
+    <t>mask_sel</t>
+  </si>
+  <si>
+    <t>inst_valid</t>
+  </si>
+  <si>
     <t>lui</t>
   </si>
   <si>
+    <t>A_PC</t>
+  </si>
+  <si>
+    <t>B_IMM</t>
+  </si>
+  <si>
+    <t>ALU_COPY_B</t>
+  </si>
+  <si>
+    <t>IMM_U</t>
+  </si>
+  <si>
+    <t>INST_VALID</t>
+  </si>
+  <si>
+    <t>auipc</t>
+  </si>
+  <si>
+    <t>ALU_ADD</t>
+  </si>
+  <si>
+    <t>default</t>
+  </si>
+  <si>
     <t>PC_4</t>
   </si>
   <si>
-    <t>A_PC</t>
-  </si>
-  <si>
-    <t>ALU_COPY_B</t>
-  </si>
-  <si>
-    <t>IMM_U</t>
-  </si>
-  <si>
-    <t>WB_ALU</t>
-  </si>
-  <si>
-    <t>auipc</t>
-  </si>
-  <si>
-    <t>ALU_ADD</t>
-  </si>
-  <si>
-    <t>default</t>
-  </si>
-  <si>
     <t>A_RS1</t>
   </si>
   <si>
-    <t>B_IMM</t>
-  </si>
-  <si>
     <t>IMM_I</t>
+  </si>
+  <si>
+    <t>WB_XX</t>
+  </si>
+  <si>
+    <t>LD_XX</t>
+  </si>
+  <si>
+    <t>MASK_XX</t>
+  </si>
+  <si>
+    <t>INST_INVALID</t>
   </si>
 </sst>
 </file>
@@ -82,8 +106,8 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="4">
     <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="41" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
     <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="41" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
     <numFmt numFmtId="42" formatCode="_ &quot;￥&quot;* #,##0_ ;_ &quot;￥&quot;* \-#,##0_ ;_ &quot;￥&quot;* &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
   <fonts count="22">
@@ -108,6 +132,13 @@
     </font>
     <font>
       <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
       <color theme="1"/>
       <name val="宋体"/>
       <charset val="0"/>
@@ -122,8 +153,23 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <u/>
       <sz val="11"/>
-      <color rgb="FFFA7D00"/>
+      <color rgb="FF0000FF"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF006100"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="0"/>
       <name val="宋体"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -136,24 +182,55 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <b/>
       <sz val="11"/>
-      <color theme="0"/>
+      <color rgb="FF3F3F3F"/>
       <name val="宋体"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <u/>
+      <b/>
+      <sz val="15"/>
+      <color theme="3"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <sz val="11"/>
-      <color rgb="FF800080"/>
+      <color rgb="FF9C6500"/>
       <name val="宋体"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <u/>
+      <b/>
       <sz val="11"/>
-      <color rgb="FF0000FF"/>
+      <color rgb="FFFA7D00"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF3F3F76"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="18"/>
+      <color theme="3"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color rgb="FF7F7F7F"/>
       <name val="宋体"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -168,22 +245,15 @@
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FF9C6500"/>
+      <color rgb="FF9C0006"/>
       <name val="宋体"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
+      <u/>
       <sz val="11"/>
-      <color theme="1"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C0006"/>
+      <color rgb="FF800080"/>
       <name val="宋体"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -198,54 +268,8 @@
     </font>
     <font>
       <b/>
-      <sz val="15"/>
-      <color theme="3"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="18"/>
-      <color theme="3"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FF3F3F3F"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF006100"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="11"/>
-      <color rgb="FF7F7F7F"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF3F3F76"/>
+      <color theme="1"/>
       <name val="宋体"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -266,67 +290,139 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor theme="8" tint="0.599993896298105"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFCC99"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFA5A5A5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor theme="9" tint="0.599993896298105"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFA5A5A5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4"/>
+        <fgColor theme="6" tint="0.799981688894314"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -338,7 +434,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.799981688894314"/>
+        <fgColor theme="5"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -350,37 +446,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
+        <fgColor theme="7" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.599993896298105"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -392,55 +464,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor theme="9" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.399975585192419"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -457,43 +481,8 @@
       <left/>
       <right/>
       <top/>
-      <bottom style="medium">
-        <color theme="4" tint="0.499984740745262"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
       <bottom style="double">
         <color rgb="FFFF8001"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="double">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="double">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="double">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="double">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color theme="4"/>
-      </top>
-      <bottom style="double">
-        <color theme="4"/>
       </bottom>
       <diagonal/>
     </border>
@@ -502,22 +491,7 @@
       <right/>
       <top/>
       <bottom style="medium">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF7F7F7F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF7F7F7F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF7F7F7F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF7F7F7F"/>
+        <color theme="4" tint="0.499984740745262"/>
       </bottom>
       <diagonal/>
     </border>
@@ -551,153 +525,203 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF7F7F7F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF7F7F7F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF7F7F7F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF7F7F7F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="double">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="double">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="double">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="double">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="4"/>
+      </top>
+      <bottom style="double">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="28" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="8" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="17" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="8" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="17" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="10" borderId="3" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="17" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="8" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="11" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="21" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="11" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="18" borderId="7" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
@@ -1042,7 +1066,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:AE59"/>
+  <dimension ref="A1:AG59"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
     <col min="1" max="1" width="13.1" customWidth="1"/>
@@ -1052,21 +1076,21 @@
     <col min="5" max="5" width="11.7166666666667" customWidth="1"/>
     <col min="6" max="6" width="11.1166666666667" customWidth="1"/>
     <col min="7" max="7" width="10.9416666666667" customWidth="1"/>
-    <col min="8" max="8" width="44.0583333333333" customWidth="1"/>
-    <col min="9" max="9" width="15.075" customWidth="1"/>
-    <col min="10" max="10" width="12.1083333333333" customWidth="1"/>
-    <col min="11" max="11" width="10.8583333333333" customWidth="1"/>
-    <col min="13" max="13" width="14.2166666666667" customWidth="1"/>
-    <col min="14" max="14" width="11.8083333333333" customWidth="1"/>
-    <col min="15" max="15" width="10.6" customWidth="1"/>
-    <col min="16" max="16" width="9.70833333333333" customWidth="1"/>
-    <col min="17" max="17" width="11.1666666666667" customWidth="1"/>
-    <col min="18" max="18" width="11.4083333333333" customWidth="1"/>
-    <col min="19" max="19" width="12.0583333333333" customWidth="1"/>
-    <col min="20" max="20" width="15.575" customWidth="1"/>
+    <col min="8" max="10" width="11.9833333333333" customWidth="1"/>
+    <col min="11" max="11" width="15.075" customWidth="1"/>
+    <col min="12" max="12" width="12.1083333333333" customWidth="1"/>
+    <col min="13" max="13" width="10.8583333333333" customWidth="1"/>
+    <col min="15" max="15" width="14.2166666666667" customWidth="1"/>
+    <col min="16" max="16" width="11.8083333333333" customWidth="1"/>
+    <col min="17" max="17" width="10.6" customWidth="1"/>
+    <col min="18" max="18" width="9.70833333333333" customWidth="1"/>
+    <col min="19" max="19" width="11.1666666666667" customWidth="1"/>
+    <col min="20" max="20" width="11.4083333333333" customWidth="1"/>
+    <col min="21" max="21" width="12.0583333333333" customWidth="1"/>
+    <col min="22" max="22" width="15.575" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="15" customHeight="1" spans="1:19">
+    <row r="1" ht="15" customHeight="1" spans="1:21">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1091,49 +1115,57 @@
       <c r="H1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="2"/>
-      <c r="J1" s="2"/>
-      <c r="K1" s="2"/>
-      <c r="L1" s="2"/>
+      <c r="I1" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="2" t="s">
+        <v>11</v>
+      </c>
       <c r="M1" s="2"/>
       <c r="N1" s="2"/>
       <c r="O1" s="2"/>
       <c r="P1" s="2"/>
-      <c r="S1" s="6"/>
-    </row>
-    <row r="2" spans="1:31">
+      <c r="Q1" s="2"/>
+      <c r="R1" s="2"/>
+      <c r="U1" s="6"/>
+    </row>
+    <row r="2" spans="1:33">
       <c r="A2" s="3"/>
       <c r="B2" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>9</v>
-      </c>
+        <v>12</v>
+      </c>
+      <c r="C2" s="2"/>
       <c r="D2" s="4" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="F2" s="4" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="G2" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="H2" s="4" t="s">
-        <v>13</v>
-      </c>
+        <v>16</v>
+      </c>
+      <c r="H2" s="4"/>
       <c r="I2" s="4"/>
       <c r="J2" s="4"/>
       <c r="K2" s="4"/>
-      <c r="L2" s="4"/>
+      <c r="L2" s="4" t="s">
+        <v>17</v>
+      </c>
       <c r="M2" s="4"/>
       <c r="N2" s="4"/>
       <c r="O2" s="4"/>
       <c r="P2" s="4"/>
-      <c r="Q2" s="3"/>
-      <c r="R2" s="3"/>
+      <c r="Q2" s="4"/>
+      <c r="R2" s="4"/>
       <c r="S2" s="3"/>
       <c r="T2" s="3"/>
       <c r="U2" s="3"/>
@@ -1147,40 +1179,40 @@
       <c r="AC2" s="3"/>
       <c r="AD2" s="3"/>
       <c r="AE2" s="3"/>
-    </row>
-    <row r="3" spans="1:31">
+      <c r="AF2" s="3"/>
+      <c r="AG2" s="3"/>
+    </row>
+    <row r="3" spans="1:33">
       <c r="A3" s="3"/>
       <c r="B3" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C3" s="2"/>
+      <c r="D3" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="E3" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="C3" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="D3" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="E3" s="4" t="s">
-        <v>10</v>
-      </c>
       <c r="F3" s="4" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="G3" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="H3" s="4" t="s">
-        <v>13</v>
-      </c>
+        <v>16</v>
+      </c>
+      <c r="H3" s="4"/>
       <c r="I3" s="4"/>
       <c r="J3" s="4"/>
       <c r="K3" s="4"/>
-      <c r="L3" s="4"/>
+      <c r="L3" s="4" t="s">
+        <v>17</v>
+      </c>
       <c r="M3" s="4"/>
       <c r="N3" s="4"/>
       <c r="O3" s="4"/>
       <c r="P3" s="4"/>
-      <c r="Q3" s="3"/>
-      <c r="R3" s="3"/>
+      <c r="Q3" s="4"/>
+      <c r="R3" s="4"/>
       <c r="S3" s="3"/>
       <c r="T3" s="3"/>
       <c r="U3" s="3"/>
@@ -1194,39 +1226,49 @@
       <c r="AC3" s="3"/>
       <c r="AD3" s="3"/>
       <c r="AE3" s="3"/>
-    </row>
-    <row r="4" spans="2:31">
+      <c r="AF3" s="3"/>
+      <c r="AG3" s="3"/>
+    </row>
+    <row r="4" spans="2:33">
       <c r="B4" s="2" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>9</v>
+        <v>21</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="H4" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="I4" s="2"/>
-      <c r="J4" s="2"/>
-      <c r="K4" s="2"/>
-      <c r="L4" s="2"/>
+        <v>24</v>
+      </c>
+      <c r="I4" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="J4" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="K4" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="L4" s="2" t="s">
+        <v>27</v>
+      </c>
       <c r="M4" s="2"/>
       <c r="N4" s="2"/>
       <c r="O4" s="2"/>
       <c r="P4" s="2"/>
-      <c r="U4" s="3"/>
-      <c r="V4" s="3"/>
+      <c r="Q4" s="2"/>
+      <c r="R4" s="2"/>
       <c r="W4" s="3"/>
       <c r="X4" s="3"/>
       <c r="Y4" s="3"/>
@@ -1236,8 +1278,10 @@
       <c r="AC4" s="3"/>
       <c r="AD4" s="3"/>
       <c r="AE4" s="3"/>
-    </row>
-    <row r="5" spans="1:31">
+      <c r="AF4" s="3"/>
+      <c r="AG4" s="3"/>
+    </row>
+    <row r="5" spans="1:33">
       <c r="A5" s="3"/>
       <c r="B5" s="4"/>
       <c r="C5" s="4"/>
@@ -1254,8 +1298,8 @@
       <c r="N5" s="4"/>
       <c r="O5" s="4"/>
       <c r="P5" s="4"/>
-      <c r="Q5" s="3"/>
-      <c r="R5" s="3"/>
+      <c r="Q5" s="4"/>
+      <c r="R5" s="4"/>
       <c r="S5" s="3"/>
       <c r="T5" s="3"/>
       <c r="U5" s="3"/>
@@ -1269,8 +1313,10 @@
       <c r="AC5" s="3"/>
       <c r="AD5" s="3"/>
       <c r="AE5" s="3"/>
-    </row>
-    <row r="6" s="1" customFormat="1" spans="1:31">
+      <c r="AF5" s="3"/>
+      <c r="AG5" s="3"/>
+    </row>
+    <row r="6" s="1" customFormat="1" spans="1:33">
       <c r="A6" s="3"/>
       <c r="B6" s="4"/>
       <c r="C6" s="4"/>
@@ -1287,8 +1333,8 @@
       <c r="N6" s="4"/>
       <c r="O6" s="4"/>
       <c r="P6" s="4"/>
-      <c r="Q6" s="3"/>
-      <c r="R6" s="3"/>
+      <c r="Q6" s="4"/>
+      <c r="R6" s="4"/>
       <c r="S6" s="3"/>
       <c r="T6" s="3"/>
       <c r="U6" s="3"/>
@@ -1302,8 +1348,10 @@
       <c r="AC6" s="3"/>
       <c r="AD6" s="3"/>
       <c r="AE6" s="3"/>
-    </row>
-    <row r="7" s="1" customFormat="1" spans="1:31">
+      <c r="AF6" s="3"/>
+      <c r="AG6" s="3"/>
+    </row>
+    <row r="7" s="1" customFormat="1" spans="1:33">
       <c r="A7" s="3"/>
       <c r="B7" s="4"/>
       <c r="C7" s="4"/>
@@ -1320,8 +1368,8 @@
       <c r="N7" s="4"/>
       <c r="O7" s="4"/>
       <c r="P7" s="4"/>
-      <c r="Q7" s="3"/>
-      <c r="R7" s="3"/>
+      <c r="Q7" s="4"/>
+      <c r="R7" s="4"/>
       <c r="S7" s="3"/>
       <c r="T7" s="3"/>
       <c r="U7" s="3"/>
@@ -1335,8 +1383,10 @@
       <c r="AC7" s="3"/>
       <c r="AD7" s="3"/>
       <c r="AE7" s="3"/>
-    </row>
-    <row r="8" spans="1:31">
+      <c r="AF7" s="3"/>
+      <c r="AG7" s="3"/>
+    </row>
+    <row r="8" spans="1:33">
       <c r="A8" s="3"/>
       <c r="B8" s="4"/>
       <c r="C8" s="4"/>
@@ -1353,8 +1403,8 @@
       <c r="N8" s="4"/>
       <c r="O8" s="4"/>
       <c r="P8" s="4"/>
-      <c r="Q8" s="3"/>
-      <c r="R8" s="3"/>
+      <c r="Q8" s="4"/>
+      <c r="R8" s="4"/>
       <c r="S8" s="3"/>
       <c r="T8" s="3"/>
       <c r="U8" s="3"/>
@@ -1368,8 +1418,10 @@
       <c r="AC8" s="3"/>
       <c r="AD8" s="3"/>
       <c r="AE8" s="3"/>
-    </row>
-    <row r="9" spans="1:31">
+      <c r="AF8" s="3"/>
+      <c r="AG8" s="3"/>
+    </row>
+    <row r="9" spans="1:33">
       <c r="A9" s="3"/>
       <c r="B9" s="4"/>
       <c r="C9" s="4"/>
@@ -1386,8 +1438,8 @@
       <c r="N9" s="4"/>
       <c r="O9" s="4"/>
       <c r="P9" s="4"/>
-      <c r="Q9" s="3"/>
-      <c r="R9" s="3"/>
+      <c r="Q9" s="4"/>
+      <c r="R9" s="4"/>
       <c r="S9" s="3"/>
       <c r="T9" s="3"/>
       <c r="U9" s="3"/>
@@ -1401,8 +1453,10 @@
       <c r="AC9" s="3"/>
       <c r="AD9" s="3"/>
       <c r="AE9" s="3"/>
-    </row>
-    <row r="10" spans="1:31">
+      <c r="AF9" s="3"/>
+      <c r="AG9" s="3"/>
+    </row>
+    <row r="10" spans="1:33">
       <c r="A10" s="3"/>
       <c r="B10" s="4"/>
       <c r="C10" s="4"/>
@@ -1419,8 +1473,8 @@
       <c r="N10" s="4"/>
       <c r="O10" s="4"/>
       <c r="P10" s="4"/>
-      <c r="Q10" s="3"/>
-      <c r="R10" s="3"/>
+      <c r="Q10" s="4"/>
+      <c r="R10" s="4"/>
       <c r="S10" s="3"/>
       <c r="T10" s="3"/>
       <c r="U10" s="3"/>
@@ -1434,8 +1488,10 @@
       <c r="AC10" s="3"/>
       <c r="AD10" s="3"/>
       <c r="AE10" s="3"/>
-    </row>
-    <row r="11" spans="1:31">
+      <c r="AF10" s="3"/>
+      <c r="AG10" s="3"/>
+    </row>
+    <row r="11" spans="1:33">
       <c r="A11" s="3"/>
       <c r="B11" s="4"/>
       <c r="C11" s="4"/>
@@ -1452,8 +1508,8 @@
       <c r="N11" s="4"/>
       <c r="O11" s="4"/>
       <c r="P11" s="4"/>
-      <c r="Q11" s="3"/>
-      <c r="R11" s="3"/>
+      <c r="Q11" s="4"/>
+      <c r="R11" s="4"/>
       <c r="S11" s="3"/>
       <c r="T11" s="3"/>
       <c r="U11" s="3"/>
@@ -1467,8 +1523,10 @@
       <c r="AC11" s="3"/>
       <c r="AD11" s="3"/>
       <c r="AE11" s="3"/>
-    </row>
-    <row r="12" spans="1:31">
+      <c r="AF11" s="3"/>
+      <c r="AG11" s="3"/>
+    </row>
+    <row r="12" spans="1:33">
       <c r="A12" s="3"/>
       <c r="B12" s="4"/>
       <c r="C12" s="4"/>
@@ -1485,8 +1543,8 @@
       <c r="N12" s="4"/>
       <c r="O12" s="4"/>
       <c r="P12" s="4"/>
-      <c r="Q12" s="3"/>
-      <c r="R12" s="3"/>
+      <c r="Q12" s="4"/>
+      <c r="R12" s="4"/>
       <c r="S12" s="3"/>
       <c r="T12" s="3"/>
       <c r="U12" s="3"/>
@@ -1500,8 +1558,10 @@
       <c r="AC12" s="3"/>
       <c r="AD12" s="3"/>
       <c r="AE12" s="3"/>
-    </row>
-    <row r="13" spans="1:31">
+      <c r="AF12" s="3"/>
+      <c r="AG12" s="3"/>
+    </row>
+    <row r="13" spans="1:33">
       <c r="A13" s="3"/>
       <c r="B13" s="4"/>
       <c r="C13" s="4"/>
@@ -1518,8 +1578,8 @@
       <c r="N13" s="4"/>
       <c r="O13" s="4"/>
       <c r="P13" s="4"/>
-      <c r="Q13" s="3"/>
-      <c r="R13" s="3"/>
+      <c r="Q13" s="4"/>
+      <c r="R13" s="4"/>
       <c r="S13" s="3"/>
       <c r="T13" s="3"/>
       <c r="U13" s="3"/>
@@ -1533,8 +1593,10 @@
       <c r="AC13" s="3"/>
       <c r="AD13" s="3"/>
       <c r="AE13" s="3"/>
-    </row>
-    <row r="14" spans="1:31">
+      <c r="AF13" s="3"/>
+      <c r="AG13" s="3"/>
+    </row>
+    <row r="14" spans="1:33">
       <c r="A14" s="3"/>
       <c r="B14" s="4"/>
       <c r="C14" s="4"/>
@@ -1551,8 +1613,8 @@
       <c r="N14" s="4"/>
       <c r="O14" s="4"/>
       <c r="P14" s="4"/>
-      <c r="Q14" s="3"/>
-      <c r="R14" s="3"/>
+      <c r="Q14" s="4"/>
+      <c r="R14" s="4"/>
       <c r="S14" s="3"/>
       <c r="T14" s="3"/>
       <c r="U14" s="3"/>
@@ -1566,8 +1628,10 @@
       <c r="AC14" s="3"/>
       <c r="AD14" s="3"/>
       <c r="AE14" s="3"/>
-    </row>
-    <row r="15" spans="1:31">
+      <c r="AF14" s="3"/>
+      <c r="AG14" s="3"/>
+    </row>
+    <row r="15" spans="1:33">
       <c r="A15" s="3"/>
       <c r="B15" s="4"/>
       <c r="C15" s="4"/>
@@ -1584,8 +1648,8 @@
       <c r="N15" s="4"/>
       <c r="O15" s="4"/>
       <c r="P15" s="4"/>
-      <c r="Q15" s="3"/>
-      <c r="R15" s="3"/>
+      <c r="Q15" s="4"/>
+      <c r="R15" s="4"/>
       <c r="S15" s="3"/>
       <c r="T15" s="3"/>
       <c r="U15" s="3"/>
@@ -1599,8 +1663,10 @@
       <c r="AC15" s="3"/>
       <c r="AD15" s="3"/>
       <c r="AE15" s="3"/>
-    </row>
-    <row r="16" spans="1:31">
+      <c r="AF15" s="3"/>
+      <c r="AG15" s="3"/>
+    </row>
+    <row r="16" spans="1:33">
       <c r="A16" s="3"/>
       <c r="B16" s="4"/>
       <c r="C16" s="4"/>
@@ -1617,8 +1683,8 @@
       <c r="N16" s="4"/>
       <c r="O16" s="4"/>
       <c r="P16" s="4"/>
-      <c r="Q16" s="3"/>
-      <c r="R16" s="3"/>
+      <c r="Q16" s="4"/>
+      <c r="R16" s="4"/>
       <c r="S16" s="3"/>
       <c r="T16" s="3"/>
       <c r="U16" s="3"/>
@@ -1632,8 +1698,10 @@
       <c r="AC16" s="3"/>
       <c r="AD16" s="3"/>
       <c r="AE16" s="3"/>
-    </row>
-    <row r="17" spans="1:31">
+      <c r="AF16" s="3"/>
+      <c r="AG16" s="3"/>
+    </row>
+    <row r="17" spans="1:33">
       <c r="A17" s="3"/>
       <c r="B17" s="4"/>
       <c r="C17" s="4"/>
@@ -1650,8 +1718,8 @@
       <c r="N17" s="4"/>
       <c r="O17" s="4"/>
       <c r="P17" s="4"/>
-      <c r="Q17" s="3"/>
-      <c r="R17" s="3"/>
+      <c r="Q17" s="4"/>
+      <c r="R17" s="4"/>
       <c r="S17" s="3"/>
       <c r="T17" s="3"/>
       <c r="U17" s="3"/>
@@ -1665,8 +1733,10 @@
       <c r="AC17" s="3"/>
       <c r="AD17" s="3"/>
       <c r="AE17" s="3"/>
-    </row>
-    <row r="18" spans="1:31">
+      <c r="AF17" s="3"/>
+      <c r="AG17" s="3"/>
+    </row>
+    <row r="18" spans="1:33">
       <c r="A18" s="3"/>
       <c r="B18" s="4"/>
       <c r="C18" s="4"/>
@@ -1683,8 +1753,8 @@
       <c r="N18" s="4"/>
       <c r="O18" s="4"/>
       <c r="P18" s="4"/>
-      <c r="Q18" s="3"/>
-      <c r="R18" s="3"/>
+      <c r="Q18" s="4"/>
+      <c r="R18" s="4"/>
       <c r="S18" s="3"/>
       <c r="T18" s="3"/>
       <c r="U18" s="3"/>
@@ -1698,8 +1768,10 @@
       <c r="AC18" s="3"/>
       <c r="AD18" s="3"/>
       <c r="AE18" s="3"/>
-    </row>
-    <row r="19" spans="1:31">
+      <c r="AF18" s="3"/>
+      <c r="AG18" s="3"/>
+    </row>
+    <row r="19" spans="1:33">
       <c r="A19" s="3"/>
       <c r="B19" s="4"/>
       <c r="C19" s="4"/>
@@ -1716,8 +1788,8 @@
       <c r="N19" s="4"/>
       <c r="O19" s="4"/>
       <c r="P19" s="4"/>
-      <c r="Q19" s="3"/>
-      <c r="R19" s="3"/>
+      <c r="Q19" s="4"/>
+      <c r="R19" s="4"/>
       <c r="S19" s="3"/>
       <c r="T19" s="3"/>
       <c r="U19" s="3"/>
@@ -1731,8 +1803,10 @@
       <c r="AC19" s="3"/>
       <c r="AD19" s="3"/>
       <c r="AE19" s="3"/>
-    </row>
-    <row r="20" spans="1:31">
+      <c r="AF19" s="3"/>
+      <c r="AG19" s="3"/>
+    </row>
+    <row r="20" spans="1:33">
       <c r="A20" s="3"/>
       <c r="B20" s="4"/>
       <c r="C20" s="4"/>
@@ -1749,8 +1823,8 @@
       <c r="N20" s="4"/>
       <c r="O20" s="4"/>
       <c r="P20" s="4"/>
-      <c r="Q20" s="3"/>
-      <c r="R20" s="3"/>
+      <c r="Q20" s="4"/>
+      <c r="R20" s="4"/>
       <c r="S20" s="3"/>
       <c r="T20" s="3"/>
       <c r="U20" s="3"/>
@@ -1764,8 +1838,10 @@
       <c r="AC20" s="3"/>
       <c r="AD20" s="3"/>
       <c r="AE20" s="3"/>
-    </row>
-    <row r="21" spans="1:31">
+      <c r="AF20" s="3"/>
+      <c r="AG20" s="3"/>
+    </row>
+    <row r="21" spans="1:33">
       <c r="A21" s="3"/>
       <c r="B21" s="4"/>
       <c r="C21" s="4"/>
@@ -1782,8 +1858,8 @@
       <c r="N21" s="4"/>
       <c r="O21" s="4"/>
       <c r="P21" s="4"/>
-      <c r="Q21" s="3"/>
-      <c r="R21" s="3"/>
+      <c r="Q21" s="4"/>
+      <c r="R21" s="4"/>
       <c r="S21" s="3"/>
       <c r="T21" s="3"/>
       <c r="U21" s="3"/>
@@ -1797,8 +1873,10 @@
       <c r="AC21" s="3"/>
       <c r="AD21" s="3"/>
       <c r="AE21" s="3"/>
-    </row>
-    <row r="22" spans="1:31">
+      <c r="AF21" s="3"/>
+      <c r="AG21" s="3"/>
+    </row>
+    <row r="22" spans="1:33">
       <c r="A22" s="3"/>
       <c r="B22" s="4"/>
       <c r="C22" s="4"/>
@@ -1815,8 +1893,8 @@
       <c r="N22" s="4"/>
       <c r="O22" s="4"/>
       <c r="P22" s="4"/>
-      <c r="Q22" s="3"/>
-      <c r="R22" s="3"/>
+      <c r="Q22" s="4"/>
+      <c r="R22" s="4"/>
       <c r="S22" s="3"/>
       <c r="T22" s="3"/>
       <c r="U22" s="3"/>
@@ -1830,8 +1908,10 @@
       <c r="AC22" s="3"/>
       <c r="AD22" s="3"/>
       <c r="AE22" s="3"/>
-    </row>
-    <row r="23" spans="1:31">
+      <c r="AF22" s="3"/>
+      <c r="AG22" s="3"/>
+    </row>
+    <row r="23" spans="1:33">
       <c r="A23" s="3"/>
       <c r="B23" s="4"/>
       <c r="C23" s="4"/>
@@ -1848,8 +1928,8 @@
       <c r="N23" s="4"/>
       <c r="O23" s="4"/>
       <c r="P23" s="4"/>
-      <c r="Q23" s="3"/>
-      <c r="R23" s="3"/>
+      <c r="Q23" s="4"/>
+      <c r="R23" s="4"/>
       <c r="S23" s="3"/>
       <c r="T23" s="3"/>
       <c r="U23" s="3"/>
@@ -1863,8 +1943,10 @@
       <c r="AC23" s="3"/>
       <c r="AD23" s="3"/>
       <c r="AE23" s="3"/>
-    </row>
-    <row r="24" spans="1:31">
+      <c r="AF23" s="3"/>
+      <c r="AG23" s="3"/>
+    </row>
+    <row r="24" spans="1:33">
       <c r="A24" s="3"/>
       <c r="B24" s="4"/>
       <c r="C24" s="4"/>
@@ -1881,8 +1963,8 @@
       <c r="N24" s="4"/>
       <c r="O24" s="4"/>
       <c r="P24" s="4"/>
-      <c r="Q24" s="3"/>
-      <c r="R24" s="3"/>
+      <c r="Q24" s="4"/>
+      <c r="R24" s="4"/>
       <c r="S24" s="3"/>
       <c r="T24" s="3"/>
       <c r="U24" s="3"/>
@@ -1896,8 +1978,10 @@
       <c r="AC24" s="3"/>
       <c r="AD24" s="3"/>
       <c r="AE24" s="3"/>
-    </row>
-    <row r="25" spans="1:31">
+      <c r="AF24" s="3"/>
+      <c r="AG24" s="3"/>
+    </row>
+    <row r="25" spans="1:33">
       <c r="A25" s="3"/>
       <c r="B25" s="4"/>
       <c r="C25" s="4"/>
@@ -1914,8 +1998,8 @@
       <c r="N25" s="4"/>
       <c r="O25" s="4"/>
       <c r="P25" s="4"/>
-      <c r="Q25" s="3"/>
-      <c r="R25" s="3"/>
+      <c r="Q25" s="4"/>
+      <c r="R25" s="4"/>
       <c r="S25" s="3"/>
       <c r="T25" s="3"/>
       <c r="U25" s="3"/>
@@ -1929,8 +2013,10 @@
       <c r="AC25" s="3"/>
       <c r="AD25" s="3"/>
       <c r="AE25" s="3"/>
-    </row>
-    <row r="26" spans="1:31">
+      <c r="AF25" s="3"/>
+      <c r="AG25" s="3"/>
+    </row>
+    <row r="26" spans="1:33">
       <c r="A26" s="3"/>
       <c r="B26" s="4"/>
       <c r="C26" s="4"/>
@@ -1947,8 +2033,8 @@
       <c r="N26" s="4"/>
       <c r="O26" s="4"/>
       <c r="P26" s="4"/>
-      <c r="Q26" s="3"/>
-      <c r="R26" s="3"/>
+      <c r="Q26" s="4"/>
+      <c r="R26" s="4"/>
       <c r="S26" s="3"/>
       <c r="T26" s="3"/>
       <c r="U26" s="3"/>
@@ -1962,8 +2048,10 @@
       <c r="AC26" s="3"/>
       <c r="AD26" s="3"/>
       <c r="AE26" s="3"/>
-    </row>
-    <row r="27" spans="1:31">
+      <c r="AF26" s="3"/>
+      <c r="AG26" s="3"/>
+    </row>
+    <row r="27" spans="1:33">
       <c r="A27" s="3"/>
       <c r="B27" s="4"/>
       <c r="C27" s="4"/>
@@ -1980,8 +2068,8 @@
       <c r="N27" s="4"/>
       <c r="O27" s="4"/>
       <c r="P27" s="4"/>
-      <c r="Q27" s="3"/>
-      <c r="R27" s="3"/>
+      <c r="Q27" s="4"/>
+      <c r="R27" s="4"/>
       <c r="S27" s="3"/>
       <c r="T27" s="3"/>
       <c r="U27" s="3"/>
@@ -1995,8 +2083,10 @@
       <c r="AC27" s="3"/>
       <c r="AD27" s="3"/>
       <c r="AE27" s="3"/>
-    </row>
-    <row r="28" spans="1:31">
+      <c r="AF27" s="3"/>
+      <c r="AG27" s="3"/>
+    </row>
+    <row r="28" spans="1:33">
       <c r="A28" s="3"/>
       <c r="B28" s="4"/>
       <c r="C28" s="4"/>
@@ -2013,8 +2103,8 @@
       <c r="N28" s="4"/>
       <c r="O28" s="4"/>
       <c r="P28" s="4"/>
-      <c r="Q28" s="3"/>
-      <c r="R28" s="3"/>
+      <c r="Q28" s="4"/>
+      <c r="R28" s="4"/>
       <c r="S28" s="3"/>
       <c r="T28" s="3"/>
       <c r="U28" s="3"/>
@@ -2028,8 +2118,10 @@
       <c r="AC28" s="3"/>
       <c r="AD28" s="3"/>
       <c r="AE28" s="3"/>
-    </row>
-    <row r="29" spans="1:31">
+      <c r="AF28" s="3"/>
+      <c r="AG28" s="3"/>
+    </row>
+    <row r="29" spans="1:33">
       <c r="A29" s="3"/>
       <c r="B29" s="4"/>
       <c r="C29" s="4"/>
@@ -2046,8 +2138,8 @@
       <c r="N29" s="4"/>
       <c r="O29" s="4"/>
       <c r="P29" s="4"/>
-      <c r="Q29" s="3"/>
-      <c r="R29" s="3"/>
+      <c r="Q29" s="4"/>
+      <c r="R29" s="4"/>
       <c r="S29" s="3"/>
       <c r="T29" s="3"/>
       <c r="U29" s="3"/>
@@ -2061,8 +2153,10 @@
       <c r="AC29" s="3"/>
       <c r="AD29" s="3"/>
       <c r="AE29" s="3"/>
-    </row>
-    <row r="30" spans="1:31">
+      <c r="AF29" s="3"/>
+      <c r="AG29" s="3"/>
+    </row>
+    <row r="30" spans="1:33">
       <c r="A30" s="3"/>
       <c r="B30" s="4"/>
       <c r="C30" s="4"/>
@@ -2079,8 +2173,8 @@
       <c r="N30" s="4"/>
       <c r="O30" s="4"/>
       <c r="P30" s="4"/>
-      <c r="Q30" s="3"/>
-      <c r="R30" s="3"/>
+      <c r="Q30" s="4"/>
+      <c r="R30" s="4"/>
       <c r="S30" s="3"/>
       <c r="T30" s="3"/>
       <c r="U30" s="3"/>
@@ -2094,8 +2188,10 @@
       <c r="AC30" s="3"/>
       <c r="AD30" s="3"/>
       <c r="AE30" s="3"/>
-    </row>
-    <row r="31" spans="1:31">
+      <c r="AF30" s="3"/>
+      <c r="AG30" s="3"/>
+    </row>
+    <row r="31" spans="1:33">
       <c r="A31" s="3"/>
       <c r="B31" s="4"/>
       <c r="C31" s="4"/>
@@ -2112,8 +2208,8 @@
       <c r="N31" s="4"/>
       <c r="O31" s="4"/>
       <c r="P31" s="4"/>
-      <c r="Q31" s="3"/>
-      <c r="R31" s="3"/>
+      <c r="Q31" s="4"/>
+      <c r="R31" s="4"/>
       <c r="S31" s="3"/>
       <c r="T31" s="3"/>
       <c r="U31" s="3"/>
@@ -2127,8 +2223,10 @@
       <c r="AC31" s="3"/>
       <c r="AD31" s="3"/>
       <c r="AE31" s="3"/>
-    </row>
-    <row r="32" spans="1:31">
+      <c r="AF31" s="3"/>
+      <c r="AG31" s="3"/>
+    </row>
+    <row r="32" spans="1:33">
       <c r="A32" s="3"/>
       <c r="B32" s="4"/>
       <c r="C32" s="4"/>
@@ -2145,8 +2243,8 @@
       <c r="N32" s="4"/>
       <c r="O32" s="4"/>
       <c r="P32" s="4"/>
-      <c r="Q32" s="3"/>
-      <c r="R32" s="3"/>
+      <c r="Q32" s="4"/>
+      <c r="R32" s="4"/>
       <c r="S32" s="3"/>
       <c r="T32" s="3"/>
       <c r="U32" s="3"/>
@@ -2160,8 +2258,10 @@
       <c r="AC32" s="3"/>
       <c r="AD32" s="3"/>
       <c r="AE32" s="3"/>
-    </row>
-    <row r="33" spans="1:31">
+      <c r="AF32" s="3"/>
+      <c r="AG32" s="3"/>
+    </row>
+    <row r="33" spans="1:33">
       <c r="A33" s="3"/>
       <c r="B33" s="4"/>
       <c r="C33" s="4"/>
@@ -2178,8 +2278,8 @@
       <c r="N33" s="4"/>
       <c r="O33" s="4"/>
       <c r="P33" s="4"/>
-      <c r="Q33" s="3"/>
-      <c r="R33" s="3"/>
+      <c r="Q33" s="4"/>
+      <c r="R33" s="4"/>
       <c r="S33" s="3"/>
       <c r="T33" s="3"/>
       <c r="U33" s="3"/>
@@ -2193,8 +2293,10 @@
       <c r="AC33" s="3"/>
       <c r="AD33" s="3"/>
       <c r="AE33" s="3"/>
-    </row>
-    <row r="34" spans="1:31">
+      <c r="AF33" s="3"/>
+      <c r="AG33" s="3"/>
+    </row>
+    <row r="34" spans="1:33">
       <c r="A34" s="3"/>
       <c r="B34" s="4"/>
       <c r="C34" s="4"/>
@@ -2211,8 +2313,8 @@
       <c r="N34" s="4"/>
       <c r="O34" s="4"/>
       <c r="P34" s="4"/>
-      <c r="Q34" s="3"/>
-      <c r="R34" s="3"/>
+      <c r="Q34" s="4"/>
+      <c r="R34" s="4"/>
       <c r="S34" s="3"/>
       <c r="T34" s="3"/>
       <c r="U34" s="3"/>
@@ -2226,8 +2328,10 @@
       <c r="AC34" s="3"/>
       <c r="AD34" s="3"/>
       <c r="AE34" s="3"/>
-    </row>
-    <row r="35" spans="1:31">
+      <c r="AF34" s="3"/>
+      <c r="AG34" s="3"/>
+    </row>
+    <row r="35" spans="1:33">
       <c r="A35" s="3"/>
       <c r="B35" s="4"/>
       <c r="C35" s="4"/>
@@ -2244,8 +2348,8 @@
       <c r="N35" s="4"/>
       <c r="O35" s="4"/>
       <c r="P35" s="4"/>
-      <c r="Q35" s="3"/>
-      <c r="R35" s="3"/>
+      <c r="Q35" s="4"/>
+      <c r="R35" s="4"/>
       <c r="S35" s="3"/>
       <c r="T35" s="3"/>
       <c r="U35" s="3"/>
@@ -2259,8 +2363,10 @@
       <c r="AC35" s="3"/>
       <c r="AD35" s="3"/>
       <c r="AE35" s="3"/>
-    </row>
-    <row r="36" spans="1:31">
+      <c r="AF35" s="3"/>
+      <c r="AG35" s="3"/>
+    </row>
+    <row r="36" spans="1:33">
       <c r="A36" s="3"/>
       <c r="B36" s="4"/>
       <c r="C36" s="4"/>
@@ -2277,8 +2383,8 @@
       <c r="N36" s="4"/>
       <c r="O36" s="4"/>
       <c r="P36" s="4"/>
-      <c r="Q36" s="3"/>
-      <c r="R36" s="3"/>
+      <c r="Q36" s="4"/>
+      <c r="R36" s="4"/>
       <c r="S36" s="3"/>
       <c r="T36" s="3"/>
       <c r="U36" s="3"/>
@@ -2292,8 +2398,10 @@
       <c r="AC36" s="3"/>
       <c r="AD36" s="3"/>
       <c r="AE36" s="3"/>
-    </row>
-    <row r="37" spans="1:31">
+      <c r="AF36" s="3"/>
+      <c r="AG36" s="3"/>
+    </row>
+    <row r="37" spans="1:33">
       <c r="A37" s="3"/>
       <c r="B37" s="4"/>
       <c r="C37" s="4"/>
@@ -2310,8 +2418,8 @@
       <c r="N37" s="4"/>
       <c r="O37" s="4"/>
       <c r="P37" s="4"/>
-      <c r="Q37" s="3"/>
-      <c r="R37" s="3"/>
+      <c r="Q37" s="4"/>
+      <c r="R37" s="4"/>
       <c r="S37" s="3"/>
       <c r="T37" s="3"/>
       <c r="U37" s="3"/>
@@ -2325,8 +2433,10 @@
       <c r="AC37" s="3"/>
       <c r="AD37" s="3"/>
       <c r="AE37" s="3"/>
-    </row>
-    <row r="38" spans="1:31">
+      <c r="AF37" s="3"/>
+      <c r="AG37" s="3"/>
+    </row>
+    <row r="38" spans="1:33">
       <c r="A38" s="3"/>
       <c r="B38" s="4"/>
       <c r="C38" s="4"/>
@@ -2343,8 +2453,8 @@
       <c r="N38" s="4"/>
       <c r="O38" s="4"/>
       <c r="P38" s="4"/>
-      <c r="Q38" s="3"/>
-      <c r="R38" s="3"/>
+      <c r="Q38" s="4"/>
+      <c r="R38" s="4"/>
       <c r="S38" s="3"/>
       <c r="T38" s="3"/>
       <c r="U38" s="3"/>
@@ -2358,176 +2468,207 @@
       <c r="AC38" s="3"/>
       <c r="AD38" s="3"/>
       <c r="AE38" s="3"/>
-    </row>
-    <row r="46" spans="1:20">
+      <c r="AF38" s="3"/>
+      <c r="AG38" s="3"/>
+    </row>
+    <row r="46" spans="1:22">
       <c r="A46" s="2"/>
       <c r="B46" s="2"/>
       <c r="C46" s="2"/>
       <c r="D46" s="2"/>
-      <c r="O46" s="2"/>
       <c r="Q46" s="2"/>
-      <c r="R46" s="2"/>
       <c r="S46" s="2"/>
       <c r="T46" s="2"/>
-    </row>
-    <row r="47" spans="1:20">
+      <c r="U46" s="2"/>
+      <c r="V46" s="2"/>
+    </row>
+    <row r="47" spans="1:22">
       <c r="A47" s="2"/>
       <c r="B47" s="2"/>
       <c r="C47" s="2"/>
       <c r="D47" s="2"/>
       <c r="E47" s="2"/>
-      <c r="O47" s="2"/>
-      <c r="P47" s="2"/>
       <c r="Q47" s="2"/>
       <c r="R47" s="2"/>
       <c r="S47" s="2"/>
       <c r="T47" s="2"/>
-    </row>
-    <row r="48" spans="1:20">
+      <c r="U47" s="2"/>
+      <c r="V47" s="2"/>
+    </row>
+    <row r="48" spans="1:22">
       <c r="A48" s="2"/>
       <c r="B48" s="2"/>
       <c r="C48" s="2"/>
       <c r="D48" s="2"/>
-      <c r="O48" s="2"/>
-      <c r="P48" s="2"/>
       <c r="Q48" s="2"/>
       <c r="R48" s="2"/>
       <c r="S48" s="2"/>
       <c r="T48" s="2"/>
-    </row>
-    <row r="49" spans="1:20">
+      <c r="U48" s="2"/>
+      <c r="V48" s="2"/>
+    </row>
+    <row r="49" spans="1:22">
       <c r="A49" s="2"/>
       <c r="B49" s="2"/>
       <c r="C49" s="2"/>
       <c r="D49" s="2"/>
-      <c r="O49" s="2"/>
-      <c r="P49" s="2"/>
       <c r="Q49" s="2"/>
       <c r="R49" s="2"/>
       <c r="S49" s="2"/>
       <c r="T49" s="2"/>
-    </row>
-    <row r="50" spans="1:20">
+      <c r="U49" s="2"/>
+      <c r="V49" s="2"/>
+    </row>
+    <row r="50" spans="1:22">
       <c r="A50" s="2"/>
       <c r="B50" s="2"/>
       <c r="C50" s="2"/>
       <c r="D50" s="2"/>
-      <c r="O50" s="2"/>
-      <c r="P50" s="2"/>
       <c r="Q50" s="2"/>
       <c r="R50" s="2"/>
       <c r="S50" s="2"/>
       <c r="T50" s="2"/>
-    </row>
-    <row r="51" spans="1:20">
+      <c r="U50" s="2"/>
+      <c r="V50" s="2"/>
+    </row>
+    <row r="51" spans="1:22">
       <c r="A51" s="2"/>
       <c r="B51" s="2"/>
       <c r="C51" s="2"/>
       <c r="D51" s="2"/>
-      <c r="O51" s="2"/>
-      <c r="P51" s="2"/>
       <c r="Q51" s="2"/>
       <c r="R51" s="2"/>
       <c r="S51" s="2"/>
       <c r="T51" s="2"/>
-    </row>
-    <row r="52" spans="1:20">
+      <c r="U51" s="2"/>
+      <c r="V51" s="2"/>
+    </row>
+    <row r="52" spans="1:22">
       <c r="A52" s="2"/>
       <c r="B52" s="2"/>
       <c r="C52" s="2"/>
       <c r="D52" s="2"/>
-      <c r="O52" s="2"/>
-      <c r="P52" s="2"/>
       <c r="Q52" s="2"/>
       <c r="R52" s="2"/>
       <c r="S52" s="2"/>
       <c r="T52" s="2"/>
-    </row>
-    <row r="53" spans="1:20">
+      <c r="U52" s="2"/>
+      <c r="V52" s="2"/>
+    </row>
+    <row r="53" spans="1:22">
       <c r="A53" s="2"/>
       <c r="B53" s="2"/>
       <c r="C53" s="2"/>
       <c r="D53" s="2"/>
-      <c r="O53" s="2"/>
-      <c r="P53" s="2"/>
       <c r="Q53" s="2"/>
       <c r="R53" s="2"/>
       <c r="S53" s="2"/>
       <c r="T53" s="2"/>
-    </row>
-    <row r="54" spans="1:20">
+      <c r="U53" s="2"/>
+      <c r="V53" s="2"/>
+    </row>
+    <row r="54" spans="1:22">
       <c r="A54" s="2"/>
       <c r="B54" s="2"/>
       <c r="C54" s="2"/>
       <c r="D54" s="2"/>
-      <c r="O54" s="2"/>
-      <c r="P54" s="2"/>
       <c r="Q54" s="2"/>
       <c r="R54" s="2"/>
       <c r="S54" s="2"/>
       <c r="T54" s="2"/>
-    </row>
-    <row r="55" spans="1:20">
+      <c r="U54" s="2"/>
+      <c r="V54" s="2"/>
+    </row>
+    <row r="55" spans="1:22">
       <c r="A55" s="2"/>
       <c r="B55" s="2"/>
       <c r="C55" s="2"/>
       <c r="D55" s="2"/>
-      <c r="O55" s="2"/>
-      <c r="P55" s="2"/>
       <c r="Q55" s="2"/>
       <c r="R55" s="2"/>
       <c r="S55" s="2"/>
       <c r="T55" s="2"/>
-    </row>
-    <row r="56" spans="1:20">
+      <c r="U55" s="2"/>
+      <c r="V55" s="2"/>
+    </row>
+    <row r="56" spans="1:22">
       <c r="A56" s="2"/>
       <c r="B56" s="2"/>
       <c r="C56" s="2"/>
       <c r="D56" s="2"/>
-      <c r="O56" s="2"/>
-      <c r="P56" s="2"/>
       <c r="Q56" s="2"/>
       <c r="R56" s="2"/>
       <c r="S56" s="2"/>
       <c r="T56" s="2"/>
-    </row>
-    <row r="57" spans="1:20">
+      <c r="U56" s="2"/>
+      <c r="V56" s="2"/>
+    </row>
+    <row r="57" spans="1:22">
       <c r="A57" s="2"/>
       <c r="B57" s="2"/>
       <c r="C57" s="2"/>
       <c r="D57" s="2"/>
-      <c r="O57" s="2"/>
-      <c r="P57" s="2"/>
       <c r="Q57" s="2"/>
       <c r="R57" s="2"/>
       <c r="S57" s="2"/>
       <c r="T57" s="2"/>
-    </row>
-    <row r="58" spans="1:20">
+      <c r="U57" s="2"/>
+      <c r="V57" s="2"/>
+    </row>
+    <row r="58" spans="1:22">
       <c r="A58" s="2"/>
       <c r="B58" s="2"/>
       <c r="C58" s="2"/>
       <c r="D58" s="2"/>
-      <c r="O58" s="2"/>
-      <c r="P58" s="2"/>
       <c r="Q58" s="2"/>
       <c r="R58" s="2"/>
       <c r="S58" s="2"/>
       <c r="T58" s="2"/>
-    </row>
-    <row r="59" spans="1:20">
+      <c r="U58" s="2"/>
+      <c r="V58" s="2"/>
+    </row>
+    <row r="59" spans="1:22">
       <c r="A59" s="2"/>
       <c r="B59" s="2"/>
       <c r="C59" s="2"/>
       <c r="D59" s="2"/>
-      <c r="O59" s="2"/>
-      <c r="P59" s="2"/>
       <c r="Q59" s="2"/>
       <c r="R59" s="2"/>
       <c r="S59" s="2"/>
       <c r="T59" s="2"/>
+      <c r="U59" s="2"/>
+      <c r="V59" s="2"/>
     </row>
   </sheetData>
+  <dataValidations count="9">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K2:K1048576">
+      <formula1>"MASK_XX,MASK_B,MASK_H,MASK_W,MASK_D"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L2:L1048576">
+      <formula1>"INST_VALID,INST_INVALID"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I2:I1048576">
+      <formula1>"LD_LB,LD_LH,LD_LW,LD_LBU,LD_LHU,LD_XX"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H2:H1048576 J2:J1048576">
+      <formula1>"WB_ALU,WB_MEM,WB_PC,WB_XX"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G2:G1048576">
+      <formula1>"IMM_I,IMM_J,IMM_U,IMM_S,IMM_B"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F2:F1048576">
+      <formula1>"ALU_ADD,ALU_SUB,ALU_AND,ALU_OR,ALU_XOR,ALU_SLL,ALU_SRL,ALU_SLT,ALU_SLTU,ALU_COPY_A,ALU_COPY_B"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D2:D1048576">
+      <formula1>"A_PC,A_RS1"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E2:E1048576">
+      <formula1>"B_IMM,B_RS2"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C2:C1048576">
+      <formula1>"PC_4,PC_0,PC_ALU"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>
 </worksheet>

</xml_diff>

<commit_message>
> sim RTL ysyx_23060246 韩炳晋 Linux archlinux 6.6.60-1-lts #1 SMP PREEMPT_DYNAMIC Fri, 08 Nov 2024 16:03:02 +0000 x86_64 GNU/Linux  14:02:03 up 20:17,  2 users,  load average: 0.88, 1.52, 1.72
</commit_message>
<xml_diff>
--- a/npc/tools/control_gen/control_table.xlsx
+++ b/npc/tools/control_gen/control_table.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="30">
   <si>
     <t>commont</t>
   </si>
@@ -76,16 +76,22 @@
     <t>ALU_ADD</t>
   </si>
   <si>
+    <t>addi</t>
+  </si>
+  <si>
+    <t>A_RS1</t>
+  </si>
+  <si>
+    <t>IMM_I</t>
+  </si>
+  <si>
+    <t>WB_ALU</t>
+  </si>
+  <si>
     <t>default</t>
   </si>
   <si>
     <t>PC_4</t>
-  </si>
-  <si>
-    <t>A_RS1</t>
-  </si>
-  <si>
-    <t>IMM_I</t>
   </si>
   <si>
     <t>WB_XX</t>
@@ -1066,7 +1072,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:AG59"/>
+  <dimension ref="A1:AG60"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
     <col min="1" max="1" width="13.1" customWidth="1"/>
@@ -1229,46 +1235,43 @@
       <c r="AF3" s="3"/>
       <c r="AG3" s="3"/>
     </row>
-    <row r="4" spans="2:33">
-      <c r="B4" s="2" t="s">
+    <row r="4" spans="1:33">
+      <c r="A4" s="3"/>
+      <c r="B4" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="C4" s="2"/>
+      <c r="D4" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="D4" s="2" t="s">
+      <c r="E4" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="F4" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="G4" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="E4" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="F4" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="G4" s="2" t="s">
+      <c r="H4" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="H4" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="I4" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="J4" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="K4" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="L4" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="M4" s="2"/>
-      <c r="N4" s="2"/>
-      <c r="O4" s="2"/>
-      <c r="P4" s="2"/>
-      <c r="Q4" s="2"/>
-      <c r="R4" s="2"/>
+      <c r="I4" s="4"/>
+      <c r="J4" s="4"/>
+      <c r="K4" s="4"/>
+      <c r="L4" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="M4" s="4"/>
+      <c r="N4" s="4"/>
+      <c r="O4" s="4"/>
+      <c r="P4" s="4"/>
+      <c r="Q4" s="4"/>
+      <c r="R4" s="4"/>
+      <c r="S4" s="3"/>
+      <c r="T4" s="3"/>
+      <c r="U4" s="3"/>
+      <c r="V4" s="3"/>
       <c r="W4" s="3"/>
       <c r="X4" s="3"/>
       <c r="Y4" s="3"/>
@@ -1281,29 +1284,46 @@
       <c r="AF4" s="3"/>
       <c r="AG4" s="3"/>
     </row>
-    <row r="5" spans="1:33">
-      <c r="A5" s="3"/>
-      <c r="B5" s="4"/>
-      <c r="C5" s="4"/>
-      <c r="D5" s="4"/>
-      <c r="E5" s="4"/>
-      <c r="F5" s="4"/>
-      <c r="G5" s="4"/>
-      <c r="H5" s="4"/>
-      <c r="I5" s="4"/>
-      <c r="J5" s="4"/>
-      <c r="K5" s="4"/>
-      <c r="L5" s="4"/>
-      <c r="M5" s="4"/>
-      <c r="N5" s="4"/>
-      <c r="O5" s="4"/>
-      <c r="P5" s="4"/>
-      <c r="Q5" s="4"/>
-      <c r="R5" s="4"/>
-      <c r="S5" s="3"/>
-      <c r="T5" s="3"/>
-      <c r="U5" s="3"/>
-      <c r="V5" s="3"/>
+    <row r="5" spans="2:33">
+      <c r="B5" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="G5" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="H5" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="I5" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="J5" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="K5" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="L5" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="M5" s="2"/>
+      <c r="N5" s="2"/>
+      <c r="O5" s="2"/>
+      <c r="P5" s="2"/>
+      <c r="Q5" s="2"/>
+      <c r="R5" s="2"/>
       <c r="W5" s="3"/>
       <c r="X5" s="3"/>
       <c r="Y5" s="3"/>
@@ -1316,7 +1336,7 @@
       <c r="AF5" s="3"/>
       <c r="AG5" s="3"/>
     </row>
-    <row r="6" s="1" customFormat="1" spans="1:33">
+    <row r="6" spans="1:33">
       <c r="A6" s="3"/>
       <c r="B6" s="4"/>
       <c r="C6" s="4"/>
@@ -1386,7 +1406,7 @@
       <c r="AF7" s="3"/>
       <c r="AG7" s="3"/>
     </row>
-    <row r="8" spans="1:33">
+    <row r="8" s="1" customFormat="1" spans="1:33">
       <c r="A8" s="3"/>
       <c r="B8" s="4"/>
       <c r="C8" s="4"/>
@@ -1916,7 +1936,7 @@
       <c r="B23" s="4"/>
       <c r="C23" s="4"/>
       <c r="D23" s="4"/>
-      <c r="E23" s="5"/>
+      <c r="E23" s="4"/>
       <c r="F23" s="4"/>
       <c r="G23" s="4"/>
       <c r="H23" s="4"/>
@@ -2021,7 +2041,7 @@
       <c r="B26" s="4"/>
       <c r="C26" s="4"/>
       <c r="D26" s="4"/>
-      <c r="E26" s="4"/>
+      <c r="E26" s="5"/>
       <c r="F26" s="4"/>
       <c r="G26" s="4"/>
       <c r="H26" s="4"/>
@@ -2161,7 +2181,7 @@
       <c r="B30" s="4"/>
       <c r="C30" s="4"/>
       <c r="D30" s="4"/>
-      <c r="E30" s="5"/>
+      <c r="E30" s="4"/>
       <c r="F30" s="4"/>
       <c r="G30" s="4"/>
       <c r="H30" s="4"/>
@@ -2196,7 +2216,7 @@
       <c r="B31" s="4"/>
       <c r="C31" s="4"/>
       <c r="D31" s="4"/>
-      <c r="E31" s="4"/>
+      <c r="E31" s="5"/>
       <c r="F31" s="4"/>
       <c r="G31" s="4"/>
       <c r="H31" s="4"/>
@@ -2471,25 +2491,47 @@
       <c r="AF38" s="3"/>
       <c r="AG38" s="3"/>
     </row>
-    <row r="46" spans="1:22">
-      <c r="A46" s="2"/>
-      <c r="B46" s="2"/>
-      <c r="C46" s="2"/>
-      <c r="D46" s="2"/>
-      <c r="Q46" s="2"/>
-      <c r="S46" s="2"/>
-      <c r="T46" s="2"/>
-      <c r="U46" s="2"/>
-      <c r="V46" s="2"/>
+    <row r="39" spans="1:33">
+      <c r="A39" s="3"/>
+      <c r="B39" s="4"/>
+      <c r="C39" s="4"/>
+      <c r="D39" s="4"/>
+      <c r="E39" s="4"/>
+      <c r="F39" s="4"/>
+      <c r="G39" s="4"/>
+      <c r="H39" s="4"/>
+      <c r="I39" s="4"/>
+      <c r="J39" s="4"/>
+      <c r="K39" s="4"/>
+      <c r="L39" s="4"/>
+      <c r="M39" s="4"/>
+      <c r="N39" s="4"/>
+      <c r="O39" s="4"/>
+      <c r="P39" s="4"/>
+      <c r="Q39" s="4"/>
+      <c r="R39" s="4"/>
+      <c r="S39" s="3"/>
+      <c r="T39" s="3"/>
+      <c r="U39" s="3"/>
+      <c r="V39" s="3"/>
+      <c r="W39" s="3"/>
+      <c r="X39" s="3"/>
+      <c r="Y39" s="3"/>
+      <c r="Z39" s="3"/>
+      <c r="AA39" s="3"/>
+      <c r="AB39" s="3"/>
+      <c r="AC39" s="3"/>
+      <c r="AD39" s="3"/>
+      <c r="AE39" s="3"/>
+      <c r="AF39" s="3"/>
+      <c r="AG39" s="3"/>
     </row>
     <row r="47" spans="1:22">
       <c r="A47" s="2"/>
       <c r="B47" s="2"/>
       <c r="C47" s="2"/>
       <c r="D47" s="2"/>
-      <c r="E47" s="2"/>
       <c r="Q47" s="2"/>
-      <c r="R47" s="2"/>
       <c r="S47" s="2"/>
       <c r="T47" s="2"/>
       <c r="U47" s="2"/>
@@ -2500,6 +2542,7 @@
       <c r="B48" s="2"/>
       <c r="C48" s="2"/>
       <c r="D48" s="2"/>
+      <c r="E48" s="2"/>
       <c r="Q48" s="2"/>
       <c r="R48" s="2"/>
       <c r="S48" s="2"/>
@@ -2639,33 +2682,45 @@
       <c r="U59" s="2"/>
       <c r="V59" s="2"/>
     </row>
+    <row r="60" spans="1:22">
+      <c r="A60" s="2"/>
+      <c r="B60" s="2"/>
+      <c r="C60" s="2"/>
+      <c r="D60" s="2"/>
+      <c r="Q60" s="2"/>
+      <c r="R60" s="2"/>
+      <c r="S60" s="2"/>
+      <c r="T60" s="2"/>
+      <c r="U60" s="2"/>
+      <c r="V60" s="2"/>
+    </row>
   </sheetData>
   <dataValidations count="9">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K2:K1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K4 K2:K3 K5:K1048576">
       <formula1>"MASK_XX,MASK_B,MASK_H,MASK_W,MASK_D"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L2:L1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L4 L2:L3 L5:L1048576">
       <formula1>"INST_VALID,INST_INVALID"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I2:I1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I4 I2:I3 I5:I1048576">
       <formula1>"LD_LB,LD_LH,LD_LW,LD_LBU,LD_LHU,LD_XX"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H2:H1048576 J2:J1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H4 J4 H2:H3 H5:H1048576 J2:J3 J5:J1048576">
       <formula1>"WB_ALU,WB_MEM,WB_PC,WB_XX"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G2:G1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G4 G2:G3 G5:G1048576">
       <formula1>"IMM_I,IMM_J,IMM_U,IMM_S,IMM_B"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F2:F1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F4 F2:F3 F5:F1048576">
       <formula1>"ALU_ADD,ALU_SUB,ALU_AND,ALU_OR,ALU_XOR,ALU_SLL,ALU_SRL,ALU_SLT,ALU_SLTU,ALU_COPY_A,ALU_COPY_B"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D2:D1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D4 D2:D3 D5:D1048576">
       <formula1>"A_PC,A_RS1"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E2:E1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E4 E2:E3 E5:E1048576">
       <formula1>"B_IMM,B_RS2"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C2:C1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C4 C2:C3 C5:C1048576">
       <formula1>"PC_4,PC_0,PC_ALU"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
> sim RTL ysyx_23060246 韩炳晋 Linux archlinux 6.6.60-1-lts #1 SMP PREEMPT_DYNAMIC Fri, 08 Nov 2024 16:03:02 +0000 x86_64 GNU/Linux  16:40:47 up 22:55,  2 users,  load average: 2.71, 2.16, 2.38
</commit_message>
<xml_diff>
--- a/npc/tools/control_gen/control_table.xlsx
+++ b/npc/tools/control_gen/control_table.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="34">
   <si>
     <t>commont</t>
   </si>
@@ -55,24 +55,27 @@
     <t>lui</t>
   </si>
   <si>
+    <t>B_IMM</t>
+  </si>
+  <si>
+    <t>ALU_COPY_B</t>
+  </si>
+  <si>
+    <t>IMM_U</t>
+  </si>
+  <si>
+    <t>WB_ALU</t>
+  </si>
+  <si>
+    <t>INST_VALID</t>
+  </si>
+  <si>
+    <t>auipc</t>
+  </si>
+  <si>
     <t>A_PC</t>
   </si>
   <si>
-    <t>B_IMM</t>
-  </si>
-  <si>
-    <t>ALU_COPY_B</t>
-  </si>
-  <si>
-    <t>IMM_U</t>
-  </si>
-  <si>
-    <t>INST_VALID</t>
-  </si>
-  <si>
-    <t>auipc</t>
-  </si>
-  <si>
     <t>ALU_ADD</t>
   </si>
   <si>
@@ -85,7 +88,16 @@
     <t>IMM_I</t>
   </si>
   <si>
-    <t>WB_ALU</t>
+    <t>jal</t>
+  </si>
+  <si>
+    <t>PC_ALU</t>
+  </si>
+  <si>
+    <t>IMM_J</t>
+  </si>
+  <si>
+    <t>WB_PC</t>
   </si>
   <si>
     <t>default</t>
@@ -1072,7 +1084,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:AG60"/>
+  <dimension ref="A1:AG61"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
     <col min="1" max="1" width="13.1" customWidth="1"/>
@@ -1147,19 +1159,19 @@
         <v>12</v>
       </c>
       <c r="C2" s="2"/>
-      <c r="D2" s="4" t="s">
+      <c r="D2" s="4"/>
+      <c r="E2" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="E2" s="4" t="s">
+      <c r="F2" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="F2" s="4" t="s">
+      <c r="G2" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="G2" s="4" t="s">
+      <c r="H2" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="H2" s="4"/>
       <c r="I2" s="4"/>
       <c r="J2" s="4"/>
       <c r="K2" s="4"/>
@@ -1195,18 +1207,20 @@
       </c>
       <c r="C3" s="2"/>
       <c r="D3" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="E3" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="E3" s="4" t="s">
-        <v>14</v>
-      </c>
       <c r="F3" s="4" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="G3" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="H3" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="H3" s="4"/>
       <c r="I3" s="4"/>
       <c r="J3" s="4"/>
       <c r="K3" s="4"/>
@@ -1238,23 +1252,23 @@
     <row r="4" spans="1:33">
       <c r="A4" s="3"/>
       <c r="B4" s="4" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C4" s="2"/>
       <c r="D4" s="4" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="H4" s="4" t="s">
-        <v>23</v>
+        <v>16</v>
       </c>
       <c r="I4" s="4"/>
       <c r="J4" s="4"/>
@@ -1284,46 +1298,45 @@
       <c r="AF4" s="3"/>
       <c r="AG4" s="3"/>
     </row>
-    <row r="5" spans="2:33">
-      <c r="B5" s="2" t="s">
+    <row r="5" spans="1:33">
+      <c r="A5" s="3"/>
+      <c r="B5" s="4" t="s">
         <v>24</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="D5" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="E5" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="F5" s="2" t="s">
+      <c r="D5" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="G5" s="2" t="s">
-        <v>22</v>
+      <c r="E5" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F5" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="G5" s="4" t="s">
+        <v>26</v>
       </c>
       <c r="H5" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="I5" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="J5" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="K5" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="L5" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="M5" s="2"/>
-      <c r="N5" s="2"/>
-      <c r="O5" s="2"/>
-      <c r="P5" s="2"/>
-      <c r="Q5" s="2"/>
-      <c r="R5" s="2"/>
+      <c r="I5" s="4"/>
+      <c r="J5" s="4"/>
+      <c r="K5" s="4"/>
+      <c r="L5" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="M5" s="4"/>
+      <c r="N5" s="4"/>
+      <c r="O5" s="4"/>
+      <c r="P5" s="4"/>
+      <c r="Q5" s="4"/>
+      <c r="R5" s="4"/>
+      <c r="S5" s="3"/>
+      <c r="T5" s="3"/>
+      <c r="U5" s="3"/>
+      <c r="V5" s="3"/>
       <c r="W5" s="3"/>
       <c r="X5" s="3"/>
       <c r="Y5" s="3"/>
@@ -1336,29 +1349,46 @@
       <c r="AF5" s="3"/>
       <c r="AG5" s="3"/>
     </row>
-    <row r="6" spans="1:33">
-      <c r="A6" s="3"/>
-      <c r="B6" s="4"/>
-      <c r="C6" s="4"/>
-      <c r="D6" s="4"/>
-      <c r="E6" s="4"/>
-      <c r="F6" s="4"/>
-      <c r="G6" s="4"/>
-      <c r="H6" s="4"/>
-      <c r="I6" s="4"/>
-      <c r="J6" s="4"/>
-      <c r="K6" s="4"/>
-      <c r="L6" s="4"/>
-      <c r="M6" s="4"/>
-      <c r="N6" s="4"/>
-      <c r="O6" s="4"/>
-      <c r="P6" s="4"/>
-      <c r="Q6" s="4"/>
-      <c r="R6" s="4"/>
-      <c r="S6" s="3"/>
-      <c r="T6" s="3"/>
-      <c r="U6" s="3"/>
-      <c r="V6" s="3"/>
+    <row r="6" spans="2:33">
+      <c r="B6" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="G6" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="H6" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="I6" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="J6" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="K6" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="L6" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="M6" s="2"/>
+      <c r="N6" s="2"/>
+      <c r="O6" s="2"/>
+      <c r="P6" s="2"/>
+      <c r="Q6" s="2"/>
+      <c r="R6" s="2"/>
       <c r="W6" s="3"/>
       <c r="X6" s="3"/>
       <c r="Y6" s="3"/>
@@ -1371,7 +1401,7 @@
       <c r="AF6" s="3"/>
       <c r="AG6" s="3"/>
     </row>
-    <row r="7" s="1" customFormat="1" spans="1:33">
+    <row r="7" spans="1:33">
       <c r="A7" s="3"/>
       <c r="B7" s="4"/>
       <c r="C7" s="4"/>
@@ -1441,7 +1471,7 @@
       <c r="AF8" s="3"/>
       <c r="AG8" s="3"/>
     </row>
-    <row r="9" spans="1:33">
+    <row r="9" s="1" customFormat="1" spans="1:33">
       <c r="A9" s="3"/>
       <c r="B9" s="4"/>
       <c r="C9" s="4"/>
@@ -1971,7 +2001,7 @@
       <c r="B24" s="4"/>
       <c r="C24" s="4"/>
       <c r="D24" s="4"/>
-      <c r="E24" s="5"/>
+      <c r="E24" s="4"/>
       <c r="F24" s="4"/>
       <c r="G24" s="4"/>
       <c r="H24" s="4"/>
@@ -2076,7 +2106,7 @@
       <c r="B27" s="4"/>
       <c r="C27" s="4"/>
       <c r="D27" s="4"/>
-      <c r="E27" s="4"/>
+      <c r="E27" s="5"/>
       <c r="F27" s="4"/>
       <c r="G27" s="4"/>
       <c r="H27" s="4"/>
@@ -2216,7 +2246,7 @@
       <c r="B31" s="4"/>
       <c r="C31" s="4"/>
       <c r="D31" s="4"/>
-      <c r="E31" s="5"/>
+      <c r="E31" s="4"/>
       <c r="F31" s="4"/>
       <c r="G31" s="4"/>
       <c r="H31" s="4"/>
@@ -2251,7 +2281,7 @@
       <c r="B32" s="4"/>
       <c r="C32" s="4"/>
       <c r="D32" s="4"/>
-      <c r="E32" s="4"/>
+      <c r="E32" s="5"/>
       <c r="F32" s="4"/>
       <c r="G32" s="4"/>
       <c r="H32" s="4"/>
@@ -2526,25 +2556,47 @@
       <c r="AF39" s="3"/>
       <c r="AG39" s="3"/>
     </row>
-    <row r="47" spans="1:22">
-      <c r="A47" s="2"/>
-      <c r="B47" s="2"/>
-      <c r="C47" s="2"/>
-      <c r="D47" s="2"/>
-      <c r="Q47" s="2"/>
-      <c r="S47" s="2"/>
-      <c r="T47" s="2"/>
-      <c r="U47" s="2"/>
-      <c r="V47" s="2"/>
+    <row r="40" spans="1:33">
+      <c r="A40" s="3"/>
+      <c r="B40" s="4"/>
+      <c r="C40" s="4"/>
+      <c r="D40" s="4"/>
+      <c r="E40" s="4"/>
+      <c r="F40" s="4"/>
+      <c r="G40" s="4"/>
+      <c r="H40" s="4"/>
+      <c r="I40" s="4"/>
+      <c r="J40" s="4"/>
+      <c r="K40" s="4"/>
+      <c r="L40" s="4"/>
+      <c r="M40" s="4"/>
+      <c r="N40" s="4"/>
+      <c r="O40" s="4"/>
+      <c r="P40" s="4"/>
+      <c r="Q40" s="4"/>
+      <c r="R40" s="4"/>
+      <c r="S40" s="3"/>
+      <c r="T40" s="3"/>
+      <c r="U40" s="3"/>
+      <c r="V40" s="3"/>
+      <c r="W40" s="3"/>
+      <c r="X40" s="3"/>
+      <c r="Y40" s="3"/>
+      <c r="Z40" s="3"/>
+      <c r="AA40" s="3"/>
+      <c r="AB40" s="3"/>
+      <c r="AC40" s="3"/>
+      <c r="AD40" s="3"/>
+      <c r="AE40" s="3"/>
+      <c r="AF40" s="3"/>
+      <c r="AG40" s="3"/>
     </row>
     <row r="48" spans="1:22">
       <c r="A48" s="2"/>
       <c r="B48" s="2"/>
       <c r="C48" s="2"/>
       <c r="D48" s="2"/>
-      <c r="E48" s="2"/>
       <c r="Q48" s="2"/>
-      <c r="R48" s="2"/>
       <c r="S48" s="2"/>
       <c r="T48" s="2"/>
       <c r="U48" s="2"/>
@@ -2555,6 +2607,7 @@
       <c r="B49" s="2"/>
       <c r="C49" s="2"/>
       <c r="D49" s="2"/>
+      <c r="E49" s="2"/>
       <c r="Q49" s="2"/>
       <c r="R49" s="2"/>
       <c r="S49" s="2"/>
@@ -2694,33 +2747,45 @@
       <c r="U60" s="2"/>
       <c r="V60" s="2"/>
     </row>
+    <row r="61" spans="1:22">
+      <c r="A61" s="2"/>
+      <c r="B61" s="2"/>
+      <c r="C61" s="2"/>
+      <c r="D61" s="2"/>
+      <c r="Q61" s="2"/>
+      <c r="R61" s="2"/>
+      <c r="S61" s="2"/>
+      <c r="T61" s="2"/>
+      <c r="U61" s="2"/>
+      <c r="V61" s="2"/>
+    </row>
   </sheetData>
   <dataValidations count="9">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K4 K2:K3 K5:K1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K4 K5 K2:K3 K6:K1048576">
       <formula1>"MASK_XX,MASK_B,MASK_H,MASK_W,MASK_D"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L4 L2:L3 L5:L1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L4 L5 L2:L3 L6:L1048576">
       <formula1>"INST_VALID,INST_INVALID"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I4 I2:I3 I5:I1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I4 I5 I2:I3 I6:I1048576">
       <formula1>"LD_LB,LD_LH,LD_LW,LD_LBU,LD_LHU,LD_XX"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H4 J4 H2:H3 H5:H1048576 J2:J3 J5:J1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H4 J4 H5 J5 H2:H3 H6:H1048576 J2:J3 J6:J1048576">
       <formula1>"WB_ALU,WB_MEM,WB_PC,WB_XX"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G4 G2:G3 G5:G1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G4 G5 G2:G3 G6:G1048576">
       <formula1>"IMM_I,IMM_J,IMM_U,IMM_S,IMM_B"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F4 F2:F3 F5:F1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F4 F5 F2:F3 F6:F1048576">
       <formula1>"ALU_ADD,ALU_SUB,ALU_AND,ALU_OR,ALU_XOR,ALU_SLL,ALU_SRL,ALU_SLT,ALU_SLTU,ALU_COPY_A,ALU_COPY_B"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D4 D2:D3 D5:D1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D4 D5 D2:D3 D6:D1048576">
       <formula1>"A_PC,A_RS1"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E4 E2:E3 E5:E1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E4 E5 E2:E3 E6:E1048576">
       <formula1>"B_IMM,B_RS2"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C4 C2:C3 C5:C1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C4 C5 C2:C3 C6:C1048576">
       <formula1>"PC_4,PC_0,PC_ALU"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
> sim RTL ysyx_23060246 韩炳晋 Linux archlinux 6.6.60-1-lts #1 SMP PREEMPT_DYNAMIC Fri, 08 Nov 2024 16:03:02 +0000 x86_64 GNU/Linux  16:48:24 up 23:03,  2 users,  load average: 2.46, 2.41, 2.44
</commit_message>
<xml_diff>
--- a/npc/tools/control_gen/control_table.xlsx
+++ b/npc/tools/control_gen/control_table.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="41">
   <si>
     <t>commont</t>
   </si>
@@ -100,16 +100,37 @@
     <t>WB_PC</t>
   </si>
   <si>
+    <t>sw</t>
+  </si>
+  <si>
+    <t>IMM_S</t>
+  </si>
+  <si>
+    <t>ST_SW</t>
+  </si>
+  <si>
+    <t>MASK_W</t>
+  </si>
+  <si>
+    <t>lw</t>
+  </si>
+  <si>
+    <t>PC_4</t>
+  </si>
+  <si>
+    <t>LD_LW</t>
+  </si>
+  <si>
     <t>default</t>
   </si>
   <si>
-    <t>PC_4</t>
-  </si>
-  <si>
     <t>WB_XX</t>
   </si>
   <si>
     <t>LD_XX</t>
+  </si>
+  <si>
+    <t>ST_XX</t>
   </si>
   <si>
     <t>MASK_XX</t>
@@ -1084,7 +1105,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:AG61"/>
+  <dimension ref="A1:AG63"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
     <col min="1" max="1" width="13.1" customWidth="1"/>
@@ -1349,46 +1370,45 @@
       <c r="AF5" s="3"/>
       <c r="AG5" s="3"/>
     </row>
-    <row r="6" spans="2:33">
-      <c r="B6" s="2" t="s">
+    <row r="6" spans="1:33">
+      <c r="A6" s="3"/>
+      <c r="B6" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="C6" s="2" t="s">
+      <c r="C6" s="2"/>
+      <c r="D6" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F6" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="G6" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="D6" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="E6" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="F6" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="G6" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="H6" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="I6" s="4" t="s">
-        <v>31</v>
-      </c>
+      <c r="H6" s="4"/>
+      <c r="I6" s="4"/>
       <c r="J6" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="K6" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="L6" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="M6" s="2"/>
-      <c r="N6" s="2"/>
-      <c r="O6" s="2"/>
-      <c r="P6" s="2"/>
-      <c r="Q6" s="2"/>
-      <c r="R6" s="2"/>
+      <c r="K6" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="L6" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="M6" s="4"/>
+      <c r="N6" s="4"/>
+      <c r="O6" s="4"/>
+      <c r="P6" s="4"/>
+      <c r="Q6" s="4"/>
+      <c r="R6" s="4"/>
+      <c r="S6" s="3"/>
+      <c r="T6" s="3"/>
+      <c r="U6" s="3"/>
+      <c r="V6" s="3"/>
       <c r="W6" s="3"/>
       <c r="X6" s="3"/>
       <c r="Y6" s="3"/>
@@ -1403,17 +1423,33 @@
     </row>
     <row r="7" spans="1:33">
       <c r="A7" s="3"/>
-      <c r="B7" s="4"/>
-      <c r="C7" s="4"/>
-      <c r="D7" s="4"/>
-      <c r="E7" s="4"/>
-      <c r="F7" s="4"/>
-      <c r="G7" s="4"/>
+      <c r="B7" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="E7" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F7" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="G7" s="4" t="s">
+        <v>23</v>
+      </c>
       <c r="H7" s="4"/>
-      <c r="I7" s="4"/>
+      <c r="I7" s="4" t="s">
+        <v>34</v>
+      </c>
       <c r="J7" s="4"/>
       <c r="K7" s="4"/>
-      <c r="L7" s="4"/>
+      <c r="L7" s="4" t="s">
+        <v>17</v>
+      </c>
       <c r="M7" s="4"/>
       <c r="N7" s="4"/>
       <c r="O7" s="4"/>
@@ -1436,29 +1472,46 @@
       <c r="AF7" s="3"/>
       <c r="AG7" s="3"/>
     </row>
-    <row r="8" s="1" customFormat="1" spans="1:33">
-      <c r="A8" s="3"/>
-      <c r="B8" s="4"/>
-      <c r="C8" s="4"/>
-      <c r="D8" s="4"/>
-      <c r="E8" s="4"/>
-      <c r="F8" s="4"/>
-      <c r="G8" s="4"/>
-      <c r="H8" s="4"/>
-      <c r="I8" s="4"/>
-      <c r="J8" s="4"/>
-      <c r="K8" s="4"/>
-      <c r="L8" s="4"/>
-      <c r="M8" s="4"/>
-      <c r="N8" s="4"/>
-      <c r="O8" s="4"/>
-      <c r="P8" s="4"/>
-      <c r="Q8" s="4"/>
-      <c r="R8" s="4"/>
-      <c r="S8" s="3"/>
-      <c r="T8" s="3"/>
-      <c r="U8" s="3"/>
-      <c r="V8" s="3"/>
+    <row r="8" spans="2:33">
+      <c r="B8" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="G8" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="H8" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="I8" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="J8" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="K8" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="L8" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="M8" s="2"/>
+      <c r="N8" s="2"/>
+      <c r="O8" s="2"/>
+      <c r="P8" s="2"/>
+      <c r="Q8" s="2"/>
+      <c r="R8" s="2"/>
       <c r="W8" s="3"/>
       <c r="X8" s="3"/>
       <c r="Y8" s="3"/>
@@ -1471,7 +1524,7 @@
       <c r="AF8" s="3"/>
       <c r="AG8" s="3"/>
     </row>
-    <row r="9" s="1" customFormat="1" spans="1:33">
+    <row r="9" spans="1:33">
       <c r="A9" s="3"/>
       <c r="B9" s="4"/>
       <c r="C9" s="4"/>
@@ -1506,7 +1559,7 @@
       <c r="AF9" s="3"/>
       <c r="AG9" s="3"/>
     </row>
-    <row r="10" spans="1:33">
+    <row r="10" s="1" customFormat="1" spans="1:33">
       <c r="A10" s="3"/>
       <c r="B10" s="4"/>
       <c r="C10" s="4"/>
@@ -1541,7 +1594,7 @@
       <c r="AF10" s="3"/>
       <c r="AG10" s="3"/>
     </row>
-    <row r="11" spans="1:33">
+    <row r="11" s="1" customFormat="1" spans="1:33">
       <c r="A11" s="3"/>
       <c r="B11" s="4"/>
       <c r="C11" s="4"/>
@@ -2036,7 +2089,7 @@
       <c r="B25" s="4"/>
       <c r="C25" s="4"/>
       <c r="D25" s="4"/>
-      <c r="E25" s="5"/>
+      <c r="E25" s="4"/>
       <c r="F25" s="4"/>
       <c r="G25" s="4"/>
       <c r="H25" s="4"/>
@@ -2071,7 +2124,7 @@
       <c r="B26" s="4"/>
       <c r="C26" s="4"/>
       <c r="D26" s="4"/>
-      <c r="E26" s="5"/>
+      <c r="E26" s="4"/>
       <c r="F26" s="4"/>
       <c r="G26" s="4"/>
       <c r="H26" s="4"/>
@@ -2141,7 +2194,7 @@
       <c r="B28" s="4"/>
       <c r="C28" s="4"/>
       <c r="D28" s="4"/>
-      <c r="E28" s="4"/>
+      <c r="E28" s="5"/>
       <c r="F28" s="4"/>
       <c r="G28" s="4"/>
       <c r="H28" s="4"/>
@@ -2176,7 +2229,7 @@
       <c r="B29" s="4"/>
       <c r="C29" s="4"/>
       <c r="D29" s="4"/>
-      <c r="E29" s="4"/>
+      <c r="E29" s="5"/>
       <c r="F29" s="4"/>
       <c r="G29" s="4"/>
       <c r="H29" s="4"/>
@@ -2281,7 +2334,7 @@
       <c r="B32" s="4"/>
       <c r="C32" s="4"/>
       <c r="D32" s="4"/>
-      <c r="E32" s="5"/>
+      <c r="E32" s="4"/>
       <c r="F32" s="4"/>
       <c r="G32" s="4"/>
       <c r="H32" s="4"/>
@@ -2351,7 +2404,7 @@
       <c r="B34" s="4"/>
       <c r="C34" s="4"/>
       <c r="D34" s="4"/>
-      <c r="E34" s="4"/>
+      <c r="E34" s="5"/>
       <c r="F34" s="4"/>
       <c r="G34" s="4"/>
       <c r="H34" s="4"/>
@@ -2591,29 +2644,75 @@
       <c r="AF40" s="3"/>
       <c r="AG40" s="3"/>
     </row>
-    <row r="48" spans="1:22">
-      <c r="A48" s="2"/>
-      <c r="B48" s="2"/>
-      <c r="C48" s="2"/>
-      <c r="D48" s="2"/>
-      <c r="Q48" s="2"/>
-      <c r="S48" s="2"/>
-      <c r="T48" s="2"/>
-      <c r="U48" s="2"/>
-      <c r="V48" s="2"/>
-    </row>
-    <row r="49" spans="1:22">
-      <c r="A49" s="2"/>
-      <c r="B49" s="2"/>
-      <c r="C49" s="2"/>
-      <c r="D49" s="2"/>
-      <c r="E49" s="2"/>
-      <c r="Q49" s="2"/>
-      <c r="R49" s="2"/>
-      <c r="S49" s="2"/>
-      <c r="T49" s="2"/>
-      <c r="U49" s="2"/>
-      <c r="V49" s="2"/>
+    <row r="41" spans="1:33">
+      <c r="A41" s="3"/>
+      <c r="B41" s="4"/>
+      <c r="C41" s="4"/>
+      <c r="D41" s="4"/>
+      <c r="E41" s="4"/>
+      <c r="F41" s="4"/>
+      <c r="G41" s="4"/>
+      <c r="H41" s="4"/>
+      <c r="I41" s="4"/>
+      <c r="J41" s="4"/>
+      <c r="K41" s="4"/>
+      <c r="L41" s="4"/>
+      <c r="M41" s="4"/>
+      <c r="N41" s="4"/>
+      <c r="O41" s="4"/>
+      <c r="P41" s="4"/>
+      <c r="Q41" s="4"/>
+      <c r="R41" s="4"/>
+      <c r="S41" s="3"/>
+      <c r="T41" s="3"/>
+      <c r="U41" s="3"/>
+      <c r="V41" s="3"/>
+      <c r="W41" s="3"/>
+      <c r="X41" s="3"/>
+      <c r="Y41" s="3"/>
+      <c r="Z41" s="3"/>
+      <c r="AA41" s="3"/>
+      <c r="AB41" s="3"/>
+      <c r="AC41" s="3"/>
+      <c r="AD41" s="3"/>
+      <c r="AE41" s="3"/>
+      <c r="AF41" s="3"/>
+      <c r="AG41" s="3"/>
+    </row>
+    <row r="42" spans="1:33">
+      <c r="A42" s="3"/>
+      <c r="B42" s="4"/>
+      <c r="C42" s="4"/>
+      <c r="D42" s="4"/>
+      <c r="E42" s="4"/>
+      <c r="F42" s="4"/>
+      <c r="G42" s="4"/>
+      <c r="H42" s="4"/>
+      <c r="I42" s="4"/>
+      <c r="J42" s="4"/>
+      <c r="K42" s="4"/>
+      <c r="L42" s="4"/>
+      <c r="M42" s="4"/>
+      <c r="N42" s="4"/>
+      <c r="O42" s="4"/>
+      <c r="P42" s="4"/>
+      <c r="Q42" s="4"/>
+      <c r="R42" s="4"/>
+      <c r="S42" s="3"/>
+      <c r="T42" s="3"/>
+      <c r="U42" s="3"/>
+      <c r="V42" s="3"/>
+      <c r="W42" s="3"/>
+      <c r="X42" s="3"/>
+      <c r="Y42" s="3"/>
+      <c r="Z42" s="3"/>
+      <c r="AA42" s="3"/>
+      <c r="AB42" s="3"/>
+      <c r="AC42" s="3"/>
+      <c r="AD42" s="3"/>
+      <c r="AE42" s="3"/>
+      <c r="AF42" s="3"/>
+      <c r="AG42" s="3"/>
     </row>
     <row r="50" spans="1:22">
       <c r="A50" s="2"/>
@@ -2621,7 +2720,6 @@
       <c r="C50" s="2"/>
       <c r="D50" s="2"/>
       <c r="Q50" s="2"/>
-      <c r="R50" s="2"/>
       <c r="S50" s="2"/>
       <c r="T50" s="2"/>
       <c r="U50" s="2"/>
@@ -2632,6 +2730,7 @@
       <c r="B51" s="2"/>
       <c r="C51" s="2"/>
       <c r="D51" s="2"/>
+      <c r="E51" s="2"/>
       <c r="Q51" s="2"/>
       <c r="R51" s="2"/>
       <c r="S51" s="2"/>
@@ -2759,33 +2858,60 @@
       <c r="U61" s="2"/>
       <c r="V61" s="2"/>
     </row>
+    <row r="62" spans="1:22">
+      <c r="A62" s="2"/>
+      <c r="B62" s="2"/>
+      <c r="C62" s="2"/>
+      <c r="D62" s="2"/>
+      <c r="Q62" s="2"/>
+      <c r="R62" s="2"/>
+      <c r="S62" s="2"/>
+      <c r="T62" s="2"/>
+      <c r="U62" s="2"/>
+      <c r="V62" s="2"/>
+    </row>
+    <row r="63" spans="1:22">
+      <c r="A63" s="2"/>
+      <c r="B63" s="2"/>
+      <c r="C63" s="2"/>
+      <c r="D63" s="2"/>
+      <c r="Q63" s="2"/>
+      <c r="R63" s="2"/>
+      <c r="S63" s="2"/>
+      <c r="T63" s="2"/>
+      <c r="U63" s="2"/>
+      <c r="V63" s="2"/>
+    </row>
   </sheetData>
-  <dataValidations count="9">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K4 K5 K2:K3 K6:K1048576">
+  <dataValidations count="10">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J7 J2:J6 J8:J1048576">
+      <formula1>"ST_SW,ST_SH,ST_SB,ST_XX"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K4 K5 K6 K7 K2:K3 K8:K1048576">
       <formula1>"MASK_XX,MASK_B,MASK_H,MASK_W,MASK_D"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L4 L5 L2:L3 L6:L1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L4 L5 L6 L7 L2:L3 L8:L1048576">
       <formula1>"INST_VALID,INST_INVALID"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I4 I5 I2:I3 I6:I1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I4 I5 I6 I7 I2:I3 I8:I1048576">
       <formula1>"LD_LB,LD_LH,LD_LW,LD_LBU,LD_LHU,LD_XX"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H4 J4 H5 J5 H2:H3 H6:H1048576 J2:J3 J6:J1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H4 H5 H6 H7 H2:H3 H8:H1048576">
       <formula1>"WB_ALU,WB_MEM,WB_PC,WB_XX"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G4 G5 G2:G3 G6:G1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G4 G5 G6 G7 G2:G3 G8:G1048576">
       <formula1>"IMM_I,IMM_J,IMM_U,IMM_S,IMM_B"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F4 F5 F2:F3 F6:F1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F4 F5 F6 F7 F2:F3 F8:F1048576">
       <formula1>"ALU_ADD,ALU_SUB,ALU_AND,ALU_OR,ALU_XOR,ALU_SLL,ALU_SRL,ALU_SLT,ALU_SLTU,ALU_COPY_A,ALU_COPY_B"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D4 D5 D2:D3 D6:D1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D4 D5 D6 D7 D2:D3 D8:D1048576">
       <formula1>"A_PC,A_RS1"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E4 E5 E2:E3 E6:E1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E4 E5 E6 E7 E2:E3 E8:E1048576">
       <formula1>"B_IMM,B_RS2"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C4 C5 C2:C3 C6:C1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C4 C5 C6 C7 C2:C3 C8:C1048576">
       <formula1>"PC_4,PC_0,PC_ALU"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
> sim RTL ysyx_23060246 韩炳晋 Linux archlinux 6.6.60-1-lts #1 SMP PREEMPT_DYNAMIC Fri, 08 Nov 2024 16:03:02 +0000 x86_64 GNU/Linux  17:07:00 up 23:22,  2 users,  load average: 3.22, 3.50, 3.50
</commit_message>
<xml_diff>
--- a/npc/tools/control_gen/control_table.xlsx
+++ b/npc/tools/control_gen/control_table.xlsx
@@ -97,7 +97,7 @@
     <t>IMM_J</t>
   </si>
   <si>
-    <t>WB_PC</t>
+    <t>WB_PC4</t>
   </si>
   <si>
     <t>sw</t>
@@ -2896,14 +2896,14 @@
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I4 I5 I6 I7 I2:I3 I8:I1048576">
       <formula1>"LD_LB,LD_LH,LD_LW,LD_LBU,LD_LHU,LD_XX"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H4 H5 H6 H7 H2:H3 H8:H1048576">
-      <formula1>"WB_ALU,WB_MEM,WB_PC,WB_XX"</formula1>
-    </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G4 G5 G6 G7 G2:G3 G8:G1048576">
       <formula1>"IMM_I,IMM_J,IMM_U,IMM_S,IMM_B"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F4 F5 F6 F7 F2:F3 F8:F1048576">
       <formula1>"ALU_ADD,ALU_SUB,ALU_AND,ALU_OR,ALU_XOR,ALU_SLL,ALU_SRL,ALU_SLT,ALU_SLTU,ALU_COPY_A,ALU_COPY_B"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H2:H1048576">
+      <formula1>"WB_ALU,WB_MEM,WB_PC4,WB_XX"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D4 D5 D6 D7 D2:D3 D8:D1048576">
       <formula1>"A_PC,A_RS1"</formula1>

</xml_diff>

<commit_message>
> sim RTL ysyx_23060246 韩炳晋 Linux archlinux 6.6.60-1-lts #1 SMP PREEMPT_DYNAMIC Fri, 08 Nov 2024 16:03:02 +0000 x86_64 GNU/Linux  17:38:33 up 23:53,  2 users,  load average: 4.06, 3.63, 3.48
</commit_message>
<xml_diff>
--- a/npc/tools/control_gen/control_table.xlsx
+++ b/npc/tools/control_gen/control_table.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="42">
   <si>
     <t>commont</t>
   </si>
@@ -88,16 +88,19 @@
     <t>IMM_I</t>
   </si>
   <si>
+    <t>jalr</t>
+  </si>
+  <si>
+    <t>PC_ALU</t>
+  </si>
+  <si>
+    <t>WB_PC4</t>
+  </si>
+  <si>
     <t>jal</t>
   </si>
   <si>
-    <t>PC_ALU</t>
-  </si>
-  <si>
     <t>IMM_J</t>
-  </si>
-  <si>
-    <t>WB_PC4</t>
   </si>
   <si>
     <t>sw</t>
@@ -1105,7 +1108,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:AG63"/>
+  <dimension ref="A1:AG64"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
     <col min="1" max="1" width="13.1" customWidth="1"/>
@@ -1328,7 +1331,7 @@
         <v>25</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="E5" s="4" t="s">
         <v>13</v>
@@ -1336,18 +1339,14 @@
       <c r="F5" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="G5" s="4" t="s">
+      <c r="G5" s="4"/>
+      <c r="H5" s="4" t="s">
         <v>26</v>
-      </c>
-      <c r="H5" s="4" t="s">
-        <v>27</v>
       </c>
       <c r="I5" s="4"/>
       <c r="J5" s="4"/>
       <c r="K5" s="4"/>
-      <c r="L5" s="4" t="s">
-        <v>17</v>
-      </c>
+      <c r="L5" s="4"/>
       <c r="M5" s="4"/>
       <c r="N5" s="4"/>
       <c r="O5" s="4"/>
@@ -1373,11 +1372,13 @@
     <row r="6" spans="1:33">
       <c r="A6" s="3"/>
       <c r="B6" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="C6" s="2"/>
+        <v>27</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>25</v>
+      </c>
       <c r="D6" s="4" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="E6" s="4" t="s">
         <v>13</v>
@@ -1386,16 +1387,14 @@
         <v>20</v>
       </c>
       <c r="G6" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="H6" s="4"/>
+        <v>28</v>
+      </c>
+      <c r="H6" s="4" t="s">
+        <v>26</v>
+      </c>
       <c r="I6" s="4"/>
-      <c r="J6" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="K6" s="4" t="s">
-        <v>31</v>
-      </c>
+      <c r="J6" s="4"/>
+      <c r="K6" s="4"/>
       <c r="L6" s="4" t="s">
         <v>17</v>
       </c>
@@ -1424,11 +1423,9 @@
     <row r="7" spans="1:33">
       <c r="A7" s="3"/>
       <c r="B7" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>33</v>
-      </c>
+        <v>29</v>
+      </c>
+      <c r="C7" s="2"/>
       <c r="D7" s="4" t="s">
         <v>22</v>
       </c>
@@ -1439,14 +1436,16 @@
         <v>20</v>
       </c>
       <c r="G7" s="4" t="s">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="H7" s="4"/>
-      <c r="I7" s="4" t="s">
-        <v>34</v>
-      </c>
-      <c r="J7" s="4"/>
-      <c r="K7" s="4"/>
+      <c r="I7" s="4"/>
+      <c r="J7" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="K7" s="4" t="s">
+        <v>32</v>
+      </c>
       <c r="L7" s="4" t="s">
         <v>17</v>
       </c>
@@ -1472,46 +1471,45 @@
       <c r="AF7" s="3"/>
       <c r="AG7" s="3"/>
     </row>
-    <row r="8" spans="2:33">
-      <c r="B8" s="2" t="s">
+    <row r="8" spans="1:33">
+      <c r="A8" s="3"/>
+      <c r="B8" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="E8" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F8" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="G8" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="H8" s="4"/>
+      <c r="I8" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="C8" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="D8" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="E8" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="F8" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="G8" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="H8" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="I8" s="4" t="s">
-        <v>37</v>
-      </c>
-      <c r="J8" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="K8" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="L8" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="M8" s="2"/>
-      <c r="N8" s="2"/>
-      <c r="O8" s="2"/>
-      <c r="P8" s="2"/>
-      <c r="Q8" s="2"/>
-      <c r="R8" s="2"/>
+      <c r="J8" s="4"/>
+      <c r="K8" s="4"/>
+      <c r="L8" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="M8" s="4"/>
+      <c r="N8" s="4"/>
+      <c r="O8" s="4"/>
+      <c r="P8" s="4"/>
+      <c r="Q8" s="4"/>
+      <c r="R8" s="4"/>
+      <c r="S8" s="3"/>
+      <c r="T8" s="3"/>
+      <c r="U8" s="3"/>
+      <c r="V8" s="3"/>
       <c r="W8" s="3"/>
       <c r="X8" s="3"/>
       <c r="Y8" s="3"/>
@@ -1524,29 +1522,46 @@
       <c r="AF8" s="3"/>
       <c r="AG8" s="3"/>
     </row>
-    <row r="9" spans="1:33">
-      <c r="A9" s="3"/>
-      <c r="B9" s="4"/>
-      <c r="C9" s="4"/>
-      <c r="D9" s="4"/>
-      <c r="E9" s="4"/>
-      <c r="F9" s="4"/>
-      <c r="G9" s="4"/>
-      <c r="H9" s="4"/>
-      <c r="I9" s="4"/>
-      <c r="J9" s="4"/>
-      <c r="K9" s="4"/>
-      <c r="L9" s="4"/>
-      <c r="M9" s="4"/>
-      <c r="N9" s="4"/>
-      <c r="O9" s="4"/>
-      <c r="P9" s="4"/>
-      <c r="Q9" s="4"/>
-      <c r="R9" s="4"/>
-      <c r="S9" s="3"/>
-      <c r="T9" s="3"/>
-      <c r="U9" s="3"/>
-      <c r="V9" s="3"/>
+    <row r="9" spans="2:33">
+      <c r="B9" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="F9" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="G9" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="H9" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="I9" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="J9" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="K9" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="L9" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="M9" s="2"/>
+      <c r="N9" s="2"/>
+      <c r="O9" s="2"/>
+      <c r="P9" s="2"/>
+      <c r="Q9" s="2"/>
+      <c r="R9" s="2"/>
       <c r="W9" s="3"/>
       <c r="X9" s="3"/>
       <c r="Y9" s="3"/>
@@ -1559,7 +1574,7 @@
       <c r="AF9" s="3"/>
       <c r="AG9" s="3"/>
     </row>
-    <row r="10" s="1" customFormat="1" spans="1:33">
+    <row r="10" spans="1:33">
       <c r="A10" s="3"/>
       <c r="B10" s="4"/>
       <c r="C10" s="4"/>
@@ -1629,7 +1644,7 @@
       <c r="AF11" s="3"/>
       <c r="AG11" s="3"/>
     </row>
-    <row r="12" spans="1:33">
+    <row r="12" s="1" customFormat="1" spans="1:33">
       <c r="A12" s="3"/>
       <c r="B12" s="4"/>
       <c r="C12" s="4"/>
@@ -2159,7 +2174,7 @@
       <c r="B27" s="4"/>
       <c r="C27" s="4"/>
       <c r="D27" s="4"/>
-      <c r="E27" s="5"/>
+      <c r="E27" s="4"/>
       <c r="F27" s="4"/>
       <c r="G27" s="4"/>
       <c r="H27" s="4"/>
@@ -2264,7 +2279,7 @@
       <c r="B30" s="4"/>
       <c r="C30" s="4"/>
       <c r="D30" s="4"/>
-      <c r="E30" s="4"/>
+      <c r="E30" s="5"/>
       <c r="F30" s="4"/>
       <c r="G30" s="4"/>
       <c r="H30" s="4"/>
@@ -2404,7 +2419,7 @@
       <c r="B34" s="4"/>
       <c r="C34" s="4"/>
       <c r="D34" s="4"/>
-      <c r="E34" s="5"/>
+      <c r="E34" s="4"/>
       <c r="F34" s="4"/>
       <c r="G34" s="4"/>
       <c r="H34" s="4"/>
@@ -2439,7 +2454,7 @@
       <c r="B35" s="4"/>
       <c r="C35" s="4"/>
       <c r="D35" s="4"/>
-      <c r="E35" s="4"/>
+      <c r="E35" s="5"/>
       <c r="F35" s="4"/>
       <c r="G35" s="4"/>
       <c r="H35" s="4"/>
@@ -2714,25 +2729,47 @@
       <c r="AF42" s="3"/>
       <c r="AG42" s="3"/>
     </row>
-    <row r="50" spans="1:22">
-      <c r="A50" s="2"/>
-      <c r="B50" s="2"/>
-      <c r="C50" s="2"/>
-      <c r="D50" s="2"/>
-      <c r="Q50" s="2"/>
-      <c r="S50" s="2"/>
-      <c r="T50" s="2"/>
-      <c r="U50" s="2"/>
-      <c r="V50" s="2"/>
+    <row r="43" spans="1:33">
+      <c r="A43" s="3"/>
+      <c r="B43" s="4"/>
+      <c r="C43" s="4"/>
+      <c r="D43" s="4"/>
+      <c r="E43" s="4"/>
+      <c r="F43" s="4"/>
+      <c r="G43" s="4"/>
+      <c r="H43" s="4"/>
+      <c r="I43" s="4"/>
+      <c r="J43" s="4"/>
+      <c r="K43" s="4"/>
+      <c r="L43" s="4"/>
+      <c r="M43" s="4"/>
+      <c r="N43" s="4"/>
+      <c r="O43" s="4"/>
+      <c r="P43" s="4"/>
+      <c r="Q43" s="4"/>
+      <c r="R43" s="4"/>
+      <c r="S43" s="3"/>
+      <c r="T43" s="3"/>
+      <c r="U43" s="3"/>
+      <c r="V43" s="3"/>
+      <c r="W43" s="3"/>
+      <c r="X43" s="3"/>
+      <c r="Y43" s="3"/>
+      <c r="Z43" s="3"/>
+      <c r="AA43" s="3"/>
+      <c r="AB43" s="3"/>
+      <c r="AC43" s="3"/>
+      <c r="AD43" s="3"/>
+      <c r="AE43" s="3"/>
+      <c r="AF43" s="3"/>
+      <c r="AG43" s="3"/>
     </row>
     <row r="51" spans="1:22">
       <c r="A51" s="2"/>
       <c r="B51" s="2"/>
       <c r="C51" s="2"/>
       <c r="D51" s="2"/>
-      <c r="E51" s="2"/>
       <c r="Q51" s="2"/>
-      <c r="R51" s="2"/>
       <c r="S51" s="2"/>
       <c r="T51" s="2"/>
       <c r="U51" s="2"/>
@@ -2743,6 +2780,7 @@
       <c r="B52" s="2"/>
       <c r="C52" s="2"/>
       <c r="D52" s="2"/>
+      <c r="E52" s="2"/>
       <c r="Q52" s="2"/>
       <c r="R52" s="2"/>
       <c r="S52" s="2"/>
@@ -2882,36 +2920,48 @@
       <c r="U63" s="2"/>
       <c r="V63" s="2"/>
     </row>
+    <row r="64" spans="1:22">
+      <c r="A64" s="2"/>
+      <c r="B64" s="2"/>
+      <c r="C64" s="2"/>
+      <c r="D64" s="2"/>
+      <c r="Q64" s="2"/>
+      <c r="R64" s="2"/>
+      <c r="S64" s="2"/>
+      <c r="T64" s="2"/>
+      <c r="U64" s="2"/>
+      <c r="V64" s="2"/>
+    </row>
   </sheetData>
   <dataValidations count="10">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J7 J2:J6 J8:J1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J5 J8 J2:J4 J6:J7 J9:J1048576">
       <formula1>"ST_SW,ST_SH,ST_SB,ST_XX"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K4 K5 K6 K7 K2:K3 K8:K1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K4 K5 K6 K7 K8 K2:K3 K9:K1048576">
       <formula1>"MASK_XX,MASK_B,MASK_H,MASK_W,MASK_D"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L4 L5 L6 L7 L2:L3 L8:L1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L4 L5 L6 L7 L8 L2:L3 L9:L1048576">
       <formula1>"INST_VALID,INST_INVALID"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I4 I5 I6 I7 I2:I3 I8:I1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I4 I5 I6 I7 I8 I2:I3 I9:I1048576">
       <formula1>"LD_LB,LD_LH,LD_LW,LD_LBU,LD_LHU,LD_XX"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G4 G5 G6 G7 G2:G3 G8:G1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G4 G5 G6 G7 G8 G2:G3 G9:G1048576">
       <formula1>"IMM_I,IMM_J,IMM_U,IMM_S,IMM_B"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F4 F5 F6 F7 F2:F3 F8:F1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F4 F5 F6 F7 F8 F2:F3 F9:F1048576">
       <formula1>"ALU_ADD,ALU_SUB,ALU_AND,ALU_OR,ALU_XOR,ALU_SLL,ALU_SRL,ALU_SLT,ALU_SLTU,ALU_COPY_A,ALU_COPY_B"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H2:H1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H5 H2:H4 H6:H1048576">
       <formula1>"WB_ALU,WB_MEM,WB_PC4,WB_XX"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D4 D5 D6 D7 D2:D3 D8:D1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D4 D5 D6 D7 D8 D2:D3 D9:D1048576">
       <formula1>"A_PC,A_RS1"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E4 E5 E6 E7 E2:E3 E8:E1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E4 E5 E6 E7 E8 E2:E3 E9:E1048576">
       <formula1>"B_IMM,B_RS2"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C4 C5 C6 C7 C2:C3 C8:C1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C4 C5 C6 C7 C8 C2:C3 C9:C1048576">
       <formula1>"PC_4,PC_0,PC_ALU"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
> sim RTL ysyx_23060246 韩炳晋 Linux archlinux 6.6.60-1-lts #1 SMP PREEMPT_DYNAMIC Fri, 08 Nov 2024 16:03:02 +0000 x86_64 GNU/Linux  17:39:30 up 23:54,  2 users,  load average: 5.19, 3.96, 3.60
</commit_message>
<xml_diff>
--- a/npc/tools/control_gen/control_table.xlsx
+++ b/npc/tools/control_gen/control_table.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="42">
   <si>
     <t>commont</t>
   </si>
@@ -1346,7 +1346,9 @@
       <c r="I5" s="4"/>
       <c r="J5" s="4"/>
       <c r="K5" s="4"/>
-      <c r="L5" s="4"/>
+      <c r="L5" s="4" t="s">
+        <v>17</v>
+      </c>
       <c r="M5" s="4"/>
       <c r="N5" s="4"/>
       <c r="O5" s="4"/>

</xml_diff>

<commit_message>
> sim RTL ysyx_23060246 韩炳晋 Linux archlinux 6.6.60-1-lts #1 SMP PREEMPT_DYNAMIC Fri, 08 Nov 2024 16:03:02 +0000 x86_64 GNU/Linux  18:25:35 up 1 day, 40 min,  2 users,  load average: 3.85, 3.54, 3.38
</commit_message>
<xml_diff>
--- a/npc/tools/control_gen/control_table.xlsx
+++ b/npc/tools/control_gen/control_table.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="46">
   <si>
     <t>commont</t>
   </si>
@@ -49,6 +49,9 @@
     <t>mask_sel</t>
   </si>
   <si>
+    <t>br_sel</t>
+  </si>
+  <si>
     <t>inst_valid</t>
   </si>
   <si>
@@ -124,6 +127,12 @@
     <t>LD_LW</t>
   </si>
   <si>
+    <t>bgeu</t>
+  </si>
+  <si>
+    <t>BR_GEU</t>
+  </si>
+  <si>
     <t>default</t>
   </si>
   <si>
@@ -137,6 +146,9 @@
   </si>
   <si>
     <t>MASK_XX</t>
+  </si>
+  <si>
+    <t>BR_XX</t>
   </si>
   <si>
     <t>INST_INVALID</t>
@@ -1108,7 +1120,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:AG64"/>
+  <dimension ref="A1:AH65"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
     <col min="1" max="1" width="13.1" customWidth="1"/>
@@ -1120,19 +1132,19 @@
     <col min="7" max="7" width="10.9416666666667" customWidth="1"/>
     <col min="8" max="10" width="11.9833333333333" customWidth="1"/>
     <col min="11" max="11" width="15.075" customWidth="1"/>
-    <col min="12" max="12" width="12.1083333333333" customWidth="1"/>
-    <col min="13" max="13" width="10.8583333333333" customWidth="1"/>
-    <col min="15" max="15" width="14.2166666666667" customWidth="1"/>
-    <col min="16" max="16" width="11.8083333333333" customWidth="1"/>
-    <col min="17" max="17" width="10.6" customWidth="1"/>
-    <col min="18" max="18" width="9.70833333333333" customWidth="1"/>
-    <col min="19" max="19" width="11.1666666666667" customWidth="1"/>
-    <col min="20" max="20" width="11.4083333333333" customWidth="1"/>
-    <col min="21" max="21" width="12.0583333333333" customWidth="1"/>
-    <col min="22" max="22" width="15.575" customWidth="1"/>
+    <col min="12" max="13" width="12.1083333333333" customWidth="1"/>
+    <col min="14" max="14" width="10.8583333333333" customWidth="1"/>
+    <col min="16" max="16" width="14.2166666666667" customWidth="1"/>
+    <col min="17" max="17" width="11.8083333333333" customWidth="1"/>
+    <col min="18" max="18" width="10.6" customWidth="1"/>
+    <col min="19" max="19" width="9.70833333333333" customWidth="1"/>
+    <col min="20" max="20" width="11.1666666666667" customWidth="1"/>
+    <col min="21" max="21" width="11.4083333333333" customWidth="1"/>
+    <col min="22" max="22" width="12.0583333333333" customWidth="1"/>
+    <col min="23" max="23" width="15.575" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="15" customHeight="1" spans="1:21">
+    <row r="1" ht="15" customHeight="1" spans="1:22">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1169,46 +1181,49 @@
       <c r="L1" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="2"/>
+      <c r="M1" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="N1" s="2"/>
       <c r="O1" s="2"/>
       <c r="P1" s="2"/>
       <c r="Q1" s="2"/>
       <c r="R1" s="2"/>
-      <c r="U1" s="6"/>
-    </row>
-    <row r="2" spans="1:33">
+      <c r="S1" s="2"/>
+      <c r="V1" s="6"/>
+    </row>
+    <row r="2" spans="1:34">
       <c r="A2" s="3"/>
       <c r="B2" s="4" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="4"/>
       <c r="E2" s="4" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F2" s="4" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G2" s="4" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="H2" s="4" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="I2" s="4"/>
       <c r="J2" s="4"/>
       <c r="K2" s="4"/>
-      <c r="L2" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="M2" s="4"/>
+      <c r="L2" s="4"/>
+      <c r="M2" s="4" t="s">
+        <v>18</v>
+      </c>
       <c r="N2" s="4"/>
       <c r="O2" s="4"/>
       <c r="P2" s="4"/>
       <c r="Q2" s="4"/>
       <c r="R2" s="4"/>
-      <c r="S2" s="3"/>
+      <c r="S2" s="4"/>
       <c r="T2" s="3"/>
       <c r="U2" s="3"/>
       <c r="V2" s="3"/>
@@ -1223,41 +1238,42 @@
       <c r="AE2" s="3"/>
       <c r="AF2" s="3"/>
       <c r="AG2" s="3"/>
-    </row>
-    <row r="3" spans="1:33">
+      <c r="AH2" s="3"/>
+    </row>
+    <row r="3" spans="1:34">
       <c r="A3" s="3"/>
       <c r="B3" s="4" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C3" s="2"/>
       <c r="D3" s="4" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="G3" s="4" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="H3" s="4" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="I3" s="4"/>
       <c r="J3" s="4"/>
       <c r="K3" s="4"/>
-      <c r="L3" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="M3" s="4"/>
+      <c r="L3" s="4"/>
+      <c r="M3" s="4" t="s">
+        <v>18</v>
+      </c>
       <c r="N3" s="4"/>
       <c r="O3" s="4"/>
       <c r="P3" s="4"/>
       <c r="Q3" s="4"/>
       <c r="R3" s="4"/>
-      <c r="S3" s="3"/>
+      <c r="S3" s="4"/>
       <c r="T3" s="3"/>
       <c r="U3" s="3"/>
       <c r="V3" s="3"/>
@@ -1272,41 +1288,42 @@
       <c r="AE3" s="3"/>
       <c r="AF3" s="3"/>
       <c r="AG3" s="3"/>
-    </row>
-    <row r="4" spans="1:33">
+      <c r="AH3" s="3"/>
+    </row>
+    <row r="4" spans="1:34">
       <c r="A4" s="3"/>
       <c r="B4" s="4" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C4" s="2"/>
       <c r="D4" s="4" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="H4" s="4" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="I4" s="4"/>
       <c r="J4" s="4"/>
       <c r="K4" s="4"/>
-      <c r="L4" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="M4" s="4"/>
+      <c r="L4" s="4"/>
+      <c r="M4" s="4" t="s">
+        <v>18</v>
+      </c>
       <c r="N4" s="4"/>
       <c r="O4" s="4"/>
       <c r="P4" s="4"/>
       <c r="Q4" s="4"/>
       <c r="R4" s="4"/>
-      <c r="S4" s="3"/>
+      <c r="S4" s="4"/>
       <c r="T4" s="3"/>
       <c r="U4" s="3"/>
       <c r="V4" s="3"/>
@@ -1321,41 +1338,42 @@
       <c r="AE4" s="3"/>
       <c r="AF4" s="3"/>
       <c r="AG4" s="3"/>
-    </row>
-    <row r="5" spans="1:33">
+      <c r="AH4" s="3"/>
+    </row>
+    <row r="5" spans="1:34">
       <c r="A5" s="3"/>
       <c r="B5" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="G5" s="4"/>
       <c r="H5" s="4" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="I5" s="4"/>
       <c r="J5" s="4"/>
       <c r="K5" s="4"/>
-      <c r="L5" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="M5" s="4"/>
+      <c r="L5" s="4"/>
+      <c r="M5" s="4" t="s">
+        <v>18</v>
+      </c>
       <c r="N5" s="4"/>
       <c r="O5" s="4"/>
       <c r="P5" s="4"/>
       <c r="Q5" s="4"/>
       <c r="R5" s="4"/>
-      <c r="S5" s="3"/>
+      <c r="S5" s="4"/>
       <c r="T5" s="3"/>
       <c r="U5" s="3"/>
       <c r="V5" s="3"/>
@@ -1370,43 +1388,44 @@
       <c r="AE5" s="3"/>
       <c r="AF5" s="3"/>
       <c r="AG5" s="3"/>
-    </row>
-    <row r="6" spans="1:33">
+      <c r="AH5" s="3"/>
+    </row>
+    <row r="6" spans="1:34">
       <c r="A6" s="3"/>
       <c r="B6" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="F6" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="G6" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="H6" s="4" t="s">
         <v>27</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="D6" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="E6" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="F6" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="G6" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="H6" s="4" t="s">
-        <v>26</v>
       </c>
       <c r="I6" s="4"/>
       <c r="J6" s="4"/>
       <c r="K6" s="4"/>
-      <c r="L6" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="M6" s="4"/>
+      <c r="L6" s="4"/>
+      <c r="M6" s="4" t="s">
+        <v>18</v>
+      </c>
       <c r="N6" s="4"/>
       <c r="O6" s="4"/>
       <c r="P6" s="4"/>
       <c r="Q6" s="4"/>
       <c r="R6" s="4"/>
-      <c r="S6" s="3"/>
+      <c r="S6" s="4"/>
       <c r="T6" s="3"/>
       <c r="U6" s="3"/>
       <c r="V6" s="3"/>
@@ -1421,43 +1440,44 @@
       <c r="AE6" s="3"/>
       <c r="AF6" s="3"/>
       <c r="AG6" s="3"/>
-    </row>
-    <row r="7" spans="1:33">
+      <c r="AH6" s="3"/>
+    </row>
+    <row r="7" spans="1:34">
       <c r="A7" s="3"/>
       <c r="B7" s="4" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C7" s="2"/>
       <c r="D7" s="4" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="G7" s="4" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="H7" s="4"/>
       <c r="I7" s="4"/>
       <c r="J7" s="4" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="K7" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="L7" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="M7" s="4"/>
+        <v>33</v>
+      </c>
+      <c r="L7" s="4"/>
+      <c r="M7" s="4" t="s">
+        <v>18</v>
+      </c>
       <c r="N7" s="4"/>
       <c r="O7" s="4"/>
       <c r="P7" s="4"/>
       <c r="Q7" s="4"/>
       <c r="R7" s="4"/>
-      <c r="S7" s="3"/>
+      <c r="S7" s="4"/>
       <c r="T7" s="3"/>
       <c r="U7" s="3"/>
       <c r="V7" s="3"/>
@@ -1472,43 +1492,44 @@
       <c r="AE7" s="3"/>
       <c r="AF7" s="3"/>
       <c r="AG7" s="3"/>
-    </row>
-    <row r="8" spans="1:33">
+      <c r="AH7" s="3"/>
+    </row>
+    <row r="8" spans="1:34">
       <c r="A8" s="3"/>
       <c r="B8" s="4" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F8" s="4" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="G8" s="4" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="H8" s="4"/>
       <c r="I8" s="4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="J8" s="4"/>
       <c r="K8" s="4"/>
-      <c r="L8" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="M8" s="4"/>
+      <c r="L8" s="4"/>
+      <c r="M8" s="4" t="s">
+        <v>18</v>
+      </c>
       <c r="N8" s="4"/>
       <c r="O8" s="4"/>
       <c r="P8" s="4"/>
       <c r="Q8" s="4"/>
       <c r="R8" s="4"/>
-      <c r="S8" s="3"/>
+      <c r="S8" s="4"/>
       <c r="T8" s="3"/>
       <c r="U8" s="3"/>
       <c r="V8" s="3"/>
@@ -1523,47 +1544,45 @@
       <c r="AE8" s="3"/>
       <c r="AF8" s="3"/>
       <c r="AG8" s="3"/>
-    </row>
-    <row r="9" spans="2:33">
-      <c r="B9" s="2" t="s">
-        <v>36</v>
+      <c r="AH8" s="3"/>
+    </row>
+    <row r="9" spans="1:34">
+      <c r="A9" s="3"/>
+      <c r="B9" s="4" t="s">
+        <v>37</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="D9" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="E9" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="F9" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="D9" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="G9" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="H9" s="4" t="s">
-        <v>37</v>
-      </c>
-      <c r="I9" s="4" t="s">
+      <c r="E9" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="F9" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="G9" s="4"/>
+      <c r="H9" s="4"/>
+      <c r="I9" s="4"/>
+      <c r="J9" s="4"/>
+      <c r="K9" s="4"/>
+      <c r="L9" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="J9" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="K9" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="L9" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="M9" s="2"/>
-      <c r="N9" s="2"/>
-      <c r="O9" s="2"/>
-      <c r="P9" s="2"/>
-      <c r="Q9" s="2"/>
-      <c r="R9" s="2"/>
+      <c r="M9" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="N9" s="4"/>
+      <c r="O9" s="4"/>
+      <c r="P9" s="4"/>
+      <c r="Q9" s="4"/>
+      <c r="R9" s="4"/>
+      <c r="S9" s="4"/>
+      <c r="T9" s="3"/>
+      <c r="U9" s="3"/>
+      <c r="V9" s="3"/>
       <c r="W9" s="3"/>
       <c r="X9" s="3"/>
       <c r="Y9" s="3"/>
@@ -1575,31 +1594,51 @@
       <c r="AE9" s="3"/>
       <c r="AF9" s="3"/>
       <c r="AG9" s="3"/>
-    </row>
-    <row r="10" spans="1:33">
-      <c r="A10" s="3"/>
-      <c r="B10" s="4"/>
-      <c r="C10" s="4"/>
-      <c r="D10" s="4"/>
-      <c r="E10" s="4"/>
-      <c r="F10" s="4"/>
-      <c r="G10" s="4"/>
-      <c r="H10" s="4"/>
-      <c r="I10" s="4"/>
-      <c r="J10" s="4"/>
-      <c r="K10" s="4"/>
-      <c r="L10" s="4"/>
-      <c r="M10" s="4"/>
-      <c r="N10" s="4"/>
-      <c r="O10" s="4"/>
-      <c r="P10" s="4"/>
-      <c r="Q10" s="4"/>
-      <c r="R10" s="4"/>
-      <c r="S10" s="3"/>
-      <c r="T10" s="3"/>
-      <c r="U10" s="3"/>
-      <c r="V10" s="3"/>
-      <c r="W10" s="3"/>
+      <c r="AH9" s="3"/>
+    </row>
+    <row r="10" spans="2:34">
+      <c r="B10" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="F10" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="G10" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="H10" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="I10" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="J10" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="K10" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="L10" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="M10" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="N10" s="2"/>
+      <c r="O10" s="2"/>
+      <c r="P10" s="2"/>
+      <c r="Q10" s="2"/>
+      <c r="R10" s="2"/>
+      <c r="S10" s="2"/>
       <c r="X10" s="3"/>
       <c r="Y10" s="3"/>
       <c r="Z10" s="3"/>
@@ -1610,8 +1649,9 @@
       <c r="AE10" s="3"/>
       <c r="AF10" s="3"/>
       <c r="AG10" s="3"/>
-    </row>
-    <row r="11" s="1" customFormat="1" spans="1:33">
+      <c r="AH10" s="3"/>
+    </row>
+    <row r="11" spans="1:34">
       <c r="A11" s="3"/>
       <c r="B11" s="4"/>
       <c r="C11" s="4"/>
@@ -1630,7 +1670,7 @@
       <c r="P11" s="4"/>
       <c r="Q11" s="4"/>
       <c r="R11" s="4"/>
-      <c r="S11" s="3"/>
+      <c r="S11" s="4"/>
       <c r="T11" s="3"/>
       <c r="U11" s="3"/>
       <c r="V11" s="3"/>
@@ -1645,8 +1685,9 @@
       <c r="AE11" s="3"/>
       <c r="AF11" s="3"/>
       <c r="AG11" s="3"/>
-    </row>
-    <row r="12" s="1" customFormat="1" spans="1:33">
+      <c r="AH11" s="3"/>
+    </row>
+    <row r="12" s="1" customFormat="1" spans="1:34">
       <c r="A12" s="3"/>
       <c r="B12" s="4"/>
       <c r="C12" s="4"/>
@@ -1665,7 +1706,7 @@
       <c r="P12" s="4"/>
       <c r="Q12" s="4"/>
       <c r="R12" s="4"/>
-      <c r="S12" s="3"/>
+      <c r="S12" s="4"/>
       <c r="T12" s="3"/>
       <c r="U12" s="3"/>
       <c r="V12" s="3"/>
@@ -1680,8 +1721,9 @@
       <c r="AE12" s="3"/>
       <c r="AF12" s="3"/>
       <c r="AG12" s="3"/>
-    </row>
-    <row r="13" spans="1:33">
+      <c r="AH12" s="3"/>
+    </row>
+    <row r="13" s="1" customFormat="1" spans="1:34">
       <c r="A13" s="3"/>
       <c r="B13" s="4"/>
       <c r="C13" s="4"/>
@@ -1700,7 +1742,7 @@
       <c r="P13" s="4"/>
       <c r="Q13" s="4"/>
       <c r="R13" s="4"/>
-      <c r="S13" s="3"/>
+      <c r="S13" s="4"/>
       <c r="T13" s="3"/>
       <c r="U13" s="3"/>
       <c r="V13" s="3"/>
@@ -1715,8 +1757,9 @@
       <c r="AE13" s="3"/>
       <c r="AF13" s="3"/>
       <c r="AG13" s="3"/>
-    </row>
-    <row r="14" spans="1:33">
+      <c r="AH13" s="3"/>
+    </row>
+    <row r="14" spans="1:34">
       <c r="A14" s="3"/>
       <c r="B14" s="4"/>
       <c r="C14" s="4"/>
@@ -1735,7 +1778,7 @@
       <c r="P14" s="4"/>
       <c r="Q14" s="4"/>
       <c r="R14" s="4"/>
-      <c r="S14" s="3"/>
+      <c r="S14" s="4"/>
       <c r="T14" s="3"/>
       <c r="U14" s="3"/>
       <c r="V14" s="3"/>
@@ -1750,8 +1793,9 @@
       <c r="AE14" s="3"/>
       <c r="AF14" s="3"/>
       <c r="AG14" s="3"/>
-    </row>
-    <row r="15" spans="1:33">
+      <c r="AH14" s="3"/>
+    </row>
+    <row r="15" spans="1:34">
       <c r="A15" s="3"/>
       <c r="B15" s="4"/>
       <c r="C15" s="4"/>
@@ -1770,7 +1814,7 @@
       <c r="P15" s="4"/>
       <c r="Q15" s="4"/>
       <c r="R15" s="4"/>
-      <c r="S15" s="3"/>
+      <c r="S15" s="4"/>
       <c r="T15" s="3"/>
       <c r="U15" s="3"/>
       <c r="V15" s="3"/>
@@ -1785,8 +1829,9 @@
       <c r="AE15" s="3"/>
       <c r="AF15" s="3"/>
       <c r="AG15" s="3"/>
-    </row>
-    <row r="16" spans="1:33">
+      <c r="AH15" s="3"/>
+    </row>
+    <row r="16" spans="1:34">
       <c r="A16" s="3"/>
       <c r="B16" s="4"/>
       <c r="C16" s="4"/>
@@ -1805,7 +1850,7 @@
       <c r="P16" s="4"/>
       <c r="Q16" s="4"/>
       <c r="R16" s="4"/>
-      <c r="S16" s="3"/>
+      <c r="S16" s="4"/>
       <c r="T16" s="3"/>
       <c r="U16" s="3"/>
       <c r="V16" s="3"/>
@@ -1820,8 +1865,9 @@
       <c r="AE16" s="3"/>
       <c r="AF16" s="3"/>
       <c r="AG16" s="3"/>
-    </row>
-    <row r="17" spans="1:33">
+      <c r="AH16" s="3"/>
+    </row>
+    <row r="17" spans="1:34">
       <c r="A17" s="3"/>
       <c r="B17" s="4"/>
       <c r="C17" s="4"/>
@@ -1840,7 +1886,7 @@
       <c r="P17" s="4"/>
       <c r="Q17" s="4"/>
       <c r="R17" s="4"/>
-      <c r="S17" s="3"/>
+      <c r="S17" s="4"/>
       <c r="T17" s="3"/>
       <c r="U17" s="3"/>
       <c r="V17" s="3"/>
@@ -1855,8 +1901,9 @@
       <c r="AE17" s="3"/>
       <c r="AF17" s="3"/>
       <c r="AG17" s="3"/>
-    </row>
-    <row r="18" spans="1:33">
+      <c r="AH17" s="3"/>
+    </row>
+    <row r="18" spans="1:34">
       <c r="A18" s="3"/>
       <c r="B18" s="4"/>
       <c r="C18" s="4"/>
@@ -1875,7 +1922,7 @@
       <c r="P18" s="4"/>
       <c r="Q18" s="4"/>
       <c r="R18" s="4"/>
-      <c r="S18" s="3"/>
+      <c r="S18" s="4"/>
       <c r="T18" s="3"/>
       <c r="U18" s="3"/>
       <c r="V18" s="3"/>
@@ -1890,8 +1937,9 @@
       <c r="AE18" s="3"/>
       <c r="AF18" s="3"/>
       <c r="AG18" s="3"/>
-    </row>
-    <row r="19" spans="1:33">
+      <c r="AH18" s="3"/>
+    </row>
+    <row r="19" spans="1:34">
       <c r="A19" s="3"/>
       <c r="B19" s="4"/>
       <c r="C19" s="4"/>
@@ -1910,7 +1958,7 @@
       <c r="P19" s="4"/>
       <c r="Q19" s="4"/>
       <c r="R19" s="4"/>
-      <c r="S19" s="3"/>
+      <c r="S19" s="4"/>
       <c r="T19" s="3"/>
       <c r="U19" s="3"/>
       <c r="V19" s="3"/>
@@ -1925,8 +1973,9 @@
       <c r="AE19" s="3"/>
       <c r="AF19" s="3"/>
       <c r="AG19" s="3"/>
-    </row>
-    <row r="20" spans="1:33">
+      <c r="AH19" s="3"/>
+    </row>
+    <row r="20" spans="1:34">
       <c r="A20" s="3"/>
       <c r="B20" s="4"/>
       <c r="C20" s="4"/>
@@ -1945,7 +1994,7 @@
       <c r="P20" s="4"/>
       <c r="Q20" s="4"/>
       <c r="R20" s="4"/>
-      <c r="S20" s="3"/>
+      <c r="S20" s="4"/>
       <c r="T20" s="3"/>
       <c r="U20" s="3"/>
       <c r="V20" s="3"/>
@@ -1960,8 +2009,9 @@
       <c r="AE20" s="3"/>
       <c r="AF20" s="3"/>
       <c r="AG20" s="3"/>
-    </row>
-    <row r="21" spans="1:33">
+      <c r="AH20" s="3"/>
+    </row>
+    <row r="21" spans="1:34">
       <c r="A21" s="3"/>
       <c r="B21" s="4"/>
       <c r="C21" s="4"/>
@@ -1980,7 +2030,7 @@
       <c r="P21" s="4"/>
       <c r="Q21" s="4"/>
       <c r="R21" s="4"/>
-      <c r="S21" s="3"/>
+      <c r="S21" s="4"/>
       <c r="T21" s="3"/>
       <c r="U21" s="3"/>
       <c r="V21" s="3"/>
@@ -1995,8 +2045,9 @@
       <c r="AE21" s="3"/>
       <c r="AF21" s="3"/>
       <c r="AG21" s="3"/>
-    </row>
-    <row r="22" spans="1:33">
+      <c r="AH21" s="3"/>
+    </row>
+    <row r="22" spans="1:34">
       <c r="A22" s="3"/>
       <c r="B22" s="4"/>
       <c r="C22" s="4"/>
@@ -2015,7 +2066,7 @@
       <c r="P22" s="4"/>
       <c r="Q22" s="4"/>
       <c r="R22" s="4"/>
-      <c r="S22" s="3"/>
+      <c r="S22" s="4"/>
       <c r="T22" s="3"/>
       <c r="U22" s="3"/>
       <c r="V22" s="3"/>
@@ -2030,8 +2081,9 @@
       <c r="AE22" s="3"/>
       <c r="AF22" s="3"/>
       <c r="AG22" s="3"/>
-    </row>
-    <row r="23" spans="1:33">
+      <c r="AH22" s="3"/>
+    </row>
+    <row r="23" spans="1:34">
       <c r="A23" s="3"/>
       <c r="B23" s="4"/>
       <c r="C23" s="4"/>
@@ -2050,7 +2102,7 @@
       <c r="P23" s="4"/>
       <c r="Q23" s="4"/>
       <c r="R23" s="4"/>
-      <c r="S23" s="3"/>
+      <c r="S23" s="4"/>
       <c r="T23" s="3"/>
       <c r="U23" s="3"/>
       <c r="V23" s="3"/>
@@ -2065,8 +2117,9 @@
       <c r="AE23" s="3"/>
       <c r="AF23" s="3"/>
       <c r="AG23" s="3"/>
-    </row>
-    <row r="24" spans="1:33">
+      <c r="AH23" s="3"/>
+    </row>
+    <row r="24" spans="1:34">
       <c r="A24" s="3"/>
       <c r="B24" s="4"/>
       <c r="C24" s="4"/>
@@ -2085,7 +2138,7 @@
       <c r="P24" s="4"/>
       <c r="Q24" s="4"/>
       <c r="R24" s="4"/>
-      <c r="S24" s="3"/>
+      <c r="S24" s="4"/>
       <c r="T24" s="3"/>
       <c r="U24" s="3"/>
       <c r="V24" s="3"/>
@@ -2100,8 +2153,9 @@
       <c r="AE24" s="3"/>
       <c r="AF24" s="3"/>
       <c r="AG24" s="3"/>
-    </row>
-    <row r="25" spans="1:33">
+      <c r="AH24" s="3"/>
+    </row>
+    <row r="25" spans="1:34">
       <c r="A25" s="3"/>
       <c r="B25" s="4"/>
       <c r="C25" s="4"/>
@@ -2120,7 +2174,7 @@
       <c r="P25" s="4"/>
       <c r="Q25" s="4"/>
       <c r="R25" s="4"/>
-      <c r="S25" s="3"/>
+      <c r="S25" s="4"/>
       <c r="T25" s="3"/>
       <c r="U25" s="3"/>
       <c r="V25" s="3"/>
@@ -2135,8 +2189,9 @@
       <c r="AE25" s="3"/>
       <c r="AF25" s="3"/>
       <c r="AG25" s="3"/>
-    </row>
-    <row r="26" spans="1:33">
+      <c r="AH25" s="3"/>
+    </row>
+    <row r="26" spans="1:34">
       <c r="A26" s="3"/>
       <c r="B26" s="4"/>
       <c r="C26" s="4"/>
@@ -2155,7 +2210,7 @@
       <c r="P26" s="4"/>
       <c r="Q26" s="4"/>
       <c r="R26" s="4"/>
-      <c r="S26" s="3"/>
+      <c r="S26" s="4"/>
       <c r="T26" s="3"/>
       <c r="U26" s="3"/>
       <c r="V26" s="3"/>
@@ -2170,8 +2225,9 @@
       <c r="AE26" s="3"/>
       <c r="AF26" s="3"/>
       <c r="AG26" s="3"/>
-    </row>
-    <row r="27" spans="1:33">
+      <c r="AH26" s="3"/>
+    </row>
+    <row r="27" spans="1:34">
       <c r="A27" s="3"/>
       <c r="B27" s="4"/>
       <c r="C27" s="4"/>
@@ -2190,7 +2246,7 @@
       <c r="P27" s="4"/>
       <c r="Q27" s="4"/>
       <c r="R27" s="4"/>
-      <c r="S27" s="3"/>
+      <c r="S27" s="4"/>
       <c r="T27" s="3"/>
       <c r="U27" s="3"/>
       <c r="V27" s="3"/>
@@ -2205,13 +2261,14 @@
       <c r="AE27" s="3"/>
       <c r="AF27" s="3"/>
       <c r="AG27" s="3"/>
-    </row>
-    <row r="28" spans="1:33">
+      <c r="AH27" s="3"/>
+    </row>
+    <row r="28" spans="1:34">
       <c r="A28" s="3"/>
       <c r="B28" s="4"/>
       <c r="C28" s="4"/>
       <c r="D28" s="4"/>
-      <c r="E28" s="5"/>
+      <c r="E28" s="4"/>
       <c r="F28" s="4"/>
       <c r="G28" s="4"/>
       <c r="H28" s="4"/>
@@ -2225,7 +2282,7 @@
       <c r="P28" s="4"/>
       <c r="Q28" s="4"/>
       <c r="R28" s="4"/>
-      <c r="S28" s="3"/>
+      <c r="S28" s="4"/>
       <c r="T28" s="3"/>
       <c r="U28" s="3"/>
       <c r="V28" s="3"/>
@@ -2240,8 +2297,9 @@
       <c r="AE28" s="3"/>
       <c r="AF28" s="3"/>
       <c r="AG28" s="3"/>
-    </row>
-    <row r="29" spans="1:33">
+      <c r="AH28" s="3"/>
+    </row>
+    <row r="29" spans="1:34">
       <c r="A29" s="3"/>
       <c r="B29" s="4"/>
       <c r="C29" s="4"/>
@@ -2260,7 +2318,7 @@
       <c r="P29" s="4"/>
       <c r="Q29" s="4"/>
       <c r="R29" s="4"/>
-      <c r="S29" s="3"/>
+      <c r="S29" s="4"/>
       <c r="T29" s="3"/>
       <c r="U29" s="3"/>
       <c r="V29" s="3"/>
@@ -2275,8 +2333,9 @@
       <c r="AE29" s="3"/>
       <c r="AF29" s="3"/>
       <c r="AG29" s="3"/>
-    </row>
-    <row r="30" spans="1:33">
+      <c r="AH29" s="3"/>
+    </row>
+    <row r="30" spans="1:34">
       <c r="A30" s="3"/>
       <c r="B30" s="4"/>
       <c r="C30" s="4"/>
@@ -2295,7 +2354,7 @@
       <c r="P30" s="4"/>
       <c r="Q30" s="4"/>
       <c r="R30" s="4"/>
-      <c r="S30" s="3"/>
+      <c r="S30" s="4"/>
       <c r="T30" s="3"/>
       <c r="U30" s="3"/>
       <c r="V30" s="3"/>
@@ -2310,13 +2369,14 @@
       <c r="AE30" s="3"/>
       <c r="AF30" s="3"/>
       <c r="AG30" s="3"/>
-    </row>
-    <row r="31" spans="1:33">
+      <c r="AH30" s="3"/>
+    </row>
+    <row r="31" spans="1:34">
       <c r="A31" s="3"/>
       <c r="B31" s="4"/>
       <c r="C31" s="4"/>
       <c r="D31" s="4"/>
-      <c r="E31" s="4"/>
+      <c r="E31" s="5"/>
       <c r="F31" s="4"/>
       <c r="G31" s="4"/>
       <c r="H31" s="4"/>
@@ -2330,7 +2390,7 @@
       <c r="P31" s="4"/>
       <c r="Q31" s="4"/>
       <c r="R31" s="4"/>
-      <c r="S31" s="3"/>
+      <c r="S31" s="4"/>
       <c r="T31" s="3"/>
       <c r="U31" s="3"/>
       <c r="V31" s="3"/>
@@ -2345,8 +2405,9 @@
       <c r="AE31" s="3"/>
       <c r="AF31" s="3"/>
       <c r="AG31" s="3"/>
-    </row>
-    <row r="32" spans="1:33">
+      <c r="AH31" s="3"/>
+    </row>
+    <row r="32" spans="1:34">
       <c r="A32" s="3"/>
       <c r="B32" s="4"/>
       <c r="C32" s="4"/>
@@ -2365,7 +2426,7 @@
       <c r="P32" s="4"/>
       <c r="Q32" s="4"/>
       <c r="R32" s="4"/>
-      <c r="S32" s="3"/>
+      <c r="S32" s="4"/>
       <c r="T32" s="3"/>
       <c r="U32" s="3"/>
       <c r="V32" s="3"/>
@@ -2380,8 +2441,9 @@
       <c r="AE32" s="3"/>
       <c r="AF32" s="3"/>
       <c r="AG32" s="3"/>
-    </row>
-    <row r="33" spans="1:33">
+      <c r="AH32" s="3"/>
+    </row>
+    <row r="33" spans="1:34">
       <c r="A33" s="3"/>
       <c r="B33" s="4"/>
       <c r="C33" s="4"/>
@@ -2400,7 +2462,7 @@
       <c r="P33" s="4"/>
       <c r="Q33" s="4"/>
       <c r="R33" s="4"/>
-      <c r="S33" s="3"/>
+      <c r="S33" s="4"/>
       <c r="T33" s="3"/>
       <c r="U33" s="3"/>
       <c r="V33" s="3"/>
@@ -2415,8 +2477,9 @@
       <c r="AE33" s="3"/>
       <c r="AF33" s="3"/>
       <c r="AG33" s="3"/>
-    </row>
-    <row r="34" spans="1:33">
+      <c r="AH33" s="3"/>
+    </row>
+    <row r="34" spans="1:34">
       <c r="A34" s="3"/>
       <c r="B34" s="4"/>
       <c r="C34" s="4"/>
@@ -2435,7 +2498,7 @@
       <c r="P34" s="4"/>
       <c r="Q34" s="4"/>
       <c r="R34" s="4"/>
-      <c r="S34" s="3"/>
+      <c r="S34" s="4"/>
       <c r="T34" s="3"/>
       <c r="U34" s="3"/>
       <c r="V34" s="3"/>
@@ -2450,13 +2513,14 @@
       <c r="AE34" s="3"/>
       <c r="AF34" s="3"/>
       <c r="AG34" s="3"/>
-    </row>
-    <row r="35" spans="1:33">
+      <c r="AH34" s="3"/>
+    </row>
+    <row r="35" spans="1:34">
       <c r="A35" s="3"/>
       <c r="B35" s="4"/>
       <c r="C35" s="4"/>
       <c r="D35" s="4"/>
-      <c r="E35" s="5"/>
+      <c r="E35" s="4"/>
       <c r="F35" s="4"/>
       <c r="G35" s="4"/>
       <c r="H35" s="4"/>
@@ -2470,7 +2534,7 @@
       <c r="P35" s="4"/>
       <c r="Q35" s="4"/>
       <c r="R35" s="4"/>
-      <c r="S35" s="3"/>
+      <c r="S35" s="4"/>
       <c r="T35" s="3"/>
       <c r="U35" s="3"/>
       <c r="V35" s="3"/>
@@ -2485,13 +2549,14 @@
       <c r="AE35" s="3"/>
       <c r="AF35" s="3"/>
       <c r="AG35" s="3"/>
-    </row>
-    <row r="36" spans="1:33">
+      <c r="AH35" s="3"/>
+    </row>
+    <row r="36" spans="1:34">
       <c r="A36" s="3"/>
       <c r="B36" s="4"/>
       <c r="C36" s="4"/>
       <c r="D36" s="4"/>
-      <c r="E36" s="4"/>
+      <c r="E36" s="5"/>
       <c r="F36" s="4"/>
       <c r="G36" s="4"/>
       <c r="H36" s="4"/>
@@ -2505,7 +2570,7 @@
       <c r="P36" s="4"/>
       <c r="Q36" s="4"/>
       <c r="R36" s="4"/>
-      <c r="S36" s="3"/>
+      <c r="S36" s="4"/>
       <c r="T36" s="3"/>
       <c r="U36" s="3"/>
       <c r="V36" s="3"/>
@@ -2520,8 +2585,9 @@
       <c r="AE36" s="3"/>
       <c r="AF36" s="3"/>
       <c r="AG36" s="3"/>
-    </row>
-    <row r="37" spans="1:33">
+      <c r="AH36" s="3"/>
+    </row>
+    <row r="37" spans="1:34">
       <c r="A37" s="3"/>
       <c r="B37" s="4"/>
       <c r="C37" s="4"/>
@@ -2540,7 +2606,7 @@
       <c r="P37" s="4"/>
       <c r="Q37" s="4"/>
       <c r="R37" s="4"/>
-      <c r="S37" s="3"/>
+      <c r="S37" s="4"/>
       <c r="T37" s="3"/>
       <c r="U37" s="3"/>
       <c r="V37" s="3"/>
@@ -2555,8 +2621,9 @@
       <c r="AE37" s="3"/>
       <c r="AF37" s="3"/>
       <c r="AG37" s="3"/>
-    </row>
-    <row r="38" spans="1:33">
+      <c r="AH37" s="3"/>
+    </row>
+    <row r="38" spans="1:34">
       <c r="A38" s="3"/>
       <c r="B38" s="4"/>
       <c r="C38" s="4"/>
@@ -2575,7 +2642,7 @@
       <c r="P38" s="4"/>
       <c r="Q38" s="4"/>
       <c r="R38" s="4"/>
-      <c r="S38" s="3"/>
+      <c r="S38" s="4"/>
       <c r="T38" s="3"/>
       <c r="U38" s="3"/>
       <c r="V38" s="3"/>
@@ -2590,8 +2657,9 @@
       <c r="AE38" s="3"/>
       <c r="AF38" s="3"/>
       <c r="AG38" s="3"/>
-    </row>
-    <row r="39" spans="1:33">
+      <c r="AH38" s="3"/>
+    </row>
+    <row r="39" spans="1:34">
       <c r="A39" s="3"/>
       <c r="B39" s="4"/>
       <c r="C39" s="4"/>
@@ -2610,7 +2678,7 @@
       <c r="P39" s="4"/>
       <c r="Q39" s="4"/>
       <c r="R39" s="4"/>
-      <c r="S39" s="3"/>
+      <c r="S39" s="4"/>
       <c r="T39" s="3"/>
       <c r="U39" s="3"/>
       <c r="V39" s="3"/>
@@ -2625,8 +2693,9 @@
       <c r="AE39" s="3"/>
       <c r="AF39" s="3"/>
       <c r="AG39" s="3"/>
-    </row>
-    <row r="40" spans="1:33">
+      <c r="AH39" s="3"/>
+    </row>
+    <row r="40" spans="1:34">
       <c r="A40" s="3"/>
       <c r="B40" s="4"/>
       <c r="C40" s="4"/>
@@ -2645,7 +2714,7 @@
       <c r="P40" s="4"/>
       <c r="Q40" s="4"/>
       <c r="R40" s="4"/>
-      <c r="S40" s="3"/>
+      <c r="S40" s="4"/>
       <c r="T40" s="3"/>
       <c r="U40" s="3"/>
       <c r="V40" s="3"/>
@@ -2660,8 +2729,9 @@
       <c r="AE40" s="3"/>
       <c r="AF40" s="3"/>
       <c r="AG40" s="3"/>
-    </row>
-    <row r="41" spans="1:33">
+      <c r="AH40" s="3"/>
+    </row>
+    <row r="41" spans="1:34">
       <c r="A41" s="3"/>
       <c r="B41" s="4"/>
       <c r="C41" s="4"/>
@@ -2680,7 +2750,7 @@
       <c r="P41" s="4"/>
       <c r="Q41" s="4"/>
       <c r="R41" s="4"/>
-      <c r="S41" s="3"/>
+      <c r="S41" s="4"/>
       <c r="T41" s="3"/>
       <c r="U41" s="3"/>
       <c r="V41" s="3"/>
@@ -2695,8 +2765,9 @@
       <c r="AE41" s="3"/>
       <c r="AF41" s="3"/>
       <c r="AG41" s="3"/>
-    </row>
-    <row r="42" spans="1:33">
+      <c r="AH41" s="3"/>
+    </row>
+    <row r="42" spans="1:34">
       <c r="A42" s="3"/>
       <c r="B42" s="4"/>
       <c r="C42" s="4"/>
@@ -2715,7 +2786,7 @@
       <c r="P42" s="4"/>
       <c r="Q42" s="4"/>
       <c r="R42" s="4"/>
-      <c r="S42" s="3"/>
+      <c r="S42" s="4"/>
       <c r="T42" s="3"/>
       <c r="U42" s="3"/>
       <c r="V42" s="3"/>
@@ -2730,8 +2801,9 @@
       <c r="AE42" s="3"/>
       <c r="AF42" s="3"/>
       <c r="AG42" s="3"/>
-    </row>
-    <row r="43" spans="1:33">
+      <c r="AH42" s="3"/>
+    </row>
+    <row r="43" spans="1:34">
       <c r="A43" s="3"/>
       <c r="B43" s="4"/>
       <c r="C43" s="4"/>
@@ -2750,7 +2822,7 @@
       <c r="P43" s="4"/>
       <c r="Q43" s="4"/>
       <c r="R43" s="4"/>
-      <c r="S43" s="3"/>
+      <c r="S43" s="4"/>
       <c r="T43" s="3"/>
       <c r="U43" s="3"/>
       <c r="V43" s="3"/>
@@ -2765,205 +2837,245 @@
       <c r="AE43" s="3"/>
       <c r="AF43" s="3"/>
       <c r="AG43" s="3"/>
-    </row>
-    <row r="51" spans="1:22">
-      <c r="A51" s="2"/>
-      <c r="B51" s="2"/>
-      <c r="C51" s="2"/>
-      <c r="D51" s="2"/>
-      <c r="Q51" s="2"/>
-      <c r="S51" s="2"/>
-      <c r="T51" s="2"/>
-      <c r="U51" s="2"/>
-      <c r="V51" s="2"/>
-    </row>
-    <row r="52" spans="1:22">
+      <c r="AH43" s="3"/>
+    </row>
+    <row r="44" spans="1:34">
+      <c r="A44" s="3"/>
+      <c r="B44" s="4"/>
+      <c r="C44" s="4"/>
+      <c r="D44" s="4"/>
+      <c r="E44" s="4"/>
+      <c r="F44" s="4"/>
+      <c r="G44" s="4"/>
+      <c r="H44" s="4"/>
+      <c r="I44" s="4"/>
+      <c r="J44" s="4"/>
+      <c r="K44" s="4"/>
+      <c r="L44" s="4"/>
+      <c r="M44" s="4"/>
+      <c r="N44" s="4"/>
+      <c r="O44" s="4"/>
+      <c r="P44" s="4"/>
+      <c r="Q44" s="4"/>
+      <c r="R44" s="4"/>
+      <c r="S44" s="4"/>
+      <c r="T44" s="3"/>
+      <c r="U44" s="3"/>
+      <c r="V44" s="3"/>
+      <c r="W44" s="3"/>
+      <c r="X44" s="3"/>
+      <c r="Y44" s="3"/>
+      <c r="Z44" s="3"/>
+      <c r="AA44" s="3"/>
+      <c r="AB44" s="3"/>
+      <c r="AC44" s="3"/>
+      <c r="AD44" s="3"/>
+      <c r="AE44" s="3"/>
+      <c r="AF44" s="3"/>
+      <c r="AG44" s="3"/>
+      <c r="AH44" s="3"/>
+    </row>
+    <row r="52" spans="1:23">
       <c r="A52" s="2"/>
       <c r="B52" s="2"/>
       <c r="C52" s="2"/>
       <c r="D52" s="2"/>
-      <c r="E52" s="2"/>
-      <c r="Q52" s="2"/>
       <c r="R52" s="2"/>
-      <c r="S52" s="2"/>
       <c r="T52" s="2"/>
       <c r="U52" s="2"/>
       <c r="V52" s="2"/>
-    </row>
-    <row r="53" spans="1:22">
+      <c r="W52" s="2"/>
+    </row>
+    <row r="53" spans="1:23">
       <c r="A53" s="2"/>
       <c r="B53" s="2"/>
       <c r="C53" s="2"/>
       <c r="D53" s="2"/>
-      <c r="Q53" s="2"/>
+      <c r="E53" s="2"/>
       <c r="R53" s="2"/>
       <c r="S53" s="2"/>
       <c r="T53" s="2"/>
       <c r="U53" s="2"/>
       <c r="V53" s="2"/>
-    </row>
-    <row r="54" spans="1:22">
+      <c r="W53" s="2"/>
+    </row>
+    <row r="54" spans="1:23">
       <c r="A54" s="2"/>
       <c r="B54" s="2"/>
       <c r="C54" s="2"/>
       <c r="D54" s="2"/>
-      <c r="Q54" s="2"/>
       <c r="R54" s="2"/>
       <c r="S54" s="2"/>
       <c r="T54" s="2"/>
       <c r="U54" s="2"/>
       <c r="V54" s="2"/>
-    </row>
-    <row r="55" spans="1:22">
+      <c r="W54" s="2"/>
+    </row>
+    <row r="55" spans="1:23">
       <c r="A55" s="2"/>
       <c r="B55" s="2"/>
       <c r="C55" s="2"/>
       <c r="D55" s="2"/>
-      <c r="Q55" s="2"/>
       <c r="R55" s="2"/>
       <c r="S55" s="2"/>
       <c r="T55" s="2"/>
       <c r="U55" s="2"/>
       <c r="V55" s="2"/>
-    </row>
-    <row r="56" spans="1:22">
+      <c r="W55" s="2"/>
+    </row>
+    <row r="56" spans="1:23">
       <c r="A56" s="2"/>
       <c r="B56" s="2"/>
       <c r="C56" s="2"/>
       <c r="D56" s="2"/>
-      <c r="Q56" s="2"/>
       <c r="R56" s="2"/>
       <c r="S56" s="2"/>
       <c r="T56" s="2"/>
       <c r="U56" s="2"/>
       <c r="V56" s="2"/>
-    </row>
-    <row r="57" spans="1:22">
+      <c r="W56" s="2"/>
+    </row>
+    <row r="57" spans="1:23">
       <c r="A57" s="2"/>
       <c r="B57" s="2"/>
       <c r="C57" s="2"/>
       <c r="D57" s="2"/>
-      <c r="Q57" s="2"/>
       <c r="R57" s="2"/>
       <c r="S57" s="2"/>
       <c r="T57" s="2"/>
       <c r="U57" s="2"/>
       <c r="V57" s="2"/>
-    </row>
-    <row r="58" spans="1:22">
+      <c r="W57" s="2"/>
+    </row>
+    <row r="58" spans="1:23">
       <c r="A58" s="2"/>
       <c r="B58" s="2"/>
       <c r="C58" s="2"/>
       <c r="D58" s="2"/>
-      <c r="Q58" s="2"/>
       <c r="R58" s="2"/>
       <c r="S58" s="2"/>
       <c r="T58" s="2"/>
       <c r="U58" s="2"/>
       <c r="V58" s="2"/>
-    </row>
-    <row r="59" spans="1:22">
+      <c r="W58" s="2"/>
+    </row>
+    <row r="59" spans="1:23">
       <c r="A59" s="2"/>
       <c r="B59" s="2"/>
       <c r="C59" s="2"/>
       <c r="D59" s="2"/>
-      <c r="Q59" s="2"/>
       <c r="R59" s="2"/>
       <c r="S59" s="2"/>
       <c r="T59" s="2"/>
       <c r="U59" s="2"/>
       <c r="V59" s="2"/>
-    </row>
-    <row r="60" spans="1:22">
+      <c r="W59" s="2"/>
+    </row>
+    <row r="60" spans="1:23">
       <c r="A60" s="2"/>
       <c r="B60" s="2"/>
       <c r="C60" s="2"/>
       <c r="D60" s="2"/>
-      <c r="Q60" s="2"/>
       <c r="R60" s="2"/>
       <c r="S60" s="2"/>
       <c r="T60" s="2"/>
       <c r="U60" s="2"/>
       <c r="V60" s="2"/>
-    </row>
-    <row r="61" spans="1:22">
+      <c r="W60" s="2"/>
+    </row>
+    <row r="61" spans="1:23">
       <c r="A61" s="2"/>
       <c r="B61" s="2"/>
       <c r="C61" s="2"/>
       <c r="D61" s="2"/>
-      <c r="Q61" s="2"/>
       <c r="R61" s="2"/>
       <c r="S61" s="2"/>
       <c r="T61" s="2"/>
       <c r="U61" s="2"/>
       <c r="V61" s="2"/>
-    </row>
-    <row r="62" spans="1:22">
+      <c r="W61" s="2"/>
+    </row>
+    <row r="62" spans="1:23">
       <c r="A62" s="2"/>
       <c r="B62" s="2"/>
       <c r="C62" s="2"/>
       <c r="D62" s="2"/>
-      <c r="Q62" s="2"/>
       <c r="R62" s="2"/>
       <c r="S62" s="2"/>
       <c r="T62" s="2"/>
       <c r="U62" s="2"/>
       <c r="V62" s="2"/>
-    </row>
-    <row r="63" spans="1:22">
+      <c r="W62" s="2"/>
+    </row>
+    <row r="63" spans="1:23">
       <c r="A63" s="2"/>
       <c r="B63" s="2"/>
       <c r="C63" s="2"/>
       <c r="D63" s="2"/>
-      <c r="Q63" s="2"/>
       <c r="R63" s="2"/>
       <c r="S63" s="2"/>
       <c r="T63" s="2"/>
       <c r="U63" s="2"/>
       <c r="V63" s="2"/>
-    </row>
-    <row r="64" spans="1:22">
+      <c r="W63" s="2"/>
+    </row>
+    <row r="64" spans="1:23">
       <c r="A64" s="2"/>
       <c r="B64" s="2"/>
       <c r="C64" s="2"/>
       <c r="D64" s="2"/>
-      <c r="Q64" s="2"/>
       <c r="R64" s="2"/>
       <c r="S64" s="2"/>
       <c r="T64" s="2"/>
       <c r="U64" s="2"/>
       <c r="V64" s="2"/>
+      <c r="W64" s="2"/>
+    </row>
+    <row r="65" spans="1:23">
+      <c r="A65" s="2"/>
+      <c r="B65" s="2"/>
+      <c r="C65" s="2"/>
+      <c r="D65" s="2"/>
+      <c r="R65" s="2"/>
+      <c r="S65" s="2"/>
+      <c r="T65" s="2"/>
+      <c r="U65" s="2"/>
+      <c r="V65" s="2"/>
+      <c r="W65" s="2"/>
     </row>
   </sheetData>
-  <dataValidations count="10">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J5 J8 J2:J4 J6:J7 J9:J1048576">
+  <dataValidations count="11">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L2:L1048576">
+      <formula1>"BR_EQ,BR_NE,BR_LTU,BR_GE,BR_GEU,BR_LT,BR_XX"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J5 J8 J9 J2:J4 J6:J7 J10:J1048576">
       <formula1>"ST_SW,ST_SH,ST_SB,ST_XX"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K4 K5 K6 K7 K8 K2:K3 K9:K1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K4 K5 K6 K7 K8 K9 K2:K3 K10:K1048576">
       <formula1>"MASK_XX,MASK_B,MASK_H,MASK_W,MASK_D"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L4 L5 L6 L7 L8 L2:L3 L9:L1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="M4 M5 M6 M7 M8 M9 M2:M3 M10:M1048576">
       <formula1>"INST_VALID,INST_INVALID"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I4 I5 I6 I7 I8 I2:I3 I9:I1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I4 I5 I6 I7 I8 I9 I2:I3 I10:I1048576">
       <formula1>"LD_LB,LD_LH,LD_LW,LD_LBU,LD_LHU,LD_XX"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G4 G5 G6 G7 G8 G2:G3 G9:G1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G4 G5 G6 G7 G8 G9 G2:G3 G10:G1048576">
       <formula1>"IMM_I,IMM_J,IMM_U,IMM_S,IMM_B"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F4 F5 F6 F7 F8 F2:F3 F9:F1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F4 F5 F6 F7 F8 F9 F2:F3 F10:F1048576">
       <formula1>"ALU_ADD,ALU_SUB,ALU_AND,ALU_OR,ALU_XOR,ALU_SLL,ALU_SRL,ALU_SLT,ALU_SLTU,ALU_COPY_A,ALU_COPY_B"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H5 H2:H4 H6:H1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H5 H9 H2:H4 H6:H8 H10:H1048576">
       <formula1>"WB_ALU,WB_MEM,WB_PC4,WB_XX"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D4 D5 D6 D7 D8 D2:D3 D9:D1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D4 D5 D6 D7 D8 D9 D2:D3 D10:D1048576">
       <formula1>"A_PC,A_RS1"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E4 E5 E6 E7 E8 E2:E3 E9:E1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E4 E5 E6 E7 E8 E9 E2:E3 E10:E1048576">
       <formula1>"B_IMM,B_RS2"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C4 C5 C6 C7 C8 C2:C3 C9:C1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C4 C5 C6 C7 C8 C9 C2:C3 C10:C1048576">
       <formula1>"PC_4,PC_0,PC_ALU"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
> sim RTL ysyx_23060246 韩炳晋 Linux archlinux 6.6.60-1-lts #1 SMP PREEMPT_DYNAMIC Fri, 08 Nov 2024 16:03:02 +0000 x86_64 GNU/Linux  18:28:29 up 1 day, 43 min,  2 users,  load average: 4.28, 3.54, 3.38
</commit_message>
<xml_diff>
--- a/npc/tools/control_gen/control_table.xlsx
+++ b/npc/tools/control_gen/control_table.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="47">
   <si>
     <t>commont</t>
   </si>
@@ -128,6 +128,9 @@
   </si>
   <si>
     <t>bgeu</t>
+  </si>
+  <si>
+    <t>IMM_B</t>
   </si>
   <si>
     <t>BR_GEU</t>
@@ -1563,13 +1566,15 @@
       <c r="F9" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="G9" s="4"/>
+      <c r="G9" s="4" t="s">
+        <v>38</v>
+      </c>
       <c r="H9" s="4"/>
       <c r="I9" s="4"/>
       <c r="J9" s="4"/>
       <c r="K9" s="4"/>
       <c r="L9" s="4" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="M9" s="4" t="s">
         <v>18</v>
@@ -1598,7 +1603,7 @@
     </row>
     <row r="10" spans="2:34">
       <c r="B10" s="2" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C10" s="2" t="s">
         <v>35</v>
@@ -1616,22 +1621,22 @@
         <v>24</v>
       </c>
       <c r="H10" s="4" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="I10" s="4" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="J10" s="4" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="K10" s="2" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="L10" s="2" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="M10" s="2" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="N10" s="2"/>
       <c r="O10" s="2"/>

</xml_diff>

<commit_message>
> compile NEMU ysyx_23060246 韩炳晋 Linux archlinux 6.6.60-1-lts #1 SMP PREEMPT_DYNAMIC Fri, 08 Nov 2024 16:03:02 +0000 x86_64 GNU/Linux  18:30:43 up 1 day, 45 min,  2 users,  load average: 5.19, 3.97, 3.55
</commit_message>
<xml_diff>
--- a/npc/tools/control_gen/control_table.xlsx
+++ b/npc/tools/control_gen/control_table.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="49">
   <si>
     <t>commont</t>
   </si>
@@ -134,6 +134,12 @@
   </si>
   <si>
     <t>BR_GEU</t>
+  </si>
+  <si>
+    <t>slli</t>
+  </si>
+  <si>
+    <t>ALU_SLL</t>
   </si>
   <si>
     <t>default</t>
@@ -1123,7 +1129,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:AH65"/>
+  <dimension ref="A1:AH66"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
     <col min="1" max="1" width="13.1" customWidth="1"/>
@@ -1601,49 +1607,44 @@
       <c r="AG9" s="3"/>
       <c r="AH9" s="3"/>
     </row>
-    <row r="10" spans="2:34">
-      <c r="B10" s="2" t="s">
+    <row r="10" spans="1:34">
+      <c r="A10" s="3"/>
+      <c r="B10" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="C10" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="D10" s="2" t="s">
+      <c r="C10" s="2"/>
+      <c r="D10" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="E10" s="2" t="s">
+      <c r="E10" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="F10" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="G10" s="2" t="s">
+      <c r="F10" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="G10" s="4" t="s">
         <v>24</v>
       </c>
       <c r="H10" s="4" t="s">
-        <v>41</v>
-      </c>
-      <c r="I10" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="J10" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="K10" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="L10" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="M10" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="N10" s="2"/>
-      <c r="O10" s="2"/>
-      <c r="P10" s="2"/>
-      <c r="Q10" s="2"/>
-      <c r="R10" s="2"/>
-      <c r="S10" s="2"/>
+        <v>17</v>
+      </c>
+      <c r="I10" s="4"/>
+      <c r="J10" s="4"/>
+      <c r="K10" s="4"/>
+      <c r="L10" s="4"/>
+      <c r="M10" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="N10" s="4"/>
+      <c r="O10" s="4"/>
+      <c r="P10" s="4"/>
+      <c r="Q10" s="4"/>
+      <c r="R10" s="4"/>
+      <c r="S10" s="4"/>
+      <c r="T10" s="3"/>
+      <c r="U10" s="3"/>
+      <c r="V10" s="3"/>
+      <c r="W10" s="3"/>
       <c r="X10" s="3"/>
       <c r="Y10" s="3"/>
       <c r="Z10" s="3"/>
@@ -1656,30 +1657,49 @@
       <c r="AG10" s="3"/>
       <c r="AH10" s="3"/>
     </row>
-    <row r="11" spans="1:34">
-      <c r="A11" s="3"/>
-      <c r="B11" s="4"/>
-      <c r="C11" s="4"/>
-      <c r="D11" s="4"/>
-      <c r="E11" s="4"/>
-      <c r="F11" s="4"/>
-      <c r="G11" s="4"/>
-      <c r="H11" s="4"/>
-      <c r="I11" s="4"/>
-      <c r="J11" s="4"/>
-      <c r="K11" s="4"/>
-      <c r="L11" s="4"/>
-      <c r="M11" s="4"/>
-      <c r="N11" s="4"/>
-      <c r="O11" s="4"/>
-      <c r="P11" s="4"/>
-      <c r="Q11" s="4"/>
-      <c r="R11" s="4"/>
-      <c r="S11" s="4"/>
-      <c r="T11" s="3"/>
-      <c r="U11" s="3"/>
-      <c r="V11" s="3"/>
-      <c r="W11" s="3"/>
+    <row r="11" spans="2:34">
+      <c r="B11" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="F11" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="G11" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="H11" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="I11" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="J11" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="K11" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="L11" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="M11" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="N11" s="2"/>
+      <c r="O11" s="2"/>
+      <c r="P11" s="2"/>
+      <c r="Q11" s="2"/>
+      <c r="R11" s="2"/>
+      <c r="S11" s="2"/>
       <c r="X11" s="3"/>
       <c r="Y11" s="3"/>
       <c r="Z11" s="3"/>
@@ -1692,7 +1712,7 @@
       <c r="AG11" s="3"/>
       <c r="AH11" s="3"/>
     </row>
-    <row r="12" s="1" customFormat="1" spans="1:34">
+    <row r="12" spans="1:34">
       <c r="A12" s="3"/>
       <c r="B12" s="4"/>
       <c r="C12" s="4"/>
@@ -1764,7 +1784,7 @@
       <c r="AG13" s="3"/>
       <c r="AH13" s="3"/>
     </row>
-    <row r="14" spans="1:34">
+    <row r="14" s="1" customFormat="1" spans="1:34">
       <c r="A14" s="3"/>
       <c r="B14" s="4"/>
       <c r="C14" s="4"/>
@@ -2309,7 +2329,7 @@
       <c r="B29" s="4"/>
       <c r="C29" s="4"/>
       <c r="D29" s="4"/>
-      <c r="E29" s="5"/>
+      <c r="E29" s="4"/>
       <c r="F29" s="4"/>
       <c r="G29" s="4"/>
       <c r="H29" s="4"/>
@@ -2417,7 +2437,7 @@
       <c r="B32" s="4"/>
       <c r="C32" s="4"/>
       <c r="D32" s="4"/>
-      <c r="E32" s="4"/>
+      <c r="E32" s="5"/>
       <c r="F32" s="4"/>
       <c r="G32" s="4"/>
       <c r="H32" s="4"/>
@@ -2561,7 +2581,7 @@
       <c r="B36" s="4"/>
       <c r="C36" s="4"/>
       <c r="D36" s="4"/>
-      <c r="E36" s="5"/>
+      <c r="E36" s="4"/>
       <c r="F36" s="4"/>
       <c r="G36" s="4"/>
       <c r="H36" s="4"/>
@@ -2597,7 +2617,7 @@
       <c r="B37" s="4"/>
       <c r="C37" s="4"/>
       <c r="D37" s="4"/>
-      <c r="E37" s="4"/>
+      <c r="E37" s="5"/>
       <c r="F37" s="4"/>
       <c r="G37" s="4"/>
       <c r="H37" s="4"/>
@@ -2880,25 +2900,48 @@
       <c r="AG44" s="3"/>
       <c r="AH44" s="3"/>
     </row>
-    <row r="52" spans="1:23">
-      <c r="A52" s="2"/>
-      <c r="B52" s="2"/>
-      <c r="C52" s="2"/>
-      <c r="D52" s="2"/>
-      <c r="R52" s="2"/>
-      <c r="T52" s="2"/>
-      <c r="U52" s="2"/>
-      <c r="V52" s="2"/>
-      <c r="W52" s="2"/>
+    <row r="45" spans="1:34">
+      <c r="A45" s="3"/>
+      <c r="B45" s="4"/>
+      <c r="C45" s="4"/>
+      <c r="D45" s="4"/>
+      <c r="E45" s="4"/>
+      <c r="F45" s="4"/>
+      <c r="G45" s="4"/>
+      <c r="H45" s="4"/>
+      <c r="I45" s="4"/>
+      <c r="J45" s="4"/>
+      <c r="K45" s="4"/>
+      <c r="L45" s="4"/>
+      <c r="M45" s="4"/>
+      <c r="N45" s="4"/>
+      <c r="O45" s="4"/>
+      <c r="P45" s="4"/>
+      <c r="Q45" s="4"/>
+      <c r="R45" s="4"/>
+      <c r="S45" s="4"/>
+      <c r="T45" s="3"/>
+      <c r="U45" s="3"/>
+      <c r="V45" s="3"/>
+      <c r="W45" s="3"/>
+      <c r="X45" s="3"/>
+      <c r="Y45" s="3"/>
+      <c r="Z45" s="3"/>
+      <c r="AA45" s="3"/>
+      <c r="AB45" s="3"/>
+      <c r="AC45" s="3"/>
+      <c r="AD45" s="3"/>
+      <c r="AE45" s="3"/>
+      <c r="AF45" s="3"/>
+      <c r="AG45" s="3"/>
+      <c r="AH45" s="3"/>
     </row>
     <row r="53" spans="1:23">
       <c r="A53" s="2"/>
       <c r="B53" s="2"/>
       <c r="C53" s="2"/>
       <c r="D53" s="2"/>
-      <c r="E53" s="2"/>
       <c r="R53" s="2"/>
-      <c r="S53" s="2"/>
       <c r="T53" s="2"/>
       <c r="U53" s="2"/>
       <c r="V53" s="2"/>
@@ -2909,6 +2952,7 @@
       <c r="B54" s="2"/>
       <c r="C54" s="2"/>
       <c r="D54" s="2"/>
+      <c r="E54" s="2"/>
       <c r="R54" s="2"/>
       <c r="S54" s="2"/>
       <c r="T54" s="2"/>
@@ -3048,39 +3092,51 @@
       <c r="V65" s="2"/>
       <c r="W65" s="2"/>
     </row>
+    <row r="66" spans="1:23">
+      <c r="A66" s="2"/>
+      <c r="B66" s="2"/>
+      <c r="C66" s="2"/>
+      <c r="D66" s="2"/>
+      <c r="R66" s="2"/>
+      <c r="S66" s="2"/>
+      <c r="T66" s="2"/>
+      <c r="U66" s="2"/>
+      <c r="V66" s="2"/>
+      <c r="W66" s="2"/>
+    </row>
   </sheetData>
   <dataValidations count="11">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L2:L1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L10 L2:L9 L11:L1048576">
       <formula1>"BR_EQ,BR_NE,BR_LTU,BR_GE,BR_GEU,BR_LT,BR_XX"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J5 J8 J9 J2:J4 J6:J7 J10:J1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J5 J8 J9 J10 J2:J4 J6:J7 J11:J1048576">
       <formula1>"ST_SW,ST_SH,ST_SB,ST_XX"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K4 K5 K6 K7 K8 K9 K2:K3 K10:K1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K4 K5 K6 K7 K8 K9 K10 K2:K3 K11:K1048576">
       <formula1>"MASK_XX,MASK_B,MASK_H,MASK_W,MASK_D"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="M4 M5 M6 M7 M8 M9 M2:M3 M10:M1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="M4 M5 M6 M7 M8 M9 M10 M2:M3 M11:M1048576">
       <formula1>"INST_VALID,INST_INVALID"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I4 I5 I6 I7 I8 I9 I2:I3 I10:I1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I4 I5 I6 I7 I8 I9 I10 I2:I3 I11:I1048576">
       <formula1>"LD_LB,LD_LH,LD_LW,LD_LBU,LD_LHU,LD_XX"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G4 G5 G6 G7 G8 G9 G2:G3 G10:G1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G4 G5 G6 G7 G8 G9 G10 G2:G3 G11:G1048576">
       <formula1>"IMM_I,IMM_J,IMM_U,IMM_S,IMM_B"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F4 F5 F6 F7 F8 F9 F2:F3 F10:F1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F4 F5 F6 F7 F8 F9 F10 F2:F3 F11:F1048576">
       <formula1>"ALU_ADD,ALU_SUB,ALU_AND,ALU_OR,ALU_XOR,ALU_SLL,ALU_SRL,ALU_SLT,ALU_SLTU,ALU_COPY_A,ALU_COPY_B"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H5 H9 H2:H4 H6:H8 H10:H1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H5 H9 H10 H2:H4 H6:H8 H11:H1048576">
       <formula1>"WB_ALU,WB_MEM,WB_PC4,WB_XX"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D4 D5 D6 D7 D8 D9 D2:D3 D10:D1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D4 D5 D6 D7 D8 D9 D10 D2:D3 D11:D1048576">
       <formula1>"A_PC,A_RS1"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E4 E5 E6 E7 E8 E9 E2:E3 E10:E1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E4 E5 E6 E7 E8 E9 E10 E2:E3 E11:E1048576">
       <formula1>"B_IMM,B_RS2"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C4 C5 C6 C7 C8 C9 C2:C3 C10:C1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C4 C5 C6 C7 C8 C9 C10 C2:C3 C11:C1048576">
       <formula1>"PC_4,PC_0,PC_ALU"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
> sim RTL ysyx_23060246 韩炳晋 Linux archlinux 6.6.60-1-lts #1 SMP PREEMPT_DYNAMIC Fri, 08 Nov 2024 16:03:02 +0000 x86_64 GNU/Linux  18:32:57 up 1 day, 48 min,  2 users,  load average: 7.27, 5.20, 4.07
</commit_message>
<xml_diff>
--- a/npc/tools/control_gen/control_table.xlsx
+++ b/npc/tools/control_gen/control_table.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="97" uniqueCount="51">
   <si>
     <t>commont</t>
   </si>
@@ -140,6 +140,12 @@
   </si>
   <si>
     <t>ALU_SLL</t>
+  </si>
+  <si>
+    <t>add</t>
+  </si>
+  <si>
+    <t>B_RS2</t>
   </si>
   <si>
     <t>default</t>
@@ -1129,7 +1135,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:AH66"/>
+  <dimension ref="A1:AH67"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
     <col min="1" max="1" width="13.1" customWidth="1"/>
@@ -1657,49 +1663,42 @@
       <c r="AG10" s="3"/>
       <c r="AH10" s="3"/>
     </row>
-    <row r="11" spans="2:34">
-      <c r="B11" s="2" t="s">
+    <row r="11" spans="1:34">
+      <c r="A11" s="3"/>
+      <c r="B11" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="C11" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="D11" s="2" t="s">
+      <c r="C11" s="2"/>
+      <c r="D11" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="E11" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="F11" s="2" t="s">
+      <c r="E11" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="F11" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="G11" s="2" t="s">
-        <v>24</v>
-      </c>
+      <c r="G11" s="4"/>
       <c r="H11" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="I11" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="J11" s="4" t="s">
-        <v>45</v>
-      </c>
-      <c r="K11" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="L11" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="M11" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="N11" s="2"/>
-      <c r="O11" s="2"/>
-      <c r="P11" s="2"/>
-      <c r="Q11" s="2"/>
-      <c r="R11" s="2"/>
-      <c r="S11" s="2"/>
+        <v>17</v>
+      </c>
+      <c r="I11" s="4"/>
+      <c r="J11" s="4"/>
+      <c r="K11" s="4"/>
+      <c r="L11" s="4"/>
+      <c r="M11" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="N11" s="4"/>
+      <c r="O11" s="4"/>
+      <c r="P11" s="4"/>
+      <c r="Q11" s="4"/>
+      <c r="R11" s="4"/>
+      <c r="S11" s="4"/>
+      <c r="T11" s="3"/>
+      <c r="U11" s="3"/>
+      <c r="V11" s="3"/>
+      <c r="W11" s="3"/>
       <c r="X11" s="3"/>
       <c r="Y11" s="3"/>
       <c r="Z11" s="3"/>
@@ -1712,30 +1711,49 @@
       <c r="AG11" s="3"/>
       <c r="AH11" s="3"/>
     </row>
-    <row r="12" spans="1:34">
-      <c r="A12" s="3"/>
-      <c r="B12" s="4"/>
-      <c r="C12" s="4"/>
-      <c r="D12" s="4"/>
-      <c r="E12" s="4"/>
-      <c r="F12" s="4"/>
-      <c r="G12" s="4"/>
-      <c r="H12" s="4"/>
-      <c r="I12" s="4"/>
-      <c r="J12" s="4"/>
-      <c r="K12" s="4"/>
-      <c r="L12" s="4"/>
-      <c r="M12" s="4"/>
-      <c r="N12" s="4"/>
-      <c r="O12" s="4"/>
-      <c r="P12" s="4"/>
-      <c r="Q12" s="4"/>
-      <c r="R12" s="4"/>
-      <c r="S12" s="4"/>
-      <c r="T12" s="3"/>
-      <c r="U12" s="3"/>
-      <c r="V12" s="3"/>
-      <c r="W12" s="3"/>
+    <row r="12" spans="2:34">
+      <c r="B12" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="F12" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="G12" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="H12" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="I12" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="J12" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="K12" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="L12" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="M12" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="N12" s="2"/>
+      <c r="O12" s="2"/>
+      <c r="P12" s="2"/>
+      <c r="Q12" s="2"/>
+      <c r="R12" s="2"/>
+      <c r="S12" s="2"/>
       <c r="X12" s="3"/>
       <c r="Y12" s="3"/>
       <c r="Z12" s="3"/>
@@ -1748,7 +1766,7 @@
       <c r="AG12" s="3"/>
       <c r="AH12" s="3"/>
     </row>
-    <row r="13" s="1" customFormat="1" spans="1:34">
+    <row r="13" spans="1:34">
       <c r="A13" s="3"/>
       <c r="B13" s="4"/>
       <c r="C13" s="4"/>
@@ -1820,7 +1838,7 @@
       <c r="AG14" s="3"/>
       <c r="AH14" s="3"/>
     </row>
-    <row r="15" spans="1:34">
+    <row r="15" s="1" customFormat="1" spans="1:34">
       <c r="A15" s="3"/>
       <c r="B15" s="4"/>
       <c r="C15" s="4"/>
@@ -2365,7 +2383,7 @@
       <c r="B30" s="4"/>
       <c r="C30" s="4"/>
       <c r="D30" s="4"/>
-      <c r="E30" s="5"/>
+      <c r="E30" s="4"/>
       <c r="F30" s="4"/>
       <c r="G30" s="4"/>
       <c r="H30" s="4"/>
@@ -2473,7 +2491,7 @@
       <c r="B33" s="4"/>
       <c r="C33" s="4"/>
       <c r="D33" s="4"/>
-      <c r="E33" s="4"/>
+      <c r="E33" s="5"/>
       <c r="F33" s="4"/>
       <c r="G33" s="4"/>
       <c r="H33" s="4"/>
@@ -2617,7 +2635,7 @@
       <c r="B37" s="4"/>
       <c r="C37" s="4"/>
       <c r="D37" s="4"/>
-      <c r="E37" s="5"/>
+      <c r="E37" s="4"/>
       <c r="F37" s="4"/>
       <c r="G37" s="4"/>
       <c r="H37" s="4"/>
@@ -2653,7 +2671,7 @@
       <c r="B38" s="4"/>
       <c r="C38" s="4"/>
       <c r="D38" s="4"/>
-      <c r="E38" s="4"/>
+      <c r="E38" s="5"/>
       <c r="F38" s="4"/>
       <c r="G38" s="4"/>
       <c r="H38" s="4"/>
@@ -2936,25 +2954,48 @@
       <c r="AG45" s="3"/>
       <c r="AH45" s="3"/>
     </row>
-    <row r="53" spans="1:23">
-      <c r="A53" s="2"/>
-      <c r="B53" s="2"/>
-      <c r="C53" s="2"/>
-      <c r="D53" s="2"/>
-      <c r="R53" s="2"/>
-      <c r="T53" s="2"/>
-      <c r="U53" s="2"/>
-      <c r="V53" s="2"/>
-      <c r="W53" s="2"/>
+    <row r="46" spans="1:34">
+      <c r="A46" s="3"/>
+      <c r="B46" s="4"/>
+      <c r="C46" s="4"/>
+      <c r="D46" s="4"/>
+      <c r="E46" s="4"/>
+      <c r="F46" s="4"/>
+      <c r="G46" s="4"/>
+      <c r="H46" s="4"/>
+      <c r="I46" s="4"/>
+      <c r="J46" s="4"/>
+      <c r="K46" s="4"/>
+      <c r="L46" s="4"/>
+      <c r="M46" s="4"/>
+      <c r="N46" s="4"/>
+      <c r="O46" s="4"/>
+      <c r="P46" s="4"/>
+      <c r="Q46" s="4"/>
+      <c r="R46" s="4"/>
+      <c r="S46" s="4"/>
+      <c r="T46" s="3"/>
+      <c r="U46" s="3"/>
+      <c r="V46" s="3"/>
+      <c r="W46" s="3"/>
+      <c r="X46" s="3"/>
+      <c r="Y46" s="3"/>
+      <c r="Z46" s="3"/>
+      <c r="AA46" s="3"/>
+      <c r="AB46" s="3"/>
+      <c r="AC46" s="3"/>
+      <c r="AD46" s="3"/>
+      <c r="AE46" s="3"/>
+      <c r="AF46" s="3"/>
+      <c r="AG46" s="3"/>
+      <c r="AH46" s="3"/>
     </row>
     <row r="54" spans="1:23">
       <c r="A54" s="2"/>
       <c r="B54" s="2"/>
       <c r="C54" s="2"/>
       <c r="D54" s="2"/>
-      <c r="E54" s="2"/>
       <c r="R54" s="2"/>
-      <c r="S54" s="2"/>
       <c r="T54" s="2"/>
       <c r="U54" s="2"/>
       <c r="V54" s="2"/>
@@ -2965,6 +3006,7 @@
       <c r="B55" s="2"/>
       <c r="C55" s="2"/>
       <c r="D55" s="2"/>
+      <c r="E55" s="2"/>
       <c r="R55" s="2"/>
       <c r="S55" s="2"/>
       <c r="T55" s="2"/>
@@ -3104,39 +3146,51 @@
       <c r="V66" s="2"/>
       <c r="W66" s="2"/>
     </row>
+    <row r="67" spans="1:23">
+      <c r="A67" s="2"/>
+      <c r="B67" s="2"/>
+      <c r="C67" s="2"/>
+      <c r="D67" s="2"/>
+      <c r="R67" s="2"/>
+      <c r="S67" s="2"/>
+      <c r="T67" s="2"/>
+      <c r="U67" s="2"/>
+      <c r="V67" s="2"/>
+      <c r="W67" s="2"/>
+    </row>
   </sheetData>
   <dataValidations count="11">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L10 L2:L9 L11:L1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L10 L11 L2:L9 L12:L1048576">
       <formula1>"BR_EQ,BR_NE,BR_LTU,BR_GE,BR_GEU,BR_LT,BR_XX"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J5 J8 J9 J10 J2:J4 J6:J7 J11:J1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J5 J8 J9 J10 J11 J2:J4 J6:J7 J12:J1048576">
       <formula1>"ST_SW,ST_SH,ST_SB,ST_XX"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K4 K5 K6 K7 K8 K9 K10 K2:K3 K11:K1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K4 K5 K6 K7 K8 K9 K10 K11 K2:K3 K12:K1048576">
       <formula1>"MASK_XX,MASK_B,MASK_H,MASK_W,MASK_D"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="M4 M5 M6 M7 M8 M9 M10 M2:M3 M11:M1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="M4 M5 M6 M7 M8 M9 M10 M11 M2:M3 M12:M1048576">
       <formula1>"INST_VALID,INST_INVALID"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I4 I5 I6 I7 I8 I9 I10 I2:I3 I11:I1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I4 I5 I6 I7 I8 I9 I10 I11 I2:I3 I12:I1048576">
       <formula1>"LD_LB,LD_LH,LD_LW,LD_LBU,LD_LHU,LD_XX"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G4 G5 G6 G7 G8 G9 G10 G2:G3 G11:G1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G4 G5 G6 G7 G8 G9 G10 G11 G2:G3 G12:G1048576">
       <formula1>"IMM_I,IMM_J,IMM_U,IMM_S,IMM_B"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F4 F5 F6 F7 F8 F9 F10 F2:F3 F11:F1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F4 F5 F6 F7 F8 F9 F10 F11 F2:F3 F12:F1048576">
       <formula1>"ALU_ADD,ALU_SUB,ALU_AND,ALU_OR,ALU_XOR,ALU_SLL,ALU_SRL,ALU_SLT,ALU_SLTU,ALU_COPY_A,ALU_COPY_B"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H5 H9 H10 H2:H4 H6:H8 H11:H1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H5 H9 H10 H11 H2:H4 H6:H8 H12:H1048576">
       <formula1>"WB_ALU,WB_MEM,WB_PC4,WB_XX"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D4 D5 D6 D7 D8 D9 D10 D2:D3 D11:D1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D4 D5 D6 D7 D8 D9 D10 D11 D2:D3 D12:D1048576">
       <formula1>"A_PC,A_RS1"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E4 E5 E6 E7 E8 E9 E10 E2:E3 E11:E1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E4 E5 E6 E7 E8 E9 E10 E11 E2:E3 E12:E1048576">
       <formula1>"B_IMM,B_RS2"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C4 C5 C6 C7 C8 C9 C10 C2:C3 C11:C1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C4 C5 C6 C7 C8 C9 C10 C11 C2:C3 C12:C1048576">
       <formula1>"PC_4,PC_0,PC_ALU"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
> sim RTL ysyx_23060246 韩炳晋 Linux archlinux 6.6.60-1-lts #1 SMP PREEMPT_DYNAMIC Fri, 08 Nov 2024 16:03:02 +0000 x86_64 GNU/Linux  18:34:02 up 1 day, 49 min,  2 users,  load average: 5.88, 5.13, 4.12
</commit_message>
<xml_diff>
--- a/npc/tools/control_gen/control_table.xlsx
+++ b/npc/tools/control_gen/control_table.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="97" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="53">
   <si>
     <t>commont</t>
   </si>
@@ -146,6 +146,12 @@
   </si>
   <si>
     <t>B_RS2</t>
+  </si>
+  <si>
+    <t>sub</t>
+  </si>
+  <si>
+    <t>ALU_SUB</t>
   </si>
   <si>
     <t>default</t>
@@ -1135,7 +1141,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:AH67"/>
+  <dimension ref="A1:AH68"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
     <col min="1" max="1" width="13.1" customWidth="1"/>
@@ -1711,49 +1717,42 @@
       <c r="AG11" s="3"/>
       <c r="AH11" s="3"/>
     </row>
-    <row r="12" spans="2:34">
-      <c r="B12" s="2" t="s">
+    <row r="12" spans="1:34">
+      <c r="A12" s="3"/>
+      <c r="B12" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="C12" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="D12" s="2" t="s">
+      <c r="C12" s="2"/>
+      <c r="D12" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="E12" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="F12" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="G12" s="2" t="s">
-        <v>24</v>
-      </c>
+      <c r="E12" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="F12" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="G12" s="4"/>
       <c r="H12" s="4" t="s">
-        <v>45</v>
-      </c>
-      <c r="I12" s="4" t="s">
-        <v>46</v>
-      </c>
-      <c r="J12" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="K12" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="L12" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="M12" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="N12" s="2"/>
-      <c r="O12" s="2"/>
-      <c r="P12" s="2"/>
-      <c r="Q12" s="2"/>
-      <c r="R12" s="2"/>
-      <c r="S12" s="2"/>
+        <v>17</v>
+      </c>
+      <c r="I12" s="4"/>
+      <c r="J12" s="4"/>
+      <c r="K12" s="4"/>
+      <c r="L12" s="4"/>
+      <c r="M12" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="N12" s="4"/>
+      <c r="O12" s="4"/>
+      <c r="P12" s="4"/>
+      <c r="Q12" s="4"/>
+      <c r="R12" s="4"/>
+      <c r="S12" s="4"/>
+      <c r="T12" s="3"/>
+      <c r="U12" s="3"/>
+      <c r="V12" s="3"/>
+      <c r="W12" s="3"/>
       <c r="X12" s="3"/>
       <c r="Y12" s="3"/>
       <c r="Z12" s="3"/>
@@ -1766,30 +1765,49 @@
       <c r="AG12" s="3"/>
       <c r="AH12" s="3"/>
     </row>
-    <row r="13" spans="1:34">
-      <c r="A13" s="3"/>
-      <c r="B13" s="4"/>
-      <c r="C13" s="4"/>
-      <c r="D13" s="4"/>
-      <c r="E13" s="4"/>
-      <c r="F13" s="4"/>
-      <c r="G13" s="4"/>
-      <c r="H13" s="4"/>
-      <c r="I13" s="4"/>
-      <c r="J13" s="4"/>
-      <c r="K13" s="4"/>
-      <c r="L13" s="4"/>
-      <c r="M13" s="4"/>
-      <c r="N13" s="4"/>
-      <c r="O13" s="4"/>
-      <c r="P13" s="4"/>
-      <c r="Q13" s="4"/>
-      <c r="R13" s="4"/>
-      <c r="S13" s="4"/>
-      <c r="T13" s="3"/>
-      <c r="U13" s="3"/>
-      <c r="V13" s="3"/>
-      <c r="W13" s="3"/>
+    <row r="13" spans="2:34">
+      <c r="B13" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="E13" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="F13" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="G13" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="H13" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="I13" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="J13" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="K13" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="L13" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="M13" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="N13" s="2"/>
+      <c r="O13" s="2"/>
+      <c r="P13" s="2"/>
+      <c r="Q13" s="2"/>
+      <c r="R13" s="2"/>
+      <c r="S13" s="2"/>
       <c r="X13" s="3"/>
       <c r="Y13" s="3"/>
       <c r="Z13" s="3"/>
@@ -1802,7 +1820,7 @@
       <c r="AG13" s="3"/>
       <c r="AH13" s="3"/>
     </row>
-    <row r="14" s="1" customFormat="1" spans="1:34">
+    <row r="14" spans="1:34">
       <c r="A14" s="3"/>
       <c r="B14" s="4"/>
       <c r="C14" s="4"/>
@@ -1874,7 +1892,7 @@
       <c r="AG15" s="3"/>
       <c r="AH15" s="3"/>
     </row>
-    <row r="16" spans="1:34">
+    <row r="16" s="1" customFormat="1" spans="1:34">
       <c r="A16" s="3"/>
       <c r="B16" s="4"/>
       <c r="C16" s="4"/>
@@ -2419,7 +2437,7 @@
       <c r="B31" s="4"/>
       <c r="C31" s="4"/>
       <c r="D31" s="4"/>
-      <c r="E31" s="5"/>
+      <c r="E31" s="4"/>
       <c r="F31" s="4"/>
       <c r="G31" s="4"/>
       <c r="H31" s="4"/>
@@ -2527,7 +2545,7 @@
       <c r="B34" s="4"/>
       <c r="C34" s="4"/>
       <c r="D34" s="4"/>
-      <c r="E34" s="4"/>
+      <c r="E34" s="5"/>
       <c r="F34" s="4"/>
       <c r="G34" s="4"/>
       <c r="H34" s="4"/>
@@ -2671,7 +2689,7 @@
       <c r="B38" s="4"/>
       <c r="C38" s="4"/>
       <c r="D38" s="4"/>
-      <c r="E38" s="5"/>
+      <c r="E38" s="4"/>
       <c r="F38" s="4"/>
       <c r="G38" s="4"/>
       <c r="H38" s="4"/>
@@ -2707,7 +2725,7 @@
       <c r="B39" s="4"/>
       <c r="C39" s="4"/>
       <c r="D39" s="4"/>
-      <c r="E39" s="4"/>
+      <c r="E39" s="5"/>
       <c r="F39" s="4"/>
       <c r="G39" s="4"/>
       <c r="H39" s="4"/>
@@ -2990,25 +3008,48 @@
       <c r="AG46" s="3"/>
       <c r="AH46" s="3"/>
     </row>
-    <row r="54" spans="1:23">
-      <c r="A54" s="2"/>
-      <c r="B54" s="2"/>
-      <c r="C54" s="2"/>
-      <c r="D54" s="2"/>
-      <c r="R54" s="2"/>
-      <c r="T54" s="2"/>
-      <c r="U54" s="2"/>
-      <c r="V54" s="2"/>
-      <c r="W54" s="2"/>
+    <row r="47" spans="1:34">
+      <c r="A47" s="3"/>
+      <c r="B47" s="4"/>
+      <c r="C47" s="4"/>
+      <c r="D47" s="4"/>
+      <c r="E47" s="4"/>
+      <c r="F47" s="4"/>
+      <c r="G47" s="4"/>
+      <c r="H47" s="4"/>
+      <c r="I47" s="4"/>
+      <c r="J47" s="4"/>
+      <c r="K47" s="4"/>
+      <c r="L47" s="4"/>
+      <c r="M47" s="4"/>
+      <c r="N47" s="4"/>
+      <c r="O47" s="4"/>
+      <c r="P47" s="4"/>
+      <c r="Q47" s="4"/>
+      <c r="R47" s="4"/>
+      <c r="S47" s="4"/>
+      <c r="T47" s="3"/>
+      <c r="U47" s="3"/>
+      <c r="V47" s="3"/>
+      <c r="W47" s="3"/>
+      <c r="X47" s="3"/>
+      <c r="Y47" s="3"/>
+      <c r="Z47" s="3"/>
+      <c r="AA47" s="3"/>
+      <c r="AB47" s="3"/>
+      <c r="AC47" s="3"/>
+      <c r="AD47" s="3"/>
+      <c r="AE47" s="3"/>
+      <c r="AF47" s="3"/>
+      <c r="AG47" s="3"/>
+      <c r="AH47" s="3"/>
     </row>
     <row r="55" spans="1:23">
       <c r="A55" s="2"/>
       <c r="B55" s="2"/>
       <c r="C55" s="2"/>
       <c r="D55" s="2"/>
-      <c r="E55" s="2"/>
       <c r="R55" s="2"/>
-      <c r="S55" s="2"/>
       <c r="T55" s="2"/>
       <c r="U55" s="2"/>
       <c r="V55" s="2"/>
@@ -3019,6 +3060,7 @@
       <c r="B56" s="2"/>
       <c r="C56" s="2"/>
       <c r="D56" s="2"/>
+      <c r="E56" s="2"/>
       <c r="R56" s="2"/>
       <c r="S56" s="2"/>
       <c r="T56" s="2"/>
@@ -3158,39 +3200,51 @@
       <c r="V67" s="2"/>
       <c r="W67" s="2"/>
     </row>
+    <row r="68" spans="1:23">
+      <c r="A68" s="2"/>
+      <c r="B68" s="2"/>
+      <c r="C68" s="2"/>
+      <c r="D68" s="2"/>
+      <c r="R68" s="2"/>
+      <c r="S68" s="2"/>
+      <c r="T68" s="2"/>
+      <c r="U68" s="2"/>
+      <c r="V68" s="2"/>
+      <c r="W68" s="2"/>
+    </row>
   </sheetData>
   <dataValidations count="11">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L10 L11 L2:L9 L12:L1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L10 L11 L12 L2:L9 L13:L1048576">
       <formula1>"BR_EQ,BR_NE,BR_LTU,BR_GE,BR_GEU,BR_LT,BR_XX"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J5 J8 J9 J10 J11 J2:J4 J6:J7 J12:J1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J5 J8 J9 J10 J11 J12 J2:J4 J6:J7 J13:J1048576">
       <formula1>"ST_SW,ST_SH,ST_SB,ST_XX"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K4 K5 K6 K7 K8 K9 K10 K11 K2:K3 K12:K1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K4 K5 K6 K7 K8 K9 K10 K11 K12 K2:K3 K13:K1048576">
       <formula1>"MASK_XX,MASK_B,MASK_H,MASK_W,MASK_D"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="M4 M5 M6 M7 M8 M9 M10 M11 M2:M3 M12:M1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="M4 M5 M6 M7 M8 M9 M10 M11 M12 M2:M3 M13:M1048576">
       <formula1>"INST_VALID,INST_INVALID"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I4 I5 I6 I7 I8 I9 I10 I11 I2:I3 I12:I1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I4 I5 I6 I7 I8 I9 I10 I11 I12 I2:I3 I13:I1048576">
       <formula1>"LD_LB,LD_LH,LD_LW,LD_LBU,LD_LHU,LD_XX"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G4 G5 G6 G7 G8 G9 G10 G11 G2:G3 G12:G1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G4 G5 G6 G7 G8 G9 G10 G11 G12 G2:G3 G13:G1048576">
       <formula1>"IMM_I,IMM_J,IMM_U,IMM_S,IMM_B"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F4 F5 F6 F7 F8 F9 F10 F11 F2:F3 F12:F1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F4 F5 F6 F7 F8 F9 F10 F11 F12 F2:F3 F13:F1048576">
       <formula1>"ALU_ADD,ALU_SUB,ALU_AND,ALU_OR,ALU_XOR,ALU_SLL,ALU_SRL,ALU_SLT,ALU_SLTU,ALU_COPY_A,ALU_COPY_B"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H5 H9 H10 H11 H2:H4 H6:H8 H12:H1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H5 H9 H10 H11 H12 H2:H4 H6:H8 H13:H1048576">
       <formula1>"WB_ALU,WB_MEM,WB_PC4,WB_XX"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D4 D5 D6 D7 D8 D9 D10 D11 D2:D3 D12:D1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D4 D5 D6 D7 D8 D9 D10 D11 D12 D2:D3 D13:D1048576">
       <formula1>"A_PC,A_RS1"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E4 E5 E6 E7 E8 E9 E10 E11 E2:E3 E12:E1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E4 E5 E6 E7 E8 E9 E10 E11 E12 E2:E3 E13:E1048576">
       <formula1>"B_IMM,B_RS2"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C4 C5 C6 C7 C8 C9 C10 C11 C2:C3 C12:C1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C4 C5 C6 C7 C8 C9 C10 C11 C12 C2:C3 C13:C1048576">
       <formula1>"PC_4,PC_0,PC_ALU"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
> sim RTL ysyx_23060246 韩炳晋 Linux archlinux 6.6.60-1-lts #1 SMP PREEMPT_DYNAMIC Fri, 08 Nov 2024 16:03:02 +0000 x86_64 GNU/Linux  18:36:47 up 1 day, 51 min,  2 users,  load average: 4.39, 4.48, 4.01
</commit_message>
<xml_diff>
--- a/npc/tools/control_gen/control_table.xlsx
+++ b/npc/tools/control_gen/control_table.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="55">
   <si>
     <t>commont</t>
   </si>
@@ -140,6 +140,12 @@
   </si>
   <si>
     <t>ALU_SLL</t>
+  </si>
+  <si>
+    <t>sltiu</t>
+  </si>
+  <si>
+    <t>ALU_SLTU</t>
   </si>
   <si>
     <t>add</t>
@@ -1141,7 +1147,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:AH68"/>
+  <dimension ref="A1:AH69"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
     <col min="1" max="1" width="13.1" customWidth="1"/>
@@ -1679,12 +1685,14 @@
         <v>23</v>
       </c>
       <c r="E11" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="F11" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="F11" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="G11" s="4"/>
+      <c r="G11" s="4" t="s">
+        <v>24</v>
+      </c>
       <c r="H11" s="4" t="s">
         <v>17</v>
       </c>
@@ -1727,10 +1735,10 @@
         <v>23</v>
       </c>
       <c r="E12" s="4" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="F12" s="4" t="s">
-        <v>45</v>
+        <v>21</v>
       </c>
       <c r="G12" s="4"/>
       <c r="H12" s="4" t="s">
@@ -1765,49 +1773,42 @@
       <c r="AG12" s="3"/>
       <c r="AH12" s="3"/>
     </row>
-    <row r="13" spans="2:34">
-      <c r="B13" s="2" t="s">
+    <row r="13" spans="1:34">
+      <c r="A13" s="3"/>
+      <c r="B13" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="C13" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="D13" s="2" t="s">
+      <c r="C13" s="2"/>
+      <c r="D13" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="E13" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="F13" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="G13" s="2" t="s">
-        <v>24</v>
-      </c>
+      <c r="E13" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="F13" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="G13" s="4"/>
       <c r="H13" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="I13" s="4" t="s">
-        <v>48</v>
-      </c>
-      <c r="J13" s="4" t="s">
-        <v>49</v>
-      </c>
-      <c r="K13" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="L13" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="M13" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="N13" s="2"/>
-      <c r="O13" s="2"/>
-      <c r="P13" s="2"/>
-      <c r="Q13" s="2"/>
-      <c r="R13" s="2"/>
-      <c r="S13" s="2"/>
+        <v>17</v>
+      </c>
+      <c r="I13" s="4"/>
+      <c r="J13" s="4"/>
+      <c r="K13" s="4"/>
+      <c r="L13" s="4"/>
+      <c r="M13" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="N13" s="4"/>
+      <c r="O13" s="4"/>
+      <c r="P13" s="4"/>
+      <c r="Q13" s="4"/>
+      <c r="R13" s="4"/>
+      <c r="S13" s="4"/>
+      <c r="T13" s="3"/>
+      <c r="U13" s="3"/>
+      <c r="V13" s="3"/>
+      <c r="W13" s="3"/>
       <c r="X13" s="3"/>
       <c r="Y13" s="3"/>
       <c r="Z13" s="3"/>
@@ -1820,30 +1821,49 @@
       <c r="AG13" s="3"/>
       <c r="AH13" s="3"/>
     </row>
-    <row r="14" spans="1:34">
-      <c r="A14" s="3"/>
-      <c r="B14" s="4"/>
-      <c r="C14" s="4"/>
-      <c r="D14" s="4"/>
-      <c r="E14" s="4"/>
-      <c r="F14" s="4"/>
-      <c r="G14" s="4"/>
-      <c r="H14" s="4"/>
-      <c r="I14" s="4"/>
-      <c r="J14" s="4"/>
-      <c r="K14" s="4"/>
-      <c r="L14" s="4"/>
-      <c r="M14" s="4"/>
-      <c r="N14" s="4"/>
-      <c r="O14" s="4"/>
-      <c r="P14" s="4"/>
-      <c r="Q14" s="4"/>
-      <c r="R14" s="4"/>
-      <c r="S14" s="4"/>
-      <c r="T14" s="3"/>
-      <c r="U14" s="3"/>
-      <c r="V14" s="3"/>
-      <c r="W14" s="3"/>
+    <row r="14" spans="2:34">
+      <c r="B14" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="F14" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="G14" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="H14" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="I14" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="J14" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="K14" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="L14" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="M14" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="N14" s="2"/>
+      <c r="O14" s="2"/>
+      <c r="P14" s="2"/>
+      <c r="Q14" s="2"/>
+      <c r="R14" s="2"/>
+      <c r="S14" s="2"/>
       <c r="X14" s="3"/>
       <c r="Y14" s="3"/>
       <c r="Z14" s="3"/>
@@ -1856,7 +1876,7 @@
       <c r="AG14" s="3"/>
       <c r="AH14" s="3"/>
     </row>
-    <row r="15" s="1" customFormat="1" spans="1:34">
+    <row r="15" spans="1:34">
       <c r="A15" s="3"/>
       <c r="B15" s="4"/>
       <c r="C15" s="4"/>
@@ -1928,7 +1948,7 @@
       <c r="AG16" s="3"/>
       <c r="AH16" s="3"/>
     </row>
-    <row r="17" spans="1:34">
+    <row r="17" s="1" customFormat="1" spans="1:34">
       <c r="A17" s="3"/>
       <c r="B17" s="4"/>
       <c r="C17" s="4"/>
@@ -2473,7 +2493,7 @@
       <c r="B32" s="4"/>
       <c r="C32" s="4"/>
       <c r="D32" s="4"/>
-      <c r="E32" s="5"/>
+      <c r="E32" s="4"/>
       <c r="F32" s="4"/>
       <c r="G32" s="4"/>
       <c r="H32" s="4"/>
@@ -2581,7 +2601,7 @@
       <c r="B35" s="4"/>
       <c r="C35" s="4"/>
       <c r="D35" s="4"/>
-      <c r="E35" s="4"/>
+      <c r="E35" s="5"/>
       <c r="F35" s="4"/>
       <c r="G35" s="4"/>
       <c r="H35" s="4"/>
@@ -2725,7 +2745,7 @@
       <c r="B39" s="4"/>
       <c r="C39" s="4"/>
       <c r="D39" s="4"/>
-      <c r="E39" s="5"/>
+      <c r="E39" s="4"/>
       <c r="F39" s="4"/>
       <c r="G39" s="4"/>
       <c r="H39" s="4"/>
@@ -2761,7 +2781,7 @@
       <c r="B40" s="4"/>
       <c r="C40" s="4"/>
       <c r="D40" s="4"/>
-      <c r="E40" s="4"/>
+      <c r="E40" s="5"/>
       <c r="F40" s="4"/>
       <c r="G40" s="4"/>
       <c r="H40" s="4"/>
@@ -3044,25 +3064,48 @@
       <c r="AG47" s="3"/>
       <c r="AH47" s="3"/>
     </row>
-    <row r="55" spans="1:23">
-      <c r="A55" s="2"/>
-      <c r="B55" s="2"/>
-      <c r="C55" s="2"/>
-      <c r="D55" s="2"/>
-      <c r="R55" s="2"/>
-      <c r="T55" s="2"/>
-      <c r="U55" s="2"/>
-      <c r="V55" s="2"/>
-      <c r="W55" s="2"/>
+    <row r="48" spans="1:34">
+      <c r="A48" s="3"/>
+      <c r="B48" s="4"/>
+      <c r="C48" s="4"/>
+      <c r="D48" s="4"/>
+      <c r="E48" s="4"/>
+      <c r="F48" s="4"/>
+      <c r="G48" s="4"/>
+      <c r="H48" s="4"/>
+      <c r="I48" s="4"/>
+      <c r="J48" s="4"/>
+      <c r="K48" s="4"/>
+      <c r="L48" s="4"/>
+      <c r="M48" s="4"/>
+      <c r="N48" s="4"/>
+      <c r="O48" s="4"/>
+      <c r="P48" s="4"/>
+      <c r="Q48" s="4"/>
+      <c r="R48" s="4"/>
+      <c r="S48" s="4"/>
+      <c r="T48" s="3"/>
+      <c r="U48" s="3"/>
+      <c r="V48" s="3"/>
+      <c r="W48" s="3"/>
+      <c r="X48" s="3"/>
+      <c r="Y48" s="3"/>
+      <c r="Z48" s="3"/>
+      <c r="AA48" s="3"/>
+      <c r="AB48" s="3"/>
+      <c r="AC48" s="3"/>
+      <c r="AD48" s="3"/>
+      <c r="AE48" s="3"/>
+      <c r="AF48" s="3"/>
+      <c r="AG48" s="3"/>
+      <c r="AH48" s="3"/>
     </row>
     <row r="56" spans="1:23">
       <c r="A56" s="2"/>
       <c r="B56" s="2"/>
       <c r="C56" s="2"/>
       <c r="D56" s="2"/>
-      <c r="E56" s="2"/>
       <c r="R56" s="2"/>
-      <c r="S56" s="2"/>
       <c r="T56" s="2"/>
       <c r="U56" s="2"/>
       <c r="V56" s="2"/>
@@ -3073,6 +3116,7 @@
       <c r="B57" s="2"/>
       <c r="C57" s="2"/>
       <c r="D57" s="2"/>
+      <c r="E57" s="2"/>
       <c r="R57" s="2"/>
       <c r="S57" s="2"/>
       <c r="T57" s="2"/>
@@ -3212,39 +3256,51 @@
       <c r="V68" s="2"/>
       <c r="W68" s="2"/>
     </row>
+    <row r="69" spans="1:23">
+      <c r="A69" s="2"/>
+      <c r="B69" s="2"/>
+      <c r="C69" s="2"/>
+      <c r="D69" s="2"/>
+      <c r="R69" s="2"/>
+      <c r="S69" s="2"/>
+      <c r="T69" s="2"/>
+      <c r="U69" s="2"/>
+      <c r="V69" s="2"/>
+      <c r="W69" s="2"/>
+    </row>
   </sheetData>
   <dataValidations count="11">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L10 L11 L12 L2:L9 L13:L1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L10 L11 L12 L13 L2:L9 L14:L1048576">
       <formula1>"BR_EQ,BR_NE,BR_LTU,BR_GE,BR_GEU,BR_LT,BR_XX"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J5 J8 J9 J10 J11 J12 J2:J4 J6:J7 J13:J1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J5 J8 J9 J10 J11 J12 J13 J2:J4 J6:J7 J14:J1048576">
       <formula1>"ST_SW,ST_SH,ST_SB,ST_XX"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K4 K5 K6 K7 K8 K9 K10 K11 K12 K2:K3 K13:K1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K4 K5 K6 K7 K8 K9 K10 K11 K12 K13 K2:K3 K14:K1048576">
       <formula1>"MASK_XX,MASK_B,MASK_H,MASK_W,MASK_D"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="M4 M5 M6 M7 M8 M9 M10 M11 M12 M2:M3 M13:M1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="M4 M5 M6 M7 M8 M9 M10 M11 M12 M13 M2:M3 M14:M1048576">
       <formula1>"INST_VALID,INST_INVALID"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I4 I5 I6 I7 I8 I9 I10 I11 I12 I2:I3 I13:I1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I4 I5 I6 I7 I8 I9 I10 I11 I12 I13 I2:I3 I14:I1048576">
       <formula1>"LD_LB,LD_LH,LD_LW,LD_LBU,LD_LHU,LD_XX"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G4 G5 G6 G7 G8 G9 G10 G11 G12 G2:G3 G13:G1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G4 G5 G6 G7 G8 G9 G10 G11 G12 G13 G2:G3 G14:G1048576">
       <formula1>"IMM_I,IMM_J,IMM_U,IMM_S,IMM_B"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F4 F5 F6 F7 F8 F9 F10 F11 F12 F2:F3 F13:F1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F4 F5 F6 F7 F8 F9 F10 F11 F12 F13 F2:F3 F14:F1048576">
       <formula1>"ALU_ADD,ALU_SUB,ALU_AND,ALU_OR,ALU_XOR,ALU_SLL,ALU_SRL,ALU_SLT,ALU_SLTU,ALU_COPY_A,ALU_COPY_B"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H5 H9 H10 H11 H12 H2:H4 H6:H8 H13:H1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H5 H9 H10 H11 H12 H13 H2:H4 H6:H8 H14:H1048576">
       <formula1>"WB_ALU,WB_MEM,WB_PC4,WB_XX"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D4 D5 D6 D7 D8 D9 D10 D11 D12 D2:D3 D13:D1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D4 D5 D6 D7 D8 D9 D10 D11 D12 D13 D2:D3 D14:D1048576">
       <formula1>"A_PC,A_RS1"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E4 E5 E6 E7 E8 E9 E10 E11 E12 E2:E3 E13:E1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E4 E5 E6 E7 E8 E9 E10 E11 E12 E13 E2:E3 E14:E1048576">
       <formula1>"B_IMM,B_RS2"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C4 C5 C6 C7 C8 C9 C10 C11 C12 C2:C3 C13:C1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C4 C5 C6 C7 C8 C9 C10 C11 C12 C13 C2:C3 C14:C1048576">
       <formula1>"PC_4,PC_0,PC_ALU"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
> sim RTL ysyx_23060246 韩炳晋 Linux archlinux 6.6.60-1-lts #1 SMP PREEMPT_DYNAMIC Fri, 08 Nov 2024 16:03:02 +0000 x86_64 GNU/Linux  18:38:18 up 1 day, 53 min,  2 users,  load average: 5.93, 4.71, 4.12
</commit_message>
<xml_diff>
--- a/npc/tools/control_gen/control_table.xlsx
+++ b/npc/tools/control_gen/control_table.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="118" uniqueCount="57">
   <si>
     <t>commont</t>
   </si>
@@ -89,6 +89,12 @@
   </si>
   <si>
     <t>IMM_I</t>
+  </si>
+  <si>
+    <t>andi</t>
+  </si>
+  <si>
+    <t>ALU_AND</t>
   </si>
   <si>
     <t>jalr</t>
@@ -1147,7 +1153,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:AH69"/>
+  <dimension ref="A1:AH70"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
     <col min="1" max="1" width="13.1" customWidth="1"/>
@@ -1372,9 +1378,7 @@
       <c r="B5" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="C5" s="2" t="s">
-        <v>26</v>
-      </c>
+      <c r="C5" s="2"/>
       <c r="D5" s="4" t="s">
         <v>23</v>
       </c>
@@ -1382,11 +1386,13 @@
         <v>14</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="G5" s="4"/>
+        <v>26</v>
+      </c>
+      <c r="G5" s="4" t="s">
+        <v>24</v>
+      </c>
       <c r="H5" s="4" t="s">
-        <v>27</v>
+        <v>17</v>
       </c>
       <c r="I5" s="4"/>
       <c r="J5" s="4"/>
@@ -1420,13 +1426,13 @@
     <row r="6" spans="1:34">
       <c r="A6" s="3"/>
       <c r="B6" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="C6" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="C6" s="2" t="s">
-        <v>26</v>
-      </c>
       <c r="D6" s="4" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="E6" s="4" t="s">
         <v>14</v>
@@ -1435,10 +1441,10 @@
         <v>21</v>
       </c>
       <c r="G6" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="H6" s="4" t="s">
         <v>29</v>
-      </c>
-      <c r="H6" s="4" t="s">
-        <v>27</v>
       </c>
       <c r="I6" s="4"/>
       <c r="J6" s="4"/>
@@ -1474,9 +1480,11 @@
       <c r="B7" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="C7" s="2"/>
+      <c r="C7" s="2" t="s">
+        <v>28</v>
+      </c>
       <c r="D7" s="4" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="E7" s="4" t="s">
         <v>14</v>
@@ -1487,14 +1495,12 @@
       <c r="G7" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="H7" s="4"/>
+      <c r="H7" s="4" t="s">
+        <v>29</v>
+      </c>
       <c r="I7" s="4"/>
-      <c r="J7" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="K7" s="4" t="s">
-        <v>33</v>
-      </c>
+      <c r="J7" s="4"/>
+      <c r="K7" s="4"/>
       <c r="L7" s="4"/>
       <c r="M7" s="4" t="s">
         <v>18</v>
@@ -1524,11 +1530,9 @@
     <row r="8" spans="1:34">
       <c r="A8" s="3"/>
       <c r="B8" s="4" t="s">
-        <v>34</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>35</v>
-      </c>
+        <v>32</v>
+      </c>
+      <c r="C8" s="2"/>
       <c r="D8" s="4" t="s">
         <v>23</v>
       </c>
@@ -1539,14 +1543,16 @@
         <v>21</v>
       </c>
       <c r="G8" s="4" t="s">
-        <v>24</v>
+        <v>33</v>
       </c>
       <c r="H8" s="4"/>
-      <c r="I8" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="J8" s="4"/>
-      <c r="K8" s="4"/>
+      <c r="I8" s="4"/>
+      <c r="J8" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="K8" s="4" t="s">
+        <v>35</v>
+      </c>
       <c r="L8" s="4"/>
       <c r="M8" s="4" t="s">
         <v>18</v>
@@ -1576,13 +1582,13 @@
     <row r="9" spans="1:34">
       <c r="A9" s="3"/>
       <c r="B9" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="C9" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="C9" s="2" t="s">
-        <v>26</v>
-      </c>
       <c r="D9" s="4" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="E9" s="4" t="s">
         <v>14</v>
@@ -1591,15 +1597,15 @@
         <v>21</v>
       </c>
       <c r="G9" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="H9" s="4"/>
+      <c r="I9" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="H9" s="4"/>
-      <c r="I9" s="4"/>
       <c r="J9" s="4"/>
       <c r="K9" s="4"/>
-      <c r="L9" s="4" t="s">
-        <v>39</v>
-      </c>
+      <c r="L9" s="4"/>
       <c r="M9" s="4" t="s">
         <v>18</v>
       </c>
@@ -1628,28 +1634,30 @@
     <row r="10" spans="1:34">
       <c r="A10" s="3"/>
       <c r="B10" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="C10" s="2"/>
+        <v>39</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>28</v>
+      </c>
       <c r="D10" s="4" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="E10" s="4" t="s">
         <v>14</v>
       </c>
       <c r="F10" s="4" t="s">
-        <v>41</v>
+        <v>21</v>
       </c>
       <c r="G10" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="H10" s="4" t="s">
-        <v>17</v>
-      </c>
+        <v>40</v>
+      </c>
+      <c r="H10" s="4"/>
       <c r="I10" s="4"/>
       <c r="J10" s="4"/>
       <c r="K10" s="4"/>
-      <c r="L10" s="4"/>
+      <c r="L10" s="4" t="s">
+        <v>41</v>
+      </c>
       <c r="M10" s="4" t="s">
         <v>18</v>
       </c>
@@ -1735,12 +1743,14 @@
         <v>23</v>
       </c>
       <c r="E12" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="F12" s="4" t="s">
         <v>45</v>
       </c>
-      <c r="F12" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="G12" s="4"/>
+      <c r="G12" s="4" t="s">
+        <v>24</v>
+      </c>
       <c r="H12" s="4" t="s">
         <v>17</v>
       </c>
@@ -1783,10 +1793,10 @@
         <v>23</v>
       </c>
       <c r="E13" s="4" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="F13" s="4" t="s">
-        <v>47</v>
+        <v>21</v>
       </c>
       <c r="G13" s="4"/>
       <c r="H13" s="4" t="s">
@@ -1821,49 +1831,42 @@
       <c r="AG13" s="3"/>
       <c r="AH13" s="3"/>
     </row>
-    <row r="14" spans="2:34">
-      <c r="B14" s="2" t="s">
+    <row r="14" spans="1:34">
+      <c r="A14" s="3"/>
+      <c r="B14" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="C14" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="D14" s="2" t="s">
+      <c r="C14" s="2"/>
+      <c r="D14" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="E14" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="F14" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="G14" s="2" t="s">
-        <v>24</v>
-      </c>
+      <c r="E14" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="F14" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="G14" s="4"/>
       <c r="H14" s="4" t="s">
-        <v>49</v>
-      </c>
-      <c r="I14" s="4" t="s">
-        <v>50</v>
-      </c>
-      <c r="J14" s="4" t="s">
-        <v>51</v>
-      </c>
-      <c r="K14" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="L14" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="M14" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="N14" s="2"/>
-      <c r="O14" s="2"/>
-      <c r="P14" s="2"/>
-      <c r="Q14" s="2"/>
-      <c r="R14" s="2"/>
-      <c r="S14" s="2"/>
+        <v>17</v>
+      </c>
+      <c r="I14" s="4"/>
+      <c r="J14" s="4"/>
+      <c r="K14" s="4"/>
+      <c r="L14" s="4"/>
+      <c r="M14" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="N14" s="4"/>
+      <c r="O14" s="4"/>
+      <c r="P14" s="4"/>
+      <c r="Q14" s="4"/>
+      <c r="R14" s="4"/>
+      <c r="S14" s="4"/>
+      <c r="T14" s="3"/>
+      <c r="U14" s="3"/>
+      <c r="V14" s="3"/>
+      <c r="W14" s="3"/>
       <c r="X14" s="3"/>
       <c r="Y14" s="3"/>
       <c r="Z14" s="3"/>
@@ -1876,30 +1879,49 @@
       <c r="AG14" s="3"/>
       <c r="AH14" s="3"/>
     </row>
-    <row r="15" spans="1:34">
-      <c r="A15" s="3"/>
-      <c r="B15" s="4"/>
-      <c r="C15" s="4"/>
-      <c r="D15" s="4"/>
-      <c r="E15" s="4"/>
-      <c r="F15" s="4"/>
-      <c r="G15" s="4"/>
-      <c r="H15" s="4"/>
-      <c r="I15" s="4"/>
-      <c r="J15" s="4"/>
-      <c r="K15" s="4"/>
-      <c r="L15" s="4"/>
-      <c r="M15" s="4"/>
-      <c r="N15" s="4"/>
-      <c r="O15" s="4"/>
-      <c r="P15" s="4"/>
-      <c r="Q15" s="4"/>
-      <c r="R15" s="4"/>
-      <c r="S15" s="4"/>
-      <c r="T15" s="3"/>
-      <c r="U15" s="3"/>
-      <c r="V15" s="3"/>
-      <c r="W15" s="3"/>
+    <row r="15" spans="2:34">
+      <c r="B15" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="E15" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="F15" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="G15" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="H15" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="I15" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="J15" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="K15" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="L15" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="M15" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="N15" s="2"/>
+      <c r="O15" s="2"/>
+      <c r="P15" s="2"/>
+      <c r="Q15" s="2"/>
+      <c r="R15" s="2"/>
+      <c r="S15" s="2"/>
       <c r="X15" s="3"/>
       <c r="Y15" s="3"/>
       <c r="Z15" s="3"/>
@@ -1912,7 +1934,7 @@
       <c r="AG15" s="3"/>
       <c r="AH15" s="3"/>
     </row>
-    <row r="16" s="1" customFormat="1" spans="1:34">
+    <row r="16" spans="1:34">
       <c r="A16" s="3"/>
       <c r="B16" s="4"/>
       <c r="C16" s="4"/>
@@ -1984,7 +2006,7 @@
       <c r="AG17" s="3"/>
       <c r="AH17" s="3"/>
     </row>
-    <row r="18" spans="1:34">
+    <row r="18" s="1" customFormat="1" spans="1:34">
       <c r="A18" s="3"/>
       <c r="B18" s="4"/>
       <c r="C18" s="4"/>
@@ -2529,7 +2551,7 @@
       <c r="B33" s="4"/>
       <c r="C33" s="4"/>
       <c r="D33" s="4"/>
-      <c r="E33" s="5"/>
+      <c r="E33" s="4"/>
       <c r="F33" s="4"/>
       <c r="G33" s="4"/>
       <c r="H33" s="4"/>
@@ -2637,7 +2659,7 @@
       <c r="B36" s="4"/>
       <c r="C36" s="4"/>
       <c r="D36" s="4"/>
-      <c r="E36" s="4"/>
+      <c r="E36" s="5"/>
       <c r="F36" s="4"/>
       <c r="G36" s="4"/>
       <c r="H36" s="4"/>
@@ -2781,7 +2803,7 @@
       <c r="B40" s="4"/>
       <c r="C40" s="4"/>
       <c r="D40" s="4"/>
-      <c r="E40" s="5"/>
+      <c r="E40" s="4"/>
       <c r="F40" s="4"/>
       <c r="G40" s="4"/>
       <c r="H40" s="4"/>
@@ -2817,7 +2839,7 @@
       <c r="B41" s="4"/>
       <c r="C41" s="4"/>
       <c r="D41" s="4"/>
-      <c r="E41" s="4"/>
+      <c r="E41" s="5"/>
       <c r="F41" s="4"/>
       <c r="G41" s="4"/>
       <c r="H41" s="4"/>
@@ -3100,25 +3122,48 @@
       <c r="AG48" s="3"/>
       <c r="AH48" s="3"/>
     </row>
-    <row r="56" spans="1:23">
-      <c r="A56" s="2"/>
-      <c r="B56" s="2"/>
-      <c r="C56" s="2"/>
-      <c r="D56" s="2"/>
-      <c r="R56" s="2"/>
-      <c r="T56" s="2"/>
-      <c r="U56" s="2"/>
-      <c r="V56" s="2"/>
-      <c r="W56" s="2"/>
+    <row r="49" spans="1:34">
+      <c r="A49" s="3"/>
+      <c r="B49" s="4"/>
+      <c r="C49" s="4"/>
+      <c r="D49" s="4"/>
+      <c r="E49" s="4"/>
+      <c r="F49" s="4"/>
+      <c r="G49" s="4"/>
+      <c r="H49" s="4"/>
+      <c r="I49" s="4"/>
+      <c r="J49" s="4"/>
+      <c r="K49" s="4"/>
+      <c r="L49" s="4"/>
+      <c r="M49" s="4"/>
+      <c r="N49" s="4"/>
+      <c r="O49" s="4"/>
+      <c r="P49" s="4"/>
+      <c r="Q49" s="4"/>
+      <c r="R49" s="4"/>
+      <c r="S49" s="4"/>
+      <c r="T49" s="3"/>
+      <c r="U49" s="3"/>
+      <c r="V49" s="3"/>
+      <c r="W49" s="3"/>
+      <c r="X49" s="3"/>
+      <c r="Y49" s="3"/>
+      <c r="Z49" s="3"/>
+      <c r="AA49" s="3"/>
+      <c r="AB49" s="3"/>
+      <c r="AC49" s="3"/>
+      <c r="AD49" s="3"/>
+      <c r="AE49" s="3"/>
+      <c r="AF49" s="3"/>
+      <c r="AG49" s="3"/>
+      <c r="AH49" s="3"/>
     </row>
     <row r="57" spans="1:23">
       <c r="A57" s="2"/>
       <c r="B57" s="2"/>
       <c r="C57" s="2"/>
       <c r="D57" s="2"/>
-      <c r="E57" s="2"/>
       <c r="R57" s="2"/>
-      <c r="S57" s="2"/>
       <c r="T57" s="2"/>
       <c r="U57" s="2"/>
       <c r="V57" s="2"/>
@@ -3129,6 +3174,7 @@
       <c r="B58" s="2"/>
       <c r="C58" s="2"/>
       <c r="D58" s="2"/>
+      <c r="E58" s="2"/>
       <c r="R58" s="2"/>
       <c r="S58" s="2"/>
       <c r="T58" s="2"/>
@@ -3268,39 +3314,51 @@
       <c r="V69" s="2"/>
       <c r="W69" s="2"/>
     </row>
+    <row r="70" spans="1:23">
+      <c r="A70" s="2"/>
+      <c r="B70" s="2"/>
+      <c r="C70" s="2"/>
+      <c r="D70" s="2"/>
+      <c r="R70" s="2"/>
+      <c r="S70" s="2"/>
+      <c r="T70" s="2"/>
+      <c r="U70" s="2"/>
+      <c r="V70" s="2"/>
+      <c r="W70" s="2"/>
+    </row>
   </sheetData>
   <dataValidations count="11">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L10 L11 L12 L13 L2:L9 L14:L1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L5 L11 L12 L13 L14 L2:L4 L6:L10 L15:L1048576">
       <formula1>"BR_EQ,BR_NE,BR_LTU,BR_GE,BR_GEU,BR_LT,BR_XX"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J5 J8 J9 J10 J11 J12 J13 J2:J4 J6:J7 J14:J1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J5 J6 J9 J10 J11 J12 J13 J14 J2:J4 J7:J8 J15:J1048576">
       <formula1>"ST_SW,ST_SH,ST_SB,ST_XX"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K4 K5 K6 K7 K8 K9 K10 K11 K12 K13 K2:K3 K14:K1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K4 K5 K6 K7 K8 K9 K10 K11 K12 K13 K14 K2:K3 K15:K1048576">
       <formula1>"MASK_XX,MASK_B,MASK_H,MASK_W,MASK_D"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="M4 M5 M6 M7 M8 M9 M10 M11 M12 M13 M2:M3 M14:M1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="M4 M5 M6 M7 M8 M9 M10 M11 M12 M13 M14 M2:M3 M15:M1048576">
       <formula1>"INST_VALID,INST_INVALID"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I4 I5 I6 I7 I8 I9 I10 I11 I12 I13 I2:I3 I14:I1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I4 I5 I6 I7 I8 I9 I10 I11 I12 I13 I14 I2:I3 I15:I1048576">
       <formula1>"LD_LB,LD_LH,LD_LW,LD_LBU,LD_LHU,LD_XX"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G4 G5 G6 G7 G8 G9 G10 G11 G12 G13 G2:G3 G14:G1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G4 G5 G6 G7 G8 G9 G10 G11 G12 G13 G14 G2:G3 G15:G1048576">
       <formula1>"IMM_I,IMM_J,IMM_U,IMM_S,IMM_B"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F4 F5 F6 F7 F8 F9 F10 F11 F12 F13 F2:F3 F14:F1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F4 F5 F6 F7 F8 F9 F10 F11 F12 F13 F14 F2:F3 F15:F1048576">
       <formula1>"ALU_ADD,ALU_SUB,ALU_AND,ALU_OR,ALU_XOR,ALU_SLL,ALU_SRL,ALU_SLT,ALU_SLTU,ALU_COPY_A,ALU_COPY_B"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H5 H9 H10 H11 H12 H13 H2:H4 H6:H8 H14:H1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H5 H6 H10 H11 H12 H13 H14 H2:H4 H7:H9 H15:H1048576">
       <formula1>"WB_ALU,WB_MEM,WB_PC4,WB_XX"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D4 D5 D6 D7 D8 D9 D10 D11 D12 D13 D2:D3 D14:D1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D4 D5 D6 D7 D8 D9 D10 D11 D12 D13 D14 D2:D3 D15:D1048576">
       <formula1>"A_PC,A_RS1"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E4 E5 E6 E7 E8 E9 E10 E11 E12 E13 E2:E3 E14:E1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E4 E5 E6 E7 E8 E9 E10 E11 E12 E13 E14 E2:E3 E15:E1048576">
       <formula1>"B_IMM,B_RS2"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C4 C5 C6 C7 C8 C9 C10 C11 C12 C13 C2:C3 C14:C1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C4 C5 C6 C7 C8 C9 C10 C11 C12 C13 C14 C2:C3 C15:C1048576">
       <formula1>"PC_4,PC_0,PC_ALU"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
> sim RTL ysyx_23060246 韩炳晋 Linux archlinux 6.6.60-1-lts #1 SMP PREEMPT_DYNAMIC Fri, 08 Nov 2024 16:03:02 +0000 x86_64 GNU/Linux  18:39:30 up 1 day, 54 min,  2 users,  load average: 6.18, 4.87, 4.21
</commit_message>
<xml_diff>
--- a/npc/tools/control_gen/control_table.xlsx
+++ b/npc/tools/control_gen/control_table.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="118" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="126" uniqueCount="60">
   <si>
     <t>commont</t>
   </si>
@@ -112,10 +112,19 @@
     <t>IMM_J</t>
   </si>
   <si>
+    <t>sb</t>
+  </si>
+  <si>
+    <t>IMM_S</t>
+  </si>
+  <si>
+    <t>ST_SB</t>
+  </si>
+  <si>
+    <t>MASK_B</t>
+  </si>
+  <si>
     <t>sw</t>
-  </si>
-  <si>
-    <t>IMM_S</t>
   </si>
   <si>
     <t>ST_SW</t>
@@ -1153,7 +1162,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:AH70"/>
+  <dimension ref="A1:AH71"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
     <col min="1" max="1" width="13.1" customWidth="1"/>
@@ -1584,9 +1593,7 @@
       <c r="B9" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="C9" s="2" t="s">
-        <v>37</v>
-      </c>
+      <c r="C9" s="2"/>
       <c r="D9" s="4" t="s">
         <v>23</v>
       </c>
@@ -1597,14 +1604,16 @@
         <v>21</v>
       </c>
       <c r="G9" s="4" t="s">
-        <v>24</v>
+        <v>33</v>
       </c>
       <c r="H9" s="4"/>
-      <c r="I9" s="4" t="s">
+      <c r="I9" s="4"/>
+      <c r="J9" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="K9" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="J9" s="4"/>
-      <c r="K9" s="4"/>
       <c r="L9" s="4"/>
       <c r="M9" s="4" t="s">
         <v>18</v>
@@ -1637,10 +1646,10 @@
         <v>39</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>28</v>
+        <v>40</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="E10" s="4" t="s">
         <v>14</v>
@@ -1649,15 +1658,15 @@
         <v>21</v>
       </c>
       <c r="G10" s="4" t="s">
-        <v>40</v>
+        <v>24</v>
       </c>
       <c r="H10" s="4"/>
-      <c r="I10" s="4"/>
+      <c r="I10" s="4" t="s">
+        <v>41</v>
+      </c>
       <c r="J10" s="4"/>
       <c r="K10" s="4"/>
-      <c r="L10" s="4" t="s">
-        <v>41</v>
-      </c>
+      <c r="L10" s="4"/>
       <c r="M10" s="4" t="s">
         <v>18</v>
       </c>
@@ -1688,26 +1697,28 @@
       <c r="B11" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="C11" s="2"/>
+      <c r="C11" s="2" t="s">
+        <v>28</v>
+      </c>
       <c r="D11" s="4" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="E11" s="4" t="s">
         <v>14</v>
       </c>
       <c r="F11" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="G11" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="G11" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="H11" s="4" t="s">
-        <v>17</v>
-      </c>
+      <c r="H11" s="4"/>
       <c r="I11" s="4"/>
       <c r="J11" s="4"/>
       <c r="K11" s="4"/>
-      <c r="L11" s="4"/>
+      <c r="L11" s="4" t="s">
+        <v>44</v>
+      </c>
       <c r="M11" s="4" t="s">
         <v>18</v>
       </c>
@@ -1736,7 +1747,7 @@
     <row r="12" spans="1:34">
       <c r="A12" s="3"/>
       <c r="B12" s="4" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C12" s="2"/>
       <c r="D12" s="4" t="s">
@@ -1746,7 +1757,7 @@
         <v>14</v>
       </c>
       <c r="F12" s="4" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="G12" s="4" t="s">
         <v>24</v>
@@ -1786,19 +1797,21 @@
     <row r="13" spans="1:34">
       <c r="A13" s="3"/>
       <c r="B13" s="4" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C13" s="2"/>
       <c r="D13" s="4" t="s">
         <v>23</v>
       </c>
       <c r="E13" s="4" t="s">
-        <v>47</v>
+        <v>14</v>
       </c>
       <c r="F13" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="G13" s="4"/>
+        <v>48</v>
+      </c>
+      <c r="G13" s="4" t="s">
+        <v>24</v>
+      </c>
       <c r="H13" s="4" t="s">
         <v>17</v>
       </c>
@@ -1834,17 +1847,17 @@
     <row r="14" spans="1:34">
       <c r="A14" s="3"/>
       <c r="B14" s="4" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C14" s="2"/>
       <c r="D14" s="4" t="s">
         <v>23</v>
       </c>
       <c r="E14" s="4" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="F14" s="4" t="s">
-        <v>49</v>
+        <v>21</v>
       </c>
       <c r="G14" s="4"/>
       <c r="H14" s="4" t="s">
@@ -1879,49 +1892,42 @@
       <c r="AG14" s="3"/>
       <c r="AH14" s="3"/>
     </row>
-    <row r="15" spans="2:34">
-      <c r="B15" s="2" t="s">
+    <row r="15" spans="1:34">
+      <c r="A15" s="3"/>
+      <c r="B15" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="C15" s="2"/>
+      <c r="D15" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="E15" s="4" t="s">
         <v>50</v>
       </c>
-      <c r="C15" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="D15" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="E15" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="F15" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="G15" s="2" t="s">
-        <v>24</v>
-      </c>
+      <c r="F15" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="G15" s="4"/>
       <c r="H15" s="4" t="s">
-        <v>51</v>
-      </c>
-      <c r="I15" s="4" t="s">
-        <v>52</v>
-      </c>
-      <c r="J15" s="4" t="s">
-        <v>53</v>
-      </c>
-      <c r="K15" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="L15" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="M15" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="N15" s="2"/>
-      <c r="O15" s="2"/>
-      <c r="P15" s="2"/>
-      <c r="Q15" s="2"/>
-      <c r="R15" s="2"/>
-      <c r="S15" s="2"/>
+        <v>17</v>
+      </c>
+      <c r="I15" s="4"/>
+      <c r="J15" s="4"/>
+      <c r="K15" s="4"/>
+      <c r="L15" s="4"/>
+      <c r="M15" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="N15" s="4"/>
+      <c r="O15" s="4"/>
+      <c r="P15" s="4"/>
+      <c r="Q15" s="4"/>
+      <c r="R15" s="4"/>
+      <c r="S15" s="4"/>
+      <c r="T15" s="3"/>
+      <c r="U15" s="3"/>
+      <c r="V15" s="3"/>
+      <c r="W15" s="3"/>
       <c r="X15" s="3"/>
       <c r="Y15" s="3"/>
       <c r="Z15" s="3"/>
@@ -1934,30 +1940,49 @@
       <c r="AG15" s="3"/>
       <c r="AH15" s="3"/>
     </row>
-    <row r="16" spans="1:34">
-      <c r="A16" s="3"/>
-      <c r="B16" s="4"/>
-      <c r="C16" s="4"/>
-      <c r="D16" s="4"/>
-      <c r="E16" s="4"/>
-      <c r="F16" s="4"/>
-      <c r="G16" s="4"/>
-      <c r="H16" s="4"/>
-      <c r="I16" s="4"/>
-      <c r="J16" s="4"/>
-      <c r="K16" s="4"/>
-      <c r="L16" s="4"/>
-      <c r="M16" s="4"/>
-      <c r="N16" s="4"/>
-      <c r="O16" s="4"/>
-      <c r="P16" s="4"/>
-      <c r="Q16" s="4"/>
-      <c r="R16" s="4"/>
-      <c r="S16" s="4"/>
-      <c r="T16" s="3"/>
-      <c r="U16" s="3"/>
-      <c r="V16" s="3"/>
-      <c r="W16" s="3"/>
+    <row r="16" spans="2:34">
+      <c r="B16" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="E16" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="F16" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="G16" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="H16" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="I16" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="J16" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="K16" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="L16" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="M16" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="N16" s="2"/>
+      <c r="O16" s="2"/>
+      <c r="P16" s="2"/>
+      <c r="Q16" s="2"/>
+      <c r="R16" s="2"/>
+      <c r="S16" s="2"/>
       <c r="X16" s="3"/>
       <c r="Y16" s="3"/>
       <c r="Z16" s="3"/>
@@ -1970,7 +1995,7 @@
       <c r="AG16" s="3"/>
       <c r="AH16" s="3"/>
     </row>
-    <row r="17" s="1" customFormat="1" spans="1:34">
+    <row r="17" spans="1:34">
       <c r="A17" s="3"/>
       <c r="B17" s="4"/>
       <c r="C17" s="4"/>
@@ -2042,7 +2067,7 @@
       <c r="AG18" s="3"/>
       <c r="AH18" s="3"/>
     </row>
-    <row r="19" spans="1:34">
+    <row r="19" s="1" customFormat="1" spans="1:34">
       <c r="A19" s="3"/>
       <c r="B19" s="4"/>
       <c r="C19" s="4"/>
@@ -2587,7 +2612,7 @@
       <c r="B34" s="4"/>
       <c r="C34" s="4"/>
       <c r="D34" s="4"/>
-      <c r="E34" s="5"/>
+      <c r="E34" s="4"/>
       <c r="F34" s="4"/>
       <c r="G34" s="4"/>
       <c r="H34" s="4"/>
@@ -2695,7 +2720,7 @@
       <c r="B37" s="4"/>
       <c r="C37" s="4"/>
       <c r="D37" s="4"/>
-      <c r="E37" s="4"/>
+      <c r="E37" s="5"/>
       <c r="F37" s="4"/>
       <c r="G37" s="4"/>
       <c r="H37" s="4"/>
@@ -2839,7 +2864,7 @@
       <c r="B41" s="4"/>
       <c r="C41" s="4"/>
       <c r="D41" s="4"/>
-      <c r="E41" s="5"/>
+      <c r="E41" s="4"/>
       <c r="F41" s="4"/>
       <c r="G41" s="4"/>
       <c r="H41" s="4"/>
@@ -2875,7 +2900,7 @@
       <c r="B42" s="4"/>
       <c r="C42" s="4"/>
       <c r="D42" s="4"/>
-      <c r="E42" s="4"/>
+      <c r="E42" s="5"/>
       <c r="F42" s="4"/>
       <c r="G42" s="4"/>
       <c r="H42" s="4"/>
@@ -3158,25 +3183,48 @@
       <c r="AG49" s="3"/>
       <c r="AH49" s="3"/>
     </row>
-    <row r="57" spans="1:23">
-      <c r="A57" s="2"/>
-      <c r="B57" s="2"/>
-      <c r="C57" s="2"/>
-      <c r="D57" s="2"/>
-      <c r="R57" s="2"/>
-      <c r="T57" s="2"/>
-      <c r="U57" s="2"/>
-      <c r="V57" s="2"/>
-      <c r="W57" s="2"/>
+    <row r="50" spans="1:34">
+      <c r="A50" s="3"/>
+      <c r="B50" s="4"/>
+      <c r="C50" s="4"/>
+      <c r="D50" s="4"/>
+      <c r="E50" s="4"/>
+      <c r="F50" s="4"/>
+      <c r="G50" s="4"/>
+      <c r="H50" s="4"/>
+      <c r="I50" s="4"/>
+      <c r="J50" s="4"/>
+      <c r="K50" s="4"/>
+      <c r="L50" s="4"/>
+      <c r="M50" s="4"/>
+      <c r="N50" s="4"/>
+      <c r="O50" s="4"/>
+      <c r="P50" s="4"/>
+      <c r="Q50" s="4"/>
+      <c r="R50" s="4"/>
+      <c r="S50" s="4"/>
+      <c r="T50" s="3"/>
+      <c r="U50" s="3"/>
+      <c r="V50" s="3"/>
+      <c r="W50" s="3"/>
+      <c r="X50" s="3"/>
+      <c r="Y50" s="3"/>
+      <c r="Z50" s="3"/>
+      <c r="AA50" s="3"/>
+      <c r="AB50" s="3"/>
+      <c r="AC50" s="3"/>
+      <c r="AD50" s="3"/>
+      <c r="AE50" s="3"/>
+      <c r="AF50" s="3"/>
+      <c r="AG50" s="3"/>
+      <c r="AH50" s="3"/>
     </row>
     <row r="58" spans="1:23">
       <c r="A58" s="2"/>
       <c r="B58" s="2"/>
       <c r="C58" s="2"/>
       <c r="D58" s="2"/>
-      <c r="E58" s="2"/>
       <c r="R58" s="2"/>
-      <c r="S58" s="2"/>
       <c r="T58" s="2"/>
       <c r="U58" s="2"/>
       <c r="V58" s="2"/>
@@ -3187,6 +3235,7 @@
       <c r="B59" s="2"/>
       <c r="C59" s="2"/>
       <c r="D59" s="2"/>
+      <c r="E59" s="2"/>
       <c r="R59" s="2"/>
       <c r="S59" s="2"/>
       <c r="T59" s="2"/>
@@ -3326,39 +3375,51 @@
       <c r="V70" s="2"/>
       <c r="W70" s="2"/>
     </row>
+    <row r="71" spans="1:23">
+      <c r="A71" s="2"/>
+      <c r="B71" s="2"/>
+      <c r="C71" s="2"/>
+      <c r="D71" s="2"/>
+      <c r="R71" s="2"/>
+      <c r="S71" s="2"/>
+      <c r="T71" s="2"/>
+      <c r="U71" s="2"/>
+      <c r="V71" s="2"/>
+      <c r="W71" s="2"/>
+    </row>
   </sheetData>
   <dataValidations count="11">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L5 L11 L12 L13 L14 L2:L4 L6:L10 L15:L1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L5 L8 L12 L13 L14 L15 L2:L4 L6:L7 L9:L11 L16:L1048576">
       <formula1>"BR_EQ,BR_NE,BR_LTU,BR_GE,BR_GEU,BR_LT,BR_XX"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J5 J6 J9 J10 J11 J12 J13 J14 J2:J4 J7:J8 J15:J1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J5 J6 J7 J8 J9 J10 J11 J12 J13 J14 J15 J2:J4 J16:J1048576">
       <formula1>"ST_SW,ST_SH,ST_SB,ST_XX"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K4 K5 K6 K7 K8 K9 K10 K11 K12 K13 K14 K2:K3 K15:K1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K4 K5 K6 K7 K8 K9 K10 K11 K12 K13 K14 K15 K2:K3 K16:K1048576">
       <formula1>"MASK_XX,MASK_B,MASK_H,MASK_W,MASK_D"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="M4 M5 M6 M7 M8 M9 M10 M11 M12 M13 M14 M2:M3 M15:M1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="M4 M5 M6 M7 M8 M9 M10 M11 M12 M13 M14 M15 M2:M3 M16:M1048576">
       <formula1>"INST_VALID,INST_INVALID"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I4 I5 I6 I7 I8 I9 I10 I11 I12 I13 I14 I2:I3 I15:I1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I4 I5 I6 I7 I8 I9 I10 I11 I12 I13 I14 I15 I2:I3 I16:I1048576">
       <formula1>"LD_LB,LD_LH,LD_LW,LD_LBU,LD_LHU,LD_XX"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G4 G5 G6 G7 G8 G9 G10 G11 G12 G13 G14 G2:G3 G15:G1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G4 G5 G6 G7 G8 G9 G10 G11 G12 G13 G14 G15 G2:G3 G16:G1048576">
       <formula1>"IMM_I,IMM_J,IMM_U,IMM_S,IMM_B"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F4 F5 F6 F7 F8 F9 F10 F11 F12 F13 F14 F2:F3 F15:F1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F4 F5 F6 F7 F8 F9 F10 F11 F12 F13 F14 F15 F2:F3 F16:F1048576">
       <formula1>"ALU_ADD,ALU_SUB,ALU_AND,ALU_OR,ALU_XOR,ALU_SLL,ALU_SRL,ALU_SLT,ALU_SLTU,ALU_COPY_A,ALU_COPY_B"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H5 H6 H10 H11 H12 H13 H14 H2:H4 H7:H9 H15:H1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H5 H6 H7 H8 H11 H12 H13 H14 H15 H2:H4 H9:H10 H16:H1048576">
       <formula1>"WB_ALU,WB_MEM,WB_PC4,WB_XX"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D4 D5 D6 D7 D8 D9 D10 D11 D12 D13 D14 D2:D3 D15:D1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D4 D5 D6 D7 D8 D9 D10 D11 D12 D13 D14 D15 D2:D3 D16:D1048576">
       <formula1>"A_PC,A_RS1"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E4 E5 E6 E7 E8 E9 E10 E11 E12 E13 E14 E2:E3 E15:E1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E4 E5 E6 E7 E8 E9 E10 E11 E12 E13 E14 E15 E2:E3 E16:E1048576">
       <formula1>"B_IMM,B_RS2"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C4 C5 C6 C7 C8 C9 C10 C11 C12 C13 C14 C2:C3 C15:C1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C4 C5 C6 C7 C8 C9 C10 C11 C12 C13 C14 C15 C2:C3 C16:C1048576">
       <formula1>"PC_4,PC_0,PC_ALU"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
> sim RTL ysyx_23060246 韩炳晋 Linux archlinux 6.6.60-1-lts #1 SMP PREEMPT_DYNAMIC Fri, 08 Nov 2024 16:03:02 +0000 x86_64 GNU/Linux  18:43:51 up 1 day, 58 min,  2 users,  load average: 4.64, 4.37, 4.14
</commit_message>
<xml_diff>
--- a/npc/tools/control_gen/control_table.xlsx
+++ b/npc/tools/control_gen/control_table.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="126" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="139" uniqueCount="64">
   <si>
     <t>commont</t>
   </si>
@@ -136,46 +136,58 @@
     <t>lw</t>
   </si>
   <si>
+    <t>LD_LW</t>
+  </si>
+  <si>
+    <t>lb</t>
+  </si>
+  <si>
+    <t>LD_LB</t>
+  </si>
+  <si>
+    <t>lbu</t>
+  </si>
+  <si>
+    <t>LD_LBU</t>
+  </si>
+  <si>
+    <t>bgeu</t>
+  </si>
+  <si>
+    <t>IMM_B</t>
+  </si>
+  <si>
+    <t>BR_GEU</t>
+  </si>
+  <si>
+    <t>slli</t>
+  </si>
+  <si>
+    <t>ALU_SLL</t>
+  </si>
+  <si>
+    <t>sltiu</t>
+  </si>
+  <si>
+    <t>ALU_SLTU</t>
+  </si>
+  <si>
+    <t>add</t>
+  </si>
+  <si>
+    <t>B_RS2</t>
+  </si>
+  <si>
+    <t>sub</t>
+  </si>
+  <si>
+    <t>ALU_SUB</t>
+  </si>
+  <si>
+    <t>default</t>
+  </si>
+  <si>
     <t>PC_4</t>
-  </si>
-  <si>
-    <t>LD_LW</t>
-  </si>
-  <si>
-    <t>bgeu</t>
-  </si>
-  <si>
-    <t>IMM_B</t>
-  </si>
-  <si>
-    <t>BR_GEU</t>
-  </si>
-  <si>
-    <t>slli</t>
-  </si>
-  <si>
-    <t>ALU_SLL</t>
-  </si>
-  <si>
-    <t>sltiu</t>
-  </si>
-  <si>
-    <t>ALU_SLTU</t>
-  </si>
-  <si>
-    <t>add</t>
-  </si>
-  <si>
-    <t>B_RS2</t>
-  </si>
-  <si>
-    <t>sub</t>
-  </si>
-  <si>
-    <t>ALU_SUB</t>
-  </si>
-  <si>
-    <t>default</t>
   </si>
   <si>
     <t>WB_XX</t>
@@ -1162,7 +1174,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:AH71"/>
+  <dimension ref="A1:AH73"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
     <col min="1" max="1" width="13.1" customWidth="1"/>
@@ -1645,9 +1657,7 @@
       <c r="B10" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="C10" s="2" t="s">
-        <v>40</v>
-      </c>
+      <c r="C10" s="2"/>
       <c r="D10" s="4" t="s">
         <v>23</v>
       </c>
@@ -1662,7 +1672,7 @@
       </c>
       <c r="H10" s="4"/>
       <c r="I10" s="4" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="J10" s="4"/>
       <c r="K10" s="4"/>
@@ -1695,13 +1705,11 @@
     <row r="11" spans="1:34">
       <c r="A11" s="3"/>
       <c r="B11" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="C11" s="2" t="s">
-        <v>28</v>
-      </c>
+        <v>41</v>
+      </c>
+      <c r="C11" s="2"/>
       <c r="D11" s="4" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="E11" s="4" t="s">
         <v>14</v>
@@ -1710,15 +1718,15 @@
         <v>21</v>
       </c>
       <c r="G11" s="4" t="s">
-        <v>43</v>
+        <v>24</v>
       </c>
       <c r="H11" s="4"/>
-      <c r="I11" s="4"/>
+      <c r="I11" s="4" t="s">
+        <v>42</v>
+      </c>
       <c r="J11" s="4"/>
       <c r="K11" s="4"/>
-      <c r="L11" s="4" t="s">
-        <v>44</v>
-      </c>
+      <c r="L11" s="4"/>
       <c r="M11" s="4" t="s">
         <v>18</v>
       </c>
@@ -1747,7 +1755,7 @@
     <row r="12" spans="1:34">
       <c r="A12" s="3"/>
       <c r="B12" s="4" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="C12" s="2"/>
       <c r="D12" s="4" t="s">
@@ -1757,15 +1765,15 @@
         <v>14</v>
       </c>
       <c r="F12" s="4" t="s">
-        <v>46</v>
+        <v>21</v>
       </c>
       <c r="G12" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="H12" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="I12" s="4"/>
+      <c r="H12" s="4"/>
+      <c r="I12" s="4" t="s">
+        <v>44</v>
+      </c>
       <c r="J12" s="4"/>
       <c r="K12" s="4"/>
       <c r="L12" s="4"/>
@@ -1797,28 +1805,30 @@
     <row r="13" spans="1:34">
       <c r="A13" s="3"/>
       <c r="B13" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="C13" s="2"/>
+        <v>45</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>28</v>
+      </c>
       <c r="D13" s="4" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="E13" s="4" t="s">
         <v>14</v>
       </c>
       <c r="F13" s="4" t="s">
-        <v>48</v>
+        <v>21</v>
       </c>
       <c r="G13" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="H13" s="4" t="s">
-        <v>17</v>
-      </c>
+        <v>46</v>
+      </c>
+      <c r="H13" s="4"/>
       <c r="I13" s="4"/>
       <c r="J13" s="4"/>
       <c r="K13" s="4"/>
-      <c r="L13" s="4"/>
+      <c r="L13" s="4" t="s">
+        <v>47</v>
+      </c>
       <c r="M13" s="4" t="s">
         <v>18</v>
       </c>
@@ -1847,19 +1857,21 @@
     <row r="14" spans="1:34">
       <c r="A14" s="3"/>
       <c r="B14" s="4" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C14" s="2"/>
       <c r="D14" s="4" t="s">
         <v>23</v>
       </c>
       <c r="E14" s="4" t="s">
-        <v>50</v>
+        <v>14</v>
       </c>
       <c r="F14" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="G14" s="4"/>
+        <v>49</v>
+      </c>
+      <c r="G14" s="4" t="s">
+        <v>24</v>
+      </c>
       <c r="H14" s="4" t="s">
         <v>17</v>
       </c>
@@ -1895,19 +1907,21 @@
     <row r="15" spans="1:34">
       <c r="A15" s="3"/>
       <c r="B15" s="4" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C15" s="2"/>
       <c r="D15" s="4" t="s">
         <v>23</v>
       </c>
       <c r="E15" s="4" t="s">
-        <v>50</v>
+        <v>14</v>
       </c>
       <c r="F15" s="4" t="s">
-        <v>52</v>
-      </c>
-      <c r="G15" s="4"/>
+        <v>51</v>
+      </c>
+      <c r="G15" s="4" t="s">
+        <v>24</v>
+      </c>
       <c r="H15" s="4" t="s">
         <v>17</v>
       </c>
@@ -1940,49 +1954,42 @@
       <c r="AG15" s="3"/>
       <c r="AH15" s="3"/>
     </row>
-    <row r="16" spans="2:34">
-      <c r="B16" s="2" t="s">
+    <row r="16" spans="1:34">
+      <c r="A16" s="3"/>
+      <c r="B16" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="C16" s="2"/>
+      <c r="D16" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="E16" s="4" t="s">
         <v>53</v>
       </c>
-      <c r="C16" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="D16" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="E16" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="F16" s="2" t="s">
+      <c r="F16" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="G16" s="2" t="s">
-        <v>24</v>
-      </c>
+      <c r="G16" s="4"/>
       <c r="H16" s="4" t="s">
-        <v>54</v>
-      </c>
-      <c r="I16" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="J16" s="4" t="s">
-        <v>56</v>
-      </c>
-      <c r="K16" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="L16" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="M16" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="N16" s="2"/>
-      <c r="O16" s="2"/>
-      <c r="P16" s="2"/>
-      <c r="Q16" s="2"/>
-      <c r="R16" s="2"/>
-      <c r="S16" s="2"/>
+        <v>17</v>
+      </c>
+      <c r="I16" s="4"/>
+      <c r="J16" s="4"/>
+      <c r="K16" s="4"/>
+      <c r="L16" s="4"/>
+      <c r="M16" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="N16" s="4"/>
+      <c r="O16" s="4"/>
+      <c r="P16" s="4"/>
+      <c r="Q16" s="4"/>
+      <c r="R16" s="4"/>
+      <c r="S16" s="4"/>
+      <c r="T16" s="3"/>
+      <c r="U16" s="3"/>
+      <c r="V16" s="3"/>
+      <c r="W16" s="3"/>
       <c r="X16" s="3"/>
       <c r="Y16" s="3"/>
       <c r="Z16" s="3"/>
@@ -1997,18 +2004,30 @@
     </row>
     <row r="17" spans="1:34">
       <c r="A17" s="3"/>
-      <c r="B17" s="4"/>
-      <c r="C17" s="4"/>
-      <c r="D17" s="4"/>
-      <c r="E17" s="4"/>
-      <c r="F17" s="4"/>
+      <c r="B17" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="C17" s="2"/>
+      <c r="D17" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="E17" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="F17" s="4" t="s">
+        <v>55</v>
+      </c>
       <c r="G17" s="4"/>
-      <c r="H17" s="4"/>
+      <c r="H17" s="4" t="s">
+        <v>17</v>
+      </c>
       <c r="I17" s="4"/>
       <c r="J17" s="4"/>
       <c r="K17" s="4"/>
       <c r="L17" s="4"/>
-      <c r="M17" s="4"/>
+      <c r="M17" s="4" t="s">
+        <v>18</v>
+      </c>
       <c r="N17" s="4"/>
       <c r="O17" s="4"/>
       <c r="P17" s="4"/>
@@ -2031,30 +2050,49 @@
       <c r="AG17" s="3"/>
       <c r="AH17" s="3"/>
     </row>
-    <row r="18" s="1" customFormat="1" spans="1:34">
-      <c r="A18" s="3"/>
-      <c r="B18" s="4"/>
-      <c r="C18" s="4"/>
-      <c r="D18" s="4"/>
-      <c r="E18" s="4"/>
-      <c r="F18" s="4"/>
-      <c r="G18" s="4"/>
-      <c r="H18" s="4"/>
-      <c r="I18" s="4"/>
-      <c r="J18" s="4"/>
-      <c r="K18" s="4"/>
-      <c r="L18" s="4"/>
-      <c r="M18" s="4"/>
-      <c r="N18" s="4"/>
-      <c r="O18" s="4"/>
-      <c r="P18" s="4"/>
-      <c r="Q18" s="4"/>
-      <c r="R18" s="4"/>
-      <c r="S18" s="4"/>
-      <c r="T18" s="3"/>
-      <c r="U18" s="3"/>
-      <c r="V18" s="3"/>
-      <c r="W18" s="3"/>
+    <row r="18" spans="2:34">
+      <c r="B18" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="E18" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="F18" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="G18" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="H18" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="I18" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="J18" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="K18" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="L18" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="M18" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="N18" s="2"/>
+      <c r="O18" s="2"/>
+      <c r="P18" s="2"/>
+      <c r="Q18" s="2"/>
+      <c r="R18" s="2"/>
+      <c r="S18" s="2"/>
       <c r="X18" s="3"/>
       <c r="Y18" s="3"/>
       <c r="Z18" s="3"/>
@@ -2067,7 +2105,7 @@
       <c r="AG18" s="3"/>
       <c r="AH18" s="3"/>
     </row>
-    <row r="19" s="1" customFormat="1" spans="1:34">
+    <row r="19" spans="1:34">
       <c r="A19" s="3"/>
       <c r="B19" s="4"/>
       <c r="C19" s="4"/>
@@ -2103,7 +2141,7 @@
       <c r="AG19" s="3"/>
       <c r="AH19" s="3"/>
     </row>
-    <row r="20" spans="1:34">
+    <row r="20" s="1" customFormat="1" spans="1:34">
       <c r="A20" s="3"/>
       <c r="B20" s="4"/>
       <c r="C20" s="4"/>
@@ -2139,7 +2177,7 @@
       <c r="AG20" s="3"/>
       <c r="AH20" s="3"/>
     </row>
-    <row r="21" spans="1:34">
+    <row r="21" s="1" customFormat="1" spans="1:34">
       <c r="A21" s="3"/>
       <c r="B21" s="4"/>
       <c r="C21" s="4"/>
@@ -2648,7 +2686,7 @@
       <c r="B35" s="4"/>
       <c r="C35" s="4"/>
       <c r="D35" s="4"/>
-      <c r="E35" s="5"/>
+      <c r="E35" s="4"/>
       <c r="F35" s="4"/>
       <c r="G35" s="4"/>
       <c r="H35" s="4"/>
@@ -2684,7 +2722,7 @@
       <c r="B36" s="4"/>
       <c r="C36" s="4"/>
       <c r="D36" s="4"/>
-      <c r="E36" s="5"/>
+      <c r="E36" s="4"/>
       <c r="F36" s="4"/>
       <c r="G36" s="4"/>
       <c r="H36" s="4"/>
@@ -2756,7 +2794,7 @@
       <c r="B38" s="4"/>
       <c r="C38" s="4"/>
       <c r="D38" s="4"/>
-      <c r="E38" s="4"/>
+      <c r="E38" s="5"/>
       <c r="F38" s="4"/>
       <c r="G38" s="4"/>
       <c r="H38" s="4"/>
@@ -2792,7 +2830,7 @@
       <c r="B39" s="4"/>
       <c r="C39" s="4"/>
       <c r="D39" s="4"/>
-      <c r="E39" s="4"/>
+      <c r="E39" s="5"/>
       <c r="F39" s="4"/>
       <c r="G39" s="4"/>
       <c r="H39" s="4"/>
@@ -2900,7 +2938,7 @@
       <c r="B42" s="4"/>
       <c r="C42" s="4"/>
       <c r="D42" s="4"/>
-      <c r="E42" s="5"/>
+      <c r="E42" s="4"/>
       <c r="F42" s="4"/>
       <c r="G42" s="4"/>
       <c r="H42" s="4"/>
@@ -2972,7 +3010,7 @@
       <c r="B44" s="4"/>
       <c r="C44" s="4"/>
       <c r="D44" s="4"/>
-      <c r="E44" s="4"/>
+      <c r="E44" s="5"/>
       <c r="F44" s="4"/>
       <c r="G44" s="4"/>
       <c r="H44" s="4"/>
@@ -3219,29 +3257,77 @@
       <c r="AG50" s="3"/>
       <c r="AH50" s="3"/>
     </row>
-    <row r="58" spans="1:23">
-      <c r="A58" s="2"/>
-      <c r="B58" s="2"/>
-      <c r="C58" s="2"/>
-      <c r="D58" s="2"/>
-      <c r="R58" s="2"/>
-      <c r="T58" s="2"/>
-      <c r="U58" s="2"/>
-      <c r="V58" s="2"/>
-      <c r="W58" s="2"/>
-    </row>
-    <row r="59" spans="1:23">
-      <c r="A59" s="2"/>
-      <c r="B59" s="2"/>
-      <c r="C59" s="2"/>
-      <c r="D59" s="2"/>
-      <c r="E59" s="2"/>
-      <c r="R59" s="2"/>
-      <c r="S59" s="2"/>
-      <c r="T59" s="2"/>
-      <c r="U59" s="2"/>
-      <c r="V59" s="2"/>
-      <c r="W59" s="2"/>
+    <row r="51" spans="1:34">
+      <c r="A51" s="3"/>
+      <c r="B51" s="4"/>
+      <c r="C51" s="4"/>
+      <c r="D51" s="4"/>
+      <c r="E51" s="4"/>
+      <c r="F51" s="4"/>
+      <c r="G51" s="4"/>
+      <c r="H51" s="4"/>
+      <c r="I51" s="4"/>
+      <c r="J51" s="4"/>
+      <c r="K51" s="4"/>
+      <c r="L51" s="4"/>
+      <c r="M51" s="4"/>
+      <c r="N51" s="4"/>
+      <c r="O51" s="4"/>
+      <c r="P51" s="4"/>
+      <c r="Q51" s="4"/>
+      <c r="R51" s="4"/>
+      <c r="S51" s="4"/>
+      <c r="T51" s="3"/>
+      <c r="U51" s="3"/>
+      <c r="V51" s="3"/>
+      <c r="W51" s="3"/>
+      <c r="X51" s="3"/>
+      <c r="Y51" s="3"/>
+      <c r="Z51" s="3"/>
+      <c r="AA51" s="3"/>
+      <c r="AB51" s="3"/>
+      <c r="AC51" s="3"/>
+      <c r="AD51" s="3"/>
+      <c r="AE51" s="3"/>
+      <c r="AF51" s="3"/>
+      <c r="AG51" s="3"/>
+      <c r="AH51" s="3"/>
+    </row>
+    <row r="52" spans="1:34">
+      <c r="A52" s="3"/>
+      <c r="B52" s="4"/>
+      <c r="C52" s="4"/>
+      <c r="D52" s="4"/>
+      <c r="E52" s="4"/>
+      <c r="F52" s="4"/>
+      <c r="G52" s="4"/>
+      <c r="H52" s="4"/>
+      <c r="I52" s="4"/>
+      <c r="J52" s="4"/>
+      <c r="K52" s="4"/>
+      <c r="L52" s="4"/>
+      <c r="M52" s="4"/>
+      <c r="N52" s="4"/>
+      <c r="O52" s="4"/>
+      <c r="P52" s="4"/>
+      <c r="Q52" s="4"/>
+      <c r="R52" s="4"/>
+      <c r="S52" s="4"/>
+      <c r="T52" s="3"/>
+      <c r="U52" s="3"/>
+      <c r="V52" s="3"/>
+      <c r="W52" s="3"/>
+      <c r="X52" s="3"/>
+      <c r="Y52" s="3"/>
+      <c r="Z52" s="3"/>
+      <c r="AA52" s="3"/>
+      <c r="AB52" s="3"/>
+      <c r="AC52" s="3"/>
+      <c r="AD52" s="3"/>
+      <c r="AE52" s="3"/>
+      <c r="AF52" s="3"/>
+      <c r="AG52" s="3"/>
+      <c r="AH52" s="3"/>
     </row>
     <row r="60" spans="1:23">
       <c r="A60" s="2"/>
@@ -3249,7 +3335,6 @@
       <c r="C60" s="2"/>
       <c r="D60" s="2"/>
       <c r="R60" s="2"/>
-      <c r="S60" s="2"/>
       <c r="T60" s="2"/>
       <c r="U60" s="2"/>
       <c r="V60" s="2"/>
@@ -3260,6 +3345,7 @@
       <c r="B61" s="2"/>
       <c r="C61" s="2"/>
       <c r="D61" s="2"/>
+      <c r="E61" s="2"/>
       <c r="R61" s="2"/>
       <c r="S61" s="2"/>
       <c r="T61" s="2"/>
@@ -3387,39 +3473,63 @@
       <c r="V71" s="2"/>
       <c r="W71" s="2"/>
     </row>
+    <row r="72" spans="1:23">
+      <c r="A72" s="2"/>
+      <c r="B72" s="2"/>
+      <c r="C72" s="2"/>
+      <c r="D72" s="2"/>
+      <c r="R72" s="2"/>
+      <c r="S72" s="2"/>
+      <c r="T72" s="2"/>
+      <c r="U72" s="2"/>
+      <c r="V72" s="2"/>
+      <c r="W72" s="2"/>
+    </row>
+    <row r="73" spans="1:23">
+      <c r="A73" s="2"/>
+      <c r="B73" s="2"/>
+      <c r="C73" s="2"/>
+      <c r="D73" s="2"/>
+      <c r="R73" s="2"/>
+      <c r="S73" s="2"/>
+      <c r="T73" s="2"/>
+      <c r="U73" s="2"/>
+      <c r="V73" s="2"/>
+      <c r="W73" s="2"/>
+    </row>
   </sheetData>
   <dataValidations count="11">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L5 L8 L12 L13 L14 L15 L2:L4 L6:L7 L9:L11 L16:L1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L5 L8 L11 L12 L13 L14 L15 L16 L17 L2:L4 L6:L7 L9:L10 L18:L1048576">
       <formula1>"BR_EQ,BR_NE,BR_LTU,BR_GE,BR_GEU,BR_LT,BR_XX"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J5 J6 J7 J8 J9 J10 J11 J12 J13 J14 J15 J2:J4 J16:J1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J5 J6 J7 J8 J9 J10 J11 J12 J13 J14 J15 J16 J17 J2:J4 J18:J1048576">
       <formula1>"ST_SW,ST_SH,ST_SB,ST_XX"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K4 K5 K6 K7 K8 K9 K10 K11 K12 K13 K14 K15 K2:K3 K16:K1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K4 K5 K6 K7 K8 K9 K10 K11 K12 K13 K14 K15 K16 K17 K2:K3 K18:K1048576">
       <formula1>"MASK_XX,MASK_B,MASK_H,MASK_W,MASK_D"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="M4 M5 M6 M7 M8 M9 M10 M11 M12 M13 M14 M15 M2:M3 M16:M1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="M4 M5 M6 M7 M8 M9 M10 M11 M12 M13 M14 M15 M16 M17 M2:M3 M18:M1048576">
       <formula1>"INST_VALID,INST_INVALID"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I4 I5 I6 I7 I8 I9 I10 I11 I12 I13 I14 I15 I2:I3 I16:I1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I4 I5 I6 I7 I8 I9 I10 I11 I12 I13 I14 I15 I16 I17 I2:I3 I18:I1048576">
       <formula1>"LD_LB,LD_LH,LD_LW,LD_LBU,LD_LHU,LD_XX"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G4 G5 G6 G7 G8 G9 G10 G11 G12 G13 G14 G15 G2:G3 G16:G1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G4 G5 G6 G7 G8 G9 G10 G11 G12 G13 G14 G15 G16 G17 G2:G3 G18:G1048576">
       <formula1>"IMM_I,IMM_J,IMM_U,IMM_S,IMM_B"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F4 F5 F6 F7 F8 F9 F10 F11 F12 F13 F14 F15 F2:F3 F16:F1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F4 F5 F6 F7 F8 F9 F10 F11 F12 F13 F14 F15 F16 F17 F2:F3 F18:F1048576">
       <formula1>"ALU_ADD,ALU_SUB,ALU_AND,ALU_OR,ALU_XOR,ALU_SLL,ALU_SRL,ALU_SLT,ALU_SLTU,ALU_COPY_A,ALU_COPY_B"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H5 H6 H7 H8 H11 H12 H13 H14 H15 H2:H4 H9:H10 H16:H1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H5 H6 H7 H8 H11 H12 H13 H14 H15 H16 H17 H2:H4 H9:H10 H18:H1048576">
       <formula1>"WB_ALU,WB_MEM,WB_PC4,WB_XX"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D4 D5 D6 D7 D8 D9 D10 D11 D12 D13 D14 D15 D2:D3 D16:D1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D4 D5 D6 D7 D8 D9 D10 D11 D12 D13 D14 D15 D16 D17 D2:D3 D18:D1048576">
       <formula1>"A_PC,A_RS1"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E4 E5 E6 E7 E8 E9 E10 E11 E12 E13 E14 E15 E2:E3 E16:E1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E4 E5 E6 E7 E8 E9 E10 E11 E12 E13 E14 E15 E16 E17 E2:E3 E18:E1048576">
       <formula1>"B_IMM,B_RS2"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C4 C5 C6 C7 C8 C9 C10 C11 C12 C13 C14 C15 C2:C3 C16:C1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C4 C5 C6 C7 C8 C9 C10 C11 C12 C13 C14 C15 C16 C17 C2:C3 C18:C1048576">
       <formula1>"PC_4,PC_0,PC_ALU"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
> sim RTL ysyx_23060246 韩炳晋 Linux archlinux 6.6.60-1-lts #1 SMP PREEMPT_DYNAMIC Fri, 08 Nov 2024 16:03:02 +0000 x86_64 GNU/Linux  18:45:38 up 1 day,  1:00,  2 users,  load average: 5.39, 4.53, 4.21
</commit_message>
<xml_diff>
--- a/npc/tools/control_gen/control_table.xlsx
+++ b/npc/tools/control_gen/control_table.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="139" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="146" uniqueCount="66">
   <si>
     <t>commont</t>
   </si>
@@ -95,6 +95,12 @@
   </si>
   <si>
     <t>ALU_AND</t>
+  </si>
+  <si>
+    <t>xori</t>
+  </si>
+  <si>
+    <t>ALU_XOR</t>
   </si>
   <si>
     <t>jalr</t>
@@ -1174,7 +1180,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:AH73"/>
+  <dimension ref="A1:AH74"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
     <col min="1" max="1" width="13.1" customWidth="1"/>
@@ -1449,9 +1455,7 @@
       <c r="B6" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="C6" s="2" t="s">
-        <v>28</v>
-      </c>
+      <c r="C6" s="2"/>
       <c r="D6" s="4" t="s">
         <v>23</v>
       </c>
@@ -1459,13 +1463,13 @@
         <v>14</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>21</v>
+        <v>28</v>
       </c>
       <c r="G6" s="4" t="s">
         <v>24</v>
       </c>
       <c r="H6" s="4" t="s">
-        <v>29</v>
+        <v>17</v>
       </c>
       <c r="I6" s="4"/>
       <c r="J6" s="4"/>
@@ -1499,13 +1503,13 @@
     <row r="7" spans="1:34">
       <c r="A7" s="3"/>
       <c r="B7" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="C7" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="C7" s="2" t="s">
-        <v>28</v>
-      </c>
       <c r="D7" s="4" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="E7" s="4" t="s">
         <v>14</v>
@@ -1514,10 +1518,10 @@
         <v>21</v>
       </c>
       <c r="G7" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="H7" s="4" t="s">
         <v>31</v>
-      </c>
-      <c r="H7" s="4" t="s">
-        <v>29</v>
       </c>
       <c r="I7" s="4"/>
       <c r="J7" s="4"/>
@@ -1553,9 +1557,11 @@
       <c r="B8" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="C8" s="2"/>
+      <c r="C8" s="2" t="s">
+        <v>30</v>
+      </c>
       <c r="D8" s="4" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="E8" s="4" t="s">
         <v>14</v>
@@ -1566,14 +1572,12 @@
       <c r="G8" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="H8" s="4"/>
+      <c r="H8" s="4" t="s">
+        <v>31</v>
+      </c>
       <c r="I8" s="4"/>
-      <c r="J8" s="4" t="s">
-        <v>34</v>
-      </c>
-      <c r="K8" s="4" t="s">
-        <v>35</v>
-      </c>
+      <c r="J8" s="4"/>
+      <c r="K8" s="4"/>
       <c r="L8" s="4"/>
       <c r="M8" s="4" t="s">
         <v>18</v>
@@ -1603,7 +1607,7 @@
     <row r="9" spans="1:34">
       <c r="A9" s="3"/>
       <c r="B9" s="4" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="C9" s="2"/>
       <c r="D9" s="4" t="s">
@@ -1616,15 +1620,15 @@
         <v>21</v>
       </c>
       <c r="G9" s="4" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="H9" s="4"/>
       <c r="I9" s="4"/>
       <c r="J9" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="K9" s="4" t="s">
         <v>37</v>
-      </c>
-      <c r="K9" s="4" t="s">
-        <v>38</v>
       </c>
       <c r="L9" s="4"/>
       <c r="M9" s="4" t="s">
@@ -1655,7 +1659,7 @@
     <row r="10" spans="1:34">
       <c r="A10" s="3"/>
       <c r="B10" s="4" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C10" s="2"/>
       <c r="D10" s="4" t="s">
@@ -1668,14 +1672,16 @@
         <v>21</v>
       </c>
       <c r="G10" s="4" t="s">
-        <v>24</v>
+        <v>35</v>
       </c>
       <c r="H10" s="4"/>
-      <c r="I10" s="4" t="s">
+      <c r="I10" s="4"/>
+      <c r="J10" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="K10" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="J10" s="4"/>
-      <c r="K10" s="4"/>
       <c r="L10" s="4"/>
       <c r="M10" s="4" t="s">
         <v>18</v>
@@ -1807,11 +1813,9 @@
       <c r="B13" s="4" t="s">
         <v>45</v>
       </c>
-      <c r="C13" s="2" t="s">
-        <v>28</v>
-      </c>
+      <c r="C13" s="2"/>
       <c r="D13" s="4" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="E13" s="4" t="s">
         <v>14</v>
@@ -1820,15 +1824,15 @@
         <v>21</v>
       </c>
       <c r="G13" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="H13" s="4"/>
+      <c r="I13" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="H13" s="4"/>
-      <c r="I13" s="4"/>
       <c r="J13" s="4"/>
       <c r="K13" s="4"/>
-      <c r="L13" s="4" t="s">
-        <v>47</v>
-      </c>
+      <c r="L13" s="4"/>
       <c r="M13" s="4" t="s">
         <v>18</v>
       </c>
@@ -1857,28 +1861,30 @@
     <row r="14" spans="1:34">
       <c r="A14" s="3"/>
       <c r="B14" s="4" t="s">
-        <v>48</v>
-      </c>
-      <c r="C14" s="2"/>
+        <v>47</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>30</v>
+      </c>
       <c r="D14" s="4" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="E14" s="4" t="s">
         <v>14</v>
       </c>
       <c r="F14" s="4" t="s">
-        <v>49</v>
+        <v>21</v>
       </c>
       <c r="G14" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="H14" s="4" t="s">
-        <v>17</v>
-      </c>
+        <v>48</v>
+      </c>
+      <c r="H14" s="4"/>
       <c r="I14" s="4"/>
       <c r="J14" s="4"/>
       <c r="K14" s="4"/>
-      <c r="L14" s="4"/>
+      <c r="L14" s="4" t="s">
+        <v>49</v>
+      </c>
       <c r="M14" s="4" t="s">
         <v>18</v>
       </c>
@@ -1964,12 +1970,14 @@
         <v>23</v>
       </c>
       <c r="E16" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="F16" s="4" t="s">
         <v>53</v>
       </c>
-      <c r="F16" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="G16" s="4"/>
+      <c r="G16" s="4" t="s">
+        <v>24</v>
+      </c>
       <c r="H16" s="4" t="s">
         <v>17</v>
       </c>
@@ -2012,10 +2020,10 @@
         <v>23</v>
       </c>
       <c r="E17" s="4" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="F17" s="4" t="s">
-        <v>55</v>
+        <v>21</v>
       </c>
       <c r="G17" s="4"/>
       <c r="H17" s="4" t="s">
@@ -2050,49 +2058,42 @@
       <c r="AG17" s="3"/>
       <c r="AH17" s="3"/>
     </row>
-    <row r="18" spans="2:34">
-      <c r="B18" s="2" t="s">
+    <row r="18" spans="1:34">
+      <c r="A18" s="3"/>
+      <c r="B18" s="4" t="s">
         <v>56</v>
       </c>
-      <c r="C18" s="2" t="s">
+      <c r="C18" s="2"/>
+      <c r="D18" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="E18" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="F18" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="D18" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="E18" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="F18" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="G18" s="2" t="s">
-        <v>24</v>
-      </c>
+      <c r="G18" s="4"/>
       <c r="H18" s="4" t="s">
-        <v>58</v>
-      </c>
-      <c r="I18" s="4" t="s">
-        <v>59</v>
-      </c>
-      <c r="J18" s="4" t="s">
-        <v>60</v>
-      </c>
-      <c r="K18" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="L18" s="2" t="s">
-        <v>62</v>
-      </c>
-      <c r="M18" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="N18" s="2"/>
-      <c r="O18" s="2"/>
-      <c r="P18" s="2"/>
-      <c r="Q18" s="2"/>
-      <c r="R18" s="2"/>
-      <c r="S18" s="2"/>
+        <v>17</v>
+      </c>
+      <c r="I18" s="4"/>
+      <c r="J18" s="4"/>
+      <c r="K18" s="4"/>
+      <c r="L18" s="4"/>
+      <c r="M18" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="N18" s="4"/>
+      <c r="O18" s="4"/>
+      <c r="P18" s="4"/>
+      <c r="Q18" s="4"/>
+      <c r="R18" s="4"/>
+      <c r="S18" s="4"/>
+      <c r="T18" s="3"/>
+      <c r="U18" s="3"/>
+      <c r="V18" s="3"/>
+      <c r="W18" s="3"/>
       <c r="X18" s="3"/>
       <c r="Y18" s="3"/>
       <c r="Z18" s="3"/>
@@ -2105,30 +2106,49 @@
       <c r="AG18" s="3"/>
       <c r="AH18" s="3"/>
     </row>
-    <row r="19" spans="1:34">
-      <c r="A19" s="3"/>
-      <c r="B19" s="4"/>
-      <c r="C19" s="4"/>
-      <c r="D19" s="4"/>
-      <c r="E19" s="4"/>
-      <c r="F19" s="4"/>
-      <c r="G19" s="4"/>
-      <c r="H19" s="4"/>
-      <c r="I19" s="4"/>
-      <c r="J19" s="4"/>
-      <c r="K19" s="4"/>
-      <c r="L19" s="4"/>
-      <c r="M19" s="4"/>
-      <c r="N19" s="4"/>
-      <c r="O19" s="4"/>
-      <c r="P19" s="4"/>
-      <c r="Q19" s="4"/>
-      <c r="R19" s="4"/>
-      <c r="S19" s="4"/>
-      <c r="T19" s="3"/>
-      <c r="U19" s="3"/>
-      <c r="V19" s="3"/>
-      <c r="W19" s="3"/>
+    <row r="19" spans="2:34">
+      <c r="B19" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="E19" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="F19" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="G19" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="H19" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="I19" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="J19" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="K19" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="L19" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="M19" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="N19" s="2"/>
+      <c r="O19" s="2"/>
+      <c r="P19" s="2"/>
+      <c r="Q19" s="2"/>
+      <c r="R19" s="2"/>
+      <c r="S19" s="2"/>
       <c r="X19" s="3"/>
       <c r="Y19" s="3"/>
       <c r="Z19" s="3"/>
@@ -2141,7 +2161,7 @@
       <c r="AG19" s="3"/>
       <c r="AH19" s="3"/>
     </row>
-    <row r="20" s="1" customFormat="1" spans="1:34">
+    <row r="20" spans="1:34">
       <c r="A20" s="3"/>
       <c r="B20" s="4"/>
       <c r="C20" s="4"/>
@@ -2213,7 +2233,7 @@
       <c r="AG21" s="3"/>
       <c r="AH21" s="3"/>
     </row>
-    <row r="22" spans="1:34">
+    <row r="22" s="1" customFormat="1" spans="1:34">
       <c r="A22" s="3"/>
       <c r="B22" s="4"/>
       <c r="C22" s="4"/>
@@ -2758,7 +2778,7 @@
       <c r="B37" s="4"/>
       <c r="C37" s="4"/>
       <c r="D37" s="4"/>
-      <c r="E37" s="5"/>
+      <c r="E37" s="4"/>
       <c r="F37" s="4"/>
       <c r="G37" s="4"/>
       <c r="H37" s="4"/>
@@ -2866,7 +2886,7 @@
       <c r="B40" s="4"/>
       <c r="C40" s="4"/>
       <c r="D40" s="4"/>
-      <c r="E40" s="4"/>
+      <c r="E40" s="5"/>
       <c r="F40" s="4"/>
       <c r="G40" s="4"/>
       <c r="H40" s="4"/>
@@ -3010,7 +3030,7 @@
       <c r="B44" s="4"/>
       <c r="C44" s="4"/>
       <c r="D44" s="4"/>
-      <c r="E44" s="5"/>
+      <c r="E44" s="4"/>
       <c r="F44" s="4"/>
       <c r="G44" s="4"/>
       <c r="H44" s="4"/>
@@ -3046,7 +3066,7 @@
       <c r="B45" s="4"/>
       <c r="C45" s="4"/>
       <c r="D45" s="4"/>
-      <c r="E45" s="4"/>
+      <c r="E45" s="5"/>
       <c r="F45" s="4"/>
       <c r="G45" s="4"/>
       <c r="H45" s="4"/>
@@ -3329,25 +3349,48 @@
       <c r="AG52" s="3"/>
       <c r="AH52" s="3"/>
     </row>
-    <row r="60" spans="1:23">
-      <c r="A60" s="2"/>
-      <c r="B60" s="2"/>
-      <c r="C60" s="2"/>
-      <c r="D60" s="2"/>
-      <c r="R60" s="2"/>
-      <c r="T60" s="2"/>
-      <c r="U60" s="2"/>
-      <c r="V60" s="2"/>
-      <c r="W60" s="2"/>
+    <row r="53" spans="1:34">
+      <c r="A53" s="3"/>
+      <c r="B53" s="4"/>
+      <c r="C53" s="4"/>
+      <c r="D53" s="4"/>
+      <c r="E53" s="4"/>
+      <c r="F53" s="4"/>
+      <c r="G53" s="4"/>
+      <c r="H53" s="4"/>
+      <c r="I53" s="4"/>
+      <c r="J53" s="4"/>
+      <c r="K53" s="4"/>
+      <c r="L53" s="4"/>
+      <c r="M53" s="4"/>
+      <c r="N53" s="4"/>
+      <c r="O53" s="4"/>
+      <c r="P53" s="4"/>
+      <c r="Q53" s="4"/>
+      <c r="R53" s="4"/>
+      <c r="S53" s="4"/>
+      <c r="T53" s="3"/>
+      <c r="U53" s="3"/>
+      <c r="V53" s="3"/>
+      <c r="W53" s="3"/>
+      <c r="X53" s="3"/>
+      <c r="Y53" s="3"/>
+      <c r="Z53" s="3"/>
+      <c r="AA53" s="3"/>
+      <c r="AB53" s="3"/>
+      <c r="AC53" s="3"/>
+      <c r="AD53" s="3"/>
+      <c r="AE53" s="3"/>
+      <c r="AF53" s="3"/>
+      <c r="AG53" s="3"/>
+      <c r="AH53" s="3"/>
     </row>
     <row r="61" spans="1:23">
       <c r="A61" s="2"/>
       <c r="B61" s="2"/>
       <c r="C61" s="2"/>
       <c r="D61" s="2"/>
-      <c r="E61" s="2"/>
       <c r="R61" s="2"/>
-      <c r="S61" s="2"/>
       <c r="T61" s="2"/>
       <c r="U61" s="2"/>
       <c r="V61" s="2"/>
@@ -3358,6 +3401,7 @@
       <c r="B62" s="2"/>
       <c r="C62" s="2"/>
       <c r="D62" s="2"/>
+      <c r="E62" s="2"/>
       <c r="R62" s="2"/>
       <c r="S62" s="2"/>
       <c r="T62" s="2"/>
@@ -3497,39 +3541,51 @@
       <c r="V73" s="2"/>
       <c r="W73" s="2"/>
     </row>
+    <row r="74" spans="1:23">
+      <c r="A74" s="2"/>
+      <c r="B74" s="2"/>
+      <c r="C74" s="2"/>
+      <c r="D74" s="2"/>
+      <c r="R74" s="2"/>
+      <c r="S74" s="2"/>
+      <c r="T74" s="2"/>
+      <c r="U74" s="2"/>
+      <c r="V74" s="2"/>
+      <c r="W74" s="2"/>
+    </row>
   </sheetData>
   <dataValidations count="11">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L5 L8 L11 L12 L13 L14 L15 L16 L17 L2:L4 L6:L7 L9:L10 L18:L1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L5 L6 L9 L12 L13 L14 L15 L16 L17 L18 L2:L4 L7:L8 L10:L11 L19:L1048576">
       <formula1>"BR_EQ,BR_NE,BR_LTU,BR_GE,BR_GEU,BR_LT,BR_XX"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J5 J6 J7 J8 J9 J10 J11 J12 J13 J14 J15 J16 J17 J2:J4 J18:J1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J5 J6 J7 J8 J9 J10 J11 J12 J13 J14 J15 J16 J17 J18 J2:J4 J19:J1048576">
       <formula1>"ST_SW,ST_SH,ST_SB,ST_XX"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K4 K5 K6 K7 K8 K9 K10 K11 K12 K13 K14 K15 K16 K17 K2:K3 K18:K1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K4 K5 K6 K7 K8 K9 K10 K11 K12 K13 K14 K15 K16 K17 K18 K2:K3 K19:K1048576">
       <formula1>"MASK_XX,MASK_B,MASK_H,MASK_W,MASK_D"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="M4 M5 M6 M7 M8 M9 M10 M11 M12 M13 M14 M15 M16 M17 M2:M3 M18:M1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="M4 M5 M6 M7 M8 M9 M10 M11 M12 M13 M14 M15 M16 M17 M18 M2:M3 M19:M1048576">
       <formula1>"INST_VALID,INST_INVALID"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I4 I5 I6 I7 I8 I9 I10 I11 I12 I13 I14 I15 I16 I17 I2:I3 I18:I1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I4 I5 I6 I7 I8 I9 I10 I11 I12 I13 I14 I15 I16 I17 I18 I2:I3 I19:I1048576">
       <formula1>"LD_LB,LD_LH,LD_LW,LD_LBU,LD_LHU,LD_XX"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G4 G5 G6 G7 G8 G9 G10 G11 G12 G13 G14 G15 G16 G17 G2:G3 G18:G1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G4 G5 G6 G7 G8 G9 G10 G11 G12 G13 G14 G15 G16 G17 G18 G2:G3 G19:G1048576">
       <formula1>"IMM_I,IMM_J,IMM_U,IMM_S,IMM_B"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F4 F5 F6 F7 F8 F9 F10 F11 F12 F13 F14 F15 F16 F17 F2:F3 F18:F1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F4 F5 F6 F7 F8 F9 F10 F11 F12 F13 F14 F15 F16 F17 F18 F2:F3 F19:F1048576">
       <formula1>"ALU_ADD,ALU_SUB,ALU_AND,ALU_OR,ALU_XOR,ALU_SLL,ALU_SRL,ALU_SLT,ALU_SLTU,ALU_COPY_A,ALU_COPY_B"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H5 H6 H7 H8 H11 H12 H13 H14 H15 H16 H17 H2:H4 H9:H10 H18:H1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H5 H6 H7 H8 H9 H12 H13 H14 H15 H16 H17 H18 H2:H4 H10:H11 H19:H1048576">
       <formula1>"WB_ALU,WB_MEM,WB_PC4,WB_XX"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D4 D5 D6 D7 D8 D9 D10 D11 D12 D13 D14 D15 D16 D17 D2:D3 D18:D1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D4 D5 D6 D7 D8 D9 D10 D11 D12 D13 D14 D15 D16 D17 D18 D2:D3 D19:D1048576">
       <formula1>"A_PC,A_RS1"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E4 E5 E6 E7 E8 E9 E10 E11 E12 E13 E14 E15 E16 E17 E2:E3 E18:E1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E4 E5 E6 E7 E8 E9 E10 E11 E12 E13 E14 E15 E16 E17 E18 E2:E3 E19:E1048576">
       <formula1>"B_IMM,B_RS2"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C4 C5 C6 C7 C8 C9 C10 C11 C12 C13 C14 C15 C16 C17 C2:C3 C18:C1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C4 C5 C6 C7 C8 C9 C10 C11 C12 C13 C14 C15 C16 C17 C18 C2:C3 C19:C1048576">
       <formula1>"PC_4,PC_0,PC_ALU"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
> sim RTL ysyx_23060246 韩炳晋 Linux archlinux 6.6.60-1-lts #1 SMP PREEMPT_DYNAMIC Fri, 08 Nov 2024 16:03:02 +0000 x86_64 GNU/Linux  19:33:40 up 1 day,  1:48,  2 users,  load average: 1.58, 1.05, 1.50
</commit_message>
<xml_diff>
--- a/npc/tools/control_gen/control_table.xlsx
+++ b/npc/tools/control_gen/control_table.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="27795" windowHeight="12075"/>
+    <workbookView windowWidth="27795" windowHeight="12735"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="146" uniqueCount="66">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="154" uniqueCount="68">
   <si>
     <t>comment</t>
   </si>
@@ -157,10 +157,16 @@
     <t>LD_LBU</t>
   </si>
   <si>
+    <t>beq</t>
+  </si>
+  <si>
+    <t>IMM_B</t>
+  </si>
+  <si>
+    <t>BR_EQ</t>
+  </si>
+  <si>
     <t>bgeu</t>
-  </si>
-  <si>
-    <t>IMM_B</t>
   </si>
   <si>
     <t>BR_GEU</t>
@@ -220,9 +226,9 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="4">
     <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="41" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
     <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="42" formatCode="_ &quot;￥&quot;* #,##0_ ;_ &quot;￥&quot;* \-#,##0_ ;_ &quot;￥&quot;* &quot;-&quot;_ ;_ @_ "/>
+    <numFmt numFmtId="41" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
   <fonts count="22">
     <font>
@@ -253,7 +259,7 @@
     </font>
     <font>
       <sz val="11"/>
-      <color theme="1"/>
+      <color theme="0"/>
       <name val="宋体"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -276,16 +282,17 @@
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FF006100"/>
+      <color theme="1"/>
       <name val="宋体"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color theme="0"/>
+      <b/>
+      <sz val="18"/>
+      <color theme="3"/>
       <name val="宋体"/>
-      <charset val="0"/>
+      <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -296,9 +303,15 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
       <sz val="11"/>
-      <color rgb="FF3F3F3F"/>
+      <color rgb="FF9C0006"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF006100"/>
       <name val="宋体"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -309,6 +322,38 @@
       <color theme="3"/>
       <name val="宋体"/>
       <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color rgb="FF7F7F7F"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="13"/>
+      <color theme="3"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF3F3F3F"/>
+      <name val="宋体"/>
+      <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -327,44 +372,6 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color rgb="FF3F3F76"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="18"/>
-      <color theme="3"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="11"/>
-      <color rgb="FF7F7F7F"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C0006"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <u/>
       <sz val="11"/>
       <color rgb="FF800080"/>
@@ -374,16 +381,15 @@
     </font>
     <font>
       <b/>
-      <sz val="13"/>
-      <color theme="3"/>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="宋体"/>
-      <charset val="134"/>
+      <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
       <sz val="11"/>
-      <color theme="1"/>
+      <color rgb="FF3F3F76"/>
       <name val="宋体"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -398,37 +404,19 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.599993896298105"/>
+        <fgColor theme="9"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
+        <fgColor theme="8" tint="0.599993896298105"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="9" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.399975585192419"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -446,60 +434,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor theme="8" tint="0.399975585192419"/>
         <bgColor indexed="64"/>
       </patternFill>
@@ -512,7 +446,43 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFA5A5A5"/>
+        <fgColor theme="6" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.799981688894314"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -524,7 +494,61 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="9"/>
+        <fgColor rgb="FFFFFFCC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFA5A5A5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.599993896298105"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -536,43 +560,25 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.799981688894314"/>
+        <fgColor theme="4"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
+        <fgColor theme="4" tint="0.599993896298105"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7"/>
+        <fgColor rgb="FFFFCC99"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="7" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.399975585192419"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -625,6 +631,30 @@
       <diagonal/>
     </border>
     <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="double">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="double">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="double">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="double">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
       <left style="thin">
         <color rgb="FF3F3F3F"/>
       </left>
@@ -636,15 +666,6 @@
       </top>
       <bottom style="thin">
         <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4"/>
       </bottom>
       <diagonal/>
     </border>
@@ -664,21 +685,6 @@
       <diagonal/>
     </border>
     <border>
-      <left style="double">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="double">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="double">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="double">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
       <left/>
       <right/>
       <top style="thin">
@@ -694,145 +700,145 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="17" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="4" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="30" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="4" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="11" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="4" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="18" fillId="21" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="19" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="21" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="17" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="21" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="11" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
@@ -1180,7 +1186,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:AH74"/>
+  <dimension ref="A1:AH75"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
     <col min="1" max="1" width="13.1" customWidth="1"/>
@@ -1915,26 +1921,28 @@
       <c r="B15" s="4" t="s">
         <v>50</v>
       </c>
-      <c r="C15" s="2"/>
+      <c r="C15" s="2" t="s">
+        <v>30</v>
+      </c>
       <c r="D15" s="4" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="E15" s="4" t="s">
         <v>14</v>
       </c>
       <c r="F15" s="4" t="s">
-        <v>51</v>
+        <v>21</v>
       </c>
       <c r="G15" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="H15" s="4" t="s">
-        <v>17</v>
-      </c>
+        <v>48</v>
+      </c>
+      <c r="H15" s="4"/>
       <c r="I15" s="4"/>
       <c r="J15" s="4"/>
       <c r="K15" s="4"/>
-      <c r="L15" s="4"/>
+      <c r="L15" s="4" t="s">
+        <v>51</v>
+      </c>
       <c r="M15" s="4" t="s">
         <v>18</v>
       </c>
@@ -2020,12 +2028,14 @@
         <v>23</v>
       </c>
       <c r="E17" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="F17" s="4" t="s">
         <v>55</v>
       </c>
-      <c r="F17" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="G17" s="4"/>
+      <c r="G17" s="4" t="s">
+        <v>24</v>
+      </c>
       <c r="H17" s="4" t="s">
         <v>17</v>
       </c>
@@ -2068,10 +2078,10 @@
         <v>23</v>
       </c>
       <c r="E18" s="4" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="F18" s="4" t="s">
-        <v>57</v>
+        <v>21</v>
       </c>
       <c r="G18" s="4"/>
       <c r="H18" s="4" t="s">
@@ -2106,49 +2116,42 @@
       <c r="AG18" s="3"/>
       <c r="AH18" s="3"/>
     </row>
-    <row r="19" spans="2:34">
-      <c r="B19" s="2" t="s">
+    <row r="19" spans="1:34">
+      <c r="A19" s="3"/>
+      <c r="B19" s="4" t="s">
         <v>58</v>
       </c>
-      <c r="C19" s="2" t="s">
+      <c r="C19" s="2"/>
+      <c r="D19" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="E19" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="F19" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="D19" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="E19" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="F19" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="G19" s="2" t="s">
-        <v>24</v>
-      </c>
+      <c r="G19" s="4"/>
       <c r="H19" s="4" t="s">
-        <v>60</v>
-      </c>
-      <c r="I19" s="4" t="s">
-        <v>61</v>
-      </c>
-      <c r="J19" s="4" t="s">
-        <v>62</v>
-      </c>
-      <c r="K19" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="L19" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="M19" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="N19" s="2"/>
-      <c r="O19" s="2"/>
-      <c r="P19" s="2"/>
-      <c r="Q19" s="2"/>
-      <c r="R19" s="2"/>
-      <c r="S19" s="2"/>
+        <v>17</v>
+      </c>
+      <c r="I19" s="4"/>
+      <c r="J19" s="4"/>
+      <c r="K19" s="4"/>
+      <c r="L19" s="4"/>
+      <c r="M19" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="N19" s="4"/>
+      <c r="O19" s="4"/>
+      <c r="P19" s="4"/>
+      <c r="Q19" s="4"/>
+      <c r="R19" s="4"/>
+      <c r="S19" s="4"/>
+      <c r="T19" s="3"/>
+      <c r="U19" s="3"/>
+      <c r="V19" s="3"/>
+      <c r="W19" s="3"/>
       <c r="X19" s="3"/>
       <c r="Y19" s="3"/>
       <c r="Z19" s="3"/>
@@ -2161,30 +2164,49 @@
       <c r="AG19" s="3"/>
       <c r="AH19" s="3"/>
     </row>
-    <row r="20" spans="1:34">
-      <c r="A20" s="3"/>
-      <c r="B20" s="4"/>
-      <c r="C20" s="4"/>
-      <c r="D20" s="4"/>
-      <c r="E20" s="4"/>
-      <c r="F20" s="4"/>
-      <c r="G20" s="4"/>
-      <c r="H20" s="4"/>
-      <c r="I20" s="4"/>
-      <c r="J20" s="4"/>
-      <c r="K20" s="4"/>
-      <c r="L20" s="4"/>
-      <c r="M20" s="4"/>
-      <c r="N20" s="4"/>
-      <c r="O20" s="4"/>
-      <c r="P20" s="4"/>
-      <c r="Q20" s="4"/>
-      <c r="R20" s="4"/>
-      <c r="S20" s="4"/>
-      <c r="T20" s="3"/>
-      <c r="U20" s="3"/>
-      <c r="V20" s="3"/>
-      <c r="W20" s="3"/>
+    <row r="20" spans="2:34">
+      <c r="B20" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="E20" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="F20" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="G20" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="H20" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="I20" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="J20" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="K20" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="L20" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="M20" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="N20" s="2"/>
+      <c r="O20" s="2"/>
+      <c r="P20" s="2"/>
+      <c r="Q20" s="2"/>
+      <c r="R20" s="2"/>
+      <c r="S20" s="2"/>
       <c r="X20" s="3"/>
       <c r="Y20" s="3"/>
       <c r="Z20" s="3"/>
@@ -2197,7 +2219,7 @@
       <c r="AG20" s="3"/>
       <c r="AH20" s="3"/>
     </row>
-    <row r="21" s="1" customFormat="1" spans="1:34">
+    <row r="21" spans="1:34">
       <c r="A21" s="3"/>
       <c r="B21" s="4"/>
       <c r="C21" s="4"/>
@@ -2269,7 +2291,7 @@
       <c r="AG22" s="3"/>
       <c r="AH22" s="3"/>
     </row>
-    <row r="23" spans="1:34">
+    <row r="23" s="1" customFormat="1" spans="1:34">
       <c r="A23" s="3"/>
       <c r="B23" s="4"/>
       <c r="C23" s="4"/>
@@ -2814,7 +2836,7 @@
       <c r="B38" s="4"/>
       <c r="C38" s="4"/>
       <c r="D38" s="4"/>
-      <c r="E38" s="5"/>
+      <c r="E38" s="4"/>
       <c r="F38" s="4"/>
       <c r="G38" s="4"/>
       <c r="H38" s="4"/>
@@ -2922,7 +2944,7 @@
       <c r="B41" s="4"/>
       <c r="C41" s="4"/>
       <c r="D41" s="4"/>
-      <c r="E41" s="4"/>
+      <c r="E41" s="5"/>
       <c r="F41" s="4"/>
       <c r="G41" s="4"/>
       <c r="H41" s="4"/>
@@ -3066,7 +3088,7 @@
       <c r="B45" s="4"/>
       <c r="C45" s="4"/>
       <c r="D45" s="4"/>
-      <c r="E45" s="5"/>
+      <c r="E45" s="4"/>
       <c r="F45" s="4"/>
       <c r="G45" s="4"/>
       <c r="H45" s="4"/>
@@ -3102,7 +3124,7 @@
       <c r="B46" s="4"/>
       <c r="C46" s="4"/>
       <c r="D46" s="4"/>
-      <c r="E46" s="4"/>
+      <c r="E46" s="5"/>
       <c r="F46" s="4"/>
       <c r="G46" s="4"/>
       <c r="H46" s="4"/>
@@ -3385,25 +3407,48 @@
       <c r="AG53" s="3"/>
       <c r="AH53" s="3"/>
     </row>
-    <row r="61" spans="1:23">
-      <c r="A61" s="2"/>
-      <c r="B61" s="2"/>
-      <c r="C61" s="2"/>
-      <c r="D61" s="2"/>
-      <c r="R61" s="2"/>
-      <c r="T61" s="2"/>
-      <c r="U61" s="2"/>
-      <c r="V61" s="2"/>
-      <c r="W61" s="2"/>
+    <row r="54" spans="1:34">
+      <c r="A54" s="3"/>
+      <c r="B54" s="4"/>
+      <c r="C54" s="4"/>
+      <c r="D54" s="4"/>
+      <c r="E54" s="4"/>
+      <c r="F54" s="4"/>
+      <c r="G54" s="4"/>
+      <c r="H54" s="4"/>
+      <c r="I54" s="4"/>
+      <c r="J54" s="4"/>
+      <c r="K54" s="4"/>
+      <c r="L54" s="4"/>
+      <c r="M54" s="4"/>
+      <c r="N54" s="4"/>
+      <c r="O54" s="4"/>
+      <c r="P54" s="4"/>
+      <c r="Q54" s="4"/>
+      <c r="R54" s="4"/>
+      <c r="S54" s="4"/>
+      <c r="T54" s="3"/>
+      <c r="U54" s="3"/>
+      <c r="V54" s="3"/>
+      <c r="W54" s="3"/>
+      <c r="X54" s="3"/>
+      <c r="Y54" s="3"/>
+      <c r="Z54" s="3"/>
+      <c r="AA54" s="3"/>
+      <c r="AB54" s="3"/>
+      <c r="AC54" s="3"/>
+      <c r="AD54" s="3"/>
+      <c r="AE54" s="3"/>
+      <c r="AF54" s="3"/>
+      <c r="AG54" s="3"/>
+      <c r="AH54" s="3"/>
     </row>
     <row r="62" spans="1:23">
       <c r="A62" s="2"/>
       <c r="B62" s="2"/>
       <c r="C62" s="2"/>
       <c r="D62" s="2"/>
-      <c r="E62" s="2"/>
       <c r="R62" s="2"/>
-      <c r="S62" s="2"/>
       <c r="T62" s="2"/>
       <c r="U62" s="2"/>
       <c r="V62" s="2"/>
@@ -3414,6 +3459,7 @@
       <c r="B63" s="2"/>
       <c r="C63" s="2"/>
       <c r="D63" s="2"/>
+      <c r="E63" s="2"/>
       <c r="R63" s="2"/>
       <c r="S63" s="2"/>
       <c r="T63" s="2"/>
@@ -3553,39 +3599,51 @@
       <c r="V74" s="2"/>
       <c r="W74" s="2"/>
     </row>
+    <row r="75" spans="1:23">
+      <c r="A75" s="2"/>
+      <c r="B75" s="2"/>
+      <c r="C75" s="2"/>
+      <c r="D75" s="2"/>
+      <c r="R75" s="2"/>
+      <c r="S75" s="2"/>
+      <c r="T75" s="2"/>
+      <c r="U75" s="2"/>
+      <c r="V75" s="2"/>
+      <c r="W75" s="2"/>
+    </row>
   </sheetData>
   <dataValidations count="11">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L5 L6 L9 L12 L13 L14 L15 L16 L17 L18 L2:L4 L7:L8 L10:L11 L19:L1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L5 L6 L9 L12 L13 L14 L15 L16 L17 L18 L19 L2:L4 L7:L8 L10:L11 L20:L1048576">
       <formula1>"BR_EQ,BR_NE,BR_LTU,BR_GE,BR_GEU,BR_LT,BR_XX"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J5 J6 J7 J8 J9 J10 J11 J12 J13 J14 J15 J16 J17 J18 J2:J4 J19:J1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J5 J6 J7 J8 J9 J10 J11 J12 J13 J14 J15 J16 J17 J18 J19 J2:J4 J20:J1048576">
       <formula1>"ST_SW,ST_SH,ST_SB,ST_XX"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K4 K5 K6 K7 K8 K9 K10 K11 K12 K13 K14 K15 K16 K17 K18 K2:K3 K19:K1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H5 H6 H7 H8 H9 H12 H13 H14 H15 H16 H17 H18 H19 H2:H4 H10:H11 H20:H1048576">
+      <formula1>"WB_ALU,WB_MEM,WB_PC4,WB_XX"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="M4 M5 M6 M7 M8 M9 M10 M11 M12 M13 M14 M15 M16 M17 M18 M19 M2:M3 M20:M1048576">
+      <formula1>"INST_VALID,INST_INVALID"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K4 K5 K6 K7 K8 K9 K10 K11 K12 K13 K14 K15 K16 K17 K18 K19 K2:K3 K20:K1048576">
       <formula1>"MASK_XX,MASK_B,MASK_H,MASK_W,MASK_D"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="M4 M5 M6 M7 M8 M9 M10 M11 M12 M13 M14 M15 M16 M17 M18 M2:M3 M19:M1048576">
-      <formula1>"INST_VALID,INST_INVALID"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I4 I5 I6 I7 I8 I9 I10 I11 I12 I13 I14 I15 I16 I17 I18 I2:I3 I19:I1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I4 I5 I6 I7 I8 I9 I10 I11 I12 I13 I14 I15 I16 I17 I18 I19 I2:I3 I20:I1048576">
       <formula1>"LD_LB,LD_LH,LD_LW,LD_LBU,LD_LHU,LD_XX"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G4 G5 G6 G7 G8 G9 G10 G11 G12 G13 G14 G15 G16 G17 G18 G2:G3 G19:G1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F4 F5 F6 F7 F8 F9 F10 F11 F12 F13 F14 F15 F16 F17 F18 F19 F2:F3 F20:F1048576">
+      <formula1>"ALU_ADD,ALU_SUB,ALU_AND,ALU_OR,ALU_XOR,ALU_SLL,ALU_SRL,ALU_SLT,ALU_SLTU,ALU_COPY_A,ALU_COPY_B"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E4 E5 E6 E7 E8 E9 E10 E11 E12 E13 E14 E15 E16 E17 E18 E19 E2:E3 E20:E1048576">
+      <formula1>"B_IMM,B_RS2"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G4 G5 G6 G7 G8 G9 G10 G11 G12 G13 G14 G15 G16 G17 G18 G19 G2:G3 G20:G1048576">
       <formula1>"IMM_I,IMM_J,IMM_U,IMM_S,IMM_B"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F4 F5 F6 F7 F8 F9 F10 F11 F12 F13 F14 F15 F16 F17 F18 F2:F3 F19:F1048576">
-      <formula1>"ALU_ADD,ALU_SUB,ALU_AND,ALU_OR,ALU_XOR,ALU_SLL,ALU_SRL,ALU_SLT,ALU_SLTU,ALU_COPY_A,ALU_COPY_B"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H5 H6 H7 H8 H9 H12 H13 H14 H15 H16 H17 H18 H2:H4 H10:H11 H19:H1048576">
-      <formula1>"WB_ALU,WB_MEM,WB_PC4,WB_XX"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D4 D5 D6 D7 D8 D9 D10 D11 D12 D13 D14 D15 D16 D17 D18 D2:D3 D19:D1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D4 D5 D6 D7 D8 D9 D10 D11 D12 D13 D14 D15 D16 D17 D18 D19 D2:D3 D20:D1048576">
       <formula1>"A_PC,A_RS1"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E4 E5 E6 E7 E8 E9 E10 E11 E12 E13 E14 E15 E16 E17 E18 E2:E3 E19:E1048576">
-      <formula1>"B_IMM,B_RS2"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C4 C5 C6 C7 C8 C9 C10 C11 C12 C13 C14 C15 C16 C17 C18 C2:C3 C19:C1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C4 C5 C6 C7 C8 C9 C10 C11 C12 C13 C14 C15 C16 C17 C18 C19 C2:C3 C20:C1048576">
       <formula1>"PC_4,PC_0,PC_ALU"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
> sim RTL ysyx_23060246 韩炳晋 Linux archlinux 6.6.60-1-lts #1 SMP PREEMPT_DYNAMIC Fri, 08 Nov 2024 16:03:02 +0000 x86_64 GNU/Linux  19:38:16 up 1 day,  1:53,  2 users,  load average: 3.62, 2.16, 1.82
</commit_message>
<xml_diff>
--- a/npc/tools/control_gen/control_table.xlsx
+++ b/npc/tools/control_gen/control_table.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="154" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="162" uniqueCount="70">
   <si>
     <t>comment</t>
   </si>
@@ -170,6 +170,12 @@
   </si>
   <si>
     <t>BR_GEU</t>
+  </si>
+  <si>
+    <t>bge</t>
+  </si>
+  <si>
+    <t>BR_GE</t>
   </si>
   <si>
     <t>slli</t>
@@ -1186,7 +1192,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:AH75"/>
+  <dimension ref="A1:AH76"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
     <col min="1" max="1" width="13.1" customWidth="1"/>
@@ -1973,26 +1979,28 @@
       <c r="B16" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="C16" s="2"/>
+      <c r="C16" s="2" t="s">
+        <v>30</v>
+      </c>
       <c r="D16" s="4" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="E16" s="4" t="s">
         <v>14</v>
       </c>
       <c r="F16" s="4" t="s">
-        <v>53</v>
+        <v>21</v>
       </c>
       <c r="G16" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="H16" s="4" t="s">
-        <v>17</v>
-      </c>
+        <v>48</v>
+      </c>
+      <c r="H16" s="4"/>
       <c r="I16" s="4"/>
       <c r="J16" s="4"/>
       <c r="K16" s="4"/>
-      <c r="L16" s="4"/>
+      <c r="L16" s="4" t="s">
+        <v>53</v>
+      </c>
       <c r="M16" s="4" t="s">
         <v>18</v>
       </c>
@@ -2078,12 +2086,14 @@
         <v>23</v>
       </c>
       <c r="E18" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="F18" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="F18" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="G18" s="4"/>
+      <c r="G18" s="4" t="s">
+        <v>24</v>
+      </c>
       <c r="H18" s="4" t="s">
         <v>17</v>
       </c>
@@ -2126,10 +2136,10 @@
         <v>23</v>
       </c>
       <c r="E19" s="4" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="F19" s="4" t="s">
-        <v>59</v>
+        <v>21</v>
       </c>
       <c r="G19" s="4"/>
       <c r="H19" s="4" t="s">
@@ -2164,49 +2174,42 @@
       <c r="AG19" s="3"/>
       <c r="AH19" s="3"/>
     </row>
-    <row r="20" spans="2:34">
-      <c r="B20" s="2" t="s">
+    <row r="20" spans="1:34">
+      <c r="A20" s="3"/>
+      <c r="B20" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="C20" s="2" t="s">
+      <c r="C20" s="2"/>
+      <c r="D20" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="E20" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="F20" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="D20" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="E20" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="F20" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="G20" s="2" t="s">
-        <v>24</v>
-      </c>
+      <c r="G20" s="4"/>
       <c r="H20" s="4" t="s">
-        <v>62</v>
-      </c>
-      <c r="I20" s="4" t="s">
-        <v>63</v>
-      </c>
-      <c r="J20" s="4" t="s">
-        <v>64</v>
-      </c>
-      <c r="K20" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="L20" s="2" t="s">
-        <v>66</v>
-      </c>
-      <c r="M20" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="N20" s="2"/>
-      <c r="O20" s="2"/>
-      <c r="P20" s="2"/>
-      <c r="Q20" s="2"/>
-      <c r="R20" s="2"/>
-      <c r="S20" s="2"/>
+        <v>17</v>
+      </c>
+      <c r="I20" s="4"/>
+      <c r="J20" s="4"/>
+      <c r="K20" s="4"/>
+      <c r="L20" s="4"/>
+      <c r="M20" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="N20" s="4"/>
+      <c r="O20" s="4"/>
+      <c r="P20" s="4"/>
+      <c r="Q20" s="4"/>
+      <c r="R20" s="4"/>
+      <c r="S20" s="4"/>
+      <c r="T20" s="3"/>
+      <c r="U20" s="3"/>
+      <c r="V20" s="3"/>
+      <c r="W20" s="3"/>
       <c r="X20" s="3"/>
       <c r="Y20" s="3"/>
       <c r="Z20" s="3"/>
@@ -2219,30 +2222,49 @@
       <c r="AG20" s="3"/>
       <c r="AH20" s="3"/>
     </row>
-    <row r="21" spans="1:34">
-      <c r="A21" s="3"/>
-      <c r="B21" s="4"/>
-      <c r="C21" s="4"/>
-      <c r="D21" s="4"/>
-      <c r="E21" s="4"/>
-      <c r="F21" s="4"/>
-      <c r="G21" s="4"/>
-      <c r="H21" s="4"/>
-      <c r="I21" s="4"/>
-      <c r="J21" s="4"/>
-      <c r="K21" s="4"/>
-      <c r="L21" s="4"/>
-      <c r="M21" s="4"/>
-      <c r="N21" s="4"/>
-      <c r="O21" s="4"/>
-      <c r="P21" s="4"/>
-      <c r="Q21" s="4"/>
-      <c r="R21" s="4"/>
-      <c r="S21" s="4"/>
-      <c r="T21" s="3"/>
-      <c r="U21" s="3"/>
-      <c r="V21" s="3"/>
-      <c r="W21" s="3"/>
+    <row r="21" spans="2:34">
+      <c r="B21" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="D21" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="E21" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="F21" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="G21" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="H21" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="I21" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="J21" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="K21" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="L21" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="M21" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="N21" s="2"/>
+      <c r="O21" s="2"/>
+      <c r="P21" s="2"/>
+      <c r="Q21" s="2"/>
+      <c r="R21" s="2"/>
+      <c r="S21" s="2"/>
       <c r="X21" s="3"/>
       <c r="Y21" s="3"/>
       <c r="Z21" s="3"/>
@@ -2255,7 +2277,7 @@
       <c r="AG21" s="3"/>
       <c r="AH21" s="3"/>
     </row>
-    <row r="22" s="1" customFormat="1" spans="1:34">
+    <row r="22" spans="1:34">
       <c r="A22" s="3"/>
       <c r="B22" s="4"/>
       <c r="C22" s="4"/>
@@ -2327,7 +2349,7 @@
       <c r="AG23" s="3"/>
       <c r="AH23" s="3"/>
     </row>
-    <row r="24" spans="1:34">
+    <row r="24" s="1" customFormat="1" spans="1:34">
       <c r="A24" s="3"/>
       <c r="B24" s="4"/>
       <c r="C24" s="4"/>
@@ -2872,7 +2894,7 @@
       <c r="B39" s="4"/>
       <c r="C39" s="4"/>
       <c r="D39" s="4"/>
-      <c r="E39" s="5"/>
+      <c r="E39" s="4"/>
       <c r="F39" s="4"/>
       <c r="G39" s="4"/>
       <c r="H39" s="4"/>
@@ -2980,7 +3002,7 @@
       <c r="B42" s="4"/>
       <c r="C42" s="4"/>
       <c r="D42" s="4"/>
-      <c r="E42" s="4"/>
+      <c r="E42" s="5"/>
       <c r="F42" s="4"/>
       <c r="G42" s="4"/>
       <c r="H42" s="4"/>
@@ -3124,7 +3146,7 @@
       <c r="B46" s="4"/>
       <c r="C46" s="4"/>
       <c r="D46" s="4"/>
-      <c r="E46" s="5"/>
+      <c r="E46" s="4"/>
       <c r="F46" s="4"/>
       <c r="G46" s="4"/>
       <c r="H46" s="4"/>
@@ -3160,7 +3182,7 @@
       <c r="B47" s="4"/>
       <c r="C47" s="4"/>
       <c r="D47" s="4"/>
-      <c r="E47" s="4"/>
+      <c r="E47" s="5"/>
       <c r="F47" s="4"/>
       <c r="G47" s="4"/>
       <c r="H47" s="4"/>
@@ -3443,25 +3465,48 @@
       <c r="AG54" s="3"/>
       <c r="AH54" s="3"/>
     </row>
-    <row r="62" spans="1:23">
-      <c r="A62" s="2"/>
-      <c r="B62" s="2"/>
-      <c r="C62" s="2"/>
-      <c r="D62" s="2"/>
-      <c r="R62" s="2"/>
-      <c r="T62" s="2"/>
-      <c r="U62" s="2"/>
-      <c r="V62" s="2"/>
-      <c r="W62" s="2"/>
+    <row r="55" spans="1:34">
+      <c r="A55" s="3"/>
+      <c r="B55" s="4"/>
+      <c r="C55" s="4"/>
+      <c r="D55" s="4"/>
+      <c r="E55" s="4"/>
+      <c r="F55" s="4"/>
+      <c r="G55" s="4"/>
+      <c r="H55" s="4"/>
+      <c r="I55" s="4"/>
+      <c r="J55" s="4"/>
+      <c r="K55" s="4"/>
+      <c r="L55" s="4"/>
+      <c r="M55" s="4"/>
+      <c r="N55" s="4"/>
+      <c r="O55" s="4"/>
+      <c r="P55" s="4"/>
+      <c r="Q55" s="4"/>
+      <c r="R55" s="4"/>
+      <c r="S55" s="4"/>
+      <c r="T55" s="3"/>
+      <c r="U55" s="3"/>
+      <c r="V55" s="3"/>
+      <c r="W55" s="3"/>
+      <c r="X55" s="3"/>
+      <c r="Y55" s="3"/>
+      <c r="Z55" s="3"/>
+      <c r="AA55" s="3"/>
+      <c r="AB55" s="3"/>
+      <c r="AC55" s="3"/>
+      <c r="AD55" s="3"/>
+      <c r="AE55" s="3"/>
+      <c r="AF55" s="3"/>
+      <c r="AG55" s="3"/>
+      <c r="AH55" s="3"/>
     </row>
     <row r="63" spans="1:23">
       <c r="A63" s="2"/>
       <c r="B63" s="2"/>
       <c r="C63" s="2"/>
       <c r="D63" s="2"/>
-      <c r="E63" s="2"/>
       <c r="R63" s="2"/>
-      <c r="S63" s="2"/>
       <c r="T63" s="2"/>
       <c r="U63" s="2"/>
       <c r="V63" s="2"/>
@@ -3472,6 +3517,7 @@
       <c r="B64" s="2"/>
       <c r="C64" s="2"/>
       <c r="D64" s="2"/>
+      <c r="E64" s="2"/>
       <c r="R64" s="2"/>
       <c r="S64" s="2"/>
       <c r="T64" s="2"/>
@@ -3611,39 +3657,51 @@
       <c r="V75" s="2"/>
       <c r="W75" s="2"/>
     </row>
+    <row r="76" spans="1:23">
+      <c r="A76" s="2"/>
+      <c r="B76" s="2"/>
+      <c r="C76" s="2"/>
+      <c r="D76" s="2"/>
+      <c r="R76" s="2"/>
+      <c r="S76" s="2"/>
+      <c r="T76" s="2"/>
+      <c r="U76" s="2"/>
+      <c r="V76" s="2"/>
+      <c r="W76" s="2"/>
+    </row>
   </sheetData>
   <dataValidations count="11">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L5 L6 L9 L12 L13 L14 L15 L16 L17 L18 L19 L2:L4 L7:L8 L10:L11 L20:L1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L5 L6 L9 L12 L13 L14 L15 L16 L17 L18 L19 L20 L2:L4 L7:L8 L10:L11 L21:L1048576">
       <formula1>"BR_EQ,BR_NE,BR_LTU,BR_GE,BR_GEU,BR_LT,BR_XX"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J5 J6 J7 J8 J9 J10 J11 J12 J13 J14 J15 J16 J17 J18 J19 J2:J4 J20:J1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J5 J6 J7 J8 J9 J10 J11 J12 J13 J14 J15 J16 J17 J18 J19 J20 J2:J4 J21:J1048576">
       <formula1>"ST_SW,ST_SH,ST_SB,ST_XX"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H5 H6 H7 H8 H9 H12 H13 H14 H15 H16 H17 H18 H19 H2:H4 H10:H11 H20:H1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H5 H6 H7 H8 H9 H12 H13 H14 H15 H16 H17 H18 H19 H20 H2:H4 H10:H11 H21:H1048576">
       <formula1>"WB_ALU,WB_MEM,WB_PC4,WB_XX"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="M4 M5 M6 M7 M8 M9 M10 M11 M12 M13 M14 M15 M16 M17 M18 M19 M2:M3 M20:M1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="M4 M5 M6 M7 M8 M9 M10 M11 M12 M13 M14 M15 M16 M17 M18 M19 M20 M2:M3 M21:M1048576">
       <formula1>"INST_VALID,INST_INVALID"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K4 K5 K6 K7 K8 K9 K10 K11 K12 K13 K14 K15 K16 K17 K18 K19 K2:K3 K20:K1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K4 K5 K6 K7 K8 K9 K10 K11 K12 K13 K14 K15 K16 K17 K18 K19 K20 K2:K3 K21:K1048576">
       <formula1>"MASK_XX,MASK_B,MASK_H,MASK_W,MASK_D"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I4 I5 I6 I7 I8 I9 I10 I11 I12 I13 I14 I15 I16 I17 I18 I19 I2:I3 I20:I1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I4 I5 I6 I7 I8 I9 I10 I11 I12 I13 I14 I15 I16 I17 I18 I19 I20 I2:I3 I21:I1048576">
       <formula1>"LD_LB,LD_LH,LD_LW,LD_LBU,LD_LHU,LD_XX"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F4 F5 F6 F7 F8 F9 F10 F11 F12 F13 F14 F15 F16 F17 F18 F19 F2:F3 F20:F1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F4 F5 F6 F7 F8 F9 F10 F11 F12 F13 F14 F15 F16 F17 F18 F19 F20 F2:F3 F21:F1048576">
       <formula1>"ALU_ADD,ALU_SUB,ALU_AND,ALU_OR,ALU_XOR,ALU_SLL,ALU_SRL,ALU_SLT,ALU_SLTU,ALU_COPY_A,ALU_COPY_B"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E4 E5 E6 E7 E8 E9 E10 E11 E12 E13 E14 E15 E16 E17 E18 E19 E2:E3 E20:E1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E4 E5 E6 E7 E8 E9 E10 E11 E12 E13 E14 E15 E16 E17 E18 E19 E20 E2:E3 E21:E1048576">
       <formula1>"B_IMM,B_RS2"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G4 G5 G6 G7 G8 G9 G10 G11 G12 G13 G14 G15 G16 G17 G18 G19 G2:G3 G20:G1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G4 G5 G6 G7 G8 G9 G10 G11 G12 G13 G14 G15 G16 G17 G18 G19 G20 G2:G3 G21:G1048576">
       <formula1>"IMM_I,IMM_J,IMM_U,IMM_S,IMM_B"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D4 D5 D6 D7 D8 D9 D10 D11 D12 D13 D14 D15 D16 D17 D18 D19 D2:D3 D20:D1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D4 D5 D6 D7 D8 D9 D10 D11 D12 D13 D14 D15 D16 D17 D18 D19 D20 D2:D3 D21:D1048576">
       <formula1>"A_PC,A_RS1"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C4 C5 C6 C7 C8 C9 C10 C11 C12 C13 C14 C15 C16 C17 C18 C19 C2:C3 C20:C1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C4 C5 C6 C7 C8 C9 C10 C11 C12 C13 C14 C15 C16 C17 C18 C19 C20 C2:C3 C21:C1048576">
       <formula1>"PC_4,PC_0,PC_ALU"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
> sim RTL ysyx_23060246 韩炳晋 Linux archlinux 6.6.60-1-lts #1 SMP PREEMPT_DYNAMIC Fri, 08 Nov 2024 16:03:02 +0000 x86_64 GNU/Linux  20:00:18 up 1 day,  2:15,  2 users,  load average: 3.22, 2.75, 2.48
</commit_message>
<xml_diff>
--- a/npc/tools/control_gen/control_table.xlsx
+++ b/npc/tools/control_gen/control_table.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="162" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="164" uniqueCount="71">
   <si>
     <t>comment</t>
   </si>
@@ -140,6 +140,9 @@
   </si>
   <si>
     <t>lw</t>
+  </si>
+  <si>
+    <t>WB_MEM</t>
   </si>
   <si>
     <t>LD_LW</t>
@@ -1738,9 +1741,11 @@
       <c r="G11" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="H11" s="4"/>
+      <c r="H11" s="4" t="s">
+        <v>42</v>
+      </c>
       <c r="I11" s="4" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="J11" s="4"/>
       <c r="K11" s="4"/>
@@ -1773,7 +1778,7 @@
     <row r="12" spans="1:34">
       <c r="A12" s="3"/>
       <c r="B12" s="4" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C12" s="2"/>
       <c r="D12" s="4" t="s">
@@ -1788,9 +1793,11 @@
       <c r="G12" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="H12" s="4"/>
+      <c r="H12" s="4" t="s">
+        <v>42</v>
+      </c>
       <c r="I12" s="4" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="J12" s="4"/>
       <c r="K12" s="4"/>
@@ -1823,7 +1830,7 @@
     <row r="13" spans="1:34">
       <c r="A13" s="3"/>
       <c r="B13" s="4" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C13" s="2"/>
       <c r="D13" s="4" t="s">
@@ -1840,7 +1847,7 @@
       </c>
       <c r="H13" s="4"/>
       <c r="I13" s="4" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="J13" s="4"/>
       <c r="K13" s="4"/>
@@ -1873,7 +1880,7 @@
     <row r="14" spans="1:34">
       <c r="A14" s="3"/>
       <c r="B14" s="4" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C14" s="2" t="s">
         <v>30</v>
@@ -1888,14 +1895,14 @@
         <v>21</v>
       </c>
       <c r="G14" s="4" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="H14" s="4"/>
       <c r="I14" s="4"/>
       <c r="J14" s="4"/>
       <c r="K14" s="4"/>
       <c r="L14" s="4" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="M14" s="4" t="s">
         <v>18</v>
@@ -1925,7 +1932,7 @@
     <row r="15" spans="1:34">
       <c r="A15" s="3"/>
       <c r="B15" s="4" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C15" s="2" t="s">
         <v>30</v>
@@ -1940,14 +1947,14 @@
         <v>21</v>
       </c>
       <c r="G15" s="4" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="H15" s="4"/>
       <c r="I15" s="4"/>
       <c r="J15" s="4"/>
       <c r="K15" s="4"/>
       <c r="L15" s="4" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="M15" s="4" t="s">
         <v>18</v>
@@ -1977,7 +1984,7 @@
     <row r="16" spans="1:34">
       <c r="A16" s="3"/>
       <c r="B16" s="4" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C16" s="2" t="s">
         <v>30</v>
@@ -1992,14 +1999,14 @@
         <v>21</v>
       </c>
       <c r="G16" s="4" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="H16" s="4"/>
       <c r="I16" s="4"/>
       <c r="J16" s="4"/>
       <c r="K16" s="4"/>
       <c r="L16" s="4" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="M16" s="4" t="s">
         <v>18</v>
@@ -2029,7 +2036,7 @@
     <row r="17" spans="1:34">
       <c r="A17" s="3"/>
       <c r="B17" s="4" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C17" s="2"/>
       <c r="D17" s="4" t="s">
@@ -2039,7 +2046,7 @@
         <v>14</v>
       </c>
       <c r="F17" s="4" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="G17" s="4" t="s">
         <v>24</v>
@@ -2079,7 +2086,7 @@
     <row r="18" spans="1:34">
       <c r="A18" s="3"/>
       <c r="B18" s="4" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C18" s="2"/>
       <c r="D18" s="4" t="s">
@@ -2089,7 +2096,7 @@
         <v>14</v>
       </c>
       <c r="F18" s="4" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="G18" s="4" t="s">
         <v>24</v>
@@ -2129,14 +2136,14 @@
     <row r="19" spans="1:34">
       <c r="A19" s="3"/>
       <c r="B19" s="4" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C19" s="2"/>
       <c r="D19" s="4" t="s">
         <v>23</v>
       </c>
       <c r="E19" s="4" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="F19" s="4" t="s">
         <v>21</v>
@@ -2177,17 +2184,17 @@
     <row r="20" spans="1:34">
       <c r="A20" s="3"/>
       <c r="B20" s="4" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C20" s="2"/>
       <c r="D20" s="4" t="s">
         <v>23</v>
       </c>
       <c r="E20" s="4" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="F20" s="4" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="G20" s="4"/>
       <c r="H20" s="4" t="s">
@@ -2224,10 +2231,10 @@
     </row>
     <row r="21" spans="2:34">
       <c r="B21" s="2" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="D21" s="2" t="s">
         <v>23</v>
@@ -2242,22 +2249,22 @@
         <v>24</v>
       </c>
       <c r="H21" s="4" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="I21" s="4" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="J21" s="4" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="K21" s="2" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="L21" s="2" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="M21" s="2" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="N21" s="2"/>
       <c r="O21" s="2"/>

</xml_diff>

<commit_message>
> sim RTL ysyx_23060246 韩炳晋 Linux archlinux 6.6.60-1-lts #1 SMP PREEMPT_DYNAMIC Fri, 08 Nov 2024 16:03:02 +0000 x86_64 GNU/Linux  20:17:21 up 1 day,  2:32,  2 users,  load average: 1.73, 1.35, 1.81
</commit_message>
<xml_diff>
--- a/npc/tools/control_gen/control_table.xlsx
+++ b/npc/tools/control_gen/control_table.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="164" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="161" uniqueCount="71">
   <si>
     <t>comment</t>
   </si>
@@ -1882,9 +1882,7 @@
       <c r="B14" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="C14" s="2" t="s">
-        <v>30</v>
-      </c>
+      <c r="C14" s="2"/>
       <c r="D14" s="4" t="s">
         <v>20</v>
       </c>
@@ -1934,9 +1932,7 @@
       <c r="B15" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="C15" s="2" t="s">
-        <v>30</v>
-      </c>
+      <c r="C15" s="2"/>
       <c r="D15" s="4" t="s">
         <v>20</v>
       </c>
@@ -1986,9 +1982,7 @@
       <c r="B16" s="4" t="s">
         <v>53</v>
       </c>
-      <c r="C16" s="2" t="s">
-        <v>30</v>
-      </c>
+      <c r="C16" s="2"/>
       <c r="D16" s="4" t="s">
         <v>20</v>
       </c>

</xml_diff>

<commit_message>
> sim RTL ysyx_23060246 韩炳晋 Linux archlinux 6.6.60-1-lts #1 SMP PREEMPT_DYNAMIC Fri, 08 Nov 2024 16:03:02 +0000 x86_64 GNU/Linux  20:22:04 up 1 day,  2:37,  2 users,  load average: 1.12, 1.14, 1.60
</commit_message>
<xml_diff>
--- a/npc/tools/control_gen/control_table.xlsx
+++ b/npc/tools/control_gen/control_table.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="161" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="177" uniqueCount="76">
   <si>
     <t>comment</t>
   </si>
@@ -130,6 +130,15 @@
     <t>MASK_B</t>
   </si>
   <si>
+    <t>sh</t>
+  </si>
+  <si>
+    <t>ST_SH</t>
+  </si>
+  <si>
+    <t>MASK_H</t>
+  </si>
+  <si>
     <t>sw</t>
   </si>
   <si>
@@ -146,6 +155,12 @@
   </si>
   <si>
     <t>LD_LW</t>
+  </si>
+  <si>
+    <t>lhu</t>
+  </si>
+  <si>
+    <t>LD_LHU</t>
   </si>
   <si>
     <t>lb</t>
@@ -1195,7 +1210,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:AH76"/>
+  <dimension ref="A1:AH78"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
     <col min="1" max="1" width="13.1" customWidth="1"/>
@@ -1739,16 +1754,16 @@
         <v>21</v>
       </c>
       <c r="G11" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="H11" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="H11" s="4"/>
+      <c r="I11" s="4"/>
+      <c r="J11" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="I11" s="4" t="s">
+      <c r="K11" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="J11" s="4"/>
-      <c r="K11" s="4"/>
       <c r="L11" s="4"/>
       <c r="M11" s="4" t="s">
         <v>18</v>
@@ -1794,10 +1809,10 @@
         <v>24</v>
       </c>
       <c r="H12" s="4" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="I12" s="4" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="J12" s="4"/>
       <c r="K12" s="4"/>
@@ -1830,7 +1845,7 @@
     <row r="13" spans="1:34">
       <c r="A13" s="3"/>
       <c r="B13" s="4" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C13" s="2"/>
       <c r="D13" s="4" t="s">
@@ -1845,9 +1860,11 @@
       <c r="G13" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="H13" s="4"/>
+      <c r="H13" s="4" t="s">
+        <v>45</v>
+      </c>
       <c r="I13" s="4" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="J13" s="4"/>
       <c r="K13" s="4"/>
@@ -1880,11 +1897,11 @@
     <row r="14" spans="1:34">
       <c r="A14" s="3"/>
       <c r="B14" s="4" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C14" s="2"/>
       <c r="D14" s="4" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="E14" s="4" t="s">
         <v>14</v>
@@ -1893,15 +1910,17 @@
         <v>21</v>
       </c>
       <c r="G14" s="4" t="s">
-        <v>49</v>
-      </c>
-      <c r="H14" s="4"/>
-      <c r="I14" s="4"/>
+        <v>24</v>
+      </c>
+      <c r="H14" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="I14" s="4" t="s">
+        <v>50</v>
+      </c>
       <c r="J14" s="4"/>
       <c r="K14" s="4"/>
-      <c r="L14" s="4" t="s">
-        <v>50</v>
-      </c>
+      <c r="L14" s="4"/>
       <c r="M14" s="4" t="s">
         <v>18</v>
       </c>
@@ -1934,7 +1953,7 @@
       </c>
       <c r="C15" s="2"/>
       <c r="D15" s="4" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="E15" s="4" t="s">
         <v>14</v>
@@ -1943,15 +1962,15 @@
         <v>21</v>
       </c>
       <c r="G15" s="4" t="s">
-        <v>49</v>
+        <v>24</v>
       </c>
       <c r="H15" s="4"/>
-      <c r="I15" s="4"/>
+      <c r="I15" s="4" t="s">
+        <v>52</v>
+      </c>
       <c r="J15" s="4"/>
       <c r="K15" s="4"/>
-      <c r="L15" s="4" t="s">
-        <v>52</v>
-      </c>
+      <c r="L15" s="4"/>
       <c r="M15" s="4" t="s">
         <v>18</v>
       </c>
@@ -1993,14 +2012,14 @@
         <v>21</v>
       </c>
       <c r="G16" s="4" t="s">
-        <v>49</v>
+        <v>54</v>
       </c>
       <c r="H16" s="4"/>
       <c r="I16" s="4"/>
       <c r="J16" s="4"/>
       <c r="K16" s="4"/>
       <c r="L16" s="4" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="M16" s="4" t="s">
         <v>18</v>
@@ -2030,28 +2049,28 @@
     <row r="17" spans="1:34">
       <c r="A17" s="3"/>
       <c r="B17" s="4" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C17" s="2"/>
       <c r="D17" s="4" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="E17" s="4" t="s">
         <v>14</v>
       </c>
       <c r="F17" s="4" t="s">
-        <v>56</v>
+        <v>21</v>
       </c>
       <c r="G17" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="H17" s="4" t="s">
-        <v>17</v>
-      </c>
+        <v>54</v>
+      </c>
+      <c r="H17" s="4"/>
       <c r="I17" s="4"/>
       <c r="J17" s="4"/>
       <c r="K17" s="4"/>
-      <c r="L17" s="4"/>
+      <c r="L17" s="4" t="s">
+        <v>57</v>
+      </c>
       <c r="M17" s="4" t="s">
         <v>18</v>
       </c>
@@ -2080,28 +2099,28 @@
     <row r="18" spans="1:34">
       <c r="A18" s="3"/>
       <c r="B18" s="4" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C18" s="2"/>
       <c r="D18" s="4" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="E18" s="4" t="s">
         <v>14</v>
       </c>
       <c r="F18" s="4" t="s">
-        <v>58</v>
+        <v>21</v>
       </c>
       <c r="G18" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="H18" s="4" t="s">
-        <v>17</v>
-      </c>
+        <v>54</v>
+      </c>
+      <c r="H18" s="4"/>
       <c r="I18" s="4"/>
       <c r="J18" s="4"/>
       <c r="K18" s="4"/>
-      <c r="L18" s="4"/>
+      <c r="L18" s="4" t="s">
+        <v>59</v>
+      </c>
       <c r="M18" s="4" t="s">
         <v>18</v>
       </c>
@@ -2130,19 +2149,21 @@
     <row r="19" spans="1:34">
       <c r="A19" s="3"/>
       <c r="B19" s="4" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C19" s="2"/>
       <c r="D19" s="4" t="s">
         <v>23</v>
       </c>
       <c r="E19" s="4" t="s">
-        <v>60</v>
+        <v>14</v>
       </c>
       <c r="F19" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="G19" s="4"/>
+        <v>61</v>
+      </c>
+      <c r="G19" s="4" t="s">
+        <v>24</v>
+      </c>
       <c r="H19" s="4" t="s">
         <v>17</v>
       </c>
@@ -2178,19 +2199,21 @@
     <row r="20" spans="1:34">
       <c r="A20" s="3"/>
       <c r="B20" s="4" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C20" s="2"/>
       <c r="D20" s="4" t="s">
         <v>23</v>
       </c>
       <c r="E20" s="4" t="s">
-        <v>60</v>
+        <v>14</v>
       </c>
       <c r="F20" s="4" t="s">
-        <v>62</v>
-      </c>
-      <c r="G20" s="4"/>
+        <v>63</v>
+      </c>
+      <c r="G20" s="4" t="s">
+        <v>24</v>
+      </c>
       <c r="H20" s="4" t="s">
         <v>17</v>
       </c>
@@ -2223,49 +2246,42 @@
       <c r="AG20" s="3"/>
       <c r="AH20" s="3"/>
     </row>
-    <row r="21" spans="2:34">
-      <c r="B21" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="C21" s="2" t="s">
+    <row r="21" spans="1:34">
+      <c r="A21" s="3"/>
+      <c r="B21" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="D21" s="2" t="s">
+      <c r="C21" s="2"/>
+      <c r="D21" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="E21" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="F21" s="2" t="s">
+      <c r="E21" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="F21" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="G21" s="2" t="s">
-        <v>24</v>
-      </c>
+      <c r="G21" s="4"/>
       <c r="H21" s="4" t="s">
-        <v>65</v>
-      </c>
-      <c r="I21" s="4" t="s">
-        <v>66</v>
-      </c>
-      <c r="J21" s="4" t="s">
-        <v>67</v>
-      </c>
-      <c r="K21" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="L21" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="M21" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="N21" s="2"/>
-      <c r="O21" s="2"/>
-      <c r="P21" s="2"/>
-      <c r="Q21" s="2"/>
-      <c r="R21" s="2"/>
-      <c r="S21" s="2"/>
+        <v>17</v>
+      </c>
+      <c r="I21" s="4"/>
+      <c r="J21" s="4"/>
+      <c r="K21" s="4"/>
+      <c r="L21" s="4"/>
+      <c r="M21" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="N21" s="4"/>
+      <c r="O21" s="4"/>
+      <c r="P21" s="4"/>
+      <c r="Q21" s="4"/>
+      <c r="R21" s="4"/>
+      <c r="S21" s="4"/>
+      <c r="T21" s="3"/>
+      <c r="U21" s="3"/>
+      <c r="V21" s="3"/>
+      <c r="W21" s="3"/>
       <c r="X21" s="3"/>
       <c r="Y21" s="3"/>
       <c r="Z21" s="3"/>
@@ -2280,18 +2296,30 @@
     </row>
     <row r="22" spans="1:34">
       <c r="A22" s="3"/>
-      <c r="B22" s="4"/>
-      <c r="C22" s="4"/>
-      <c r="D22" s="4"/>
-      <c r="E22" s="4"/>
-      <c r="F22" s="4"/>
+      <c r="B22" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="C22" s="2"/>
+      <c r="D22" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="E22" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="F22" s="4" t="s">
+        <v>67</v>
+      </c>
       <c r="G22" s="4"/>
-      <c r="H22" s="4"/>
+      <c r="H22" s="4" t="s">
+        <v>17</v>
+      </c>
       <c r="I22" s="4"/>
       <c r="J22" s="4"/>
       <c r="K22" s="4"/>
       <c r="L22" s="4"/>
-      <c r="M22" s="4"/>
+      <c r="M22" s="4" t="s">
+        <v>18</v>
+      </c>
       <c r="N22" s="4"/>
       <c r="O22" s="4"/>
       <c r="P22" s="4"/>
@@ -2314,30 +2342,49 @@
       <c r="AG22" s="3"/>
       <c r="AH22" s="3"/>
     </row>
-    <row r="23" s="1" customFormat="1" spans="1:34">
-      <c r="A23" s="3"/>
-      <c r="B23" s="4"/>
-      <c r="C23" s="4"/>
-      <c r="D23" s="4"/>
-      <c r="E23" s="4"/>
-      <c r="F23" s="4"/>
-      <c r="G23" s="4"/>
-      <c r="H23" s="4"/>
-      <c r="I23" s="4"/>
-      <c r="J23" s="4"/>
-      <c r="K23" s="4"/>
-      <c r="L23" s="4"/>
-      <c r="M23" s="4"/>
-      <c r="N23" s="4"/>
-      <c r="O23" s="4"/>
-      <c r="P23" s="4"/>
-      <c r="Q23" s="4"/>
-      <c r="R23" s="4"/>
-      <c r="S23" s="4"/>
-      <c r="T23" s="3"/>
-      <c r="U23" s="3"/>
-      <c r="V23" s="3"/>
-      <c r="W23" s="3"/>
+    <row r="23" spans="2:34">
+      <c r="B23" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="C23" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="D23" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="E23" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="F23" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="G23" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="H23" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="I23" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="J23" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="K23" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="L23" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="M23" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="N23" s="2"/>
+      <c r="O23" s="2"/>
+      <c r="P23" s="2"/>
+      <c r="Q23" s="2"/>
+      <c r="R23" s="2"/>
+      <c r="S23" s="2"/>
       <c r="X23" s="3"/>
       <c r="Y23" s="3"/>
       <c r="Z23" s="3"/>
@@ -2350,7 +2397,7 @@
       <c r="AG23" s="3"/>
       <c r="AH23" s="3"/>
     </row>
-    <row r="24" s="1" customFormat="1" spans="1:34">
+    <row r="24" spans="1:34">
       <c r="A24" s="3"/>
       <c r="B24" s="4"/>
       <c r="C24" s="4"/>
@@ -2386,7 +2433,7 @@
       <c r="AG24" s="3"/>
       <c r="AH24" s="3"/>
     </row>
-    <row r="25" spans="1:34">
+    <row r="25" s="1" customFormat="1" spans="1:34">
       <c r="A25" s="3"/>
       <c r="B25" s="4"/>
       <c r="C25" s="4"/>
@@ -2422,7 +2469,7 @@
       <c r="AG25" s="3"/>
       <c r="AH25" s="3"/>
     </row>
-    <row r="26" spans="1:34">
+    <row r="26" s="1" customFormat="1" spans="1:34">
       <c r="A26" s="3"/>
       <c r="B26" s="4"/>
       <c r="C26" s="4"/>
@@ -2931,7 +2978,7 @@
       <c r="B40" s="4"/>
       <c r="C40" s="4"/>
       <c r="D40" s="4"/>
-      <c r="E40" s="5"/>
+      <c r="E40" s="4"/>
       <c r="F40" s="4"/>
       <c r="G40" s="4"/>
       <c r="H40" s="4"/>
@@ -2967,7 +3014,7 @@
       <c r="B41" s="4"/>
       <c r="C41" s="4"/>
       <c r="D41" s="4"/>
-      <c r="E41" s="5"/>
+      <c r="E41" s="4"/>
       <c r="F41" s="4"/>
       <c r="G41" s="4"/>
       <c r="H41" s="4"/>
@@ -3039,7 +3086,7 @@
       <c r="B43" s="4"/>
       <c r="C43" s="4"/>
       <c r="D43" s="4"/>
-      <c r="E43" s="4"/>
+      <c r="E43" s="5"/>
       <c r="F43" s="4"/>
       <c r="G43" s="4"/>
       <c r="H43" s="4"/>
@@ -3075,7 +3122,7 @@
       <c r="B44" s="4"/>
       <c r="C44" s="4"/>
       <c r="D44" s="4"/>
-      <c r="E44" s="4"/>
+      <c r="E44" s="5"/>
       <c r="F44" s="4"/>
       <c r="G44" s="4"/>
       <c r="H44" s="4"/>
@@ -3183,7 +3230,7 @@
       <c r="B47" s="4"/>
       <c r="C47" s="4"/>
       <c r="D47" s="4"/>
-      <c r="E47" s="5"/>
+      <c r="E47" s="4"/>
       <c r="F47" s="4"/>
       <c r="G47" s="4"/>
       <c r="H47" s="4"/>
@@ -3255,7 +3302,7 @@
       <c r="B49" s="4"/>
       <c r="C49" s="4"/>
       <c r="D49" s="4"/>
-      <c r="E49" s="4"/>
+      <c r="E49" s="5"/>
       <c r="F49" s="4"/>
       <c r="G49" s="4"/>
       <c r="H49" s="4"/>
@@ -3502,29 +3549,77 @@
       <c r="AG55" s="3"/>
       <c r="AH55" s="3"/>
     </row>
-    <row r="63" spans="1:23">
-      <c r="A63" s="2"/>
-      <c r="B63" s="2"/>
-      <c r="C63" s="2"/>
-      <c r="D63" s="2"/>
-      <c r="R63" s="2"/>
-      <c r="T63" s="2"/>
-      <c r="U63" s="2"/>
-      <c r="V63" s="2"/>
-      <c r="W63" s="2"/>
-    </row>
-    <row r="64" spans="1:23">
-      <c r="A64" s="2"/>
-      <c r="B64" s="2"/>
-      <c r="C64" s="2"/>
-      <c r="D64" s="2"/>
-      <c r="E64" s="2"/>
-      <c r="R64" s="2"/>
-      <c r="S64" s="2"/>
-      <c r="T64" s="2"/>
-      <c r="U64" s="2"/>
-      <c r="V64" s="2"/>
-      <c r="W64" s="2"/>
+    <row r="56" spans="1:34">
+      <c r="A56" s="3"/>
+      <c r="B56" s="4"/>
+      <c r="C56" s="4"/>
+      <c r="D56" s="4"/>
+      <c r="E56" s="4"/>
+      <c r="F56" s="4"/>
+      <c r="G56" s="4"/>
+      <c r="H56" s="4"/>
+      <c r="I56" s="4"/>
+      <c r="J56" s="4"/>
+      <c r="K56" s="4"/>
+      <c r="L56" s="4"/>
+      <c r="M56" s="4"/>
+      <c r="N56" s="4"/>
+      <c r="O56" s="4"/>
+      <c r="P56" s="4"/>
+      <c r="Q56" s="4"/>
+      <c r="R56" s="4"/>
+      <c r="S56" s="4"/>
+      <c r="T56" s="3"/>
+      <c r="U56" s="3"/>
+      <c r="V56" s="3"/>
+      <c r="W56" s="3"/>
+      <c r="X56" s="3"/>
+      <c r="Y56" s="3"/>
+      <c r="Z56" s="3"/>
+      <c r="AA56" s="3"/>
+      <c r="AB56" s="3"/>
+      <c r="AC56" s="3"/>
+      <c r="AD56" s="3"/>
+      <c r="AE56" s="3"/>
+      <c r="AF56" s="3"/>
+      <c r="AG56" s="3"/>
+      <c r="AH56" s="3"/>
+    </row>
+    <row r="57" spans="1:34">
+      <c r="A57" s="3"/>
+      <c r="B57" s="4"/>
+      <c r="C57" s="4"/>
+      <c r="D57" s="4"/>
+      <c r="E57" s="4"/>
+      <c r="F57" s="4"/>
+      <c r="G57" s="4"/>
+      <c r="H57" s="4"/>
+      <c r="I57" s="4"/>
+      <c r="J57" s="4"/>
+      <c r="K57" s="4"/>
+      <c r="L57" s="4"/>
+      <c r="M57" s="4"/>
+      <c r="N57" s="4"/>
+      <c r="O57" s="4"/>
+      <c r="P57" s="4"/>
+      <c r="Q57" s="4"/>
+      <c r="R57" s="4"/>
+      <c r="S57" s="4"/>
+      <c r="T57" s="3"/>
+      <c r="U57" s="3"/>
+      <c r="V57" s="3"/>
+      <c r="W57" s="3"/>
+      <c r="X57" s="3"/>
+      <c r="Y57" s="3"/>
+      <c r="Z57" s="3"/>
+      <c r="AA57" s="3"/>
+      <c r="AB57" s="3"/>
+      <c r="AC57" s="3"/>
+      <c r="AD57" s="3"/>
+      <c r="AE57" s="3"/>
+      <c r="AF57" s="3"/>
+      <c r="AG57" s="3"/>
+      <c r="AH57" s="3"/>
     </row>
     <row r="65" spans="1:23">
       <c r="A65" s="2"/>
@@ -3532,7 +3627,6 @@
       <c r="C65" s="2"/>
       <c r="D65" s="2"/>
       <c r="R65" s="2"/>
-      <c r="S65" s="2"/>
       <c r="T65" s="2"/>
       <c r="U65" s="2"/>
       <c r="V65" s="2"/>
@@ -3543,6 +3637,7 @@
       <c r="B66" s="2"/>
       <c r="C66" s="2"/>
       <c r="D66" s="2"/>
+      <c r="E66" s="2"/>
       <c r="R66" s="2"/>
       <c r="S66" s="2"/>
       <c r="T66" s="2"/>
@@ -3670,39 +3765,63 @@
       <c r="V76" s="2"/>
       <c r="W76" s="2"/>
     </row>
+    <row r="77" spans="1:23">
+      <c r="A77" s="2"/>
+      <c r="B77" s="2"/>
+      <c r="C77" s="2"/>
+      <c r="D77" s="2"/>
+      <c r="R77" s="2"/>
+      <c r="S77" s="2"/>
+      <c r="T77" s="2"/>
+      <c r="U77" s="2"/>
+      <c r="V77" s="2"/>
+      <c r="W77" s="2"/>
+    </row>
+    <row r="78" spans="1:23">
+      <c r="A78" s="2"/>
+      <c r="B78" s="2"/>
+      <c r="C78" s="2"/>
+      <c r="D78" s="2"/>
+      <c r="R78" s="2"/>
+      <c r="S78" s="2"/>
+      <c r="T78" s="2"/>
+      <c r="U78" s="2"/>
+      <c r="V78" s="2"/>
+      <c r="W78" s="2"/>
+    </row>
   </sheetData>
   <dataValidations count="11">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L5 L6 L9 L12 L13 L14 L15 L16 L17 L18 L19 L20 L2:L4 L7:L8 L10:L11 L21:L1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L5 L6 L9 L10 L13 L14 L15 L16 L17 L18 L19 L20 L21 L22 L2:L4 L7:L8 L11:L12 L23:L1048576">
       <formula1>"BR_EQ,BR_NE,BR_LTU,BR_GE,BR_GEU,BR_LT,BR_XX"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J5 J6 J7 J8 J9 J10 J11 J12 J13 J14 J15 J16 J17 J18 J19 J20 J2:J4 J21:J1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J5 J6 J7 J8 J9 J10 J11 J12 J13 J14 J15 J16 J17 J18 J19 J20 J21 J22 J2:J4 J23:J1048576">
       <formula1>"ST_SW,ST_SH,ST_SB,ST_XX"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H5 H6 H7 H8 H9 H12 H13 H14 H15 H16 H17 H18 H19 H20 H2:H4 H10:H11 H21:H1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H5 H6 H7 H8 H9 H10 H13 H14 H15 H16 H17 H18 H19 H20 H21 H22 H2:H4 H11:H12 H23:H1048576">
       <formula1>"WB_ALU,WB_MEM,WB_PC4,WB_XX"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="M4 M5 M6 M7 M8 M9 M10 M11 M12 M13 M14 M15 M16 M17 M18 M19 M20 M2:M3 M21:M1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="M4 M5 M6 M7 M8 M9 M10 M11 M12 M13 M14 M15 M16 M17 M18 M19 M20 M21 M22 M2:M3 M23:M1048576">
       <formula1>"INST_VALID,INST_INVALID"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K4 K5 K6 K7 K8 K9 K10 K11 K12 K13 K14 K15 K16 K17 K18 K19 K20 K2:K3 K21:K1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K4 K5 K6 K7 K8 K9 K10 K11 K12 K13 K14 K15 K16 K17 K18 K19 K20 K21 K22 K2:K3 K23:K1048576">
       <formula1>"MASK_XX,MASK_B,MASK_H,MASK_W,MASK_D"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I4 I5 I6 I7 I8 I9 I10 I11 I12 I13 I14 I15 I16 I17 I18 I19 I20 I2:I3 I21:I1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I4 I5 I6 I7 I8 I9 I10 I11 I12 I13 I14 I15 I16 I17 I18 I19 I20 I21 I22 I2:I3 I23:I1048576">
       <formula1>"LD_LB,LD_LH,LD_LW,LD_LBU,LD_LHU,LD_XX"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F4 F5 F6 F7 F8 F9 F10 F11 F12 F13 F14 F15 F16 F17 F18 F19 F20 F2:F3 F21:F1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F4 F5 F6 F7 F8 F9 F10 F11 F12 F13 F14 F15 F16 F17 F18 F19 F20 F21 F22 F2:F3 F23:F1048576">
       <formula1>"ALU_ADD,ALU_SUB,ALU_AND,ALU_OR,ALU_XOR,ALU_SLL,ALU_SRL,ALU_SLT,ALU_SLTU,ALU_COPY_A,ALU_COPY_B"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E4 E5 E6 E7 E8 E9 E10 E11 E12 E13 E14 E15 E16 E17 E18 E19 E20 E2:E3 E21:E1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E4 E5 E6 E7 E8 E9 E10 E11 E12 E13 E14 E15 E16 E17 E18 E19 E20 E21 E22 E2:E3 E23:E1048576">
       <formula1>"B_IMM,B_RS2"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G4 G5 G6 G7 G8 G9 G10 G11 G12 G13 G14 G15 G16 G17 G18 G19 G20 G2:G3 G21:G1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G4 G5 G6 G7 G8 G9 G10 G11 G12 G13 G14 G15 G16 G17 G18 G19 G20 G21 G22 G2:G3 G23:G1048576">
       <formula1>"IMM_I,IMM_J,IMM_U,IMM_S,IMM_B"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D4 D5 D6 D7 D8 D9 D10 D11 D12 D13 D14 D15 D16 D17 D18 D19 D20 D2:D3 D21:D1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D4 D5 D6 D7 D8 D9 D10 D11 D12 D13 D14 D15 D16 D17 D18 D19 D20 D21 D22 D2:D3 D23:D1048576">
       <formula1>"A_PC,A_RS1"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C4 C5 C6 C7 C8 C9 C10 C11 C12 C13 C14 C15 C16 C17 C18 C19 C20 C2:C3 C21:C1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C4 C5 C6 C7 C8 C9 C10 C11 C12 C13 C14 C15 C16 C17 C18 C19 C20 C21 C22 C2:C3 C23:C1048576">
       <formula1>"PC_4,PC_0,PC_ALU"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
> sim RTL ysyx_23060246 韩炳晋 Linux archlinux 6.6.60-1-lts #1 SMP PREEMPT_DYNAMIC Fri, 08 Nov 2024 16:03:02 +0000 x86_64 GNU/Linux  20:24:09 up 1 day,  2:39,  2 users,  load average: 1.93, 1.39, 1.63
</commit_message>
<xml_diff>
--- a/npc/tools/control_gen/control_table.xlsx
+++ b/npc/tools/control_gen/control_table.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="177" uniqueCount="76">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="184" uniqueCount="78">
   <si>
     <t>comment</t>
   </si>
@@ -194,6 +194,12 @@
   </si>
   <si>
     <t>BR_GE</t>
+  </si>
+  <si>
+    <t>srai</t>
+  </si>
+  <si>
+    <t>ALU_SRA</t>
   </si>
   <si>
     <t>slli</t>
@@ -1210,7 +1216,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:AH78"/>
+  <dimension ref="A1:AH79"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
     <col min="1" max="1" width="13.1" customWidth="1"/>
@@ -2256,12 +2262,14 @@
         <v>23</v>
       </c>
       <c r="E21" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="F21" s="4" t="s">
         <v>65</v>
       </c>
-      <c r="F21" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="G21" s="4"/>
+      <c r="G21" s="4" t="s">
+        <v>24</v>
+      </c>
       <c r="H21" s="4" t="s">
         <v>17</v>
       </c>
@@ -2304,10 +2312,10 @@
         <v>23</v>
       </c>
       <c r="E22" s="4" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="F22" s="4" t="s">
-        <v>67</v>
+        <v>21</v>
       </c>
       <c r="G22" s="4"/>
       <c r="H22" s="4" t="s">
@@ -2342,49 +2350,42 @@
       <c r="AG22" s="3"/>
       <c r="AH22" s="3"/>
     </row>
-    <row r="23" spans="2:34">
-      <c r="B23" s="2" t="s">
+    <row r="23" spans="1:34">
+      <c r="A23" s="3"/>
+      <c r="B23" s="4" t="s">
         <v>68</v>
       </c>
-      <c r="C23" s="2" t="s">
+      <c r="C23" s="2"/>
+      <c r="D23" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="E23" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="F23" s="4" t="s">
         <v>69</v>
       </c>
-      <c r="D23" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="E23" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="F23" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="G23" s="2" t="s">
-        <v>24</v>
-      </c>
+      <c r="G23" s="4"/>
       <c r="H23" s="4" t="s">
-        <v>70</v>
-      </c>
-      <c r="I23" s="4" t="s">
-        <v>71</v>
-      </c>
-      <c r="J23" s="4" t="s">
-        <v>72</v>
-      </c>
-      <c r="K23" s="2" t="s">
-        <v>73</v>
-      </c>
-      <c r="L23" s="2" t="s">
-        <v>74</v>
-      </c>
-      <c r="M23" s="2" t="s">
-        <v>75</v>
-      </c>
-      <c r="N23" s="2"/>
-      <c r="O23" s="2"/>
-      <c r="P23" s="2"/>
-      <c r="Q23" s="2"/>
-      <c r="R23" s="2"/>
-      <c r="S23" s="2"/>
+        <v>17</v>
+      </c>
+      <c r="I23" s="4"/>
+      <c r="J23" s="4"/>
+      <c r="K23" s="4"/>
+      <c r="L23" s="4"/>
+      <c r="M23" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="N23" s="4"/>
+      <c r="O23" s="4"/>
+      <c r="P23" s="4"/>
+      <c r="Q23" s="4"/>
+      <c r="R23" s="4"/>
+      <c r="S23" s="4"/>
+      <c r="T23" s="3"/>
+      <c r="U23" s="3"/>
+      <c r="V23" s="3"/>
+      <c r="W23" s="3"/>
       <c r="X23" s="3"/>
       <c r="Y23" s="3"/>
       <c r="Z23" s="3"/>
@@ -2397,30 +2398,49 @@
       <c r="AG23" s="3"/>
       <c r="AH23" s="3"/>
     </row>
-    <row r="24" spans="1:34">
-      <c r="A24" s="3"/>
-      <c r="B24" s="4"/>
-      <c r="C24" s="4"/>
-      <c r="D24" s="4"/>
-      <c r="E24" s="4"/>
-      <c r="F24" s="4"/>
-      <c r="G24" s="4"/>
-      <c r="H24" s="4"/>
-      <c r="I24" s="4"/>
-      <c r="J24" s="4"/>
-      <c r="K24" s="4"/>
-      <c r="L24" s="4"/>
-      <c r="M24" s="4"/>
-      <c r="N24" s="4"/>
-      <c r="O24" s="4"/>
-      <c r="P24" s="4"/>
-      <c r="Q24" s="4"/>
-      <c r="R24" s="4"/>
-      <c r="S24" s="4"/>
-      <c r="T24" s="3"/>
-      <c r="U24" s="3"/>
-      <c r="V24" s="3"/>
-      <c r="W24" s="3"/>
+    <row r="24" spans="2:34">
+      <c r="B24" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="C24" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="D24" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="E24" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="F24" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="G24" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="H24" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="I24" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="J24" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="K24" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="L24" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="M24" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="N24" s="2"/>
+      <c r="O24" s="2"/>
+      <c r="P24" s="2"/>
+      <c r="Q24" s="2"/>
+      <c r="R24" s="2"/>
+      <c r="S24" s="2"/>
       <c r="X24" s="3"/>
       <c r="Y24" s="3"/>
       <c r="Z24" s="3"/>
@@ -2433,7 +2453,7 @@
       <c r="AG24" s="3"/>
       <c r="AH24" s="3"/>
     </row>
-    <row r="25" s="1" customFormat="1" spans="1:34">
+    <row r="25" spans="1:34">
       <c r="A25" s="3"/>
       <c r="B25" s="4"/>
       <c r="C25" s="4"/>
@@ -2505,7 +2525,7 @@
       <c r="AG26" s="3"/>
       <c r="AH26" s="3"/>
     </row>
-    <row r="27" spans="1:34">
+    <row r="27" s="1" customFormat="1" spans="1:34">
       <c r="A27" s="3"/>
       <c r="B27" s="4"/>
       <c r="C27" s="4"/>
@@ -3050,7 +3070,7 @@
       <c r="B42" s="4"/>
       <c r="C42" s="4"/>
       <c r="D42" s="4"/>
-      <c r="E42" s="5"/>
+      <c r="E42" s="4"/>
       <c r="F42" s="4"/>
       <c r="G42" s="4"/>
       <c r="H42" s="4"/>
@@ -3158,7 +3178,7 @@
       <c r="B45" s="4"/>
       <c r="C45" s="4"/>
       <c r="D45" s="4"/>
-      <c r="E45" s="4"/>
+      <c r="E45" s="5"/>
       <c r="F45" s="4"/>
       <c r="G45" s="4"/>
       <c r="H45" s="4"/>
@@ -3302,7 +3322,7 @@
       <c r="B49" s="4"/>
       <c r="C49" s="4"/>
       <c r="D49" s="4"/>
-      <c r="E49" s="5"/>
+      <c r="E49" s="4"/>
       <c r="F49" s="4"/>
       <c r="G49" s="4"/>
       <c r="H49" s="4"/>
@@ -3338,7 +3358,7 @@
       <c r="B50" s="4"/>
       <c r="C50" s="4"/>
       <c r="D50" s="4"/>
-      <c r="E50" s="4"/>
+      <c r="E50" s="5"/>
       <c r="F50" s="4"/>
       <c r="G50" s="4"/>
       <c r="H50" s="4"/>
@@ -3621,25 +3641,48 @@
       <c r="AG57" s="3"/>
       <c r="AH57" s="3"/>
     </row>
-    <row r="65" spans="1:23">
-      <c r="A65" s="2"/>
-      <c r="B65" s="2"/>
-      <c r="C65" s="2"/>
-      <c r="D65" s="2"/>
-      <c r="R65" s="2"/>
-      <c r="T65" s="2"/>
-      <c r="U65" s="2"/>
-      <c r="V65" s="2"/>
-      <c r="W65" s="2"/>
+    <row r="58" spans="1:34">
+      <c r="A58" s="3"/>
+      <c r="B58" s="4"/>
+      <c r="C58" s="4"/>
+      <c r="D58" s="4"/>
+      <c r="E58" s="4"/>
+      <c r="F58" s="4"/>
+      <c r="G58" s="4"/>
+      <c r="H58" s="4"/>
+      <c r="I58" s="4"/>
+      <c r="J58" s="4"/>
+      <c r="K58" s="4"/>
+      <c r="L58" s="4"/>
+      <c r="M58" s="4"/>
+      <c r="N58" s="4"/>
+      <c r="O58" s="4"/>
+      <c r="P58" s="4"/>
+      <c r="Q58" s="4"/>
+      <c r="R58" s="4"/>
+      <c r="S58" s="4"/>
+      <c r="T58" s="3"/>
+      <c r="U58" s="3"/>
+      <c r="V58" s="3"/>
+      <c r="W58" s="3"/>
+      <c r="X58" s="3"/>
+      <c r="Y58" s="3"/>
+      <c r="Z58" s="3"/>
+      <c r="AA58" s="3"/>
+      <c r="AB58" s="3"/>
+      <c r="AC58" s="3"/>
+      <c r="AD58" s="3"/>
+      <c r="AE58" s="3"/>
+      <c r="AF58" s="3"/>
+      <c r="AG58" s="3"/>
+      <c r="AH58" s="3"/>
     </row>
     <row r="66" spans="1:23">
       <c r="A66" s="2"/>
       <c r="B66" s="2"/>
       <c r="C66" s="2"/>
       <c r="D66" s="2"/>
-      <c r="E66" s="2"/>
       <c r="R66" s="2"/>
-      <c r="S66" s="2"/>
       <c r="T66" s="2"/>
       <c r="U66" s="2"/>
       <c r="V66" s="2"/>
@@ -3650,6 +3693,7 @@
       <c r="B67" s="2"/>
       <c r="C67" s="2"/>
       <c r="D67" s="2"/>
+      <c r="E67" s="2"/>
       <c r="R67" s="2"/>
       <c r="S67" s="2"/>
       <c r="T67" s="2"/>
@@ -3789,39 +3833,51 @@
       <c r="V78" s="2"/>
       <c r="W78" s="2"/>
     </row>
+    <row r="79" spans="1:23">
+      <c r="A79" s="2"/>
+      <c r="B79" s="2"/>
+      <c r="C79" s="2"/>
+      <c r="D79" s="2"/>
+      <c r="R79" s="2"/>
+      <c r="S79" s="2"/>
+      <c r="T79" s="2"/>
+      <c r="U79" s="2"/>
+      <c r="V79" s="2"/>
+      <c r="W79" s="2"/>
+    </row>
   </sheetData>
   <dataValidations count="11">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L5 L6 L9 L10 L13 L14 L15 L16 L17 L18 L19 L20 L21 L22 L2:L4 L7:L8 L11:L12 L23:L1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F2:F1048576">
+      <formula1>"ALU_ADD,ALU_SUB,ALU_AND,ALU_OR,ALU_XOR,ALU_SLL,ALU_SRL,ALU_SLT,ALU_SLTU,ALU_COPY_A,ALU_COPY_B,ALU_SRA"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L5 L6 L9 L10 L13 L14 L15 L16 L17 L18 L19 L20 L21 L22 L23 L2:L4 L7:L8 L11:L12 L24:L1048576">
       <formula1>"BR_EQ,BR_NE,BR_LTU,BR_GE,BR_GEU,BR_LT,BR_XX"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J5 J6 J7 J8 J9 J10 J11 J12 J13 J14 J15 J16 J17 J18 J19 J20 J21 J22 J2:J4 J23:J1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J5 J6 J7 J8 J9 J10 J11 J12 J13 J14 J15 J16 J17 J18 J19 J20 J21 J22 J23 J2:J4 J24:J1048576">
       <formula1>"ST_SW,ST_SH,ST_SB,ST_XX"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H5 H6 H7 H8 H9 H10 H13 H14 H15 H16 H17 H18 H19 H20 H21 H22 H2:H4 H11:H12 H23:H1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H5 H6 H7 H8 H9 H10 H13 H14 H15 H16 H17 H18 H19 H20 H21 H22 H23 H2:H4 H11:H12 H24:H1048576">
       <formula1>"WB_ALU,WB_MEM,WB_PC4,WB_XX"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="M4 M5 M6 M7 M8 M9 M10 M11 M12 M13 M14 M15 M16 M17 M18 M19 M20 M21 M22 M2:M3 M23:M1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="M4 M5 M6 M7 M8 M9 M10 M11 M12 M13 M14 M15 M16 M17 M18 M19 M20 M21 M22 M23 M2:M3 M24:M1048576">
       <formula1>"INST_VALID,INST_INVALID"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K4 K5 K6 K7 K8 K9 K10 K11 K12 K13 K14 K15 K16 K17 K18 K19 K20 K21 K22 K2:K3 K23:K1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K4 K5 K6 K7 K8 K9 K10 K11 K12 K13 K14 K15 K16 K17 K18 K19 K20 K21 K22 K23 K2:K3 K24:K1048576">
       <formula1>"MASK_XX,MASK_B,MASK_H,MASK_W,MASK_D"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I4 I5 I6 I7 I8 I9 I10 I11 I12 I13 I14 I15 I16 I17 I18 I19 I20 I21 I22 I2:I3 I23:I1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I4 I5 I6 I7 I8 I9 I10 I11 I12 I13 I14 I15 I16 I17 I18 I19 I20 I21 I22 I23 I2:I3 I24:I1048576">
       <formula1>"LD_LB,LD_LH,LD_LW,LD_LBU,LD_LHU,LD_XX"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F4 F5 F6 F7 F8 F9 F10 F11 F12 F13 F14 F15 F16 F17 F18 F19 F20 F21 F22 F2:F3 F23:F1048576">
-      <formula1>"ALU_ADD,ALU_SUB,ALU_AND,ALU_OR,ALU_XOR,ALU_SLL,ALU_SRL,ALU_SLT,ALU_SLTU,ALU_COPY_A,ALU_COPY_B"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E4 E5 E6 E7 E8 E9 E10 E11 E12 E13 E14 E15 E16 E17 E18 E19 E20 E21 E22 E2:E3 E23:E1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E4 E5 E6 E7 E8 E9 E10 E11 E12 E13 E14 E15 E16 E17 E18 E19 E20 E21 E22 E23 E2:E3 E24:E1048576">
       <formula1>"B_IMM,B_RS2"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G4 G5 G6 G7 G8 G9 G10 G11 G12 G13 G14 G15 G16 G17 G18 G19 G20 G21 G22 G2:G3 G23:G1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G4 G5 G6 G7 G8 G9 G10 G11 G12 G13 G14 G15 G16 G17 G18 G19 G20 G21 G22 G23 G2:G3 G24:G1048576">
       <formula1>"IMM_I,IMM_J,IMM_U,IMM_S,IMM_B"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D4 D5 D6 D7 D8 D9 D10 D11 D12 D13 D14 D15 D16 D17 D18 D19 D20 D21 D22 D2:D3 D23:D1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D4 D5 D6 D7 D8 D9 D10 D11 D12 D13 D14 D15 D16 D17 D18 D19 D20 D21 D22 D23 D2:D3 D24:D1048576">
       <formula1>"A_PC,A_RS1"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C4 C5 C6 C7 C8 C9 C10 C11 C12 C13 C14 C15 C16 C17 C18 C19 C20 C21 C22 C2:C3 C23:C1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C4 C5 C6 C7 C8 C9 C10 C11 C12 C13 C14 C15 C16 C17 C18 C19 C20 C21 C22 C23 C2:C3 C24:C1048576">
       <formula1>"PC_4,PC_0,PC_ALU"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
> sim RTL ysyx_23060246 韩炳晋 Linux archlinux 6.6.60-1-lts #1 SMP PREEMPT_DYNAMIC Fri, 08 Nov 2024 16:03:02 +0000 x86_64 GNU/Linux  20:25:28 up 1 day,  2:40,  2 users,  load average: 2.03, 1.48, 1.64
</commit_message>
<xml_diff>
--- a/npc/tools/control_gen/control_table.xlsx
+++ b/npc/tools/control_gen/control_table.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="184" uniqueCount="78">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="190" uniqueCount="79">
   <si>
     <t>comment</t>
   </si>
@@ -214,10 +214,13 @@
     <t>ALU_SLTU</t>
   </si>
   <si>
+    <t>sll</t>
+  </si>
+  <si>
+    <t>B_RS2</t>
+  </si>
+  <si>
     <t>add</t>
-  </si>
-  <si>
-    <t>B_RS2</t>
   </si>
   <si>
     <t>sub</t>
@@ -1216,7 +1219,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:AH79"/>
+  <dimension ref="A1:AH80"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
     <col min="1" max="1" width="13.1" customWidth="1"/>
@@ -2315,7 +2318,7 @@
         <v>67</v>
       </c>
       <c r="F22" s="4" t="s">
-        <v>21</v>
+        <v>63</v>
       </c>
       <c r="G22" s="4"/>
       <c r="H22" s="4" t="s">
@@ -2363,7 +2366,7 @@
         <v>67</v>
       </c>
       <c r="F23" s="4" t="s">
-        <v>69</v>
+        <v>21</v>
       </c>
       <c r="G23" s="4"/>
       <c r="H23" s="4" t="s">
@@ -2398,49 +2401,42 @@
       <c r="AG23" s="3"/>
       <c r="AH23" s="3"/>
     </row>
-    <row r="24" spans="2:34">
-      <c r="B24" s="2" t="s">
+    <row r="24" spans="1:34">
+      <c r="A24" s="3"/>
+      <c r="B24" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="C24" s="2"/>
+      <c r="D24" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="E24" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="F24" s="4" t="s">
         <v>70</v>
       </c>
-      <c r="C24" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="D24" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="E24" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="F24" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="G24" s="2" t="s">
-        <v>24</v>
-      </c>
+      <c r="G24" s="4"/>
       <c r="H24" s="4" t="s">
-        <v>72</v>
-      </c>
-      <c r="I24" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="J24" s="4" t="s">
-        <v>74</v>
-      </c>
-      <c r="K24" s="2" t="s">
-        <v>75</v>
-      </c>
-      <c r="L24" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="M24" s="2" t="s">
-        <v>77</v>
-      </c>
-      <c r="N24" s="2"/>
-      <c r="O24" s="2"/>
-      <c r="P24" s="2"/>
-      <c r="Q24" s="2"/>
-      <c r="R24" s="2"/>
-      <c r="S24" s="2"/>
+        <v>17</v>
+      </c>
+      <c r="I24" s="4"/>
+      <c r="J24" s="4"/>
+      <c r="K24" s="4"/>
+      <c r="L24" s="4"/>
+      <c r="M24" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="N24" s="4"/>
+      <c r="O24" s="4"/>
+      <c r="P24" s="4"/>
+      <c r="Q24" s="4"/>
+      <c r="R24" s="4"/>
+      <c r="S24" s="4"/>
+      <c r="T24" s="3"/>
+      <c r="U24" s="3"/>
+      <c r="V24" s="3"/>
+      <c r="W24" s="3"/>
       <c r="X24" s="3"/>
       <c r="Y24" s="3"/>
       <c r="Z24" s="3"/>
@@ -2453,30 +2449,49 @@
       <c r="AG24" s="3"/>
       <c r="AH24" s="3"/>
     </row>
-    <row r="25" spans="1:34">
-      <c r="A25" s="3"/>
-      <c r="B25" s="4"/>
-      <c r="C25" s="4"/>
-      <c r="D25" s="4"/>
-      <c r="E25" s="4"/>
-      <c r="F25" s="4"/>
-      <c r="G25" s="4"/>
-      <c r="H25" s="4"/>
-      <c r="I25" s="4"/>
-      <c r="J25" s="4"/>
-      <c r="K25" s="4"/>
-      <c r="L25" s="4"/>
-      <c r="M25" s="4"/>
-      <c r="N25" s="4"/>
-      <c r="O25" s="4"/>
-      <c r="P25" s="4"/>
-      <c r="Q25" s="4"/>
-      <c r="R25" s="4"/>
-      <c r="S25" s="4"/>
-      <c r="T25" s="3"/>
-      <c r="U25" s="3"/>
-      <c r="V25" s="3"/>
-      <c r="W25" s="3"/>
+    <row r="25" spans="2:34">
+      <c r="B25" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="C25" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="D25" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="E25" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="F25" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="G25" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="H25" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="I25" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="J25" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="K25" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="L25" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="M25" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="N25" s="2"/>
+      <c r="O25" s="2"/>
+      <c r="P25" s="2"/>
+      <c r="Q25" s="2"/>
+      <c r="R25" s="2"/>
+      <c r="S25" s="2"/>
       <c r="X25" s="3"/>
       <c r="Y25" s="3"/>
       <c r="Z25" s="3"/>
@@ -2489,7 +2504,7 @@
       <c r="AG25" s="3"/>
       <c r="AH25" s="3"/>
     </row>
-    <row r="26" s="1" customFormat="1" spans="1:34">
+    <row r="26" spans="1:34">
       <c r="A26" s="3"/>
       <c r="B26" s="4"/>
       <c r="C26" s="4"/>
@@ -2561,7 +2576,7 @@
       <c r="AG27" s="3"/>
       <c r="AH27" s="3"/>
     </row>
-    <row r="28" spans="1:34">
+    <row r="28" s="1" customFormat="1" spans="1:34">
       <c r="A28" s="3"/>
       <c r="B28" s="4"/>
       <c r="C28" s="4"/>
@@ -3106,7 +3121,7 @@
       <c r="B43" s="4"/>
       <c r="C43" s="4"/>
       <c r="D43" s="4"/>
-      <c r="E43" s="5"/>
+      <c r="E43" s="4"/>
       <c r="F43" s="4"/>
       <c r="G43" s="4"/>
       <c r="H43" s="4"/>
@@ -3214,7 +3229,7 @@
       <c r="B46" s="4"/>
       <c r="C46" s="4"/>
       <c r="D46" s="4"/>
-      <c r="E46" s="4"/>
+      <c r="E46" s="5"/>
       <c r="F46" s="4"/>
       <c r="G46" s="4"/>
       <c r="H46" s="4"/>
@@ -3358,7 +3373,7 @@
       <c r="B50" s="4"/>
       <c r="C50" s="4"/>
       <c r="D50" s="4"/>
-      <c r="E50" s="5"/>
+      <c r="E50" s="4"/>
       <c r="F50" s="4"/>
       <c r="G50" s="4"/>
       <c r="H50" s="4"/>
@@ -3394,7 +3409,7 @@
       <c r="B51" s="4"/>
       <c r="C51" s="4"/>
       <c r="D51" s="4"/>
-      <c r="E51" s="4"/>
+      <c r="E51" s="5"/>
       <c r="F51" s="4"/>
       <c r="G51" s="4"/>
       <c r="H51" s="4"/>
@@ -3677,25 +3692,48 @@
       <c r="AG58" s="3"/>
       <c r="AH58" s="3"/>
     </row>
-    <row r="66" spans="1:23">
-      <c r="A66" s="2"/>
-      <c r="B66" s="2"/>
-      <c r="C66" s="2"/>
-      <c r="D66" s="2"/>
-      <c r="R66" s="2"/>
-      <c r="T66" s="2"/>
-      <c r="U66" s="2"/>
-      <c r="V66" s="2"/>
-      <c r="W66" s="2"/>
+    <row r="59" spans="1:34">
+      <c r="A59" s="3"/>
+      <c r="B59" s="4"/>
+      <c r="C59" s="4"/>
+      <c r="D59" s="4"/>
+      <c r="E59" s="4"/>
+      <c r="F59" s="4"/>
+      <c r="G59" s="4"/>
+      <c r="H59" s="4"/>
+      <c r="I59" s="4"/>
+      <c r="J59" s="4"/>
+      <c r="K59" s="4"/>
+      <c r="L59" s="4"/>
+      <c r="M59" s="4"/>
+      <c r="N59" s="4"/>
+      <c r="O59" s="4"/>
+      <c r="P59" s="4"/>
+      <c r="Q59" s="4"/>
+      <c r="R59" s="4"/>
+      <c r="S59" s="4"/>
+      <c r="T59" s="3"/>
+      <c r="U59" s="3"/>
+      <c r="V59" s="3"/>
+      <c r="W59" s="3"/>
+      <c r="X59" s="3"/>
+      <c r="Y59" s="3"/>
+      <c r="Z59" s="3"/>
+      <c r="AA59" s="3"/>
+      <c r="AB59" s="3"/>
+      <c r="AC59" s="3"/>
+      <c r="AD59" s="3"/>
+      <c r="AE59" s="3"/>
+      <c r="AF59" s="3"/>
+      <c r="AG59" s="3"/>
+      <c r="AH59" s="3"/>
     </row>
     <row r="67" spans="1:23">
       <c r="A67" s="2"/>
       <c r="B67" s="2"/>
       <c r="C67" s="2"/>
       <c r="D67" s="2"/>
-      <c r="E67" s="2"/>
       <c r="R67" s="2"/>
-      <c r="S67" s="2"/>
       <c r="T67" s="2"/>
       <c r="U67" s="2"/>
       <c r="V67" s="2"/>
@@ -3706,6 +3744,7 @@
       <c r="B68" s="2"/>
       <c r="C68" s="2"/>
       <c r="D68" s="2"/>
+      <c r="E68" s="2"/>
       <c r="R68" s="2"/>
       <c r="S68" s="2"/>
       <c r="T68" s="2"/>
@@ -3845,39 +3884,51 @@
       <c r="V79" s="2"/>
       <c r="W79" s="2"/>
     </row>
+    <row r="80" spans="1:23">
+      <c r="A80" s="2"/>
+      <c r="B80" s="2"/>
+      <c r="C80" s="2"/>
+      <c r="D80" s="2"/>
+      <c r="R80" s="2"/>
+      <c r="S80" s="2"/>
+      <c r="T80" s="2"/>
+      <c r="U80" s="2"/>
+      <c r="V80" s="2"/>
+      <c r="W80" s="2"/>
+    </row>
   </sheetData>
   <dataValidations count="11">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F2:F1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F22 F2:F21 F23:F1048576">
       <formula1>"ALU_ADD,ALU_SUB,ALU_AND,ALU_OR,ALU_XOR,ALU_SLL,ALU_SRL,ALU_SLT,ALU_SLTU,ALU_COPY_A,ALU_COPY_B,ALU_SRA"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L5 L6 L9 L10 L13 L14 L15 L16 L17 L18 L19 L20 L21 L22 L23 L2:L4 L7:L8 L11:L12 L24:L1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L5 L6 L9 L10 L13 L14 L15 L16 L17 L18 L19 L20 L21 L22 L23 L24 L2:L4 L7:L8 L11:L12 L25:L1048576">
       <formula1>"BR_EQ,BR_NE,BR_LTU,BR_GE,BR_GEU,BR_LT,BR_XX"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J5 J6 J7 J8 J9 J10 J11 J12 J13 J14 J15 J16 J17 J18 J19 J20 J21 J22 J23 J2:J4 J24:J1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J5 J6 J7 J8 J9 J10 J11 J12 J13 J14 J15 J16 J17 J18 J19 J20 J21 J22 J23 J24 J2:J4 J25:J1048576">
       <formula1>"ST_SW,ST_SH,ST_SB,ST_XX"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H5 H6 H7 H8 H9 H10 H13 H14 H15 H16 H17 H18 H19 H20 H21 H22 H23 H2:H4 H11:H12 H24:H1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H5 H6 H7 H8 H9 H10 H13 H14 H15 H16 H17 H18 H19 H20 H21 H22 H23 H24 H2:H4 H11:H12 H25:H1048576">
       <formula1>"WB_ALU,WB_MEM,WB_PC4,WB_XX"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="M4 M5 M6 M7 M8 M9 M10 M11 M12 M13 M14 M15 M16 M17 M18 M19 M20 M21 M22 M23 M2:M3 M24:M1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="M4 M5 M6 M7 M8 M9 M10 M11 M12 M13 M14 M15 M16 M17 M18 M19 M20 M21 M22 M23 M24 M2:M3 M25:M1048576">
       <formula1>"INST_VALID,INST_INVALID"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K4 K5 K6 K7 K8 K9 K10 K11 K12 K13 K14 K15 K16 K17 K18 K19 K20 K21 K22 K23 K2:K3 K24:K1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K4 K5 K6 K7 K8 K9 K10 K11 K12 K13 K14 K15 K16 K17 K18 K19 K20 K21 K22 K23 K24 K2:K3 K25:K1048576">
       <formula1>"MASK_XX,MASK_B,MASK_H,MASK_W,MASK_D"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I4 I5 I6 I7 I8 I9 I10 I11 I12 I13 I14 I15 I16 I17 I18 I19 I20 I21 I22 I23 I2:I3 I24:I1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I4 I5 I6 I7 I8 I9 I10 I11 I12 I13 I14 I15 I16 I17 I18 I19 I20 I21 I22 I23 I24 I2:I3 I25:I1048576">
       <formula1>"LD_LB,LD_LH,LD_LW,LD_LBU,LD_LHU,LD_XX"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E4 E5 E6 E7 E8 E9 E10 E11 E12 E13 E14 E15 E16 E17 E18 E19 E20 E21 E22 E23 E2:E3 E24:E1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E4 E5 E6 E7 E8 E9 E10 E11 E12 E13 E14 E15 E16 E17 E18 E19 E20 E21 E22 E23 E24 E2:E3 E25:E1048576">
       <formula1>"B_IMM,B_RS2"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G4 G5 G6 G7 G8 G9 G10 G11 G12 G13 G14 G15 G16 G17 G18 G19 G20 G21 G22 G23 G2:G3 G24:G1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G4 G5 G6 G7 G8 G9 G10 G11 G12 G13 G14 G15 G16 G17 G18 G19 G20 G21 G22 G23 G24 G2:G3 G25:G1048576">
       <formula1>"IMM_I,IMM_J,IMM_U,IMM_S,IMM_B"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D4 D5 D6 D7 D8 D9 D10 D11 D12 D13 D14 D15 D16 D17 D18 D19 D20 D21 D22 D23 D2:D3 D24:D1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D4 D5 D6 D7 D8 D9 D10 D11 D12 D13 D14 D15 D16 D17 D18 D19 D20 D21 D22 D23 D24 D2:D3 D25:D1048576">
       <formula1>"A_PC,A_RS1"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C4 C5 C6 C7 C8 C9 C10 C11 C12 C13 C14 C15 C16 C17 C18 C19 C20 C21 C22 C23 C2:C3 C24:C1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C4 C5 C6 C7 C8 C9 C10 C11 C12 C13 C14 C15 C16 C17 C18 C19 C20 C21 C22 C23 C24 C2:C3 C25:C1048576">
       <formula1>"PC_4,PC_0,PC_ALU"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
> sim RTL ysyx_23060246 韩炳晋 Linux archlinux 6.6.60-1-lts #1 SMP PREEMPT_DYNAMIC Fri, 08 Nov 2024 16:03:02 +0000 x86_64 GNU/Linux  20:32:26 up 1 day,  2:47,  2 users,  load average: 3.52, 2.06, 1.75
</commit_message>
<xml_diff>
--- a/npc/tools/control_gen/control_table.xlsx
+++ b/npc/tools/control_gen/control_table.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="27795" windowHeight="12735"/>
+    <workbookView windowWidth="27795" windowHeight="12075"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="190" uniqueCount="79">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="243" uniqueCount="92">
   <si>
     <t>comment</t>
   </si>
@@ -97,6 +97,12 @@
     <t>ALU_AND</t>
   </si>
   <si>
+    <t>ori</t>
+  </si>
+  <si>
+    <t>ALU_OR</t>
+  </si>
+  <si>
     <t>xori</t>
   </si>
   <si>
@@ -175,15 +181,33 @@
     <t>LD_LBU</t>
   </si>
   <si>
+    <t>bne</t>
+  </si>
+  <si>
+    <t>IMM_B</t>
+  </si>
+  <si>
+    <t>BR_NE</t>
+  </si>
+  <si>
     <t>beq</t>
   </si>
   <si>
-    <t>IMM_B</t>
-  </si>
-  <si>
     <t>BR_EQ</t>
   </si>
   <si>
+    <t>blt</t>
+  </si>
+  <si>
+    <t>BR_LT</t>
+  </si>
+  <si>
+    <t>bltu</t>
+  </si>
+  <si>
+    <t>BR_LTU</t>
+  </si>
+  <si>
     <t>bgeu</t>
   </si>
   <si>
@@ -196,6 +220,12 @@
     <t>BR_GE</t>
   </si>
   <si>
+    <t>srli</t>
+  </si>
+  <si>
+    <t>ALU_SRL</t>
+  </si>
+  <si>
     <t>srai</t>
   </si>
   <si>
@@ -227,6 +257,15 @@
   </si>
   <si>
     <t>ALU_SUB</t>
+  </si>
+  <si>
+    <t>xor</t>
+  </si>
+  <si>
+    <t>and</t>
+  </si>
+  <si>
+    <t>or</t>
   </si>
   <si>
     <t>default</t>
@@ -1219,7 +1258,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:AH80"/>
+  <dimension ref="A1:AH88"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
     <col min="1" max="1" width="13.1" customWidth="1"/>
@@ -1544,9 +1583,7 @@
       <c r="B7" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="C7" s="2" t="s">
-        <v>30</v>
-      </c>
+      <c r="C7" s="2"/>
       <c r="D7" s="4" t="s">
         <v>23</v>
       </c>
@@ -1554,13 +1591,13 @@
         <v>14</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>21</v>
+        <v>30</v>
       </c>
       <c r="G7" s="4" t="s">
         <v>24</v>
       </c>
       <c r="H7" s="4" t="s">
-        <v>31</v>
+        <v>17</v>
       </c>
       <c r="I7" s="4"/>
       <c r="J7" s="4"/>
@@ -1594,13 +1631,13 @@
     <row r="8" spans="1:34">
       <c r="A8" s="3"/>
       <c r="B8" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="C8" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="C8" s="2" t="s">
-        <v>30</v>
-      </c>
       <c r="D8" s="4" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="E8" s="4" t="s">
         <v>14</v>
@@ -1609,10 +1646,10 @@
         <v>21</v>
       </c>
       <c r="G8" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="H8" s="4" t="s">
         <v>33</v>
-      </c>
-      <c r="H8" s="4" t="s">
-        <v>31</v>
       </c>
       <c r="I8" s="4"/>
       <c r="J8" s="4"/>
@@ -1648,9 +1685,11 @@
       <c r="B9" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="C9" s="2"/>
+      <c r="C9" s="2" t="s">
+        <v>32</v>
+      </c>
       <c r="D9" s="4" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="E9" s="4" t="s">
         <v>14</v>
@@ -1661,14 +1700,12 @@
       <c r="G9" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="H9" s="4"/>
+      <c r="H9" s="4" t="s">
+        <v>33</v>
+      </c>
       <c r="I9" s="4"/>
-      <c r="J9" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="K9" s="4" t="s">
-        <v>37</v>
-      </c>
+      <c r="J9" s="4"/>
+      <c r="K9" s="4"/>
       <c r="L9" s="4"/>
       <c r="M9" s="4" t="s">
         <v>18</v>
@@ -1698,7 +1735,7 @@
     <row r="10" spans="1:34">
       <c r="A10" s="3"/>
       <c r="B10" s="4" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="C10" s="2"/>
       <c r="D10" s="4" t="s">
@@ -1711,15 +1748,15 @@
         <v>21</v>
       </c>
       <c r="G10" s="4" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="H10" s="4"/>
       <c r="I10" s="4"/>
       <c r="J10" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="K10" s="4" t="s">
         <v>39</v>
-      </c>
-      <c r="K10" s="4" t="s">
-        <v>40</v>
       </c>
       <c r="L10" s="4"/>
       <c r="M10" s="4" t="s">
@@ -1750,7 +1787,7 @@
     <row r="11" spans="1:34">
       <c r="A11" s="3"/>
       <c r="B11" s="4" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C11" s="2"/>
       <c r="D11" s="4" t="s">
@@ -1763,15 +1800,15 @@
         <v>21</v>
       </c>
       <c r="G11" s="4" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="H11" s="4"/>
       <c r="I11" s="4"/>
       <c r="J11" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="K11" s="4" t="s">
         <v>42</v>
-      </c>
-      <c r="K11" s="4" t="s">
-        <v>43</v>
       </c>
       <c r="L11" s="4"/>
       <c r="M11" s="4" t="s">
@@ -1802,7 +1839,7 @@
     <row r="12" spans="1:34">
       <c r="A12" s="3"/>
       <c r="B12" s="4" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C12" s="2"/>
       <c r="D12" s="4" t="s">
@@ -1815,16 +1852,16 @@
         <v>21</v>
       </c>
       <c r="G12" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="H12" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="H12" s="4"/>
+      <c r="I12" s="4"/>
+      <c r="J12" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="K12" s="4" t="s">
         <v>45</v>
       </c>
-      <c r="I12" s="4" t="s">
-        <v>46</v>
-      </c>
-      <c r="J12" s="4"/>
-      <c r="K12" s="4"/>
       <c r="L12" s="4"/>
       <c r="M12" s="4" t="s">
         <v>18</v>
@@ -1854,7 +1891,7 @@
     <row r="13" spans="1:34">
       <c r="A13" s="3"/>
       <c r="B13" s="4" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C13" s="2"/>
       <c r="D13" s="4" t="s">
@@ -1870,7 +1907,7 @@
         <v>24</v>
       </c>
       <c r="H13" s="4" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="I13" s="4" t="s">
         <v>48</v>
@@ -1922,7 +1959,7 @@
         <v>24</v>
       </c>
       <c r="H14" s="4" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="I14" s="4" t="s">
         <v>50</v>
@@ -1973,7 +2010,9 @@
       <c r="G15" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="H15" s="4"/>
+      <c r="H15" s="4" t="s">
+        <v>47</v>
+      </c>
       <c r="I15" s="4" t="s">
         <v>52</v>
       </c>
@@ -2012,7 +2051,7 @@
       </c>
       <c r="C16" s="2"/>
       <c r="D16" s="4" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="E16" s="4" t="s">
         <v>14</v>
@@ -2021,15 +2060,15 @@
         <v>21</v>
       </c>
       <c r="G16" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="H16" s="4"/>
+      <c r="I16" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="H16" s="4"/>
-      <c r="I16" s="4"/>
       <c r="J16" s="4"/>
       <c r="K16" s="4"/>
-      <c r="L16" s="4" t="s">
-        <v>55</v>
-      </c>
+      <c r="L16" s="4"/>
       <c r="M16" s="4" t="s">
         <v>18</v>
       </c>
@@ -2058,7 +2097,7 @@
     <row r="17" spans="1:34">
       <c r="A17" s="3"/>
       <c r="B17" s="4" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C17" s="2"/>
       <c r="D17" s="4" t="s">
@@ -2071,7 +2110,7 @@
         <v>21</v>
       </c>
       <c r="G17" s="4" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="H17" s="4"/>
       <c r="I17" s="4"/>
@@ -2121,7 +2160,7 @@
         <v>21</v>
       </c>
       <c r="G18" s="4" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="H18" s="4"/>
       <c r="I18" s="4"/>
@@ -2162,24 +2201,24 @@
       </c>
       <c r="C19" s="2"/>
       <c r="D19" s="4" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="E19" s="4" t="s">
         <v>14</v>
       </c>
       <c r="F19" s="4" t="s">
-        <v>61</v>
+        <v>21</v>
       </c>
       <c r="G19" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="H19" s="4" t="s">
-        <v>17</v>
-      </c>
+        <v>56</v>
+      </c>
+      <c r="H19" s="4"/>
       <c r="I19" s="4"/>
       <c r="J19" s="4"/>
       <c r="K19" s="4"/>
-      <c r="L19" s="4"/>
+      <c r="L19" s="4" t="s">
+        <v>61</v>
+      </c>
       <c r="M19" s="4" t="s">
         <v>18</v>
       </c>
@@ -2212,24 +2251,24 @@
       </c>
       <c r="C20" s="2"/>
       <c r="D20" s="4" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="E20" s="4" t="s">
         <v>14</v>
       </c>
       <c r="F20" s="4" t="s">
-        <v>63</v>
+        <v>21</v>
       </c>
       <c r="G20" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="H20" s="4" t="s">
-        <v>17</v>
-      </c>
+        <v>56</v>
+      </c>
+      <c r="H20" s="4"/>
       <c r="I20" s="4"/>
       <c r="J20" s="4"/>
       <c r="K20" s="4"/>
-      <c r="L20" s="4"/>
+      <c r="L20" s="4" t="s">
+        <v>63</v>
+      </c>
       <c r="M20" s="4" t="s">
         <v>18</v>
       </c>
@@ -2262,24 +2301,24 @@
       </c>
       <c r="C21" s="2"/>
       <c r="D21" s="4" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="E21" s="4" t="s">
         <v>14</v>
       </c>
       <c r="F21" s="4" t="s">
-        <v>65</v>
+        <v>21</v>
       </c>
       <c r="G21" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="H21" s="4" t="s">
-        <v>17</v>
-      </c>
+        <v>56</v>
+      </c>
+      <c r="H21" s="4"/>
       <c r="I21" s="4"/>
       <c r="J21" s="4"/>
       <c r="K21" s="4"/>
-      <c r="L21" s="4"/>
+      <c r="L21" s="4" t="s">
+        <v>65</v>
+      </c>
       <c r="M21" s="4" t="s">
         <v>18</v>
       </c>
@@ -2312,22 +2351,24 @@
       </c>
       <c r="C22" s="2"/>
       <c r="D22" s="4" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="E22" s="4" t="s">
-        <v>67</v>
+        <v>14</v>
       </c>
       <c r="F22" s="4" t="s">
-        <v>63</v>
-      </c>
-      <c r="G22" s="4"/>
-      <c r="H22" s="4" t="s">
-        <v>17</v>
-      </c>
+        <v>21</v>
+      </c>
+      <c r="G22" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="H22" s="4"/>
       <c r="I22" s="4"/>
       <c r="J22" s="4"/>
       <c r="K22" s="4"/>
-      <c r="L22" s="4"/>
+      <c r="L22" s="4" t="s">
+        <v>67</v>
+      </c>
       <c r="M22" s="4" t="s">
         <v>18</v>
       </c>
@@ -2363,12 +2404,14 @@
         <v>23</v>
       </c>
       <c r="E23" s="4" t="s">
-        <v>67</v>
+        <v>14</v>
       </c>
       <c r="F23" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="G23" s="4"/>
+        <v>69</v>
+      </c>
+      <c r="G23" s="4" t="s">
+        <v>24</v>
+      </c>
       <c r="H23" s="4" t="s">
         <v>17</v>
       </c>
@@ -2404,19 +2447,21 @@
     <row r="24" spans="1:34">
       <c r="A24" s="3"/>
       <c r="B24" s="4" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="C24" s="2"/>
       <c r="D24" s="4" t="s">
         <v>23</v>
       </c>
       <c r="E24" s="4" t="s">
-        <v>67</v>
+        <v>14</v>
       </c>
       <c r="F24" s="4" t="s">
-        <v>70</v>
-      </c>
-      <c r="G24" s="4"/>
+        <v>71</v>
+      </c>
+      <c r="G24" s="4" t="s">
+        <v>24</v>
+      </c>
       <c r="H24" s="4" t="s">
         <v>17</v>
       </c>
@@ -2449,49 +2494,44 @@
       <c r="AG24" s="3"/>
       <c r="AH24" s="3"/>
     </row>
-    <row r="25" spans="2:34">
-      <c r="B25" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="C25" s="2" t="s">
+    <row r="25" spans="1:34">
+      <c r="A25" s="3"/>
+      <c r="B25" s="4" t="s">
         <v>72</v>
       </c>
-      <c r="D25" s="2" t="s">
+      <c r="C25" s="2"/>
+      <c r="D25" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="E25" s="2" t="s">
+      <c r="E25" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="F25" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="G25" s="2" t="s">
+      <c r="F25" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="G25" s="4" t="s">
         <v>24</v>
       </c>
       <c r="H25" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="I25" s="4" t="s">
-        <v>74</v>
-      </c>
-      <c r="J25" s="4" t="s">
-        <v>75</v>
-      </c>
-      <c r="K25" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="L25" s="2" t="s">
-        <v>77</v>
-      </c>
-      <c r="M25" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="N25" s="2"/>
-      <c r="O25" s="2"/>
-      <c r="P25" s="2"/>
-      <c r="Q25" s="2"/>
-      <c r="R25" s="2"/>
-      <c r="S25" s="2"/>
+        <v>17</v>
+      </c>
+      <c r="I25" s="4"/>
+      <c r="J25" s="4"/>
+      <c r="K25" s="4"/>
+      <c r="L25" s="4"/>
+      <c r="M25" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="N25" s="4"/>
+      <c r="O25" s="4"/>
+      <c r="P25" s="4"/>
+      <c r="Q25" s="4"/>
+      <c r="R25" s="4"/>
+      <c r="S25" s="4"/>
+      <c r="T25" s="3"/>
+      <c r="U25" s="3"/>
+      <c r="V25" s="3"/>
+      <c r="W25" s="3"/>
       <c r="X25" s="3"/>
       <c r="Y25" s="3"/>
       <c r="Z25" s="3"/>
@@ -2506,18 +2546,32 @@
     </row>
     <row r="26" spans="1:34">
       <c r="A26" s="3"/>
-      <c r="B26" s="4"/>
-      <c r="C26" s="4"/>
-      <c r="D26" s="4"/>
-      <c r="E26" s="4"/>
-      <c r="F26" s="4"/>
-      <c r="G26" s="4"/>
-      <c r="H26" s="4"/>
+      <c r="B26" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="C26" s="2"/>
+      <c r="D26" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="E26" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="F26" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="G26" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="H26" s="4" t="s">
+        <v>17</v>
+      </c>
       <c r="I26" s="4"/>
       <c r="J26" s="4"/>
       <c r="K26" s="4"/>
       <c r="L26" s="4"/>
-      <c r="M26" s="4"/>
+      <c r="M26" s="4" t="s">
+        <v>18</v>
+      </c>
       <c r="N26" s="4"/>
       <c r="O26" s="4"/>
       <c r="P26" s="4"/>
@@ -2540,20 +2594,32 @@
       <c r="AG26" s="3"/>
       <c r="AH26" s="3"/>
     </row>
-    <row r="27" s="1" customFormat="1" spans="1:34">
+    <row r="27" spans="1:34">
       <c r="A27" s="3"/>
-      <c r="B27" s="4"/>
-      <c r="C27" s="4"/>
-      <c r="D27" s="4"/>
-      <c r="E27" s="4"/>
-      <c r="F27" s="4"/>
+      <c r="B27" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="C27" s="2"/>
+      <c r="D27" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="E27" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="F27" s="4" t="s">
+        <v>73</v>
+      </c>
       <c r="G27" s="4"/>
-      <c r="H27" s="4"/>
+      <c r="H27" s="4" t="s">
+        <v>17</v>
+      </c>
       <c r="I27" s="4"/>
       <c r="J27" s="4"/>
       <c r="K27" s="4"/>
       <c r="L27" s="4"/>
-      <c r="M27" s="4"/>
+      <c r="M27" s="4" t="s">
+        <v>18</v>
+      </c>
       <c r="N27" s="4"/>
       <c r="O27" s="4"/>
       <c r="P27" s="4"/>
@@ -2576,20 +2642,32 @@
       <c r="AG27" s="3"/>
       <c r="AH27" s="3"/>
     </row>
-    <row r="28" s="1" customFormat="1" spans="1:34">
+    <row r="28" spans="1:34">
       <c r="A28" s="3"/>
-      <c r="B28" s="4"/>
-      <c r="C28" s="4"/>
-      <c r="D28" s="4"/>
-      <c r="E28" s="4"/>
-      <c r="F28" s="4"/>
+      <c r="B28" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="C28" s="2"/>
+      <c r="D28" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="E28" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="F28" s="4" t="s">
+        <v>21</v>
+      </c>
       <c r="G28" s="4"/>
-      <c r="H28" s="4"/>
+      <c r="H28" s="4" t="s">
+        <v>17</v>
+      </c>
       <c r="I28" s="4"/>
       <c r="J28" s="4"/>
       <c r="K28" s="4"/>
       <c r="L28" s="4"/>
-      <c r="M28" s="4"/>
+      <c r="M28" s="4" t="s">
+        <v>18</v>
+      </c>
       <c r="N28" s="4"/>
       <c r="O28" s="4"/>
       <c r="P28" s="4"/>
@@ -2614,18 +2692,30 @@
     </row>
     <row r="29" spans="1:34">
       <c r="A29" s="3"/>
-      <c r="B29" s="4"/>
-      <c r="C29" s="4"/>
-      <c r="D29" s="4"/>
-      <c r="E29" s="4"/>
-      <c r="F29" s="4"/>
+      <c r="B29" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="C29" s="2"/>
+      <c r="D29" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="E29" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="F29" s="4" t="s">
+        <v>80</v>
+      </c>
       <c r="G29" s="4"/>
-      <c r="H29" s="4"/>
+      <c r="H29" s="4" t="s">
+        <v>17</v>
+      </c>
       <c r="I29" s="4"/>
       <c r="J29" s="4"/>
       <c r="K29" s="4"/>
       <c r="L29" s="4"/>
-      <c r="M29" s="4"/>
+      <c r="M29" s="4" t="s">
+        <v>18</v>
+      </c>
       <c r="N29" s="4"/>
       <c r="O29" s="4"/>
       <c r="P29" s="4"/>
@@ -2650,18 +2740,30 @@
     </row>
     <row r="30" spans="1:34">
       <c r="A30" s="3"/>
-      <c r="B30" s="4"/>
-      <c r="C30" s="4"/>
-      <c r="D30" s="4"/>
-      <c r="E30" s="4"/>
-      <c r="F30" s="4"/>
+      <c r="B30" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="C30" s="2"/>
+      <c r="D30" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="E30" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="F30" s="4" t="s">
+        <v>30</v>
+      </c>
       <c r="G30" s="4"/>
-      <c r="H30" s="4"/>
+      <c r="H30" s="4" t="s">
+        <v>17</v>
+      </c>
       <c r="I30" s="4"/>
       <c r="J30" s="4"/>
       <c r="K30" s="4"/>
       <c r="L30" s="4"/>
-      <c r="M30" s="4"/>
+      <c r="M30" s="4" t="s">
+        <v>18</v>
+      </c>
       <c r="N30" s="4"/>
       <c r="O30" s="4"/>
       <c r="P30" s="4"/>
@@ -2686,18 +2788,30 @@
     </row>
     <row r="31" spans="1:34">
       <c r="A31" s="3"/>
-      <c r="B31" s="4"/>
-      <c r="C31" s="4"/>
-      <c r="D31" s="4"/>
-      <c r="E31" s="4"/>
-      <c r="F31" s="4"/>
+      <c r="B31" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="C31" s="2"/>
+      <c r="D31" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="E31" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="F31" s="4" t="s">
+        <v>26</v>
+      </c>
       <c r="G31" s="4"/>
-      <c r="H31" s="4"/>
+      <c r="H31" s="4" t="s">
+        <v>17</v>
+      </c>
       <c r="I31" s="4"/>
       <c r="J31" s="4"/>
       <c r="K31" s="4"/>
       <c r="L31" s="4"/>
-      <c r="M31" s="4"/>
+      <c r="M31" s="4" t="s">
+        <v>18</v>
+      </c>
       <c r="N31" s="4"/>
       <c r="O31" s="4"/>
       <c r="P31" s="4"/>
@@ -2722,18 +2836,30 @@
     </row>
     <row r="32" spans="1:34">
       <c r="A32" s="3"/>
-      <c r="B32" s="4"/>
-      <c r="C32" s="4"/>
-      <c r="D32" s="4"/>
-      <c r="E32" s="4"/>
-      <c r="F32" s="4"/>
+      <c r="B32" s="4" t="s">
+        <v>83</v>
+      </c>
+      <c r="C32" s="2"/>
+      <c r="D32" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="E32" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="F32" s="4" t="s">
+        <v>28</v>
+      </c>
       <c r="G32" s="4"/>
-      <c r="H32" s="4"/>
+      <c r="H32" s="4" t="s">
+        <v>17</v>
+      </c>
       <c r="I32" s="4"/>
       <c r="J32" s="4"/>
       <c r="K32" s="4"/>
       <c r="L32" s="4"/>
-      <c r="M32" s="4"/>
+      <c r="M32" s="4" t="s">
+        <v>18</v>
+      </c>
       <c r="N32" s="4"/>
       <c r="O32" s="4"/>
       <c r="P32" s="4"/>
@@ -2756,30 +2882,49 @@
       <c r="AG32" s="3"/>
       <c r="AH32" s="3"/>
     </row>
-    <row r="33" spans="1:34">
-      <c r="A33" s="3"/>
-      <c r="B33" s="4"/>
-      <c r="C33" s="4"/>
-      <c r="D33" s="4"/>
-      <c r="E33" s="4"/>
-      <c r="F33" s="4"/>
-      <c r="G33" s="4"/>
-      <c r="H33" s="4"/>
-      <c r="I33" s="4"/>
-      <c r="J33" s="4"/>
-      <c r="K33" s="4"/>
-      <c r="L33" s="4"/>
-      <c r="M33" s="4"/>
-      <c r="N33" s="4"/>
-      <c r="O33" s="4"/>
-      <c r="P33" s="4"/>
-      <c r="Q33" s="4"/>
-      <c r="R33" s="4"/>
-      <c r="S33" s="4"/>
-      <c r="T33" s="3"/>
-      <c r="U33" s="3"/>
-      <c r="V33" s="3"/>
-      <c r="W33" s="3"/>
+    <row r="33" spans="2:34">
+      <c r="B33" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="C33" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="D33" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="E33" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="F33" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="G33" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="H33" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="I33" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="J33" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="K33" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="L33" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="M33" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="N33" s="2"/>
+      <c r="O33" s="2"/>
+      <c r="P33" s="2"/>
+      <c r="Q33" s="2"/>
+      <c r="R33" s="2"/>
+      <c r="S33" s="2"/>
       <c r="X33" s="3"/>
       <c r="Y33" s="3"/>
       <c r="Z33" s="3"/>
@@ -2828,7 +2973,7 @@
       <c r="AG34" s="3"/>
       <c r="AH34" s="3"/>
     </row>
-    <row r="35" spans="1:34">
+    <row r="35" s="1" customFormat="1" spans="1:34">
       <c r="A35" s="3"/>
       <c r="B35" s="4"/>
       <c r="C35" s="4"/>
@@ -2864,7 +3009,7 @@
       <c r="AG35" s="3"/>
       <c r="AH35" s="3"/>
     </row>
-    <row r="36" spans="1:34">
+    <row r="36" s="1" customFormat="1" spans="1:34">
       <c r="A36" s="3"/>
       <c r="B36" s="4"/>
       <c r="C36" s="4"/>
@@ -3157,7 +3302,7 @@
       <c r="B44" s="4"/>
       <c r="C44" s="4"/>
       <c r="D44" s="4"/>
-      <c r="E44" s="5"/>
+      <c r="E44" s="4"/>
       <c r="F44" s="4"/>
       <c r="G44" s="4"/>
       <c r="H44" s="4"/>
@@ -3193,7 +3338,7 @@
       <c r="B45" s="4"/>
       <c r="C45" s="4"/>
       <c r="D45" s="4"/>
-      <c r="E45" s="5"/>
+      <c r="E45" s="4"/>
       <c r="F45" s="4"/>
       <c r="G45" s="4"/>
       <c r="H45" s="4"/>
@@ -3229,7 +3374,7 @@
       <c r="B46" s="4"/>
       <c r="C46" s="4"/>
       <c r="D46" s="4"/>
-      <c r="E46" s="5"/>
+      <c r="E46" s="4"/>
       <c r="F46" s="4"/>
       <c r="G46" s="4"/>
       <c r="H46" s="4"/>
@@ -3409,7 +3554,7 @@
       <c r="B51" s="4"/>
       <c r="C51" s="4"/>
       <c r="D51" s="4"/>
-      <c r="E51" s="5"/>
+      <c r="E51" s="4"/>
       <c r="F51" s="4"/>
       <c r="G51" s="4"/>
       <c r="H51" s="4"/>
@@ -3445,7 +3590,7 @@
       <c r="B52" s="4"/>
       <c r="C52" s="4"/>
       <c r="D52" s="4"/>
-      <c r="E52" s="4"/>
+      <c r="E52" s="5"/>
       <c r="F52" s="4"/>
       <c r="G52" s="4"/>
       <c r="H52" s="4"/>
@@ -3481,7 +3626,7 @@
       <c r="B53" s="4"/>
       <c r="C53" s="4"/>
       <c r="D53" s="4"/>
-      <c r="E53" s="4"/>
+      <c r="E53" s="5"/>
       <c r="F53" s="4"/>
       <c r="G53" s="4"/>
       <c r="H53" s="4"/>
@@ -3517,7 +3662,7 @@
       <c r="B54" s="4"/>
       <c r="C54" s="4"/>
       <c r="D54" s="4"/>
-      <c r="E54" s="4"/>
+      <c r="E54" s="5"/>
       <c r="F54" s="4"/>
       <c r="G54" s="4"/>
       <c r="H54" s="4"/>
@@ -3697,7 +3842,7 @@
       <c r="B59" s="4"/>
       <c r="C59" s="4"/>
       <c r="D59" s="4"/>
-      <c r="E59" s="4"/>
+      <c r="E59" s="5"/>
       <c r="F59" s="4"/>
       <c r="G59" s="4"/>
       <c r="H59" s="4"/>
@@ -3728,101 +3873,293 @@
       <c r="AG59" s="3"/>
       <c r="AH59" s="3"/>
     </row>
-    <row r="67" spans="1:23">
-      <c r="A67" s="2"/>
-      <c r="B67" s="2"/>
-      <c r="C67" s="2"/>
-      <c r="D67" s="2"/>
-      <c r="R67" s="2"/>
-      <c r="T67" s="2"/>
-      <c r="U67" s="2"/>
-      <c r="V67" s="2"/>
-      <c r="W67" s="2"/>
-    </row>
-    <row r="68" spans="1:23">
-      <c r="A68" s="2"/>
-      <c r="B68" s="2"/>
-      <c r="C68" s="2"/>
-      <c r="D68" s="2"/>
-      <c r="E68" s="2"/>
-      <c r="R68" s="2"/>
-      <c r="S68" s="2"/>
-      <c r="T68" s="2"/>
-      <c r="U68" s="2"/>
-      <c r="V68" s="2"/>
-      <c r="W68" s="2"/>
-    </row>
-    <row r="69" spans="1:23">
-      <c r="A69" s="2"/>
-      <c r="B69" s="2"/>
-      <c r="C69" s="2"/>
-      <c r="D69" s="2"/>
-      <c r="R69" s="2"/>
-      <c r="S69" s="2"/>
-      <c r="T69" s="2"/>
-      <c r="U69" s="2"/>
-      <c r="V69" s="2"/>
-      <c r="W69" s="2"/>
-    </row>
-    <row r="70" spans="1:23">
-      <c r="A70" s="2"/>
-      <c r="B70" s="2"/>
-      <c r="C70" s="2"/>
-      <c r="D70" s="2"/>
-      <c r="R70" s="2"/>
-      <c r="S70" s="2"/>
-      <c r="T70" s="2"/>
-      <c r="U70" s="2"/>
-      <c r="V70" s="2"/>
-      <c r="W70" s="2"/>
-    </row>
-    <row r="71" spans="1:23">
-      <c r="A71" s="2"/>
-      <c r="B71" s="2"/>
-      <c r="C71" s="2"/>
-      <c r="D71" s="2"/>
-      <c r="R71" s="2"/>
-      <c r="S71" s="2"/>
-      <c r="T71" s="2"/>
-      <c r="U71" s="2"/>
-      <c r="V71" s="2"/>
-      <c r="W71" s="2"/>
-    </row>
-    <row r="72" spans="1:23">
-      <c r="A72" s="2"/>
-      <c r="B72" s="2"/>
-      <c r="C72" s="2"/>
-      <c r="D72" s="2"/>
-      <c r="R72" s="2"/>
-      <c r="S72" s="2"/>
-      <c r="T72" s="2"/>
-      <c r="U72" s="2"/>
-      <c r="V72" s="2"/>
-      <c r="W72" s="2"/>
-    </row>
-    <row r="73" spans="1:23">
-      <c r="A73" s="2"/>
-      <c r="B73" s="2"/>
-      <c r="C73" s="2"/>
-      <c r="D73" s="2"/>
-      <c r="R73" s="2"/>
-      <c r="S73" s="2"/>
-      <c r="T73" s="2"/>
-      <c r="U73" s="2"/>
-      <c r="V73" s="2"/>
-      <c r="W73" s="2"/>
-    </row>
-    <row r="74" spans="1:23">
-      <c r="A74" s="2"/>
-      <c r="B74" s="2"/>
-      <c r="C74" s="2"/>
-      <c r="D74" s="2"/>
-      <c r="R74" s="2"/>
-      <c r="S74" s="2"/>
-      <c r="T74" s="2"/>
-      <c r="U74" s="2"/>
-      <c r="V74" s="2"/>
-      <c r="W74" s="2"/>
+    <row r="60" spans="1:34">
+      <c r="A60" s="3"/>
+      <c r="B60" s="4"/>
+      <c r="C60" s="4"/>
+      <c r="D60" s="4"/>
+      <c r="E60" s="4"/>
+      <c r="F60" s="4"/>
+      <c r="G60" s="4"/>
+      <c r="H60" s="4"/>
+      <c r="I60" s="4"/>
+      <c r="J60" s="4"/>
+      <c r="K60" s="4"/>
+      <c r="L60" s="4"/>
+      <c r="M60" s="4"/>
+      <c r="N60" s="4"/>
+      <c r="O60" s="4"/>
+      <c r="P60" s="4"/>
+      <c r="Q60" s="4"/>
+      <c r="R60" s="4"/>
+      <c r="S60" s="4"/>
+      <c r="T60" s="3"/>
+      <c r="U60" s="3"/>
+      <c r="V60" s="3"/>
+      <c r="W60" s="3"/>
+      <c r="X60" s="3"/>
+      <c r="Y60" s="3"/>
+      <c r="Z60" s="3"/>
+      <c r="AA60" s="3"/>
+      <c r="AB60" s="3"/>
+      <c r="AC60" s="3"/>
+      <c r="AD60" s="3"/>
+      <c r="AE60" s="3"/>
+      <c r="AF60" s="3"/>
+      <c r="AG60" s="3"/>
+      <c r="AH60" s="3"/>
+    </row>
+    <row r="61" spans="1:34">
+      <c r="A61" s="3"/>
+      <c r="B61" s="4"/>
+      <c r="C61" s="4"/>
+      <c r="D61" s="4"/>
+      <c r="E61" s="4"/>
+      <c r="F61" s="4"/>
+      <c r="G61" s="4"/>
+      <c r="H61" s="4"/>
+      <c r="I61" s="4"/>
+      <c r="J61" s="4"/>
+      <c r="K61" s="4"/>
+      <c r="L61" s="4"/>
+      <c r="M61" s="4"/>
+      <c r="N61" s="4"/>
+      <c r="O61" s="4"/>
+      <c r="P61" s="4"/>
+      <c r="Q61" s="4"/>
+      <c r="R61" s="4"/>
+      <c r="S61" s="4"/>
+      <c r="T61" s="3"/>
+      <c r="U61" s="3"/>
+      <c r="V61" s="3"/>
+      <c r="W61" s="3"/>
+      <c r="X61" s="3"/>
+      <c r="Y61" s="3"/>
+      <c r="Z61" s="3"/>
+      <c r="AA61" s="3"/>
+      <c r="AB61" s="3"/>
+      <c r="AC61" s="3"/>
+      <c r="AD61" s="3"/>
+      <c r="AE61" s="3"/>
+      <c r="AF61" s="3"/>
+      <c r="AG61" s="3"/>
+      <c r="AH61" s="3"/>
+    </row>
+    <row r="62" spans="1:34">
+      <c r="A62" s="3"/>
+      <c r="B62" s="4"/>
+      <c r="C62" s="4"/>
+      <c r="D62" s="4"/>
+      <c r="E62" s="4"/>
+      <c r="F62" s="4"/>
+      <c r="G62" s="4"/>
+      <c r="H62" s="4"/>
+      <c r="I62" s="4"/>
+      <c r="J62" s="4"/>
+      <c r="K62" s="4"/>
+      <c r="L62" s="4"/>
+      <c r="M62" s="4"/>
+      <c r="N62" s="4"/>
+      <c r="O62" s="4"/>
+      <c r="P62" s="4"/>
+      <c r="Q62" s="4"/>
+      <c r="R62" s="4"/>
+      <c r="S62" s="4"/>
+      <c r="T62" s="3"/>
+      <c r="U62" s="3"/>
+      <c r="V62" s="3"/>
+      <c r="W62" s="3"/>
+      <c r="X62" s="3"/>
+      <c r="Y62" s="3"/>
+      <c r="Z62" s="3"/>
+      <c r="AA62" s="3"/>
+      <c r="AB62" s="3"/>
+      <c r="AC62" s="3"/>
+      <c r="AD62" s="3"/>
+      <c r="AE62" s="3"/>
+      <c r="AF62" s="3"/>
+      <c r="AG62" s="3"/>
+      <c r="AH62" s="3"/>
+    </row>
+    <row r="63" spans="1:34">
+      <c r="A63" s="3"/>
+      <c r="B63" s="4"/>
+      <c r="C63" s="4"/>
+      <c r="D63" s="4"/>
+      <c r="E63" s="4"/>
+      <c r="F63" s="4"/>
+      <c r="G63" s="4"/>
+      <c r="H63" s="4"/>
+      <c r="I63" s="4"/>
+      <c r="J63" s="4"/>
+      <c r="K63" s="4"/>
+      <c r="L63" s="4"/>
+      <c r="M63" s="4"/>
+      <c r="N63" s="4"/>
+      <c r="O63" s="4"/>
+      <c r="P63" s="4"/>
+      <c r="Q63" s="4"/>
+      <c r="R63" s="4"/>
+      <c r="S63" s="4"/>
+      <c r="T63" s="3"/>
+      <c r="U63" s="3"/>
+      <c r="V63" s="3"/>
+      <c r="W63" s="3"/>
+      <c r="X63" s="3"/>
+      <c r="Y63" s="3"/>
+      <c r="Z63" s="3"/>
+      <c r="AA63" s="3"/>
+      <c r="AB63" s="3"/>
+      <c r="AC63" s="3"/>
+      <c r="AD63" s="3"/>
+      <c r="AE63" s="3"/>
+      <c r="AF63" s="3"/>
+      <c r="AG63" s="3"/>
+      <c r="AH63" s="3"/>
+    </row>
+    <row r="64" spans="1:34">
+      <c r="A64" s="3"/>
+      <c r="B64" s="4"/>
+      <c r="C64" s="4"/>
+      <c r="D64" s="4"/>
+      <c r="E64" s="4"/>
+      <c r="F64" s="4"/>
+      <c r="G64" s="4"/>
+      <c r="H64" s="4"/>
+      <c r="I64" s="4"/>
+      <c r="J64" s="4"/>
+      <c r="K64" s="4"/>
+      <c r="L64" s="4"/>
+      <c r="M64" s="4"/>
+      <c r="N64" s="4"/>
+      <c r="O64" s="4"/>
+      <c r="P64" s="4"/>
+      <c r="Q64" s="4"/>
+      <c r="R64" s="4"/>
+      <c r="S64" s="4"/>
+      <c r="T64" s="3"/>
+      <c r="U64" s="3"/>
+      <c r="V64" s="3"/>
+      <c r="W64" s="3"/>
+      <c r="X64" s="3"/>
+      <c r="Y64" s="3"/>
+      <c r="Z64" s="3"/>
+      <c r="AA64" s="3"/>
+      <c r="AB64" s="3"/>
+      <c r="AC64" s="3"/>
+      <c r="AD64" s="3"/>
+      <c r="AE64" s="3"/>
+      <c r="AF64" s="3"/>
+      <c r="AG64" s="3"/>
+      <c r="AH64" s="3"/>
+    </row>
+    <row r="65" spans="1:34">
+      <c r="A65" s="3"/>
+      <c r="B65" s="4"/>
+      <c r="C65" s="4"/>
+      <c r="D65" s="4"/>
+      <c r="E65" s="4"/>
+      <c r="F65" s="4"/>
+      <c r="G65" s="4"/>
+      <c r="H65" s="4"/>
+      <c r="I65" s="4"/>
+      <c r="J65" s="4"/>
+      <c r="K65" s="4"/>
+      <c r="L65" s="4"/>
+      <c r="M65" s="4"/>
+      <c r="N65" s="4"/>
+      <c r="O65" s="4"/>
+      <c r="P65" s="4"/>
+      <c r="Q65" s="4"/>
+      <c r="R65" s="4"/>
+      <c r="S65" s="4"/>
+      <c r="T65" s="3"/>
+      <c r="U65" s="3"/>
+      <c r="V65" s="3"/>
+      <c r="W65" s="3"/>
+      <c r="X65" s="3"/>
+      <c r="Y65" s="3"/>
+      <c r="Z65" s="3"/>
+      <c r="AA65" s="3"/>
+      <c r="AB65" s="3"/>
+      <c r="AC65" s="3"/>
+      <c r="AD65" s="3"/>
+      <c r="AE65" s="3"/>
+      <c r="AF65" s="3"/>
+      <c r="AG65" s="3"/>
+      <c r="AH65" s="3"/>
+    </row>
+    <row r="66" spans="1:34">
+      <c r="A66" s="3"/>
+      <c r="B66" s="4"/>
+      <c r="C66" s="4"/>
+      <c r="D66" s="4"/>
+      <c r="E66" s="4"/>
+      <c r="F66" s="4"/>
+      <c r="G66" s="4"/>
+      <c r="H66" s="4"/>
+      <c r="I66" s="4"/>
+      <c r="J66" s="4"/>
+      <c r="K66" s="4"/>
+      <c r="L66" s="4"/>
+      <c r="M66" s="4"/>
+      <c r="N66" s="4"/>
+      <c r="O66" s="4"/>
+      <c r="P66" s="4"/>
+      <c r="Q66" s="4"/>
+      <c r="R66" s="4"/>
+      <c r="S66" s="4"/>
+      <c r="T66" s="3"/>
+      <c r="U66" s="3"/>
+      <c r="V66" s="3"/>
+      <c r="W66" s="3"/>
+      <c r="X66" s="3"/>
+      <c r="Y66" s="3"/>
+      <c r="Z66" s="3"/>
+      <c r="AA66" s="3"/>
+      <c r="AB66" s="3"/>
+      <c r="AC66" s="3"/>
+      <c r="AD66" s="3"/>
+      <c r="AE66" s="3"/>
+      <c r="AF66" s="3"/>
+      <c r="AG66" s="3"/>
+      <c r="AH66" s="3"/>
+    </row>
+    <row r="67" spans="1:34">
+      <c r="A67" s="3"/>
+      <c r="B67" s="4"/>
+      <c r="C67" s="4"/>
+      <c r="D67" s="4"/>
+      <c r="E67" s="4"/>
+      <c r="F67" s="4"/>
+      <c r="G67" s="4"/>
+      <c r="H67" s="4"/>
+      <c r="I67" s="4"/>
+      <c r="J67" s="4"/>
+      <c r="K67" s="4"/>
+      <c r="L67" s="4"/>
+      <c r="M67" s="4"/>
+      <c r="N67" s="4"/>
+      <c r="O67" s="4"/>
+      <c r="P67" s="4"/>
+      <c r="Q67" s="4"/>
+      <c r="R67" s="4"/>
+      <c r="S67" s="4"/>
+      <c r="T67" s="3"/>
+      <c r="U67" s="3"/>
+      <c r="V67" s="3"/>
+      <c r="W67" s="3"/>
+      <c r="X67" s="3"/>
+      <c r="Y67" s="3"/>
+      <c r="Z67" s="3"/>
+      <c r="AA67" s="3"/>
+      <c r="AB67" s="3"/>
+      <c r="AC67" s="3"/>
+      <c r="AD67" s="3"/>
+      <c r="AE67" s="3"/>
+      <c r="AF67" s="3"/>
+      <c r="AG67" s="3"/>
+      <c r="AH67" s="3"/>
     </row>
     <row r="75" spans="1:23">
       <c r="A75" s="2"/>
@@ -3830,7 +4167,6 @@
       <c r="C75" s="2"/>
       <c r="D75" s="2"/>
       <c r="R75" s="2"/>
-      <c r="S75" s="2"/>
       <c r="T75" s="2"/>
       <c r="U75" s="2"/>
       <c r="V75" s="2"/>
@@ -3841,6 +4177,7 @@
       <c r="B76" s="2"/>
       <c r="C76" s="2"/>
       <c r="D76" s="2"/>
+      <c r="E76" s="2"/>
       <c r="R76" s="2"/>
       <c r="S76" s="2"/>
       <c r="T76" s="2"/>
@@ -3896,39 +4233,135 @@
       <c r="V80" s="2"/>
       <c r="W80" s="2"/>
     </row>
+    <row r="81" spans="1:23">
+      <c r="A81" s="2"/>
+      <c r="B81" s="2"/>
+      <c r="C81" s="2"/>
+      <c r="D81" s="2"/>
+      <c r="R81" s="2"/>
+      <c r="S81" s="2"/>
+      <c r="T81" s="2"/>
+      <c r="U81" s="2"/>
+      <c r="V81" s="2"/>
+      <c r="W81" s="2"/>
+    </row>
+    <row r="82" spans="1:23">
+      <c r="A82" s="2"/>
+      <c r="B82" s="2"/>
+      <c r="C82" s="2"/>
+      <c r="D82" s="2"/>
+      <c r="R82" s="2"/>
+      <c r="S82" s="2"/>
+      <c r="T82" s="2"/>
+      <c r="U82" s="2"/>
+      <c r="V82" s="2"/>
+      <c r="W82" s="2"/>
+    </row>
+    <row r="83" spans="1:23">
+      <c r="A83" s="2"/>
+      <c r="B83" s="2"/>
+      <c r="C83" s="2"/>
+      <c r="D83" s="2"/>
+      <c r="R83" s="2"/>
+      <c r="S83" s="2"/>
+      <c r="T83" s="2"/>
+      <c r="U83" s="2"/>
+      <c r="V83" s="2"/>
+      <c r="W83" s="2"/>
+    </row>
+    <row r="84" spans="1:23">
+      <c r="A84" s="2"/>
+      <c r="B84" s="2"/>
+      <c r="C84" s="2"/>
+      <c r="D84" s="2"/>
+      <c r="R84" s="2"/>
+      <c r="S84" s="2"/>
+      <c r="T84" s="2"/>
+      <c r="U84" s="2"/>
+      <c r="V84" s="2"/>
+      <c r="W84" s="2"/>
+    </row>
+    <row r="85" spans="1:23">
+      <c r="A85" s="2"/>
+      <c r="B85" s="2"/>
+      <c r="C85" s="2"/>
+      <c r="D85" s="2"/>
+      <c r="R85" s="2"/>
+      <c r="S85" s="2"/>
+      <c r="T85" s="2"/>
+      <c r="U85" s="2"/>
+      <c r="V85" s="2"/>
+      <c r="W85" s="2"/>
+    </row>
+    <row r="86" spans="1:23">
+      <c r="A86" s="2"/>
+      <c r="B86" s="2"/>
+      <c r="C86" s="2"/>
+      <c r="D86" s="2"/>
+      <c r="R86" s="2"/>
+      <c r="S86" s="2"/>
+      <c r="T86" s="2"/>
+      <c r="U86" s="2"/>
+      <c r="V86" s="2"/>
+      <c r="W86" s="2"/>
+    </row>
+    <row r="87" spans="1:23">
+      <c r="A87" s="2"/>
+      <c r="B87" s="2"/>
+      <c r="C87" s="2"/>
+      <c r="D87" s="2"/>
+      <c r="R87" s="2"/>
+      <c r="S87" s="2"/>
+      <c r="T87" s="2"/>
+      <c r="U87" s="2"/>
+      <c r="V87" s="2"/>
+      <c r="W87" s="2"/>
+    </row>
+    <row r="88" spans="1:23">
+      <c r="A88" s="2"/>
+      <c r="B88" s="2"/>
+      <c r="C88" s="2"/>
+      <c r="D88" s="2"/>
+      <c r="R88" s="2"/>
+      <c r="S88" s="2"/>
+      <c r="T88" s="2"/>
+      <c r="U88" s="2"/>
+      <c r="V88" s="2"/>
+      <c r="W88" s="2"/>
+    </row>
   </sheetData>
   <dataValidations count="11">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F22 F2:F21 F23:F1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F6 F17 F18 F19 F20 F23 F27 F30 F31 F32 F2:F5 F7:F16 F21:F22 F24:F26 F28:F29 F33:F1048576">
       <formula1>"ALU_ADD,ALU_SUB,ALU_AND,ALU_OR,ALU_XOR,ALU_SLL,ALU_SRL,ALU_SLT,ALU_SLTU,ALU_COPY_A,ALU_COPY_B,ALU_SRA"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L5 L6 L9 L10 L13 L14 L15 L16 L17 L18 L19 L20 L21 L22 L23 L24 L2:L4 L7:L8 L11:L12 L25:L1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L5 L6 L7 L10 L11 L14 L15 L16 L17 L18 L19 L20 L21 L22 L23 L24 L25 L26 L27 L28 L29 L30 L31 L32 L2:L4 L8:L9 L12:L13 L33:L1048576">
       <formula1>"BR_EQ,BR_NE,BR_LTU,BR_GE,BR_GEU,BR_LT,BR_XX"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J5 J6 J7 J8 J9 J10 J11 J12 J13 J14 J15 J16 J17 J18 J19 J20 J21 J22 J23 J24 J2:J4 J25:J1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J5 J6 J7 J8 J9 J10 J11 J12 J13 J14 J15 J16 J17 J18 J19 J20 J21 J22 J23 J24 J25 J26 J27 J28 J29 J30 J31 J32 J2:J4 J33:J1048576">
       <formula1>"ST_SW,ST_SH,ST_SB,ST_XX"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H5 H6 H7 H8 H9 H10 H13 H14 H15 H16 H17 H18 H19 H20 H21 H22 H23 H24 H2:H4 H11:H12 H25:H1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H5 H6 H7 H8 H9 H10 H11 H14 H15 H16 H17 H18 H19 H20 H21 H22 H23 H24 H25 H26 H27 H28 H29 H30 H31 H32 H2:H4 H12:H13 H33:H1048576">
       <formula1>"WB_ALU,WB_MEM,WB_PC4,WB_XX"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="M4 M5 M6 M7 M8 M9 M10 M11 M12 M13 M14 M15 M16 M17 M18 M19 M20 M21 M22 M23 M24 M2:M3 M25:M1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="M4 M5 M6 M7 M8 M9 M10 M11 M12 M13 M14 M15 M16 M17 M18 M19 M20 M21 M22 M23 M24 M25 M26 M27 M28 M29 M30 M31 M32 M2:M3 M33:M1048576">
       <formula1>"INST_VALID,INST_INVALID"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K4 K5 K6 K7 K8 K9 K10 K11 K12 K13 K14 K15 K16 K17 K18 K19 K20 K21 K22 K23 K24 K2:K3 K25:K1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K4 K5 K6 K7 K8 K9 K10 K11 K12 K13 K14 K15 K16 K17 K18 K19 K20 K21 K22 K23 K24 K25 K26 K27 K28 K29 K30 K31 K32 K2:K3 K33:K1048576">
       <formula1>"MASK_XX,MASK_B,MASK_H,MASK_W,MASK_D"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I4 I5 I6 I7 I8 I9 I10 I11 I12 I13 I14 I15 I16 I17 I18 I19 I20 I21 I22 I23 I24 I2:I3 I25:I1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I4 I5 I6 I7 I8 I9 I10 I11 I12 I13 I14 I15 I16 I17 I18 I19 I20 I21 I22 I23 I24 I25 I26 I27 I28 I29 I30 I31 I32 I2:I3 I33:I1048576">
       <formula1>"LD_LB,LD_LH,LD_LW,LD_LBU,LD_LHU,LD_XX"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E4 E5 E6 E7 E8 E9 E10 E11 E12 E13 E14 E15 E16 E17 E18 E19 E20 E21 E22 E23 E24 E2:E3 E25:E1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E4 E5 E6 E7 E8 E9 E10 E11 E12 E13 E14 E15 E16 E17 E18 E19 E20 E21 E22 E23 E24 E25 E26 E27 E28 E29 E30 E31 E32 E2:E3 E33:E1048576">
       <formula1>"B_IMM,B_RS2"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G4 G5 G6 G7 G8 G9 G10 G11 G12 G13 G14 G15 G16 G17 G18 G19 G20 G21 G22 G23 G24 G2:G3 G25:G1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G4 G5 G6 G7 G8 G9 G10 G11 G12 G13 G14 G15 G16 G17 G18 G19 G20 G21 G22 G23 G24 G25 G26 G27 G28 G29 G30 G31 G32 G2:G3 G33:G1048576">
       <formula1>"IMM_I,IMM_J,IMM_U,IMM_S,IMM_B"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D4 D5 D6 D7 D8 D9 D10 D11 D12 D13 D14 D15 D16 D17 D18 D19 D20 D21 D22 D23 D24 D2:D3 D25:D1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D4 D5 D6 D7 D8 D9 D10 D11 D12 D13 D14 D15 D16 D17 D18 D19 D20 D21 D22 D23 D24 D25 D26 D27 D28 D29 D30 D31 D32 D2:D3 D33:D1048576">
       <formula1>"A_PC,A_RS1"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C4 C5 C6 C7 C8 C9 C10 C11 C12 C13 C14 C15 C16 C17 C18 C19 C20 C21 C22 C23 C24 C2:C3 C25:C1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C4 C5 C6 C7 C8 C9 C10 C11 C12 C13 C14 C15 C16 C17 C18 C19 C20 C21 C22 C23 C24 C25 C26 C27 C28 C29 C30 C31 C32 C2:C3 C33:C1048576">
       <formula1>"PC_4,PC_0,PC_ALU"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
> sim RTL ysyx_23060246 韩炳晋 Linux archlinux 6.6.60-1-lts #1 SMP PREEMPT_DYNAMIC Fri, 08 Nov 2024 16:03:02 +0000 x86_64 GNU/Linux  20:35:19 up 1 day,  2:50,  2 users,  load average: 3.46, 2.51, 1.97
</commit_message>
<xml_diff>
--- a/npc/tools/control_gen/control_table.xlsx
+++ b/npc/tools/control_gen/control_table.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="243" uniqueCount="92">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="263" uniqueCount="96">
   <si>
     <t>comment</t>
   </si>
@@ -169,6 +169,12 @@
     <t>LD_LHU</t>
   </si>
   <si>
+    <t>lh</t>
+  </si>
+  <si>
+    <t>LD_LH</t>
+  </si>
+  <si>
     <t>lb</t>
   </si>
   <si>
@@ -232,6 +238,15 @@
     <t>ALU_SRA</t>
   </si>
   <si>
+    <t>srl</t>
+  </si>
+  <si>
+    <t>B_RS2</t>
+  </si>
+  <si>
+    <t>sra</t>
+  </si>
+  <si>
     <t>slli</t>
   </si>
   <si>
@@ -245,9 +260,6 @@
   </si>
   <si>
     <t>sll</t>
-  </si>
-  <si>
-    <t>B_RS2</t>
   </si>
   <si>
     <t>add</t>
@@ -1258,7 +1270,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:AH88"/>
+  <dimension ref="A1:AH91"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
     <col min="1" max="1" width="13.1" customWidth="1"/>
@@ -2062,7 +2074,9 @@
       <c r="G16" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="H16" s="4"/>
+      <c r="H16" s="4" t="s">
+        <v>47</v>
+      </c>
       <c r="I16" s="4" t="s">
         <v>54</v>
       </c>
@@ -2101,7 +2115,7 @@
       </c>
       <c r="C17" s="2"/>
       <c r="D17" s="4" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="E17" s="4" t="s">
         <v>14</v>
@@ -2110,15 +2124,15 @@
         <v>21</v>
       </c>
       <c r="G17" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="H17" s="4"/>
+      <c r="I17" s="4" t="s">
         <v>56</v>
       </c>
-      <c r="H17" s="4"/>
-      <c r="I17" s="4"/>
       <c r="J17" s="4"/>
       <c r="K17" s="4"/>
-      <c r="L17" s="4" t="s">
-        <v>57</v>
-      </c>
+      <c r="L17" s="4"/>
       <c r="M17" s="4" t="s">
         <v>18</v>
       </c>
@@ -2147,7 +2161,7 @@
     <row r="18" spans="1:34">
       <c r="A18" s="3"/>
       <c r="B18" s="4" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C18" s="2"/>
       <c r="D18" s="4" t="s">
@@ -2160,7 +2174,7 @@
         <v>21</v>
       </c>
       <c r="G18" s="4" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="H18" s="4"/>
       <c r="I18" s="4"/>
@@ -2210,7 +2224,7 @@
         <v>21</v>
       </c>
       <c r="G19" s="4" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="H19" s="4"/>
       <c r="I19" s="4"/>
@@ -2260,7 +2274,7 @@
         <v>21</v>
       </c>
       <c r="G20" s="4" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="H20" s="4"/>
       <c r="I20" s="4"/>
@@ -2310,7 +2324,7 @@
         <v>21</v>
       </c>
       <c r="G21" s="4" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="H21" s="4"/>
       <c r="I21" s="4"/>
@@ -2360,7 +2374,7 @@
         <v>21</v>
       </c>
       <c r="G22" s="4" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="H22" s="4"/>
       <c r="I22" s="4"/>
@@ -2401,24 +2415,24 @@
       </c>
       <c r="C23" s="2"/>
       <c r="D23" s="4" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="E23" s="4" t="s">
         <v>14</v>
       </c>
       <c r="F23" s="4" t="s">
-        <v>69</v>
+        <v>21</v>
       </c>
       <c r="G23" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="H23" s="4" t="s">
-        <v>17</v>
-      </c>
+        <v>58</v>
+      </c>
+      <c r="H23" s="4"/>
       <c r="I23" s="4"/>
       <c r="J23" s="4"/>
       <c r="K23" s="4"/>
-      <c r="L23" s="4"/>
+      <c r="L23" s="4" t="s">
+        <v>69</v>
+      </c>
       <c r="M23" s="4" t="s">
         <v>18</v>
       </c>
@@ -2554,14 +2568,12 @@
         <v>23</v>
       </c>
       <c r="E26" s="4" t="s">
-        <v>14</v>
+        <v>75</v>
       </c>
       <c r="F26" s="4" t="s">
-        <v>75</v>
-      </c>
-      <c r="G26" s="4" t="s">
-        <v>24</v>
-      </c>
+        <v>71</v>
+      </c>
+      <c r="G26" s="4"/>
       <c r="H26" s="4" t="s">
         <v>17</v>
       </c>
@@ -2604,7 +2616,7 @@
         <v>23</v>
       </c>
       <c r="E27" s="4" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="F27" s="4" t="s">
         <v>73</v>
@@ -2645,19 +2657,21 @@
     <row r="28" spans="1:34">
       <c r="A28" s="3"/>
       <c r="B28" s="4" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C28" s="2"/>
       <c r="D28" s="4" t="s">
         <v>23</v>
       </c>
       <c r="E28" s="4" t="s">
-        <v>77</v>
+        <v>14</v>
       </c>
       <c r="F28" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="G28" s="4"/>
+        <v>78</v>
+      </c>
+      <c r="G28" s="4" t="s">
+        <v>24</v>
+      </c>
       <c r="H28" s="4" t="s">
         <v>17</v>
       </c>
@@ -2700,12 +2714,14 @@
         <v>23</v>
       </c>
       <c r="E29" s="4" t="s">
-        <v>77</v>
+        <v>14</v>
       </c>
       <c r="F29" s="4" t="s">
         <v>80</v>
       </c>
-      <c r="G29" s="4"/>
+      <c r="G29" s="4" t="s">
+        <v>24</v>
+      </c>
       <c r="H29" s="4" t="s">
         <v>17</v>
       </c>
@@ -2748,10 +2764,10 @@
         <v>23</v>
       </c>
       <c r="E30" s="4" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="F30" s="4" t="s">
-        <v>30</v>
+        <v>78</v>
       </c>
       <c r="G30" s="4"/>
       <c r="H30" s="4" t="s">
@@ -2796,10 +2812,10 @@
         <v>23</v>
       </c>
       <c r="E31" s="4" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="F31" s="4" t="s">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="G31" s="4"/>
       <c r="H31" s="4" t="s">
@@ -2844,10 +2860,10 @@
         <v>23</v>
       </c>
       <c r="E32" s="4" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="F32" s="4" t="s">
-        <v>28</v>
+        <v>84</v>
       </c>
       <c r="G32" s="4"/>
       <c r="H32" s="4" t="s">
@@ -2882,49 +2898,42 @@
       <c r="AG32" s="3"/>
       <c r="AH32" s="3"/>
     </row>
-    <row r="33" spans="2:34">
-      <c r="B33" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="C33" s="2" t="s">
+    <row r="33" spans="1:34">
+      <c r="A33" s="3"/>
+      <c r="B33" s="4" t="s">
         <v>85</v>
       </c>
-      <c r="D33" s="2" t="s">
+      <c r="C33" s="2"/>
+      <c r="D33" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="E33" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="F33" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="G33" s="2" t="s">
-        <v>24</v>
-      </c>
+      <c r="E33" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="F33" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="G33" s="4"/>
       <c r="H33" s="4" t="s">
-        <v>86</v>
-      </c>
-      <c r="I33" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="J33" s="4" t="s">
-        <v>88</v>
-      </c>
-      <c r="K33" s="2" t="s">
-        <v>89</v>
-      </c>
-      <c r="L33" s="2" t="s">
-        <v>90</v>
-      </c>
-      <c r="M33" s="2" t="s">
-        <v>91</v>
-      </c>
-      <c r="N33" s="2"/>
-      <c r="O33" s="2"/>
-      <c r="P33" s="2"/>
-      <c r="Q33" s="2"/>
-      <c r="R33" s="2"/>
-      <c r="S33" s="2"/>
+        <v>17</v>
+      </c>
+      <c r="I33" s="4"/>
+      <c r="J33" s="4"/>
+      <c r="K33" s="4"/>
+      <c r="L33" s="4"/>
+      <c r="M33" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="N33" s="4"/>
+      <c r="O33" s="4"/>
+      <c r="P33" s="4"/>
+      <c r="Q33" s="4"/>
+      <c r="R33" s="4"/>
+      <c r="S33" s="4"/>
+      <c r="T33" s="3"/>
+      <c r="U33" s="3"/>
+      <c r="V33" s="3"/>
+      <c r="W33" s="3"/>
       <c r="X33" s="3"/>
       <c r="Y33" s="3"/>
       <c r="Z33" s="3"/>
@@ -2939,18 +2948,30 @@
     </row>
     <row r="34" spans="1:34">
       <c r="A34" s="3"/>
-      <c r="B34" s="4"/>
-      <c r="C34" s="4"/>
-      <c r="D34" s="4"/>
-      <c r="E34" s="4"/>
-      <c r="F34" s="4"/>
+      <c r="B34" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="C34" s="2"/>
+      <c r="D34" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="E34" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="F34" s="4" t="s">
+        <v>26</v>
+      </c>
       <c r="G34" s="4"/>
-      <c r="H34" s="4"/>
+      <c r="H34" s="4" t="s">
+        <v>17</v>
+      </c>
       <c r="I34" s="4"/>
       <c r="J34" s="4"/>
       <c r="K34" s="4"/>
       <c r="L34" s="4"/>
-      <c r="M34" s="4"/>
+      <c r="M34" s="4" t="s">
+        <v>18</v>
+      </c>
       <c r="N34" s="4"/>
       <c r="O34" s="4"/>
       <c r="P34" s="4"/>
@@ -2973,20 +2994,32 @@
       <c r="AG34" s="3"/>
       <c r="AH34" s="3"/>
     </row>
-    <row r="35" s="1" customFormat="1" spans="1:34">
+    <row r="35" spans="1:34">
       <c r="A35" s="3"/>
-      <c r="B35" s="4"/>
-      <c r="C35" s="4"/>
-      <c r="D35" s="4"/>
-      <c r="E35" s="4"/>
-      <c r="F35" s="4"/>
+      <c r="B35" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="C35" s="2"/>
+      <c r="D35" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="E35" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="F35" s="4" t="s">
+        <v>28</v>
+      </c>
       <c r="G35" s="4"/>
-      <c r="H35" s="4"/>
+      <c r="H35" s="4" t="s">
+        <v>17</v>
+      </c>
       <c r="I35" s="4"/>
       <c r="J35" s="4"/>
       <c r="K35" s="4"/>
       <c r="L35" s="4"/>
-      <c r="M35" s="4"/>
+      <c r="M35" s="4" t="s">
+        <v>18</v>
+      </c>
       <c r="N35" s="4"/>
       <c r="O35" s="4"/>
       <c r="P35" s="4"/>
@@ -3009,30 +3042,49 @@
       <c r="AG35" s="3"/>
       <c r="AH35" s="3"/>
     </row>
-    <row r="36" s="1" customFormat="1" spans="1:34">
-      <c r="A36" s="3"/>
-      <c r="B36" s="4"/>
-      <c r="C36" s="4"/>
-      <c r="D36" s="4"/>
-      <c r="E36" s="4"/>
-      <c r="F36" s="4"/>
-      <c r="G36" s="4"/>
-      <c r="H36" s="4"/>
-      <c r="I36" s="4"/>
-      <c r="J36" s="4"/>
-      <c r="K36" s="4"/>
-      <c r="L36" s="4"/>
-      <c r="M36" s="4"/>
-      <c r="N36" s="4"/>
-      <c r="O36" s="4"/>
-      <c r="P36" s="4"/>
-      <c r="Q36" s="4"/>
-      <c r="R36" s="4"/>
-      <c r="S36" s="4"/>
-      <c r="T36" s="3"/>
-      <c r="U36" s="3"/>
-      <c r="V36" s="3"/>
-      <c r="W36" s="3"/>
+    <row r="36" spans="2:34">
+      <c r="B36" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="C36" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="D36" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="E36" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="F36" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="G36" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="H36" s="4" t="s">
+        <v>90</v>
+      </c>
+      <c r="I36" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="J36" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="K36" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="L36" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="M36" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="N36" s="2"/>
+      <c r="O36" s="2"/>
+      <c r="P36" s="2"/>
+      <c r="Q36" s="2"/>
+      <c r="R36" s="2"/>
+      <c r="S36" s="2"/>
       <c r="X36" s="3"/>
       <c r="Y36" s="3"/>
       <c r="Z36" s="3"/>
@@ -3081,7 +3133,7 @@
       <c r="AG37" s="3"/>
       <c r="AH37" s="3"/>
     </row>
-    <row r="38" spans="1:34">
+    <row r="38" s="1" customFormat="1" spans="1:34">
       <c r="A38" s="3"/>
       <c r="B38" s="4"/>
       <c r="C38" s="4"/>
@@ -3117,7 +3169,7 @@
       <c r="AG38" s="3"/>
       <c r="AH38" s="3"/>
     </row>
-    <row r="39" spans="1:34">
+    <row r="39" s="1" customFormat="1" spans="1:34">
       <c r="A39" s="3"/>
       <c r="B39" s="4"/>
       <c r="C39" s="4"/>
@@ -3590,7 +3642,7 @@
       <c r="B52" s="4"/>
       <c r="C52" s="4"/>
       <c r="D52" s="4"/>
-      <c r="E52" s="5"/>
+      <c r="E52" s="4"/>
       <c r="F52" s="4"/>
       <c r="G52" s="4"/>
       <c r="H52" s="4"/>
@@ -3626,7 +3678,7 @@
       <c r="B53" s="4"/>
       <c r="C53" s="4"/>
       <c r="D53" s="4"/>
-      <c r="E53" s="5"/>
+      <c r="E53" s="4"/>
       <c r="F53" s="4"/>
       <c r="G53" s="4"/>
       <c r="H53" s="4"/>
@@ -3662,7 +3714,7 @@
       <c r="B54" s="4"/>
       <c r="C54" s="4"/>
       <c r="D54" s="4"/>
-      <c r="E54" s="5"/>
+      <c r="E54" s="4"/>
       <c r="F54" s="4"/>
       <c r="G54" s="4"/>
       <c r="H54" s="4"/>
@@ -3698,7 +3750,7 @@
       <c r="B55" s="4"/>
       <c r="C55" s="4"/>
       <c r="D55" s="4"/>
-      <c r="E55" s="4"/>
+      <c r="E55" s="5"/>
       <c r="F55" s="4"/>
       <c r="G55" s="4"/>
       <c r="H55" s="4"/>
@@ -3734,7 +3786,7 @@
       <c r="B56" s="4"/>
       <c r="C56" s="4"/>
       <c r="D56" s="4"/>
-      <c r="E56" s="4"/>
+      <c r="E56" s="5"/>
       <c r="F56" s="4"/>
       <c r="G56" s="4"/>
       <c r="H56" s="4"/>
@@ -3770,7 +3822,7 @@
       <c r="B57" s="4"/>
       <c r="C57" s="4"/>
       <c r="D57" s="4"/>
-      <c r="E57" s="4"/>
+      <c r="E57" s="5"/>
       <c r="F57" s="4"/>
       <c r="G57" s="4"/>
       <c r="H57" s="4"/>
@@ -3842,7 +3894,7 @@
       <c r="B59" s="4"/>
       <c r="C59" s="4"/>
       <c r="D59" s="4"/>
-      <c r="E59" s="5"/>
+      <c r="E59" s="4"/>
       <c r="F59" s="4"/>
       <c r="G59" s="4"/>
       <c r="H59" s="4"/>
@@ -3950,7 +4002,7 @@
       <c r="B62" s="4"/>
       <c r="C62" s="4"/>
       <c r="D62" s="4"/>
-      <c r="E62" s="4"/>
+      <c r="E62" s="5"/>
       <c r="F62" s="4"/>
       <c r="G62" s="4"/>
       <c r="H62" s="4"/>
@@ -4161,41 +4213,113 @@
       <c r="AG67" s="3"/>
       <c r="AH67" s="3"/>
     </row>
-    <row r="75" spans="1:23">
-      <c r="A75" s="2"/>
-      <c r="B75" s="2"/>
-      <c r="C75" s="2"/>
-      <c r="D75" s="2"/>
-      <c r="R75" s="2"/>
-      <c r="T75" s="2"/>
-      <c r="U75" s="2"/>
-      <c r="V75" s="2"/>
-      <c r="W75" s="2"/>
-    </row>
-    <row r="76" spans="1:23">
-      <c r="A76" s="2"/>
-      <c r="B76" s="2"/>
-      <c r="C76" s="2"/>
-      <c r="D76" s="2"/>
-      <c r="E76" s="2"/>
-      <c r="R76" s="2"/>
-      <c r="S76" s="2"/>
-      <c r="T76" s="2"/>
-      <c r="U76" s="2"/>
-      <c r="V76" s="2"/>
-      <c r="W76" s="2"/>
-    </row>
-    <row r="77" spans="1:23">
-      <c r="A77" s="2"/>
-      <c r="B77" s="2"/>
-      <c r="C77" s="2"/>
-      <c r="D77" s="2"/>
-      <c r="R77" s="2"/>
-      <c r="S77" s="2"/>
-      <c r="T77" s="2"/>
-      <c r="U77" s="2"/>
-      <c r="V77" s="2"/>
-      <c r="W77" s="2"/>
+    <row r="68" spans="1:34">
+      <c r="A68" s="3"/>
+      <c r="B68" s="4"/>
+      <c r="C68" s="4"/>
+      <c r="D68" s="4"/>
+      <c r="E68" s="4"/>
+      <c r="F68" s="4"/>
+      <c r="G68" s="4"/>
+      <c r="H68" s="4"/>
+      <c r="I68" s="4"/>
+      <c r="J68" s="4"/>
+      <c r="K68" s="4"/>
+      <c r="L68" s="4"/>
+      <c r="M68" s="4"/>
+      <c r="N68" s="4"/>
+      <c r="O68" s="4"/>
+      <c r="P68" s="4"/>
+      <c r="Q68" s="4"/>
+      <c r="R68" s="4"/>
+      <c r="S68" s="4"/>
+      <c r="T68" s="3"/>
+      <c r="U68" s="3"/>
+      <c r="V68" s="3"/>
+      <c r="W68" s="3"/>
+      <c r="X68" s="3"/>
+      <c r="Y68" s="3"/>
+      <c r="Z68" s="3"/>
+      <c r="AA68" s="3"/>
+      <c r="AB68" s="3"/>
+      <c r="AC68" s="3"/>
+      <c r="AD68" s="3"/>
+      <c r="AE68" s="3"/>
+      <c r="AF68" s="3"/>
+      <c r="AG68" s="3"/>
+      <c r="AH68" s="3"/>
+    </row>
+    <row r="69" spans="1:34">
+      <c r="A69" s="3"/>
+      <c r="B69" s="4"/>
+      <c r="C69" s="4"/>
+      <c r="D69" s="4"/>
+      <c r="E69" s="4"/>
+      <c r="F69" s="4"/>
+      <c r="G69" s="4"/>
+      <c r="H69" s="4"/>
+      <c r="I69" s="4"/>
+      <c r="J69" s="4"/>
+      <c r="K69" s="4"/>
+      <c r="L69" s="4"/>
+      <c r="M69" s="4"/>
+      <c r="N69" s="4"/>
+      <c r="O69" s="4"/>
+      <c r="P69" s="4"/>
+      <c r="Q69" s="4"/>
+      <c r="R69" s="4"/>
+      <c r="S69" s="4"/>
+      <c r="T69" s="3"/>
+      <c r="U69" s="3"/>
+      <c r="V69" s="3"/>
+      <c r="W69" s="3"/>
+      <c r="X69" s="3"/>
+      <c r="Y69" s="3"/>
+      <c r="Z69" s="3"/>
+      <c r="AA69" s="3"/>
+      <c r="AB69" s="3"/>
+      <c r="AC69" s="3"/>
+      <c r="AD69" s="3"/>
+      <c r="AE69" s="3"/>
+      <c r="AF69" s="3"/>
+      <c r="AG69" s="3"/>
+      <c r="AH69" s="3"/>
+    </row>
+    <row r="70" spans="1:34">
+      <c r="A70" s="3"/>
+      <c r="B70" s="4"/>
+      <c r="C70" s="4"/>
+      <c r="D70" s="4"/>
+      <c r="E70" s="4"/>
+      <c r="F70" s="4"/>
+      <c r="G70" s="4"/>
+      <c r="H70" s="4"/>
+      <c r="I70" s="4"/>
+      <c r="J70" s="4"/>
+      <c r="K70" s="4"/>
+      <c r="L70" s="4"/>
+      <c r="M70" s="4"/>
+      <c r="N70" s="4"/>
+      <c r="O70" s="4"/>
+      <c r="P70" s="4"/>
+      <c r="Q70" s="4"/>
+      <c r="R70" s="4"/>
+      <c r="S70" s="4"/>
+      <c r="T70" s="3"/>
+      <c r="U70" s="3"/>
+      <c r="V70" s="3"/>
+      <c r="W70" s="3"/>
+      <c r="X70" s="3"/>
+      <c r="Y70" s="3"/>
+      <c r="Z70" s="3"/>
+      <c r="AA70" s="3"/>
+      <c r="AB70" s="3"/>
+      <c r="AC70" s="3"/>
+      <c r="AD70" s="3"/>
+      <c r="AE70" s="3"/>
+      <c r="AF70" s="3"/>
+      <c r="AG70" s="3"/>
+      <c r="AH70" s="3"/>
     </row>
     <row r="78" spans="1:23">
       <c r="A78" s="2"/>
@@ -4203,7 +4327,6 @@
       <c r="C78" s="2"/>
       <c r="D78" s="2"/>
       <c r="R78" s="2"/>
-      <c r="S78" s="2"/>
       <c r="T78" s="2"/>
       <c r="U78" s="2"/>
       <c r="V78" s="2"/>
@@ -4214,6 +4337,7 @@
       <c r="B79" s="2"/>
       <c r="C79" s="2"/>
       <c r="D79" s="2"/>
+      <c r="E79" s="2"/>
       <c r="R79" s="2"/>
       <c r="S79" s="2"/>
       <c r="T79" s="2"/>
@@ -4329,39 +4453,75 @@
       <c r="V88" s="2"/>
       <c r="W88" s="2"/>
     </row>
+    <row r="89" spans="1:23">
+      <c r="A89" s="2"/>
+      <c r="B89" s="2"/>
+      <c r="C89" s="2"/>
+      <c r="D89" s="2"/>
+      <c r="R89" s="2"/>
+      <c r="S89" s="2"/>
+      <c r="T89" s="2"/>
+      <c r="U89" s="2"/>
+      <c r="V89" s="2"/>
+      <c r="W89" s="2"/>
+    </row>
+    <row r="90" spans="1:23">
+      <c r="A90" s="2"/>
+      <c r="B90" s="2"/>
+      <c r="C90" s="2"/>
+      <c r="D90" s="2"/>
+      <c r="R90" s="2"/>
+      <c r="S90" s="2"/>
+      <c r="T90" s="2"/>
+      <c r="U90" s="2"/>
+      <c r="V90" s="2"/>
+      <c r="W90" s="2"/>
+    </row>
+    <row r="91" spans="1:23">
+      <c r="A91" s="2"/>
+      <c r="B91" s="2"/>
+      <c r="C91" s="2"/>
+      <c r="D91" s="2"/>
+      <c r="R91" s="2"/>
+      <c r="S91" s="2"/>
+      <c r="T91" s="2"/>
+      <c r="U91" s="2"/>
+      <c r="V91" s="2"/>
+      <c r="W91" s="2"/>
+    </row>
   </sheetData>
   <dataValidations count="11">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F6 F17 F18 F19 F20 F23 F27 F30 F31 F32 F2:F5 F7:F16 F21:F22 F24:F26 F28:F29 F33:F1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F6 F15 F18 F19 F20 F21 F24 F25 F26 F27 F30 F33 F34 F35 F2:F5 F7:F14 F16:F17 F22:F23 F28:F29 F31:F32 F36:F1048576">
       <formula1>"ALU_ADD,ALU_SUB,ALU_AND,ALU_OR,ALU_XOR,ALU_SLL,ALU_SRL,ALU_SLT,ALU_SLTU,ALU_COPY_A,ALU_COPY_B,ALU_SRA"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L5 L6 L7 L10 L11 L14 L15 L16 L17 L18 L19 L20 L21 L22 L23 L24 L25 L26 L27 L28 L29 L30 L31 L32 L2:L4 L8:L9 L12:L13 L33:L1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L5 L6 L7 L10 L11 L14 L15 L16 L17 L18 L19 L20 L21 L22 L23 L24 L25 L26 L27 L28 L29 L30 L31 L32 L33 L34 L35 L2:L4 L8:L9 L12:L13 L36:L1048576">
       <formula1>"BR_EQ,BR_NE,BR_LTU,BR_GE,BR_GEU,BR_LT,BR_XX"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J5 J6 J7 J8 J9 J10 J11 J12 J13 J14 J15 J16 J17 J18 J19 J20 J21 J22 J23 J24 J25 J26 J27 J28 J29 J30 J31 J32 J2:J4 J33:J1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J5 J6 J7 J8 J9 J10 J11 J12 J13 J14 J15 J16 J17 J18 J19 J20 J21 J22 J23 J24 J25 J26 J27 J28 J29 J30 J31 J32 J33 J34 J35 J2:J4 J36:J1048576">
       <formula1>"ST_SW,ST_SH,ST_SB,ST_XX"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H5 H6 H7 H8 H9 H10 H11 H14 H15 H16 H17 H18 H19 H20 H21 H22 H23 H24 H25 H26 H27 H28 H29 H30 H31 H32 H2:H4 H12:H13 H33:H1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H5 H6 H7 H8 H9 H10 H11 H14 H15 H16 H17 H18 H19 H20 H21 H22 H23 H24 H25 H26 H27 H28 H29 H30 H31 H32 H33 H34 H35 H2:H4 H12:H13 H36:H1048576">
       <formula1>"WB_ALU,WB_MEM,WB_PC4,WB_XX"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="M4 M5 M6 M7 M8 M9 M10 M11 M12 M13 M14 M15 M16 M17 M18 M19 M20 M21 M22 M23 M24 M25 M26 M27 M28 M29 M30 M31 M32 M2:M3 M33:M1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="M4 M5 M6 M7 M8 M9 M10 M11 M12 M13 M14 M15 M16 M17 M18 M19 M20 M21 M22 M23 M24 M25 M26 M27 M28 M29 M30 M31 M32 M33 M34 M35 M2:M3 M36:M1048576">
       <formula1>"INST_VALID,INST_INVALID"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K4 K5 K6 K7 K8 K9 K10 K11 K12 K13 K14 K15 K16 K17 K18 K19 K20 K21 K22 K23 K24 K25 K26 K27 K28 K29 K30 K31 K32 K2:K3 K33:K1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K4 K5 K6 K7 K8 K9 K10 K11 K12 K13 K14 K15 K16 K17 K18 K19 K20 K21 K22 K23 K24 K25 K26 K27 K28 K29 K30 K31 K32 K33 K34 K35 K2:K3 K36:K1048576">
       <formula1>"MASK_XX,MASK_B,MASK_H,MASK_W,MASK_D"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I4 I5 I6 I7 I8 I9 I10 I11 I12 I13 I14 I15 I16 I17 I18 I19 I20 I21 I22 I23 I24 I25 I26 I27 I28 I29 I30 I31 I32 I2:I3 I33:I1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I4 I5 I6 I7 I8 I9 I10 I11 I12 I13 I14 I15 I16 I17 I18 I19 I20 I21 I22 I23 I24 I25 I26 I27 I28 I29 I30 I31 I32 I33 I34 I35 I2:I3 I36:I1048576">
       <formula1>"LD_LB,LD_LH,LD_LW,LD_LBU,LD_LHU,LD_XX"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E4 E5 E6 E7 E8 E9 E10 E11 E12 E13 E14 E15 E16 E17 E18 E19 E20 E21 E22 E23 E24 E25 E26 E27 E28 E29 E30 E31 E32 E2:E3 E33:E1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E4 E5 E6 E7 E8 E9 E10 E11 E12 E13 E14 E15 E16 E17 E18 E19 E20 E21 E22 E23 E24 E25 E26 E27 E28 E29 E30 E31 E32 E33 E34 E35 E2:E3 E36:E1048576">
       <formula1>"B_IMM,B_RS2"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G4 G5 G6 G7 G8 G9 G10 G11 G12 G13 G14 G15 G16 G17 G18 G19 G20 G21 G22 G23 G24 G25 G26 G27 G28 G29 G30 G31 G32 G2:G3 G33:G1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G4 G5 G6 G7 G8 G9 G10 G11 G12 G13 G14 G15 G16 G17 G18 G19 G20 G21 G22 G23 G24 G25 G26 G27 G28 G29 G30 G31 G32 G33 G34 G35 G2:G3 G36:G1048576">
       <formula1>"IMM_I,IMM_J,IMM_U,IMM_S,IMM_B"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D4 D5 D6 D7 D8 D9 D10 D11 D12 D13 D14 D15 D16 D17 D18 D19 D20 D21 D22 D23 D24 D25 D26 D27 D28 D29 D30 D31 D32 D2:D3 D33:D1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D4 D5 D6 D7 D8 D9 D10 D11 D12 D13 D14 D15 D16 D17 D18 D19 D20 D21 D22 D23 D24 D25 D26 D27 D28 D29 D30 D31 D32 D33 D34 D35 D2:D3 D36:D1048576">
       <formula1>"A_PC,A_RS1"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C4 C5 C6 C7 C8 C9 C10 C11 C12 C13 C14 C15 C16 C17 C18 C19 C20 C21 C22 C23 C24 C25 C26 C27 C28 C29 C30 C31 C32 C2:C3 C33:C1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C4 C5 C6 C7 C8 C9 C10 C11 C12 C13 C14 C15 C16 C17 C18 C19 C20 C21 C22 C23 C24 C25 C26 C27 C28 C29 C30 C31 C32 C33 C34 C35 C2:C3 C36:C1048576">
       <formula1>"PC_4,PC_0,PC_ALU"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
> sim RTL ysyx_23060246 韩炳晋 Linux archlinux 6.6.60-1-lts #1 SMP PREEMPT_DYNAMIC Fri, 08 Nov 2024 16:03:02 +0000 x86_64 GNU/Linux  20:37:52 up 1 day,  2:52,  2 users,  load average: 5.45, 3.76, 2.53
</commit_message>
<xml_diff>
--- a/npc/tools/control_gen/control_table.xlsx
+++ b/npc/tools/control_gen/control_table.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="263" uniqueCount="96">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="269" uniqueCount="97">
   <si>
     <t>comment</t>
   </si>
@@ -253,10 +253,13 @@
     <t>ALU_SLL</t>
   </si>
   <si>
+    <t>sltu</t>
+  </si>
+  <si>
+    <t>ALU_SLTU</t>
+  </si>
+  <si>
     <t>sltiu</t>
-  </si>
-  <si>
-    <t>ALU_SLTU</t>
   </si>
   <si>
     <t>sll</t>
@@ -1270,7 +1273,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:AH91"/>
+  <dimension ref="A1:AH92"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
     <col min="1" max="1" width="13.1" customWidth="1"/>
@@ -2714,14 +2717,12 @@
         <v>23</v>
       </c>
       <c r="E29" s="4" t="s">
-        <v>14</v>
+        <v>75</v>
       </c>
       <c r="F29" s="4" t="s">
         <v>80</v>
       </c>
-      <c r="G29" s="4" t="s">
-        <v>24</v>
-      </c>
+      <c r="G29" s="4"/>
       <c r="H29" s="4" t="s">
         <v>17</v>
       </c>
@@ -2764,12 +2765,14 @@
         <v>23</v>
       </c>
       <c r="E30" s="4" t="s">
-        <v>75</v>
+        <v>14</v>
       </c>
       <c r="F30" s="4" t="s">
-        <v>78</v>
-      </c>
-      <c r="G30" s="4"/>
+        <v>80</v>
+      </c>
+      <c r="G30" s="4" t="s">
+        <v>24</v>
+      </c>
       <c r="H30" s="4" t="s">
         <v>17</v>
       </c>
@@ -2815,7 +2818,7 @@
         <v>75</v>
       </c>
       <c r="F31" s="4" t="s">
-        <v>21</v>
+        <v>78</v>
       </c>
       <c r="G31" s="4"/>
       <c r="H31" s="4" t="s">
@@ -2863,7 +2866,7 @@
         <v>75</v>
       </c>
       <c r="F32" s="4" t="s">
-        <v>84</v>
+        <v>21</v>
       </c>
       <c r="G32" s="4"/>
       <c r="H32" s="4" t="s">
@@ -2901,7 +2904,7 @@
     <row r="33" spans="1:34">
       <c r="A33" s="3"/>
       <c r="B33" s="4" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="C33" s="2"/>
       <c r="D33" s="4" t="s">
@@ -2911,7 +2914,7 @@
         <v>75</v>
       </c>
       <c r="F33" s="4" t="s">
-        <v>30</v>
+        <v>85</v>
       </c>
       <c r="G33" s="4"/>
       <c r="H33" s="4" t="s">
@@ -2959,7 +2962,7 @@
         <v>75</v>
       </c>
       <c r="F34" s="4" t="s">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="G34" s="4"/>
       <c r="H34" s="4" t="s">
@@ -3007,7 +3010,7 @@
         <v>75</v>
       </c>
       <c r="F35" s="4" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="G35" s="4"/>
       <c r="H35" s="4" t="s">
@@ -3042,49 +3045,42 @@
       <c r="AG35" s="3"/>
       <c r="AH35" s="3"/>
     </row>
-    <row r="36" spans="2:34">
-      <c r="B36" s="2" t="s">
+    <row r="36" spans="1:34">
+      <c r="A36" s="3"/>
+      <c r="B36" s="4" t="s">
         <v>88</v>
       </c>
-      <c r="C36" s="2" t="s">
-        <v>89</v>
-      </c>
-      <c r="D36" s="2" t="s">
+      <c r="C36" s="2"/>
+      <c r="D36" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="E36" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="F36" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="G36" s="2" t="s">
-        <v>24</v>
-      </c>
+      <c r="E36" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="F36" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="G36" s="4"/>
       <c r="H36" s="4" t="s">
-        <v>90</v>
-      </c>
-      <c r="I36" s="4" t="s">
-        <v>91</v>
-      </c>
-      <c r="J36" s="4" t="s">
-        <v>92</v>
-      </c>
-      <c r="K36" s="2" t="s">
-        <v>93</v>
-      </c>
-      <c r="L36" s="2" t="s">
-        <v>94</v>
-      </c>
-      <c r="M36" s="2" t="s">
-        <v>95</v>
-      </c>
-      <c r="N36" s="2"/>
-      <c r="O36" s="2"/>
-      <c r="P36" s="2"/>
-      <c r="Q36" s="2"/>
-      <c r="R36" s="2"/>
-      <c r="S36" s="2"/>
+        <v>17</v>
+      </c>
+      <c r="I36" s="4"/>
+      <c r="J36" s="4"/>
+      <c r="K36" s="4"/>
+      <c r="L36" s="4"/>
+      <c r="M36" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="N36" s="4"/>
+      <c r="O36" s="4"/>
+      <c r="P36" s="4"/>
+      <c r="Q36" s="4"/>
+      <c r="R36" s="4"/>
+      <c r="S36" s="4"/>
+      <c r="T36" s="3"/>
+      <c r="U36" s="3"/>
+      <c r="V36" s="3"/>
+      <c r="W36" s="3"/>
       <c r="X36" s="3"/>
       <c r="Y36" s="3"/>
       <c r="Z36" s="3"/>
@@ -3097,30 +3093,49 @@
       <c r="AG36" s="3"/>
       <c r="AH36" s="3"/>
     </row>
-    <row r="37" spans="1:34">
-      <c r="A37" s="3"/>
-      <c r="B37" s="4"/>
-      <c r="C37" s="4"/>
-      <c r="D37" s="4"/>
-      <c r="E37" s="4"/>
-      <c r="F37" s="4"/>
-      <c r="G37" s="4"/>
-      <c r="H37" s="4"/>
-      <c r="I37" s="4"/>
-      <c r="J37" s="4"/>
-      <c r="K37" s="4"/>
-      <c r="L37" s="4"/>
-      <c r="M37" s="4"/>
-      <c r="N37" s="4"/>
-      <c r="O37" s="4"/>
-      <c r="P37" s="4"/>
-      <c r="Q37" s="4"/>
-      <c r="R37" s="4"/>
-      <c r="S37" s="4"/>
-      <c r="T37" s="3"/>
-      <c r="U37" s="3"/>
-      <c r="V37" s="3"/>
-      <c r="W37" s="3"/>
+    <row r="37" spans="2:34">
+      <c r="B37" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="C37" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="D37" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="E37" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="F37" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="G37" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="H37" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="I37" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="J37" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="K37" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="L37" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="M37" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="N37" s="2"/>
+      <c r="O37" s="2"/>
+      <c r="P37" s="2"/>
+      <c r="Q37" s="2"/>
+      <c r="R37" s="2"/>
+      <c r="S37" s="2"/>
       <c r="X37" s="3"/>
       <c r="Y37" s="3"/>
       <c r="Z37" s="3"/>
@@ -3133,7 +3148,7 @@
       <c r="AG37" s="3"/>
       <c r="AH37" s="3"/>
     </row>
-    <row r="38" s="1" customFormat="1" spans="1:34">
+    <row r="38" spans="1:34">
       <c r="A38" s="3"/>
       <c r="B38" s="4"/>
       <c r="C38" s="4"/>
@@ -3205,7 +3220,7 @@
       <c r="AG39" s="3"/>
       <c r="AH39" s="3"/>
     </row>
-    <row r="40" spans="1:34">
+    <row r="40" s="1" customFormat="1" spans="1:34">
       <c r="A40" s="3"/>
       <c r="B40" s="4"/>
       <c r="C40" s="4"/>
@@ -3750,7 +3765,7 @@
       <c r="B55" s="4"/>
       <c r="C55" s="4"/>
       <c r="D55" s="4"/>
-      <c r="E55" s="5"/>
+      <c r="E55" s="4"/>
       <c r="F55" s="4"/>
       <c r="G55" s="4"/>
       <c r="H55" s="4"/>
@@ -3858,7 +3873,7 @@
       <c r="B58" s="4"/>
       <c r="C58" s="4"/>
       <c r="D58" s="4"/>
-      <c r="E58" s="4"/>
+      <c r="E58" s="5"/>
       <c r="F58" s="4"/>
       <c r="G58" s="4"/>
       <c r="H58" s="4"/>
@@ -4002,7 +4017,7 @@
       <c r="B62" s="4"/>
       <c r="C62" s="4"/>
       <c r="D62" s="4"/>
-      <c r="E62" s="5"/>
+      <c r="E62" s="4"/>
       <c r="F62" s="4"/>
       <c r="G62" s="4"/>
       <c r="H62" s="4"/>
@@ -4038,7 +4053,7 @@
       <c r="B63" s="4"/>
       <c r="C63" s="4"/>
       <c r="D63" s="4"/>
-      <c r="E63" s="4"/>
+      <c r="E63" s="5"/>
       <c r="F63" s="4"/>
       <c r="G63" s="4"/>
       <c r="H63" s="4"/>
@@ -4321,25 +4336,48 @@
       <c r="AG70" s="3"/>
       <c r="AH70" s="3"/>
     </row>
-    <row r="78" spans="1:23">
-      <c r="A78" s="2"/>
-      <c r="B78" s="2"/>
-      <c r="C78" s="2"/>
-      <c r="D78" s="2"/>
-      <c r="R78" s="2"/>
-      <c r="T78" s="2"/>
-      <c r="U78" s="2"/>
-      <c r="V78" s="2"/>
-      <c r="W78" s="2"/>
+    <row r="71" spans="1:34">
+      <c r="A71" s="3"/>
+      <c r="B71" s="4"/>
+      <c r="C71" s="4"/>
+      <c r="D71" s="4"/>
+      <c r="E71" s="4"/>
+      <c r="F71" s="4"/>
+      <c r="G71" s="4"/>
+      <c r="H71" s="4"/>
+      <c r="I71" s="4"/>
+      <c r="J71" s="4"/>
+      <c r="K71" s="4"/>
+      <c r="L71" s="4"/>
+      <c r="M71" s="4"/>
+      <c r="N71" s="4"/>
+      <c r="O71" s="4"/>
+      <c r="P71" s="4"/>
+      <c r="Q71" s="4"/>
+      <c r="R71" s="4"/>
+      <c r="S71" s="4"/>
+      <c r="T71" s="3"/>
+      <c r="U71" s="3"/>
+      <c r="V71" s="3"/>
+      <c r="W71" s="3"/>
+      <c r="X71" s="3"/>
+      <c r="Y71" s="3"/>
+      <c r="Z71" s="3"/>
+      <c r="AA71" s="3"/>
+      <c r="AB71" s="3"/>
+      <c r="AC71" s="3"/>
+      <c r="AD71" s="3"/>
+      <c r="AE71" s="3"/>
+      <c r="AF71" s="3"/>
+      <c r="AG71" s="3"/>
+      <c r="AH71" s="3"/>
     </row>
     <row r="79" spans="1:23">
       <c r="A79" s="2"/>
       <c r="B79" s="2"/>
       <c r="C79" s="2"/>
       <c r="D79" s="2"/>
-      <c r="E79" s="2"/>
       <c r="R79" s="2"/>
-      <c r="S79" s="2"/>
       <c r="T79" s="2"/>
       <c r="U79" s="2"/>
       <c r="V79" s="2"/>
@@ -4350,6 +4388,7 @@
       <c r="B80" s="2"/>
       <c r="C80" s="2"/>
       <c r="D80" s="2"/>
+      <c r="E80" s="2"/>
       <c r="R80" s="2"/>
       <c r="S80" s="2"/>
       <c r="T80" s="2"/>
@@ -4489,39 +4528,51 @@
       <c r="V91" s="2"/>
       <c r="W91" s="2"/>
     </row>
+    <row r="92" spans="1:23">
+      <c r="A92" s="2"/>
+      <c r="B92" s="2"/>
+      <c r="C92" s="2"/>
+      <c r="D92" s="2"/>
+      <c r="R92" s="2"/>
+      <c r="S92" s="2"/>
+      <c r="T92" s="2"/>
+      <c r="U92" s="2"/>
+      <c r="V92" s="2"/>
+      <c r="W92" s="2"/>
+    </row>
   </sheetData>
   <dataValidations count="11">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F6 F15 F18 F19 F20 F21 F24 F25 F26 F27 F30 F33 F34 F35 F2:F5 F7:F14 F16:F17 F22:F23 F28:F29 F31:F32 F36:F1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F6 F15 F18 F19 F20 F21 F24 F25 F26 F27 F28 F29 F30 F31 F34 F35 F36 F2:F5 F7:F14 F16:F17 F22:F23 F32:F33 F37:F1048576">
       <formula1>"ALU_ADD,ALU_SUB,ALU_AND,ALU_OR,ALU_XOR,ALU_SLL,ALU_SRL,ALU_SLT,ALU_SLTU,ALU_COPY_A,ALU_COPY_B,ALU_SRA"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L5 L6 L7 L10 L11 L14 L15 L16 L17 L18 L19 L20 L21 L22 L23 L24 L25 L26 L27 L28 L29 L30 L31 L32 L33 L34 L35 L2:L4 L8:L9 L12:L13 L36:L1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L5 L6 L7 L10 L11 L14 L15 L16 L17 L18 L19 L20 L21 L22 L23 L24 L25 L26 L27 L28 L29 L30 L31 L32 L33 L34 L35 L36 L2:L4 L8:L9 L12:L13 L37:L1048576">
       <formula1>"BR_EQ,BR_NE,BR_LTU,BR_GE,BR_GEU,BR_LT,BR_XX"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J5 J6 J7 J8 J9 J10 J11 J12 J13 J14 J15 J16 J17 J18 J19 J20 J21 J22 J23 J24 J25 J26 J27 J28 J29 J30 J31 J32 J33 J34 J35 J2:J4 J36:J1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J5 J6 J7 J8 J9 J10 J11 J12 J13 J14 J15 J16 J17 J18 J19 J20 J21 J22 J23 J24 J25 J26 J27 J28 J29 J30 J31 J32 J33 J34 J35 J36 J2:J4 J37:J1048576">
       <formula1>"ST_SW,ST_SH,ST_SB,ST_XX"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H5 H6 H7 H8 H9 H10 H11 H14 H15 H16 H17 H18 H19 H20 H21 H22 H23 H24 H25 H26 H27 H28 H29 H30 H31 H32 H33 H34 H35 H2:H4 H12:H13 H36:H1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H5 H6 H7 H8 H9 H10 H11 H14 H15 H16 H17 H18 H19 H20 H21 H22 H23 H24 H25 H26 H27 H28 H29 H30 H31 H32 H33 H34 H35 H36 H2:H4 H12:H13 H37:H1048576">
       <formula1>"WB_ALU,WB_MEM,WB_PC4,WB_XX"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="M4 M5 M6 M7 M8 M9 M10 M11 M12 M13 M14 M15 M16 M17 M18 M19 M20 M21 M22 M23 M24 M25 M26 M27 M28 M29 M30 M31 M32 M33 M34 M35 M2:M3 M36:M1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="M4 M5 M6 M7 M8 M9 M10 M11 M12 M13 M14 M15 M16 M17 M18 M19 M20 M21 M22 M23 M24 M25 M26 M27 M28 M29 M30 M31 M32 M33 M34 M35 M36 M2:M3 M37:M1048576">
       <formula1>"INST_VALID,INST_INVALID"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K4 K5 K6 K7 K8 K9 K10 K11 K12 K13 K14 K15 K16 K17 K18 K19 K20 K21 K22 K23 K24 K25 K26 K27 K28 K29 K30 K31 K32 K33 K34 K35 K2:K3 K36:K1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K4 K5 K6 K7 K8 K9 K10 K11 K12 K13 K14 K15 K16 K17 K18 K19 K20 K21 K22 K23 K24 K25 K26 K27 K28 K29 K30 K31 K32 K33 K34 K35 K36 K2:K3 K37:K1048576">
       <formula1>"MASK_XX,MASK_B,MASK_H,MASK_W,MASK_D"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I4 I5 I6 I7 I8 I9 I10 I11 I12 I13 I14 I15 I16 I17 I18 I19 I20 I21 I22 I23 I24 I25 I26 I27 I28 I29 I30 I31 I32 I33 I34 I35 I2:I3 I36:I1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I4 I5 I6 I7 I8 I9 I10 I11 I12 I13 I14 I15 I16 I17 I18 I19 I20 I21 I22 I23 I24 I25 I26 I27 I28 I29 I30 I31 I32 I33 I34 I35 I36 I2:I3 I37:I1048576">
       <formula1>"LD_LB,LD_LH,LD_LW,LD_LBU,LD_LHU,LD_XX"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E4 E5 E6 E7 E8 E9 E10 E11 E12 E13 E14 E15 E16 E17 E18 E19 E20 E21 E22 E23 E24 E25 E26 E27 E28 E29 E30 E31 E32 E33 E34 E35 E2:E3 E36:E1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E4 E5 E6 E7 E8 E9 E10 E11 E12 E13 E14 E15 E16 E17 E18 E19 E20 E21 E22 E23 E24 E25 E26 E27 E28 E29 E30 E31 E32 E33 E34 E35 E36 E2:E3 E37:E1048576">
       <formula1>"B_IMM,B_RS2"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G4 G5 G6 G7 G8 G9 G10 G11 G12 G13 G14 G15 G16 G17 G18 G19 G20 G21 G22 G23 G24 G25 G26 G27 G28 G29 G30 G31 G32 G33 G34 G35 G2:G3 G36:G1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G4 G5 G6 G7 G8 G9 G10 G11 G12 G13 G14 G15 G16 G17 G18 G19 G20 G21 G22 G23 G24 G25 G26 G27 G28 G29 G30 G31 G32 G33 G34 G35 G36 G2:G3 G37:G1048576">
       <formula1>"IMM_I,IMM_J,IMM_U,IMM_S,IMM_B"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D4 D5 D6 D7 D8 D9 D10 D11 D12 D13 D14 D15 D16 D17 D18 D19 D20 D21 D22 D23 D24 D25 D26 D27 D28 D29 D30 D31 D32 D33 D34 D35 D2:D3 D36:D1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D4 D5 D6 D7 D8 D9 D10 D11 D12 D13 D14 D15 D16 D17 D18 D19 D20 D21 D22 D23 D24 D25 D26 D27 D28 D29 D30 D31 D32 D33 D34 D35 D36 D2:D3 D37:D1048576">
       <formula1>"A_PC,A_RS1"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C4 C5 C6 C7 C8 C9 C10 C11 C12 C13 C14 C15 C16 C17 C18 C19 C20 C21 C22 C23 C24 C25 C26 C27 C28 C29 C30 C31 C32 C33 C34 C35 C2:C3 C36:C1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C4 C5 C6 C7 C8 C9 C10 C11 C12 C13 C14 C15 C16 C17 C18 C19 C20 C21 C22 C23 C24 C25 C26 C27 C28 C29 C30 C31 C32 C33 C34 C35 C36 C2:C3 C37:C1048576">
       <formula1>"PC_4,PC_0,PC_ALU"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
> sim RTL ysyx_23060246 韩炳晋 Linux archlinux 6.6.60-1-lts #1 SMP PREEMPT_DYNAMIC Fri, 08 Nov 2024 16:03:02 +0000 x86_64 GNU/Linux  20:46:04 up 1 day,  3:01,  2 users,  load average: 4.30, 4.85, 3.71
</commit_message>
<xml_diff>
--- a/npc/tools/control_gen/control_table.xlsx
+++ b/npc/tools/control_gen/control_table.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="269" uniqueCount="97">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="270" uniqueCount="97">
   <si>
     <t>comment</t>
   </si>
@@ -2129,7 +2129,9 @@
       <c r="G17" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="H17" s="4"/>
+      <c r="H17" s="4" t="s">
+        <v>47</v>
+      </c>
       <c r="I17" s="4" t="s">
         <v>56</v>
       </c>

</xml_diff>

<commit_message>
> sim RTL ysyx_23060246 韩炳晋 Linux archlinux 6.6.60-1-lts #1 SMP PREEMPT_DYNAMIC Fri, 08 Nov 2024 16:03:02 +0000 x86_64 GNU/Linux  17:56:52 up  2:16,  2 users,  load average: 2.27, 2.06, 1.88
</commit_message>
<xml_diff>
--- a/npc/tools/control_gen/control_table.xlsx
+++ b/npc/tools/control_gen/control_table.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="27795" windowHeight="12075"/>
+    <workbookView windowWidth="27795" windowHeight="12735"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="270" uniqueCount="97">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="296" uniqueCount="109">
   <si>
     <t>comment</t>
   </si>
@@ -52,6 +52,9 @@
     <t>br_sel</t>
   </si>
   <si>
+    <t>csr_sel</t>
+  </si>
+  <si>
     <t>inst_valid</t>
   </si>
   <si>
@@ -283,12 +286,42 @@
     <t>or</t>
   </si>
   <si>
+    <t>csrrw</t>
+  </si>
+  <si>
+    <t>PC_0</t>
+  </si>
+  <si>
+    <t>WB_CSR</t>
+  </si>
+  <si>
+    <t>CSR_W</t>
+  </si>
+  <si>
+    <t>csrrs</t>
+  </si>
+  <si>
+    <t>CSR_S</t>
+  </si>
+  <si>
+    <t>ecall</t>
+  </si>
+  <si>
+    <t>PC_4</t>
+  </si>
+  <si>
+    <t>CSR_P</t>
+  </si>
+  <si>
+    <t>mret</t>
+  </si>
+  <si>
+    <t>PC_EPC</t>
+  </si>
+  <si>
     <t>default</t>
   </si>
   <si>
-    <t>PC_4</t>
-  </si>
-  <si>
     <t>WB_XX</t>
   </si>
   <si>
@@ -302,6 +335,9 @@
   </si>
   <si>
     <t>BR_XX</t>
+  </si>
+  <si>
+    <t>CSR_XX</t>
   </si>
   <si>
     <t>INST_INVALID</t>
@@ -312,10 +348,10 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="4">
+    <numFmt numFmtId="41" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
+    <numFmt numFmtId="42" formatCode="_ &quot;￥&quot;* #,##0_ ;_ &quot;￥&quot;* \-#,##0_ ;_ &quot;￥&quot;* &quot;-&quot;_ ;_ @_ "/>
     <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="42" formatCode="_ &quot;￥&quot;* #,##0_ ;_ &quot;￥&quot;* \-#,##0_ ;_ &quot;￥&quot;* &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="41" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
   <fonts count="22">
     <font>
@@ -346,7 +382,22 @@
     </font>
     <font>
       <sz val="11"/>
+      <color theme="1"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
       <color theme="0"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color rgb="FF7F7F7F"/>
       <name val="宋体"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -354,6 +405,22 @@
     <font>
       <b/>
       <sz val="11"/>
+      <color theme="3"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="13"/>
       <color theme="3"/>
       <name val="宋体"/>
       <charset val="134"/>
@@ -369,22 +436,7 @@
     </font>
     <font>
       <sz val="11"/>
-      <color theme="1"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="18"/>
-      <color theme="3"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
+      <color rgb="FF9C6500"/>
       <name val="宋体"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -392,6 +444,22 @@
     <font>
       <sz val="11"/>
       <color rgb="FF9C0006"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF3F3F3F"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
       <name val="宋体"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -412,48 +480,8 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
       <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="11"/>
-      <color rgb="FF7F7F7F"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="13"/>
-      <color theme="3"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FF3F3F3F"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C6500"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
+      <color rgb="FFFF0000"/>
       <name val="宋体"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -475,6 +503,14 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <b/>
+      <sz val="18"/>
+      <color theme="3"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <sz val="11"/>
       <color rgb="FF3F3F76"/>
       <name val="宋体"/>
@@ -491,7 +527,49 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -503,7 +581,103 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFA5A5A5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor theme="9" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.399975585192419"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -515,103 +689,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor theme="6" tint="0.799981688894314"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFA5A5A5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
+        <fgColor theme="6" tint="0.599993896298105"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -623,55 +707,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="FFFFCC99"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.399975585192419"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -704,6 +740,30 @@
     </border>
     <border>
       <left style="thin">
+        <color rgb="FF7F7F7F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF7F7F7F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF7F7F7F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF7F7F7F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
         <color rgb="FFB2B2B2"/>
       </left>
       <right style="thin">
@@ -718,11 +778,17 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4"/>
+      <left style="thin">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF3F3F3F"/>
       </bottom>
       <diagonal/>
     </border>
@@ -742,36 +808,6 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF7F7F7F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF7F7F7F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF7F7F7F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF7F7F7F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
       <left/>
       <right/>
       <top style="thin">
@@ -787,145 +823,145 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="30" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="5" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="32" borderId="3" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="3" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="17" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="5" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="21" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="19" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="21" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="17" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
@@ -1273,7 +1309,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:AH92"/>
+  <dimension ref="A1:AI96"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
     <col min="1" max="1" width="13.1" customWidth="1"/>
@@ -1285,19 +1321,19 @@
     <col min="7" max="7" width="10.9416666666667" customWidth="1"/>
     <col min="8" max="10" width="11.9833333333333" customWidth="1"/>
     <col min="11" max="11" width="15.075" customWidth="1"/>
-    <col min="12" max="13" width="12.1083333333333" customWidth="1"/>
-    <col min="14" max="14" width="10.8583333333333" customWidth="1"/>
-    <col min="16" max="16" width="14.2166666666667" customWidth="1"/>
-    <col min="17" max="17" width="11.8083333333333" customWidth="1"/>
-    <col min="18" max="18" width="10.6" customWidth="1"/>
-    <col min="19" max="19" width="9.70833333333333" customWidth="1"/>
-    <col min="20" max="20" width="11.1666666666667" customWidth="1"/>
-    <col min="21" max="21" width="11.4083333333333" customWidth="1"/>
-    <col min="22" max="22" width="12.0583333333333" customWidth="1"/>
-    <col min="23" max="23" width="15.575" customWidth="1"/>
+    <col min="12" max="14" width="12.1083333333333" customWidth="1"/>
+    <col min="15" max="15" width="10.8583333333333" customWidth="1"/>
+    <col min="17" max="17" width="14.2166666666667" customWidth="1"/>
+    <col min="18" max="18" width="11.8083333333333" customWidth="1"/>
+    <col min="19" max="19" width="10.6" customWidth="1"/>
+    <col min="20" max="20" width="9.70833333333333" customWidth="1"/>
+    <col min="21" max="21" width="11.1666666666667" customWidth="1"/>
+    <col min="22" max="22" width="11.4083333333333" customWidth="1"/>
+    <col min="23" max="23" width="12.0583333333333" customWidth="1"/>
+    <col min="24" max="24" width="15.575" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="15" customHeight="1" spans="1:22">
+    <row r="1" ht="15" customHeight="1" spans="1:23">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1337,47 +1373,50 @@
       <c r="M1" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="2"/>
+      <c r="N1" s="2" t="s">
+        <v>13</v>
+      </c>
       <c r="O1" s="2"/>
       <c r="P1" s="2"/>
       <c r="Q1" s="2"/>
       <c r="R1" s="2"/>
       <c r="S1" s="2"/>
-      <c r="V1" s="6"/>
-    </row>
-    <row r="2" spans="1:34">
+      <c r="T1" s="2"/>
+      <c r="W1" s="6"/>
+    </row>
+    <row r="2" spans="1:35">
       <c r="A2" s="3"/>
       <c r="B2" s="4" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="4"/>
       <c r="E2" s="4" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F2" s="4" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="G2" s="4" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="H2" s="4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="I2" s="4"/>
       <c r="J2" s="4"/>
       <c r="K2" s="4"/>
       <c r="L2" s="4"/>
-      <c r="M2" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="N2" s="4"/>
+      <c r="M2" s="4"/>
+      <c r="N2" s="4" t="s">
+        <v>19</v>
+      </c>
       <c r="O2" s="4"/>
       <c r="P2" s="4"/>
       <c r="Q2" s="4"/>
       <c r="R2" s="4"/>
       <c r="S2" s="4"/>
-      <c r="T2" s="3"/>
+      <c r="T2" s="4"/>
       <c r="U2" s="3"/>
       <c r="V2" s="3"/>
       <c r="W2" s="3"/>
@@ -1392,42 +1431,43 @@
       <c r="AF2" s="3"/>
       <c r="AG2" s="3"/>
       <c r="AH2" s="3"/>
-    </row>
-    <row r="3" spans="1:34">
+      <c r="AI2" s="3"/>
+    </row>
+    <row r="3" spans="1:35">
       <c r="A3" s="3"/>
       <c r="B3" s="4" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C3" s="2"/>
       <c r="D3" s="4" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="G3" s="4" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="H3" s="4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="I3" s="4"/>
       <c r="J3" s="4"/>
       <c r="K3" s="4"/>
       <c r="L3" s="4"/>
-      <c r="M3" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="N3" s="4"/>
+      <c r="M3" s="4"/>
+      <c r="N3" s="4" t="s">
+        <v>19</v>
+      </c>
       <c r="O3" s="4"/>
       <c r="P3" s="4"/>
       <c r="Q3" s="4"/>
       <c r="R3" s="4"/>
       <c r="S3" s="4"/>
-      <c r="T3" s="3"/>
+      <c r="T3" s="4"/>
       <c r="U3" s="3"/>
       <c r="V3" s="3"/>
       <c r="W3" s="3"/>
@@ -1442,42 +1482,43 @@
       <c r="AF3" s="3"/>
       <c r="AG3" s="3"/>
       <c r="AH3" s="3"/>
-    </row>
-    <row r="4" spans="1:34">
+      <c r="AI3" s="3"/>
+    </row>
+    <row r="4" spans="1:35">
       <c r="A4" s="3"/>
       <c r="B4" s="4" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C4" s="2"/>
       <c r="D4" s="4" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="H4" s="4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="I4" s="4"/>
       <c r="J4" s="4"/>
       <c r="K4" s="4"/>
       <c r="L4" s="4"/>
-      <c r="M4" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="N4" s="4"/>
+      <c r="M4" s="4"/>
+      <c r="N4" s="4" t="s">
+        <v>19</v>
+      </c>
       <c r="O4" s="4"/>
       <c r="P4" s="4"/>
       <c r="Q4" s="4"/>
       <c r="R4" s="4"/>
       <c r="S4" s="4"/>
-      <c r="T4" s="3"/>
+      <c r="T4" s="4"/>
       <c r="U4" s="3"/>
       <c r="V4" s="3"/>
       <c r="W4" s="3"/>
@@ -1492,42 +1533,43 @@
       <c r="AF4" s="3"/>
       <c r="AG4" s="3"/>
       <c r="AH4" s="3"/>
-    </row>
-    <row r="5" spans="1:34">
+      <c r="AI4" s="3"/>
+    </row>
+    <row r="5" spans="1:35">
       <c r="A5" s="3"/>
       <c r="B5" s="4" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C5" s="2"/>
       <c r="D5" s="4" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="H5" s="4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="I5" s="4"/>
       <c r="J5" s="4"/>
       <c r="K5" s="4"/>
       <c r="L5" s="4"/>
-      <c r="M5" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="N5" s="4"/>
+      <c r="M5" s="4"/>
+      <c r="N5" s="4" t="s">
+        <v>19</v>
+      </c>
       <c r="O5" s="4"/>
       <c r="P5" s="4"/>
       <c r="Q5" s="4"/>
       <c r="R5" s="4"/>
       <c r="S5" s="4"/>
-      <c r="T5" s="3"/>
+      <c r="T5" s="4"/>
       <c r="U5" s="3"/>
       <c r="V5" s="3"/>
       <c r="W5" s="3"/>
@@ -1542,42 +1584,43 @@
       <c r="AF5" s="3"/>
       <c r="AG5" s="3"/>
       <c r="AH5" s="3"/>
-    </row>
-    <row r="6" spans="1:34">
+      <c r="AI5" s="3"/>
+    </row>
+    <row r="6" spans="1:35">
       <c r="A6" s="3"/>
       <c r="B6" s="4" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C6" s="2"/>
       <c r="D6" s="4" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="G6" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="H6" s="4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="I6" s="4"/>
       <c r="J6" s="4"/>
       <c r="K6" s="4"/>
       <c r="L6" s="4"/>
-      <c r="M6" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="N6" s="4"/>
+      <c r="M6" s="4"/>
+      <c r="N6" s="4" t="s">
+        <v>19</v>
+      </c>
       <c r="O6" s="4"/>
       <c r="P6" s="4"/>
       <c r="Q6" s="4"/>
       <c r="R6" s="4"/>
       <c r="S6" s="4"/>
-      <c r="T6" s="3"/>
+      <c r="T6" s="4"/>
       <c r="U6" s="3"/>
       <c r="V6" s="3"/>
       <c r="W6" s="3"/>
@@ -1592,42 +1635,43 @@
       <c r="AF6" s="3"/>
       <c r="AG6" s="3"/>
       <c r="AH6" s="3"/>
-    </row>
-    <row r="7" spans="1:34">
+      <c r="AI6" s="3"/>
+    </row>
+    <row r="7" spans="1:35">
       <c r="A7" s="3"/>
       <c r="B7" s="4" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C7" s="2"/>
       <c r="D7" s="4" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="G7" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="H7" s="4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="I7" s="4"/>
       <c r="J7" s="4"/>
       <c r="K7" s="4"/>
       <c r="L7" s="4"/>
-      <c r="M7" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="N7" s="4"/>
+      <c r="M7" s="4"/>
+      <c r="N7" s="4" t="s">
+        <v>19</v>
+      </c>
       <c r="O7" s="4"/>
       <c r="P7" s="4"/>
       <c r="Q7" s="4"/>
       <c r="R7" s="4"/>
       <c r="S7" s="4"/>
-      <c r="T7" s="3"/>
+      <c r="T7" s="4"/>
       <c r="U7" s="3"/>
       <c r="V7" s="3"/>
       <c r="W7" s="3"/>
@@ -1642,44 +1686,45 @@
       <c r="AF7" s="3"/>
       <c r="AG7" s="3"/>
       <c r="AH7" s="3"/>
-    </row>
-    <row r="8" spans="1:34">
+      <c r="AI7" s="3"/>
+    </row>
+    <row r="8" spans="1:35">
       <c r="A8" s="3"/>
       <c r="B8" s="4" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F8" s="4" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="G8" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="H8" s="4" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="I8" s="4"/>
       <c r="J8" s="4"/>
       <c r="K8" s="4"/>
       <c r="L8" s="4"/>
-      <c r="M8" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="N8" s="4"/>
+      <c r="M8" s="4"/>
+      <c r="N8" s="4" t="s">
+        <v>19</v>
+      </c>
       <c r="O8" s="4"/>
       <c r="P8" s="4"/>
       <c r="Q8" s="4"/>
       <c r="R8" s="4"/>
       <c r="S8" s="4"/>
-      <c r="T8" s="3"/>
+      <c r="T8" s="4"/>
       <c r="U8" s="3"/>
       <c r="V8" s="3"/>
       <c r="W8" s="3"/>
@@ -1694,44 +1739,45 @@
       <c r="AF8" s="3"/>
       <c r="AG8" s="3"/>
       <c r="AH8" s="3"/>
-    </row>
-    <row r="9" spans="1:34">
+      <c r="AI8" s="3"/>
+    </row>
+    <row r="9" spans="1:35">
       <c r="A9" s="3"/>
       <c r="B9" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="D9" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="E9" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="F9" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="G9" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="H9" s="4" t="s">
         <v>34</v>
-      </c>
-      <c r="C9" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="D9" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="E9" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="F9" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="G9" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="H9" s="4" t="s">
-        <v>33</v>
       </c>
       <c r="I9" s="4"/>
       <c r="J9" s="4"/>
       <c r="K9" s="4"/>
       <c r="L9" s="4"/>
-      <c r="M9" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="N9" s="4"/>
+      <c r="M9" s="4"/>
+      <c r="N9" s="4" t="s">
+        <v>19</v>
+      </c>
       <c r="O9" s="4"/>
       <c r="P9" s="4"/>
       <c r="Q9" s="4"/>
       <c r="R9" s="4"/>
       <c r="S9" s="4"/>
-      <c r="T9" s="3"/>
+      <c r="T9" s="4"/>
       <c r="U9" s="3"/>
       <c r="V9" s="3"/>
       <c r="W9" s="3"/>
@@ -1746,44 +1792,45 @@
       <c r="AF9" s="3"/>
       <c r="AG9" s="3"/>
       <c r="AH9" s="3"/>
-    </row>
-    <row r="10" spans="1:34">
+      <c r="AI9" s="3"/>
+    </row>
+    <row r="10" spans="1:35">
       <c r="A10" s="3"/>
       <c r="B10" s="4" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C10" s="2"/>
       <c r="D10" s="4" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F10" s="4" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="G10" s="4" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="H10" s="4"/>
       <c r="I10" s="4"/>
       <c r="J10" s="4" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="K10" s="4" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="L10" s="4"/>
-      <c r="M10" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="N10" s="4"/>
+      <c r="M10" s="4"/>
+      <c r="N10" s="4" t="s">
+        <v>19</v>
+      </c>
       <c r="O10" s="4"/>
       <c r="P10" s="4"/>
       <c r="Q10" s="4"/>
       <c r="R10" s="4"/>
       <c r="S10" s="4"/>
-      <c r="T10" s="3"/>
+      <c r="T10" s="4"/>
       <c r="U10" s="3"/>
       <c r="V10" s="3"/>
       <c r="W10" s="3"/>
@@ -1798,44 +1845,45 @@
       <c r="AF10" s="3"/>
       <c r="AG10" s="3"/>
       <c r="AH10" s="3"/>
-    </row>
-    <row r="11" spans="1:34">
+      <c r="AI10" s="3"/>
+    </row>
+    <row r="11" spans="1:35">
       <c r="A11" s="3"/>
       <c r="B11" s="4" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C11" s="2"/>
       <c r="D11" s="4" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E11" s="4" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F11" s="4" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="G11" s="4" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="H11" s="4"/>
       <c r="I11" s="4"/>
       <c r="J11" s="4" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="K11" s="4" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="L11" s="4"/>
-      <c r="M11" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="N11" s="4"/>
+      <c r="M11" s="4"/>
+      <c r="N11" s="4" t="s">
+        <v>19</v>
+      </c>
       <c r="O11" s="4"/>
       <c r="P11" s="4"/>
       <c r="Q11" s="4"/>
       <c r="R11" s="4"/>
       <c r="S11" s="4"/>
-      <c r="T11" s="3"/>
+      <c r="T11" s="4"/>
       <c r="U11" s="3"/>
       <c r="V11" s="3"/>
       <c r="W11" s="3"/>
@@ -1850,44 +1898,45 @@
       <c r="AF11" s="3"/>
       <c r="AG11" s="3"/>
       <c r="AH11" s="3"/>
-    </row>
-    <row r="12" spans="1:34">
+      <c r="AI11" s="3"/>
+    </row>
+    <row r="12" spans="1:35">
       <c r="A12" s="3"/>
       <c r="B12" s="4" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C12" s="2"/>
       <c r="D12" s="4" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E12" s="4" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F12" s="4" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="G12" s="4" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="H12" s="4"/>
       <c r="I12" s="4"/>
       <c r="J12" s="4" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="K12" s="4" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="L12" s="4"/>
-      <c r="M12" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="N12" s="4"/>
+      <c r="M12" s="4"/>
+      <c r="N12" s="4" t="s">
+        <v>19</v>
+      </c>
       <c r="O12" s="4"/>
       <c r="P12" s="4"/>
       <c r="Q12" s="4"/>
       <c r="R12" s="4"/>
       <c r="S12" s="4"/>
-      <c r="T12" s="3"/>
+      <c r="T12" s="4"/>
       <c r="U12" s="3"/>
       <c r="V12" s="3"/>
       <c r="W12" s="3"/>
@@ -1902,44 +1951,45 @@
       <c r="AF12" s="3"/>
       <c r="AG12" s="3"/>
       <c r="AH12" s="3"/>
-    </row>
-    <row r="13" spans="1:34">
+      <c r="AI12" s="3"/>
+    </row>
+    <row r="13" spans="1:35">
       <c r="A13" s="3"/>
       <c r="B13" s="4" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C13" s="2"/>
       <c r="D13" s="4" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E13" s="4" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F13" s="4" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="G13" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="H13" s="4" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="I13" s="4" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="J13" s="4"/>
       <c r="K13" s="4"/>
       <c r="L13" s="4"/>
-      <c r="M13" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="N13" s="4"/>
+      <c r="M13" s="4"/>
+      <c r="N13" s="4" t="s">
+        <v>19</v>
+      </c>
       <c r="O13" s="4"/>
       <c r="P13" s="4"/>
       <c r="Q13" s="4"/>
       <c r="R13" s="4"/>
       <c r="S13" s="4"/>
-      <c r="T13" s="3"/>
+      <c r="T13" s="4"/>
       <c r="U13" s="3"/>
       <c r="V13" s="3"/>
       <c r="W13" s="3"/>
@@ -1954,44 +2004,45 @@
       <c r="AF13" s="3"/>
       <c r="AG13" s="3"/>
       <c r="AH13" s="3"/>
-    </row>
-    <row r="14" spans="1:34">
+      <c r="AI13" s="3"/>
+    </row>
+    <row r="14" spans="1:35">
       <c r="A14" s="3"/>
       <c r="B14" s="4" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C14" s="2"/>
       <c r="D14" s="4" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E14" s="4" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F14" s="4" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="G14" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="H14" s="4" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="I14" s="4" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="J14" s="4"/>
       <c r="K14" s="4"/>
       <c r="L14" s="4"/>
-      <c r="M14" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="N14" s="4"/>
+      <c r="M14" s="4"/>
+      <c r="N14" s="4" t="s">
+        <v>19</v>
+      </c>
       <c r="O14" s="4"/>
       <c r="P14" s="4"/>
       <c r="Q14" s="4"/>
       <c r="R14" s="4"/>
       <c r="S14" s="4"/>
-      <c r="T14" s="3"/>
+      <c r="T14" s="4"/>
       <c r="U14" s="3"/>
       <c r="V14" s="3"/>
       <c r="W14" s="3"/>
@@ -2006,44 +2057,45 @@
       <c r="AF14" s="3"/>
       <c r="AG14" s="3"/>
       <c r="AH14" s="3"/>
-    </row>
-    <row r="15" spans="1:34">
+      <c r="AI14" s="3"/>
+    </row>
+    <row r="15" spans="1:35">
       <c r="A15" s="3"/>
       <c r="B15" s="4" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C15" s="2"/>
       <c r="D15" s="4" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E15" s="4" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F15" s="4" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="G15" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="H15" s="4" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="I15" s="4" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="J15" s="4"/>
       <c r="K15" s="4"/>
       <c r="L15" s="4"/>
-      <c r="M15" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="N15" s="4"/>
+      <c r="M15" s="4"/>
+      <c r="N15" s="4" t="s">
+        <v>19</v>
+      </c>
       <c r="O15" s="4"/>
       <c r="P15" s="4"/>
       <c r="Q15" s="4"/>
       <c r="R15" s="4"/>
       <c r="S15" s="4"/>
-      <c r="T15" s="3"/>
+      <c r="T15" s="4"/>
       <c r="U15" s="3"/>
       <c r="V15" s="3"/>
       <c r="W15" s="3"/>
@@ -2058,44 +2110,45 @@
       <c r="AF15" s="3"/>
       <c r="AG15" s="3"/>
       <c r="AH15" s="3"/>
-    </row>
-    <row r="16" spans="1:34">
+      <c r="AI15" s="3"/>
+    </row>
+    <row r="16" spans="1:35">
       <c r="A16" s="3"/>
       <c r="B16" s="4" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C16" s="2"/>
       <c r="D16" s="4" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E16" s="4" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F16" s="4" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="G16" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="H16" s="4" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="I16" s="4" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="J16" s="4"/>
       <c r="K16" s="4"/>
       <c r="L16" s="4"/>
-      <c r="M16" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="N16" s="4"/>
+      <c r="M16" s="4"/>
+      <c r="N16" s="4" t="s">
+        <v>19</v>
+      </c>
       <c r="O16" s="4"/>
       <c r="P16" s="4"/>
       <c r="Q16" s="4"/>
       <c r="R16" s="4"/>
       <c r="S16" s="4"/>
-      <c r="T16" s="3"/>
+      <c r="T16" s="4"/>
       <c r="U16" s="3"/>
       <c r="V16" s="3"/>
       <c r="W16" s="3"/>
@@ -2110,44 +2163,45 @@
       <c r="AF16" s="3"/>
       <c r="AG16" s="3"/>
       <c r="AH16" s="3"/>
-    </row>
-    <row r="17" spans="1:34">
+      <c r="AI16" s="3"/>
+    </row>
+    <row r="17" spans="1:35">
       <c r="A17" s="3"/>
       <c r="B17" s="4" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C17" s="2"/>
       <c r="D17" s="4" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E17" s="4" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F17" s="4" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="G17" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="H17" s="4" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="I17" s="4" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="J17" s="4"/>
       <c r="K17" s="4"/>
       <c r="L17" s="4"/>
-      <c r="M17" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="N17" s="4"/>
+      <c r="M17" s="4"/>
+      <c r="N17" s="4" t="s">
+        <v>19</v>
+      </c>
       <c r="O17" s="4"/>
       <c r="P17" s="4"/>
       <c r="Q17" s="4"/>
       <c r="R17" s="4"/>
       <c r="S17" s="4"/>
-      <c r="T17" s="3"/>
+      <c r="T17" s="4"/>
       <c r="U17" s="3"/>
       <c r="V17" s="3"/>
       <c r="W17" s="3"/>
@@ -2162,42 +2216,43 @@
       <c r="AF17" s="3"/>
       <c r="AG17" s="3"/>
       <c r="AH17" s="3"/>
-    </row>
-    <row r="18" spans="1:34">
+      <c r="AI17" s="3"/>
+    </row>
+    <row r="18" spans="1:35">
       <c r="A18" s="3"/>
       <c r="B18" s="4" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C18" s="2"/>
       <c r="D18" s="4" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E18" s="4" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F18" s="4" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="G18" s="4" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="H18" s="4"/>
       <c r="I18" s="4"/>
       <c r="J18" s="4"/>
       <c r="K18" s="4"/>
       <c r="L18" s="4" t="s">
-        <v>59</v>
-      </c>
-      <c r="M18" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="N18" s="4"/>
+        <v>60</v>
+      </c>
+      <c r="M18" s="4"/>
+      <c r="N18" s="4" t="s">
+        <v>19</v>
+      </c>
       <c r="O18" s="4"/>
       <c r="P18" s="4"/>
       <c r="Q18" s="4"/>
       <c r="R18" s="4"/>
       <c r="S18" s="4"/>
-      <c r="T18" s="3"/>
+      <c r="T18" s="4"/>
       <c r="U18" s="3"/>
       <c r="V18" s="3"/>
       <c r="W18" s="3"/>
@@ -2212,42 +2267,43 @@
       <c r="AF18" s="3"/>
       <c r="AG18" s="3"/>
       <c r="AH18" s="3"/>
-    </row>
-    <row r="19" spans="1:34">
+      <c r="AI18" s="3"/>
+    </row>
+    <row r="19" spans="1:35">
       <c r="A19" s="3"/>
       <c r="B19" s="4" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C19" s="2"/>
       <c r="D19" s="4" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E19" s="4" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F19" s="4" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="G19" s="4" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="H19" s="4"/>
       <c r="I19" s="4"/>
       <c r="J19" s="4"/>
       <c r="K19" s="4"/>
       <c r="L19" s="4" t="s">
-        <v>61</v>
-      </c>
-      <c r="M19" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="N19" s="4"/>
+        <v>62</v>
+      </c>
+      <c r="M19" s="4"/>
+      <c r="N19" s="4" t="s">
+        <v>19</v>
+      </c>
       <c r="O19" s="4"/>
       <c r="P19" s="4"/>
       <c r="Q19" s="4"/>
       <c r="R19" s="4"/>
       <c r="S19" s="4"/>
-      <c r="T19" s="3"/>
+      <c r="T19" s="4"/>
       <c r="U19" s="3"/>
       <c r="V19" s="3"/>
       <c r="W19" s="3"/>
@@ -2262,42 +2318,43 @@
       <c r="AF19" s="3"/>
       <c r="AG19" s="3"/>
       <c r="AH19" s="3"/>
-    </row>
-    <row r="20" spans="1:34">
+      <c r="AI19" s="3"/>
+    </row>
+    <row r="20" spans="1:35">
       <c r="A20" s="3"/>
       <c r="B20" s="4" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C20" s="2"/>
       <c r="D20" s="4" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E20" s="4" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F20" s="4" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="G20" s="4" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="H20" s="4"/>
       <c r="I20" s="4"/>
       <c r="J20" s="4"/>
       <c r="K20" s="4"/>
       <c r="L20" s="4" t="s">
-        <v>63</v>
-      </c>
-      <c r="M20" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="N20" s="4"/>
+        <v>64</v>
+      </c>
+      <c r="M20" s="4"/>
+      <c r="N20" s="4" t="s">
+        <v>19</v>
+      </c>
       <c r="O20" s="4"/>
       <c r="P20" s="4"/>
       <c r="Q20" s="4"/>
       <c r="R20" s="4"/>
       <c r="S20" s="4"/>
-      <c r="T20" s="3"/>
+      <c r="T20" s="4"/>
       <c r="U20" s="3"/>
       <c r="V20" s="3"/>
       <c r="W20" s="3"/>
@@ -2312,42 +2369,43 @@
       <c r="AF20" s="3"/>
       <c r="AG20" s="3"/>
       <c r="AH20" s="3"/>
-    </row>
-    <row r="21" spans="1:34">
+      <c r="AI20" s="3"/>
+    </row>
+    <row r="21" spans="1:35">
       <c r="A21" s="3"/>
       <c r="B21" s="4" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C21" s="2"/>
       <c r="D21" s="4" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E21" s="4" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F21" s="4" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="G21" s="4" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="H21" s="4"/>
       <c r="I21" s="4"/>
       <c r="J21" s="4"/>
       <c r="K21" s="4"/>
       <c r="L21" s="4" t="s">
-        <v>65</v>
-      </c>
-      <c r="M21" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="N21" s="4"/>
+        <v>66</v>
+      </c>
+      <c r="M21" s="4"/>
+      <c r="N21" s="4" t="s">
+        <v>19</v>
+      </c>
       <c r="O21" s="4"/>
       <c r="P21" s="4"/>
       <c r="Q21" s="4"/>
       <c r="R21" s="4"/>
       <c r="S21" s="4"/>
-      <c r="T21" s="3"/>
+      <c r="T21" s="4"/>
       <c r="U21" s="3"/>
       <c r="V21" s="3"/>
       <c r="W21" s="3"/>
@@ -2362,42 +2420,43 @@
       <c r="AF21" s="3"/>
       <c r="AG21" s="3"/>
       <c r="AH21" s="3"/>
-    </row>
-    <row r="22" spans="1:34">
+      <c r="AI21" s="3"/>
+    </row>
+    <row r="22" spans="1:35">
       <c r="A22" s="3"/>
       <c r="B22" s="4" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C22" s="2"/>
       <c r="D22" s="4" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E22" s="4" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F22" s="4" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="G22" s="4" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="H22" s="4"/>
       <c r="I22" s="4"/>
       <c r="J22" s="4"/>
       <c r="K22" s="4"/>
       <c r="L22" s="4" t="s">
-        <v>67</v>
-      </c>
-      <c r="M22" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="N22" s="4"/>
+        <v>68</v>
+      </c>
+      <c r="M22" s="4"/>
+      <c r="N22" s="4" t="s">
+        <v>19</v>
+      </c>
       <c r="O22" s="4"/>
       <c r="P22" s="4"/>
       <c r="Q22" s="4"/>
       <c r="R22" s="4"/>
       <c r="S22" s="4"/>
-      <c r="T22" s="3"/>
+      <c r="T22" s="4"/>
       <c r="U22" s="3"/>
       <c r="V22" s="3"/>
       <c r="W22" s="3"/>
@@ -2412,42 +2471,43 @@
       <c r="AF22" s="3"/>
       <c r="AG22" s="3"/>
       <c r="AH22" s="3"/>
-    </row>
-    <row r="23" spans="1:34">
+      <c r="AI22" s="3"/>
+    </row>
+    <row r="23" spans="1:35">
       <c r="A23" s="3"/>
       <c r="B23" s="4" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="C23" s="2"/>
       <c r="D23" s="4" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E23" s="4" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F23" s="4" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="G23" s="4" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="H23" s="4"/>
       <c r="I23" s="4"/>
       <c r="J23" s="4"/>
       <c r="K23" s="4"/>
       <c r="L23" s="4" t="s">
-        <v>69</v>
-      </c>
-      <c r="M23" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="N23" s="4"/>
+        <v>70</v>
+      </c>
+      <c r="M23" s="4"/>
+      <c r="N23" s="4" t="s">
+        <v>19</v>
+      </c>
       <c r="O23" s="4"/>
       <c r="P23" s="4"/>
       <c r="Q23" s="4"/>
       <c r="R23" s="4"/>
       <c r="S23" s="4"/>
-      <c r="T23" s="3"/>
+      <c r="T23" s="4"/>
       <c r="U23" s="3"/>
       <c r="V23" s="3"/>
       <c r="W23" s="3"/>
@@ -2462,42 +2522,43 @@
       <c r="AF23" s="3"/>
       <c r="AG23" s="3"/>
       <c r="AH23" s="3"/>
-    </row>
-    <row r="24" spans="1:34">
+      <c r="AI23" s="3"/>
+    </row>
+    <row r="24" spans="1:35">
       <c r="A24" s="3"/>
       <c r="B24" s="4" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C24" s="2"/>
       <c r="D24" s="4" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E24" s="4" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F24" s="4" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="G24" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="H24" s="4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="I24" s="4"/>
       <c r="J24" s="4"/>
       <c r="K24" s="4"/>
       <c r="L24" s="4"/>
-      <c r="M24" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="N24" s="4"/>
+      <c r="M24" s="4"/>
+      <c r="N24" s="4" t="s">
+        <v>19</v>
+      </c>
       <c r="O24" s="4"/>
       <c r="P24" s="4"/>
       <c r="Q24" s="4"/>
       <c r="R24" s="4"/>
       <c r="S24" s="4"/>
-      <c r="T24" s="3"/>
+      <c r="T24" s="4"/>
       <c r="U24" s="3"/>
       <c r="V24" s="3"/>
       <c r="W24" s="3"/>
@@ -2512,42 +2573,43 @@
       <c r="AF24" s="3"/>
       <c r="AG24" s="3"/>
       <c r="AH24" s="3"/>
-    </row>
-    <row r="25" spans="1:34">
+      <c r="AI24" s="3"/>
+    </row>
+    <row r="25" spans="1:35">
       <c r="A25" s="3"/>
       <c r="B25" s="4" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C25" s="2"/>
       <c r="D25" s="4" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E25" s="4" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F25" s="4" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="G25" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="H25" s="4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="I25" s="4"/>
       <c r="J25" s="4"/>
       <c r="K25" s="4"/>
       <c r="L25" s="4"/>
-      <c r="M25" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="N25" s="4"/>
+      <c r="M25" s="4"/>
+      <c r="N25" s="4" t="s">
+        <v>19</v>
+      </c>
       <c r="O25" s="4"/>
       <c r="P25" s="4"/>
       <c r="Q25" s="4"/>
       <c r="R25" s="4"/>
       <c r="S25" s="4"/>
-      <c r="T25" s="3"/>
+      <c r="T25" s="4"/>
       <c r="U25" s="3"/>
       <c r="V25" s="3"/>
       <c r="W25" s="3"/>
@@ -2562,40 +2624,41 @@
       <c r="AF25" s="3"/>
       <c r="AG25" s="3"/>
       <c r="AH25" s="3"/>
-    </row>
-    <row r="26" spans="1:34">
+      <c r="AI25" s="3"/>
+    </row>
+    <row r="26" spans="1:35">
       <c r="A26" s="3"/>
       <c r="B26" s="4" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="C26" s="2"/>
       <c r="D26" s="4" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E26" s="4" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F26" s="4" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="G26" s="4"/>
       <c r="H26" s="4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="I26" s="4"/>
       <c r="J26" s="4"/>
       <c r="K26" s="4"/>
       <c r="L26" s="4"/>
-      <c r="M26" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="N26" s="4"/>
+      <c r="M26" s="4"/>
+      <c r="N26" s="4" t="s">
+        <v>19</v>
+      </c>
       <c r="O26" s="4"/>
       <c r="P26" s="4"/>
       <c r="Q26" s="4"/>
       <c r="R26" s="4"/>
       <c r="S26" s="4"/>
-      <c r="T26" s="3"/>
+      <c r="T26" s="4"/>
       <c r="U26" s="3"/>
       <c r="V26" s="3"/>
       <c r="W26" s="3"/>
@@ -2610,40 +2673,41 @@
       <c r="AF26" s="3"/>
       <c r="AG26" s="3"/>
       <c r="AH26" s="3"/>
-    </row>
-    <row r="27" spans="1:34">
+      <c r="AI26" s="3"/>
+    </row>
+    <row r="27" spans="1:35">
       <c r="A27" s="3"/>
       <c r="B27" s="4" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C27" s="2"/>
       <c r="D27" s="4" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E27" s="4" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F27" s="4" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="G27" s="4"/>
       <c r="H27" s="4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="I27" s="4"/>
       <c r="J27" s="4"/>
       <c r="K27" s="4"/>
       <c r="L27" s="4"/>
-      <c r="M27" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="N27" s="4"/>
+      <c r="M27" s="4"/>
+      <c r="N27" s="4" t="s">
+        <v>19</v>
+      </c>
       <c r="O27" s="4"/>
       <c r="P27" s="4"/>
       <c r="Q27" s="4"/>
       <c r="R27" s="4"/>
       <c r="S27" s="4"/>
-      <c r="T27" s="3"/>
+      <c r="T27" s="4"/>
       <c r="U27" s="3"/>
       <c r="V27" s="3"/>
       <c r="W27" s="3"/>
@@ -2658,42 +2722,43 @@
       <c r="AF27" s="3"/>
       <c r="AG27" s="3"/>
       <c r="AH27" s="3"/>
-    </row>
-    <row r="28" spans="1:34">
+      <c r="AI27" s="3"/>
+    </row>
+    <row r="28" spans="1:35">
       <c r="A28" s="3"/>
       <c r="B28" s="4" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="C28" s="2"/>
       <c r="D28" s="4" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E28" s="4" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F28" s="4" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="G28" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="H28" s="4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="I28" s="4"/>
       <c r="J28" s="4"/>
       <c r="K28" s="4"/>
       <c r="L28" s="4"/>
-      <c r="M28" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="N28" s="4"/>
+      <c r="M28" s="4"/>
+      <c r="N28" s="4" t="s">
+        <v>19</v>
+      </c>
       <c r="O28" s="4"/>
       <c r="P28" s="4"/>
       <c r="Q28" s="4"/>
       <c r="R28" s="4"/>
       <c r="S28" s="4"/>
-      <c r="T28" s="3"/>
+      <c r="T28" s="4"/>
       <c r="U28" s="3"/>
       <c r="V28" s="3"/>
       <c r="W28" s="3"/>
@@ -2708,40 +2773,41 @@
       <c r="AF28" s="3"/>
       <c r="AG28" s="3"/>
       <c r="AH28" s="3"/>
-    </row>
-    <row r="29" spans="1:34">
+      <c r="AI28" s="3"/>
+    </row>
+    <row r="29" spans="1:35">
       <c r="A29" s="3"/>
       <c r="B29" s="4" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C29" s="2"/>
       <c r="D29" s="4" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E29" s="4" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F29" s="4" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="G29" s="4"/>
       <c r="H29" s="4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="I29" s="4"/>
       <c r="J29" s="4"/>
       <c r="K29" s="4"/>
       <c r="L29" s="4"/>
-      <c r="M29" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="N29" s="4"/>
+      <c r="M29" s="4"/>
+      <c r="N29" s="4" t="s">
+        <v>19</v>
+      </c>
       <c r="O29" s="4"/>
       <c r="P29" s="4"/>
       <c r="Q29" s="4"/>
       <c r="R29" s="4"/>
       <c r="S29" s="4"/>
-      <c r="T29" s="3"/>
+      <c r="T29" s="4"/>
       <c r="U29" s="3"/>
       <c r="V29" s="3"/>
       <c r="W29" s="3"/>
@@ -2756,42 +2822,43 @@
       <c r="AF29" s="3"/>
       <c r="AG29" s="3"/>
       <c r="AH29" s="3"/>
-    </row>
-    <row r="30" spans="1:34">
+      <c r="AI29" s="3"/>
+    </row>
+    <row r="30" spans="1:35">
       <c r="A30" s="3"/>
       <c r="B30" s="4" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="C30" s="2"/>
       <c r="D30" s="4" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E30" s="4" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F30" s="4" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="G30" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="H30" s="4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="I30" s="4"/>
       <c r="J30" s="4"/>
       <c r="K30" s="4"/>
       <c r="L30" s="4"/>
-      <c r="M30" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="N30" s="4"/>
+      <c r="M30" s="4"/>
+      <c r="N30" s="4" t="s">
+        <v>19</v>
+      </c>
       <c r="O30" s="4"/>
       <c r="P30" s="4"/>
       <c r="Q30" s="4"/>
       <c r="R30" s="4"/>
       <c r="S30" s="4"/>
-      <c r="T30" s="3"/>
+      <c r="T30" s="4"/>
       <c r="U30" s="3"/>
       <c r="V30" s="3"/>
       <c r="W30" s="3"/>
@@ -2806,40 +2873,41 @@
       <c r="AF30" s="3"/>
       <c r="AG30" s="3"/>
       <c r="AH30" s="3"/>
-    </row>
-    <row r="31" spans="1:34">
+      <c r="AI30" s="3"/>
+    </row>
+    <row r="31" spans="1:35">
       <c r="A31" s="3"/>
       <c r="B31" s="4" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="C31" s="2"/>
       <c r="D31" s="4" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E31" s="4" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F31" s="4" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="G31" s="4"/>
       <c r="H31" s="4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="I31" s="4"/>
       <c r="J31" s="4"/>
       <c r="K31" s="4"/>
       <c r="L31" s="4"/>
-      <c r="M31" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="N31" s="4"/>
+      <c r="M31" s="4"/>
+      <c r="N31" s="4" t="s">
+        <v>19</v>
+      </c>
       <c r="O31" s="4"/>
       <c r="P31" s="4"/>
       <c r="Q31" s="4"/>
       <c r="R31" s="4"/>
       <c r="S31" s="4"/>
-      <c r="T31" s="3"/>
+      <c r="T31" s="4"/>
       <c r="U31" s="3"/>
       <c r="V31" s="3"/>
       <c r="W31" s="3"/>
@@ -2854,40 +2922,41 @@
       <c r="AF31" s="3"/>
       <c r="AG31" s="3"/>
       <c r="AH31" s="3"/>
-    </row>
-    <row r="32" spans="1:34">
+      <c r="AI31" s="3"/>
+    </row>
+    <row r="32" spans="1:35">
       <c r="A32" s="3"/>
       <c r="B32" s="4" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="C32" s="2"/>
       <c r="D32" s="4" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E32" s="4" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F32" s="4" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="G32" s="4"/>
       <c r="H32" s="4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="I32" s="4"/>
       <c r="J32" s="4"/>
       <c r="K32" s="4"/>
       <c r="L32" s="4"/>
-      <c r="M32" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="N32" s="4"/>
+      <c r="M32" s="4"/>
+      <c r="N32" s="4" t="s">
+        <v>19</v>
+      </c>
       <c r="O32" s="4"/>
       <c r="P32" s="4"/>
       <c r="Q32" s="4"/>
       <c r="R32" s="4"/>
       <c r="S32" s="4"/>
-      <c r="T32" s="3"/>
+      <c r="T32" s="4"/>
       <c r="U32" s="3"/>
       <c r="V32" s="3"/>
       <c r="W32" s="3"/>
@@ -2902,40 +2971,41 @@
       <c r="AF32" s="3"/>
       <c r="AG32" s="3"/>
       <c r="AH32" s="3"/>
-    </row>
-    <row r="33" spans="1:34">
+      <c r="AI32" s="3"/>
+    </row>
+    <row r="33" spans="1:35">
       <c r="A33" s="3"/>
       <c r="B33" s="4" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="C33" s="2"/>
       <c r="D33" s="4" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E33" s="4" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F33" s="4" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="G33" s="4"/>
       <c r="H33" s="4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="I33" s="4"/>
       <c r="J33" s="4"/>
       <c r="K33" s="4"/>
       <c r="L33" s="4"/>
-      <c r="M33" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="N33" s="4"/>
+      <c r="M33" s="4"/>
+      <c r="N33" s="4" t="s">
+        <v>19</v>
+      </c>
       <c r="O33" s="4"/>
       <c r="P33" s="4"/>
       <c r="Q33" s="4"/>
       <c r="R33" s="4"/>
       <c r="S33" s="4"/>
-      <c r="T33" s="3"/>
+      <c r="T33" s="4"/>
       <c r="U33" s="3"/>
       <c r="V33" s="3"/>
       <c r="W33" s="3"/>
@@ -2950,40 +3020,41 @@
       <c r="AF33" s="3"/>
       <c r="AG33" s="3"/>
       <c r="AH33" s="3"/>
-    </row>
-    <row r="34" spans="1:34">
+      <c r="AI33" s="3"/>
+    </row>
+    <row r="34" spans="1:35">
       <c r="A34" s="3"/>
       <c r="B34" s="4" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="C34" s="2"/>
       <c r="D34" s="4" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E34" s="4" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F34" s="4" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="G34" s="4"/>
       <c r="H34" s="4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="I34" s="4"/>
       <c r="J34" s="4"/>
       <c r="K34" s="4"/>
       <c r="L34" s="4"/>
-      <c r="M34" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="N34" s="4"/>
+      <c r="M34" s="4"/>
+      <c r="N34" s="4" t="s">
+        <v>19</v>
+      </c>
       <c r="O34" s="4"/>
       <c r="P34" s="4"/>
       <c r="Q34" s="4"/>
       <c r="R34" s="4"/>
       <c r="S34" s="4"/>
-      <c r="T34" s="3"/>
+      <c r="T34" s="4"/>
       <c r="U34" s="3"/>
       <c r="V34" s="3"/>
       <c r="W34" s="3"/>
@@ -2998,40 +3069,41 @@
       <c r="AF34" s="3"/>
       <c r="AG34" s="3"/>
       <c r="AH34" s="3"/>
-    </row>
-    <row r="35" spans="1:34">
+      <c r="AI34" s="3"/>
+    </row>
+    <row r="35" spans="1:35">
       <c r="A35" s="3"/>
       <c r="B35" s="4" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C35" s="2"/>
       <c r="D35" s="4" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E35" s="4" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F35" s="4" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="G35" s="4"/>
       <c r="H35" s="4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="I35" s="4"/>
       <c r="J35" s="4"/>
       <c r="K35" s="4"/>
       <c r="L35" s="4"/>
-      <c r="M35" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="N35" s="4"/>
+      <c r="M35" s="4"/>
+      <c r="N35" s="4" t="s">
+        <v>19</v>
+      </c>
       <c r="O35" s="4"/>
       <c r="P35" s="4"/>
       <c r="Q35" s="4"/>
       <c r="R35" s="4"/>
       <c r="S35" s="4"/>
-      <c r="T35" s="3"/>
+      <c r="T35" s="4"/>
       <c r="U35" s="3"/>
       <c r="V35" s="3"/>
       <c r="W35" s="3"/>
@@ -3046,40 +3118,41 @@
       <c r="AF35" s="3"/>
       <c r="AG35" s="3"/>
       <c r="AH35" s="3"/>
-    </row>
-    <row r="36" spans="1:34">
+      <c r="AI35" s="3"/>
+    </row>
+    <row r="36" spans="1:35">
       <c r="A36" s="3"/>
       <c r="B36" s="4" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C36" s="2"/>
       <c r="D36" s="4" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E36" s="4" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F36" s="4" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="G36" s="4"/>
       <c r="H36" s="4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="I36" s="4"/>
       <c r="J36" s="4"/>
       <c r="K36" s="4"/>
       <c r="L36" s="4"/>
-      <c r="M36" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="N36" s="4"/>
+      <c r="M36" s="4"/>
+      <c r="N36" s="4" t="s">
+        <v>19</v>
+      </c>
       <c r="O36" s="4"/>
       <c r="P36" s="4"/>
       <c r="Q36" s="4"/>
       <c r="R36" s="4"/>
       <c r="S36" s="4"/>
-      <c r="T36" s="3"/>
+      <c r="T36" s="4"/>
       <c r="U36" s="3"/>
       <c r="V36" s="3"/>
       <c r="W36" s="3"/>
@@ -3094,50 +3167,46 @@
       <c r="AF36" s="3"/>
       <c r="AG36" s="3"/>
       <c r="AH36" s="3"/>
-    </row>
-    <row r="37" spans="2:34">
-      <c r="B37" s="2" t="s">
-        <v>89</v>
+      <c r="AI36" s="3"/>
+    </row>
+    <row r="37" spans="1:35">
+      <c r="A37" s="3"/>
+      <c r="B37" s="4" t="s">
+        <v>90</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>90</v>
-      </c>
-      <c r="D37" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="E37" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="F37" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="G37" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="D37" s="4" t="s">
         <v>24</v>
       </c>
+      <c r="E37" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="F37" s="4"/>
+      <c r="G37" s="4"/>
       <c r="H37" s="4" t="s">
-        <v>91</v>
-      </c>
-      <c r="I37" s="4" t="s">
         <v>92</v>
       </c>
-      <c r="J37" s="4" t="s">
+      <c r="I37" s="4"/>
+      <c r="J37" s="4"/>
+      <c r="K37" s="4"/>
+      <c r="L37" s="4"/>
+      <c r="M37" s="4" t="s">
         <v>93</v>
       </c>
-      <c r="K37" s="2" t="s">
-        <v>94</v>
-      </c>
-      <c r="L37" s="2" t="s">
-        <v>95</v>
-      </c>
-      <c r="M37" s="2" t="s">
-        <v>96</v>
-      </c>
-      <c r="N37" s="2"/>
-      <c r="O37" s="2"/>
-      <c r="P37" s="2"/>
-      <c r="Q37" s="2"/>
-      <c r="R37" s="2"/>
-      <c r="S37" s="2"/>
+      <c r="N37" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="O37" s="4"/>
+      <c r="P37" s="4"/>
+      <c r="Q37" s="4"/>
+      <c r="R37" s="4"/>
+      <c r="S37" s="4"/>
+      <c r="T37" s="4"/>
+      <c r="U37" s="3"/>
+      <c r="V37" s="3"/>
+      <c r="W37" s="3"/>
       <c r="X37" s="3"/>
       <c r="Y37" s="3"/>
       <c r="Z37" s="3"/>
@@ -3149,28 +3218,43 @@
       <c r="AF37" s="3"/>
       <c r="AG37" s="3"/>
       <c r="AH37" s="3"/>
-    </row>
-    <row r="38" spans="1:34">
+      <c r="AI37" s="3"/>
+    </row>
+    <row r="38" spans="1:35">
       <c r="A38" s="3"/>
-      <c r="B38" s="4"/>
-      <c r="C38" s="4"/>
-      <c r="D38" s="4"/>
-      <c r="E38" s="4"/>
+      <c r="B38" s="4" t="s">
+        <v>94</v>
+      </c>
+      <c r="C38" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="D38" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="E38" s="4" t="s">
+        <v>76</v>
+      </c>
       <c r="F38" s="4"/>
       <c r="G38" s="4"/>
-      <c r="H38" s="4"/>
+      <c r="H38" s="4" t="s">
+        <v>92</v>
+      </c>
       <c r="I38" s="4"/>
       <c r="J38" s="4"/>
       <c r="K38" s="4"/>
       <c r="L38" s="4"/>
-      <c r="M38" s="4"/>
-      <c r="N38" s="4"/>
+      <c r="M38" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="N38" s="4" t="s">
+        <v>19</v>
+      </c>
       <c r="O38" s="4"/>
       <c r="P38" s="4"/>
       <c r="Q38" s="4"/>
       <c r="R38" s="4"/>
       <c r="S38" s="4"/>
-      <c r="T38" s="3"/>
+      <c r="T38" s="4"/>
       <c r="U38" s="3"/>
       <c r="V38" s="3"/>
       <c r="W38" s="3"/>
@@ -3185,28 +3269,39 @@
       <c r="AF38" s="3"/>
       <c r="AG38" s="3"/>
       <c r="AH38" s="3"/>
-    </row>
-    <row r="39" s="1" customFormat="1" spans="1:34">
+      <c r="AI38" s="3"/>
+    </row>
+    <row r="39" spans="1:35">
       <c r="A39" s="3"/>
-      <c r="B39" s="4"/>
-      <c r="C39" s="4"/>
+      <c r="B39" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="C39" s="2" t="s">
+        <v>97</v>
+      </c>
       <c r="D39" s="4"/>
       <c r="E39" s="4"/>
       <c r="F39" s="4"/>
       <c r="G39" s="4"/>
-      <c r="H39" s="4"/>
+      <c r="H39" s="4" t="s">
+        <v>92</v>
+      </c>
       <c r="I39" s="4"/>
       <c r="J39" s="4"/>
       <c r="K39" s="4"/>
       <c r="L39" s="4"/>
-      <c r="M39" s="4"/>
-      <c r="N39" s="4"/>
+      <c r="M39" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="N39" s="4" t="s">
+        <v>19</v>
+      </c>
       <c r="O39" s="4"/>
       <c r="P39" s="4"/>
       <c r="Q39" s="4"/>
       <c r="R39" s="4"/>
       <c r="S39" s="4"/>
-      <c r="T39" s="3"/>
+      <c r="T39" s="4"/>
       <c r="U39" s="3"/>
       <c r="V39" s="3"/>
       <c r="W39" s="3"/>
@@ -3221,28 +3316,39 @@
       <c r="AF39" s="3"/>
       <c r="AG39" s="3"/>
       <c r="AH39" s="3"/>
-    </row>
-    <row r="40" s="1" customFormat="1" spans="1:34">
+      <c r="AI39" s="3"/>
+    </row>
+    <row r="40" spans="1:35">
       <c r="A40" s="3"/>
-      <c r="B40" s="4"/>
-      <c r="C40" s="4"/>
+      <c r="B40" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="C40" s="2" t="s">
+        <v>100</v>
+      </c>
       <c r="D40" s="4"/>
       <c r="E40" s="4"/>
       <c r="F40" s="4"/>
       <c r="G40" s="4"/>
-      <c r="H40" s="4"/>
+      <c r="H40" s="4" t="s">
+        <v>92</v>
+      </c>
       <c r="I40" s="4"/>
       <c r="J40" s="4"/>
       <c r="K40" s="4"/>
       <c r="L40" s="4"/>
-      <c r="M40" s="4"/>
-      <c r="N40" s="4"/>
+      <c r="M40" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="N40" s="4" t="s">
+        <v>19</v>
+      </c>
       <c r="O40" s="4"/>
       <c r="P40" s="4"/>
       <c r="Q40" s="4"/>
       <c r="R40" s="4"/>
       <c r="S40" s="4"/>
-      <c r="T40" s="3"/>
+      <c r="T40" s="4"/>
       <c r="U40" s="3"/>
       <c r="V40" s="3"/>
       <c r="W40" s="3"/>
@@ -3257,32 +3363,54 @@
       <c r="AF40" s="3"/>
       <c r="AG40" s="3"/>
       <c r="AH40" s="3"/>
-    </row>
-    <row r="41" spans="1:34">
-      <c r="A41" s="3"/>
-      <c r="B41" s="4"/>
-      <c r="C41" s="4"/>
-      <c r="D41" s="4"/>
-      <c r="E41" s="4"/>
-      <c r="F41" s="4"/>
-      <c r="G41" s="4"/>
-      <c r="H41" s="4"/>
-      <c r="I41" s="4"/>
-      <c r="J41" s="4"/>
-      <c r="K41" s="4"/>
-      <c r="L41" s="4"/>
-      <c r="M41" s="4"/>
-      <c r="N41" s="4"/>
-      <c r="O41" s="4"/>
-      <c r="P41" s="4"/>
-      <c r="Q41" s="4"/>
-      <c r="R41" s="4"/>
-      <c r="S41" s="4"/>
-      <c r="T41" s="3"/>
-      <c r="U41" s="3"/>
-      <c r="V41" s="3"/>
-      <c r="W41" s="3"/>
-      <c r="X41" s="3"/>
+      <c r="AI40" s="3"/>
+    </row>
+    <row r="41" spans="2:35">
+      <c r="B41" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="C41" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="D41" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="E41" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="F41" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="G41" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="H41" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="I41" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="J41" s="4" t="s">
+        <v>104</v>
+      </c>
+      <c r="K41" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="L41" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="M41" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="N41" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="O41" s="2"/>
+      <c r="P41" s="2"/>
+      <c r="Q41" s="2"/>
+      <c r="R41" s="2"/>
+      <c r="S41" s="2"/>
+      <c r="T41" s="2"/>
       <c r="Y41" s="3"/>
       <c r="Z41" s="3"/>
       <c r="AA41" s="3"/>
@@ -3293,8 +3421,9 @@
       <c r="AF41" s="3"/>
       <c r="AG41" s="3"/>
       <c r="AH41" s="3"/>
-    </row>
-    <row r="42" spans="1:34">
+      <c r="AI41" s="3"/>
+    </row>
+    <row r="42" spans="1:35">
       <c r="A42" s="3"/>
       <c r="B42" s="4"/>
       <c r="C42" s="4"/>
@@ -3314,7 +3443,7 @@
       <c r="Q42" s="4"/>
       <c r="R42" s="4"/>
       <c r="S42" s="4"/>
-      <c r="T42" s="3"/>
+      <c r="T42" s="4"/>
       <c r="U42" s="3"/>
       <c r="V42" s="3"/>
       <c r="W42" s="3"/>
@@ -3329,8 +3458,9 @@
       <c r="AF42" s="3"/>
       <c r="AG42" s="3"/>
       <c r="AH42" s="3"/>
-    </row>
-    <row r="43" spans="1:34">
+      <c r="AI42" s="3"/>
+    </row>
+    <row r="43" s="1" customFormat="1" spans="1:35">
       <c r="A43" s="3"/>
       <c r="B43" s="4"/>
       <c r="C43" s="4"/>
@@ -3350,7 +3480,7 @@
       <c r="Q43" s="4"/>
       <c r="R43" s="4"/>
       <c r="S43" s="4"/>
-      <c r="T43" s="3"/>
+      <c r="T43" s="4"/>
       <c r="U43" s="3"/>
       <c r="V43" s="3"/>
       <c r="W43" s="3"/>
@@ -3365,8 +3495,9 @@
       <c r="AF43" s="3"/>
       <c r="AG43" s="3"/>
       <c r="AH43" s="3"/>
-    </row>
-    <row r="44" spans="1:34">
+      <c r="AI43" s="3"/>
+    </row>
+    <row r="44" s="1" customFormat="1" spans="1:35">
       <c r="A44" s="3"/>
       <c r="B44" s="4"/>
       <c r="C44" s="4"/>
@@ -3386,7 +3517,7 @@
       <c r="Q44" s="4"/>
       <c r="R44" s="4"/>
       <c r="S44" s="4"/>
-      <c r="T44" s="3"/>
+      <c r="T44" s="4"/>
       <c r="U44" s="3"/>
       <c r="V44" s="3"/>
       <c r="W44" s="3"/>
@@ -3401,8 +3532,9 @@
       <c r="AF44" s="3"/>
       <c r="AG44" s="3"/>
       <c r="AH44" s="3"/>
-    </row>
-    <row r="45" spans="1:34">
+      <c r="AI44" s="3"/>
+    </row>
+    <row r="45" spans="1:35">
       <c r="A45" s="3"/>
       <c r="B45" s="4"/>
       <c r="C45" s="4"/>
@@ -3422,7 +3554,7 @@
       <c r="Q45" s="4"/>
       <c r="R45" s="4"/>
       <c r="S45" s="4"/>
-      <c r="T45" s="3"/>
+      <c r="T45" s="4"/>
       <c r="U45" s="3"/>
       <c r="V45" s="3"/>
       <c r="W45" s="3"/>
@@ -3437,8 +3569,9 @@
       <c r="AF45" s="3"/>
       <c r="AG45" s="3"/>
       <c r="AH45" s="3"/>
-    </row>
-    <row r="46" spans="1:34">
+      <c r="AI45" s="3"/>
+    </row>
+    <row r="46" spans="1:35">
       <c r="A46" s="3"/>
       <c r="B46" s="4"/>
       <c r="C46" s="4"/>
@@ -3458,7 +3591,7 @@
       <c r="Q46" s="4"/>
       <c r="R46" s="4"/>
       <c r="S46" s="4"/>
-      <c r="T46" s="3"/>
+      <c r="T46" s="4"/>
       <c r="U46" s="3"/>
       <c r="V46" s="3"/>
       <c r="W46" s="3"/>
@@ -3473,8 +3606,9 @@
       <c r="AF46" s="3"/>
       <c r="AG46" s="3"/>
       <c r="AH46" s="3"/>
-    </row>
-    <row r="47" spans="1:34">
+      <c r="AI46" s="3"/>
+    </row>
+    <row r="47" spans="1:35">
       <c r="A47" s="3"/>
       <c r="B47" s="4"/>
       <c r="C47" s="4"/>
@@ -3494,7 +3628,7 @@
       <c r="Q47" s="4"/>
       <c r="R47" s="4"/>
       <c r="S47" s="4"/>
-      <c r="T47" s="3"/>
+      <c r="T47" s="4"/>
       <c r="U47" s="3"/>
       <c r="V47" s="3"/>
       <c r="W47" s="3"/>
@@ -3509,8 +3643,9 @@
       <c r="AF47" s="3"/>
       <c r="AG47" s="3"/>
       <c r="AH47" s="3"/>
-    </row>
-    <row r="48" spans="1:34">
+      <c r="AI47" s="3"/>
+    </row>
+    <row r="48" spans="1:35">
       <c r="A48" s="3"/>
       <c r="B48" s="4"/>
       <c r="C48" s="4"/>
@@ -3530,7 +3665,7 @@
       <c r="Q48" s="4"/>
       <c r="R48" s="4"/>
       <c r="S48" s="4"/>
-      <c r="T48" s="3"/>
+      <c r="T48" s="4"/>
       <c r="U48" s="3"/>
       <c r="V48" s="3"/>
       <c r="W48" s="3"/>
@@ -3545,8 +3680,9 @@
       <c r="AF48" s="3"/>
       <c r="AG48" s="3"/>
       <c r="AH48" s="3"/>
-    </row>
-    <row r="49" spans="1:34">
+      <c r="AI48" s="3"/>
+    </row>
+    <row r="49" spans="1:35">
       <c r="A49" s="3"/>
       <c r="B49" s="4"/>
       <c r="C49" s="4"/>
@@ -3566,7 +3702,7 @@
       <c r="Q49" s="4"/>
       <c r="R49" s="4"/>
       <c r="S49" s="4"/>
-      <c r="T49" s="3"/>
+      <c r="T49" s="4"/>
       <c r="U49" s="3"/>
       <c r="V49" s="3"/>
       <c r="W49" s="3"/>
@@ -3581,8 +3717,9 @@
       <c r="AF49" s="3"/>
       <c r="AG49" s="3"/>
       <c r="AH49" s="3"/>
-    </row>
-    <row r="50" spans="1:34">
+      <c r="AI49" s="3"/>
+    </row>
+    <row r="50" spans="1:35">
       <c r="A50" s="3"/>
       <c r="B50" s="4"/>
       <c r="C50" s="4"/>
@@ -3602,7 +3739,7 @@
       <c r="Q50" s="4"/>
       <c r="R50" s="4"/>
       <c r="S50" s="4"/>
-      <c r="T50" s="3"/>
+      <c r="T50" s="4"/>
       <c r="U50" s="3"/>
       <c r="V50" s="3"/>
       <c r="W50" s="3"/>
@@ -3617,8 +3754,9 @@
       <c r="AF50" s="3"/>
       <c r="AG50" s="3"/>
       <c r="AH50" s="3"/>
-    </row>
-    <row r="51" spans="1:34">
+      <c r="AI50" s="3"/>
+    </row>
+    <row r="51" spans="1:35">
       <c r="A51" s="3"/>
       <c r="B51" s="4"/>
       <c r="C51" s="4"/>
@@ -3638,7 +3776,7 @@
       <c r="Q51" s="4"/>
       <c r="R51" s="4"/>
       <c r="S51" s="4"/>
-      <c r="T51" s="3"/>
+      <c r="T51" s="4"/>
       <c r="U51" s="3"/>
       <c r="V51" s="3"/>
       <c r="W51" s="3"/>
@@ -3653,8 +3791,9 @@
       <c r="AF51" s="3"/>
       <c r="AG51" s="3"/>
       <c r="AH51" s="3"/>
-    </row>
-    <row r="52" spans="1:34">
+      <c r="AI51" s="3"/>
+    </row>
+    <row r="52" spans="1:35">
       <c r="A52" s="3"/>
       <c r="B52" s="4"/>
       <c r="C52" s="4"/>
@@ -3674,7 +3813,7 @@
       <c r="Q52" s="4"/>
       <c r="R52" s="4"/>
       <c r="S52" s="4"/>
-      <c r="T52" s="3"/>
+      <c r="T52" s="4"/>
       <c r="U52" s="3"/>
       <c r="V52" s="3"/>
       <c r="W52" s="3"/>
@@ -3689,8 +3828,9 @@
       <c r="AF52" s="3"/>
       <c r="AG52" s="3"/>
       <c r="AH52" s="3"/>
-    </row>
-    <row r="53" spans="1:34">
+      <c r="AI52" s="3"/>
+    </row>
+    <row r="53" spans="1:35">
       <c r="A53" s="3"/>
       <c r="B53" s="4"/>
       <c r="C53" s="4"/>
@@ -3710,7 +3850,7 @@
       <c r="Q53" s="4"/>
       <c r="R53" s="4"/>
       <c r="S53" s="4"/>
-      <c r="T53" s="3"/>
+      <c r="T53" s="4"/>
       <c r="U53" s="3"/>
       <c r="V53" s="3"/>
       <c r="W53" s="3"/>
@@ -3725,8 +3865,9 @@
       <c r="AF53" s="3"/>
       <c r="AG53" s="3"/>
       <c r="AH53" s="3"/>
-    </row>
-    <row r="54" spans="1:34">
+      <c r="AI53" s="3"/>
+    </row>
+    <row r="54" spans="1:35">
       <c r="A54" s="3"/>
       <c r="B54" s="4"/>
       <c r="C54" s="4"/>
@@ -3746,7 +3887,7 @@
       <c r="Q54" s="4"/>
       <c r="R54" s="4"/>
       <c r="S54" s="4"/>
-      <c r="T54" s="3"/>
+      <c r="T54" s="4"/>
       <c r="U54" s="3"/>
       <c r="V54" s="3"/>
       <c r="W54" s="3"/>
@@ -3761,8 +3902,9 @@
       <c r="AF54" s="3"/>
       <c r="AG54" s="3"/>
       <c r="AH54" s="3"/>
-    </row>
-    <row r="55" spans="1:34">
+      <c r="AI54" s="3"/>
+    </row>
+    <row r="55" spans="1:35">
       <c r="A55" s="3"/>
       <c r="B55" s="4"/>
       <c r="C55" s="4"/>
@@ -3782,7 +3924,7 @@
       <c r="Q55" s="4"/>
       <c r="R55" s="4"/>
       <c r="S55" s="4"/>
-      <c r="T55" s="3"/>
+      <c r="T55" s="4"/>
       <c r="U55" s="3"/>
       <c r="V55" s="3"/>
       <c r="W55" s="3"/>
@@ -3797,13 +3939,14 @@
       <c r="AF55" s="3"/>
       <c r="AG55" s="3"/>
       <c r="AH55" s="3"/>
-    </row>
-    <row r="56" spans="1:34">
+      <c r="AI55" s="3"/>
+    </row>
+    <row r="56" spans="1:35">
       <c r="A56" s="3"/>
       <c r="B56" s="4"/>
       <c r="C56" s="4"/>
       <c r="D56" s="4"/>
-      <c r="E56" s="5"/>
+      <c r="E56" s="4"/>
       <c r="F56" s="4"/>
       <c r="G56" s="4"/>
       <c r="H56" s="4"/>
@@ -3818,7 +3961,7 @@
       <c r="Q56" s="4"/>
       <c r="R56" s="4"/>
       <c r="S56" s="4"/>
-      <c r="T56" s="3"/>
+      <c r="T56" s="4"/>
       <c r="U56" s="3"/>
       <c r="V56" s="3"/>
       <c r="W56" s="3"/>
@@ -3833,13 +3976,14 @@
       <c r="AF56" s="3"/>
       <c r="AG56" s="3"/>
       <c r="AH56" s="3"/>
-    </row>
-    <row r="57" spans="1:34">
+      <c r="AI56" s="3"/>
+    </row>
+    <row r="57" spans="1:35">
       <c r="A57" s="3"/>
       <c r="B57" s="4"/>
       <c r="C57" s="4"/>
       <c r="D57" s="4"/>
-      <c r="E57" s="5"/>
+      <c r="E57" s="4"/>
       <c r="F57" s="4"/>
       <c r="G57" s="4"/>
       <c r="H57" s="4"/>
@@ -3854,7 +3998,7 @@
       <c r="Q57" s="4"/>
       <c r="R57" s="4"/>
       <c r="S57" s="4"/>
-      <c r="T57" s="3"/>
+      <c r="T57" s="4"/>
       <c r="U57" s="3"/>
       <c r="V57" s="3"/>
       <c r="W57" s="3"/>
@@ -3869,13 +4013,14 @@
       <c r="AF57" s="3"/>
       <c r="AG57" s="3"/>
       <c r="AH57" s="3"/>
-    </row>
-    <row r="58" spans="1:34">
+      <c r="AI57" s="3"/>
+    </row>
+    <row r="58" spans="1:35">
       <c r="A58" s="3"/>
       <c r="B58" s="4"/>
       <c r="C58" s="4"/>
       <c r="D58" s="4"/>
-      <c r="E58" s="5"/>
+      <c r="E58" s="4"/>
       <c r="F58" s="4"/>
       <c r="G58" s="4"/>
       <c r="H58" s="4"/>
@@ -3890,7 +4035,7 @@
       <c r="Q58" s="4"/>
       <c r="R58" s="4"/>
       <c r="S58" s="4"/>
-      <c r="T58" s="3"/>
+      <c r="T58" s="4"/>
       <c r="U58" s="3"/>
       <c r="V58" s="3"/>
       <c r="W58" s="3"/>
@@ -3905,8 +4050,9 @@
       <c r="AF58" s="3"/>
       <c r="AG58" s="3"/>
       <c r="AH58" s="3"/>
-    </row>
-    <row r="59" spans="1:34">
+      <c r="AI58" s="3"/>
+    </row>
+    <row r="59" spans="1:35">
       <c r="A59" s="3"/>
       <c r="B59" s="4"/>
       <c r="C59" s="4"/>
@@ -3926,7 +4072,7 @@
       <c r="Q59" s="4"/>
       <c r="R59" s="4"/>
       <c r="S59" s="4"/>
-      <c r="T59" s="3"/>
+      <c r="T59" s="4"/>
       <c r="U59" s="3"/>
       <c r="V59" s="3"/>
       <c r="W59" s="3"/>
@@ -3941,13 +4087,14 @@
       <c r="AF59" s="3"/>
       <c r="AG59" s="3"/>
       <c r="AH59" s="3"/>
-    </row>
-    <row r="60" spans="1:34">
+      <c r="AI59" s="3"/>
+    </row>
+    <row r="60" spans="1:35">
       <c r="A60" s="3"/>
       <c r="B60" s="4"/>
       <c r="C60" s="4"/>
       <c r="D60" s="4"/>
-      <c r="E60" s="4"/>
+      <c r="E60" s="5"/>
       <c r="F60" s="4"/>
       <c r="G60" s="4"/>
       <c r="H60" s="4"/>
@@ -3962,7 +4109,7 @@
       <c r="Q60" s="4"/>
       <c r="R60" s="4"/>
       <c r="S60" s="4"/>
-      <c r="T60" s="3"/>
+      <c r="T60" s="4"/>
       <c r="U60" s="3"/>
       <c r="V60" s="3"/>
       <c r="W60" s="3"/>
@@ -3977,13 +4124,14 @@
       <c r="AF60" s="3"/>
       <c r="AG60" s="3"/>
       <c r="AH60" s="3"/>
-    </row>
-    <row r="61" spans="1:34">
+      <c r="AI60" s="3"/>
+    </row>
+    <row r="61" spans="1:35">
       <c r="A61" s="3"/>
       <c r="B61" s="4"/>
       <c r="C61" s="4"/>
       <c r="D61" s="4"/>
-      <c r="E61" s="4"/>
+      <c r="E61" s="5"/>
       <c r="F61" s="4"/>
       <c r="G61" s="4"/>
       <c r="H61" s="4"/>
@@ -3998,7 +4146,7 @@
       <c r="Q61" s="4"/>
       <c r="R61" s="4"/>
       <c r="S61" s="4"/>
-      <c r="T61" s="3"/>
+      <c r="T61" s="4"/>
       <c r="U61" s="3"/>
       <c r="V61" s="3"/>
       <c r="W61" s="3"/>
@@ -4013,13 +4161,14 @@
       <c r="AF61" s="3"/>
       <c r="AG61" s="3"/>
       <c r="AH61" s="3"/>
-    </row>
-    <row r="62" spans="1:34">
+      <c r="AI61" s="3"/>
+    </row>
+    <row r="62" spans="1:35">
       <c r="A62" s="3"/>
       <c r="B62" s="4"/>
       <c r="C62" s="4"/>
       <c r="D62" s="4"/>
-      <c r="E62" s="4"/>
+      <c r="E62" s="5"/>
       <c r="F62" s="4"/>
       <c r="G62" s="4"/>
       <c r="H62" s="4"/>
@@ -4034,7 +4183,7 @@
       <c r="Q62" s="4"/>
       <c r="R62" s="4"/>
       <c r="S62" s="4"/>
-      <c r="T62" s="3"/>
+      <c r="T62" s="4"/>
       <c r="U62" s="3"/>
       <c r="V62" s="3"/>
       <c r="W62" s="3"/>
@@ -4049,13 +4198,14 @@
       <c r="AF62" s="3"/>
       <c r="AG62" s="3"/>
       <c r="AH62" s="3"/>
-    </row>
-    <row r="63" spans="1:34">
+      <c r="AI62" s="3"/>
+    </row>
+    <row r="63" spans="1:35">
       <c r="A63" s="3"/>
       <c r="B63" s="4"/>
       <c r="C63" s="4"/>
       <c r="D63" s="4"/>
-      <c r="E63" s="5"/>
+      <c r="E63" s="4"/>
       <c r="F63" s="4"/>
       <c r="G63" s="4"/>
       <c r="H63" s="4"/>
@@ -4070,7 +4220,7 @@
       <c r="Q63" s="4"/>
       <c r="R63" s="4"/>
       <c r="S63" s="4"/>
-      <c r="T63" s="3"/>
+      <c r="T63" s="4"/>
       <c r="U63" s="3"/>
       <c r="V63" s="3"/>
       <c r="W63" s="3"/>
@@ -4085,8 +4235,9 @@
       <c r="AF63" s="3"/>
       <c r="AG63" s="3"/>
       <c r="AH63" s="3"/>
-    </row>
-    <row r="64" spans="1:34">
+      <c r="AI63" s="3"/>
+    </row>
+    <row r="64" spans="1:35">
       <c r="A64" s="3"/>
       <c r="B64" s="4"/>
       <c r="C64" s="4"/>
@@ -4106,7 +4257,7 @@
       <c r="Q64" s="4"/>
       <c r="R64" s="4"/>
       <c r="S64" s="4"/>
-      <c r="T64" s="3"/>
+      <c r="T64" s="4"/>
       <c r="U64" s="3"/>
       <c r="V64" s="3"/>
       <c r="W64" s="3"/>
@@ -4121,8 +4272,9 @@
       <c r="AF64" s="3"/>
       <c r="AG64" s="3"/>
       <c r="AH64" s="3"/>
-    </row>
-    <row r="65" spans="1:34">
+      <c r="AI64" s="3"/>
+    </row>
+    <row r="65" spans="1:35">
       <c r="A65" s="3"/>
       <c r="B65" s="4"/>
       <c r="C65" s="4"/>
@@ -4142,7 +4294,7 @@
       <c r="Q65" s="4"/>
       <c r="R65" s="4"/>
       <c r="S65" s="4"/>
-      <c r="T65" s="3"/>
+      <c r="T65" s="4"/>
       <c r="U65" s="3"/>
       <c r="V65" s="3"/>
       <c r="W65" s="3"/>
@@ -4157,8 +4309,9 @@
       <c r="AF65" s="3"/>
       <c r="AG65" s="3"/>
       <c r="AH65" s="3"/>
-    </row>
-    <row r="66" spans="1:34">
+      <c r="AI65" s="3"/>
+    </row>
+    <row r="66" spans="1:35">
       <c r="A66" s="3"/>
       <c r="B66" s="4"/>
       <c r="C66" s="4"/>
@@ -4178,7 +4331,7 @@
       <c r="Q66" s="4"/>
       <c r="R66" s="4"/>
       <c r="S66" s="4"/>
-      <c r="T66" s="3"/>
+      <c r="T66" s="4"/>
       <c r="U66" s="3"/>
       <c r="V66" s="3"/>
       <c r="W66" s="3"/>
@@ -4193,13 +4346,14 @@
       <c r="AF66" s="3"/>
       <c r="AG66" s="3"/>
       <c r="AH66" s="3"/>
-    </row>
-    <row r="67" spans="1:34">
+      <c r="AI66" s="3"/>
+    </row>
+    <row r="67" spans="1:35">
       <c r="A67" s="3"/>
       <c r="B67" s="4"/>
       <c r="C67" s="4"/>
       <c r="D67" s="4"/>
-      <c r="E67" s="4"/>
+      <c r="E67" s="5"/>
       <c r="F67" s="4"/>
       <c r="G67" s="4"/>
       <c r="H67" s="4"/>
@@ -4214,7 +4368,7 @@
       <c r="Q67" s="4"/>
       <c r="R67" s="4"/>
       <c r="S67" s="4"/>
-      <c r="T67" s="3"/>
+      <c r="T67" s="4"/>
       <c r="U67" s="3"/>
       <c r="V67" s="3"/>
       <c r="W67" s="3"/>
@@ -4229,8 +4383,9 @@
       <c r="AF67" s="3"/>
       <c r="AG67" s="3"/>
       <c r="AH67" s="3"/>
-    </row>
-    <row r="68" spans="1:34">
+      <c r="AI67" s="3"/>
+    </row>
+    <row r="68" spans="1:35">
       <c r="A68" s="3"/>
       <c r="B68" s="4"/>
       <c r="C68" s="4"/>
@@ -4250,7 +4405,7 @@
       <c r="Q68" s="4"/>
       <c r="R68" s="4"/>
       <c r="S68" s="4"/>
-      <c r="T68" s="3"/>
+      <c r="T68" s="4"/>
       <c r="U68" s="3"/>
       <c r="V68" s="3"/>
       <c r="W68" s="3"/>
@@ -4265,8 +4420,9 @@
       <c r="AF68" s="3"/>
       <c r="AG68" s="3"/>
       <c r="AH68" s="3"/>
-    </row>
-    <row r="69" spans="1:34">
+      <c r="AI68" s="3"/>
+    </row>
+    <row r="69" spans="1:35">
       <c r="A69" s="3"/>
       <c r="B69" s="4"/>
       <c r="C69" s="4"/>
@@ -4286,7 +4442,7 @@
       <c r="Q69" s="4"/>
       <c r="R69" s="4"/>
       <c r="S69" s="4"/>
-      <c r="T69" s="3"/>
+      <c r="T69" s="4"/>
       <c r="U69" s="3"/>
       <c r="V69" s="3"/>
       <c r="W69" s="3"/>
@@ -4301,8 +4457,9 @@
       <c r="AF69" s="3"/>
       <c r="AG69" s="3"/>
       <c r="AH69" s="3"/>
-    </row>
-    <row r="70" spans="1:34">
+      <c r="AI69" s="3"/>
+    </row>
+    <row r="70" spans="1:35">
       <c r="A70" s="3"/>
       <c r="B70" s="4"/>
       <c r="C70" s="4"/>
@@ -4322,7 +4479,7 @@
       <c r="Q70" s="4"/>
       <c r="R70" s="4"/>
       <c r="S70" s="4"/>
-      <c r="T70" s="3"/>
+      <c r="T70" s="4"/>
       <c r="U70" s="3"/>
       <c r="V70" s="3"/>
       <c r="W70" s="3"/>
@@ -4337,8 +4494,9 @@
       <c r="AF70" s="3"/>
       <c r="AG70" s="3"/>
       <c r="AH70" s="3"/>
-    </row>
-    <row r="71" spans="1:34">
+      <c r="AI70" s="3"/>
+    </row>
+    <row r="71" spans="1:35">
       <c r="A71" s="3"/>
       <c r="B71" s="4"/>
       <c r="C71" s="4"/>
@@ -4358,7 +4516,7 @@
       <c r="Q71" s="4"/>
       <c r="R71" s="4"/>
       <c r="S71" s="4"/>
-      <c r="T71" s="3"/>
+      <c r="T71" s="4"/>
       <c r="U71" s="3"/>
       <c r="V71" s="3"/>
       <c r="W71" s="3"/>
@@ -4373,209 +4531,364 @@
       <c r="AF71" s="3"/>
       <c r="AG71" s="3"/>
       <c r="AH71" s="3"/>
-    </row>
-    <row r="79" spans="1:23">
-      <c r="A79" s="2"/>
-      <c r="B79" s="2"/>
-      <c r="C79" s="2"/>
-      <c r="D79" s="2"/>
-      <c r="R79" s="2"/>
-      <c r="T79" s="2"/>
-      <c r="U79" s="2"/>
-      <c r="V79" s="2"/>
-      <c r="W79" s="2"/>
-    </row>
-    <row r="80" spans="1:23">
-      <c r="A80" s="2"/>
-      <c r="B80" s="2"/>
-      <c r="C80" s="2"/>
-      <c r="D80" s="2"/>
-      <c r="E80" s="2"/>
-      <c r="R80" s="2"/>
-      <c r="S80" s="2"/>
-      <c r="T80" s="2"/>
-      <c r="U80" s="2"/>
-      <c r="V80" s="2"/>
-      <c r="W80" s="2"/>
-    </row>
-    <row r="81" spans="1:23">
-      <c r="A81" s="2"/>
-      <c r="B81" s="2"/>
-      <c r="C81" s="2"/>
-      <c r="D81" s="2"/>
-      <c r="R81" s="2"/>
-      <c r="S81" s="2"/>
-      <c r="T81" s="2"/>
-      <c r="U81" s="2"/>
-      <c r="V81" s="2"/>
-      <c r="W81" s="2"/>
-    </row>
-    <row r="82" spans="1:23">
-      <c r="A82" s="2"/>
-      <c r="B82" s="2"/>
-      <c r="C82" s="2"/>
-      <c r="D82" s="2"/>
-      <c r="R82" s="2"/>
-      <c r="S82" s="2"/>
-      <c r="T82" s="2"/>
-      <c r="U82" s="2"/>
-      <c r="V82" s="2"/>
-      <c r="W82" s="2"/>
-    </row>
-    <row r="83" spans="1:23">
+      <c r="AI71" s="3"/>
+    </row>
+    <row r="72" spans="1:35">
+      <c r="A72" s="3"/>
+      <c r="B72" s="4"/>
+      <c r="C72" s="4"/>
+      <c r="D72" s="4"/>
+      <c r="E72" s="4"/>
+      <c r="F72" s="4"/>
+      <c r="G72" s="4"/>
+      <c r="H72" s="4"/>
+      <c r="I72" s="4"/>
+      <c r="J72" s="4"/>
+      <c r="K72" s="4"/>
+      <c r="L72" s="4"/>
+      <c r="M72" s="4"/>
+      <c r="N72" s="4"/>
+      <c r="O72" s="4"/>
+      <c r="P72" s="4"/>
+      <c r="Q72" s="4"/>
+      <c r="R72" s="4"/>
+      <c r="S72" s="4"/>
+      <c r="T72" s="4"/>
+      <c r="U72" s="3"/>
+      <c r="V72" s="3"/>
+      <c r="W72" s="3"/>
+      <c r="X72" s="3"/>
+      <c r="Y72" s="3"/>
+      <c r="Z72" s="3"/>
+      <c r="AA72" s="3"/>
+      <c r="AB72" s="3"/>
+      <c r="AC72" s="3"/>
+      <c r="AD72" s="3"/>
+      <c r="AE72" s="3"/>
+      <c r="AF72" s="3"/>
+      <c r="AG72" s="3"/>
+      <c r="AH72" s="3"/>
+      <c r="AI72" s="3"/>
+    </row>
+    <row r="73" spans="1:35">
+      <c r="A73" s="3"/>
+      <c r="B73" s="4"/>
+      <c r="C73" s="4"/>
+      <c r="D73" s="4"/>
+      <c r="E73" s="4"/>
+      <c r="F73" s="4"/>
+      <c r="G73" s="4"/>
+      <c r="H73" s="4"/>
+      <c r="I73" s="4"/>
+      <c r="J73" s="4"/>
+      <c r="K73" s="4"/>
+      <c r="L73" s="4"/>
+      <c r="M73" s="4"/>
+      <c r="N73" s="4"/>
+      <c r="O73" s="4"/>
+      <c r="P73" s="4"/>
+      <c r="Q73" s="4"/>
+      <c r="R73" s="4"/>
+      <c r="S73" s="4"/>
+      <c r="T73" s="4"/>
+      <c r="U73" s="3"/>
+      <c r="V73" s="3"/>
+      <c r="W73" s="3"/>
+      <c r="X73" s="3"/>
+      <c r="Y73" s="3"/>
+      <c r="Z73" s="3"/>
+      <c r="AA73" s="3"/>
+      <c r="AB73" s="3"/>
+      <c r="AC73" s="3"/>
+      <c r="AD73" s="3"/>
+      <c r="AE73" s="3"/>
+      <c r="AF73" s="3"/>
+      <c r="AG73" s="3"/>
+      <c r="AH73" s="3"/>
+      <c r="AI73" s="3"/>
+    </row>
+    <row r="74" spans="1:35">
+      <c r="A74" s="3"/>
+      <c r="B74" s="4"/>
+      <c r="C74" s="4"/>
+      <c r="D74" s="4"/>
+      <c r="E74" s="4"/>
+      <c r="F74" s="4"/>
+      <c r="G74" s="4"/>
+      <c r="H74" s="4"/>
+      <c r="I74" s="4"/>
+      <c r="J74" s="4"/>
+      <c r="K74" s="4"/>
+      <c r="L74" s="4"/>
+      <c r="M74" s="4"/>
+      <c r="N74" s="4"/>
+      <c r="O74" s="4"/>
+      <c r="P74" s="4"/>
+      <c r="Q74" s="4"/>
+      <c r="R74" s="4"/>
+      <c r="S74" s="4"/>
+      <c r="T74" s="4"/>
+      <c r="U74" s="3"/>
+      <c r="V74" s="3"/>
+      <c r="W74" s="3"/>
+      <c r="X74" s="3"/>
+      <c r="Y74" s="3"/>
+      <c r="Z74" s="3"/>
+      <c r="AA74" s="3"/>
+      <c r="AB74" s="3"/>
+      <c r="AC74" s="3"/>
+      <c r="AD74" s="3"/>
+      <c r="AE74" s="3"/>
+      <c r="AF74" s="3"/>
+      <c r="AG74" s="3"/>
+      <c r="AH74" s="3"/>
+      <c r="AI74" s="3"/>
+    </row>
+    <row r="75" spans="1:35">
+      <c r="A75" s="3"/>
+      <c r="B75" s="4"/>
+      <c r="C75" s="4"/>
+      <c r="D75" s="4"/>
+      <c r="E75" s="4"/>
+      <c r="F75" s="4"/>
+      <c r="G75" s="4"/>
+      <c r="H75" s="4"/>
+      <c r="I75" s="4"/>
+      <c r="J75" s="4"/>
+      <c r="K75" s="4"/>
+      <c r="L75" s="4"/>
+      <c r="M75" s="4"/>
+      <c r="N75" s="4"/>
+      <c r="O75" s="4"/>
+      <c r="P75" s="4"/>
+      <c r="Q75" s="4"/>
+      <c r="R75" s="4"/>
+      <c r="S75" s="4"/>
+      <c r="T75" s="4"/>
+      <c r="U75" s="3"/>
+      <c r="V75" s="3"/>
+      <c r="W75" s="3"/>
+      <c r="X75" s="3"/>
+      <c r="Y75" s="3"/>
+      <c r="Z75" s="3"/>
+      <c r="AA75" s="3"/>
+      <c r="AB75" s="3"/>
+      <c r="AC75" s="3"/>
+      <c r="AD75" s="3"/>
+      <c r="AE75" s="3"/>
+      <c r="AF75" s="3"/>
+      <c r="AG75" s="3"/>
+      <c r="AH75" s="3"/>
+      <c r="AI75" s="3"/>
+    </row>
+    <row r="83" spans="1:24">
       <c r="A83" s="2"/>
       <c r="B83" s="2"/>
       <c r="C83" s="2"/>
       <c r="D83" s="2"/>
-      <c r="R83" s="2"/>
       <c r="S83" s="2"/>
-      <c r="T83" s="2"/>
       <c r="U83" s="2"/>
       <c r="V83" s="2"/>
       <c r="W83" s="2"/>
-    </row>
-    <row r="84" spans="1:23">
+      <c r="X83" s="2"/>
+    </row>
+    <row r="84" spans="1:24">
       <c r="A84" s="2"/>
       <c r="B84" s="2"/>
       <c r="C84" s="2"/>
       <c r="D84" s="2"/>
-      <c r="R84" s="2"/>
+      <c r="E84" s="2"/>
       <c r="S84" s="2"/>
       <c r="T84" s="2"/>
       <c r="U84" s="2"/>
       <c r="V84" s="2"/>
       <c r="W84" s="2"/>
-    </row>
-    <row r="85" spans="1:23">
+      <c r="X84" s="2"/>
+    </row>
+    <row r="85" spans="1:24">
       <c r="A85" s="2"/>
       <c r="B85" s="2"/>
       <c r="C85" s="2"/>
       <c r="D85" s="2"/>
-      <c r="R85" s="2"/>
       <c r="S85" s="2"/>
       <c r="T85" s="2"/>
       <c r="U85" s="2"/>
       <c r="V85" s="2"/>
       <c r="W85" s="2"/>
-    </row>
-    <row r="86" spans="1:23">
+      <c r="X85" s="2"/>
+    </row>
+    <row r="86" spans="1:24">
       <c r="A86" s="2"/>
       <c r="B86" s="2"/>
       <c r="C86" s="2"/>
       <c r="D86" s="2"/>
-      <c r="R86" s="2"/>
       <c r="S86" s="2"/>
       <c r="T86" s="2"/>
       <c r="U86" s="2"/>
       <c r="V86" s="2"/>
       <c r="W86" s="2"/>
-    </row>
-    <row r="87" spans="1:23">
+      <c r="X86" s="2"/>
+    </row>
+    <row r="87" spans="1:24">
       <c r="A87" s="2"/>
       <c r="B87" s="2"/>
       <c r="C87" s="2"/>
       <c r="D87" s="2"/>
-      <c r="R87" s="2"/>
       <c r="S87" s="2"/>
       <c r="T87" s="2"/>
       <c r="U87" s="2"/>
       <c r="V87" s="2"/>
       <c r="W87" s="2"/>
-    </row>
-    <row r="88" spans="1:23">
+      <c r="X87" s="2"/>
+    </row>
+    <row r="88" spans="1:24">
       <c r="A88" s="2"/>
       <c r="B88" s="2"/>
       <c r="C88" s="2"/>
       <c r="D88" s="2"/>
-      <c r="R88" s="2"/>
       <c r="S88" s="2"/>
       <c r="T88" s="2"/>
       <c r="U88" s="2"/>
       <c r="V88" s="2"/>
       <c r="W88" s="2"/>
-    </row>
-    <row r="89" spans="1:23">
+      <c r="X88" s="2"/>
+    </row>
+    <row r="89" spans="1:24">
       <c r="A89" s="2"/>
       <c r="B89" s="2"/>
       <c r="C89" s="2"/>
       <c r="D89" s="2"/>
-      <c r="R89" s="2"/>
       <c r="S89" s="2"/>
       <c r="T89" s="2"/>
       <c r="U89" s="2"/>
       <c r="V89" s="2"/>
       <c r="W89" s="2"/>
-    </row>
-    <row r="90" spans="1:23">
+      <c r="X89" s="2"/>
+    </row>
+    <row r="90" spans="1:24">
       <c r="A90" s="2"/>
       <c r="B90" s="2"/>
       <c r="C90" s="2"/>
       <c r="D90" s="2"/>
-      <c r="R90" s="2"/>
       <c r="S90" s="2"/>
       <c r="T90" s="2"/>
       <c r="U90" s="2"/>
       <c r="V90" s="2"/>
       <c r="W90" s="2"/>
-    </row>
-    <row r="91" spans="1:23">
+      <c r="X90" s="2"/>
+    </row>
+    <row r="91" spans="1:24">
       <c r="A91" s="2"/>
       <c r="B91" s="2"/>
       <c r="C91" s="2"/>
       <c r="D91" s="2"/>
-      <c r="R91" s="2"/>
       <c r="S91" s="2"/>
       <c r="T91" s="2"/>
       <c r="U91" s="2"/>
       <c r="V91" s="2"/>
       <c r="W91" s="2"/>
-    </row>
-    <row r="92" spans="1:23">
+      <c r="X91" s="2"/>
+    </row>
+    <row r="92" spans="1:24">
       <c r="A92" s="2"/>
       <c r="B92" s="2"/>
       <c r="C92" s="2"/>
       <c r="D92" s="2"/>
-      <c r="R92" s="2"/>
       <c r="S92" s="2"/>
       <c r="T92" s="2"/>
       <c r="U92" s="2"/>
       <c r="V92" s="2"/>
       <c r="W92" s="2"/>
+      <c r="X92" s="2"/>
+    </row>
+    <row r="93" spans="1:24">
+      <c r="A93" s="2"/>
+      <c r="B93" s="2"/>
+      <c r="C93" s="2"/>
+      <c r="D93" s="2"/>
+      <c r="S93" s="2"/>
+      <c r="T93" s="2"/>
+      <c r="U93" s="2"/>
+      <c r="V93" s="2"/>
+      <c r="W93" s="2"/>
+      <c r="X93" s="2"/>
+    </row>
+    <row r="94" spans="1:24">
+      <c r="A94" s="2"/>
+      <c r="B94" s="2"/>
+      <c r="C94" s="2"/>
+      <c r="D94" s="2"/>
+      <c r="S94" s="2"/>
+      <c r="T94" s="2"/>
+      <c r="U94" s="2"/>
+      <c r="V94" s="2"/>
+      <c r="W94" s="2"/>
+      <c r="X94" s="2"/>
+    </row>
+    <row r="95" spans="1:24">
+      <c r="A95" s="2"/>
+      <c r="B95" s="2"/>
+      <c r="C95" s="2"/>
+      <c r="D95" s="2"/>
+      <c r="S95" s="2"/>
+      <c r="T95" s="2"/>
+      <c r="U95" s="2"/>
+      <c r="V95" s="2"/>
+      <c r="W95" s="2"/>
+      <c r="X95" s="2"/>
+    </row>
+    <row r="96" spans="1:24">
+      <c r="A96" s="2"/>
+      <c r="B96" s="2"/>
+      <c r="C96" s="2"/>
+      <c r="D96" s="2"/>
+      <c r="S96" s="2"/>
+      <c r="T96" s="2"/>
+      <c r="U96" s="2"/>
+      <c r="V96" s="2"/>
+      <c r="W96" s="2"/>
+      <c r="X96" s="2"/>
     </row>
   </sheetData>
-  <dataValidations count="11">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F6 F15 F18 F19 F20 F21 F24 F25 F26 F27 F28 F29 F30 F31 F34 F35 F36 F2:F5 F7:F14 F16:F17 F22:F23 F32:F33 F37:F1048576">
+  <dataValidations count="13">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C2:C1048576">
+      <formula1>"PC_4,PC_0,PC_ALU,PC_EPC"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H38 H39 H40 H10:H37 H41:H1048576">
+      <formula1>"WB_ALU,WB_MEM,WB_PC4,WB_XX,WB_CSR"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D4 D5 D6 D7 D8 D9 D10 D11 D12 D13 D14 D15 D16 D17 D18 D19 D20 D21 D22 D23 D24 D25 D26 D27 D28 D29 D30 D31 D32 D33 D34 D35 D36 D37 D38 D39 D40 D2:D3 D41:D1048576">
+      <formula1>"A_PC,A_RS1"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="M37 M38 M39 M40 M2:M36 M41:M1048576">
+      <formula1>"CSR_W,CSR_S,CSR_C,CSR_P,CSR_XX"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="N4 N5 N6 N7 N8 N9 N10 N11 N12 N13 N14 N15 N16 N17 N18 N19 N20 N21 N22 N23 N24 N25 N26 N27 N28 N29 N30 N31 N32 N33 N34 N35 N36 N37 N38 N39 N40 N2:N3 N41:N1048576">
+      <formula1>"INST_VALID,INST_INVALID"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J5 J6 J7 J8 J9 J10 J11 J12 J13 J14 J15 J16 J17 J18 J19 J20 J21 J22 J23 J24 J25 J26 J27 J28 J29 J30 J31 J32 J33 J34 J35 J36 J37 J38 J39 J40 J2:J4 J41:J1048576">
+      <formula1>"ST_SW,ST_SH,ST_SB,ST_XX"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F6 F15 F18 F19 F20 F21 F24 F25 F26 F27 F28 F29 F30 F31 F34 F35 F36 F37 F38 F39 F40 F2:F5 F7:F14 F16:F17 F22:F23 F32:F33 F41:F1048576">
       <formula1>"ALU_ADD,ALU_SUB,ALU_AND,ALU_OR,ALU_XOR,ALU_SLL,ALU_SRL,ALU_SLT,ALU_SLTU,ALU_COPY_A,ALU_COPY_B,ALU_SRA"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L5 L6 L7 L10 L11 L14 L15 L16 L17 L18 L19 L20 L21 L22 L23 L24 L25 L26 L27 L28 L29 L30 L31 L32 L33 L34 L35 L36 L2:L4 L8:L9 L12:L13 L37:L1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L5 L6 L7 L10 L11 L14 L15 L16 L17 L18 L19 L20 L21 L22 L23 L24 L25 L26 L27 L28 L29 L30 L31 L32 L33 L34 L35 L36 L37 L38 L39 L40 L2:L4 L8:L9 L12:L13 L41:L1048576">
       <formula1>"BR_EQ,BR_NE,BR_LTU,BR_GE,BR_GEU,BR_LT,BR_XX"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J5 J6 J7 J8 J9 J10 J11 J12 J13 J14 J15 J16 J17 J18 J19 J20 J21 J22 J23 J24 J25 J26 J27 J28 J29 J30 J31 J32 J33 J34 J35 J36 J2:J4 J37:J1048576">
-      <formula1>"ST_SW,ST_SH,ST_SB,ST_XX"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H5 H6 H7 H8 H9 H10 H11 H14 H15 H16 H17 H18 H19 H20 H21 H22 H23 H24 H25 H26 H27 H28 H29 H30 H31 H32 H33 H34 H35 H36 H2:H4 H12:H13 H37:H1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H5 H6 H7 H8 H9 H2:H4">
       <formula1>"WB_ALU,WB_MEM,WB_PC4,WB_XX"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="M4 M5 M6 M7 M8 M9 M10 M11 M12 M13 M14 M15 M16 M17 M18 M19 M20 M21 M22 M23 M24 M25 M26 M27 M28 M29 M30 M31 M32 M33 M34 M35 M36 M2:M3 M37:M1048576">
-      <formula1>"INST_VALID,INST_INVALID"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K4 K5 K6 K7 K8 K9 K10 K11 K12 K13 K14 K15 K16 K17 K18 K19 K20 K21 K22 K23 K24 K25 K26 K27 K28 K29 K30 K31 K32 K33 K34 K35 K36 K2:K3 K37:K1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K4 K5 K6 K7 K8 K9 K10 K11 K12 K13 K14 K15 K16 K17 K18 K19 K20 K21 K22 K23 K24 K25 K26 K27 K28 K29 K30 K31 K32 K33 K34 K35 K36 K37 K38 K39 K40 K2:K3 K41:K1048576">
       <formula1>"MASK_XX,MASK_B,MASK_H,MASK_W,MASK_D"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I4 I5 I6 I7 I8 I9 I10 I11 I12 I13 I14 I15 I16 I17 I18 I19 I20 I21 I22 I23 I24 I25 I26 I27 I28 I29 I30 I31 I32 I33 I34 I35 I36 I2:I3 I37:I1048576">
-      <formula1>"LD_LB,LD_LH,LD_LW,LD_LBU,LD_LHU,LD_XX"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G4 G5 G6 G7 G8 G9 G10 G11 G12 G13 G14 G15 G16 G17 G18 G19 G20 G21 G22 G23 G24 G25 G26 G27 G28 G29 G30 G31 G32 G33 G34 G35 G36 G37 G38 G39 G40 G2:G3 G41:G1048576">
+      <formula1>"IMM_I,IMM_J,IMM_U,IMM_S,IMM_B"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E4 E5 E6 E7 E8 E9 E10 E11 E12 E13 E14 E15 E16 E17 E18 E19 E20 E21 E22 E23 E24 E25 E26 E27 E28 E29 E30 E31 E32 E33 E34 E35 E36 E2:E3 E37:E1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E4 E5 E6 E7 E8 E9 E10 E11 E12 E13 E14 E15 E16 E17 E18 E19 E20 E21 E22 E23 E24 E25 E26 E27 E28 E29 E30 E31 E32 E33 E34 E35 E36 E37 E38 E39 E40 E2:E3 E41:E1048576">
       <formula1>"B_IMM,B_RS2"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G4 G5 G6 G7 G8 G9 G10 G11 G12 G13 G14 G15 G16 G17 G18 G19 G20 G21 G22 G23 G24 G25 G26 G27 G28 G29 G30 G31 G32 G33 G34 G35 G36 G2:G3 G37:G1048576">
-      <formula1>"IMM_I,IMM_J,IMM_U,IMM_S,IMM_B"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D4 D5 D6 D7 D8 D9 D10 D11 D12 D13 D14 D15 D16 D17 D18 D19 D20 D21 D22 D23 D24 D25 D26 D27 D28 D29 D30 D31 D32 D33 D34 D35 D36 D2:D3 D37:D1048576">
-      <formula1>"A_PC,A_RS1"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C4 C5 C6 C7 C8 C9 C10 C11 C12 C13 C14 C15 C16 C17 C18 C19 C20 C21 C22 C23 C24 C25 C26 C27 C28 C29 C30 C31 C32 C33 C34 C35 C36 C2:C3 C37:C1048576">
-      <formula1>"PC_4,PC_0,PC_ALU"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I4 I5 I6 I7 I8 I9 I10 I11 I12 I13 I14 I15 I16 I17 I18 I19 I20 I21 I22 I23 I24 I25 I26 I27 I28 I29 I30 I31 I32 I33 I34 I35 I36 I37 I38 I39 I40 I2:I3 I41:I1048576">
+      <formula1>"LD_LB,LD_LH,LD_LW,LD_LBU,LD_LHU,LD_XX"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
> sim RTL ysyx_23060246 韩炳晋 Linux archlinux 6.6.60-1-lts #1 SMP PREEMPT_DYNAMIC Fri, 08 Nov 2024 16:03:02 +0000 x86_64 GNU/Linux  18:44:24 up  3:03,  2 users,  load average: 1.44, 0.72, 0.59
</commit_message>
<xml_diff>
--- a/npc/tools/control_gen/control_table.xlsx
+++ b/npc/tools/control_gen/control_table.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="296" uniqueCount="109">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="296" uniqueCount="108">
   <si>
     <t>comment</t>
   </si>
@@ -289,7 +289,7 @@
     <t>csrrw</t>
   </si>
   <si>
-    <t>PC_0</t>
+    <t>PC_4</t>
   </si>
   <si>
     <t>WB_CSR</t>
@@ -305,9 +305,6 @@
   </si>
   <si>
     <t>ecall</t>
-  </si>
-  <si>
-    <t>PC_4</t>
   </si>
   <si>
     <t>CSR_P</t>
@@ -3277,7 +3274,7 @@
         <v>96</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>97</v>
+        <v>91</v>
       </c>
       <c r="D39" s="4"/>
       <c r="E39" s="4"/>
@@ -3291,7 +3288,7 @@
       <c r="K39" s="4"/>
       <c r="L39" s="4"/>
       <c r="M39" s="4" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="N39" s="4" t="s">
         <v>19</v>
@@ -3321,10 +3318,10 @@
     <row r="40" spans="1:35">
       <c r="A40" s="3"/>
       <c r="B40" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="C40" s="2" t="s">
         <v>99</v>
-      </c>
-      <c r="C40" s="2" t="s">
-        <v>100</v>
       </c>
       <c r="D40" s="4"/>
       <c r="E40" s="4"/>
@@ -3338,7 +3335,7 @@
       <c r="K40" s="4"/>
       <c r="L40" s="4"/>
       <c r="M40" s="4" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="N40" s="4" t="s">
         <v>19</v>
@@ -3367,10 +3364,10 @@
     </row>
     <row r="41" spans="2:35">
       <c r="B41" s="2" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>97</v>
+        <v>91</v>
       </c>
       <c r="D41" s="2" t="s">
         <v>24</v>
@@ -3385,25 +3382,25 @@
         <v>25</v>
       </c>
       <c r="H41" s="4" t="s">
+        <v>101</v>
+      </c>
+      <c r="I41" s="4" t="s">
         <v>102</v>
       </c>
-      <c r="I41" s="4" t="s">
+      <c r="J41" s="4" t="s">
         <v>103</v>
       </c>
-      <c r="J41" s="4" t="s">
+      <c r="K41" s="2" t="s">
         <v>104</v>
       </c>
-      <c r="K41" s="2" t="s">
+      <c r="L41" s="2" t="s">
         <v>105</v>
       </c>
-      <c r="L41" s="2" t="s">
+      <c r="M41" s="2" t="s">
         <v>106</v>
       </c>
-      <c r="M41" s="2" t="s">
+      <c r="N41" s="2" t="s">
         <v>107</v>
-      </c>
-      <c r="N41" s="2" t="s">
-        <v>108</v>
       </c>
       <c r="O41" s="2"/>
       <c r="P41" s="2"/>

</xml_diff>

<commit_message>
> sim RTL ysyx_23060246 韩炳晋 Linux archlinux 6.6.60-1-lts #1 SMP PREEMPT_DYNAMIC Fri, 08 Nov 2024 16:03:02 +0000 x86_64 GNU/Linux  18:45:34 up  3:04,  2 users,  load average: 1.25, 0.76, 0.61
</commit_message>
<xml_diff>
--- a/npc/tools/control_gen/control_table.xlsx
+++ b/npc/tools/control_gen/control_table.xlsx
@@ -307,13 +307,13 @@
     <t>ecall</t>
   </si>
   <si>
+    <t>PC_EPC</t>
+  </si>
+  <si>
     <t>CSR_P</t>
   </si>
   <si>
     <t>mret</t>
-  </si>
-  <si>
-    <t>PC_EPC</t>
   </si>
   <si>
     <t>default</t>
@@ -3274,7 +3274,7 @@
         <v>96</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>91</v>
+        <v>97</v>
       </c>
       <c r="D39" s="4"/>
       <c r="E39" s="4"/>
@@ -3288,7 +3288,7 @@
       <c r="K39" s="4"/>
       <c r="L39" s="4"/>
       <c r="M39" s="4" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="N39" s="4" t="s">
         <v>19</v>
@@ -3318,10 +3318,10 @@
     <row r="40" spans="1:35">
       <c r="A40" s="3"/>
       <c r="B40" s="4" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="D40" s="4"/>
       <c r="E40" s="4"/>
@@ -3335,7 +3335,7 @@
       <c r="K40" s="4"/>
       <c r="L40" s="4"/>
       <c r="M40" s="4" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="N40" s="4" t="s">
         <v>19</v>

</xml_diff>

<commit_message>
> sim RTL ysyx_23060246 韩炳晋 Linux archlinux 6.6.60-1-lts #1 SMP PREEMPT_DYNAMIC Fri, 08 Nov 2024 16:03:02 +0000 x86_64 GNU/Linux  19:47:20 up  4:06,  2 users,  load average: 2.75, 2.26, 1.68
</commit_message>
<xml_diff>
--- a/npc/tools/control_gen/control_table.xlsx
+++ b/npc/tools/control_gen/control_table.xlsx
@@ -307,7 +307,7 @@
     <t>ecall</t>
   </si>
   <si>
-    <t>PC_EPC</t>
+    <t>PC_CSR</t>
   </si>
   <si>
     <t>CSR_P</t>
@@ -4848,9 +4848,6 @@
     </row>
   </sheetData>
   <dataValidations count="13">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C2:C1048576">
-      <formula1>"PC_4,PC_0,PC_ALU,PC_EPC"</formula1>
-    </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H38 H39 H40 H10:H37 H41:H1048576">
       <formula1>"WB_ALU,WB_MEM,WB_PC4,WB_XX,WB_CSR"</formula1>
     </dataValidation>
@@ -4865,6 +4862,9 @@
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J5 J6 J7 J8 J9 J10 J11 J12 J13 J14 J15 J16 J17 J18 J19 J20 J21 J22 J23 J24 J25 J26 J27 J28 J29 J30 J31 J32 J33 J34 J35 J36 J37 J38 J39 J40 J2:J4 J41:J1048576">
       <formula1>"ST_SW,ST_SH,ST_SB,ST_XX"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C2:C1048576">
+      <formula1>"PC_4,PC_0,PC_ALU,PC_CSR"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F6 F15 F18 F19 F20 F21 F24 F25 F26 F27 F28 F29 F30 F31 F34 F35 F36 F37 F38 F39 F40 F2:F5 F7:F14 F16:F17 F22:F23 F32:F33 F41:F1048576">
       <formula1>"ALU_ADD,ALU_SUB,ALU_AND,ALU_OR,ALU_XOR,ALU_SLL,ALU_SRL,ALU_SLT,ALU_SLTU,ALU_COPY_A,ALU_COPY_B,ALU_SRA"</formula1>

</xml_diff>

<commit_message>
support csr to run rt-thread
</commit_message>
<xml_diff>
--- a/npc/tools/control_gen/control_table.xlsx
+++ b/npc/tools/control_gen/control_table.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="27795" windowHeight="12075"/>
+    <workbookView windowWidth="27795" windowHeight="12735"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="270" uniqueCount="97">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="296" uniqueCount="108">
   <si>
     <t>comment</t>
   </si>
@@ -52,6 +52,9 @@
     <t>br_sel</t>
   </si>
   <si>
+    <t>csr_sel</t>
+  </si>
+  <si>
     <t>inst_valid</t>
   </si>
   <si>
@@ -283,12 +286,39 @@
     <t>or</t>
   </si>
   <si>
+    <t>csrrw</t>
+  </si>
+  <si>
+    <t>PC_4</t>
+  </si>
+  <si>
+    <t>WB_CSR</t>
+  </si>
+  <si>
+    <t>CSR_W</t>
+  </si>
+  <si>
+    <t>csrrs</t>
+  </si>
+  <si>
+    <t>CSR_S</t>
+  </si>
+  <si>
+    <t>ecall</t>
+  </si>
+  <si>
+    <t>PC_CSR</t>
+  </si>
+  <si>
+    <t>CSR_P</t>
+  </si>
+  <si>
+    <t>mret</t>
+  </si>
+  <si>
     <t>default</t>
   </si>
   <si>
-    <t>PC_4</t>
-  </si>
-  <si>
     <t>WB_XX</t>
   </si>
   <si>
@@ -302,6 +332,9 @@
   </si>
   <si>
     <t>BR_XX</t>
+  </si>
+  <si>
+    <t>CSR_XX</t>
   </si>
   <si>
     <t>INST_INVALID</t>
@@ -312,10 +345,10 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="4">
+    <numFmt numFmtId="41" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
+    <numFmt numFmtId="42" formatCode="_ &quot;￥&quot;* #,##0_ ;_ &quot;￥&quot;* \-#,##0_ ;_ &quot;￥&quot;* &quot;-&quot;_ ;_ @_ "/>
     <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="42" formatCode="_ &quot;￥&quot;* #,##0_ ;_ &quot;￥&quot;* \-#,##0_ ;_ &quot;￥&quot;* &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="41" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
   <fonts count="22">
     <font>
@@ -346,7 +379,22 @@
     </font>
     <font>
       <sz val="11"/>
+      <color theme="1"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
       <color theme="0"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color rgb="FF7F7F7F"/>
       <name val="宋体"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -354,6 +402,22 @@
     <font>
       <b/>
       <sz val="11"/>
+      <color theme="3"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="13"/>
       <color theme="3"/>
       <name val="宋体"/>
       <charset val="134"/>
@@ -369,22 +433,7 @@
     </font>
     <font>
       <sz val="11"/>
-      <color theme="1"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="18"/>
-      <color theme="3"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
+      <color rgb="FF9C6500"/>
       <name val="宋体"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -392,6 +441,22 @@
     <font>
       <sz val="11"/>
       <color rgb="FF9C0006"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF3F3F3F"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
       <name val="宋体"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -412,48 +477,8 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
       <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="11"/>
-      <color rgb="FF7F7F7F"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="13"/>
-      <color theme="3"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FF3F3F3F"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C6500"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
+      <color rgb="FFFF0000"/>
       <name val="宋体"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -475,6 +500,14 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <b/>
+      <sz val="18"/>
+      <color theme="3"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <sz val="11"/>
       <color rgb="FF3F3F76"/>
       <name val="宋体"/>
@@ -491,7 +524,49 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -503,7 +578,103 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFA5A5A5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor theme="9" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.399975585192419"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -515,103 +686,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor theme="6" tint="0.799981688894314"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFA5A5A5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
+        <fgColor theme="6" tint="0.599993896298105"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -623,55 +704,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="FFFFCC99"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.399975585192419"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -704,6 +737,30 @@
     </border>
     <border>
       <left style="thin">
+        <color rgb="FF7F7F7F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF7F7F7F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF7F7F7F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF7F7F7F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
         <color rgb="FFB2B2B2"/>
       </left>
       <right style="thin">
@@ -718,11 +775,17 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4"/>
+      <left style="thin">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF3F3F3F"/>
       </bottom>
       <diagonal/>
     </border>
@@ -742,36 +805,6 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF7F7F7F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF7F7F7F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF7F7F7F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF7F7F7F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
       <left/>
       <right/>
       <top style="thin">
@@ -787,145 +820,145 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="30" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="5" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="32" borderId="3" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="3" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="17" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="5" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="21" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="19" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="21" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="17" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
@@ -1273,7 +1306,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:AH92"/>
+  <dimension ref="A1:AI96"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
     <col min="1" max="1" width="13.1" customWidth="1"/>
@@ -1285,19 +1318,19 @@
     <col min="7" max="7" width="10.9416666666667" customWidth="1"/>
     <col min="8" max="10" width="11.9833333333333" customWidth="1"/>
     <col min="11" max="11" width="15.075" customWidth="1"/>
-    <col min="12" max="13" width="12.1083333333333" customWidth="1"/>
-    <col min="14" max="14" width="10.8583333333333" customWidth="1"/>
-    <col min="16" max="16" width="14.2166666666667" customWidth="1"/>
-    <col min="17" max="17" width="11.8083333333333" customWidth="1"/>
-    <col min="18" max="18" width="10.6" customWidth="1"/>
-    <col min="19" max="19" width="9.70833333333333" customWidth="1"/>
-    <col min="20" max="20" width="11.1666666666667" customWidth="1"/>
-    <col min="21" max="21" width="11.4083333333333" customWidth="1"/>
-    <col min="22" max="22" width="12.0583333333333" customWidth="1"/>
-    <col min="23" max="23" width="15.575" customWidth="1"/>
+    <col min="12" max="14" width="12.1083333333333" customWidth="1"/>
+    <col min="15" max="15" width="10.8583333333333" customWidth="1"/>
+    <col min="17" max="17" width="14.2166666666667" customWidth="1"/>
+    <col min="18" max="18" width="11.8083333333333" customWidth="1"/>
+    <col min="19" max="19" width="10.6" customWidth="1"/>
+    <col min="20" max="20" width="9.70833333333333" customWidth="1"/>
+    <col min="21" max="21" width="11.1666666666667" customWidth="1"/>
+    <col min="22" max="22" width="11.4083333333333" customWidth="1"/>
+    <col min="23" max="23" width="12.0583333333333" customWidth="1"/>
+    <col min="24" max="24" width="15.575" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="15" customHeight="1" spans="1:22">
+    <row r="1" ht="15" customHeight="1" spans="1:23">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1337,47 +1370,50 @@
       <c r="M1" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="2"/>
+      <c r="N1" s="2" t="s">
+        <v>13</v>
+      </c>
       <c r="O1" s="2"/>
       <c r="P1" s="2"/>
       <c r="Q1" s="2"/>
       <c r="R1" s="2"/>
       <c r="S1" s="2"/>
-      <c r="V1" s="6"/>
-    </row>
-    <row r="2" spans="1:34">
+      <c r="T1" s="2"/>
+      <c r="W1" s="6"/>
+    </row>
+    <row r="2" spans="1:35">
       <c r="A2" s="3"/>
       <c r="B2" s="4" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="4"/>
       <c r="E2" s="4" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F2" s="4" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="G2" s="4" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="H2" s="4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="I2" s="4"/>
       <c r="J2" s="4"/>
       <c r="K2" s="4"/>
       <c r="L2" s="4"/>
-      <c r="M2" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="N2" s="4"/>
+      <c r="M2" s="4"/>
+      <c r="N2" s="4" t="s">
+        <v>19</v>
+      </c>
       <c r="O2" s="4"/>
       <c r="P2" s="4"/>
       <c r="Q2" s="4"/>
       <c r="R2" s="4"/>
       <c r="S2" s="4"/>
-      <c r="T2" s="3"/>
+      <c r="T2" s="4"/>
       <c r="U2" s="3"/>
       <c r="V2" s="3"/>
       <c r="W2" s="3"/>
@@ -1392,42 +1428,43 @@
       <c r="AF2" s="3"/>
       <c r="AG2" s="3"/>
       <c r="AH2" s="3"/>
-    </row>
-    <row r="3" spans="1:34">
+      <c r="AI2" s="3"/>
+    </row>
+    <row r="3" spans="1:35">
       <c r="A3" s="3"/>
       <c r="B3" s="4" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C3" s="2"/>
       <c r="D3" s="4" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="G3" s="4" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="H3" s="4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="I3" s="4"/>
       <c r="J3" s="4"/>
       <c r="K3" s="4"/>
       <c r="L3" s="4"/>
-      <c r="M3" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="N3" s="4"/>
+      <c r="M3" s="4"/>
+      <c r="N3" s="4" t="s">
+        <v>19</v>
+      </c>
       <c r="O3" s="4"/>
       <c r="P3" s="4"/>
       <c r="Q3" s="4"/>
       <c r="R3" s="4"/>
       <c r="S3" s="4"/>
-      <c r="T3" s="3"/>
+      <c r="T3" s="4"/>
       <c r="U3" s="3"/>
       <c r="V3" s="3"/>
       <c r="W3" s="3"/>
@@ -1442,42 +1479,43 @@
       <c r="AF3" s="3"/>
       <c r="AG3" s="3"/>
       <c r="AH3" s="3"/>
-    </row>
-    <row r="4" spans="1:34">
+      <c r="AI3" s="3"/>
+    </row>
+    <row r="4" spans="1:35">
       <c r="A4" s="3"/>
       <c r="B4" s="4" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C4" s="2"/>
       <c r="D4" s="4" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="H4" s="4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="I4" s="4"/>
       <c r="J4" s="4"/>
       <c r="K4" s="4"/>
       <c r="L4" s="4"/>
-      <c r="M4" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="N4" s="4"/>
+      <c r="M4" s="4"/>
+      <c r="N4" s="4" t="s">
+        <v>19</v>
+      </c>
       <c r="O4" s="4"/>
       <c r="P4" s="4"/>
       <c r="Q4" s="4"/>
       <c r="R4" s="4"/>
       <c r="S4" s="4"/>
-      <c r="T4" s="3"/>
+      <c r="T4" s="4"/>
       <c r="U4" s="3"/>
       <c r="V4" s="3"/>
       <c r="W4" s="3"/>
@@ -1492,42 +1530,43 @@
       <c r="AF4" s="3"/>
       <c r="AG4" s="3"/>
       <c r="AH4" s="3"/>
-    </row>
-    <row r="5" spans="1:34">
+      <c r="AI4" s="3"/>
+    </row>
+    <row r="5" spans="1:35">
       <c r="A5" s="3"/>
       <c r="B5" s="4" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C5" s="2"/>
       <c r="D5" s="4" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="H5" s="4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="I5" s="4"/>
       <c r="J5" s="4"/>
       <c r="K5" s="4"/>
       <c r="L5" s="4"/>
-      <c r="M5" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="N5" s="4"/>
+      <c r="M5" s="4"/>
+      <c r="N5" s="4" t="s">
+        <v>19</v>
+      </c>
       <c r="O5" s="4"/>
       <c r="P5" s="4"/>
       <c r="Q5" s="4"/>
       <c r="R5" s="4"/>
       <c r="S5" s="4"/>
-      <c r="T5" s="3"/>
+      <c r="T5" s="4"/>
       <c r="U5" s="3"/>
       <c r="V5" s="3"/>
       <c r="W5" s="3"/>
@@ -1542,42 +1581,43 @@
       <c r="AF5" s="3"/>
       <c r="AG5" s="3"/>
       <c r="AH5" s="3"/>
-    </row>
-    <row r="6" spans="1:34">
+      <c r="AI5" s="3"/>
+    </row>
+    <row r="6" spans="1:35">
       <c r="A6" s="3"/>
       <c r="B6" s="4" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C6" s="2"/>
       <c r="D6" s="4" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="G6" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="H6" s="4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="I6" s="4"/>
       <c r="J6" s="4"/>
       <c r="K6" s="4"/>
       <c r="L6" s="4"/>
-      <c r="M6" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="N6" s="4"/>
+      <c r="M6" s="4"/>
+      <c r="N6" s="4" t="s">
+        <v>19</v>
+      </c>
       <c r="O6" s="4"/>
       <c r="P6" s="4"/>
       <c r="Q6" s="4"/>
       <c r="R6" s="4"/>
       <c r="S6" s="4"/>
-      <c r="T6" s="3"/>
+      <c r="T6" s="4"/>
       <c r="U6" s="3"/>
       <c r="V6" s="3"/>
       <c r="W6" s="3"/>
@@ -1592,42 +1632,43 @@
       <c r="AF6" s="3"/>
       <c r="AG6" s="3"/>
       <c r="AH6" s="3"/>
-    </row>
-    <row r="7" spans="1:34">
+      <c r="AI6" s="3"/>
+    </row>
+    <row r="7" spans="1:35">
       <c r="A7" s="3"/>
       <c r="B7" s="4" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C7" s="2"/>
       <c r="D7" s="4" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="G7" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="H7" s="4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="I7" s="4"/>
       <c r="J7" s="4"/>
       <c r="K7" s="4"/>
       <c r="L7" s="4"/>
-      <c r="M7" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="N7" s="4"/>
+      <c r="M7" s="4"/>
+      <c r="N7" s="4" t="s">
+        <v>19</v>
+      </c>
       <c r="O7" s="4"/>
       <c r="P7" s="4"/>
       <c r="Q7" s="4"/>
       <c r="R7" s="4"/>
       <c r="S7" s="4"/>
-      <c r="T7" s="3"/>
+      <c r="T7" s="4"/>
       <c r="U7" s="3"/>
       <c r="V7" s="3"/>
       <c r="W7" s="3"/>
@@ -1642,44 +1683,45 @@
       <c r="AF7" s="3"/>
       <c r="AG7" s="3"/>
       <c r="AH7" s="3"/>
-    </row>
-    <row r="8" spans="1:34">
+      <c r="AI7" s="3"/>
+    </row>
+    <row r="8" spans="1:35">
       <c r="A8" s="3"/>
       <c r="B8" s="4" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F8" s="4" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="G8" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="H8" s="4" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="I8" s="4"/>
       <c r="J8" s="4"/>
       <c r="K8" s="4"/>
       <c r="L8" s="4"/>
-      <c r="M8" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="N8" s="4"/>
+      <c r="M8" s="4"/>
+      <c r="N8" s="4" t="s">
+        <v>19</v>
+      </c>
       <c r="O8" s="4"/>
       <c r="P8" s="4"/>
       <c r="Q8" s="4"/>
       <c r="R8" s="4"/>
       <c r="S8" s="4"/>
-      <c r="T8" s="3"/>
+      <c r="T8" s="4"/>
       <c r="U8" s="3"/>
       <c r="V8" s="3"/>
       <c r="W8" s="3"/>
@@ -1694,44 +1736,45 @@
       <c r="AF8" s="3"/>
       <c r="AG8" s="3"/>
       <c r="AH8" s="3"/>
-    </row>
-    <row r="9" spans="1:34">
+      <c r="AI8" s="3"/>
+    </row>
+    <row r="9" spans="1:35">
       <c r="A9" s="3"/>
       <c r="B9" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="D9" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="E9" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="F9" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="G9" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="H9" s="4" t="s">
         <v>34</v>
-      </c>
-      <c r="C9" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="D9" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="E9" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="F9" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="G9" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="H9" s="4" t="s">
-        <v>33</v>
       </c>
       <c r="I9" s="4"/>
       <c r="J9" s="4"/>
       <c r="K9" s="4"/>
       <c r="L9" s="4"/>
-      <c r="M9" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="N9" s="4"/>
+      <c r="M9" s="4"/>
+      <c r="N9" s="4" t="s">
+        <v>19</v>
+      </c>
       <c r="O9" s="4"/>
       <c r="P9" s="4"/>
       <c r="Q9" s="4"/>
       <c r="R9" s="4"/>
       <c r="S9" s="4"/>
-      <c r="T9" s="3"/>
+      <c r="T9" s="4"/>
       <c r="U9" s="3"/>
       <c r="V9" s="3"/>
       <c r="W9" s="3"/>
@@ -1746,44 +1789,45 @@
       <c r="AF9" s="3"/>
       <c r="AG9" s="3"/>
       <c r="AH9" s="3"/>
-    </row>
-    <row r="10" spans="1:34">
+      <c r="AI9" s="3"/>
+    </row>
+    <row r="10" spans="1:35">
       <c r="A10" s="3"/>
       <c r="B10" s="4" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C10" s="2"/>
       <c r="D10" s="4" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F10" s="4" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="G10" s="4" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="H10" s="4"/>
       <c r="I10" s="4"/>
       <c r="J10" s="4" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="K10" s="4" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="L10" s="4"/>
-      <c r="M10" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="N10" s="4"/>
+      <c r="M10" s="4"/>
+      <c r="N10" s="4" t="s">
+        <v>19</v>
+      </c>
       <c r="O10" s="4"/>
       <c r="P10" s="4"/>
       <c r="Q10" s="4"/>
       <c r="R10" s="4"/>
       <c r="S10" s="4"/>
-      <c r="T10" s="3"/>
+      <c r="T10" s="4"/>
       <c r="U10" s="3"/>
       <c r="V10" s="3"/>
       <c r="W10" s="3"/>
@@ -1798,44 +1842,45 @@
       <c r="AF10" s="3"/>
       <c r="AG10" s="3"/>
       <c r="AH10" s="3"/>
-    </row>
-    <row r="11" spans="1:34">
+      <c r="AI10" s="3"/>
+    </row>
+    <row r="11" spans="1:35">
       <c r="A11" s="3"/>
       <c r="B11" s="4" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C11" s="2"/>
       <c r="D11" s="4" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E11" s="4" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F11" s="4" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="G11" s="4" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="H11" s="4"/>
       <c r="I11" s="4"/>
       <c r="J11" s="4" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="K11" s="4" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="L11" s="4"/>
-      <c r="M11" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="N11" s="4"/>
+      <c r="M11" s="4"/>
+      <c r="N11" s="4" t="s">
+        <v>19</v>
+      </c>
       <c r="O11" s="4"/>
       <c r="P11" s="4"/>
       <c r="Q11" s="4"/>
       <c r="R11" s="4"/>
       <c r="S11" s="4"/>
-      <c r="T11" s="3"/>
+      <c r="T11" s="4"/>
       <c r="U11" s="3"/>
       <c r="V11" s="3"/>
       <c r="W11" s="3"/>
@@ -1850,44 +1895,45 @@
       <c r="AF11" s="3"/>
       <c r="AG11" s="3"/>
       <c r="AH11" s="3"/>
-    </row>
-    <row r="12" spans="1:34">
+      <c r="AI11" s="3"/>
+    </row>
+    <row r="12" spans="1:35">
       <c r="A12" s="3"/>
       <c r="B12" s="4" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C12" s="2"/>
       <c r="D12" s="4" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E12" s="4" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F12" s="4" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="G12" s="4" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="H12" s="4"/>
       <c r="I12" s="4"/>
       <c r="J12" s="4" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="K12" s="4" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="L12" s="4"/>
-      <c r="M12" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="N12" s="4"/>
+      <c r="M12" s="4"/>
+      <c r="N12" s="4" t="s">
+        <v>19</v>
+      </c>
       <c r="O12" s="4"/>
       <c r="P12" s="4"/>
       <c r="Q12" s="4"/>
       <c r="R12" s="4"/>
       <c r="S12" s="4"/>
-      <c r="T12" s="3"/>
+      <c r="T12" s="4"/>
       <c r="U12" s="3"/>
       <c r="V12" s="3"/>
       <c r="W12" s="3"/>
@@ -1902,44 +1948,45 @@
       <c r="AF12" s="3"/>
       <c r="AG12" s="3"/>
       <c r="AH12" s="3"/>
-    </row>
-    <row r="13" spans="1:34">
+      <c r="AI12" s="3"/>
+    </row>
+    <row r="13" spans="1:35">
       <c r="A13" s="3"/>
       <c r="B13" s="4" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C13" s="2"/>
       <c r="D13" s="4" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E13" s="4" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F13" s="4" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="G13" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="H13" s="4" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="I13" s="4" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="J13" s="4"/>
       <c r="K13" s="4"/>
       <c r="L13" s="4"/>
-      <c r="M13" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="N13" s="4"/>
+      <c r="M13" s="4"/>
+      <c r="N13" s="4" t="s">
+        <v>19</v>
+      </c>
       <c r="O13" s="4"/>
       <c r="P13" s="4"/>
       <c r="Q13" s="4"/>
       <c r="R13" s="4"/>
       <c r="S13" s="4"/>
-      <c r="T13" s="3"/>
+      <c r="T13" s="4"/>
       <c r="U13" s="3"/>
       <c r="V13" s="3"/>
       <c r="W13" s="3"/>
@@ -1954,44 +2001,45 @@
       <c r="AF13" s="3"/>
       <c r="AG13" s="3"/>
       <c r="AH13" s="3"/>
-    </row>
-    <row r="14" spans="1:34">
+      <c r="AI13" s="3"/>
+    </row>
+    <row r="14" spans="1:35">
       <c r="A14" s="3"/>
       <c r="B14" s="4" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C14" s="2"/>
       <c r="D14" s="4" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E14" s="4" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F14" s="4" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="G14" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="H14" s="4" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="I14" s="4" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="J14" s="4"/>
       <c r="K14" s="4"/>
       <c r="L14" s="4"/>
-      <c r="M14" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="N14" s="4"/>
+      <c r="M14" s="4"/>
+      <c r="N14" s="4" t="s">
+        <v>19</v>
+      </c>
       <c r="O14" s="4"/>
       <c r="P14" s="4"/>
       <c r="Q14" s="4"/>
       <c r="R14" s="4"/>
       <c r="S14" s="4"/>
-      <c r="T14" s="3"/>
+      <c r="T14" s="4"/>
       <c r="U14" s="3"/>
       <c r="V14" s="3"/>
       <c r="W14" s="3"/>
@@ -2006,44 +2054,45 @@
       <c r="AF14" s="3"/>
       <c r="AG14" s="3"/>
       <c r="AH14" s="3"/>
-    </row>
-    <row r="15" spans="1:34">
+      <c r="AI14" s="3"/>
+    </row>
+    <row r="15" spans="1:35">
       <c r="A15" s="3"/>
       <c r="B15" s="4" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C15" s="2"/>
       <c r="D15" s="4" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E15" s="4" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F15" s="4" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="G15" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="H15" s="4" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="I15" s="4" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="J15" s="4"/>
       <c r="K15" s="4"/>
       <c r="L15" s="4"/>
-      <c r="M15" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="N15" s="4"/>
+      <c r="M15" s="4"/>
+      <c r="N15" s="4" t="s">
+        <v>19</v>
+      </c>
       <c r="O15" s="4"/>
       <c r="P15" s="4"/>
       <c r="Q15" s="4"/>
       <c r="R15" s="4"/>
       <c r="S15" s="4"/>
-      <c r="T15" s="3"/>
+      <c r="T15" s="4"/>
       <c r="U15" s="3"/>
       <c r="V15" s="3"/>
       <c r="W15" s="3"/>
@@ -2058,44 +2107,45 @@
       <c r="AF15" s="3"/>
       <c r="AG15" s="3"/>
       <c r="AH15" s="3"/>
-    </row>
-    <row r="16" spans="1:34">
+      <c r="AI15" s="3"/>
+    </row>
+    <row r="16" spans="1:35">
       <c r="A16" s="3"/>
       <c r="B16" s="4" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C16" s="2"/>
       <c r="D16" s="4" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E16" s="4" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F16" s="4" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="G16" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="H16" s="4" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="I16" s="4" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="J16" s="4"/>
       <c r="K16" s="4"/>
       <c r="L16" s="4"/>
-      <c r="M16" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="N16" s="4"/>
+      <c r="M16" s="4"/>
+      <c r="N16" s="4" t="s">
+        <v>19</v>
+      </c>
       <c r="O16" s="4"/>
       <c r="P16" s="4"/>
       <c r="Q16" s="4"/>
       <c r="R16" s="4"/>
       <c r="S16" s="4"/>
-      <c r="T16" s="3"/>
+      <c r="T16" s="4"/>
       <c r="U16" s="3"/>
       <c r="V16" s="3"/>
       <c r="W16" s="3"/>
@@ -2110,44 +2160,45 @@
       <c r="AF16" s="3"/>
       <c r="AG16" s="3"/>
       <c r="AH16" s="3"/>
-    </row>
-    <row r="17" spans="1:34">
+      <c r="AI16" s="3"/>
+    </row>
+    <row r="17" spans="1:35">
       <c r="A17" s="3"/>
       <c r="B17" s="4" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C17" s="2"/>
       <c r="D17" s="4" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E17" s="4" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F17" s="4" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="G17" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="H17" s="4" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="I17" s="4" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="J17" s="4"/>
       <c r="K17" s="4"/>
       <c r="L17" s="4"/>
-      <c r="M17" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="N17" s="4"/>
+      <c r="M17" s="4"/>
+      <c r="N17" s="4" t="s">
+        <v>19</v>
+      </c>
       <c r="O17" s="4"/>
       <c r="P17" s="4"/>
       <c r="Q17" s="4"/>
       <c r="R17" s="4"/>
       <c r="S17" s="4"/>
-      <c r="T17" s="3"/>
+      <c r="T17" s="4"/>
       <c r="U17" s="3"/>
       <c r="V17" s="3"/>
       <c r="W17" s="3"/>
@@ -2162,42 +2213,43 @@
       <c r="AF17" s="3"/>
       <c r="AG17" s="3"/>
       <c r="AH17" s="3"/>
-    </row>
-    <row r="18" spans="1:34">
+      <c r="AI17" s="3"/>
+    </row>
+    <row r="18" spans="1:35">
       <c r="A18" s="3"/>
       <c r="B18" s="4" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C18" s="2"/>
       <c r="D18" s="4" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E18" s="4" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F18" s="4" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="G18" s="4" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="H18" s="4"/>
       <c r="I18" s="4"/>
       <c r="J18" s="4"/>
       <c r="K18" s="4"/>
       <c r="L18" s="4" t="s">
-        <v>59</v>
-      </c>
-      <c r="M18" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="N18" s="4"/>
+        <v>60</v>
+      </c>
+      <c r="M18" s="4"/>
+      <c r="N18" s="4" t="s">
+        <v>19</v>
+      </c>
       <c r="O18" s="4"/>
       <c r="P18" s="4"/>
       <c r="Q18" s="4"/>
       <c r="R18" s="4"/>
       <c r="S18" s="4"/>
-      <c r="T18" s="3"/>
+      <c r="T18" s="4"/>
       <c r="U18" s="3"/>
       <c r="V18" s="3"/>
       <c r="W18" s="3"/>
@@ -2212,42 +2264,43 @@
       <c r="AF18" s="3"/>
       <c r="AG18" s="3"/>
       <c r="AH18" s="3"/>
-    </row>
-    <row r="19" spans="1:34">
+      <c r="AI18" s="3"/>
+    </row>
+    <row r="19" spans="1:35">
       <c r="A19" s="3"/>
       <c r="B19" s="4" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C19" s="2"/>
       <c r="D19" s="4" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E19" s="4" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F19" s="4" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="G19" s="4" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="H19" s="4"/>
       <c r="I19" s="4"/>
       <c r="J19" s="4"/>
       <c r="K19" s="4"/>
       <c r="L19" s="4" t="s">
-        <v>61</v>
-      </c>
-      <c r="M19" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="N19" s="4"/>
+        <v>62</v>
+      </c>
+      <c r="M19" s="4"/>
+      <c r="N19" s="4" t="s">
+        <v>19</v>
+      </c>
       <c r="O19" s="4"/>
       <c r="P19" s="4"/>
       <c r="Q19" s="4"/>
       <c r="R19" s="4"/>
       <c r="S19" s="4"/>
-      <c r="T19" s="3"/>
+      <c r="T19" s="4"/>
       <c r="U19" s="3"/>
       <c r="V19" s="3"/>
       <c r="W19" s="3"/>
@@ -2262,42 +2315,43 @@
       <c r="AF19" s="3"/>
       <c r="AG19" s="3"/>
       <c r="AH19" s="3"/>
-    </row>
-    <row r="20" spans="1:34">
+      <c r="AI19" s="3"/>
+    </row>
+    <row r="20" spans="1:35">
       <c r="A20" s="3"/>
       <c r="B20" s="4" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C20" s="2"/>
       <c r="D20" s="4" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E20" s="4" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F20" s="4" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="G20" s="4" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="H20" s="4"/>
       <c r="I20" s="4"/>
       <c r="J20" s="4"/>
       <c r="K20" s="4"/>
       <c r="L20" s="4" t="s">
-        <v>63</v>
-      </c>
-      <c r="M20" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="N20" s="4"/>
+        <v>64</v>
+      </c>
+      <c r="M20" s="4"/>
+      <c r="N20" s="4" t="s">
+        <v>19</v>
+      </c>
       <c r="O20" s="4"/>
       <c r="P20" s="4"/>
       <c r="Q20" s="4"/>
       <c r="R20" s="4"/>
       <c r="S20" s="4"/>
-      <c r="T20" s="3"/>
+      <c r="T20" s="4"/>
       <c r="U20" s="3"/>
       <c r="V20" s="3"/>
       <c r="W20" s="3"/>
@@ -2312,42 +2366,43 @@
       <c r="AF20" s="3"/>
       <c r="AG20" s="3"/>
       <c r="AH20" s="3"/>
-    </row>
-    <row r="21" spans="1:34">
+      <c r="AI20" s="3"/>
+    </row>
+    <row r="21" spans="1:35">
       <c r="A21" s="3"/>
       <c r="B21" s="4" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C21" s="2"/>
       <c r="D21" s="4" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E21" s="4" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F21" s="4" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="G21" s="4" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="H21" s="4"/>
       <c r="I21" s="4"/>
       <c r="J21" s="4"/>
       <c r="K21" s="4"/>
       <c r="L21" s="4" t="s">
-        <v>65</v>
-      </c>
-      <c r="M21" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="N21" s="4"/>
+        <v>66</v>
+      </c>
+      <c r="M21" s="4"/>
+      <c r="N21" s="4" t="s">
+        <v>19</v>
+      </c>
       <c r="O21" s="4"/>
       <c r="P21" s="4"/>
       <c r="Q21" s="4"/>
       <c r="R21" s="4"/>
       <c r="S21" s="4"/>
-      <c r="T21" s="3"/>
+      <c r="T21" s="4"/>
       <c r="U21" s="3"/>
       <c r="V21" s="3"/>
       <c r="W21" s="3"/>
@@ -2362,42 +2417,43 @@
       <c r="AF21" s="3"/>
       <c r="AG21" s="3"/>
       <c r="AH21" s="3"/>
-    </row>
-    <row r="22" spans="1:34">
+      <c r="AI21" s="3"/>
+    </row>
+    <row r="22" spans="1:35">
       <c r="A22" s="3"/>
       <c r="B22" s="4" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C22" s="2"/>
       <c r="D22" s="4" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E22" s="4" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F22" s="4" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="G22" s="4" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="H22" s="4"/>
       <c r="I22" s="4"/>
       <c r="J22" s="4"/>
       <c r="K22" s="4"/>
       <c r="L22" s="4" t="s">
-        <v>67</v>
-      </c>
-      <c r="M22" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="N22" s="4"/>
+        <v>68</v>
+      </c>
+      <c r="M22" s="4"/>
+      <c r="N22" s="4" t="s">
+        <v>19</v>
+      </c>
       <c r="O22" s="4"/>
       <c r="P22" s="4"/>
       <c r="Q22" s="4"/>
       <c r="R22" s="4"/>
       <c r="S22" s="4"/>
-      <c r="T22" s="3"/>
+      <c r="T22" s="4"/>
       <c r="U22" s="3"/>
       <c r="V22" s="3"/>
       <c r="W22" s="3"/>
@@ -2412,42 +2468,43 @@
       <c r="AF22" s="3"/>
       <c r="AG22" s="3"/>
       <c r="AH22" s="3"/>
-    </row>
-    <row r="23" spans="1:34">
+      <c r="AI22" s="3"/>
+    </row>
+    <row r="23" spans="1:35">
       <c r="A23" s="3"/>
       <c r="B23" s="4" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="C23" s="2"/>
       <c r="D23" s="4" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E23" s="4" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F23" s="4" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="G23" s="4" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="H23" s="4"/>
       <c r="I23" s="4"/>
       <c r="J23" s="4"/>
       <c r="K23" s="4"/>
       <c r="L23" s="4" t="s">
-        <v>69</v>
-      </c>
-      <c r="M23" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="N23" s="4"/>
+        <v>70</v>
+      </c>
+      <c r="M23" s="4"/>
+      <c r="N23" s="4" t="s">
+        <v>19</v>
+      </c>
       <c r="O23" s="4"/>
       <c r="P23" s="4"/>
       <c r="Q23" s="4"/>
       <c r="R23" s="4"/>
       <c r="S23" s="4"/>
-      <c r="T23" s="3"/>
+      <c r="T23" s="4"/>
       <c r="U23" s="3"/>
       <c r="V23" s="3"/>
       <c r="W23" s="3"/>
@@ -2462,42 +2519,43 @@
       <c r="AF23" s="3"/>
       <c r="AG23" s="3"/>
       <c r="AH23" s="3"/>
-    </row>
-    <row r="24" spans="1:34">
+      <c r="AI23" s="3"/>
+    </row>
+    <row r="24" spans="1:35">
       <c r="A24" s="3"/>
       <c r="B24" s="4" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C24" s="2"/>
       <c r="D24" s="4" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E24" s="4" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F24" s="4" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="G24" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="H24" s="4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="I24" s="4"/>
       <c r="J24" s="4"/>
       <c r="K24" s="4"/>
       <c r="L24" s="4"/>
-      <c r="M24" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="N24" s="4"/>
+      <c r="M24" s="4"/>
+      <c r="N24" s="4" t="s">
+        <v>19</v>
+      </c>
       <c r="O24" s="4"/>
       <c r="P24" s="4"/>
       <c r="Q24" s="4"/>
       <c r="R24" s="4"/>
       <c r="S24" s="4"/>
-      <c r="T24" s="3"/>
+      <c r="T24" s="4"/>
       <c r="U24" s="3"/>
       <c r="V24" s="3"/>
       <c r="W24" s="3"/>
@@ -2512,42 +2570,43 @@
       <c r="AF24" s="3"/>
       <c r="AG24" s="3"/>
       <c r="AH24" s="3"/>
-    </row>
-    <row r="25" spans="1:34">
+      <c r="AI24" s="3"/>
+    </row>
+    <row r="25" spans="1:35">
       <c r="A25" s="3"/>
       <c r="B25" s="4" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C25" s="2"/>
       <c r="D25" s="4" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E25" s="4" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F25" s="4" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="G25" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="H25" s="4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="I25" s="4"/>
       <c r="J25" s="4"/>
       <c r="K25" s="4"/>
       <c r="L25" s="4"/>
-      <c r="M25" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="N25" s="4"/>
+      <c r="M25" s="4"/>
+      <c r="N25" s="4" t="s">
+        <v>19</v>
+      </c>
       <c r="O25" s="4"/>
       <c r="P25" s="4"/>
       <c r="Q25" s="4"/>
       <c r="R25" s="4"/>
       <c r="S25" s="4"/>
-      <c r="T25" s="3"/>
+      <c r="T25" s="4"/>
       <c r="U25" s="3"/>
       <c r="V25" s="3"/>
       <c r="W25" s="3"/>
@@ -2562,40 +2621,41 @@
       <c r="AF25" s="3"/>
       <c r="AG25" s="3"/>
       <c r="AH25" s="3"/>
-    </row>
-    <row r="26" spans="1:34">
+      <c r="AI25" s="3"/>
+    </row>
+    <row r="26" spans="1:35">
       <c r="A26" s="3"/>
       <c r="B26" s="4" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="C26" s="2"/>
       <c r="D26" s="4" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E26" s="4" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F26" s="4" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="G26" s="4"/>
       <c r="H26" s="4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="I26" s="4"/>
       <c r="J26" s="4"/>
       <c r="K26" s="4"/>
       <c r="L26" s="4"/>
-      <c r="M26" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="N26" s="4"/>
+      <c r="M26" s="4"/>
+      <c r="N26" s="4" t="s">
+        <v>19</v>
+      </c>
       <c r="O26" s="4"/>
       <c r="P26" s="4"/>
       <c r="Q26" s="4"/>
       <c r="R26" s="4"/>
       <c r="S26" s="4"/>
-      <c r="T26" s="3"/>
+      <c r="T26" s="4"/>
       <c r="U26" s="3"/>
       <c r="V26" s="3"/>
       <c r="W26" s="3"/>
@@ -2610,40 +2670,41 @@
       <c r="AF26" s="3"/>
       <c r="AG26" s="3"/>
       <c r="AH26" s="3"/>
-    </row>
-    <row r="27" spans="1:34">
+      <c r="AI26" s="3"/>
+    </row>
+    <row r="27" spans="1:35">
       <c r="A27" s="3"/>
       <c r="B27" s="4" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C27" s="2"/>
       <c r="D27" s="4" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E27" s="4" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F27" s="4" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="G27" s="4"/>
       <c r="H27" s="4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="I27" s="4"/>
       <c r="J27" s="4"/>
       <c r="K27" s="4"/>
       <c r="L27" s="4"/>
-      <c r="M27" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="N27" s="4"/>
+      <c r="M27" s="4"/>
+      <c r="N27" s="4" t="s">
+        <v>19</v>
+      </c>
       <c r="O27" s="4"/>
       <c r="P27" s="4"/>
       <c r="Q27" s="4"/>
       <c r="R27" s="4"/>
       <c r="S27" s="4"/>
-      <c r="T27" s="3"/>
+      <c r="T27" s="4"/>
       <c r="U27" s="3"/>
       <c r="V27" s="3"/>
       <c r="W27" s="3"/>
@@ -2658,42 +2719,43 @@
       <c r="AF27" s="3"/>
       <c r="AG27" s="3"/>
       <c r="AH27" s="3"/>
-    </row>
-    <row r="28" spans="1:34">
+      <c r="AI27" s="3"/>
+    </row>
+    <row r="28" spans="1:35">
       <c r="A28" s="3"/>
       <c r="B28" s="4" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="C28" s="2"/>
       <c r="D28" s="4" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E28" s="4" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F28" s="4" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="G28" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="H28" s="4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="I28" s="4"/>
       <c r="J28" s="4"/>
       <c r="K28" s="4"/>
       <c r="L28" s="4"/>
-      <c r="M28" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="N28" s="4"/>
+      <c r="M28" s="4"/>
+      <c r="N28" s="4" t="s">
+        <v>19</v>
+      </c>
       <c r="O28" s="4"/>
       <c r="P28" s="4"/>
       <c r="Q28" s="4"/>
       <c r="R28" s="4"/>
       <c r="S28" s="4"/>
-      <c r="T28" s="3"/>
+      <c r="T28" s="4"/>
       <c r="U28" s="3"/>
       <c r="V28" s="3"/>
       <c r="W28" s="3"/>
@@ -2708,40 +2770,41 @@
       <c r="AF28" s="3"/>
       <c r="AG28" s="3"/>
       <c r="AH28" s="3"/>
-    </row>
-    <row r="29" spans="1:34">
+      <c r="AI28" s="3"/>
+    </row>
+    <row r="29" spans="1:35">
       <c r="A29" s="3"/>
       <c r="B29" s="4" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C29" s="2"/>
       <c r="D29" s="4" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E29" s="4" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F29" s="4" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="G29" s="4"/>
       <c r="H29" s="4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="I29" s="4"/>
       <c r="J29" s="4"/>
       <c r="K29" s="4"/>
       <c r="L29" s="4"/>
-      <c r="M29" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="N29" s="4"/>
+      <c r="M29" s="4"/>
+      <c r="N29" s="4" t="s">
+        <v>19</v>
+      </c>
       <c r="O29" s="4"/>
       <c r="P29" s="4"/>
       <c r="Q29" s="4"/>
       <c r="R29" s="4"/>
       <c r="S29" s="4"/>
-      <c r="T29" s="3"/>
+      <c r="T29" s="4"/>
       <c r="U29" s="3"/>
       <c r="V29" s="3"/>
       <c r="W29" s="3"/>
@@ -2756,42 +2819,43 @@
       <c r="AF29" s="3"/>
       <c r="AG29" s="3"/>
       <c r="AH29" s="3"/>
-    </row>
-    <row r="30" spans="1:34">
+      <c r="AI29" s="3"/>
+    </row>
+    <row r="30" spans="1:35">
       <c r="A30" s="3"/>
       <c r="B30" s="4" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="C30" s="2"/>
       <c r="D30" s="4" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E30" s="4" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F30" s="4" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="G30" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="H30" s="4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="I30" s="4"/>
       <c r="J30" s="4"/>
       <c r="K30" s="4"/>
       <c r="L30" s="4"/>
-      <c r="M30" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="N30" s="4"/>
+      <c r="M30" s="4"/>
+      <c r="N30" s="4" t="s">
+        <v>19</v>
+      </c>
       <c r="O30" s="4"/>
       <c r="P30" s="4"/>
       <c r="Q30" s="4"/>
       <c r="R30" s="4"/>
       <c r="S30" s="4"/>
-      <c r="T30" s="3"/>
+      <c r="T30" s="4"/>
       <c r="U30" s="3"/>
       <c r="V30" s="3"/>
       <c r="W30" s="3"/>
@@ -2806,40 +2870,41 @@
       <c r="AF30" s="3"/>
       <c r="AG30" s="3"/>
       <c r="AH30" s="3"/>
-    </row>
-    <row r="31" spans="1:34">
+      <c r="AI30" s="3"/>
+    </row>
+    <row r="31" spans="1:35">
       <c r="A31" s="3"/>
       <c r="B31" s="4" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="C31" s="2"/>
       <c r="D31" s="4" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E31" s="4" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F31" s="4" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="G31" s="4"/>
       <c r="H31" s="4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="I31" s="4"/>
       <c r="J31" s="4"/>
       <c r="K31" s="4"/>
       <c r="L31" s="4"/>
-      <c r="M31" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="N31" s="4"/>
+      <c r="M31" s="4"/>
+      <c r="N31" s="4" t="s">
+        <v>19</v>
+      </c>
       <c r="O31" s="4"/>
       <c r="P31" s="4"/>
       <c r="Q31" s="4"/>
       <c r="R31" s="4"/>
       <c r="S31" s="4"/>
-      <c r="T31" s="3"/>
+      <c r="T31" s="4"/>
       <c r="U31" s="3"/>
       <c r="V31" s="3"/>
       <c r="W31" s="3"/>
@@ -2854,40 +2919,41 @@
       <c r="AF31" s="3"/>
       <c r="AG31" s="3"/>
       <c r="AH31" s="3"/>
-    </row>
-    <row r="32" spans="1:34">
+      <c r="AI31" s="3"/>
+    </row>
+    <row r="32" spans="1:35">
       <c r="A32" s="3"/>
       <c r="B32" s="4" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="C32" s="2"/>
       <c r="D32" s="4" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E32" s="4" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F32" s="4" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="G32" s="4"/>
       <c r="H32" s="4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="I32" s="4"/>
       <c r="J32" s="4"/>
       <c r="K32" s="4"/>
       <c r="L32" s="4"/>
-      <c r="M32" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="N32" s="4"/>
+      <c r="M32" s="4"/>
+      <c r="N32" s="4" t="s">
+        <v>19</v>
+      </c>
       <c r="O32" s="4"/>
       <c r="P32" s="4"/>
       <c r="Q32" s="4"/>
       <c r="R32" s="4"/>
       <c r="S32" s="4"/>
-      <c r="T32" s="3"/>
+      <c r="T32" s="4"/>
       <c r="U32" s="3"/>
       <c r="V32" s="3"/>
       <c r="W32" s="3"/>
@@ -2902,40 +2968,41 @@
       <c r="AF32" s="3"/>
       <c r="AG32" s="3"/>
       <c r="AH32" s="3"/>
-    </row>
-    <row r="33" spans="1:34">
+      <c r="AI32" s="3"/>
+    </row>
+    <row r="33" spans="1:35">
       <c r="A33" s="3"/>
       <c r="B33" s="4" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="C33" s="2"/>
       <c r="D33" s="4" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E33" s="4" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F33" s="4" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="G33" s="4"/>
       <c r="H33" s="4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="I33" s="4"/>
       <c r="J33" s="4"/>
       <c r="K33" s="4"/>
       <c r="L33" s="4"/>
-      <c r="M33" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="N33" s="4"/>
+      <c r="M33" s="4"/>
+      <c r="N33" s="4" t="s">
+        <v>19</v>
+      </c>
       <c r="O33" s="4"/>
       <c r="P33" s="4"/>
       <c r="Q33" s="4"/>
       <c r="R33" s="4"/>
       <c r="S33" s="4"/>
-      <c r="T33" s="3"/>
+      <c r="T33" s="4"/>
       <c r="U33" s="3"/>
       <c r="V33" s="3"/>
       <c r="W33" s="3"/>
@@ -2950,40 +3017,41 @@
       <c r="AF33" s="3"/>
       <c r="AG33" s="3"/>
       <c r="AH33" s="3"/>
-    </row>
-    <row r="34" spans="1:34">
+      <c r="AI33" s="3"/>
+    </row>
+    <row r="34" spans="1:35">
       <c r="A34" s="3"/>
       <c r="B34" s="4" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="C34" s="2"/>
       <c r="D34" s="4" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E34" s="4" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F34" s="4" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="G34" s="4"/>
       <c r="H34" s="4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="I34" s="4"/>
       <c r="J34" s="4"/>
       <c r="K34" s="4"/>
       <c r="L34" s="4"/>
-      <c r="M34" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="N34" s="4"/>
+      <c r="M34" s="4"/>
+      <c r="N34" s="4" t="s">
+        <v>19</v>
+      </c>
       <c r="O34" s="4"/>
       <c r="P34" s="4"/>
       <c r="Q34" s="4"/>
       <c r="R34" s="4"/>
       <c r="S34" s="4"/>
-      <c r="T34" s="3"/>
+      <c r="T34" s="4"/>
       <c r="U34" s="3"/>
       <c r="V34" s="3"/>
       <c r="W34" s="3"/>
@@ -2998,40 +3066,41 @@
       <c r="AF34" s="3"/>
       <c r="AG34" s="3"/>
       <c r="AH34" s="3"/>
-    </row>
-    <row r="35" spans="1:34">
+      <c r="AI34" s="3"/>
+    </row>
+    <row r="35" spans="1:35">
       <c r="A35" s="3"/>
       <c r="B35" s="4" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C35" s="2"/>
       <c r="D35" s="4" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E35" s="4" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F35" s="4" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="G35" s="4"/>
       <c r="H35" s="4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="I35" s="4"/>
       <c r="J35" s="4"/>
       <c r="K35" s="4"/>
       <c r="L35" s="4"/>
-      <c r="M35" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="N35" s="4"/>
+      <c r="M35" s="4"/>
+      <c r="N35" s="4" t="s">
+        <v>19</v>
+      </c>
       <c r="O35" s="4"/>
       <c r="P35" s="4"/>
       <c r="Q35" s="4"/>
       <c r="R35" s="4"/>
       <c r="S35" s="4"/>
-      <c r="T35" s="3"/>
+      <c r="T35" s="4"/>
       <c r="U35" s="3"/>
       <c r="V35" s="3"/>
       <c r="W35" s="3"/>
@@ -3046,40 +3115,41 @@
       <c r="AF35" s="3"/>
       <c r="AG35" s="3"/>
       <c r="AH35" s="3"/>
-    </row>
-    <row r="36" spans="1:34">
+      <c r="AI35" s="3"/>
+    </row>
+    <row r="36" spans="1:35">
       <c r="A36" s="3"/>
       <c r="B36" s="4" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C36" s="2"/>
       <c r="D36" s="4" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E36" s="4" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F36" s="4" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="G36" s="4"/>
       <c r="H36" s="4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="I36" s="4"/>
       <c r="J36" s="4"/>
       <c r="K36" s="4"/>
       <c r="L36" s="4"/>
-      <c r="M36" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="N36" s="4"/>
+      <c r="M36" s="4"/>
+      <c r="N36" s="4" t="s">
+        <v>19</v>
+      </c>
       <c r="O36" s="4"/>
       <c r="P36" s="4"/>
       <c r="Q36" s="4"/>
       <c r="R36" s="4"/>
       <c r="S36" s="4"/>
-      <c r="T36" s="3"/>
+      <c r="T36" s="4"/>
       <c r="U36" s="3"/>
       <c r="V36" s="3"/>
       <c r="W36" s="3"/>
@@ -3094,50 +3164,46 @@
       <c r="AF36" s="3"/>
       <c r="AG36" s="3"/>
       <c r="AH36" s="3"/>
-    </row>
-    <row r="37" spans="2:34">
-      <c r="B37" s="2" t="s">
-        <v>89</v>
+      <c r="AI36" s="3"/>
+    </row>
+    <row r="37" spans="1:35">
+      <c r="A37" s="3"/>
+      <c r="B37" s="4" t="s">
+        <v>90</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>90</v>
-      </c>
-      <c r="D37" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="E37" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="F37" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="G37" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="D37" s="4" t="s">
         <v>24</v>
       </c>
+      <c r="E37" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="F37" s="4"/>
+      <c r="G37" s="4"/>
       <c r="H37" s="4" t="s">
-        <v>91</v>
-      </c>
-      <c r="I37" s="4" t="s">
         <v>92</v>
       </c>
-      <c r="J37" s="4" t="s">
+      <c r="I37" s="4"/>
+      <c r="J37" s="4"/>
+      <c r="K37" s="4"/>
+      <c r="L37" s="4"/>
+      <c r="M37" s="4" t="s">
         <v>93</v>
       </c>
-      <c r="K37" s="2" t="s">
-        <v>94</v>
-      </c>
-      <c r="L37" s="2" t="s">
-        <v>95</v>
-      </c>
-      <c r="M37" s="2" t="s">
-        <v>96</v>
-      </c>
-      <c r="N37" s="2"/>
-      <c r="O37" s="2"/>
-      <c r="P37" s="2"/>
-      <c r="Q37" s="2"/>
-      <c r="R37" s="2"/>
-      <c r="S37" s="2"/>
+      <c r="N37" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="O37" s="4"/>
+      <c r="P37" s="4"/>
+      <c r="Q37" s="4"/>
+      <c r="R37" s="4"/>
+      <c r="S37" s="4"/>
+      <c r="T37" s="4"/>
+      <c r="U37" s="3"/>
+      <c r="V37" s="3"/>
+      <c r="W37" s="3"/>
       <c r="X37" s="3"/>
       <c r="Y37" s="3"/>
       <c r="Z37" s="3"/>
@@ -3149,28 +3215,43 @@
       <c r="AF37" s="3"/>
       <c r="AG37" s="3"/>
       <c r="AH37" s="3"/>
-    </row>
-    <row r="38" spans="1:34">
+      <c r="AI37" s="3"/>
+    </row>
+    <row r="38" spans="1:35">
       <c r="A38" s="3"/>
-      <c r="B38" s="4"/>
-      <c r="C38" s="4"/>
-      <c r="D38" s="4"/>
-      <c r="E38" s="4"/>
+      <c r="B38" s="4" t="s">
+        <v>94</v>
+      </c>
+      <c r="C38" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="D38" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="E38" s="4" t="s">
+        <v>76</v>
+      </c>
       <c r="F38" s="4"/>
       <c r="G38" s="4"/>
-      <c r="H38" s="4"/>
+      <c r="H38" s="4" t="s">
+        <v>92</v>
+      </c>
       <c r="I38" s="4"/>
       <c r="J38" s="4"/>
       <c r="K38" s="4"/>
       <c r="L38" s="4"/>
-      <c r="M38" s="4"/>
-      <c r="N38" s="4"/>
+      <c r="M38" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="N38" s="4" t="s">
+        <v>19</v>
+      </c>
       <c r="O38" s="4"/>
       <c r="P38" s="4"/>
       <c r="Q38" s="4"/>
       <c r="R38" s="4"/>
       <c r="S38" s="4"/>
-      <c r="T38" s="3"/>
+      <c r="T38" s="4"/>
       <c r="U38" s="3"/>
       <c r="V38" s="3"/>
       <c r="W38" s="3"/>
@@ -3185,28 +3266,39 @@
       <c r="AF38" s="3"/>
       <c r="AG38" s="3"/>
       <c r="AH38" s="3"/>
-    </row>
-    <row r="39" s="1" customFormat="1" spans="1:34">
+      <c r="AI38" s="3"/>
+    </row>
+    <row r="39" spans="1:35">
       <c r="A39" s="3"/>
-      <c r="B39" s="4"/>
-      <c r="C39" s="4"/>
+      <c r="B39" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="C39" s="2" t="s">
+        <v>97</v>
+      </c>
       <c r="D39" s="4"/>
       <c r="E39" s="4"/>
       <c r="F39" s="4"/>
       <c r="G39" s="4"/>
-      <c r="H39" s="4"/>
+      <c r="H39" s="4" t="s">
+        <v>92</v>
+      </c>
       <c r="I39" s="4"/>
       <c r="J39" s="4"/>
       <c r="K39" s="4"/>
       <c r="L39" s="4"/>
-      <c r="M39" s="4"/>
-      <c r="N39" s="4"/>
+      <c r="M39" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="N39" s="4" t="s">
+        <v>19</v>
+      </c>
       <c r="O39" s="4"/>
       <c r="P39" s="4"/>
       <c r="Q39" s="4"/>
       <c r="R39" s="4"/>
       <c r="S39" s="4"/>
-      <c r="T39" s="3"/>
+      <c r="T39" s="4"/>
       <c r="U39" s="3"/>
       <c r="V39" s="3"/>
       <c r="W39" s="3"/>
@@ -3221,28 +3313,39 @@
       <c r="AF39" s="3"/>
       <c r="AG39" s="3"/>
       <c r="AH39" s="3"/>
-    </row>
-    <row r="40" s="1" customFormat="1" spans="1:34">
+      <c r="AI39" s="3"/>
+    </row>
+    <row r="40" spans="1:35">
       <c r="A40" s="3"/>
-      <c r="B40" s="4"/>
-      <c r="C40" s="4"/>
+      <c r="B40" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="C40" s="2" t="s">
+        <v>97</v>
+      </c>
       <c r="D40" s="4"/>
       <c r="E40" s="4"/>
       <c r="F40" s="4"/>
       <c r="G40" s="4"/>
-      <c r="H40" s="4"/>
+      <c r="H40" s="4" t="s">
+        <v>92</v>
+      </c>
       <c r="I40" s="4"/>
       <c r="J40" s="4"/>
       <c r="K40" s="4"/>
       <c r="L40" s="4"/>
-      <c r="M40" s="4"/>
-      <c r="N40" s="4"/>
+      <c r="M40" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="N40" s="4" t="s">
+        <v>19</v>
+      </c>
       <c r="O40" s="4"/>
       <c r="P40" s="4"/>
       <c r="Q40" s="4"/>
       <c r="R40" s="4"/>
       <c r="S40" s="4"/>
-      <c r="T40" s="3"/>
+      <c r="T40" s="4"/>
       <c r="U40" s="3"/>
       <c r="V40" s="3"/>
       <c r="W40" s="3"/>
@@ -3257,32 +3360,54 @@
       <c r="AF40" s="3"/>
       <c r="AG40" s="3"/>
       <c r="AH40" s="3"/>
-    </row>
-    <row r="41" spans="1:34">
-      <c r="A41" s="3"/>
-      <c r="B41" s="4"/>
-      <c r="C41" s="4"/>
-      <c r="D41" s="4"/>
-      <c r="E41" s="4"/>
-      <c r="F41" s="4"/>
-      <c r="G41" s="4"/>
-      <c r="H41" s="4"/>
-      <c r="I41" s="4"/>
-      <c r="J41" s="4"/>
-      <c r="K41" s="4"/>
-      <c r="L41" s="4"/>
-      <c r="M41" s="4"/>
-      <c r="N41" s="4"/>
-      <c r="O41" s="4"/>
-      <c r="P41" s="4"/>
-      <c r="Q41" s="4"/>
-      <c r="R41" s="4"/>
-      <c r="S41" s="4"/>
-      <c r="T41" s="3"/>
-      <c r="U41" s="3"/>
-      <c r="V41" s="3"/>
-      <c r="W41" s="3"/>
-      <c r="X41" s="3"/>
+      <c r="AI40" s="3"/>
+    </row>
+    <row r="41" spans="2:35">
+      <c r="B41" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="C41" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="D41" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="E41" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="F41" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="G41" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="H41" s="4" t="s">
+        <v>101</v>
+      </c>
+      <c r="I41" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="J41" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="K41" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="L41" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="M41" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="N41" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="O41" s="2"/>
+      <c r="P41" s="2"/>
+      <c r="Q41" s="2"/>
+      <c r="R41" s="2"/>
+      <c r="S41" s="2"/>
+      <c r="T41" s="2"/>
       <c r="Y41" s="3"/>
       <c r="Z41" s="3"/>
       <c r="AA41" s="3"/>
@@ -3293,8 +3418,9 @@
       <c r="AF41" s="3"/>
       <c r="AG41" s="3"/>
       <c r="AH41" s="3"/>
-    </row>
-    <row r="42" spans="1:34">
+      <c r="AI41" s="3"/>
+    </row>
+    <row r="42" spans="1:35">
       <c r="A42" s="3"/>
       <c r="B42" s="4"/>
       <c r="C42" s="4"/>
@@ -3314,7 +3440,7 @@
       <c r="Q42" s="4"/>
       <c r="R42" s="4"/>
       <c r="S42" s="4"/>
-      <c r="T42" s="3"/>
+      <c r="T42" s="4"/>
       <c r="U42" s="3"/>
       <c r="V42" s="3"/>
       <c r="W42" s="3"/>
@@ -3329,8 +3455,9 @@
       <c r="AF42" s="3"/>
       <c r="AG42" s="3"/>
       <c r="AH42" s="3"/>
-    </row>
-    <row r="43" spans="1:34">
+      <c r="AI42" s="3"/>
+    </row>
+    <row r="43" s="1" customFormat="1" spans="1:35">
       <c r="A43" s="3"/>
       <c r="B43" s="4"/>
       <c r="C43" s="4"/>
@@ -3350,7 +3477,7 @@
       <c r="Q43" s="4"/>
       <c r="R43" s="4"/>
       <c r="S43" s="4"/>
-      <c r="T43" s="3"/>
+      <c r="T43" s="4"/>
       <c r="U43" s="3"/>
       <c r="V43" s="3"/>
       <c r="W43" s="3"/>
@@ -3365,8 +3492,9 @@
       <c r="AF43" s="3"/>
       <c r="AG43" s="3"/>
       <c r="AH43" s="3"/>
-    </row>
-    <row r="44" spans="1:34">
+      <c r="AI43" s="3"/>
+    </row>
+    <row r="44" s="1" customFormat="1" spans="1:35">
       <c r="A44" s="3"/>
       <c r="B44" s="4"/>
       <c r="C44" s="4"/>
@@ -3386,7 +3514,7 @@
       <c r="Q44" s="4"/>
       <c r="R44" s="4"/>
       <c r="S44" s="4"/>
-      <c r="T44" s="3"/>
+      <c r="T44" s="4"/>
       <c r="U44" s="3"/>
       <c r="V44" s="3"/>
       <c r="W44" s="3"/>
@@ -3401,8 +3529,9 @@
       <c r="AF44" s="3"/>
       <c r="AG44" s="3"/>
       <c r="AH44" s="3"/>
-    </row>
-    <row r="45" spans="1:34">
+      <c r="AI44" s="3"/>
+    </row>
+    <row r="45" spans="1:35">
       <c r="A45" s="3"/>
       <c r="B45" s="4"/>
       <c r="C45" s="4"/>
@@ -3422,7 +3551,7 @@
       <c r="Q45" s="4"/>
       <c r="R45" s="4"/>
       <c r="S45" s="4"/>
-      <c r="T45" s="3"/>
+      <c r="T45" s="4"/>
       <c r="U45" s="3"/>
       <c r="V45" s="3"/>
       <c r="W45" s="3"/>
@@ -3437,8 +3566,9 @@
       <c r="AF45" s="3"/>
       <c r="AG45" s="3"/>
       <c r="AH45" s="3"/>
-    </row>
-    <row r="46" spans="1:34">
+      <c r="AI45" s="3"/>
+    </row>
+    <row r="46" spans="1:35">
       <c r="A46" s="3"/>
       <c r="B46" s="4"/>
       <c r="C46" s="4"/>
@@ -3458,7 +3588,7 @@
       <c r="Q46" s="4"/>
       <c r="R46" s="4"/>
       <c r="S46" s="4"/>
-      <c r="T46" s="3"/>
+      <c r="T46" s="4"/>
       <c r="U46" s="3"/>
       <c r="V46" s="3"/>
       <c r="W46" s="3"/>
@@ -3473,8 +3603,9 @@
       <c r="AF46" s="3"/>
       <c r="AG46" s="3"/>
       <c r="AH46" s="3"/>
-    </row>
-    <row r="47" spans="1:34">
+      <c r="AI46" s="3"/>
+    </row>
+    <row r="47" spans="1:35">
       <c r="A47" s="3"/>
       <c r="B47" s="4"/>
       <c r="C47" s="4"/>
@@ -3494,7 +3625,7 @@
       <c r="Q47" s="4"/>
       <c r="R47" s="4"/>
       <c r="S47" s="4"/>
-      <c r="T47" s="3"/>
+      <c r="T47" s="4"/>
       <c r="U47" s="3"/>
       <c r="V47" s="3"/>
       <c r="W47" s="3"/>
@@ -3509,8 +3640,9 @@
       <c r="AF47" s="3"/>
       <c r="AG47" s="3"/>
       <c r="AH47" s="3"/>
-    </row>
-    <row r="48" spans="1:34">
+      <c r="AI47" s="3"/>
+    </row>
+    <row r="48" spans="1:35">
       <c r="A48" s="3"/>
       <c r="B48" s="4"/>
       <c r="C48" s="4"/>
@@ -3530,7 +3662,7 @@
       <c r="Q48" s="4"/>
       <c r="R48" s="4"/>
       <c r="S48" s="4"/>
-      <c r="T48" s="3"/>
+      <c r="T48" s="4"/>
       <c r="U48" s="3"/>
       <c r="V48" s="3"/>
       <c r="W48" s="3"/>
@@ -3545,8 +3677,9 @@
       <c r="AF48" s="3"/>
       <c r="AG48" s="3"/>
       <c r="AH48" s="3"/>
-    </row>
-    <row r="49" spans="1:34">
+      <c r="AI48" s="3"/>
+    </row>
+    <row r="49" spans="1:35">
       <c r="A49" s="3"/>
       <c r="B49" s="4"/>
       <c r="C49" s="4"/>
@@ -3566,7 +3699,7 @@
       <c r="Q49" s="4"/>
       <c r="R49" s="4"/>
       <c r="S49" s="4"/>
-      <c r="T49" s="3"/>
+      <c r="T49" s="4"/>
       <c r="U49" s="3"/>
       <c r="V49" s="3"/>
       <c r="W49" s="3"/>
@@ -3581,8 +3714,9 @@
       <c r="AF49" s="3"/>
       <c r="AG49" s="3"/>
       <c r="AH49" s="3"/>
-    </row>
-    <row r="50" spans="1:34">
+      <c r="AI49" s="3"/>
+    </row>
+    <row r="50" spans="1:35">
       <c r="A50" s="3"/>
       <c r="B50" s="4"/>
       <c r="C50" s="4"/>
@@ -3602,7 +3736,7 @@
       <c r="Q50" s="4"/>
       <c r="R50" s="4"/>
       <c r="S50" s="4"/>
-      <c r="T50" s="3"/>
+      <c r="T50" s="4"/>
       <c r="U50" s="3"/>
       <c r="V50" s="3"/>
       <c r="W50" s="3"/>
@@ -3617,8 +3751,9 @@
       <c r="AF50" s="3"/>
       <c r="AG50" s="3"/>
       <c r="AH50" s="3"/>
-    </row>
-    <row r="51" spans="1:34">
+      <c r="AI50" s="3"/>
+    </row>
+    <row r="51" spans="1:35">
       <c r="A51" s="3"/>
       <c r="B51" s="4"/>
       <c r="C51" s="4"/>
@@ -3638,7 +3773,7 @@
       <c r="Q51" s="4"/>
       <c r="R51" s="4"/>
       <c r="S51" s="4"/>
-      <c r="T51" s="3"/>
+      <c r="T51" s="4"/>
       <c r="U51" s="3"/>
       <c r="V51" s="3"/>
       <c r="W51" s="3"/>
@@ -3653,8 +3788,9 @@
       <c r="AF51" s="3"/>
       <c r="AG51" s="3"/>
       <c r="AH51" s="3"/>
-    </row>
-    <row r="52" spans="1:34">
+      <c r="AI51" s="3"/>
+    </row>
+    <row r="52" spans="1:35">
       <c r="A52" s="3"/>
       <c r="B52" s="4"/>
       <c r="C52" s="4"/>
@@ -3674,7 +3810,7 @@
       <c r="Q52" s="4"/>
       <c r="R52" s="4"/>
       <c r="S52" s="4"/>
-      <c r="T52" s="3"/>
+      <c r="T52" s="4"/>
       <c r="U52" s="3"/>
       <c r="V52" s="3"/>
       <c r="W52" s="3"/>
@@ -3689,8 +3825,9 @@
       <c r="AF52" s="3"/>
       <c r="AG52" s="3"/>
       <c r="AH52" s="3"/>
-    </row>
-    <row r="53" spans="1:34">
+      <c r="AI52" s="3"/>
+    </row>
+    <row r="53" spans="1:35">
       <c r="A53" s="3"/>
       <c r="B53" s="4"/>
       <c r="C53" s="4"/>
@@ -3710,7 +3847,7 @@
       <c r="Q53" s="4"/>
       <c r="R53" s="4"/>
       <c r="S53" s="4"/>
-      <c r="T53" s="3"/>
+      <c r="T53" s="4"/>
       <c r="U53" s="3"/>
       <c r="V53" s="3"/>
       <c r="W53" s="3"/>
@@ -3725,8 +3862,9 @@
       <c r="AF53" s="3"/>
       <c r="AG53" s="3"/>
       <c r="AH53" s="3"/>
-    </row>
-    <row r="54" spans="1:34">
+      <c r="AI53" s="3"/>
+    </row>
+    <row r="54" spans="1:35">
       <c r="A54" s="3"/>
       <c r="B54" s="4"/>
       <c r="C54" s="4"/>
@@ -3746,7 +3884,7 @@
       <c r="Q54" s="4"/>
       <c r="R54" s="4"/>
       <c r="S54" s="4"/>
-      <c r="T54" s="3"/>
+      <c r="T54" s="4"/>
       <c r="U54" s="3"/>
       <c r="V54" s="3"/>
       <c r="W54" s="3"/>
@@ -3761,8 +3899,9 @@
       <c r="AF54" s="3"/>
       <c r="AG54" s="3"/>
       <c r="AH54" s="3"/>
-    </row>
-    <row r="55" spans="1:34">
+      <c r="AI54" s="3"/>
+    </row>
+    <row r="55" spans="1:35">
       <c r="A55" s="3"/>
       <c r="B55" s="4"/>
       <c r="C55" s="4"/>
@@ -3782,7 +3921,7 @@
       <c r="Q55" s="4"/>
       <c r="R55" s="4"/>
       <c r="S55" s="4"/>
-      <c r="T55" s="3"/>
+      <c r="T55" s="4"/>
       <c r="U55" s="3"/>
       <c r="V55" s="3"/>
       <c r="W55" s="3"/>
@@ -3797,13 +3936,14 @@
       <c r="AF55" s="3"/>
       <c r="AG55" s="3"/>
       <c r="AH55" s="3"/>
-    </row>
-    <row r="56" spans="1:34">
+      <c r="AI55" s="3"/>
+    </row>
+    <row r="56" spans="1:35">
       <c r="A56" s="3"/>
       <c r="B56" s="4"/>
       <c r="C56" s="4"/>
       <c r="D56" s="4"/>
-      <c r="E56" s="5"/>
+      <c r="E56" s="4"/>
       <c r="F56" s="4"/>
       <c r="G56" s="4"/>
       <c r="H56" s="4"/>
@@ -3818,7 +3958,7 @@
       <c r="Q56" s="4"/>
       <c r="R56" s="4"/>
       <c r="S56" s="4"/>
-      <c r="T56" s="3"/>
+      <c r="T56" s="4"/>
       <c r="U56" s="3"/>
       <c r="V56" s="3"/>
       <c r="W56" s="3"/>
@@ -3833,13 +3973,14 @@
       <c r="AF56" s="3"/>
       <c r="AG56" s="3"/>
       <c r="AH56" s="3"/>
-    </row>
-    <row r="57" spans="1:34">
+      <c r="AI56" s="3"/>
+    </row>
+    <row r="57" spans="1:35">
       <c r="A57" s="3"/>
       <c r="B57" s="4"/>
       <c r="C57" s="4"/>
       <c r="D57" s="4"/>
-      <c r="E57" s="5"/>
+      <c r="E57" s="4"/>
       <c r="F57" s="4"/>
       <c r="G57" s="4"/>
       <c r="H57" s="4"/>
@@ -3854,7 +3995,7 @@
       <c r="Q57" s="4"/>
       <c r="R57" s="4"/>
       <c r="S57" s="4"/>
-      <c r="T57" s="3"/>
+      <c r="T57" s="4"/>
       <c r="U57" s="3"/>
       <c r="V57" s="3"/>
       <c r="W57" s="3"/>
@@ -3869,13 +4010,14 @@
       <c r="AF57" s="3"/>
       <c r="AG57" s="3"/>
       <c r="AH57" s="3"/>
-    </row>
-    <row r="58" spans="1:34">
+      <c r="AI57" s="3"/>
+    </row>
+    <row r="58" spans="1:35">
       <c r="A58" s="3"/>
       <c r="B58" s="4"/>
       <c r="C58" s="4"/>
       <c r="D58" s="4"/>
-      <c r="E58" s="5"/>
+      <c r="E58" s="4"/>
       <c r="F58" s="4"/>
       <c r="G58" s="4"/>
       <c r="H58" s="4"/>
@@ -3890,7 +4032,7 @@
       <c r="Q58" s="4"/>
       <c r="R58" s="4"/>
       <c r="S58" s="4"/>
-      <c r="T58" s="3"/>
+      <c r="T58" s="4"/>
       <c r="U58" s="3"/>
       <c r="V58" s="3"/>
       <c r="W58" s="3"/>
@@ -3905,8 +4047,9 @@
       <c r="AF58" s="3"/>
       <c r="AG58" s="3"/>
       <c r="AH58" s="3"/>
-    </row>
-    <row r="59" spans="1:34">
+      <c r="AI58" s="3"/>
+    </row>
+    <row r="59" spans="1:35">
       <c r="A59" s="3"/>
       <c r="B59" s="4"/>
       <c r="C59" s="4"/>
@@ -3926,7 +4069,7 @@
       <c r="Q59" s="4"/>
       <c r="R59" s="4"/>
       <c r="S59" s="4"/>
-      <c r="T59" s="3"/>
+      <c r="T59" s="4"/>
       <c r="U59" s="3"/>
       <c r="V59" s="3"/>
       <c r="W59" s="3"/>
@@ -3941,13 +4084,14 @@
       <c r="AF59" s="3"/>
       <c r="AG59" s="3"/>
       <c r="AH59" s="3"/>
-    </row>
-    <row r="60" spans="1:34">
+      <c r="AI59" s="3"/>
+    </row>
+    <row r="60" spans="1:35">
       <c r="A60" s="3"/>
       <c r="B60" s="4"/>
       <c r="C60" s="4"/>
       <c r="D60" s="4"/>
-      <c r="E60" s="4"/>
+      <c r="E60" s="5"/>
       <c r="F60" s="4"/>
       <c r="G60" s="4"/>
       <c r="H60" s="4"/>
@@ -3962,7 +4106,7 @@
       <c r="Q60" s="4"/>
       <c r="R60" s="4"/>
       <c r="S60" s="4"/>
-      <c r="T60" s="3"/>
+      <c r="T60" s="4"/>
       <c r="U60" s="3"/>
       <c r="V60" s="3"/>
       <c r="W60" s="3"/>
@@ -3977,13 +4121,14 @@
       <c r="AF60" s="3"/>
       <c r="AG60" s="3"/>
       <c r="AH60" s="3"/>
-    </row>
-    <row r="61" spans="1:34">
+      <c r="AI60" s="3"/>
+    </row>
+    <row r="61" spans="1:35">
       <c r="A61" s="3"/>
       <c r="B61" s="4"/>
       <c r="C61" s="4"/>
       <c r="D61" s="4"/>
-      <c r="E61" s="4"/>
+      <c r="E61" s="5"/>
       <c r="F61" s="4"/>
       <c r="G61" s="4"/>
       <c r="H61" s="4"/>
@@ -3998,7 +4143,7 @@
       <c r="Q61" s="4"/>
       <c r="R61" s="4"/>
       <c r="S61" s="4"/>
-      <c r="T61" s="3"/>
+      <c r="T61" s="4"/>
       <c r="U61" s="3"/>
       <c r="V61" s="3"/>
       <c r="W61" s="3"/>
@@ -4013,13 +4158,14 @@
       <c r="AF61" s="3"/>
       <c r="AG61" s="3"/>
       <c r="AH61" s="3"/>
-    </row>
-    <row r="62" spans="1:34">
+      <c r="AI61" s="3"/>
+    </row>
+    <row r="62" spans="1:35">
       <c r="A62" s="3"/>
       <c r="B62" s="4"/>
       <c r="C62" s="4"/>
       <c r="D62" s="4"/>
-      <c r="E62" s="4"/>
+      <c r="E62" s="5"/>
       <c r="F62" s="4"/>
       <c r="G62" s="4"/>
       <c r="H62" s="4"/>
@@ -4034,7 +4180,7 @@
       <c r="Q62" s="4"/>
       <c r="R62" s="4"/>
       <c r="S62" s="4"/>
-      <c r="T62" s="3"/>
+      <c r="T62" s="4"/>
       <c r="U62" s="3"/>
       <c r="V62" s="3"/>
       <c r="W62" s="3"/>
@@ -4049,13 +4195,14 @@
       <c r="AF62" s="3"/>
       <c r="AG62" s="3"/>
       <c r="AH62" s="3"/>
-    </row>
-    <row r="63" spans="1:34">
+      <c r="AI62" s="3"/>
+    </row>
+    <row r="63" spans="1:35">
       <c r="A63" s="3"/>
       <c r="B63" s="4"/>
       <c r="C63" s="4"/>
       <c r="D63" s="4"/>
-      <c r="E63" s="5"/>
+      <c r="E63" s="4"/>
       <c r="F63" s="4"/>
       <c r="G63" s="4"/>
       <c r="H63" s="4"/>
@@ -4070,7 +4217,7 @@
       <c r="Q63" s="4"/>
       <c r="R63" s="4"/>
       <c r="S63" s="4"/>
-      <c r="T63" s="3"/>
+      <c r="T63" s="4"/>
       <c r="U63" s="3"/>
       <c r="V63" s="3"/>
       <c r="W63" s="3"/>
@@ -4085,8 +4232,9 @@
       <c r="AF63" s="3"/>
       <c r="AG63" s="3"/>
       <c r="AH63" s="3"/>
-    </row>
-    <row r="64" spans="1:34">
+      <c r="AI63" s="3"/>
+    </row>
+    <row r="64" spans="1:35">
       <c r="A64" s="3"/>
       <c r="B64" s="4"/>
       <c r="C64" s="4"/>
@@ -4106,7 +4254,7 @@
       <c r="Q64" s="4"/>
       <c r="R64" s="4"/>
       <c r="S64" s="4"/>
-      <c r="T64" s="3"/>
+      <c r="T64" s="4"/>
       <c r="U64" s="3"/>
       <c r="V64" s="3"/>
       <c r="W64" s="3"/>
@@ -4121,8 +4269,9 @@
       <c r="AF64" s="3"/>
       <c r="AG64" s="3"/>
       <c r="AH64" s="3"/>
-    </row>
-    <row r="65" spans="1:34">
+      <c r="AI64" s="3"/>
+    </row>
+    <row r="65" spans="1:35">
       <c r="A65" s="3"/>
       <c r="B65" s="4"/>
       <c r="C65" s="4"/>
@@ -4142,7 +4291,7 @@
       <c r="Q65" s="4"/>
       <c r="R65" s="4"/>
       <c r="S65" s="4"/>
-      <c r="T65" s="3"/>
+      <c r="T65" s="4"/>
       <c r="U65" s="3"/>
       <c r="V65" s="3"/>
       <c r="W65" s="3"/>
@@ -4157,8 +4306,9 @@
       <c r="AF65" s="3"/>
       <c r="AG65" s="3"/>
       <c r="AH65" s="3"/>
-    </row>
-    <row r="66" spans="1:34">
+      <c r="AI65" s="3"/>
+    </row>
+    <row r="66" spans="1:35">
       <c r="A66" s="3"/>
       <c r="B66" s="4"/>
       <c r="C66" s="4"/>
@@ -4178,7 +4328,7 @@
       <c r="Q66" s="4"/>
       <c r="R66" s="4"/>
       <c r="S66" s="4"/>
-      <c r="T66" s="3"/>
+      <c r="T66" s="4"/>
       <c r="U66" s="3"/>
       <c r="V66" s="3"/>
       <c r="W66" s="3"/>
@@ -4193,13 +4343,14 @@
       <c r="AF66" s="3"/>
       <c r="AG66" s="3"/>
       <c r="AH66" s="3"/>
-    </row>
-    <row r="67" spans="1:34">
+      <c r="AI66" s="3"/>
+    </row>
+    <row r="67" spans="1:35">
       <c r="A67" s="3"/>
       <c r="B67" s="4"/>
       <c r="C67" s="4"/>
       <c r="D67" s="4"/>
-      <c r="E67" s="4"/>
+      <c r="E67" s="5"/>
       <c r="F67" s="4"/>
       <c r="G67" s="4"/>
       <c r="H67" s="4"/>
@@ -4214,7 +4365,7 @@
       <c r="Q67" s="4"/>
       <c r="R67" s="4"/>
       <c r="S67" s="4"/>
-      <c r="T67" s="3"/>
+      <c r="T67" s="4"/>
       <c r="U67" s="3"/>
       <c r="V67" s="3"/>
       <c r="W67" s="3"/>
@@ -4229,8 +4380,9 @@
       <c r="AF67" s="3"/>
       <c r="AG67" s="3"/>
       <c r="AH67" s="3"/>
-    </row>
-    <row r="68" spans="1:34">
+      <c r="AI67" s="3"/>
+    </row>
+    <row r="68" spans="1:35">
       <c r="A68" s="3"/>
       <c r="B68" s="4"/>
       <c r="C68" s="4"/>
@@ -4250,7 +4402,7 @@
       <c r="Q68" s="4"/>
       <c r="R68" s="4"/>
       <c r="S68" s="4"/>
-      <c r="T68" s="3"/>
+      <c r="T68" s="4"/>
       <c r="U68" s="3"/>
       <c r="V68" s="3"/>
       <c r="W68" s="3"/>
@@ -4265,8 +4417,9 @@
       <c r="AF68" s="3"/>
       <c r="AG68" s="3"/>
       <c r="AH68" s="3"/>
-    </row>
-    <row r="69" spans="1:34">
+      <c r="AI68" s="3"/>
+    </row>
+    <row r="69" spans="1:35">
       <c r="A69" s="3"/>
       <c r="B69" s="4"/>
       <c r="C69" s="4"/>
@@ -4286,7 +4439,7 @@
       <c r="Q69" s="4"/>
       <c r="R69" s="4"/>
       <c r="S69" s="4"/>
-      <c r="T69" s="3"/>
+      <c r="T69" s="4"/>
       <c r="U69" s="3"/>
       <c r="V69" s="3"/>
       <c r="W69" s="3"/>
@@ -4301,8 +4454,9 @@
       <c r="AF69" s="3"/>
       <c r="AG69" s="3"/>
       <c r="AH69" s="3"/>
-    </row>
-    <row r="70" spans="1:34">
+      <c r="AI69" s="3"/>
+    </row>
+    <row r="70" spans="1:35">
       <c r="A70" s="3"/>
       <c r="B70" s="4"/>
       <c r="C70" s="4"/>
@@ -4322,7 +4476,7 @@
       <c r="Q70" s="4"/>
       <c r="R70" s="4"/>
       <c r="S70" s="4"/>
-      <c r="T70" s="3"/>
+      <c r="T70" s="4"/>
       <c r="U70" s="3"/>
       <c r="V70" s="3"/>
       <c r="W70" s="3"/>
@@ -4337,8 +4491,9 @@
       <c r="AF70" s="3"/>
       <c r="AG70" s="3"/>
       <c r="AH70" s="3"/>
-    </row>
-    <row r="71" spans="1:34">
+      <c r="AI70" s="3"/>
+    </row>
+    <row r="71" spans="1:35">
       <c r="A71" s="3"/>
       <c r="B71" s="4"/>
       <c r="C71" s="4"/>
@@ -4358,7 +4513,7 @@
       <c r="Q71" s="4"/>
       <c r="R71" s="4"/>
       <c r="S71" s="4"/>
-      <c r="T71" s="3"/>
+      <c r="T71" s="4"/>
       <c r="U71" s="3"/>
       <c r="V71" s="3"/>
       <c r="W71" s="3"/>
@@ -4373,209 +4528,364 @@
       <c r="AF71" s="3"/>
       <c r="AG71" s="3"/>
       <c r="AH71" s="3"/>
-    </row>
-    <row r="79" spans="1:23">
-      <c r="A79" s="2"/>
-      <c r="B79" s="2"/>
-      <c r="C79" s="2"/>
-      <c r="D79" s="2"/>
-      <c r="R79" s="2"/>
-      <c r="T79" s="2"/>
-      <c r="U79" s="2"/>
-      <c r="V79" s="2"/>
-      <c r="W79" s="2"/>
-    </row>
-    <row r="80" spans="1:23">
-      <c r="A80" s="2"/>
-      <c r="B80" s="2"/>
-      <c r="C80" s="2"/>
-      <c r="D80" s="2"/>
-      <c r="E80" s="2"/>
-      <c r="R80" s="2"/>
-      <c r="S80" s="2"/>
-      <c r="T80" s="2"/>
-      <c r="U80" s="2"/>
-      <c r="V80" s="2"/>
-      <c r="W80" s="2"/>
-    </row>
-    <row r="81" spans="1:23">
-      <c r="A81" s="2"/>
-      <c r="B81" s="2"/>
-      <c r="C81" s="2"/>
-      <c r="D81" s="2"/>
-      <c r="R81" s="2"/>
-      <c r="S81" s="2"/>
-      <c r="T81" s="2"/>
-      <c r="U81" s="2"/>
-      <c r="V81" s="2"/>
-      <c r="W81" s="2"/>
-    </row>
-    <row r="82" spans="1:23">
-      <c r="A82" s="2"/>
-      <c r="B82" s="2"/>
-      <c r="C82" s="2"/>
-      <c r="D82" s="2"/>
-      <c r="R82" s="2"/>
-      <c r="S82" s="2"/>
-      <c r="T82" s="2"/>
-      <c r="U82" s="2"/>
-      <c r="V82" s="2"/>
-      <c r="W82" s="2"/>
-    </row>
-    <row r="83" spans="1:23">
+      <c r="AI71" s="3"/>
+    </row>
+    <row r="72" spans="1:35">
+      <c r="A72" s="3"/>
+      <c r="B72" s="4"/>
+      <c r="C72" s="4"/>
+      <c r="D72" s="4"/>
+      <c r="E72" s="4"/>
+      <c r="F72" s="4"/>
+      <c r="G72" s="4"/>
+      <c r="H72" s="4"/>
+      <c r="I72" s="4"/>
+      <c r="J72" s="4"/>
+      <c r="K72" s="4"/>
+      <c r="L72" s="4"/>
+      <c r="M72" s="4"/>
+      <c r="N72" s="4"/>
+      <c r="O72" s="4"/>
+      <c r="P72" s="4"/>
+      <c r="Q72" s="4"/>
+      <c r="R72" s="4"/>
+      <c r="S72" s="4"/>
+      <c r="T72" s="4"/>
+      <c r="U72" s="3"/>
+      <c r="V72" s="3"/>
+      <c r="W72" s="3"/>
+      <c r="X72" s="3"/>
+      <c r="Y72" s="3"/>
+      <c r="Z72" s="3"/>
+      <c r="AA72" s="3"/>
+      <c r="AB72" s="3"/>
+      <c r="AC72" s="3"/>
+      <c r="AD72" s="3"/>
+      <c r="AE72" s="3"/>
+      <c r="AF72" s="3"/>
+      <c r="AG72" s="3"/>
+      <c r="AH72" s="3"/>
+      <c r="AI72" s="3"/>
+    </row>
+    <row r="73" spans="1:35">
+      <c r="A73" s="3"/>
+      <c r="B73" s="4"/>
+      <c r="C73" s="4"/>
+      <c r="D73" s="4"/>
+      <c r="E73" s="4"/>
+      <c r="F73" s="4"/>
+      <c r="G73" s="4"/>
+      <c r="H73" s="4"/>
+      <c r="I73" s="4"/>
+      <c r="J73" s="4"/>
+      <c r="K73" s="4"/>
+      <c r="L73" s="4"/>
+      <c r="M73" s="4"/>
+      <c r="N73" s="4"/>
+      <c r="O73" s="4"/>
+      <c r="P73" s="4"/>
+      <c r="Q73" s="4"/>
+      <c r="R73" s="4"/>
+      <c r="S73" s="4"/>
+      <c r="T73" s="4"/>
+      <c r="U73" s="3"/>
+      <c r="V73" s="3"/>
+      <c r="W73" s="3"/>
+      <c r="X73" s="3"/>
+      <c r="Y73" s="3"/>
+      <c r="Z73" s="3"/>
+      <c r="AA73" s="3"/>
+      <c r="AB73" s="3"/>
+      <c r="AC73" s="3"/>
+      <c r="AD73" s="3"/>
+      <c r="AE73" s="3"/>
+      <c r="AF73" s="3"/>
+      <c r="AG73" s="3"/>
+      <c r="AH73" s="3"/>
+      <c r="AI73" s="3"/>
+    </row>
+    <row r="74" spans="1:35">
+      <c r="A74" s="3"/>
+      <c r="B74" s="4"/>
+      <c r="C74" s="4"/>
+      <c r="D74" s="4"/>
+      <c r="E74" s="4"/>
+      <c r="F74" s="4"/>
+      <c r="G74" s="4"/>
+      <c r="H74" s="4"/>
+      <c r="I74" s="4"/>
+      <c r="J74" s="4"/>
+      <c r="K74" s="4"/>
+      <c r="L74" s="4"/>
+      <c r="M74" s="4"/>
+      <c r="N74" s="4"/>
+      <c r="O74" s="4"/>
+      <c r="P74" s="4"/>
+      <c r="Q74" s="4"/>
+      <c r="R74" s="4"/>
+      <c r="S74" s="4"/>
+      <c r="T74" s="4"/>
+      <c r="U74" s="3"/>
+      <c r="V74" s="3"/>
+      <c r="W74" s="3"/>
+      <c r="X74" s="3"/>
+      <c r="Y74" s="3"/>
+      <c r="Z74" s="3"/>
+      <c r="AA74" s="3"/>
+      <c r="AB74" s="3"/>
+      <c r="AC74" s="3"/>
+      <c r="AD74" s="3"/>
+      <c r="AE74" s="3"/>
+      <c r="AF74" s="3"/>
+      <c r="AG74" s="3"/>
+      <c r="AH74" s="3"/>
+      <c r="AI74" s="3"/>
+    </row>
+    <row r="75" spans="1:35">
+      <c r="A75" s="3"/>
+      <c r="B75" s="4"/>
+      <c r="C75" s="4"/>
+      <c r="D75" s="4"/>
+      <c r="E75" s="4"/>
+      <c r="F75" s="4"/>
+      <c r="G75" s="4"/>
+      <c r="H75" s="4"/>
+      <c r="I75" s="4"/>
+      <c r="J75" s="4"/>
+      <c r="K75" s="4"/>
+      <c r="L75" s="4"/>
+      <c r="M75" s="4"/>
+      <c r="N75" s="4"/>
+      <c r="O75" s="4"/>
+      <c r="P75" s="4"/>
+      <c r="Q75" s="4"/>
+      <c r="R75" s="4"/>
+      <c r="S75" s="4"/>
+      <c r="T75" s="4"/>
+      <c r="U75" s="3"/>
+      <c r="V75" s="3"/>
+      <c r="W75" s="3"/>
+      <c r="X75" s="3"/>
+      <c r="Y75" s="3"/>
+      <c r="Z75" s="3"/>
+      <c r="AA75" s="3"/>
+      <c r="AB75" s="3"/>
+      <c r="AC75" s="3"/>
+      <c r="AD75" s="3"/>
+      <c r="AE75" s="3"/>
+      <c r="AF75" s="3"/>
+      <c r="AG75" s="3"/>
+      <c r="AH75" s="3"/>
+      <c r="AI75" s="3"/>
+    </row>
+    <row r="83" spans="1:24">
       <c r="A83" s="2"/>
       <c r="B83" s="2"/>
       <c r="C83" s="2"/>
       <c r="D83" s="2"/>
-      <c r="R83" s="2"/>
       <c r="S83" s="2"/>
-      <c r="T83" s="2"/>
       <c r="U83" s="2"/>
       <c r="V83" s="2"/>
       <c r="W83" s="2"/>
-    </row>
-    <row r="84" spans="1:23">
+      <c r="X83" s="2"/>
+    </row>
+    <row r="84" spans="1:24">
       <c r="A84" s="2"/>
       <c r="B84" s="2"/>
       <c r="C84" s="2"/>
       <c r="D84" s="2"/>
-      <c r="R84" s="2"/>
+      <c r="E84" s="2"/>
       <c r="S84" s="2"/>
       <c r="T84" s="2"/>
       <c r="U84" s="2"/>
       <c r="V84" s="2"/>
       <c r="W84" s="2"/>
-    </row>
-    <row r="85" spans="1:23">
+      <c r="X84" s="2"/>
+    </row>
+    <row r="85" spans="1:24">
       <c r="A85" s="2"/>
       <c r="B85" s="2"/>
       <c r="C85" s="2"/>
       <c r="D85" s="2"/>
-      <c r="R85" s="2"/>
       <c r="S85" s="2"/>
       <c r="T85" s="2"/>
       <c r="U85" s="2"/>
       <c r="V85" s="2"/>
       <c r="W85" s="2"/>
-    </row>
-    <row r="86" spans="1:23">
+      <c r="X85" s="2"/>
+    </row>
+    <row r="86" spans="1:24">
       <c r="A86" s="2"/>
       <c r="B86" s="2"/>
       <c r="C86" s="2"/>
       <c r="D86" s="2"/>
-      <c r="R86" s="2"/>
       <c r="S86" s="2"/>
       <c r="T86" s="2"/>
       <c r="U86" s="2"/>
       <c r="V86" s="2"/>
       <c r="W86" s="2"/>
-    </row>
-    <row r="87" spans="1:23">
+      <c r="X86" s="2"/>
+    </row>
+    <row r="87" spans="1:24">
       <c r="A87" s="2"/>
       <c r="B87" s="2"/>
       <c r="C87" s="2"/>
       <c r="D87" s="2"/>
-      <c r="R87" s="2"/>
       <c r="S87" s="2"/>
       <c r="T87" s="2"/>
       <c r="U87" s="2"/>
       <c r="V87" s="2"/>
       <c r="W87" s="2"/>
-    </row>
-    <row r="88" spans="1:23">
+      <c r="X87" s="2"/>
+    </row>
+    <row r="88" spans="1:24">
       <c r="A88" s="2"/>
       <c r="B88" s="2"/>
       <c r="C88" s="2"/>
       <c r="D88" s="2"/>
-      <c r="R88" s="2"/>
       <c r="S88" s="2"/>
       <c r="T88" s="2"/>
       <c r="U88" s="2"/>
       <c r="V88" s="2"/>
       <c r="W88" s="2"/>
-    </row>
-    <row r="89" spans="1:23">
+      <c r="X88" s="2"/>
+    </row>
+    <row r="89" spans="1:24">
       <c r="A89" s="2"/>
       <c r="B89" s="2"/>
       <c r="C89" s="2"/>
       <c r="D89" s="2"/>
-      <c r="R89" s="2"/>
       <c r="S89" s="2"/>
       <c r="T89" s="2"/>
       <c r="U89" s="2"/>
       <c r="V89" s="2"/>
       <c r="W89" s="2"/>
-    </row>
-    <row r="90" spans="1:23">
+      <c r="X89" s="2"/>
+    </row>
+    <row r="90" spans="1:24">
       <c r="A90" s="2"/>
       <c r="B90" s="2"/>
       <c r="C90" s="2"/>
       <c r="D90" s="2"/>
-      <c r="R90" s="2"/>
       <c r="S90" s="2"/>
       <c r="T90" s="2"/>
       <c r="U90" s="2"/>
       <c r="V90" s="2"/>
       <c r="W90" s="2"/>
-    </row>
-    <row r="91" spans="1:23">
+      <c r="X90" s="2"/>
+    </row>
+    <row r="91" spans="1:24">
       <c r="A91" s="2"/>
       <c r="B91" s="2"/>
       <c r="C91" s="2"/>
       <c r="D91" s="2"/>
-      <c r="R91" s="2"/>
       <c r="S91" s="2"/>
       <c r="T91" s="2"/>
       <c r="U91" s="2"/>
       <c r="V91" s="2"/>
       <c r="W91" s="2"/>
-    </row>
-    <row r="92" spans="1:23">
+      <c r="X91" s="2"/>
+    </row>
+    <row r="92" spans="1:24">
       <c r="A92" s="2"/>
       <c r="B92" s="2"/>
       <c r="C92" s="2"/>
       <c r="D92" s="2"/>
-      <c r="R92" s="2"/>
       <c r="S92" s="2"/>
       <c r="T92" s="2"/>
       <c r="U92" s="2"/>
       <c r="V92" s="2"/>
       <c r="W92" s="2"/>
+      <c r="X92" s="2"/>
+    </row>
+    <row r="93" spans="1:24">
+      <c r="A93" s="2"/>
+      <c r="B93" s="2"/>
+      <c r="C93" s="2"/>
+      <c r="D93" s="2"/>
+      <c r="S93" s="2"/>
+      <c r="T93" s="2"/>
+      <c r="U93" s="2"/>
+      <c r="V93" s="2"/>
+      <c r="W93" s="2"/>
+      <c r="X93" s="2"/>
+    </row>
+    <row r="94" spans="1:24">
+      <c r="A94" s="2"/>
+      <c r="B94" s="2"/>
+      <c r="C94" s="2"/>
+      <c r="D94" s="2"/>
+      <c r="S94" s="2"/>
+      <c r="T94" s="2"/>
+      <c r="U94" s="2"/>
+      <c r="V94" s="2"/>
+      <c r="W94" s="2"/>
+      <c r="X94" s="2"/>
+    </row>
+    <row r="95" spans="1:24">
+      <c r="A95" s="2"/>
+      <c r="B95" s="2"/>
+      <c r="C95" s="2"/>
+      <c r="D95" s="2"/>
+      <c r="S95" s="2"/>
+      <c r="T95" s="2"/>
+      <c r="U95" s="2"/>
+      <c r="V95" s="2"/>
+      <c r="W95" s="2"/>
+      <c r="X95" s="2"/>
+    </row>
+    <row r="96" spans="1:24">
+      <c r="A96" s="2"/>
+      <c r="B96" s="2"/>
+      <c r="C96" s="2"/>
+      <c r="D96" s="2"/>
+      <c r="S96" s="2"/>
+      <c r="T96" s="2"/>
+      <c r="U96" s="2"/>
+      <c r="V96" s="2"/>
+      <c r="W96" s="2"/>
+      <c r="X96" s="2"/>
     </row>
   </sheetData>
-  <dataValidations count="11">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F6 F15 F18 F19 F20 F21 F24 F25 F26 F27 F28 F29 F30 F31 F34 F35 F36 F2:F5 F7:F14 F16:F17 F22:F23 F32:F33 F37:F1048576">
+  <dataValidations count="13">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H38 H39 H40 H10:H37 H41:H1048576">
+      <formula1>"WB_ALU,WB_MEM,WB_PC4,WB_XX,WB_CSR"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D4 D5 D6 D7 D8 D9 D10 D11 D12 D13 D14 D15 D16 D17 D18 D19 D20 D21 D22 D23 D24 D25 D26 D27 D28 D29 D30 D31 D32 D33 D34 D35 D36 D37 D38 D39 D40 D2:D3 D41:D1048576">
+      <formula1>"A_PC,A_RS1"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="M37 M38 M39 M40 M2:M36 M41:M1048576">
+      <formula1>"CSR_W,CSR_S,CSR_C,CSR_P,CSR_XX"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="N4 N5 N6 N7 N8 N9 N10 N11 N12 N13 N14 N15 N16 N17 N18 N19 N20 N21 N22 N23 N24 N25 N26 N27 N28 N29 N30 N31 N32 N33 N34 N35 N36 N37 N38 N39 N40 N2:N3 N41:N1048576">
+      <formula1>"INST_VALID,INST_INVALID"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J5 J6 J7 J8 J9 J10 J11 J12 J13 J14 J15 J16 J17 J18 J19 J20 J21 J22 J23 J24 J25 J26 J27 J28 J29 J30 J31 J32 J33 J34 J35 J36 J37 J38 J39 J40 J2:J4 J41:J1048576">
+      <formula1>"ST_SW,ST_SH,ST_SB,ST_XX"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C2:C1048576">
+      <formula1>"PC_4,PC_0,PC_ALU,PC_CSR"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F6 F15 F18 F19 F20 F21 F24 F25 F26 F27 F28 F29 F30 F31 F34 F35 F36 F37 F38 F39 F40 F2:F5 F7:F14 F16:F17 F22:F23 F32:F33 F41:F1048576">
       <formula1>"ALU_ADD,ALU_SUB,ALU_AND,ALU_OR,ALU_XOR,ALU_SLL,ALU_SRL,ALU_SLT,ALU_SLTU,ALU_COPY_A,ALU_COPY_B,ALU_SRA"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L5 L6 L7 L10 L11 L14 L15 L16 L17 L18 L19 L20 L21 L22 L23 L24 L25 L26 L27 L28 L29 L30 L31 L32 L33 L34 L35 L36 L2:L4 L8:L9 L12:L13 L37:L1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L5 L6 L7 L10 L11 L14 L15 L16 L17 L18 L19 L20 L21 L22 L23 L24 L25 L26 L27 L28 L29 L30 L31 L32 L33 L34 L35 L36 L37 L38 L39 L40 L2:L4 L8:L9 L12:L13 L41:L1048576">
       <formula1>"BR_EQ,BR_NE,BR_LTU,BR_GE,BR_GEU,BR_LT,BR_XX"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J5 J6 J7 J8 J9 J10 J11 J12 J13 J14 J15 J16 J17 J18 J19 J20 J21 J22 J23 J24 J25 J26 J27 J28 J29 J30 J31 J32 J33 J34 J35 J36 J2:J4 J37:J1048576">
-      <formula1>"ST_SW,ST_SH,ST_SB,ST_XX"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H5 H6 H7 H8 H9 H10 H11 H14 H15 H16 H17 H18 H19 H20 H21 H22 H23 H24 H25 H26 H27 H28 H29 H30 H31 H32 H33 H34 H35 H36 H2:H4 H12:H13 H37:H1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H5 H6 H7 H8 H9 H2:H4">
       <formula1>"WB_ALU,WB_MEM,WB_PC4,WB_XX"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="M4 M5 M6 M7 M8 M9 M10 M11 M12 M13 M14 M15 M16 M17 M18 M19 M20 M21 M22 M23 M24 M25 M26 M27 M28 M29 M30 M31 M32 M33 M34 M35 M36 M2:M3 M37:M1048576">
-      <formula1>"INST_VALID,INST_INVALID"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K4 K5 K6 K7 K8 K9 K10 K11 K12 K13 K14 K15 K16 K17 K18 K19 K20 K21 K22 K23 K24 K25 K26 K27 K28 K29 K30 K31 K32 K33 K34 K35 K36 K2:K3 K37:K1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K4 K5 K6 K7 K8 K9 K10 K11 K12 K13 K14 K15 K16 K17 K18 K19 K20 K21 K22 K23 K24 K25 K26 K27 K28 K29 K30 K31 K32 K33 K34 K35 K36 K37 K38 K39 K40 K2:K3 K41:K1048576">
       <formula1>"MASK_XX,MASK_B,MASK_H,MASK_W,MASK_D"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I4 I5 I6 I7 I8 I9 I10 I11 I12 I13 I14 I15 I16 I17 I18 I19 I20 I21 I22 I23 I24 I25 I26 I27 I28 I29 I30 I31 I32 I33 I34 I35 I36 I2:I3 I37:I1048576">
-      <formula1>"LD_LB,LD_LH,LD_LW,LD_LBU,LD_LHU,LD_XX"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G4 G5 G6 G7 G8 G9 G10 G11 G12 G13 G14 G15 G16 G17 G18 G19 G20 G21 G22 G23 G24 G25 G26 G27 G28 G29 G30 G31 G32 G33 G34 G35 G36 G37 G38 G39 G40 G2:G3 G41:G1048576">
+      <formula1>"IMM_I,IMM_J,IMM_U,IMM_S,IMM_B"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E4 E5 E6 E7 E8 E9 E10 E11 E12 E13 E14 E15 E16 E17 E18 E19 E20 E21 E22 E23 E24 E25 E26 E27 E28 E29 E30 E31 E32 E33 E34 E35 E36 E2:E3 E37:E1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E4 E5 E6 E7 E8 E9 E10 E11 E12 E13 E14 E15 E16 E17 E18 E19 E20 E21 E22 E23 E24 E25 E26 E27 E28 E29 E30 E31 E32 E33 E34 E35 E36 E37 E38 E39 E40 E2:E3 E41:E1048576">
       <formula1>"B_IMM,B_RS2"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G4 G5 G6 G7 G8 G9 G10 G11 G12 G13 G14 G15 G16 G17 G18 G19 G20 G21 G22 G23 G24 G25 G26 G27 G28 G29 G30 G31 G32 G33 G34 G35 G36 G2:G3 G37:G1048576">
-      <formula1>"IMM_I,IMM_J,IMM_U,IMM_S,IMM_B"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D4 D5 D6 D7 D8 D9 D10 D11 D12 D13 D14 D15 D16 D17 D18 D19 D20 D21 D22 D23 D24 D25 D26 D27 D28 D29 D30 D31 D32 D33 D34 D35 D36 D2:D3 D37:D1048576">
-      <formula1>"A_PC,A_RS1"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C4 C5 C6 C7 C8 C9 C10 C11 C12 C13 C14 C15 C16 C17 C18 C19 C20 C21 C22 C23 C24 C25 C26 C27 C28 C29 C30 C31 C32 C33 C34 C35 C36 C2:C3 C37:C1048576">
-      <formula1>"PC_4,PC_0,PC_ALU"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I4 I5 I6 I7 I8 I9 I10 I11 I12 I13 I14 I15 I16 I17 I18 I19 I20 I21 I22 I23 I24 I25 I26 I27 I28 I29 I30 I31 I32 I33 I34 I35 I36 I37 I38 I39 I40 I2:I3 I41:I1048576">
+      <formula1>"LD_LB,LD_LH,LD_LW,LD_LBU,LD_LHU,LD_XX"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
> sim RTL ysyx_23060246 韩炳晋 Linux archlinux 6.6.60-1-lts #1 SMP PREEMPT_DYNAMIC Fri, 08 Nov 2024 16:03:02 +0000 x86_64 GNU/Linux  20:12:16 up 4 days, 10:28,  2 users,  load average: 5.12, 4.11, 3.76
</commit_message>
<xml_diff>
--- a/npc/tools/control_gen/control_table.xlsx
+++ b/npc/tools/control_gen/control_table.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="296" uniqueCount="108">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="302" uniqueCount="110">
   <si>
     <t>comment</t>
   </si>
@@ -254,6 +254,12 @@
   </si>
   <si>
     <t>ALU_SLL</t>
+  </si>
+  <si>
+    <t>slt</t>
+  </si>
+  <si>
+    <t>ALU_SLT</t>
   </si>
   <si>
     <t>sltu</t>
@@ -345,10 +351,10 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="4">
+    <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="42" formatCode="_ &quot;￥&quot;* #,##0_ ;_ &quot;￥&quot;* \-#,##0_ ;_ &quot;￥&quot;* &quot;-&quot;_ ;_ @_ "/>
+    <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="41" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="42" formatCode="_ &quot;￥&quot;* #,##0_ ;_ &quot;￥&quot;* \-#,##0_ ;_ &quot;￥&quot;* &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
   </numFmts>
   <fonts count="22">
     <font>
@@ -385,8 +391,70 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <b/>
+      <sz val="13"/>
+      <color theme="3"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C0006"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF0000FF"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <sz val="11"/>
       <color theme="0"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="3"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="18"/>
+      <color theme="3"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF800080"/>
       <name val="宋体"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -401,7 +469,7 @@
     </font>
     <font>
       <b/>
-      <sz val="11"/>
+      <sz val="15"/>
       <color theme="3"/>
       <name val="宋体"/>
       <charset val="134"/>
@@ -417,16 +485,15 @@
     </font>
     <font>
       <b/>
-      <sz val="13"/>
-      <color theme="3"/>
+      <sz val="11"/>
+      <color rgb="FF3F3F3F"/>
       <name val="宋体"/>
-      <charset val="134"/>
+      <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <u/>
       <sz val="11"/>
-      <color rgb="FF0000FF"/>
+      <color rgb="FF006100"/>
       <name val="宋体"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -440,53 +507,7 @@
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FF9C0006"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FF3F3F3F"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF006100"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="15"/>
-      <color theme="3"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF800080"/>
+      <color rgb="FF3F3F76"/>
       <name val="宋体"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -495,21 +516,6 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="18"/>
-      <color theme="3"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF3F3F76"/>
       <name val="宋体"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -530,7 +536,85 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="9"/>
+        <fgColor theme="8" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFA5A5A5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -542,7 +626,67 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="7"/>
+        <fgColor theme="4" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFCC99"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -554,49 +698,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="6"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
+        <fgColor theme="8" tint="0.799981688894314"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -608,103 +710,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFA5A5A5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor theme="6" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -723,30 +729,6 @@
       <top/>
       <bottom style="double">
         <color rgb="FFFF8001"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4" tint="0.499984740745262"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF7F7F7F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF7F7F7F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF7F7F7F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF7F7F7F"/>
       </bottom>
       <diagonal/>
     </border>
@@ -775,17 +757,11 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF3F3F3F"/>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4" tint="0.499984740745262"/>
       </bottom>
       <diagonal/>
     </border>
@@ -805,6 +781,36 @@
       <diagonal/>
     </border>
     <border>
+      <left style="thin">
+        <color rgb="FF7F7F7F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF7F7F7F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF7F7F7F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF7F7F7F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
       <left/>
       <right/>
       <top style="thin">
@@ -820,142 +826,142 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="32" borderId="3" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="8" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="23" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="17" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="3" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="11" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="17" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="17" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="4" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="5" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -1306,7 +1312,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:AI96"/>
+  <dimension ref="A1:AI97"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
     <col min="1" max="1" width="13.1" customWidth="1"/>
@@ -2831,14 +2837,12 @@
         <v>24</v>
       </c>
       <c r="E30" s="4" t="s">
-        <v>15</v>
+        <v>76</v>
       </c>
       <c r="F30" s="4" t="s">
-        <v>81</v>
-      </c>
-      <c r="G30" s="4" t="s">
-        <v>25</v>
-      </c>
+        <v>83</v>
+      </c>
+      <c r="G30" s="4"/>
       <c r="H30" s="4" t="s">
         <v>18</v>
       </c>
@@ -2875,19 +2879,21 @@
     <row r="31" spans="1:35">
       <c r="A31" s="3"/>
       <c r="B31" s="4" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="C31" s="2"/>
       <c r="D31" s="4" t="s">
         <v>24</v>
       </c>
       <c r="E31" s="4" t="s">
-        <v>76</v>
+        <v>15</v>
       </c>
       <c r="F31" s="4" t="s">
-        <v>79</v>
-      </c>
-      <c r="G31" s="4"/>
+        <v>83</v>
+      </c>
+      <c r="G31" s="4" t="s">
+        <v>25</v>
+      </c>
       <c r="H31" s="4" t="s">
         <v>18</v>
       </c>
@@ -2924,7 +2930,7 @@
     <row r="32" spans="1:35">
       <c r="A32" s="3"/>
       <c r="B32" s="4" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="C32" s="2"/>
       <c r="D32" s="4" t="s">
@@ -2934,7 +2940,7 @@
         <v>76</v>
       </c>
       <c r="F32" s="4" t="s">
-        <v>22</v>
+        <v>79</v>
       </c>
       <c r="G32" s="4"/>
       <c r="H32" s="4" t="s">
@@ -2973,7 +2979,7 @@
     <row r="33" spans="1:35">
       <c r="A33" s="3"/>
       <c r="B33" s="4" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="C33" s="2"/>
       <c r="D33" s="4" t="s">
@@ -2983,7 +2989,7 @@
         <v>76</v>
       </c>
       <c r="F33" s="4" t="s">
-        <v>86</v>
+        <v>22</v>
       </c>
       <c r="G33" s="4"/>
       <c r="H33" s="4" t="s">
@@ -3032,7 +3038,7 @@
         <v>76</v>
       </c>
       <c r="F34" s="4" t="s">
-        <v>31</v>
+        <v>88</v>
       </c>
       <c r="G34" s="4"/>
       <c r="H34" s="4" t="s">
@@ -3071,7 +3077,7 @@
     <row r="35" spans="1:35">
       <c r="A35" s="3"/>
       <c r="B35" s="4" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C35" s="2"/>
       <c r="D35" s="4" t="s">
@@ -3081,7 +3087,7 @@
         <v>76</v>
       </c>
       <c r="F35" s="4" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="G35" s="4"/>
       <c r="H35" s="4" t="s">
@@ -3120,7 +3126,7 @@
     <row r="36" spans="1:35">
       <c r="A36" s="3"/>
       <c r="B36" s="4" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C36" s="2"/>
       <c r="D36" s="4" t="s">
@@ -3130,7 +3136,7 @@
         <v>76</v>
       </c>
       <c r="F36" s="4" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="G36" s="4"/>
       <c r="H36" s="4" t="s">
@@ -3169,29 +3175,27 @@
     <row r="37" spans="1:35">
       <c r="A37" s="3"/>
       <c r="B37" s="4" t="s">
-        <v>90</v>
-      </c>
-      <c r="C37" s="2" t="s">
         <v>91</v>
       </c>
+      <c r="C37" s="2"/>
       <c r="D37" s="4" t="s">
         <v>24</v>
       </c>
       <c r="E37" s="4" t="s">
         <v>76</v>
       </c>
-      <c r="F37" s="4"/>
+      <c r="F37" s="4" t="s">
+        <v>29</v>
+      </c>
       <c r="G37" s="4"/>
       <c r="H37" s="4" t="s">
-        <v>92</v>
+        <v>18</v>
       </c>
       <c r="I37" s="4"/>
       <c r="J37" s="4"/>
       <c r="K37" s="4"/>
       <c r="L37" s="4"/>
-      <c r="M37" s="4" t="s">
-        <v>93</v>
-      </c>
+      <c r="M37" s="4"/>
       <c r="N37" s="4" t="s">
         <v>19</v>
       </c>
@@ -3220,10 +3224,10 @@
     <row r="38" spans="1:35">
       <c r="A38" s="3"/>
       <c r="B38" s="4" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="D38" s="4" t="s">
         <v>24</v>
@@ -3234,7 +3238,7 @@
       <c r="F38" s="4"/>
       <c r="G38" s="4"/>
       <c r="H38" s="4" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="I38" s="4"/>
       <c r="J38" s="4"/>
@@ -3274,21 +3278,25 @@
         <v>96</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>97</v>
-      </c>
-      <c r="D39" s="4"/>
-      <c r="E39" s="4"/>
+        <v>93</v>
+      </c>
+      <c r="D39" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="E39" s="4" t="s">
+        <v>76</v>
+      </c>
       <c r="F39" s="4"/>
       <c r="G39" s="4"/>
       <c r="H39" s="4" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="I39" s="4"/>
       <c r="J39" s="4"/>
       <c r="K39" s="4"/>
       <c r="L39" s="4"/>
       <c r="M39" s="4" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="N39" s="4" t="s">
         <v>19</v>
@@ -3318,24 +3326,24 @@
     <row r="40" spans="1:35">
       <c r="A40" s="3"/>
       <c r="B40" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="C40" s="2" t="s">
         <v>99</v>
-      </c>
-      <c r="C40" s="2" t="s">
-        <v>97</v>
       </c>
       <c r="D40" s="4"/>
       <c r="E40" s="4"/>
       <c r="F40" s="4"/>
       <c r="G40" s="4"/>
       <c r="H40" s="4" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="I40" s="4"/>
       <c r="J40" s="4"/>
       <c r="K40" s="4"/>
       <c r="L40" s="4"/>
       <c r="M40" s="4" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="N40" s="4" t="s">
         <v>19</v>
@@ -3362,52 +3370,41 @@
       <c r="AH40" s="3"/>
       <c r="AI40" s="3"/>
     </row>
-    <row r="41" spans="2:35">
-      <c r="B41" s="2" t="s">
+    <row r="41" spans="1:35">
+      <c r="A41" s="3"/>
+      <c r="B41" s="4" t="s">
+        <v>101</v>
+      </c>
+      <c r="C41" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="D41" s="4"/>
+      <c r="E41" s="4"/>
+      <c r="F41" s="4"/>
+      <c r="G41" s="4"/>
+      <c r="H41" s="4" t="s">
+        <v>94</v>
+      </c>
+      <c r="I41" s="4"/>
+      <c r="J41" s="4"/>
+      <c r="K41" s="4"/>
+      <c r="L41" s="4"/>
+      <c r="M41" s="4" t="s">
         <v>100</v>
       </c>
-      <c r="C41" s="2" t="s">
-        <v>91</v>
-      </c>
-      <c r="D41" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="E41" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="F41" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="G41" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="H41" s="4" t="s">
-        <v>101</v>
-      </c>
-      <c r="I41" s="4" t="s">
-        <v>102</v>
-      </c>
-      <c r="J41" s="4" t="s">
-        <v>103</v>
-      </c>
-      <c r="K41" s="2" t="s">
-        <v>104</v>
-      </c>
-      <c r="L41" s="2" t="s">
-        <v>105</v>
-      </c>
-      <c r="M41" s="2" t="s">
-        <v>106</v>
-      </c>
-      <c r="N41" s="2" t="s">
-        <v>107</v>
-      </c>
-      <c r="O41" s="2"/>
-      <c r="P41" s="2"/>
-      <c r="Q41" s="2"/>
-      <c r="R41" s="2"/>
-      <c r="S41" s="2"/>
-      <c r="T41" s="2"/>
+      <c r="N41" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="O41" s="4"/>
+      <c r="P41" s="4"/>
+      <c r="Q41" s="4"/>
+      <c r="R41" s="4"/>
+      <c r="S41" s="4"/>
+      <c r="T41" s="4"/>
+      <c r="U41" s="3"/>
+      <c r="V41" s="3"/>
+      <c r="W41" s="3"/>
+      <c r="X41" s="3"/>
       <c r="Y41" s="3"/>
       <c r="Z41" s="3"/>
       <c r="AA41" s="3"/>
@@ -3420,31 +3417,52 @@
       <c r="AH41" s="3"/>
       <c r="AI41" s="3"/>
     </row>
-    <row r="42" spans="1:35">
-      <c r="A42" s="3"/>
-      <c r="B42" s="4"/>
-      <c r="C42" s="4"/>
-      <c r="D42" s="4"/>
-      <c r="E42" s="4"/>
-      <c r="F42" s="4"/>
-      <c r="G42" s="4"/>
-      <c r="H42" s="4"/>
-      <c r="I42" s="4"/>
-      <c r="J42" s="4"/>
-      <c r="K42" s="4"/>
-      <c r="L42" s="4"/>
-      <c r="M42" s="4"/>
-      <c r="N42" s="4"/>
-      <c r="O42" s="4"/>
-      <c r="P42" s="4"/>
-      <c r="Q42" s="4"/>
-      <c r="R42" s="4"/>
-      <c r="S42" s="4"/>
-      <c r="T42" s="4"/>
-      <c r="U42" s="3"/>
-      <c r="V42" s="3"/>
-      <c r="W42" s="3"/>
-      <c r="X42" s="3"/>
+    <row r="42" spans="2:35">
+      <c r="B42" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="C42" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="D42" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="E42" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="F42" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="G42" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="H42" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="I42" s="4" t="s">
+        <v>104</v>
+      </c>
+      <c r="J42" s="4" t="s">
+        <v>105</v>
+      </c>
+      <c r="K42" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="L42" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="M42" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="N42" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="O42" s="2"/>
+      <c r="P42" s="2"/>
+      <c r="Q42" s="2"/>
+      <c r="R42" s="2"/>
+      <c r="S42" s="2"/>
+      <c r="T42" s="2"/>
       <c r="Y42" s="3"/>
       <c r="Z42" s="3"/>
       <c r="AA42" s="3"/>
@@ -3457,7 +3475,7 @@
       <c r="AH42" s="3"/>
       <c r="AI42" s="3"/>
     </row>
-    <row r="43" s="1" customFormat="1" spans="1:35">
+    <row r="43" spans="1:35">
       <c r="A43" s="3"/>
       <c r="B43" s="4"/>
       <c r="C43" s="4"/>
@@ -3531,7 +3549,7 @@
       <c r="AH44" s="3"/>
       <c r="AI44" s="3"/>
     </row>
-    <row r="45" spans="1:35">
+    <row r="45" s="1" customFormat="1" spans="1:35">
       <c r="A45" s="3"/>
       <c r="B45" s="4"/>
       <c r="C45" s="4"/>
@@ -4091,7 +4109,7 @@
       <c r="B60" s="4"/>
       <c r="C60" s="4"/>
       <c r="D60" s="4"/>
-      <c r="E60" s="5"/>
+      <c r="E60" s="4"/>
       <c r="F60" s="4"/>
       <c r="G60" s="4"/>
       <c r="H60" s="4"/>
@@ -4202,7 +4220,7 @@
       <c r="B63" s="4"/>
       <c r="C63" s="4"/>
       <c r="D63" s="4"/>
-      <c r="E63" s="4"/>
+      <c r="E63" s="5"/>
       <c r="F63" s="4"/>
       <c r="G63" s="4"/>
       <c r="H63" s="4"/>
@@ -4350,7 +4368,7 @@
       <c r="B67" s="4"/>
       <c r="C67" s="4"/>
       <c r="D67" s="4"/>
-      <c r="E67" s="5"/>
+      <c r="E67" s="4"/>
       <c r="F67" s="4"/>
       <c r="G67" s="4"/>
       <c r="H67" s="4"/>
@@ -4387,7 +4405,7 @@
       <c r="B68" s="4"/>
       <c r="C68" s="4"/>
       <c r="D68" s="4"/>
-      <c r="E68" s="4"/>
+      <c r="E68" s="5"/>
       <c r="F68" s="4"/>
       <c r="G68" s="4"/>
       <c r="H68" s="4"/>
@@ -4678,25 +4696,49 @@
       <c r="AH75" s="3"/>
       <c r="AI75" s="3"/>
     </row>
-    <row r="83" spans="1:24">
-      <c r="A83" s="2"/>
-      <c r="B83" s="2"/>
-      <c r="C83" s="2"/>
-      <c r="D83" s="2"/>
-      <c r="S83" s="2"/>
-      <c r="U83" s="2"/>
-      <c r="V83" s="2"/>
-      <c r="W83" s="2"/>
-      <c r="X83" s="2"/>
+    <row r="76" spans="1:35">
+      <c r="A76" s="3"/>
+      <c r="B76" s="4"/>
+      <c r="C76" s="4"/>
+      <c r="D76" s="4"/>
+      <c r="E76" s="4"/>
+      <c r="F76" s="4"/>
+      <c r="G76" s="4"/>
+      <c r="H76" s="4"/>
+      <c r="I76" s="4"/>
+      <c r="J76" s="4"/>
+      <c r="K76" s="4"/>
+      <c r="L76" s="4"/>
+      <c r="M76" s="4"/>
+      <c r="N76" s="4"/>
+      <c r="O76" s="4"/>
+      <c r="P76" s="4"/>
+      <c r="Q76" s="4"/>
+      <c r="R76" s="4"/>
+      <c r="S76" s="4"/>
+      <c r="T76" s="4"/>
+      <c r="U76" s="3"/>
+      <c r="V76" s="3"/>
+      <c r="W76" s="3"/>
+      <c r="X76" s="3"/>
+      <c r="Y76" s="3"/>
+      <c r="Z76" s="3"/>
+      <c r="AA76" s="3"/>
+      <c r="AB76" s="3"/>
+      <c r="AC76" s="3"/>
+      <c r="AD76" s="3"/>
+      <c r="AE76" s="3"/>
+      <c r="AF76" s="3"/>
+      <c r="AG76" s="3"/>
+      <c r="AH76" s="3"/>
+      <c r="AI76" s="3"/>
     </row>
     <row r="84" spans="1:24">
       <c r="A84" s="2"/>
       <c r="B84" s="2"/>
       <c r="C84" s="2"/>
       <c r="D84" s="2"/>
-      <c r="E84" s="2"/>
       <c r="S84" s="2"/>
-      <c r="T84" s="2"/>
       <c r="U84" s="2"/>
       <c r="V84" s="2"/>
       <c r="W84" s="2"/>
@@ -4707,6 +4749,7 @@
       <c r="B85" s="2"/>
       <c r="C85" s="2"/>
       <c r="D85" s="2"/>
+      <c r="E85" s="2"/>
       <c r="S85" s="2"/>
       <c r="T85" s="2"/>
       <c r="U85" s="2"/>
@@ -4846,46 +4889,58 @@
       <c r="W96" s="2"/>
       <c r="X96" s="2"/>
     </row>
+    <row r="97" spans="1:24">
+      <c r="A97" s="2"/>
+      <c r="B97" s="2"/>
+      <c r="C97" s="2"/>
+      <c r="D97" s="2"/>
+      <c r="S97" s="2"/>
+      <c r="T97" s="2"/>
+      <c r="U97" s="2"/>
+      <c r="V97" s="2"/>
+      <c r="W97" s="2"/>
+      <c r="X97" s="2"/>
+    </row>
   </sheetData>
   <dataValidations count="13">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H38 H39 H40 H10:H37 H41:H1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C29 C2:C28 C30:C1048576">
+      <formula1>"PC_4,PC_0,PC_ALU,PC_CSR"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="M29 M38 M39 M40 M41 M2:M28 M30:M37 M42:M1048576">
+      <formula1>"CSR_W,CSR_S,CSR_C,CSR_P,CSR_XX"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H29 H39 H40 H41 H10:H28 H30:H38 H42:H1048576">
       <formula1>"WB_ALU,WB_MEM,WB_PC4,WB_XX,WB_CSR"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D4 D5 D6 D7 D8 D9 D10 D11 D12 D13 D14 D15 D16 D17 D18 D19 D20 D21 D22 D23 D24 D25 D26 D27 D28 D29 D30 D31 D32 D33 D34 D35 D36 D37 D38 D39 D40 D2:D3 D41:D1048576">
-      <formula1>"A_PC,A_RS1"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="M37 M38 M39 M40 M2:M36 M41:M1048576">
-      <formula1>"CSR_W,CSR_S,CSR_C,CSR_P,CSR_XX"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="N4 N5 N6 N7 N8 N9 N10 N11 N12 N13 N14 N15 N16 N17 N18 N19 N20 N21 N22 N23 N24 N25 N26 N27 N28 N29 N30 N31 N32 N33 N34 N35 N36 N37 N38 N39 N40 N2:N3 N41:N1048576">
-      <formula1>"INST_VALID,INST_INVALID"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J5 J6 J7 J8 J9 J10 J11 J12 J13 J14 J15 J16 J17 J18 J19 J20 J21 J22 J23 J24 J25 J26 J27 J28 J29 J30 J31 J32 J33 J34 J35 J36 J37 J38 J39 J40 J2:J4 J41:J1048576">
-      <formula1>"ST_SW,ST_SH,ST_SB,ST_XX"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C2:C1048576">
-      <formula1>"PC_4,PC_0,PC_ALU,PC_CSR"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F6 F15 F18 F19 F20 F21 F24 F25 F26 F27 F28 F29 F30 F31 F34 F35 F36 F37 F38 F39 F40 F2:F5 F7:F14 F16:F17 F22:F23 F32:F33 F41:F1048576">
-      <formula1>"ALU_ADD,ALU_SUB,ALU_AND,ALU_OR,ALU_XOR,ALU_SLL,ALU_SRL,ALU_SLT,ALU_SLTU,ALU_COPY_A,ALU_COPY_B,ALU_SRA"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L5 L6 L7 L10 L11 L14 L15 L16 L17 L18 L19 L20 L21 L22 L23 L24 L25 L26 L27 L28 L29 L30 L31 L32 L33 L34 L35 L36 L37 L38 L39 L40 L2:L4 L8:L9 L12:L13 L41:L1048576">
-      <formula1>"BR_EQ,BR_NE,BR_LTU,BR_GE,BR_GEU,BR_LT,BR_XX"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I4 I5 I6 I7 I8 I9 I10 I11 I12 I13 I14 I15 I16 I17 I18 I19 I20 I21 I22 I23 I24 I25 I26 I27 I28 I29 I30 I31 I32 I33 I34 I35 I36 I37 I38 I39 I40 I41 I2:I3 I42:I1048576">
+      <formula1>"LD_LB,LD_LH,LD_LW,LD_LBU,LD_LHU,LD_XX"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H5 H6 H7 H8 H9 H2:H4">
       <formula1>"WB_ALU,WB_MEM,WB_PC4,WB_XX"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K4 K5 K6 K7 K8 K9 K10 K11 K12 K13 K14 K15 K16 K17 K18 K19 K20 K21 K22 K23 K24 K25 K26 K27 K28 K29 K30 K31 K32 K33 K34 K35 K36 K37 K38 K39 K40 K2:K3 K41:K1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L5 L6 L7 L10 L11 L14 L15 L16 L17 L18 L19 L20 L21 L22 L23 L24 L25 L26 L27 L28 L29 L30 L31 L32 L33 L34 L35 L36 L37 L38 L39 L40 L41 L2:L4 L8:L9 L12:L13 L42:L1048576">
+      <formula1>"BR_EQ,BR_NE,BR_LTU,BR_GE,BR_GEU,BR_LT,BR_XX"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="N4 N5 N6 N7 N8 N9 N10 N11 N12 N13 N14 N15 N16 N17 N18 N19 N20 N21 N22 N23 N24 N25 N26 N27 N28 N29 N30 N31 N32 N33 N34 N35 N36 N37 N38 N39 N40 N41 N2:N3 N42:N1048576">
+      <formula1>"INST_VALID,INST_INVALID"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F6 F15 F18 F19 F20 F21 F24 F25 F26 F27 F28 F29 F30 F31 F32 F35 F36 F37 F38 F39 F40 F41 F2:F5 F7:F14 F16:F17 F22:F23 F33:F34 F42:F1048576">
+      <formula1>"ALU_ADD,ALU_SUB,ALU_AND,ALU_OR,ALU_XOR,ALU_SLL,ALU_SRL,ALU_SLT,ALU_SLTU,ALU_COPY_A,ALU_COPY_B,ALU_SRA"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J5 J6 J7 J8 J9 J10 J11 J12 J13 J14 J15 J16 J17 J18 J19 J20 J21 J22 J23 J24 J25 J26 J27 J28 J29 J30 J31 J32 J33 J34 J35 J36 J37 J38 J39 J40 J41 J2:J4 J42:J1048576">
+      <formula1>"ST_SW,ST_SH,ST_SB,ST_XX"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G4 G5 G6 G7 G8 G9 G10 G11 G12 G13 G14 G15 G16 G17 G18 G19 G20 G21 G22 G23 G24 G25 G26 G27 G28 G29 G30 G31 G32 G33 G34 G35 G36 G37 G38 G39 G40 G41 G2:G3 G42:G1048576">
+      <formula1>"IMM_I,IMM_J,IMM_U,IMM_S,IMM_B"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E4 E5 E6 E7 E8 E9 E10 E11 E12 E13 E14 E15 E16 E17 E18 E19 E20 E21 E22 E23 E24 E25 E26 E27 E28 E29 E30 E31 E32 E33 E34 E35 E36 E37 E38 E39 E40 E41 E2:E3 E42:E1048576">
+      <formula1>"B_IMM,B_RS2"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K4 K5 K6 K7 K8 K9 K10 K11 K12 K13 K14 K15 K16 K17 K18 K19 K20 K21 K22 K23 K24 K25 K26 K27 K28 K29 K30 K31 K32 K33 K34 K35 K36 K37 K38 K39 K40 K41 K2:K3 K42:K1048576">
       <formula1>"MASK_XX,MASK_B,MASK_H,MASK_W,MASK_D"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G4 G5 G6 G7 G8 G9 G10 G11 G12 G13 G14 G15 G16 G17 G18 G19 G20 G21 G22 G23 G24 G25 G26 G27 G28 G29 G30 G31 G32 G33 G34 G35 G36 G37 G38 G39 G40 G2:G3 G41:G1048576">
-      <formula1>"IMM_I,IMM_J,IMM_U,IMM_S,IMM_B"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E4 E5 E6 E7 E8 E9 E10 E11 E12 E13 E14 E15 E16 E17 E18 E19 E20 E21 E22 E23 E24 E25 E26 E27 E28 E29 E30 E31 E32 E33 E34 E35 E36 E37 E38 E39 E40 E2:E3 E41:E1048576">
-      <formula1>"B_IMM,B_RS2"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I4 I5 I6 I7 I8 I9 I10 I11 I12 I13 I14 I15 I16 I17 I18 I19 I20 I21 I22 I23 I24 I25 I26 I27 I28 I29 I30 I31 I32 I33 I34 I35 I36 I37 I38 I39 I40 I2:I3 I41:I1048576">
-      <formula1>"LD_LB,LD_LH,LD_LW,LD_LBU,LD_LHU,LD_XX"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D4 D5 D6 D7 D8 D9 D10 D11 D12 D13 D14 D15 D16 D17 D18 D19 D20 D21 D22 D23 D24 D25 D26 D27 D28 D29 D30 D31 D32 D33 D34 D35 D36 D37 D38 D39 D40 D41 D2:D3 D42:D1048576">
+      <formula1>"A_PC,A_RS1"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
> sim RTL ysyx_23060246 韩炳晋 Linux archlinux 6.6.60-1-lts #1 SMP PREEMPT_DYNAMIC Fri, 08 Nov 2024 16:03:02 +0000 x86_64 GNU/Linux  14:10:21 up 5 days,  4:26,  2 users,  load average: 2.40, 3.81, 4.82
</commit_message>
<xml_diff>
--- a/npc/tools/control_gen/control_table.xlsx
+++ b/npc/tools/control_gen/control_table.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="302" uniqueCount="110">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="309" uniqueCount="111">
   <si>
     <t>comment</t>
   </si>
@@ -266,6 +266,9 @@
   </si>
   <si>
     <t>ALU_SLTU</t>
+  </si>
+  <si>
+    <t>slti</t>
   </si>
   <si>
     <t>sltiu</t>
@@ -352,9 +355,9 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="4">
     <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="42" formatCode="_ &quot;￥&quot;* #,##0_ ;_ &quot;￥&quot;* \-#,##0_ ;_ &quot;￥&quot;* &quot;-&quot;_ ;_ @_ "/>
     <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="41" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
+    <numFmt numFmtId="42" formatCode="_ &quot;￥&quot;* #,##0_ ;_ &quot;￥&quot;* \-#,##0_ ;_ &quot;￥&quot;* &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
   <fonts count="22">
     <font>
@@ -384,8 +387,16 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <b/>
       <sz val="11"/>
-      <color theme="1"/>
+      <color theme="3"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="0"/>
       <name val="宋体"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -399,23 +410,9 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <b/>
       <sz val="11"/>
-      <color rgb="FF9C0006"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF0000FF"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="0"/>
+      <color rgb="FF3F3F3F"/>
       <name val="宋体"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -428,25 +425,16 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
+      <u/>
       <sz val="11"/>
-      <color theme="3"/>
+      <color rgb="FF800080"/>
       <name val="宋体"/>
-      <charset val="134"/>
+      <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <sz val="18"/>
-      <color theme="3"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
+      <color theme="1"/>
       <name val="宋体"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -454,7 +442,7 @@
     <font>
       <u/>
       <sz val="11"/>
-      <color rgb="FF800080"/>
+      <color rgb="FF0000FF"/>
       <name val="宋体"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -478,6 +466,29 @@
     <font>
       <b/>
       <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C0006"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
       <color rgb="FFFA7D00"/>
       <name val="宋体"/>
       <charset val="0"/>
@@ -485,17 +496,10 @@
     </font>
     <font>
       <b/>
-      <sz val="11"/>
-      <color rgb="FF3F3F3F"/>
+      <sz val="18"/>
+      <color theme="3"/>
       <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF006100"/>
-      <name val="宋体"/>
-      <charset val="0"/>
+      <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -513,9 +517,8 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
       <sz val="11"/>
-      <color theme="1"/>
+      <color rgb="FF006100"/>
       <name val="宋体"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -530,7 +533,115 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.599993896298105"/>
+        <fgColor theme="8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFA5A5A5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFCC99"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.399975585192419"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -542,19 +653,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.399975585192419"/>
+        <fgColor theme="6" tint="0.799981688894314"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -566,67 +665,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFA5A5A5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor theme="4"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="7"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.799981688894314"/>
+        <fgColor theme="4" tint="0.599993896298105"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -644,25 +689,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.399975585192419"/>
+        <fgColor theme="9" tint="0.599993896298105"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.599993896298105"/>
+        <fgColor theme="6" tint="0.599993896298105"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -674,43 +707,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9"/>
+        <fgColor theme="5" tint="0.599993896298105"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="7" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.799981688894314"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -729,6 +732,15 @@
       <top/>
       <bottom style="double">
         <color rgb="FFFF8001"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4" tint="0.499984740745262"/>
       </bottom>
       <diagonal/>
     </border>
@@ -757,11 +769,17 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4" tint="0.499984740745262"/>
+      <left style="thin">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF3F3F3F"/>
       </bottom>
       <diagonal/>
     </border>
@@ -781,6 +799,17 @@
       <diagonal/>
     </border>
     <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="4"/>
+      </top>
+      <bottom style="double">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
       <left style="thin">
         <color rgb="FF7F7F7F"/>
       </left>
@@ -795,176 +824,150 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color theme="4"/>
-      </top>
-      <bottom style="double">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="23" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="5" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="19" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="5" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="17" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="11" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="17" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="5" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="6" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="11" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="4" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
@@ -1312,7 +1315,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:AI97"/>
+  <dimension ref="A1:AI98"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
     <col min="1" max="1" width="13.1" customWidth="1"/>
@@ -2937,12 +2940,14 @@
         <v>24</v>
       </c>
       <c r="E32" s="4" t="s">
-        <v>76</v>
+        <v>15</v>
       </c>
       <c r="F32" s="4" t="s">
-        <v>79</v>
-      </c>
-      <c r="G32" s="4"/>
+        <v>83</v>
+      </c>
+      <c r="G32" s="4" t="s">
+        <v>25</v>
+      </c>
       <c r="H32" s="4" t="s">
         <v>18</v>
       </c>
@@ -2989,7 +2994,7 @@
         <v>76</v>
       </c>
       <c r="F33" s="4" t="s">
-        <v>22</v>
+        <v>79</v>
       </c>
       <c r="G33" s="4"/>
       <c r="H33" s="4" t="s">
@@ -3038,7 +3043,7 @@
         <v>76</v>
       </c>
       <c r="F34" s="4" t="s">
-        <v>88</v>
+        <v>22</v>
       </c>
       <c r="G34" s="4"/>
       <c r="H34" s="4" t="s">
@@ -3077,7 +3082,7 @@
     <row r="35" spans="1:35">
       <c r="A35" s="3"/>
       <c r="B35" s="4" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C35" s="2"/>
       <c r="D35" s="4" t="s">
@@ -3087,7 +3092,7 @@
         <v>76</v>
       </c>
       <c r="F35" s="4" t="s">
-        <v>31</v>
+        <v>89</v>
       </c>
       <c r="G35" s="4"/>
       <c r="H35" s="4" t="s">
@@ -3136,7 +3141,7 @@
         <v>76</v>
       </c>
       <c r="F36" s="4" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="G36" s="4"/>
       <c r="H36" s="4" t="s">
@@ -3185,7 +3190,7 @@
         <v>76</v>
       </c>
       <c r="F37" s="4" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="G37" s="4"/>
       <c r="H37" s="4" t="s">
@@ -3226,27 +3231,25 @@
       <c r="B38" s="4" t="s">
         <v>92</v>
       </c>
-      <c r="C38" s="2" t="s">
-        <v>93</v>
-      </c>
+      <c r="C38" s="2"/>
       <c r="D38" s="4" t="s">
         <v>24</v>
       </c>
       <c r="E38" s="4" t="s">
         <v>76</v>
       </c>
-      <c r="F38" s="4"/>
+      <c r="F38" s="4" t="s">
+        <v>29</v>
+      </c>
       <c r="G38" s="4"/>
       <c r="H38" s="4" t="s">
-        <v>94</v>
+        <v>18</v>
       </c>
       <c r="I38" s="4"/>
       <c r="J38" s="4"/>
       <c r="K38" s="4"/>
       <c r="L38" s="4"/>
-      <c r="M38" s="4" t="s">
-        <v>95</v>
-      </c>
+      <c r="M38" s="4"/>
       <c r="N38" s="4" t="s">
         <v>19</v>
       </c>
@@ -3275,10 +3278,10 @@
     <row r="39" spans="1:35">
       <c r="A39" s="3"/>
       <c r="B39" s="4" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="D39" s="4" t="s">
         <v>24</v>
@@ -3289,14 +3292,14 @@
       <c r="F39" s="4"/>
       <c r="G39" s="4"/>
       <c r="H39" s="4" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="I39" s="4"/>
       <c r="J39" s="4"/>
       <c r="K39" s="4"/>
       <c r="L39" s="4"/>
       <c r="M39" s="4" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="N39" s="4" t="s">
         <v>19</v>
@@ -3326,24 +3329,28 @@
     <row r="40" spans="1:35">
       <c r="A40" s="3"/>
       <c r="B40" s="4" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>99</v>
-      </c>
-      <c r="D40" s="4"/>
-      <c r="E40" s="4"/>
+        <v>94</v>
+      </c>
+      <c r="D40" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="E40" s="4" t="s">
+        <v>76</v>
+      </c>
       <c r="F40" s="4"/>
       <c r="G40" s="4"/>
       <c r="H40" s="4" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="I40" s="4"/>
       <c r="J40" s="4"/>
       <c r="K40" s="4"/>
       <c r="L40" s="4"/>
       <c r="M40" s="4" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="N40" s="4" t="s">
         <v>19</v>
@@ -3373,24 +3380,24 @@
     <row r="41" spans="1:35">
       <c r="A41" s="3"/>
       <c r="B41" s="4" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="D41" s="4"/>
       <c r="E41" s="4"/>
       <c r="F41" s="4"/>
       <c r="G41" s="4"/>
       <c r="H41" s="4" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="I41" s="4"/>
       <c r="J41" s="4"/>
       <c r="K41" s="4"/>
       <c r="L41" s="4"/>
       <c r="M41" s="4" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="N41" s="4" t="s">
         <v>19</v>
@@ -3417,52 +3424,41 @@
       <c r="AH41" s="3"/>
       <c r="AI41" s="3"/>
     </row>
-    <row r="42" spans="2:35">
-      <c r="B42" s="2" t="s">
+    <row r="42" spans="1:35">
+      <c r="A42" s="3"/>
+      <c r="B42" s="4" t="s">
         <v>102</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>93</v>
-      </c>
-      <c r="D42" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="E42" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="F42" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="G42" s="2" t="s">
-        <v>25</v>
-      </c>
+        <v>100</v>
+      </c>
+      <c r="D42" s="4"/>
+      <c r="E42" s="4"/>
+      <c r="F42" s="4"/>
+      <c r="G42" s="4"/>
       <c r="H42" s="4" t="s">
-        <v>103</v>
-      </c>
-      <c r="I42" s="4" t="s">
-        <v>104</v>
-      </c>
-      <c r="J42" s="4" t="s">
-        <v>105</v>
-      </c>
-      <c r="K42" s="2" t="s">
-        <v>106</v>
-      </c>
-      <c r="L42" s="2" t="s">
-        <v>107</v>
-      </c>
-      <c r="M42" s="2" t="s">
-        <v>108</v>
-      </c>
-      <c r="N42" s="2" t="s">
-        <v>109</v>
-      </c>
-      <c r="O42" s="2"/>
-      <c r="P42" s="2"/>
-      <c r="Q42" s="2"/>
-      <c r="R42" s="2"/>
-      <c r="S42" s="2"/>
-      <c r="T42" s="2"/>
+        <v>95</v>
+      </c>
+      <c r="I42" s="4"/>
+      <c r="J42" s="4"/>
+      <c r="K42" s="4"/>
+      <c r="L42" s="4"/>
+      <c r="M42" s="4" t="s">
+        <v>101</v>
+      </c>
+      <c r="N42" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="O42" s="4"/>
+      <c r="P42" s="4"/>
+      <c r="Q42" s="4"/>
+      <c r="R42" s="4"/>
+      <c r="S42" s="4"/>
+      <c r="T42" s="4"/>
+      <c r="U42" s="3"/>
+      <c r="V42" s="3"/>
+      <c r="W42" s="3"/>
+      <c r="X42" s="3"/>
       <c r="Y42" s="3"/>
       <c r="Z42" s="3"/>
       <c r="AA42" s="3"/>
@@ -3475,31 +3471,52 @@
       <c r="AH42" s="3"/>
       <c r="AI42" s="3"/>
     </row>
-    <row r="43" spans="1:35">
-      <c r="A43" s="3"/>
-      <c r="B43" s="4"/>
-      <c r="C43" s="4"/>
-      <c r="D43" s="4"/>
-      <c r="E43" s="4"/>
-      <c r="F43" s="4"/>
-      <c r="G43" s="4"/>
-      <c r="H43" s="4"/>
-      <c r="I43" s="4"/>
-      <c r="J43" s="4"/>
-      <c r="K43" s="4"/>
-      <c r="L43" s="4"/>
-      <c r="M43" s="4"/>
-      <c r="N43" s="4"/>
-      <c r="O43" s="4"/>
-      <c r="P43" s="4"/>
-      <c r="Q43" s="4"/>
-      <c r="R43" s="4"/>
-      <c r="S43" s="4"/>
-      <c r="T43" s="4"/>
-      <c r="U43" s="3"/>
-      <c r="V43" s="3"/>
-      <c r="W43" s="3"/>
-      <c r="X43" s="3"/>
+    <row r="43" spans="2:35">
+      <c r="B43" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="C43" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="D43" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="E43" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="F43" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="G43" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="H43" s="4" t="s">
+        <v>104</v>
+      </c>
+      <c r="I43" s="4" t="s">
+        <v>105</v>
+      </c>
+      <c r="J43" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="K43" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="L43" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="M43" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="N43" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="O43" s="2"/>
+      <c r="P43" s="2"/>
+      <c r="Q43" s="2"/>
+      <c r="R43" s="2"/>
+      <c r="S43" s="2"/>
+      <c r="T43" s="2"/>
       <c r="Y43" s="3"/>
       <c r="Z43" s="3"/>
       <c r="AA43" s="3"/>
@@ -3512,7 +3529,7 @@
       <c r="AH43" s="3"/>
       <c r="AI43" s="3"/>
     </row>
-    <row r="44" s="1" customFormat="1" spans="1:35">
+    <row r="44" spans="1:35">
       <c r="A44" s="3"/>
       <c r="B44" s="4"/>
       <c r="C44" s="4"/>
@@ -3586,7 +3603,7 @@
       <c r="AH45" s="3"/>
       <c r="AI45" s="3"/>
     </row>
-    <row r="46" spans="1:35">
+    <row r="46" s="1" customFormat="1" spans="1:35">
       <c r="A46" s="3"/>
       <c r="B46" s="4"/>
       <c r="C46" s="4"/>
@@ -4146,7 +4163,7 @@
       <c r="B61" s="4"/>
       <c r="C61" s="4"/>
       <c r="D61" s="4"/>
-      <c r="E61" s="5"/>
+      <c r="E61" s="4"/>
       <c r="F61" s="4"/>
       <c r="G61" s="4"/>
       <c r="H61" s="4"/>
@@ -4257,7 +4274,7 @@
       <c r="B64" s="4"/>
       <c r="C64" s="4"/>
       <c r="D64" s="4"/>
-      <c r="E64" s="4"/>
+      <c r="E64" s="5"/>
       <c r="F64" s="4"/>
       <c r="G64" s="4"/>
       <c r="H64" s="4"/>
@@ -4405,7 +4422,7 @@
       <c r="B68" s="4"/>
       <c r="C68" s="4"/>
       <c r="D68" s="4"/>
-      <c r="E68" s="5"/>
+      <c r="E68" s="4"/>
       <c r="F68" s="4"/>
       <c r="G68" s="4"/>
       <c r="H68" s="4"/>
@@ -4442,7 +4459,7 @@
       <c r="B69" s="4"/>
       <c r="C69" s="4"/>
       <c r="D69" s="4"/>
-      <c r="E69" s="4"/>
+      <c r="E69" s="5"/>
       <c r="F69" s="4"/>
       <c r="G69" s="4"/>
       <c r="H69" s="4"/>
@@ -4733,25 +4750,49 @@
       <c r="AH76" s="3"/>
       <c r="AI76" s="3"/>
     </row>
-    <row r="84" spans="1:24">
-      <c r="A84" s="2"/>
-      <c r="B84" s="2"/>
-      <c r="C84" s="2"/>
-      <c r="D84" s="2"/>
-      <c r="S84" s="2"/>
-      <c r="U84" s="2"/>
-      <c r="V84" s="2"/>
-      <c r="W84" s="2"/>
-      <c r="X84" s="2"/>
+    <row r="77" spans="1:35">
+      <c r="A77" s="3"/>
+      <c r="B77" s="4"/>
+      <c r="C77" s="4"/>
+      <c r="D77" s="4"/>
+      <c r="E77" s="4"/>
+      <c r="F77" s="4"/>
+      <c r="G77" s="4"/>
+      <c r="H77" s="4"/>
+      <c r="I77" s="4"/>
+      <c r="J77" s="4"/>
+      <c r="K77" s="4"/>
+      <c r="L77" s="4"/>
+      <c r="M77" s="4"/>
+      <c r="N77" s="4"/>
+      <c r="O77" s="4"/>
+      <c r="P77" s="4"/>
+      <c r="Q77" s="4"/>
+      <c r="R77" s="4"/>
+      <c r="S77" s="4"/>
+      <c r="T77" s="4"/>
+      <c r="U77" s="3"/>
+      <c r="V77" s="3"/>
+      <c r="W77" s="3"/>
+      <c r="X77" s="3"/>
+      <c r="Y77" s="3"/>
+      <c r="Z77" s="3"/>
+      <c r="AA77" s="3"/>
+      <c r="AB77" s="3"/>
+      <c r="AC77" s="3"/>
+      <c r="AD77" s="3"/>
+      <c r="AE77" s="3"/>
+      <c r="AF77" s="3"/>
+      <c r="AG77" s="3"/>
+      <c r="AH77" s="3"/>
+      <c r="AI77" s="3"/>
     </row>
     <row r="85" spans="1:24">
       <c r="A85" s="2"/>
       <c r="B85" s="2"/>
       <c r="C85" s="2"/>
       <c r="D85" s="2"/>
-      <c r="E85" s="2"/>
       <c r="S85" s="2"/>
-      <c r="T85" s="2"/>
       <c r="U85" s="2"/>
       <c r="V85" s="2"/>
       <c r="W85" s="2"/>
@@ -4762,6 +4803,7 @@
       <c r="B86" s="2"/>
       <c r="C86" s="2"/>
       <c r="D86" s="2"/>
+      <c r="E86" s="2"/>
       <c r="S86" s="2"/>
       <c r="T86" s="2"/>
       <c r="U86" s="2"/>
@@ -4901,46 +4943,58 @@
       <c r="W97" s="2"/>
       <c r="X97" s="2"/>
     </row>
+    <row r="98" spans="1:24">
+      <c r="A98" s="2"/>
+      <c r="B98" s="2"/>
+      <c r="C98" s="2"/>
+      <c r="D98" s="2"/>
+      <c r="S98" s="2"/>
+      <c r="T98" s="2"/>
+      <c r="U98" s="2"/>
+      <c r="V98" s="2"/>
+      <c r="W98" s="2"/>
+      <c r="X98" s="2"/>
+    </row>
   </sheetData>
   <dataValidations count="13">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C29 C2:C28 C30:C1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G4 G5 G6 G7 G8 G9 G10 G11 G12 G13 G14 G15 G16 G17 G18 G19 G20 G21 G22 G23 G24 G25 G26 G27 G28 G29 G30 G31 G32 G33 G34 G35 G36 G37 G38 G39 G40 G41 G42 G2:G3 G43:G1048576">
+      <formula1>"IMM_I,IMM_J,IMM_U,IMM_S,IMM_B"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C29 C30 C31 C2:C28 C32:C1048576">
       <formula1>"PC_4,PC_0,PC_ALU,PC_CSR"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="M29 M38 M39 M40 M41 M2:M28 M30:M37 M42:M1048576">
-      <formula1>"CSR_W,CSR_S,CSR_C,CSR_P,CSR_XX"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H29 H39 H40 H41 H10:H28 H30:H38 H42:H1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H29 H30 H31 H40 H41 H42 H10:H28 H32:H39 H43:H1048576">
       <formula1>"WB_ALU,WB_MEM,WB_PC4,WB_XX,WB_CSR"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I4 I5 I6 I7 I8 I9 I10 I11 I12 I13 I14 I15 I16 I17 I18 I19 I20 I21 I22 I23 I24 I25 I26 I27 I28 I29 I30 I31 I32 I33 I34 I35 I36 I37 I38 I39 I40 I41 I2:I3 I42:I1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I4 I5 I6 I7 I8 I9 I10 I11 I12 I13 I14 I15 I16 I17 I18 I19 I20 I21 I22 I23 I24 I25 I26 I27 I28 I29 I30 I31 I32 I33 I34 I35 I36 I37 I38 I39 I40 I41 I42 I2:I3 I43:I1048576">
       <formula1>"LD_LB,LD_LH,LD_LW,LD_LBU,LD_LHU,LD_XX"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L5 L6 L7 L10 L11 L14 L15 L16 L17 L18 L19 L20 L21 L22 L23 L24 L25 L26 L27 L28 L29 L30 L31 L32 L33 L34 L35 L36 L37 L38 L39 L40 L41 L42 L2:L4 L8:L9 L12:L13 L43:L1048576">
+      <formula1>"BR_EQ,BR_NE,BR_LTU,BR_GE,BR_GEU,BR_LT,BR_XX"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="M29 M30 M31 M39 M40 M41 M42 M2:M28 M32:M38 M43:M1048576">
+      <formula1>"CSR_W,CSR_S,CSR_C,CSR_P,CSR_XX"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H5 H6 H7 H8 H9 H2:H4">
       <formula1>"WB_ALU,WB_MEM,WB_PC4,WB_XX"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L5 L6 L7 L10 L11 L14 L15 L16 L17 L18 L19 L20 L21 L22 L23 L24 L25 L26 L27 L28 L29 L30 L31 L32 L33 L34 L35 L36 L37 L38 L39 L40 L41 L2:L4 L8:L9 L12:L13 L42:L1048576">
-      <formula1>"BR_EQ,BR_NE,BR_LTU,BR_GE,BR_GEU,BR_LT,BR_XX"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E4 E5 E6 E7 E8 E9 E10 E11 E12 E13 E14 E15 E16 E17 E18 E19 E20 E21 E22 E23 E24 E25 E26 E27 E28 E29 E30 E31 E32 E33 E34 E35 E36 E37 E38 E39 E40 E41 E42 E2:E3 E43:E1048576">
+      <formula1>"B_IMM,B_RS2"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="N4 N5 N6 N7 N8 N9 N10 N11 N12 N13 N14 N15 N16 N17 N18 N19 N20 N21 N22 N23 N24 N25 N26 N27 N28 N29 N30 N31 N32 N33 N34 N35 N36 N37 N38 N39 N40 N41 N2:N3 N42:N1048576">
-      <formula1>"INST_VALID,INST_INVALID"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F6 F15 F18 F19 F20 F21 F24 F25 F26 F27 F28 F29 F30 F31 F32 F35 F36 F37 F38 F39 F40 F41 F2:F5 F7:F14 F16:F17 F22:F23 F33:F34 F42:F1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F6 F15 F18 F19 F20 F21 F24 F25 F26 F27 F28 F29 F30 F31 F32 F33 F36 F37 F38 F39 F40 F41 F42 F2:F5 F7:F14 F16:F17 F22:F23 F34:F35 F43:F1048576">
       <formula1>"ALU_ADD,ALU_SUB,ALU_AND,ALU_OR,ALU_XOR,ALU_SLL,ALU_SRL,ALU_SLT,ALU_SLTU,ALU_COPY_A,ALU_COPY_B,ALU_SRA"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J5 J6 J7 J8 J9 J10 J11 J12 J13 J14 J15 J16 J17 J18 J19 J20 J21 J22 J23 J24 J25 J26 J27 J28 J29 J30 J31 J32 J33 J34 J35 J36 J37 J38 J39 J40 J41 J2:J4 J42:J1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J5 J6 J7 J8 J9 J10 J11 J12 J13 J14 J15 J16 J17 J18 J19 J20 J21 J22 J23 J24 J25 J26 J27 J28 J29 J30 J31 J32 J33 J34 J35 J36 J37 J38 J39 J40 J41 J42 J2:J4 J43:J1048576">
       <formula1>"ST_SW,ST_SH,ST_SB,ST_XX"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G4 G5 G6 G7 G8 G9 G10 G11 G12 G13 G14 G15 G16 G17 G18 G19 G20 G21 G22 G23 G24 G25 G26 G27 G28 G29 G30 G31 G32 G33 G34 G35 G36 G37 G38 G39 G40 G41 G2:G3 G42:G1048576">
-      <formula1>"IMM_I,IMM_J,IMM_U,IMM_S,IMM_B"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D4 D5 D6 D7 D8 D9 D10 D11 D12 D13 D14 D15 D16 D17 D18 D19 D20 D21 D22 D23 D24 D25 D26 D27 D28 D29 D30 D31 D32 D33 D34 D35 D36 D37 D38 D39 D40 D41 D42 D2:D3 D43:D1048576">
+      <formula1>"A_PC,A_RS1"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E4 E5 E6 E7 E8 E9 E10 E11 E12 E13 E14 E15 E16 E17 E18 E19 E20 E21 E22 E23 E24 E25 E26 E27 E28 E29 E30 E31 E32 E33 E34 E35 E36 E37 E38 E39 E40 E41 E2:E3 E42:E1048576">
-      <formula1>"B_IMM,B_RS2"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K4 K5 K6 K7 K8 K9 K10 K11 K12 K13 K14 K15 K16 K17 K18 K19 K20 K21 K22 K23 K24 K25 K26 K27 K28 K29 K30 K31 K32 K33 K34 K35 K36 K37 K38 K39 K40 K41 K2:K3 K42:K1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K4 K5 K6 K7 K8 K9 K10 K11 K12 K13 K14 K15 K16 K17 K18 K19 K20 K21 K22 K23 K24 K25 K26 K27 K28 K29 K30 K31 K32 K33 K34 K35 K36 K37 K38 K39 K40 K41 K42 K2:K3 K43:K1048576">
       <formula1>"MASK_XX,MASK_B,MASK_H,MASK_W,MASK_D"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D4 D5 D6 D7 D8 D9 D10 D11 D12 D13 D14 D15 D16 D17 D18 D19 D20 D21 D22 D23 D24 D25 D26 D27 D28 D29 D30 D31 D32 D33 D34 D35 D36 D37 D38 D39 D40 D41 D2:D3 D42:D1048576">
-      <formula1>"A_PC,A_RS1"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="N4 N5 N6 N7 N8 N9 N10 N11 N12 N13 N14 N15 N16 N17 N18 N19 N20 N21 N22 N23 N24 N25 N26 N27 N28 N29 N30 N31 N32 N33 N34 N35 N36 N37 N38 N39 N40 N41 N42 N2:N3 N43:N1048576">
+      <formula1>"INST_VALID,INST_INVALID"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
> sim RTL ysyx_23060246 韩炳晋 Linux archlinux 6.6.60-1-lts #1 SMP PREEMPT_DYNAMIC Fri, 08 Nov 2024 16:03:02 +0000 x86_64 GNU/Linux  22:00:20 up 1 day,  4:41,  2 users,  load average: 2.47, 1.88, 1.56
</commit_message>
<xml_diff>
--- a/npc/tools/control_gen/control_table.xlsx
+++ b/npc/tools/control_gen/control_table.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="27795" windowHeight="12075"/>
+    <workbookView windowWidth="23370" windowHeight="12150"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="309" uniqueCount="111">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="311" uniqueCount="112">
   <si>
     <t>comment</t>
   </si>
@@ -323,6 +323,9 @@
   </si>
   <si>
     <t>mret</t>
+  </si>
+  <si>
+    <t>fencei</t>
   </si>
   <si>
     <t>default</t>
@@ -396,23 +399,14 @@
     </font>
     <font>
       <sz val="11"/>
-      <color theme="0"/>
+      <color theme="1"/>
       <name val="宋体"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <sz val="13"/>
-      <color theme="3"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
-      <color rgb="FF3F3F3F"/>
+      <color theme="0"/>
       <name val="宋体"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -425,24 +419,17 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF800080"/>
+      <b/>
+      <sz val="18"/>
+      <color theme="3"/>
       <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="宋体"/>
-      <charset val="0"/>
+      <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
       <u/>
       <sz val="11"/>
-      <color rgb="FF0000FF"/>
+      <color rgb="FF800080"/>
       <name val="宋体"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -466,6 +453,14 @@
     <font>
       <b/>
       <sz val="11"/>
+      <color rgb="FF3F3F3F"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
       <color rgb="FFFFFFFF"/>
       <name val="宋体"/>
       <charset val="0"/>
@@ -481,25 +476,16 @@
     <font>
       <b/>
       <sz val="11"/>
-      <color theme="1"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
       <color rgb="FFFA7D00"/>
       <name val="宋体"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <sz val="18"/>
-      <color theme="3"/>
+      <sz val="11"/>
+      <color rgb="FF3F3F76"/>
       <name val="宋体"/>
-      <charset val="134"/>
+      <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -510,8 +496,25 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <b/>
+      <sz val="13"/>
+      <color theme="3"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
       <sz val="11"/>
-      <color rgb="FF3F3F76"/>
+      <color rgb="FF0000FF"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="宋体"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -533,7 +536,19 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor theme="8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -545,43 +560,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
+        <fgColor theme="7" tint="0.599993896298105"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFF2F2F2"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.799981688894314"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -599,7 +584,115 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FFFFCC99"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor theme="4" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.799981688894314"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -611,85 +704,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.599993896298105"/>
+        <fgColor theme="5" tint="0.599993896298105"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -701,19 +716,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.799981688894314"/>
+        <fgColor rgb="FFC6EFCE"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -745,15 +748,6 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
       <left style="thin">
         <color rgb="FFB2B2B2"/>
       </left>
@@ -765,6 +759,15 @@
       </top>
       <bottom style="thin">
         <color rgb="FFB2B2B2"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4"/>
       </bottom>
       <diagonal/>
     </border>
@@ -799,17 +802,6 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color theme="4"/>
-      </top>
-      <bottom style="double">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
       <left style="thin">
         <color rgb="FF7F7F7F"/>
       </left>
@@ -824,150 +816,161 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="4"/>
+      </top>
+      <bottom style="double">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="19" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="6" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="10" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="6" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="7" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="8" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="7" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="6" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="11" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="4" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
@@ -1315,7 +1318,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:AI98"/>
+  <dimension ref="A1:AI99"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
     <col min="1" max="1" width="13.1" customWidth="1"/>
@@ -3475,41 +3478,19 @@
       <c r="B43" s="2" t="s">
         <v>103</v>
       </c>
-      <c r="C43" s="2" t="s">
-        <v>94</v>
-      </c>
-      <c r="D43" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="E43" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="F43" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="G43" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="H43" s="4" t="s">
-        <v>104</v>
-      </c>
-      <c r="I43" s="4" t="s">
-        <v>105</v>
-      </c>
-      <c r="J43" s="4" t="s">
-        <v>106</v>
-      </c>
-      <c r="K43" s="2" t="s">
-        <v>107</v>
-      </c>
-      <c r="L43" s="2" t="s">
-        <v>108</v>
-      </c>
-      <c r="M43" s="2" t="s">
-        <v>109</v>
-      </c>
+      <c r="C43" s="2"/>
+      <c r="D43" s="2"/>
+      <c r="E43" s="2"/>
+      <c r="F43" s="2"/>
+      <c r="G43" s="2"/>
+      <c r="H43" s="4"/>
+      <c r="I43" s="4"/>
+      <c r="J43" s="4"/>
+      <c r="K43" s="2"/>
+      <c r="L43" s="2"/>
+      <c r="M43" s="2"/>
       <c r="N43" s="2" t="s">
-        <v>110</v>
+        <v>19</v>
       </c>
       <c r="O43" s="2"/>
       <c r="P43" s="2"/>
@@ -3529,31 +3510,52 @@
       <c r="AH43" s="3"/>
       <c r="AI43" s="3"/>
     </row>
-    <row r="44" spans="1:35">
-      <c r="A44" s="3"/>
-      <c r="B44" s="4"/>
-      <c r="C44" s="4"/>
-      <c r="D44" s="4"/>
-      <c r="E44" s="4"/>
-      <c r="F44" s="4"/>
-      <c r="G44" s="4"/>
-      <c r="H44" s="4"/>
-      <c r="I44" s="4"/>
-      <c r="J44" s="4"/>
-      <c r="K44" s="4"/>
-      <c r="L44" s="4"/>
-      <c r="M44" s="4"/>
-      <c r="N44" s="4"/>
-      <c r="O44" s="4"/>
-      <c r="P44" s="4"/>
-      <c r="Q44" s="4"/>
-      <c r="R44" s="4"/>
-      <c r="S44" s="4"/>
-      <c r="T44" s="4"/>
-      <c r="U44" s="3"/>
-      <c r="V44" s="3"/>
-      <c r="W44" s="3"/>
-      <c r="X44" s="3"/>
+    <row r="44" spans="2:35">
+      <c r="B44" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="C44" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="D44" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="E44" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="F44" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="G44" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="H44" s="4" t="s">
+        <v>105</v>
+      </c>
+      <c r="I44" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="J44" s="4" t="s">
+        <v>107</v>
+      </c>
+      <c r="K44" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="L44" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="M44" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="N44" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="O44" s="2"/>
+      <c r="P44" s="2"/>
+      <c r="Q44" s="2"/>
+      <c r="R44" s="2"/>
+      <c r="S44" s="2"/>
+      <c r="T44" s="2"/>
       <c r="Y44" s="3"/>
       <c r="Z44" s="3"/>
       <c r="AA44" s="3"/>
@@ -3566,7 +3568,7 @@
       <c r="AH44" s="3"/>
       <c r="AI44" s="3"/>
     </row>
-    <row r="45" s="1" customFormat="1" spans="1:35">
+    <row r="45" spans="1:35">
       <c r="A45" s="3"/>
       <c r="B45" s="4"/>
       <c r="C45" s="4"/>
@@ -3640,7 +3642,7 @@
       <c r="AH46" s="3"/>
       <c r="AI46" s="3"/>
     </row>
-    <row r="47" spans="1:35">
+    <row r="47" s="1" customFormat="1" spans="1:35">
       <c r="A47" s="3"/>
       <c r="B47" s="4"/>
       <c r="C47" s="4"/>
@@ -4200,7 +4202,7 @@
       <c r="B62" s="4"/>
       <c r="C62" s="4"/>
       <c r="D62" s="4"/>
-      <c r="E62" s="5"/>
+      <c r="E62" s="4"/>
       <c r="F62" s="4"/>
       <c r="G62" s="4"/>
       <c r="H62" s="4"/>
@@ -4311,7 +4313,7 @@
       <c r="B65" s="4"/>
       <c r="C65" s="4"/>
       <c r="D65" s="4"/>
-      <c r="E65" s="4"/>
+      <c r="E65" s="5"/>
       <c r="F65" s="4"/>
       <c r="G65" s="4"/>
       <c r="H65" s="4"/>
@@ -4459,7 +4461,7 @@
       <c r="B69" s="4"/>
       <c r="C69" s="4"/>
       <c r="D69" s="4"/>
-      <c r="E69" s="5"/>
+      <c r="E69" s="4"/>
       <c r="F69" s="4"/>
       <c r="G69" s="4"/>
       <c r="H69" s="4"/>
@@ -4496,7 +4498,7 @@
       <c r="B70" s="4"/>
       <c r="C70" s="4"/>
       <c r="D70" s="4"/>
-      <c r="E70" s="4"/>
+      <c r="E70" s="5"/>
       <c r="F70" s="4"/>
       <c r="G70" s="4"/>
       <c r="H70" s="4"/>
@@ -4787,25 +4789,49 @@
       <c r="AH77" s="3"/>
       <c r="AI77" s="3"/>
     </row>
-    <row r="85" spans="1:24">
-      <c r="A85" s="2"/>
-      <c r="B85" s="2"/>
-      <c r="C85" s="2"/>
-      <c r="D85" s="2"/>
-      <c r="S85" s="2"/>
-      <c r="U85" s="2"/>
-      <c r="V85" s="2"/>
-      <c r="W85" s="2"/>
-      <c r="X85" s="2"/>
+    <row r="78" spans="1:35">
+      <c r="A78" s="3"/>
+      <c r="B78" s="4"/>
+      <c r="C78" s="4"/>
+      <c r="D78" s="4"/>
+      <c r="E78" s="4"/>
+      <c r="F78" s="4"/>
+      <c r="G78" s="4"/>
+      <c r="H78" s="4"/>
+      <c r="I78" s="4"/>
+      <c r="J78" s="4"/>
+      <c r="K78" s="4"/>
+      <c r="L78" s="4"/>
+      <c r="M78" s="4"/>
+      <c r="N78" s="4"/>
+      <c r="O78" s="4"/>
+      <c r="P78" s="4"/>
+      <c r="Q78" s="4"/>
+      <c r="R78" s="4"/>
+      <c r="S78" s="4"/>
+      <c r="T78" s="4"/>
+      <c r="U78" s="3"/>
+      <c r="V78" s="3"/>
+      <c r="W78" s="3"/>
+      <c r="X78" s="3"/>
+      <c r="Y78" s="3"/>
+      <c r="Z78" s="3"/>
+      <c r="AA78" s="3"/>
+      <c r="AB78" s="3"/>
+      <c r="AC78" s="3"/>
+      <c r="AD78" s="3"/>
+      <c r="AE78" s="3"/>
+      <c r="AF78" s="3"/>
+      <c r="AG78" s="3"/>
+      <c r="AH78" s="3"/>
+      <c r="AI78" s="3"/>
     </row>
     <row r="86" spans="1:24">
       <c r="A86" s="2"/>
       <c r="B86" s="2"/>
       <c r="C86" s="2"/>
       <c r="D86" s="2"/>
-      <c r="E86" s="2"/>
       <c r="S86" s="2"/>
-      <c r="T86" s="2"/>
       <c r="U86" s="2"/>
       <c r="V86" s="2"/>
       <c r="W86" s="2"/>
@@ -4816,6 +4842,7 @@
       <c r="B87" s="2"/>
       <c r="C87" s="2"/>
       <c r="D87" s="2"/>
+      <c r="E87" s="2"/>
       <c r="S87" s="2"/>
       <c r="T87" s="2"/>
       <c r="U87" s="2"/>
@@ -4955,46 +4982,58 @@
       <c r="W98" s="2"/>
       <c r="X98" s="2"/>
     </row>
+    <row r="99" spans="1:24">
+      <c r="A99" s="2"/>
+      <c r="B99" s="2"/>
+      <c r="C99" s="2"/>
+      <c r="D99" s="2"/>
+      <c r="S99" s="2"/>
+      <c r="T99" s="2"/>
+      <c r="U99" s="2"/>
+      <c r="V99" s="2"/>
+      <c r="W99" s="2"/>
+      <c r="X99" s="2"/>
+    </row>
   </sheetData>
   <dataValidations count="13">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G4 G5 G6 G7 G8 G9 G10 G11 G12 G13 G14 G15 G16 G17 G18 G19 G20 G21 G22 G23 G24 G25 G26 G27 G28 G29 G30 G31 G32 G33 G34 G35 G36 G37 G38 G39 G40 G41 G42 G2:G3 G43:G1048576">
-      <formula1>"IMM_I,IMM_J,IMM_U,IMM_S,IMM_B"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H29 H30 H31 H40 H41 H42 H43 H10:H28 H32:H39 H44:H1048576">
+      <formula1>"WB_ALU,WB_MEM,WB_PC4,WB_XX,WB_CSR"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C29 C30 C31 C2:C28 C32:C1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F6 F15 F18 F19 F20 F21 F24 F25 F26 F27 F28 F29 F30 F31 F32 F33 F36 F37 F38 F39 F40 F41 F42 F43 F2:F5 F7:F14 F16:F17 F22:F23 F34:F35 F44:F1048576">
+      <formula1>"ALU_ADD,ALU_SUB,ALU_AND,ALU_OR,ALU_XOR,ALU_SLL,ALU_SRL,ALU_SLT,ALU_SLTU,ALU_COPY_A,ALU_COPY_B,ALU_SRA"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L5 L6 L7 L10 L11 L14 L15 L16 L17 L18 L19 L20 L21 L22 L23 L24 L25 L26 L27 L28 L29 L30 L31 L32 L33 L34 L35 L36 L37 L38 L39 L40 L41 L42 L43 L2:L4 L8:L9 L12:L13 L44:L1048576">
+      <formula1>"BR_EQ,BR_NE,BR_LTU,BR_GE,BR_GEU,BR_LT,BR_XX"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C29 C30 C31 C43 C2:C28 C32:C42 C44:C1048576">
       <formula1>"PC_4,PC_0,PC_ALU,PC_CSR"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H29 H30 H31 H40 H41 H42 H10:H28 H32:H39 H43:H1048576">
-      <formula1>"WB_ALU,WB_MEM,WB_PC4,WB_XX,WB_CSR"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="N4 N5 N6 N7 N8 N9 N10 N11 N12 N13 N14 N15 N16 N17 N18 N19 N20 N21 N22 N23 N24 N25 N26 N27 N28 N29 N30 N31 N32 N33 N34 N35 N36 N37 N38 N39 N40 N41 N42 N43 N2:N3 N44:N1048576">
+      <formula1>"INST_VALID,INST_INVALID"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I4 I5 I6 I7 I8 I9 I10 I11 I12 I13 I14 I15 I16 I17 I18 I19 I20 I21 I22 I23 I24 I25 I26 I27 I28 I29 I30 I31 I32 I33 I34 I35 I36 I37 I38 I39 I40 I41 I42 I2:I3 I43:I1048576">
-      <formula1>"LD_LB,LD_LH,LD_LW,LD_LBU,LD_LHU,LD_XX"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D4 D5 D6 D7 D8 D9 D10 D11 D12 D13 D14 D15 D16 D17 D18 D19 D20 D21 D22 D23 D24 D25 D26 D27 D28 D29 D30 D31 D32 D33 D34 D35 D36 D37 D38 D39 D40 D41 D42 D43 D2:D3 D44:D1048576">
+      <formula1>"A_PC,A_RS1"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L5 L6 L7 L10 L11 L14 L15 L16 L17 L18 L19 L20 L21 L22 L23 L24 L25 L26 L27 L28 L29 L30 L31 L32 L33 L34 L35 L36 L37 L38 L39 L40 L41 L42 L2:L4 L8:L9 L12:L13 L43:L1048576">
-      <formula1>"BR_EQ,BR_NE,BR_LTU,BR_GE,BR_GEU,BR_LT,BR_XX"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="M29 M30 M31 M39 M40 M41 M42 M2:M28 M32:M38 M43:M1048576">
-      <formula1>"CSR_W,CSR_S,CSR_C,CSR_P,CSR_XX"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J5 J6 J7 J8 J9 J10 J11 J12 J13 J14 J15 J16 J17 J18 J19 J20 J21 J22 J23 J24 J25 J26 J27 J28 J29 J30 J31 J32 J33 J34 J35 J36 J37 J38 J39 J40 J41 J42 J43 J2:J4 J44:J1048576">
+      <formula1>"ST_SW,ST_SH,ST_SB,ST_XX"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H5 H6 H7 H8 H9 H2:H4">
       <formula1>"WB_ALU,WB_MEM,WB_PC4,WB_XX"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E4 E5 E6 E7 E8 E9 E10 E11 E12 E13 E14 E15 E16 E17 E18 E19 E20 E21 E22 E23 E24 E25 E26 E27 E28 E29 E30 E31 E32 E33 E34 E35 E36 E37 E38 E39 E40 E41 E42 E2:E3 E43:E1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K4 K5 K6 K7 K8 K9 K10 K11 K12 K13 K14 K15 K16 K17 K18 K19 K20 K21 K22 K23 K24 K25 K26 K27 K28 K29 K30 K31 K32 K33 K34 K35 K36 K37 K38 K39 K40 K41 K42 K43 K2:K3 K44:K1048576">
+      <formula1>"MASK_XX,MASK_B,MASK_H,MASK_W,MASK_D"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E4 E5 E6 E7 E8 E9 E10 E11 E12 E13 E14 E15 E16 E17 E18 E19 E20 E21 E22 E23 E24 E25 E26 E27 E28 E29 E30 E31 E32 E33 E34 E35 E36 E37 E38 E39 E40 E41 E42 E43 E2:E3 E44:E1048576">
       <formula1>"B_IMM,B_RS2"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F6 F15 F18 F19 F20 F21 F24 F25 F26 F27 F28 F29 F30 F31 F32 F33 F36 F37 F38 F39 F40 F41 F42 F2:F5 F7:F14 F16:F17 F22:F23 F34:F35 F43:F1048576">
-      <formula1>"ALU_ADD,ALU_SUB,ALU_AND,ALU_OR,ALU_XOR,ALU_SLL,ALU_SRL,ALU_SLT,ALU_SLTU,ALU_COPY_A,ALU_COPY_B,ALU_SRA"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="M29 M30 M31 M39 M40 M41 M42 M43 M2:M28 M32:M38 M44:M1048576">
+      <formula1>"CSR_W,CSR_S,CSR_C,CSR_P,CSR_XX"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J5 J6 J7 J8 J9 J10 J11 J12 J13 J14 J15 J16 J17 J18 J19 J20 J21 J22 J23 J24 J25 J26 J27 J28 J29 J30 J31 J32 J33 J34 J35 J36 J37 J38 J39 J40 J41 J42 J2:J4 J43:J1048576">
-      <formula1>"ST_SW,ST_SH,ST_SB,ST_XX"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I4 I5 I6 I7 I8 I9 I10 I11 I12 I13 I14 I15 I16 I17 I18 I19 I20 I21 I22 I23 I24 I25 I26 I27 I28 I29 I30 I31 I32 I33 I34 I35 I36 I37 I38 I39 I40 I41 I42 I43 I2:I3 I44:I1048576">
+      <formula1>"LD_LB,LD_LH,LD_LW,LD_LBU,LD_LHU,LD_XX"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D4 D5 D6 D7 D8 D9 D10 D11 D12 D13 D14 D15 D16 D17 D18 D19 D20 D21 D22 D23 D24 D25 D26 D27 D28 D29 D30 D31 D32 D33 D34 D35 D36 D37 D38 D39 D40 D41 D42 D2:D3 D43:D1048576">
-      <formula1>"A_PC,A_RS1"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K4 K5 K6 K7 K8 K9 K10 K11 K12 K13 K14 K15 K16 K17 K18 K19 K20 K21 K22 K23 K24 K25 K26 K27 K28 K29 K30 K31 K32 K33 K34 K35 K36 K37 K38 K39 K40 K41 K42 K2:K3 K43:K1048576">
-      <formula1>"MASK_XX,MASK_B,MASK_H,MASK_W,MASK_D"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="N4 N5 N6 N7 N8 N9 N10 N11 N12 N13 N14 N15 N16 N17 N18 N19 N20 N21 N22 N23 N24 N25 N26 N27 N28 N29 N30 N31 N32 N33 N34 N35 N36 N37 N38 N39 N40 N41 N42 N2:N3 N43:N1048576">
-      <formula1>"INST_VALID,INST_INVALID"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G4 G5 G6 G7 G8 G9 G10 G11 G12 G13 G14 G15 G16 G17 G18 G19 G20 G21 G22 G23 G24 G25 G26 G27 G28 G29 G30 G31 G32 G33 G34 G35 G36 G37 G38 G39 G40 G41 G42 G43 G2:G3 G44:G1048576">
+      <formula1>"IMM_I,IMM_J,IMM_U,IMM_S,IMM_B"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
> sim RTL ysyx_23060246 韩炳晋 Linux archlinux 6.6.68-1-lts #1 SMP PREEMPT_DYNAMIC Fri, 27 Dec 2024 15:16:06 +0000 x86_64 GNU/Linux  18:52:49 up  1:34,  1 user,  load average: 2.14, 2.40, 2.30
</commit_message>
<xml_diff>
--- a/npc/tools/control_gen/control_table.xlsx
+++ b/npc/tools/control_gen/control_table.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="311" uniqueCount="112">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="355" uniqueCount="119">
   <si>
     <t>comment</t>
   </si>
@@ -76,6 +76,9 @@
     <t>INST_VALID</t>
   </si>
   <si>
+    <t>U_TYPE</t>
+  </si>
+  <si>
     <t>auipc</t>
   </si>
   <si>
@@ -94,6 +97,9 @@
     <t>IMM_I</t>
   </si>
   <si>
+    <t>I_TYPE</t>
+  </si>
+  <si>
     <t>andi</t>
   </si>
   <si>
@@ -127,6 +133,9 @@
     <t>IMM_J</t>
   </si>
   <si>
+    <t>J_TYPE</t>
+  </si>
+  <si>
     <t>sb</t>
   </si>
   <si>
@@ -139,6 +148,9 @@
     <t>MASK_B</t>
   </si>
   <si>
+    <t>S_TYPE</t>
+  </si>
+  <si>
     <t>sh</t>
   </si>
   <si>
@@ -199,6 +211,9 @@
     <t>BR_NE</t>
   </si>
   <si>
+    <t>B_TYPE</t>
+  </si>
+  <si>
     <t>beq</t>
   </si>
   <si>
@@ -247,6 +262,9 @@
     <t>B_RS2</t>
   </si>
   <si>
+    <t>R_TYPE</t>
+  </si>
+  <si>
     <t>sra</t>
   </si>
   <si>
@@ -320,6 +338,9 @@
   </si>
   <si>
     <t>CSR_P</t>
+  </si>
+  <si>
+    <t>N_TYPE</t>
   </si>
   <si>
     <t>mret</t>
@@ -358,9 +379,9 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="4">
     <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="42" formatCode="_ &quot;￥&quot;* #,##0_ ;_ &quot;￥&quot;* \-#,##0_ ;_ &quot;￥&quot;* &quot;-&quot;_ ;_ @_ "/>
     <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="41" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="42" formatCode="_ &quot;￥&quot;* #,##0_ ;_ &quot;￥&quot;* \-#,##0_ ;_ &quot;￥&quot;* &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
   <fonts count="22">
     <font>
@@ -378,21 +399,6 @@
     </font>
     <font>
       <sz val="10.8"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="3"/>
       <name val="宋体"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -419,6 +425,29 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF0000FF"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="3"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <b/>
       <sz val="18"/>
       <color theme="3"/>
@@ -432,22 +461,6 @@
       <color rgb="FF800080"/>
       <name val="宋体"/>
       <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="11"/>
-      <color rgb="FF7F7F7F"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="15"/>
-      <color theme="3"/>
-      <name val="宋体"/>
-      <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -476,14 +489,7 @@
     <font>
       <b/>
       <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF3F3F76"/>
+      <color theme="1"/>
       <name val="宋体"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -497,6 +503,21 @@
     </font>
     <font>
       <b/>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF006100"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="13"/>
       <color theme="3"/>
       <name val="宋体"/>
@@ -504,24 +525,24 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF0000FF"/>
+      <b/>
+      <sz val="15"/>
+      <color theme="3"/>
       <name val="宋体"/>
-      <charset val="0"/>
+      <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
+      <i/>
       <sz val="11"/>
-      <color theme="1"/>
+      <color rgb="FF7F7F7F"/>
       <name val="宋体"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FF006100"/>
+      <color rgb="FF3F3F76"/>
       <name val="宋体"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -536,7 +557,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.599993896298105"/>
+        <fgColor theme="4" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -554,19 +581,67 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="9"/>
+        <fgColor theme="5" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="7" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -584,25 +659,61 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor theme="4" tint="0.799981688894314"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.799981688894314"/>
+        <fgColor theme="6" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.799981688894314"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -614,37 +725,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.399975585192419"/>
+        <fgColor rgb="FFFFCC99"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -656,67 +737,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor theme="9" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -727,24 +748,6 @@
       <right/>
       <top/>
       <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="double">
-        <color rgb="FFFF8001"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4" tint="0.499984740745262"/>
-      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -766,8 +769,17 @@
       <left/>
       <right/>
       <top/>
+      <bottom style="double">
+        <color rgb="FFFF8001"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
       <bottom style="medium">
-        <color theme="4"/>
+        <color theme="4" tint="0.499984740745262"/>
       </bottom>
       <diagonal/>
     </border>
@@ -802,6 +814,17 @@
       <diagonal/>
     </border>
     <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="4"/>
+      </top>
+      <bottom style="double">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
       <left style="thin">
         <color rgb="FF7F7F7F"/>
       </left>
@@ -819,10 +842,8 @@
     <border>
       <left/>
       <right/>
-      <top style="thin">
-        <color theme="4"/>
-      </top>
-      <bottom style="double">
+      <top/>
+      <bottom style="medium">
         <color theme="4"/>
       </bottom>
       <diagonal/>
@@ -832,148 +853,148 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="10" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="4" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="30" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="4" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="7" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="8" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="7" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="15" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="17" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="15" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
@@ -1318,7 +1339,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:AI99"/>
+  <dimension ref="A1:AJ99"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
     <col min="1" max="1" width="13.1" customWidth="1"/>
@@ -1331,18 +1352,18 @@
     <col min="8" max="10" width="11.9833333333333" customWidth="1"/>
     <col min="11" max="11" width="15.075" customWidth="1"/>
     <col min="12" max="14" width="12.1083333333333" customWidth="1"/>
-    <col min="15" max="15" width="10.8583333333333" customWidth="1"/>
-    <col min="17" max="17" width="14.2166666666667" customWidth="1"/>
-    <col min="18" max="18" width="11.8083333333333" customWidth="1"/>
-    <col min="19" max="19" width="10.6" customWidth="1"/>
-    <col min="20" max="20" width="9.70833333333333" customWidth="1"/>
-    <col min="21" max="21" width="11.1666666666667" customWidth="1"/>
-    <col min="22" max="22" width="11.4083333333333" customWidth="1"/>
-    <col min="23" max="23" width="12.0583333333333" customWidth="1"/>
-    <col min="24" max="24" width="15.575" customWidth="1"/>
+    <col min="15" max="16" width="10.8583333333333" customWidth="1"/>
+    <col min="18" max="18" width="14.2166666666667" customWidth="1"/>
+    <col min="19" max="19" width="11.8083333333333" customWidth="1"/>
+    <col min="20" max="20" width="10.6" customWidth="1"/>
+    <col min="21" max="21" width="9.70833333333333" customWidth="1"/>
+    <col min="22" max="22" width="11.1666666666667" customWidth="1"/>
+    <col min="23" max="23" width="11.4083333333333" customWidth="1"/>
+    <col min="24" max="24" width="12.0583333333333" customWidth="1"/>
+    <col min="25" max="25" width="15.575" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="15" customHeight="1" spans="1:23">
+    <row r="1" ht="15" customHeight="1" spans="1:24">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1385,15 +1406,18 @@
       <c r="N1" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="2"/>
+      <c r="O1" s="2" t="s">
+        <v>1</v>
+      </c>
       <c r="P1" s="2"/>
       <c r="Q1" s="2"/>
       <c r="R1" s="2"/>
       <c r="S1" s="2"/>
       <c r="T1" s="2"/>
-      <c r="W1" s="6"/>
-    </row>
-    <row r="2" spans="1:35">
+      <c r="U1" s="2"/>
+      <c r="X1" s="6"/>
+    </row>
+    <row r="2" spans="1:36">
       <c r="A2" s="3"/>
       <c r="B2" s="4" t="s">
         <v>14</v>
@@ -1420,13 +1444,15 @@
       <c r="N2" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O2" s="4"/>
+      <c r="O2" s="4" t="s">
+        <v>20</v>
+      </c>
       <c r="P2" s="4"/>
       <c r="Q2" s="4"/>
       <c r="R2" s="4"/>
       <c r="S2" s="4"/>
       <c r="T2" s="4"/>
-      <c r="U2" s="3"/>
+      <c r="U2" s="4"/>
       <c r="V2" s="3"/>
       <c r="W2" s="3"/>
       <c r="X2" s="3"/>
@@ -1441,21 +1467,22 @@
       <c r="AG2" s="3"/>
       <c r="AH2" s="3"/>
       <c r="AI2" s="3"/>
-    </row>
-    <row r="3" spans="1:35">
+      <c r="AJ2" s="3"/>
+    </row>
+    <row r="3" spans="1:36">
       <c r="A3" s="3"/>
       <c r="B3" s="4" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C3" s="2"/>
       <c r="D3" s="4" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E3" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="G3" s="4" t="s">
         <v>17</v>
@@ -1471,13 +1498,15 @@
       <c r="N3" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O3" s="4"/>
+      <c r="O3" s="4" t="s">
+        <v>20</v>
+      </c>
       <c r="P3" s="4"/>
       <c r="Q3" s="4"/>
       <c r="R3" s="4"/>
       <c r="S3" s="4"/>
       <c r="T3" s="4"/>
-      <c r="U3" s="3"/>
+      <c r="U3" s="4"/>
       <c r="V3" s="3"/>
       <c r="W3" s="3"/>
       <c r="X3" s="3"/>
@@ -1492,24 +1521,25 @@
       <c r="AG3" s="3"/>
       <c r="AH3" s="3"/>
       <c r="AI3" s="3"/>
-    </row>
-    <row r="4" spans="1:35">
+      <c r="AJ3" s="3"/>
+    </row>
+    <row r="4" spans="1:36">
       <c r="A4" s="3"/>
       <c r="B4" s="4" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C4" s="2"/>
       <c r="D4" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E4" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="H4" s="4" t="s">
         <v>18</v>
@@ -1522,13 +1552,15 @@
       <c r="N4" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O4" s="4"/>
+      <c r="O4" s="4" t="s">
+        <v>27</v>
+      </c>
       <c r="P4" s="4"/>
       <c r="Q4" s="4"/>
       <c r="R4" s="4"/>
       <c r="S4" s="4"/>
       <c r="T4" s="4"/>
-      <c r="U4" s="3"/>
+      <c r="U4" s="4"/>
       <c r="V4" s="3"/>
       <c r="W4" s="3"/>
       <c r="X4" s="3"/>
@@ -1543,24 +1575,25 @@
       <c r="AG4" s="3"/>
       <c r="AH4" s="3"/>
       <c r="AI4" s="3"/>
-    </row>
-    <row r="5" spans="1:35">
+      <c r="AJ4" s="3"/>
+    </row>
+    <row r="5" spans="1:36">
       <c r="A5" s="3"/>
       <c r="B5" s="4" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="C5" s="2"/>
       <c r="D5" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E5" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="H5" s="4" t="s">
         <v>18</v>
@@ -1573,13 +1606,15 @@
       <c r="N5" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O5" s="4"/>
+      <c r="O5" s="4" t="s">
+        <v>27</v>
+      </c>
       <c r="P5" s="4"/>
       <c r="Q5" s="4"/>
       <c r="R5" s="4"/>
       <c r="S5" s="4"/>
       <c r="T5" s="4"/>
-      <c r="U5" s="3"/>
+      <c r="U5" s="4"/>
       <c r="V5" s="3"/>
       <c r="W5" s="3"/>
       <c r="X5" s="3"/>
@@ -1594,24 +1629,25 @@
       <c r="AG5" s="3"/>
       <c r="AH5" s="3"/>
       <c r="AI5" s="3"/>
-    </row>
-    <row r="6" spans="1:35">
+      <c r="AJ5" s="3"/>
+    </row>
+    <row r="6" spans="1:36">
       <c r="A6" s="3"/>
       <c r="B6" s="4" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="C6" s="2"/>
       <c r="D6" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E6" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="G6" s="4" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="H6" s="4" t="s">
         <v>18</v>
@@ -1624,13 +1660,15 @@
       <c r="N6" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O6" s="4"/>
+      <c r="O6" s="4" t="s">
+        <v>27</v>
+      </c>
       <c r="P6" s="4"/>
       <c r="Q6" s="4"/>
       <c r="R6" s="4"/>
       <c r="S6" s="4"/>
       <c r="T6" s="4"/>
-      <c r="U6" s="3"/>
+      <c r="U6" s="4"/>
       <c r="V6" s="3"/>
       <c r="W6" s="3"/>
       <c r="X6" s="3"/>
@@ -1645,24 +1683,25 @@
       <c r="AG6" s="3"/>
       <c r="AH6" s="3"/>
       <c r="AI6" s="3"/>
-    </row>
-    <row r="7" spans="1:35">
+      <c r="AJ6" s="3"/>
+    </row>
+    <row r="7" spans="1:36">
       <c r="A7" s="3"/>
       <c r="B7" s="4" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="C7" s="2"/>
       <c r="D7" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E7" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="G7" s="4" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="H7" s="4" t="s">
         <v>18</v>
@@ -1675,13 +1714,15 @@
       <c r="N7" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O7" s="4"/>
+      <c r="O7" s="4" t="s">
+        <v>27</v>
+      </c>
       <c r="P7" s="4"/>
       <c r="Q7" s="4"/>
       <c r="R7" s="4"/>
       <c r="S7" s="4"/>
       <c r="T7" s="4"/>
-      <c r="U7" s="3"/>
+      <c r="U7" s="4"/>
       <c r="V7" s="3"/>
       <c r="W7" s="3"/>
       <c r="X7" s="3"/>
@@ -1696,29 +1737,30 @@
       <c r="AG7" s="3"/>
       <c r="AH7" s="3"/>
       <c r="AI7" s="3"/>
-    </row>
-    <row r="8" spans="1:35">
+      <c r="AJ7" s="3"/>
+    </row>
+    <row r="8" spans="1:36">
       <c r="A8" s="3"/>
       <c r="B8" s="4" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E8" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F8" s="4" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="G8" s="4" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="H8" s="4" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="I8" s="4"/>
       <c r="J8" s="4"/>
@@ -1728,13 +1770,15 @@
       <c r="N8" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O8" s="4"/>
+      <c r="O8" s="4" t="s">
+        <v>27</v>
+      </c>
       <c r="P8" s="4"/>
       <c r="Q8" s="4"/>
       <c r="R8" s="4"/>
       <c r="S8" s="4"/>
       <c r="T8" s="4"/>
-      <c r="U8" s="3"/>
+      <c r="U8" s="4"/>
       <c r="V8" s="3"/>
       <c r="W8" s="3"/>
       <c r="X8" s="3"/>
@@ -1749,29 +1793,30 @@
       <c r="AG8" s="3"/>
       <c r="AH8" s="3"/>
       <c r="AI8" s="3"/>
-    </row>
-    <row r="9" spans="1:35">
+      <c r="AJ8" s="3"/>
+    </row>
+    <row r="9" spans="1:36">
       <c r="A9" s="3"/>
       <c r="B9" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="C9" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="C9" s="2" t="s">
-        <v>33</v>
-      </c>
       <c r="D9" s="4" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E9" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F9" s="4" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="G9" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="H9" s="4" t="s">
         <v>36</v>
-      </c>
-      <c r="H9" s="4" t="s">
-        <v>34</v>
       </c>
       <c r="I9" s="4"/>
       <c r="J9" s="4"/>
@@ -1781,13 +1826,15 @@
       <c r="N9" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O9" s="4"/>
+      <c r="O9" s="4" t="s">
+        <v>39</v>
+      </c>
       <c r="P9" s="4"/>
       <c r="Q9" s="4"/>
       <c r="R9" s="4"/>
       <c r="S9" s="4"/>
       <c r="T9" s="4"/>
-      <c r="U9" s="3"/>
+      <c r="U9" s="4"/>
       <c r="V9" s="3"/>
       <c r="W9" s="3"/>
       <c r="X9" s="3"/>
@@ -1802,45 +1849,48 @@
       <c r="AG9" s="3"/>
       <c r="AH9" s="3"/>
       <c r="AI9" s="3"/>
-    </row>
-    <row r="10" spans="1:35">
+      <c r="AJ9" s="3"/>
+    </row>
+    <row r="10" spans="1:36">
       <c r="A10" s="3"/>
       <c r="B10" s="4" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="C10" s="2"/>
       <c r="D10" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E10" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F10" s="4" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="G10" s="4" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="H10" s="4"/>
       <c r="I10" s="4"/>
       <c r="J10" s="4" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="K10" s="4" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="L10" s="4"/>
       <c r="M10" s="4"/>
       <c r="N10" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O10" s="4"/>
+      <c r="O10" s="4" t="s">
+        <v>44</v>
+      </c>
       <c r="P10" s="4"/>
       <c r="Q10" s="4"/>
       <c r="R10" s="4"/>
       <c r="S10" s="4"/>
       <c r="T10" s="4"/>
-      <c r="U10" s="3"/>
+      <c r="U10" s="4"/>
       <c r="V10" s="3"/>
       <c r="W10" s="3"/>
       <c r="X10" s="3"/>
@@ -1855,45 +1905,48 @@
       <c r="AG10" s="3"/>
       <c r="AH10" s="3"/>
       <c r="AI10" s="3"/>
-    </row>
-    <row r="11" spans="1:35">
+      <c r="AJ10" s="3"/>
+    </row>
+    <row r="11" spans="1:36">
       <c r="A11" s="3"/>
       <c r="B11" s="4" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="C11" s="2"/>
       <c r="D11" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E11" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F11" s="4" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="G11" s="4" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="H11" s="4"/>
       <c r="I11" s="4"/>
       <c r="J11" s="4" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="K11" s="4" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="L11" s="4"/>
       <c r="M11" s="4"/>
       <c r="N11" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O11" s="4"/>
+      <c r="O11" s="4" t="s">
+        <v>44</v>
+      </c>
       <c r="P11" s="4"/>
       <c r="Q11" s="4"/>
       <c r="R11" s="4"/>
       <c r="S11" s="4"/>
       <c r="T11" s="4"/>
-      <c r="U11" s="3"/>
+      <c r="U11" s="4"/>
       <c r="V11" s="3"/>
       <c r="W11" s="3"/>
       <c r="X11" s="3"/>
@@ -1908,45 +1961,48 @@
       <c r="AG11" s="3"/>
       <c r="AH11" s="3"/>
       <c r="AI11" s="3"/>
-    </row>
-    <row r="12" spans="1:35">
+      <c r="AJ11" s="3"/>
+    </row>
+    <row r="12" spans="1:36">
       <c r="A12" s="3"/>
       <c r="B12" s="4" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="C12" s="2"/>
       <c r="D12" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E12" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F12" s="4" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="G12" s="4" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="H12" s="4"/>
       <c r="I12" s="4"/>
       <c r="J12" s="4" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="K12" s="4" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="L12" s="4"/>
       <c r="M12" s="4"/>
       <c r="N12" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O12" s="4"/>
+      <c r="O12" s="4" t="s">
+        <v>44</v>
+      </c>
       <c r="P12" s="4"/>
       <c r="Q12" s="4"/>
       <c r="R12" s="4"/>
       <c r="S12" s="4"/>
       <c r="T12" s="4"/>
-      <c r="U12" s="3"/>
+      <c r="U12" s="4"/>
       <c r="V12" s="3"/>
       <c r="W12" s="3"/>
       <c r="X12" s="3"/>
@@ -1961,30 +2017,31 @@
       <c r="AG12" s="3"/>
       <c r="AH12" s="3"/>
       <c r="AI12" s="3"/>
-    </row>
-    <row r="13" spans="1:35">
+      <c r="AJ12" s="3"/>
+    </row>
+    <row r="13" spans="1:36">
       <c r="A13" s="3"/>
       <c r="B13" s="4" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="C13" s="2"/>
       <c r="D13" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E13" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F13" s="4" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="G13" s="4" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="H13" s="4" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="I13" s="4" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="J13" s="4"/>
       <c r="K13" s="4"/>
@@ -1993,13 +2050,15 @@
       <c r="N13" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O13" s="4"/>
+      <c r="O13" s="4" t="s">
+        <v>27</v>
+      </c>
       <c r="P13" s="4"/>
       <c r="Q13" s="4"/>
       <c r="R13" s="4"/>
       <c r="S13" s="4"/>
       <c r="T13" s="4"/>
-      <c r="U13" s="3"/>
+      <c r="U13" s="4"/>
       <c r="V13" s="3"/>
       <c r="W13" s="3"/>
       <c r="X13" s="3"/>
@@ -2014,30 +2073,31 @@
       <c r="AG13" s="3"/>
       <c r="AH13" s="3"/>
       <c r="AI13" s="3"/>
-    </row>
-    <row r="14" spans="1:35">
+      <c r="AJ13" s="3"/>
+    </row>
+    <row r="14" spans="1:36">
       <c r="A14" s="3"/>
       <c r="B14" s="4" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="C14" s="2"/>
       <c r="D14" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E14" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F14" s="4" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="G14" s="4" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="H14" s="4" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="I14" s="4" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="J14" s="4"/>
       <c r="K14" s="4"/>
@@ -2046,13 +2106,15 @@
       <c r="N14" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O14" s="4"/>
+      <c r="O14" s="4" t="s">
+        <v>27</v>
+      </c>
       <c r="P14" s="4"/>
       <c r="Q14" s="4"/>
       <c r="R14" s="4"/>
       <c r="S14" s="4"/>
       <c r="T14" s="4"/>
-      <c r="U14" s="3"/>
+      <c r="U14" s="4"/>
       <c r="V14" s="3"/>
       <c r="W14" s="3"/>
       <c r="X14" s="3"/>
@@ -2067,30 +2129,31 @@
       <c r="AG14" s="3"/>
       <c r="AH14" s="3"/>
       <c r="AI14" s="3"/>
-    </row>
-    <row r="15" spans="1:35">
+      <c r="AJ14" s="3"/>
+    </row>
+    <row r="15" spans="1:36">
       <c r="A15" s="3"/>
       <c r="B15" s="4" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="C15" s="2"/>
       <c r="D15" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E15" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F15" s="4" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="G15" s="4" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="H15" s="4" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="I15" s="4" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="J15" s="4"/>
       <c r="K15" s="4"/>
@@ -2099,13 +2162,15 @@
       <c r="N15" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O15" s="4"/>
+      <c r="O15" s="4" t="s">
+        <v>27</v>
+      </c>
       <c r="P15" s="4"/>
       <c r="Q15" s="4"/>
       <c r="R15" s="4"/>
       <c r="S15" s="4"/>
       <c r="T15" s="4"/>
-      <c r="U15" s="3"/>
+      <c r="U15" s="4"/>
       <c r="V15" s="3"/>
       <c r="W15" s="3"/>
       <c r="X15" s="3"/>
@@ -2120,30 +2185,31 @@
       <c r="AG15" s="3"/>
       <c r="AH15" s="3"/>
       <c r="AI15" s="3"/>
-    </row>
-    <row r="16" spans="1:35">
+      <c r="AJ15" s="3"/>
+    </row>
+    <row r="16" spans="1:36">
       <c r="A16" s="3"/>
       <c r="B16" s="4" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="C16" s="2"/>
       <c r="D16" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E16" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F16" s="4" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="G16" s="4" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="H16" s="4" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="I16" s="4" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="J16" s="4"/>
       <c r="K16" s="4"/>
@@ -2152,13 +2218,15 @@
       <c r="N16" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O16" s="4"/>
+      <c r="O16" s="4" t="s">
+        <v>27</v>
+      </c>
       <c r="P16" s="4"/>
       <c r="Q16" s="4"/>
       <c r="R16" s="4"/>
       <c r="S16" s="4"/>
       <c r="T16" s="4"/>
-      <c r="U16" s="3"/>
+      <c r="U16" s="4"/>
       <c r="V16" s="3"/>
       <c r="W16" s="3"/>
       <c r="X16" s="3"/>
@@ -2173,30 +2241,31 @@
       <c r="AG16" s="3"/>
       <c r="AH16" s="3"/>
       <c r="AI16" s="3"/>
-    </row>
-    <row r="17" spans="1:35">
+      <c r="AJ16" s="3"/>
+    </row>
+    <row r="17" spans="1:36">
       <c r="A17" s="3"/>
       <c r="B17" s="4" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="C17" s="2"/>
       <c r="D17" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E17" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F17" s="4" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="G17" s="4" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="H17" s="4" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="I17" s="4" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="J17" s="4"/>
       <c r="K17" s="4"/>
@@ -2205,13 +2274,15 @@
       <c r="N17" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O17" s="4"/>
+      <c r="O17" s="4" t="s">
+        <v>27</v>
+      </c>
       <c r="P17" s="4"/>
       <c r="Q17" s="4"/>
       <c r="R17" s="4"/>
       <c r="S17" s="4"/>
       <c r="T17" s="4"/>
-      <c r="U17" s="3"/>
+      <c r="U17" s="4"/>
       <c r="V17" s="3"/>
       <c r="W17" s="3"/>
       <c r="X17" s="3"/>
@@ -2226,43 +2297,46 @@
       <c r="AG17" s="3"/>
       <c r="AH17" s="3"/>
       <c r="AI17" s="3"/>
-    </row>
-    <row r="18" spans="1:35">
+      <c r="AJ17" s="3"/>
+    </row>
+    <row r="18" spans="1:36">
       <c r="A18" s="3"/>
       <c r="B18" s="4" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="C18" s="2"/>
       <c r="D18" s="4" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E18" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F18" s="4" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="G18" s="4" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="H18" s="4"/>
       <c r="I18" s="4"/>
       <c r="J18" s="4"/>
       <c r="K18" s="4"/>
       <c r="L18" s="4" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="M18" s="4"/>
       <c r="N18" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O18" s="4"/>
+      <c r="O18" s="4" t="s">
+        <v>65</v>
+      </c>
       <c r="P18" s="4"/>
       <c r="Q18" s="4"/>
       <c r="R18" s="4"/>
       <c r="S18" s="4"/>
       <c r="T18" s="4"/>
-      <c r="U18" s="3"/>
+      <c r="U18" s="4"/>
       <c r="V18" s="3"/>
       <c r="W18" s="3"/>
       <c r="X18" s="3"/>
@@ -2277,43 +2351,46 @@
       <c r="AG18" s="3"/>
       <c r="AH18" s="3"/>
       <c r="AI18" s="3"/>
-    </row>
-    <row r="19" spans="1:35">
+      <c r="AJ18" s="3"/>
+    </row>
+    <row r="19" spans="1:36">
       <c r="A19" s="3"/>
       <c r="B19" s="4" t="s">
-        <v>61</v>
+        <v>66</v>
       </c>
       <c r="C19" s="2"/>
       <c r="D19" s="4" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E19" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F19" s="4" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="G19" s="4" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="H19" s="4"/>
       <c r="I19" s="4"/>
       <c r="J19" s="4"/>
       <c r="K19" s="4"/>
       <c r="L19" s="4" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="M19" s="4"/>
       <c r="N19" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O19" s="4"/>
+      <c r="O19" s="4" t="s">
+        <v>65</v>
+      </c>
       <c r="P19" s="4"/>
       <c r="Q19" s="4"/>
       <c r="R19" s="4"/>
       <c r="S19" s="4"/>
       <c r="T19" s="4"/>
-      <c r="U19" s="3"/>
+      <c r="U19" s="4"/>
       <c r="V19" s="3"/>
       <c r="W19" s="3"/>
       <c r="X19" s="3"/>
@@ -2328,43 +2405,46 @@
       <c r="AG19" s="3"/>
       <c r="AH19" s="3"/>
       <c r="AI19" s="3"/>
-    </row>
-    <row r="20" spans="1:35">
+      <c r="AJ19" s="3"/>
+    </row>
+    <row r="20" spans="1:36">
       <c r="A20" s="3"/>
       <c r="B20" s="4" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="C20" s="2"/>
       <c r="D20" s="4" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E20" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F20" s="4" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="G20" s="4" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="H20" s="4"/>
       <c r="I20" s="4"/>
       <c r="J20" s="4"/>
       <c r="K20" s="4"/>
       <c r="L20" s="4" t="s">
-        <v>64</v>
+        <v>69</v>
       </c>
       <c r="M20" s="4"/>
       <c r="N20" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O20" s="4"/>
+      <c r="O20" s="4" t="s">
+        <v>65</v>
+      </c>
       <c r="P20" s="4"/>
       <c r="Q20" s="4"/>
       <c r="R20" s="4"/>
       <c r="S20" s="4"/>
       <c r="T20" s="4"/>
-      <c r="U20" s="3"/>
+      <c r="U20" s="4"/>
       <c r="V20" s="3"/>
       <c r="W20" s="3"/>
       <c r="X20" s="3"/>
@@ -2379,43 +2459,46 @@
       <c r="AG20" s="3"/>
       <c r="AH20" s="3"/>
       <c r="AI20" s="3"/>
-    </row>
-    <row r="21" spans="1:35">
+      <c r="AJ20" s="3"/>
+    </row>
+    <row r="21" spans="1:36">
       <c r="A21" s="3"/>
       <c r="B21" s="4" t="s">
-        <v>65</v>
+        <v>70</v>
       </c>
       <c r="C21" s="2"/>
       <c r="D21" s="4" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E21" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F21" s="4" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="G21" s="4" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="H21" s="4"/>
       <c r="I21" s="4"/>
       <c r="J21" s="4"/>
       <c r="K21" s="4"/>
       <c r="L21" s="4" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="M21" s="4"/>
       <c r="N21" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O21" s="4"/>
+      <c r="O21" s="4" t="s">
+        <v>65</v>
+      </c>
       <c r="P21" s="4"/>
       <c r="Q21" s="4"/>
       <c r="R21" s="4"/>
       <c r="S21" s="4"/>
       <c r="T21" s="4"/>
-      <c r="U21" s="3"/>
+      <c r="U21" s="4"/>
       <c r="V21" s="3"/>
       <c r="W21" s="3"/>
       <c r="X21" s="3"/>
@@ -2430,43 +2513,46 @@
       <c r="AG21" s="3"/>
       <c r="AH21" s="3"/>
       <c r="AI21" s="3"/>
-    </row>
-    <row r="22" spans="1:35">
+      <c r="AJ21" s="3"/>
+    </row>
+    <row r="22" spans="1:36">
       <c r="A22" s="3"/>
       <c r="B22" s="4" t="s">
-        <v>67</v>
+        <v>72</v>
       </c>
       <c r="C22" s="2"/>
       <c r="D22" s="4" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E22" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F22" s="4" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="G22" s="4" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="H22" s="4"/>
       <c r="I22" s="4"/>
       <c r="J22" s="4"/>
       <c r="K22" s="4"/>
       <c r="L22" s="4" t="s">
-        <v>68</v>
+        <v>73</v>
       </c>
       <c r="M22" s="4"/>
       <c r="N22" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O22" s="4"/>
+      <c r="O22" s="4" t="s">
+        <v>65</v>
+      </c>
       <c r="P22" s="4"/>
       <c r="Q22" s="4"/>
       <c r="R22" s="4"/>
       <c r="S22" s="4"/>
       <c r="T22" s="4"/>
-      <c r="U22" s="3"/>
+      <c r="U22" s="4"/>
       <c r="V22" s="3"/>
       <c r="W22" s="3"/>
       <c r="X22" s="3"/>
@@ -2481,43 +2567,46 @@
       <c r="AG22" s="3"/>
       <c r="AH22" s="3"/>
       <c r="AI22" s="3"/>
-    </row>
-    <row r="23" spans="1:35">
+      <c r="AJ22" s="3"/>
+    </row>
+    <row r="23" spans="1:36">
       <c r="A23" s="3"/>
       <c r="B23" s="4" t="s">
-        <v>69</v>
+        <v>74</v>
       </c>
       <c r="C23" s="2"/>
       <c r="D23" s="4" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E23" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F23" s="4" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="G23" s="4" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="H23" s="4"/>
       <c r="I23" s="4"/>
       <c r="J23" s="4"/>
       <c r="K23" s="4"/>
       <c r="L23" s="4" t="s">
-        <v>70</v>
+        <v>75</v>
       </c>
       <c r="M23" s="4"/>
       <c r="N23" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O23" s="4"/>
+      <c r="O23" s="4" t="s">
+        <v>65</v>
+      </c>
       <c r="P23" s="4"/>
       <c r="Q23" s="4"/>
       <c r="R23" s="4"/>
       <c r="S23" s="4"/>
       <c r="T23" s="4"/>
-      <c r="U23" s="3"/>
+      <c r="U23" s="4"/>
       <c r="V23" s="3"/>
       <c r="W23" s="3"/>
       <c r="X23" s="3"/>
@@ -2532,24 +2621,25 @@
       <c r="AG23" s="3"/>
       <c r="AH23" s="3"/>
       <c r="AI23" s="3"/>
-    </row>
-    <row r="24" spans="1:35">
+      <c r="AJ23" s="3"/>
+    </row>
+    <row r="24" spans="1:36">
       <c r="A24" s="3"/>
       <c r="B24" s="4" t="s">
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="C24" s="2"/>
       <c r="D24" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E24" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F24" s="4" t="s">
-        <v>72</v>
+        <v>77</v>
       </c>
       <c r="G24" s="4" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="H24" s="4" t="s">
         <v>18</v>
@@ -2562,13 +2652,15 @@
       <c r="N24" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O24" s="4"/>
+      <c r="O24" s="4" t="s">
+        <v>27</v>
+      </c>
       <c r="P24" s="4"/>
       <c r="Q24" s="4"/>
       <c r="R24" s="4"/>
       <c r="S24" s="4"/>
       <c r="T24" s="4"/>
-      <c r="U24" s="3"/>
+      <c r="U24" s="4"/>
       <c r="V24" s="3"/>
       <c r="W24" s="3"/>
       <c r="X24" s="3"/>
@@ -2583,24 +2675,25 @@
       <c r="AG24" s="3"/>
       <c r="AH24" s="3"/>
       <c r="AI24" s="3"/>
-    </row>
-    <row r="25" spans="1:35">
+      <c r="AJ24" s="3"/>
+    </row>
+    <row r="25" spans="1:36">
       <c r="A25" s="3"/>
       <c r="B25" s="4" t="s">
-        <v>73</v>
+        <v>78</v>
       </c>
       <c r="C25" s="2"/>
       <c r="D25" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E25" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F25" s="4" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="G25" s="4" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="H25" s="4" t="s">
         <v>18</v>
@@ -2613,13 +2706,15 @@
       <c r="N25" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O25" s="4"/>
+      <c r="O25" s="4" t="s">
+        <v>27</v>
+      </c>
       <c r="P25" s="4"/>
       <c r="Q25" s="4"/>
       <c r="R25" s="4"/>
       <c r="S25" s="4"/>
       <c r="T25" s="4"/>
-      <c r="U25" s="3"/>
+      <c r="U25" s="4"/>
       <c r="V25" s="3"/>
       <c r="W25" s="3"/>
       <c r="X25" s="3"/>
@@ -2634,21 +2729,22 @@
       <c r="AG25" s="3"/>
       <c r="AH25" s="3"/>
       <c r="AI25" s="3"/>
-    </row>
-    <row r="26" spans="1:35">
+      <c r="AJ25" s="3"/>
+    </row>
+    <row r="26" spans="1:36">
       <c r="A26" s="3"/>
       <c r="B26" s="4" t="s">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="C26" s="2"/>
       <c r="D26" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E26" s="4" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="F26" s="4" t="s">
-        <v>72</v>
+        <v>77</v>
       </c>
       <c r="G26" s="4"/>
       <c r="H26" s="4" t="s">
@@ -2662,13 +2758,15 @@
       <c r="N26" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O26" s="4"/>
+      <c r="O26" s="4" t="s">
+        <v>82</v>
+      </c>
       <c r="P26" s="4"/>
       <c r="Q26" s="4"/>
       <c r="R26" s="4"/>
       <c r="S26" s="4"/>
       <c r="T26" s="4"/>
-      <c r="U26" s="3"/>
+      <c r="U26" s="4"/>
       <c r="V26" s="3"/>
       <c r="W26" s="3"/>
       <c r="X26" s="3"/>
@@ -2683,21 +2781,22 @@
       <c r="AG26" s="3"/>
       <c r="AH26" s="3"/>
       <c r="AI26" s="3"/>
-    </row>
-    <row r="27" spans="1:35">
+      <c r="AJ26" s="3"/>
+    </row>
+    <row r="27" spans="1:36">
       <c r="A27" s="3"/>
       <c r="B27" s="4" t="s">
-        <v>77</v>
+        <v>83</v>
       </c>
       <c r="C27" s="2"/>
       <c r="D27" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E27" s="4" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="F27" s="4" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="G27" s="4"/>
       <c r="H27" s="4" t="s">
@@ -2711,13 +2810,15 @@
       <c r="N27" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O27" s="4"/>
+      <c r="O27" s="4" t="s">
+        <v>82</v>
+      </c>
       <c r="P27" s="4"/>
       <c r="Q27" s="4"/>
       <c r="R27" s="4"/>
       <c r="S27" s="4"/>
       <c r="T27" s="4"/>
-      <c r="U27" s="3"/>
+      <c r="U27" s="4"/>
       <c r="V27" s="3"/>
       <c r="W27" s="3"/>
       <c r="X27" s="3"/>
@@ -2732,24 +2833,25 @@
       <c r="AG27" s="3"/>
       <c r="AH27" s="3"/>
       <c r="AI27" s="3"/>
-    </row>
-    <row r="28" spans="1:35">
+      <c r="AJ27" s="3"/>
+    </row>
+    <row r="28" spans="1:36">
       <c r="A28" s="3"/>
       <c r="B28" s="4" t="s">
-        <v>78</v>
+        <v>84</v>
       </c>
       <c r="C28" s="2"/>
       <c r="D28" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E28" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F28" s="4" t="s">
-        <v>79</v>
+        <v>85</v>
       </c>
       <c r="G28" s="4" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="H28" s="4" t="s">
         <v>18</v>
@@ -2762,13 +2864,15 @@
       <c r="N28" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O28" s="4"/>
+      <c r="O28" s="4" t="s">
+        <v>27</v>
+      </c>
       <c r="P28" s="4"/>
       <c r="Q28" s="4"/>
       <c r="R28" s="4"/>
       <c r="S28" s="4"/>
       <c r="T28" s="4"/>
-      <c r="U28" s="3"/>
+      <c r="U28" s="4"/>
       <c r="V28" s="3"/>
       <c r="W28" s="3"/>
       <c r="X28" s="3"/>
@@ -2783,21 +2887,22 @@
       <c r="AG28" s="3"/>
       <c r="AH28" s="3"/>
       <c r="AI28" s="3"/>
-    </row>
-    <row r="29" spans="1:35">
+      <c r="AJ28" s="3"/>
+    </row>
+    <row r="29" spans="1:36">
       <c r="A29" s="3"/>
       <c r="B29" s="4" t="s">
-        <v>80</v>
+        <v>86</v>
       </c>
       <c r="C29" s="2"/>
       <c r="D29" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E29" s="4" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="F29" s="4" t="s">
-        <v>81</v>
+        <v>87</v>
       </c>
       <c r="G29" s="4"/>
       <c r="H29" s="4" t="s">
@@ -2811,13 +2916,15 @@
       <c r="N29" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O29" s="4"/>
+      <c r="O29" s="4" t="s">
+        <v>82</v>
+      </c>
       <c r="P29" s="4"/>
       <c r="Q29" s="4"/>
       <c r="R29" s="4"/>
       <c r="S29" s="4"/>
       <c r="T29" s="4"/>
-      <c r="U29" s="3"/>
+      <c r="U29" s="4"/>
       <c r="V29" s="3"/>
       <c r="W29" s="3"/>
       <c r="X29" s="3"/>
@@ -2832,21 +2939,22 @@
       <c r="AG29" s="3"/>
       <c r="AH29" s="3"/>
       <c r="AI29" s="3"/>
-    </row>
-    <row r="30" spans="1:35">
+      <c r="AJ29" s="3"/>
+    </row>
+    <row r="30" spans="1:36">
       <c r="A30" s="3"/>
       <c r="B30" s="4" t="s">
-        <v>82</v>
+        <v>88</v>
       </c>
       <c r="C30" s="2"/>
       <c r="D30" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E30" s="4" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="F30" s="4" t="s">
-        <v>83</v>
+        <v>89</v>
       </c>
       <c r="G30" s="4"/>
       <c r="H30" s="4" t="s">
@@ -2860,13 +2968,15 @@
       <c r="N30" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O30" s="4"/>
+      <c r="O30" s="4" t="s">
+        <v>82</v>
+      </c>
       <c r="P30" s="4"/>
       <c r="Q30" s="4"/>
       <c r="R30" s="4"/>
       <c r="S30" s="4"/>
       <c r="T30" s="4"/>
-      <c r="U30" s="3"/>
+      <c r="U30" s="4"/>
       <c r="V30" s="3"/>
       <c r="W30" s="3"/>
       <c r="X30" s="3"/>
@@ -2881,24 +2991,25 @@
       <c r="AG30" s="3"/>
       <c r="AH30" s="3"/>
       <c r="AI30" s="3"/>
-    </row>
-    <row r="31" spans="1:35">
+      <c r="AJ30" s="3"/>
+    </row>
+    <row r="31" spans="1:36">
       <c r="A31" s="3"/>
       <c r="B31" s="4" t="s">
-        <v>84</v>
+        <v>90</v>
       </c>
       <c r="C31" s="2"/>
       <c r="D31" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E31" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F31" s="4" t="s">
-        <v>83</v>
+        <v>89</v>
       </c>
       <c r="G31" s="4" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="H31" s="4" t="s">
         <v>18</v>
@@ -2911,13 +3022,15 @@
       <c r="N31" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O31" s="4"/>
+      <c r="O31" s="4" t="s">
+        <v>27</v>
+      </c>
       <c r="P31" s="4"/>
       <c r="Q31" s="4"/>
       <c r="R31" s="4"/>
       <c r="S31" s="4"/>
       <c r="T31" s="4"/>
-      <c r="U31" s="3"/>
+      <c r="U31" s="4"/>
       <c r="V31" s="3"/>
       <c r="W31" s="3"/>
       <c r="X31" s="3"/>
@@ -2932,24 +3045,25 @@
       <c r="AG31" s="3"/>
       <c r="AH31" s="3"/>
       <c r="AI31" s="3"/>
-    </row>
-    <row r="32" spans="1:35">
+      <c r="AJ31" s="3"/>
+    </row>
+    <row r="32" spans="1:36">
       <c r="A32" s="3"/>
       <c r="B32" s="4" t="s">
-        <v>85</v>
+        <v>91</v>
       </c>
       <c r="C32" s="2"/>
       <c r="D32" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E32" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F32" s="4" t="s">
-        <v>83</v>
+        <v>89</v>
       </c>
       <c r="G32" s="4" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="H32" s="4" t="s">
         <v>18</v>
@@ -2962,13 +3076,15 @@
       <c r="N32" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O32" s="4"/>
+      <c r="O32" s="4" t="s">
+        <v>27</v>
+      </c>
       <c r="P32" s="4"/>
       <c r="Q32" s="4"/>
       <c r="R32" s="4"/>
       <c r="S32" s="4"/>
       <c r="T32" s="4"/>
-      <c r="U32" s="3"/>
+      <c r="U32" s="4"/>
       <c r="V32" s="3"/>
       <c r="W32" s="3"/>
       <c r="X32" s="3"/>
@@ -2983,21 +3099,22 @@
       <c r="AG32" s="3"/>
       <c r="AH32" s="3"/>
       <c r="AI32" s="3"/>
-    </row>
-    <row r="33" spans="1:35">
+      <c r="AJ32" s="3"/>
+    </row>
+    <row r="33" spans="1:36">
       <c r="A33" s="3"/>
       <c r="B33" s="4" t="s">
-        <v>86</v>
+        <v>92</v>
       </c>
       <c r="C33" s="2"/>
       <c r="D33" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E33" s="4" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="F33" s="4" t="s">
-        <v>79</v>
+        <v>85</v>
       </c>
       <c r="G33" s="4"/>
       <c r="H33" s="4" t="s">
@@ -3011,13 +3128,15 @@
       <c r="N33" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O33" s="4"/>
+      <c r="O33" s="4" t="s">
+        <v>82</v>
+      </c>
       <c r="P33" s="4"/>
       <c r="Q33" s="4"/>
       <c r="R33" s="4"/>
       <c r="S33" s="4"/>
       <c r="T33" s="4"/>
-      <c r="U33" s="3"/>
+      <c r="U33" s="4"/>
       <c r="V33" s="3"/>
       <c r="W33" s="3"/>
       <c r="X33" s="3"/>
@@ -3032,21 +3151,22 @@
       <c r="AG33" s="3"/>
       <c r="AH33" s="3"/>
       <c r="AI33" s="3"/>
-    </row>
-    <row r="34" spans="1:35">
+      <c r="AJ33" s="3"/>
+    </row>
+    <row r="34" spans="1:36">
       <c r="A34" s="3"/>
       <c r="B34" s="4" t="s">
-        <v>87</v>
+        <v>93</v>
       </c>
       <c r="C34" s="2"/>
       <c r="D34" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E34" s="4" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="F34" s="4" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="G34" s="4"/>
       <c r="H34" s="4" t="s">
@@ -3060,13 +3180,15 @@
       <c r="N34" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O34" s="4"/>
+      <c r="O34" s="4" t="s">
+        <v>82</v>
+      </c>
       <c r="P34" s="4"/>
       <c r="Q34" s="4"/>
       <c r="R34" s="4"/>
       <c r="S34" s="4"/>
       <c r="T34" s="4"/>
-      <c r="U34" s="3"/>
+      <c r="U34" s="4"/>
       <c r="V34" s="3"/>
       <c r="W34" s="3"/>
       <c r="X34" s="3"/>
@@ -3081,21 +3203,22 @@
       <c r="AG34" s="3"/>
       <c r="AH34" s="3"/>
       <c r="AI34" s="3"/>
-    </row>
-    <row r="35" spans="1:35">
+      <c r="AJ34" s="3"/>
+    </row>
+    <row r="35" spans="1:36">
       <c r="A35" s="3"/>
       <c r="B35" s="4" t="s">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="C35" s="2"/>
       <c r="D35" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E35" s="4" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="F35" s="4" t="s">
-        <v>89</v>
+        <v>95</v>
       </c>
       <c r="G35" s="4"/>
       <c r="H35" s="4" t="s">
@@ -3109,13 +3232,15 @@
       <c r="N35" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O35" s="4"/>
+      <c r="O35" s="4" t="s">
+        <v>82</v>
+      </c>
       <c r="P35" s="4"/>
       <c r="Q35" s="4"/>
       <c r="R35" s="4"/>
       <c r="S35" s="4"/>
       <c r="T35" s="4"/>
-      <c r="U35" s="3"/>
+      <c r="U35" s="4"/>
       <c r="V35" s="3"/>
       <c r="W35" s="3"/>
       <c r="X35" s="3"/>
@@ -3130,21 +3255,22 @@
       <c r="AG35" s="3"/>
       <c r="AH35" s="3"/>
       <c r="AI35" s="3"/>
-    </row>
-    <row r="36" spans="1:35">
+      <c r="AJ35" s="3"/>
+    </row>
+    <row r="36" spans="1:36">
       <c r="A36" s="3"/>
       <c r="B36" s="4" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="C36" s="2"/>
       <c r="D36" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E36" s="4" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="F36" s="4" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="G36" s="4"/>
       <c r="H36" s="4" t="s">
@@ -3158,13 +3284,15 @@
       <c r="N36" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O36" s="4"/>
+      <c r="O36" s="4" t="s">
+        <v>82</v>
+      </c>
       <c r="P36" s="4"/>
       <c r="Q36" s="4"/>
       <c r="R36" s="4"/>
       <c r="S36" s="4"/>
       <c r="T36" s="4"/>
-      <c r="U36" s="3"/>
+      <c r="U36" s="4"/>
       <c r="V36" s="3"/>
       <c r="W36" s="3"/>
       <c r="X36" s="3"/>
@@ -3179,21 +3307,22 @@
       <c r="AG36" s="3"/>
       <c r="AH36" s="3"/>
       <c r="AI36" s="3"/>
-    </row>
-    <row r="37" spans="1:35">
+      <c r="AJ36" s="3"/>
+    </row>
+    <row r="37" spans="1:36">
       <c r="A37" s="3"/>
       <c r="B37" s="4" t="s">
-        <v>91</v>
+        <v>97</v>
       </c>
       <c r="C37" s="2"/>
       <c r="D37" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E37" s="4" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="F37" s="4" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="G37" s="4"/>
       <c r="H37" s="4" t="s">
@@ -3207,13 +3336,15 @@
       <c r="N37" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O37" s="4"/>
+      <c r="O37" s="4" t="s">
+        <v>82</v>
+      </c>
       <c r="P37" s="4"/>
       <c r="Q37" s="4"/>
       <c r="R37" s="4"/>
       <c r="S37" s="4"/>
       <c r="T37" s="4"/>
-      <c r="U37" s="3"/>
+      <c r="U37" s="4"/>
       <c r="V37" s="3"/>
       <c r="W37" s="3"/>
       <c r="X37" s="3"/>
@@ -3228,21 +3359,22 @@
       <c r="AG37" s="3"/>
       <c r="AH37" s="3"/>
       <c r="AI37" s="3"/>
-    </row>
-    <row r="38" spans="1:35">
+      <c r="AJ37" s="3"/>
+    </row>
+    <row r="38" spans="1:36">
       <c r="A38" s="3"/>
       <c r="B38" s="4" t="s">
-        <v>92</v>
+        <v>98</v>
       </c>
       <c r="C38" s="2"/>
       <c r="D38" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E38" s="4" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="F38" s="4" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="G38" s="4"/>
       <c r="H38" s="4" t="s">
@@ -3256,13 +3388,15 @@
       <c r="N38" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O38" s="4"/>
+      <c r="O38" s="4" t="s">
+        <v>82</v>
+      </c>
       <c r="P38" s="4"/>
       <c r="Q38" s="4"/>
       <c r="R38" s="4"/>
       <c r="S38" s="4"/>
       <c r="T38" s="4"/>
-      <c r="U38" s="3"/>
+      <c r="U38" s="4"/>
       <c r="V38" s="3"/>
       <c r="W38" s="3"/>
       <c r="X38" s="3"/>
@@ -3277,43 +3411,46 @@
       <c r="AG38" s="3"/>
       <c r="AH38" s="3"/>
       <c r="AI38" s="3"/>
-    </row>
-    <row r="39" spans="1:35">
+      <c r="AJ38" s="3"/>
+    </row>
+    <row r="39" spans="1:36">
       <c r="A39" s="3"/>
       <c r="B39" s="4" t="s">
-        <v>93</v>
+        <v>99</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="D39" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E39" s="4" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="F39" s="4"/>
       <c r="G39" s="4"/>
       <c r="H39" s="4" t="s">
-        <v>95</v>
+        <v>101</v>
       </c>
       <c r="I39" s="4"/>
       <c r="J39" s="4"/>
       <c r="K39" s="4"/>
       <c r="L39" s="4"/>
       <c r="M39" s="4" t="s">
-        <v>96</v>
+        <v>102</v>
       </c>
       <c r="N39" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O39" s="4"/>
+      <c r="O39" s="4" t="s">
+        <v>82</v>
+      </c>
       <c r="P39" s="4"/>
       <c r="Q39" s="4"/>
       <c r="R39" s="4"/>
       <c r="S39" s="4"/>
       <c r="T39" s="4"/>
-      <c r="U39" s="3"/>
+      <c r="U39" s="4"/>
       <c r="V39" s="3"/>
       <c r="W39" s="3"/>
       <c r="X39" s="3"/>
@@ -3328,43 +3465,46 @@
       <c r="AG39" s="3"/>
       <c r="AH39" s="3"/>
       <c r="AI39" s="3"/>
-    </row>
-    <row r="40" spans="1:35">
+      <c r="AJ39" s="3"/>
+    </row>
+    <row r="40" spans="1:36">
       <c r="A40" s="3"/>
       <c r="B40" s="4" t="s">
-        <v>97</v>
+        <v>103</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="D40" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E40" s="4" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="F40" s="4"/>
       <c r="G40" s="4"/>
       <c r="H40" s="4" t="s">
-        <v>95</v>
+        <v>101</v>
       </c>
       <c r="I40" s="4"/>
       <c r="J40" s="4"/>
       <c r="K40" s="4"/>
       <c r="L40" s="4"/>
       <c r="M40" s="4" t="s">
-        <v>98</v>
+        <v>104</v>
       </c>
       <c r="N40" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O40" s="4"/>
+      <c r="O40" s="4" t="s">
+        <v>82</v>
+      </c>
       <c r="P40" s="4"/>
       <c r="Q40" s="4"/>
       <c r="R40" s="4"/>
       <c r="S40" s="4"/>
       <c r="T40" s="4"/>
-      <c r="U40" s="3"/>
+      <c r="U40" s="4"/>
       <c r="V40" s="3"/>
       <c r="W40" s="3"/>
       <c r="X40" s="3"/>
@@ -3379,39 +3519,42 @@
       <c r="AG40" s="3"/>
       <c r="AH40" s="3"/>
       <c r="AI40" s="3"/>
-    </row>
-    <row r="41" spans="1:35">
+      <c r="AJ40" s="3"/>
+    </row>
+    <row r="41" spans="1:36">
       <c r="A41" s="3"/>
       <c r="B41" s="4" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="D41" s="4"/>
       <c r="E41" s="4"/>
       <c r="F41" s="4"/>
       <c r="G41" s="4"/>
       <c r="H41" s="4" t="s">
-        <v>95</v>
+        <v>101</v>
       </c>
       <c r="I41" s="4"/>
       <c r="J41" s="4"/>
       <c r="K41" s="4"/>
       <c r="L41" s="4"/>
       <c r="M41" s="4" t="s">
-        <v>101</v>
+        <v>107</v>
       </c>
       <c r="N41" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O41" s="4"/>
+      <c r="O41" s="4" t="s">
+        <v>108</v>
+      </c>
       <c r="P41" s="4"/>
       <c r="Q41" s="4"/>
       <c r="R41" s="4"/>
       <c r="S41" s="4"/>
       <c r="T41" s="4"/>
-      <c r="U41" s="3"/>
+      <c r="U41" s="4"/>
       <c r="V41" s="3"/>
       <c r="W41" s="3"/>
       <c r="X41" s="3"/>
@@ -3426,39 +3569,42 @@
       <c r="AG41" s="3"/>
       <c r="AH41" s="3"/>
       <c r="AI41" s="3"/>
-    </row>
-    <row r="42" spans="1:35">
+      <c r="AJ41" s="3"/>
+    </row>
+    <row r="42" spans="1:36">
       <c r="A42" s="3"/>
       <c r="B42" s="4" t="s">
-        <v>102</v>
+        <v>109</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="D42" s="4"/>
       <c r="E42" s="4"/>
       <c r="F42" s="4"/>
       <c r="G42" s="4"/>
       <c r="H42" s="4" t="s">
-        <v>95</v>
+        <v>101</v>
       </c>
       <c r="I42" s="4"/>
       <c r="J42" s="4"/>
       <c r="K42" s="4"/>
       <c r="L42" s="4"/>
       <c r="M42" s="4" t="s">
-        <v>101</v>
+        <v>107</v>
       </c>
       <c r="N42" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O42" s="4"/>
+      <c r="O42" s="4" t="s">
+        <v>108</v>
+      </c>
       <c r="P42" s="4"/>
       <c r="Q42" s="4"/>
       <c r="R42" s="4"/>
       <c r="S42" s="4"/>
       <c r="T42" s="4"/>
-      <c r="U42" s="3"/>
+      <c r="U42" s="4"/>
       <c r="V42" s="3"/>
       <c r="W42" s="3"/>
       <c r="X42" s="3"/>
@@ -3473,10 +3619,11 @@
       <c r="AG42" s="3"/>
       <c r="AH42" s="3"/>
       <c r="AI42" s="3"/>
-    </row>
-    <row r="43" spans="2:35">
+      <c r="AJ42" s="3"/>
+    </row>
+    <row r="43" spans="2:36">
       <c r="B43" s="2" t="s">
-        <v>103</v>
+        <v>110</v>
       </c>
       <c r="C43" s="2"/>
       <c r="D43" s="2"/>
@@ -3492,13 +3639,15 @@
       <c r="N43" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="O43" s="2"/>
+      <c r="O43" s="2" t="s">
+        <v>27</v>
+      </c>
       <c r="P43" s="2"/>
       <c r="Q43" s="2"/>
       <c r="R43" s="2"/>
       <c r="S43" s="2"/>
       <c r="T43" s="2"/>
-      <c r="Y43" s="3"/>
+      <c r="U43" s="2"/>
       <c r="Z43" s="3"/>
       <c r="AA43" s="3"/>
       <c r="AB43" s="3"/>
@@ -3509,54 +3658,57 @@
       <c r="AG43" s="3"/>
       <c r="AH43" s="3"/>
       <c r="AI43" s="3"/>
-    </row>
-    <row r="44" spans="2:35">
+      <c r="AJ43" s="3"/>
+    </row>
+    <row r="44" spans="2:36">
       <c r="B44" s="2" t="s">
-        <v>104</v>
+        <v>111</v>
       </c>
       <c r="C44" s="2" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="D44" s="2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E44" s="2" t="s">
         <v>15</v>
       </c>
       <c r="F44" s="2" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="G44" s="2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="H44" s="4" t="s">
-        <v>105</v>
+        <v>112</v>
       </c>
       <c r="I44" s="4" t="s">
-        <v>106</v>
+        <v>113</v>
       </c>
       <c r="J44" s="4" t="s">
-        <v>107</v>
+        <v>114</v>
       </c>
       <c r="K44" s="2" t="s">
-        <v>108</v>
+        <v>115</v>
       </c>
       <c r="L44" s="2" t="s">
-        <v>109</v>
+        <v>116</v>
       </c>
       <c r="M44" s="2" t="s">
-        <v>110</v>
+        <v>117</v>
       </c>
       <c r="N44" s="2" t="s">
-        <v>111</v>
-      </c>
-      <c r="O44" s="2"/>
+        <v>118</v>
+      </c>
+      <c r="O44" s="2" t="s">
+        <v>82</v>
+      </c>
       <c r="P44" s="2"/>
       <c r="Q44" s="2"/>
       <c r="R44" s="2"/>
       <c r="S44" s="2"/>
       <c r="T44" s="2"/>
-      <c r="Y44" s="3"/>
+      <c r="U44" s="2"/>
       <c r="Z44" s="3"/>
       <c r="AA44" s="3"/>
       <c r="AB44" s="3"/>
@@ -3567,8 +3719,9 @@
       <c r="AG44" s="3"/>
       <c r="AH44" s="3"/>
       <c r="AI44" s="3"/>
-    </row>
-    <row r="45" spans="1:35">
+      <c r="AJ44" s="3"/>
+    </row>
+    <row r="45" spans="1:36">
       <c r="A45" s="3"/>
       <c r="B45" s="4"/>
       <c r="C45" s="4"/>
@@ -3589,7 +3742,7 @@
       <c r="R45" s="4"/>
       <c r="S45" s="4"/>
       <c r="T45" s="4"/>
-      <c r="U45" s="3"/>
+      <c r="U45" s="4"/>
       <c r="V45" s="3"/>
       <c r="W45" s="3"/>
       <c r="X45" s="3"/>
@@ -3604,8 +3757,9 @@
       <c r="AG45" s="3"/>
       <c r="AH45" s="3"/>
       <c r="AI45" s="3"/>
-    </row>
-    <row r="46" s="1" customFormat="1" spans="1:35">
+      <c r="AJ45" s="3"/>
+    </row>
+    <row r="46" s="1" customFormat="1" spans="1:36">
       <c r="A46" s="3"/>
       <c r="B46" s="4"/>
       <c r="C46" s="4"/>
@@ -3626,7 +3780,7 @@
       <c r="R46" s="4"/>
       <c r="S46" s="4"/>
       <c r="T46" s="4"/>
-      <c r="U46" s="3"/>
+      <c r="U46" s="4"/>
       <c r="V46" s="3"/>
       <c r="W46" s="3"/>
       <c r="X46" s="3"/>
@@ -3641,8 +3795,9 @@
       <c r="AG46" s="3"/>
       <c r="AH46" s="3"/>
       <c r="AI46" s="3"/>
-    </row>
-    <row r="47" s="1" customFormat="1" spans="1:35">
+      <c r="AJ46" s="3"/>
+    </row>
+    <row r="47" s="1" customFormat="1" spans="1:36">
       <c r="A47" s="3"/>
       <c r="B47" s="4"/>
       <c r="C47" s="4"/>
@@ -3663,7 +3818,7 @@
       <c r="R47" s="4"/>
       <c r="S47" s="4"/>
       <c r="T47" s="4"/>
-      <c r="U47" s="3"/>
+      <c r="U47" s="4"/>
       <c r="V47" s="3"/>
       <c r="W47" s="3"/>
       <c r="X47" s="3"/>
@@ -3678,8 +3833,9 @@
       <c r="AG47" s="3"/>
       <c r="AH47" s="3"/>
       <c r="AI47" s="3"/>
-    </row>
-    <row r="48" spans="1:35">
+      <c r="AJ47" s="3"/>
+    </row>
+    <row r="48" spans="1:36">
       <c r="A48" s="3"/>
       <c r="B48" s="4"/>
       <c r="C48" s="4"/>
@@ -3700,7 +3856,7 @@
       <c r="R48" s="4"/>
       <c r="S48" s="4"/>
       <c r="T48" s="4"/>
-      <c r="U48" s="3"/>
+      <c r="U48" s="4"/>
       <c r="V48" s="3"/>
       <c r="W48" s="3"/>
       <c r="X48" s="3"/>
@@ -3715,8 +3871,9 @@
       <c r="AG48" s="3"/>
       <c r="AH48" s="3"/>
       <c r="AI48" s="3"/>
-    </row>
-    <row r="49" spans="1:35">
+      <c r="AJ48" s="3"/>
+    </row>
+    <row r="49" spans="1:36">
       <c r="A49" s="3"/>
       <c r="B49" s="4"/>
       <c r="C49" s="4"/>
@@ -3737,7 +3894,7 @@
       <c r="R49" s="4"/>
       <c r="S49" s="4"/>
       <c r="T49" s="4"/>
-      <c r="U49" s="3"/>
+      <c r="U49" s="4"/>
       <c r="V49" s="3"/>
       <c r="W49" s="3"/>
       <c r="X49" s="3"/>
@@ -3752,8 +3909,9 @@
       <c r="AG49" s="3"/>
       <c r="AH49" s="3"/>
       <c r="AI49" s="3"/>
-    </row>
-    <row r="50" spans="1:35">
+      <c r="AJ49" s="3"/>
+    </row>
+    <row r="50" spans="1:36">
       <c r="A50" s="3"/>
       <c r="B50" s="4"/>
       <c r="C50" s="4"/>
@@ -3774,7 +3932,7 @@
       <c r="R50" s="4"/>
       <c r="S50" s="4"/>
       <c r="T50" s="4"/>
-      <c r="U50" s="3"/>
+      <c r="U50" s="4"/>
       <c r="V50" s="3"/>
       <c r="W50" s="3"/>
       <c r="X50" s="3"/>
@@ -3789,8 +3947,9 @@
       <c r="AG50" s="3"/>
       <c r="AH50" s="3"/>
       <c r="AI50" s="3"/>
-    </row>
-    <row r="51" spans="1:35">
+      <c r="AJ50" s="3"/>
+    </row>
+    <row r="51" spans="1:36">
       <c r="A51" s="3"/>
       <c r="B51" s="4"/>
       <c r="C51" s="4"/>
@@ -3811,7 +3970,7 @@
       <c r="R51" s="4"/>
       <c r="S51" s="4"/>
       <c r="T51" s="4"/>
-      <c r="U51" s="3"/>
+      <c r="U51" s="4"/>
       <c r="V51" s="3"/>
       <c r="W51" s="3"/>
       <c r="X51" s="3"/>
@@ -3826,8 +3985,9 @@
       <c r="AG51" s="3"/>
       <c r="AH51" s="3"/>
       <c r="AI51" s="3"/>
-    </row>
-    <row r="52" spans="1:35">
+      <c r="AJ51" s="3"/>
+    </row>
+    <row r="52" spans="1:36">
       <c r="A52" s="3"/>
       <c r="B52" s="4"/>
       <c r="C52" s="4"/>
@@ -3848,7 +4008,7 @@
       <c r="R52" s="4"/>
       <c r="S52" s="4"/>
       <c r="T52" s="4"/>
-      <c r="U52" s="3"/>
+      <c r="U52" s="4"/>
       <c r="V52" s="3"/>
       <c r="W52" s="3"/>
       <c r="X52" s="3"/>
@@ -3863,8 +4023,9 @@
       <c r="AG52" s="3"/>
       <c r="AH52" s="3"/>
       <c r="AI52" s="3"/>
-    </row>
-    <row r="53" spans="1:35">
+      <c r="AJ52" s="3"/>
+    </row>
+    <row r="53" spans="1:36">
       <c r="A53" s="3"/>
       <c r="B53" s="4"/>
       <c r="C53" s="4"/>
@@ -3885,7 +4046,7 @@
       <c r="R53" s="4"/>
       <c r="S53" s="4"/>
       <c r="T53" s="4"/>
-      <c r="U53" s="3"/>
+      <c r="U53" s="4"/>
       <c r="V53" s="3"/>
       <c r="W53" s="3"/>
       <c r="X53" s="3"/>
@@ -3900,8 +4061,9 @@
       <c r="AG53" s="3"/>
       <c r="AH53" s="3"/>
       <c r="AI53" s="3"/>
-    </row>
-    <row r="54" spans="1:35">
+      <c r="AJ53" s="3"/>
+    </row>
+    <row r="54" spans="1:36">
       <c r="A54" s="3"/>
       <c r="B54" s="4"/>
       <c r="C54" s="4"/>
@@ -3922,7 +4084,7 @@
       <c r="R54" s="4"/>
       <c r="S54" s="4"/>
       <c r="T54" s="4"/>
-      <c r="U54" s="3"/>
+      <c r="U54" s="4"/>
       <c r="V54" s="3"/>
       <c r="W54" s="3"/>
       <c r="X54" s="3"/>
@@ -3937,8 +4099,9 @@
       <c r="AG54" s="3"/>
       <c r="AH54" s="3"/>
       <c r="AI54" s="3"/>
-    </row>
-    <row r="55" spans="1:35">
+      <c r="AJ54" s="3"/>
+    </row>
+    <row r="55" spans="1:36">
       <c r="A55" s="3"/>
       <c r="B55" s="4"/>
       <c r="C55" s="4"/>
@@ -3959,7 +4122,7 @@
       <c r="R55" s="4"/>
       <c r="S55" s="4"/>
       <c r="T55" s="4"/>
-      <c r="U55" s="3"/>
+      <c r="U55" s="4"/>
       <c r="V55" s="3"/>
       <c r="W55" s="3"/>
       <c r="X55" s="3"/>
@@ -3974,8 +4137,9 @@
       <c r="AG55" s="3"/>
       <c r="AH55" s="3"/>
       <c r="AI55" s="3"/>
-    </row>
-    <row r="56" spans="1:35">
+      <c r="AJ55" s="3"/>
+    </row>
+    <row r="56" spans="1:36">
       <c r="A56" s="3"/>
       <c r="B56" s="4"/>
       <c r="C56" s="4"/>
@@ -3996,7 +4160,7 @@
       <c r="R56" s="4"/>
       <c r="S56" s="4"/>
       <c r="T56" s="4"/>
-      <c r="U56" s="3"/>
+      <c r="U56" s="4"/>
       <c r="V56" s="3"/>
       <c r="W56" s="3"/>
       <c r="X56" s="3"/>
@@ -4011,8 +4175,9 @@
       <c r="AG56" s="3"/>
       <c r="AH56" s="3"/>
       <c r="AI56" s="3"/>
-    </row>
-    <row r="57" spans="1:35">
+      <c r="AJ56" s="3"/>
+    </row>
+    <row r="57" spans="1:36">
       <c r="A57" s="3"/>
       <c r="B57" s="4"/>
       <c r="C57" s="4"/>
@@ -4033,7 +4198,7 @@
       <c r="R57" s="4"/>
       <c r="S57" s="4"/>
       <c r="T57" s="4"/>
-      <c r="U57" s="3"/>
+      <c r="U57" s="4"/>
       <c r="V57" s="3"/>
       <c r="W57" s="3"/>
       <c r="X57" s="3"/>
@@ -4048,8 +4213,9 @@
       <c r="AG57" s="3"/>
       <c r="AH57" s="3"/>
       <c r="AI57" s="3"/>
-    </row>
-    <row r="58" spans="1:35">
+      <c r="AJ57" s="3"/>
+    </row>
+    <row r="58" spans="1:36">
       <c r="A58" s="3"/>
       <c r="B58" s="4"/>
       <c r="C58" s="4"/>
@@ -4070,7 +4236,7 @@
       <c r="R58" s="4"/>
       <c r="S58" s="4"/>
       <c r="T58" s="4"/>
-      <c r="U58" s="3"/>
+      <c r="U58" s="4"/>
       <c r="V58" s="3"/>
       <c r="W58" s="3"/>
       <c r="X58" s="3"/>
@@ -4085,8 +4251,9 @@
       <c r="AG58" s="3"/>
       <c r="AH58" s="3"/>
       <c r="AI58" s="3"/>
-    </row>
-    <row r="59" spans="1:35">
+      <c r="AJ58" s="3"/>
+    </row>
+    <row r="59" spans="1:36">
       <c r="A59" s="3"/>
       <c r="B59" s="4"/>
       <c r="C59" s="4"/>
@@ -4107,7 +4274,7 @@
       <c r="R59" s="4"/>
       <c r="S59" s="4"/>
       <c r="T59" s="4"/>
-      <c r="U59" s="3"/>
+      <c r="U59" s="4"/>
       <c r="V59" s="3"/>
       <c r="W59" s="3"/>
       <c r="X59" s="3"/>
@@ -4122,8 +4289,9 @@
       <c r="AG59" s="3"/>
       <c r="AH59" s="3"/>
       <c r="AI59" s="3"/>
-    </row>
-    <row r="60" spans="1:35">
+      <c r="AJ59" s="3"/>
+    </row>
+    <row r="60" spans="1:36">
       <c r="A60" s="3"/>
       <c r="B60" s="4"/>
       <c r="C60" s="4"/>
@@ -4144,7 +4312,7 @@
       <c r="R60" s="4"/>
       <c r="S60" s="4"/>
       <c r="T60" s="4"/>
-      <c r="U60" s="3"/>
+      <c r="U60" s="4"/>
       <c r="V60" s="3"/>
       <c r="W60" s="3"/>
       <c r="X60" s="3"/>
@@ -4159,8 +4327,9 @@
       <c r="AG60" s="3"/>
       <c r="AH60" s="3"/>
       <c r="AI60" s="3"/>
-    </row>
-    <row r="61" spans="1:35">
+      <c r="AJ60" s="3"/>
+    </row>
+    <row r="61" spans="1:36">
       <c r="A61" s="3"/>
       <c r="B61" s="4"/>
       <c r="C61" s="4"/>
@@ -4181,7 +4350,7 @@
       <c r="R61" s="4"/>
       <c r="S61" s="4"/>
       <c r="T61" s="4"/>
-      <c r="U61" s="3"/>
+      <c r="U61" s="4"/>
       <c r="V61" s="3"/>
       <c r="W61" s="3"/>
       <c r="X61" s="3"/>
@@ -4196,8 +4365,9 @@
       <c r="AG61" s="3"/>
       <c r="AH61" s="3"/>
       <c r="AI61" s="3"/>
-    </row>
-    <row r="62" spans="1:35">
+      <c r="AJ61" s="3"/>
+    </row>
+    <row r="62" spans="1:36">
       <c r="A62" s="3"/>
       <c r="B62" s="4"/>
       <c r="C62" s="4"/>
@@ -4218,7 +4388,7 @@
       <c r="R62" s="4"/>
       <c r="S62" s="4"/>
       <c r="T62" s="4"/>
-      <c r="U62" s="3"/>
+      <c r="U62" s="4"/>
       <c r="V62" s="3"/>
       <c r="W62" s="3"/>
       <c r="X62" s="3"/>
@@ -4233,8 +4403,9 @@
       <c r="AG62" s="3"/>
       <c r="AH62" s="3"/>
       <c r="AI62" s="3"/>
-    </row>
-    <row r="63" spans="1:35">
+      <c r="AJ62" s="3"/>
+    </row>
+    <row r="63" spans="1:36">
       <c r="A63" s="3"/>
       <c r="B63" s="4"/>
       <c r="C63" s="4"/>
@@ -4255,7 +4426,7 @@
       <c r="R63" s="4"/>
       <c r="S63" s="4"/>
       <c r="T63" s="4"/>
-      <c r="U63" s="3"/>
+      <c r="U63" s="4"/>
       <c r="V63" s="3"/>
       <c r="W63" s="3"/>
       <c r="X63" s="3"/>
@@ -4270,8 +4441,9 @@
       <c r="AG63" s="3"/>
       <c r="AH63" s="3"/>
       <c r="AI63" s="3"/>
-    </row>
-    <row r="64" spans="1:35">
+      <c r="AJ63" s="3"/>
+    </row>
+    <row r="64" spans="1:36">
       <c r="A64" s="3"/>
       <c r="B64" s="4"/>
       <c r="C64" s="4"/>
@@ -4292,7 +4464,7 @@
       <c r="R64" s="4"/>
       <c r="S64" s="4"/>
       <c r="T64" s="4"/>
-      <c r="U64" s="3"/>
+      <c r="U64" s="4"/>
       <c r="V64" s="3"/>
       <c r="W64" s="3"/>
       <c r="X64" s="3"/>
@@ -4307,8 +4479,9 @@
       <c r="AG64" s="3"/>
       <c r="AH64" s="3"/>
       <c r="AI64" s="3"/>
-    </row>
-    <row r="65" spans="1:35">
+      <c r="AJ64" s="3"/>
+    </row>
+    <row r="65" spans="1:36">
       <c r="A65" s="3"/>
       <c r="B65" s="4"/>
       <c r="C65" s="4"/>
@@ -4329,7 +4502,7 @@
       <c r="R65" s="4"/>
       <c r="S65" s="4"/>
       <c r="T65" s="4"/>
-      <c r="U65" s="3"/>
+      <c r="U65" s="4"/>
       <c r="V65" s="3"/>
       <c r="W65" s="3"/>
       <c r="X65" s="3"/>
@@ -4344,8 +4517,9 @@
       <c r="AG65" s="3"/>
       <c r="AH65" s="3"/>
       <c r="AI65" s="3"/>
-    </row>
-    <row r="66" spans="1:35">
+      <c r="AJ65" s="3"/>
+    </row>
+    <row r="66" spans="1:36">
       <c r="A66" s="3"/>
       <c r="B66" s="4"/>
       <c r="C66" s="4"/>
@@ -4366,7 +4540,7 @@
       <c r="R66" s="4"/>
       <c r="S66" s="4"/>
       <c r="T66" s="4"/>
-      <c r="U66" s="3"/>
+      <c r="U66" s="4"/>
       <c r="V66" s="3"/>
       <c r="W66" s="3"/>
       <c r="X66" s="3"/>
@@ -4381,8 +4555,9 @@
       <c r="AG66" s="3"/>
       <c r="AH66" s="3"/>
       <c r="AI66" s="3"/>
-    </row>
-    <row r="67" spans="1:35">
+      <c r="AJ66" s="3"/>
+    </row>
+    <row r="67" spans="1:36">
       <c r="A67" s="3"/>
       <c r="B67" s="4"/>
       <c r="C67" s="4"/>
@@ -4403,7 +4578,7 @@
       <c r="R67" s="4"/>
       <c r="S67" s="4"/>
       <c r="T67" s="4"/>
-      <c r="U67" s="3"/>
+      <c r="U67" s="4"/>
       <c r="V67" s="3"/>
       <c r="W67" s="3"/>
       <c r="X67" s="3"/>
@@ -4418,8 +4593,9 @@
       <c r="AG67" s="3"/>
       <c r="AH67" s="3"/>
       <c r="AI67" s="3"/>
-    </row>
-    <row r="68" spans="1:35">
+      <c r="AJ67" s="3"/>
+    </row>
+    <row r="68" spans="1:36">
       <c r="A68" s="3"/>
       <c r="B68" s="4"/>
       <c r="C68" s="4"/>
@@ -4440,7 +4616,7 @@
       <c r="R68" s="4"/>
       <c r="S68" s="4"/>
       <c r="T68" s="4"/>
-      <c r="U68" s="3"/>
+      <c r="U68" s="4"/>
       <c r="V68" s="3"/>
       <c r="W68" s="3"/>
       <c r="X68" s="3"/>
@@ -4455,8 +4631,9 @@
       <c r="AG68" s="3"/>
       <c r="AH68" s="3"/>
       <c r="AI68" s="3"/>
-    </row>
-    <row r="69" spans="1:35">
+      <c r="AJ68" s="3"/>
+    </row>
+    <row r="69" spans="1:36">
       <c r="A69" s="3"/>
       <c r="B69" s="4"/>
       <c r="C69" s="4"/>
@@ -4477,7 +4654,7 @@
       <c r="R69" s="4"/>
       <c r="S69" s="4"/>
       <c r="T69" s="4"/>
-      <c r="U69" s="3"/>
+      <c r="U69" s="4"/>
       <c r="V69" s="3"/>
       <c r="W69" s="3"/>
       <c r="X69" s="3"/>
@@ -4492,8 +4669,9 @@
       <c r="AG69" s="3"/>
       <c r="AH69" s="3"/>
       <c r="AI69" s="3"/>
-    </row>
-    <row r="70" spans="1:35">
+      <c r="AJ69" s="3"/>
+    </row>
+    <row r="70" spans="1:36">
       <c r="A70" s="3"/>
       <c r="B70" s="4"/>
       <c r="C70" s="4"/>
@@ -4514,7 +4692,7 @@
       <c r="R70" s="4"/>
       <c r="S70" s="4"/>
       <c r="T70" s="4"/>
-      <c r="U70" s="3"/>
+      <c r="U70" s="4"/>
       <c r="V70" s="3"/>
       <c r="W70" s="3"/>
       <c r="X70" s="3"/>
@@ -4529,8 +4707,9 @@
       <c r="AG70" s="3"/>
       <c r="AH70" s="3"/>
       <c r="AI70" s="3"/>
-    </row>
-    <row r="71" spans="1:35">
+      <c r="AJ70" s="3"/>
+    </row>
+    <row r="71" spans="1:36">
       <c r="A71" s="3"/>
       <c r="B71" s="4"/>
       <c r="C71" s="4"/>
@@ -4551,7 +4730,7 @@
       <c r="R71" s="4"/>
       <c r="S71" s="4"/>
       <c r="T71" s="4"/>
-      <c r="U71" s="3"/>
+      <c r="U71" s="4"/>
       <c r="V71" s="3"/>
       <c r="W71" s="3"/>
       <c r="X71" s="3"/>
@@ -4566,8 +4745,9 @@
       <c r="AG71" s="3"/>
       <c r="AH71" s="3"/>
       <c r="AI71" s="3"/>
-    </row>
-    <row r="72" spans="1:35">
+      <c r="AJ71" s="3"/>
+    </row>
+    <row r="72" spans="1:36">
       <c r="A72" s="3"/>
       <c r="B72" s="4"/>
       <c r="C72" s="4"/>
@@ -4588,7 +4768,7 @@
       <c r="R72" s="4"/>
       <c r="S72" s="4"/>
       <c r="T72" s="4"/>
-      <c r="U72" s="3"/>
+      <c r="U72" s="4"/>
       <c r="V72" s="3"/>
       <c r="W72" s="3"/>
       <c r="X72" s="3"/>
@@ -4603,8 +4783,9 @@
       <c r="AG72" s="3"/>
       <c r="AH72" s="3"/>
       <c r="AI72" s="3"/>
-    </row>
-    <row r="73" spans="1:35">
+      <c r="AJ72" s="3"/>
+    </row>
+    <row r="73" spans="1:36">
       <c r="A73" s="3"/>
       <c r="B73" s="4"/>
       <c r="C73" s="4"/>
@@ -4625,7 +4806,7 @@
       <c r="R73" s="4"/>
       <c r="S73" s="4"/>
       <c r="T73" s="4"/>
-      <c r="U73" s="3"/>
+      <c r="U73" s="4"/>
       <c r="V73" s="3"/>
       <c r="W73" s="3"/>
       <c r="X73" s="3"/>
@@ -4640,8 +4821,9 @@
       <c r="AG73" s="3"/>
       <c r="AH73" s="3"/>
       <c r="AI73" s="3"/>
-    </row>
-    <row r="74" spans="1:35">
+      <c r="AJ73" s="3"/>
+    </row>
+    <row r="74" spans="1:36">
       <c r="A74" s="3"/>
       <c r="B74" s="4"/>
       <c r="C74" s="4"/>
@@ -4662,7 +4844,7 @@
       <c r="R74" s="4"/>
       <c r="S74" s="4"/>
       <c r="T74" s="4"/>
-      <c r="U74" s="3"/>
+      <c r="U74" s="4"/>
       <c r="V74" s="3"/>
       <c r="W74" s="3"/>
       <c r="X74" s="3"/>
@@ -4677,8 +4859,9 @@
       <c r="AG74" s="3"/>
       <c r="AH74" s="3"/>
       <c r="AI74" s="3"/>
-    </row>
-    <row r="75" spans="1:35">
+      <c r="AJ74" s="3"/>
+    </row>
+    <row r="75" spans="1:36">
       <c r="A75" s="3"/>
       <c r="B75" s="4"/>
       <c r="C75" s="4"/>
@@ -4699,7 +4882,7 @@
       <c r="R75" s="4"/>
       <c r="S75" s="4"/>
       <c r="T75" s="4"/>
-      <c r="U75" s="3"/>
+      <c r="U75" s="4"/>
       <c r="V75" s="3"/>
       <c r="W75" s="3"/>
       <c r="X75" s="3"/>
@@ -4714,8 +4897,9 @@
       <c r="AG75" s="3"/>
       <c r="AH75" s="3"/>
       <c r="AI75" s="3"/>
-    </row>
-    <row r="76" spans="1:35">
+      <c r="AJ75" s="3"/>
+    </row>
+    <row r="76" spans="1:36">
       <c r="A76" s="3"/>
       <c r="B76" s="4"/>
       <c r="C76" s="4"/>
@@ -4736,7 +4920,7 @@
       <c r="R76" s="4"/>
       <c r="S76" s="4"/>
       <c r="T76" s="4"/>
-      <c r="U76" s="3"/>
+      <c r="U76" s="4"/>
       <c r="V76" s="3"/>
       <c r="W76" s="3"/>
       <c r="X76" s="3"/>
@@ -4751,8 +4935,9 @@
       <c r="AG76" s="3"/>
       <c r="AH76" s="3"/>
       <c r="AI76" s="3"/>
-    </row>
-    <row r="77" spans="1:35">
+      <c r="AJ76" s="3"/>
+    </row>
+    <row r="77" spans="1:36">
       <c r="A77" s="3"/>
       <c r="B77" s="4"/>
       <c r="C77" s="4"/>
@@ -4773,7 +4958,7 @@
       <c r="R77" s="4"/>
       <c r="S77" s="4"/>
       <c r="T77" s="4"/>
-      <c r="U77" s="3"/>
+      <c r="U77" s="4"/>
       <c r="V77" s="3"/>
       <c r="W77" s="3"/>
       <c r="X77" s="3"/>
@@ -4788,8 +4973,9 @@
       <c r="AG77" s="3"/>
       <c r="AH77" s="3"/>
       <c r="AI77" s="3"/>
-    </row>
-    <row r="78" spans="1:35">
+      <c r="AJ77" s="3"/>
+    </row>
+    <row r="78" spans="1:36">
       <c r="A78" s="3"/>
       <c r="B78" s="4"/>
       <c r="C78" s="4"/>
@@ -4810,7 +4996,7 @@
       <c r="R78" s="4"/>
       <c r="S78" s="4"/>
       <c r="T78" s="4"/>
-      <c r="U78" s="3"/>
+      <c r="U78" s="4"/>
       <c r="V78" s="3"/>
       <c r="W78" s="3"/>
       <c r="X78" s="3"/>
@@ -4825,194 +5011,195 @@
       <c r="AG78" s="3"/>
       <c r="AH78" s="3"/>
       <c r="AI78" s="3"/>
-    </row>
-    <row r="86" spans="1:24">
+      <c r="AJ78" s="3"/>
+    </row>
+    <row r="86" spans="1:25">
       <c r="A86" s="2"/>
       <c r="B86" s="2"/>
       <c r="C86" s="2"/>
       <c r="D86" s="2"/>
-      <c r="S86" s="2"/>
-      <c r="U86" s="2"/>
+      <c r="T86" s="2"/>
       <c r="V86" s="2"/>
       <c r="W86" s="2"/>
       <c r="X86" s="2"/>
-    </row>
-    <row r="87" spans="1:24">
+      <c r="Y86" s="2"/>
+    </row>
+    <row r="87" spans="1:25">
       <c r="A87" s="2"/>
       <c r="B87" s="2"/>
       <c r="C87" s="2"/>
       <c r="D87" s="2"/>
       <c r="E87" s="2"/>
-      <c r="S87" s="2"/>
       <c r="T87" s="2"/>
       <c r="U87" s="2"/>
       <c r="V87" s="2"/>
       <c r="W87" s="2"/>
       <c r="X87" s="2"/>
-    </row>
-    <row r="88" spans="1:24">
+      <c r="Y87" s="2"/>
+    </row>
+    <row r="88" spans="1:25">
       <c r="A88" s="2"/>
       <c r="B88" s="2"/>
       <c r="C88" s="2"/>
       <c r="D88" s="2"/>
-      <c r="S88" s="2"/>
       <c r="T88" s="2"/>
       <c r="U88" s="2"/>
       <c r="V88" s="2"/>
       <c r="W88" s="2"/>
       <c r="X88" s="2"/>
-    </row>
-    <row r="89" spans="1:24">
+      <c r="Y88" s="2"/>
+    </row>
+    <row r="89" spans="1:25">
       <c r="A89" s="2"/>
       <c r="B89" s="2"/>
       <c r="C89" s="2"/>
       <c r="D89" s="2"/>
-      <c r="S89" s="2"/>
       <c r="T89" s="2"/>
       <c r="U89" s="2"/>
       <c r="V89" s="2"/>
       <c r="W89" s="2"/>
       <c r="X89" s="2"/>
-    </row>
-    <row r="90" spans="1:24">
+      <c r="Y89" s="2"/>
+    </row>
+    <row r="90" spans="1:25">
       <c r="A90" s="2"/>
       <c r="B90" s="2"/>
       <c r="C90" s="2"/>
       <c r="D90" s="2"/>
-      <c r="S90" s="2"/>
       <c r="T90" s="2"/>
       <c r="U90" s="2"/>
       <c r="V90" s="2"/>
       <c r="W90" s="2"/>
       <c r="X90" s="2"/>
-    </row>
-    <row r="91" spans="1:24">
+      <c r="Y90" s="2"/>
+    </row>
+    <row r="91" spans="1:25">
       <c r="A91" s="2"/>
       <c r="B91" s="2"/>
       <c r="C91" s="2"/>
       <c r="D91" s="2"/>
-      <c r="S91" s="2"/>
       <c r="T91" s="2"/>
       <c r="U91" s="2"/>
       <c r="V91" s="2"/>
       <c r="W91" s="2"/>
       <c r="X91" s="2"/>
-    </row>
-    <row r="92" spans="1:24">
+      <c r="Y91" s="2"/>
+    </row>
+    <row r="92" spans="1:25">
       <c r="A92" s="2"/>
       <c r="B92" s="2"/>
       <c r="C92" s="2"/>
       <c r="D92" s="2"/>
-      <c r="S92" s="2"/>
       <c r="T92" s="2"/>
       <c r="U92" s="2"/>
       <c r="V92" s="2"/>
       <c r="W92" s="2"/>
       <c r="X92" s="2"/>
-    </row>
-    <row r="93" spans="1:24">
+      <c r="Y92" s="2"/>
+    </row>
+    <row r="93" spans="1:25">
       <c r="A93" s="2"/>
       <c r="B93" s="2"/>
       <c r="C93" s="2"/>
       <c r="D93" s="2"/>
-      <c r="S93" s="2"/>
       <c r="T93" s="2"/>
       <c r="U93" s="2"/>
       <c r="V93" s="2"/>
       <c r="W93" s="2"/>
       <c r="X93" s="2"/>
-    </row>
-    <row r="94" spans="1:24">
+      <c r="Y93" s="2"/>
+    </row>
+    <row r="94" spans="1:25">
       <c r="A94" s="2"/>
       <c r="B94" s="2"/>
       <c r="C94" s="2"/>
       <c r="D94" s="2"/>
-      <c r="S94" s="2"/>
       <c r="T94" s="2"/>
       <c r="U94" s="2"/>
       <c r="V94" s="2"/>
       <c r="W94" s="2"/>
       <c r="X94" s="2"/>
-    </row>
-    <row r="95" spans="1:24">
+      <c r="Y94" s="2"/>
+    </row>
+    <row r="95" spans="1:25">
       <c r="A95" s="2"/>
       <c r="B95" s="2"/>
       <c r="C95" s="2"/>
       <c r="D95" s="2"/>
-      <c r="S95" s="2"/>
       <c r="T95" s="2"/>
       <c r="U95" s="2"/>
       <c r="V95" s="2"/>
       <c r="W95" s="2"/>
       <c r="X95" s="2"/>
-    </row>
-    <row r="96" spans="1:24">
+      <c r="Y95" s="2"/>
+    </row>
+    <row r="96" spans="1:25">
       <c r="A96" s="2"/>
       <c r="B96" s="2"/>
       <c r="C96" s="2"/>
       <c r="D96" s="2"/>
-      <c r="S96" s="2"/>
       <c r="T96" s="2"/>
       <c r="U96" s="2"/>
       <c r="V96" s="2"/>
       <c r="W96" s="2"/>
       <c r="X96" s="2"/>
-    </row>
-    <row r="97" spans="1:24">
+      <c r="Y96" s="2"/>
+    </row>
+    <row r="97" spans="1:25">
       <c r="A97" s="2"/>
       <c r="B97" s="2"/>
       <c r="C97" s="2"/>
       <c r="D97" s="2"/>
-      <c r="S97" s="2"/>
       <c r="T97" s="2"/>
       <c r="U97" s="2"/>
       <c r="V97" s="2"/>
       <c r="W97" s="2"/>
       <c r="X97" s="2"/>
-    </row>
-    <row r="98" spans="1:24">
+      <c r="Y97" s="2"/>
+    </row>
+    <row r="98" spans="1:25">
       <c r="A98" s="2"/>
       <c r="B98" s="2"/>
       <c r="C98" s="2"/>
       <c r="D98" s="2"/>
-      <c r="S98" s="2"/>
       <c r="T98" s="2"/>
       <c r="U98" s="2"/>
       <c r="V98" s="2"/>
       <c r="W98" s="2"/>
       <c r="X98" s="2"/>
-    </row>
-    <row r="99" spans="1:24">
+      <c r="Y98" s="2"/>
+    </row>
+    <row r="99" spans="1:25">
       <c r="A99" s="2"/>
       <c r="B99" s="2"/>
       <c r="C99" s="2"/>
       <c r="D99" s="2"/>
-      <c r="S99" s="2"/>
       <c r="T99" s="2"/>
       <c r="U99" s="2"/>
       <c r="V99" s="2"/>
       <c r="W99" s="2"/>
       <c r="X99" s="2"/>
+      <c r="Y99" s="2"/>
     </row>
   </sheetData>
-  <dataValidations count="13">
+  <dataValidations count="14">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="O2:O1048576">
+      <formula1>"R_TYPE,I_TYPE,S_TYPE,B_TYPE,U_TYPE,J_TYPE,ICSR_TYPE,FENCE_TYPE,N_TYPE"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="M29 M30 M31 M39 M40 M41 M42 M43 M2:M28 M32:M38 M44:M1048576">
+      <formula1>"CSR_W,CSR_S,CSR_C,CSR_P,CSR_XX"</formula1>
+    </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H29 H30 H31 H40 H41 H42 H43 H10:H28 H32:H39 H44:H1048576">
       <formula1>"WB_ALU,WB_MEM,WB_PC4,WB_XX,WB_CSR"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F6 F15 F18 F19 F20 F21 F24 F25 F26 F27 F28 F29 F30 F31 F32 F33 F36 F37 F38 F39 F40 F41 F42 F43 F2:F5 F7:F14 F16:F17 F22:F23 F34:F35 F44:F1048576">
-      <formula1>"ALU_ADD,ALU_SUB,ALU_AND,ALU_OR,ALU_XOR,ALU_SLL,ALU_SRL,ALU_SLT,ALU_SLTU,ALU_COPY_A,ALU_COPY_B,ALU_SRA"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L5 L6 L7 L10 L11 L14 L15 L16 L17 L18 L19 L20 L21 L22 L23 L24 L25 L26 L27 L28 L29 L30 L31 L32 L33 L34 L35 L36 L37 L38 L39 L40 L41 L42 L43 L2:L4 L8:L9 L12:L13 L44:L1048576">
-      <formula1>"BR_EQ,BR_NE,BR_LTU,BR_GE,BR_GEU,BR_LT,BR_XX"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C29 C30 C31 C43 C2:C28 C32:C42 C44:C1048576">
       <formula1>"PC_4,PC_0,PC_ALU,PC_CSR"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="N4 N5 N6 N7 N8 N9 N10 N11 N12 N13 N14 N15 N16 N17 N18 N19 N20 N21 N22 N23 N24 N25 N26 N27 N28 N29 N30 N31 N32 N33 N34 N35 N36 N37 N38 N39 N40 N41 N42 N43 N2:N3 N44:N1048576">
-      <formula1>"INST_VALID,INST_INVALID"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E4 E5 E6 E7 E8 E9 E10 E11 E12 E13 E14 E15 E16 E17 E18 E19 E20 E21 E22 E23 E24 E25 E26 E27 E28 E29 E30 E31 E32 E33 E34 E35 E36 E37 E38 E39 E40 E41 E42 E43 E2:E3 E44:E1048576">
+      <formula1>"B_IMM,B_RS2"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D4 D5 D6 D7 D8 D9 D10 D11 D12 D13 D14 D15 D16 D17 D18 D19 D20 D21 D22 D23 D24 D25 D26 D27 D28 D29 D30 D31 D32 D33 D34 D35 D36 D37 D38 D39 D40 D41 D42 D43 D2:D3 D44:D1048576">
-      <formula1>"A_PC,A_RS1"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G4 G5 G6 G7 G8 G9 G10 G11 G12 G13 G14 G15 G16 G17 G18 G19 G20 G21 G22 G23 G24 G25 G26 G27 G28 G29 G30 G31 G32 G33 G34 G35 G36 G37 G38 G39 G40 G41 G42 G43 G2:G3 G44:G1048576">
+      <formula1>"IMM_I,IMM_J,IMM_U,IMM_S,IMM_B"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J5 J6 J7 J8 J9 J10 J11 J12 J13 J14 J15 J16 J17 J18 J19 J20 J21 J22 J23 J24 J25 J26 J27 J28 J29 J30 J31 J32 J33 J34 J35 J36 J37 J38 J39 J40 J41 J42 J43 J2:J4 J44:J1048576">
       <formula1>"ST_SW,ST_SH,ST_SB,ST_XX"</formula1>
@@ -5020,20 +5207,23 @@
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H5 H6 H7 H8 H9 H2:H4">
       <formula1>"WB_ALU,WB_MEM,WB_PC4,WB_XX"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K4 K5 K6 K7 K8 K9 K10 K11 K12 K13 K14 K15 K16 K17 K18 K19 K20 K21 K22 K23 K24 K25 K26 K27 K28 K29 K30 K31 K32 K33 K34 K35 K36 K37 K38 K39 K40 K41 K42 K43 K2:K3 K44:K1048576">
-      <formula1>"MASK_XX,MASK_B,MASK_H,MASK_W,MASK_D"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L5 L6 L7 L10 L11 L14 L15 L16 L17 L18 L19 L20 L21 L22 L23 L24 L25 L26 L27 L28 L29 L30 L31 L32 L33 L34 L35 L36 L37 L38 L39 L40 L41 L42 L43 L2:L4 L8:L9 L12:L13 L44:L1048576">
+      <formula1>"BR_EQ,BR_NE,BR_LTU,BR_GE,BR_GEU,BR_LT,BR_XX"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E4 E5 E6 E7 E8 E9 E10 E11 E12 E13 E14 E15 E16 E17 E18 E19 E20 E21 E22 E23 E24 E25 E26 E27 E28 E29 E30 E31 E32 E33 E34 E35 E36 E37 E38 E39 E40 E41 E42 E43 E2:E3 E44:E1048576">
-      <formula1>"B_IMM,B_RS2"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="M29 M30 M31 M39 M40 M41 M42 M43 M2:M28 M32:M38 M44:M1048576">
-      <formula1>"CSR_W,CSR_S,CSR_C,CSR_P,CSR_XX"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="N4 N5 N6 N7 N8 N9 N10 N11 N12 N13 N14 N15 N16 N17 N18 N19 N20 N21 N22 N23 N24 N25 N26 N27 N28 N29 N30 N31 N32 N33 N34 N35 N36 N37 N38 N39 N40 N41 N42 N43 N2:N3 N44:N1048576">
+      <formula1>"INST_VALID,INST_INVALID"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I4 I5 I6 I7 I8 I9 I10 I11 I12 I13 I14 I15 I16 I17 I18 I19 I20 I21 I22 I23 I24 I25 I26 I27 I28 I29 I30 I31 I32 I33 I34 I35 I36 I37 I38 I39 I40 I41 I42 I43 I2:I3 I44:I1048576">
       <formula1>"LD_LB,LD_LH,LD_LW,LD_LBU,LD_LHU,LD_XX"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G4 G5 G6 G7 G8 G9 G10 G11 G12 G13 G14 G15 G16 G17 G18 G19 G20 G21 G22 G23 G24 G25 G26 G27 G28 G29 G30 G31 G32 G33 G34 G35 G36 G37 G38 G39 G40 G41 G42 G43 G2:G3 G44:G1048576">
-      <formula1>"IMM_I,IMM_J,IMM_U,IMM_S,IMM_B"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F6 F15 F18 F19 F20 F21 F24 F25 F26 F27 F28 F29 F30 F31 F32 F33 F36 F37 F38 F39 F40 F41 F42 F43 F2:F5 F7:F14 F16:F17 F22:F23 F34:F35 F44:F1048576">
+      <formula1>"ALU_ADD,ALU_SUB,ALU_AND,ALU_OR,ALU_XOR,ALU_SLL,ALU_SRL,ALU_SLT,ALU_SLTU,ALU_COPY_A,ALU_COPY_B,ALU_SRA"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K4 K5 K6 K7 K8 K9 K10 K11 K12 K13 K14 K15 K16 K17 K18 K19 K20 K21 K22 K23 K24 K25 K26 K27 K28 K29 K30 K31 K32 K33 K34 K35 K36 K37 K38 K39 K40 K41 K42 K43 K2:K3 K44:K1048576">
+      <formula1>"MASK_XX,MASK_B,MASK_H,MASK_W,MASK_D"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D4 D5 D6 D7 D8 D9 D10 D11 D12 D13 D14 D15 D16 D17 D18 D19 D20 D21 D22 D23 D24 D25 D26 D27 D28 D29 D30 D31 D32 D33 D34 D35 D36 D37 D38 D39 D40 D41 D42 D43 D2:D3 D44:D1048576">
+      <formula1>"A_PC,A_RS1"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
> compile NEMU ysyx_23060246 韩炳晋 Linux archlinux 6.12.17-1-lts #1 SMP PREEMPT_DYNAMIC Thu, 27 Feb 2025 14:12:30 +0000 x86_64 GNU/Linux  14:06:31 up 17:56,  1 user,  load average: 0.56, 1.11, 2.79
</commit_message>
<xml_diff>
--- a/npc/tools/control_gen/control_table.xlsx
+++ b/npc/tools/control_gen/control_table.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="355" uniqueCount="119">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="311" uniqueCount="112">
   <si>
     <t>comment</t>
   </si>
@@ -76,9 +76,6 @@
     <t>INST_VALID</t>
   </si>
   <si>
-    <t>U_TYPE</t>
-  </si>
-  <si>
     <t>auipc</t>
   </si>
   <si>
@@ -97,9 +94,6 @@
     <t>IMM_I</t>
   </si>
   <si>
-    <t>I_TYPE</t>
-  </si>
-  <si>
     <t>andi</t>
   </si>
   <si>
@@ -133,9 +127,6 @@
     <t>IMM_J</t>
   </si>
   <si>
-    <t>J_TYPE</t>
-  </si>
-  <si>
     <t>sb</t>
   </si>
   <si>
@@ -148,9 +139,6 @@
     <t>MASK_B</t>
   </si>
   <si>
-    <t>S_TYPE</t>
-  </si>
-  <si>
     <t>sh</t>
   </si>
   <si>
@@ -211,9 +199,6 @@
     <t>BR_NE</t>
   </si>
   <si>
-    <t>B_TYPE</t>
-  </si>
-  <si>
     <t>beq</t>
   </si>
   <si>
@@ -262,9 +247,6 @@
     <t>B_RS2</t>
   </si>
   <si>
-    <t>R_TYPE</t>
-  </si>
-  <si>
     <t>sra</t>
   </si>
   <si>
@@ -338,9 +320,6 @@
   </si>
   <si>
     <t>CSR_P</t>
-  </si>
-  <si>
-    <t>N_TYPE</t>
   </si>
   <si>
     <t>mret</t>
@@ -379,9 +358,9 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="4">
     <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="42" formatCode="_ &quot;￥&quot;* #,##0_ ;_ &quot;￥&quot;* \-#,##0_ ;_ &quot;￥&quot;* &quot;-&quot;_ ;_ @_ "/>
     <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="41" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
+    <numFmt numFmtId="42" formatCode="_ &quot;￥&quot;* #,##0_ ;_ &quot;￥&quot;* \-#,##0_ ;_ &quot;￥&quot;* &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
   <fonts count="22">
     <font>
@@ -399,6 +378,21 @@
     </font>
     <font>
       <sz val="10.8"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="3"/>
       <name val="宋体"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -425,29 +419,6 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF0000FF"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="3"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <b/>
       <sz val="18"/>
       <color theme="3"/>
@@ -461,6 +432,22 @@
       <color rgb="FF800080"/>
       <name val="宋体"/>
       <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color rgb="FF7F7F7F"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="15"/>
+      <color theme="3"/>
+      <name val="宋体"/>
+      <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -489,7 +476,14 @@
     <font>
       <b/>
       <sz val="11"/>
-      <color theme="1"/>
+      <color rgb="FFFA7D00"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF3F3F76"/>
       <name val="宋体"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -503,8 +497,24 @@
     </font>
     <font>
       <b/>
+      <sz val="13"/>
+      <color theme="3"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
       <sz val="11"/>
-      <color rgb="FFFA7D00"/>
+      <color rgb="FF0000FF"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="宋体"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -512,37 +522,6 @@
     <font>
       <sz val="11"/>
       <color rgb="FF006100"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="13"/>
-      <color theme="3"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="15"/>
-      <color theme="3"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="11"/>
-      <color rgb="FF7F7F7F"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF3F3F76"/>
       <name val="宋体"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -557,13 +536,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9"/>
+        <fgColor theme="8" tint="0.599993896298105"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -581,67 +554,19 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.599993896298105"/>
+        <fgColor theme="9"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.399975585192419"/>
+        <fgColor theme="7" tint="0.599993896298105"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFF2F2F2"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.599993896298105"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -659,7 +584,61 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FFFFCC99"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor theme="4" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.399975585192419"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -671,19 +650,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.799981688894314"/>
+        <fgColor theme="8" tint="0.799981688894314"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
+        <fgColor theme="7" tint="0.399975585192419"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -695,19 +668,25 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor theme="8" tint="0.399975585192419"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="4"/>
+        <fgColor theme="6" tint="0.799981688894314"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5"/>
+        <fgColor theme="9" tint="0.399975585192419"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -719,25 +698,25 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="6"/>
+        <fgColor theme="7"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
+        <fgColor theme="5" tint="0.599993896298105"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.799981688894314"/>
+        <fgColor theme="6" tint="0.599993896298105"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.399975585192419"/>
+        <fgColor rgb="FFC6EFCE"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -748,6 +727,24 @@
       <right/>
       <top/>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="double">
+        <color rgb="FFFF8001"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4" tint="0.499984740745262"/>
+      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -769,17 +766,8 @@
       <left/>
       <right/>
       <top/>
-      <bottom style="double">
-        <color rgb="FFFF8001"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
       <bottom style="medium">
-        <color theme="4" tint="0.499984740745262"/>
+        <color theme="4"/>
       </bottom>
       <diagonal/>
     </border>
@@ -814,17 +802,6 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color theme="4"/>
-      </top>
-      <bottom style="double">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
       <left style="thin">
         <color rgb="FF7F7F7F"/>
       </left>
@@ -842,8 +819,10 @@
     <border>
       <left/>
       <right/>
-      <top/>
-      <bottom style="medium">
+      <top style="thin">
+        <color theme="4"/>
+      </top>
+      <bottom style="double">
         <color theme="4"/>
       </bottom>
       <diagonal/>
@@ -853,148 +832,148 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="30" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="6" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="10" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="6" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="15" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="17" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="15" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="6" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="7" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="8" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="7" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="5" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
@@ -1339,7 +1318,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:AJ99"/>
+  <dimension ref="A1:AI99"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
     <col min="1" max="1" width="13.1" customWidth="1"/>
@@ -1352,18 +1331,18 @@
     <col min="8" max="10" width="11.9833333333333" customWidth="1"/>
     <col min="11" max="11" width="15.075" customWidth="1"/>
     <col min="12" max="14" width="12.1083333333333" customWidth="1"/>
-    <col min="15" max="16" width="10.8583333333333" customWidth="1"/>
-    <col min="18" max="18" width="14.2166666666667" customWidth="1"/>
-    <col min="19" max="19" width="11.8083333333333" customWidth="1"/>
-    <col min="20" max="20" width="10.6" customWidth="1"/>
-    <col min="21" max="21" width="9.70833333333333" customWidth="1"/>
-    <col min="22" max="22" width="11.1666666666667" customWidth="1"/>
-    <col min="23" max="23" width="11.4083333333333" customWidth="1"/>
-    <col min="24" max="24" width="12.0583333333333" customWidth="1"/>
-    <col min="25" max="25" width="15.575" customWidth="1"/>
+    <col min="15" max="15" width="10.8583333333333" customWidth="1"/>
+    <col min="17" max="17" width="14.2166666666667" customWidth="1"/>
+    <col min="18" max="18" width="11.8083333333333" customWidth="1"/>
+    <col min="19" max="19" width="10.6" customWidth="1"/>
+    <col min="20" max="20" width="9.70833333333333" customWidth="1"/>
+    <col min="21" max="21" width="11.1666666666667" customWidth="1"/>
+    <col min="22" max="22" width="11.4083333333333" customWidth="1"/>
+    <col min="23" max="23" width="12.0583333333333" customWidth="1"/>
+    <col min="24" max="24" width="15.575" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="15" customHeight="1" spans="1:24">
+    <row r="1" ht="15" customHeight="1" spans="1:23">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1406,18 +1385,15 @@
       <c r="N1" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="2" t="s">
-        <v>1</v>
-      </c>
+      <c r="O1" s="2"/>
       <c r="P1" s="2"/>
       <c r="Q1" s="2"/>
       <c r="R1" s="2"/>
       <c r="S1" s="2"/>
       <c r="T1" s="2"/>
-      <c r="U1" s="2"/>
-      <c r="X1" s="6"/>
-    </row>
-    <row r="2" spans="1:36">
+      <c r="W1" s="6"/>
+    </row>
+    <row r="2" spans="1:35">
       <c r="A2" s="3"/>
       <c r="B2" s="4" t="s">
         <v>14</v>
@@ -1444,15 +1420,13 @@
       <c r="N2" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O2" s="4" t="s">
-        <v>20</v>
-      </c>
+      <c r="O2" s="4"/>
       <c r="P2" s="4"/>
       <c r="Q2" s="4"/>
       <c r="R2" s="4"/>
       <c r="S2" s="4"/>
       <c r="T2" s="4"/>
-      <c r="U2" s="4"/>
+      <c r="U2" s="3"/>
       <c r="V2" s="3"/>
       <c r="W2" s="3"/>
       <c r="X2" s="3"/>
@@ -1467,22 +1441,21 @@
       <c r="AG2" s="3"/>
       <c r="AH2" s="3"/>
       <c r="AI2" s="3"/>
-      <c r="AJ2" s="3"/>
-    </row>
-    <row r="3" spans="1:36">
+    </row>
+    <row r="3" spans="1:35">
       <c r="A3" s="3"/>
       <c r="B3" s="4" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C3" s="2"/>
       <c r="D3" s="4" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E3" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G3" s="4" t="s">
         <v>17</v>
@@ -1498,15 +1471,13 @@
       <c r="N3" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O3" s="4" t="s">
-        <v>20</v>
-      </c>
+      <c r="O3" s="4"/>
       <c r="P3" s="4"/>
       <c r="Q3" s="4"/>
       <c r="R3" s="4"/>
       <c r="S3" s="4"/>
       <c r="T3" s="4"/>
-      <c r="U3" s="4"/>
+      <c r="U3" s="3"/>
       <c r="V3" s="3"/>
       <c r="W3" s="3"/>
       <c r="X3" s="3"/>
@@ -1521,25 +1492,24 @@
       <c r="AG3" s="3"/>
       <c r="AH3" s="3"/>
       <c r="AI3" s="3"/>
-      <c r="AJ3" s="3"/>
-    </row>
-    <row r="4" spans="1:36">
+    </row>
+    <row r="4" spans="1:35">
       <c r="A4" s="3"/>
       <c r="B4" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C4" s="2"/>
       <c r="D4" s="4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E4" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="H4" s="4" t="s">
         <v>18</v>
@@ -1552,15 +1522,13 @@
       <c r="N4" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O4" s="4" t="s">
-        <v>27</v>
-      </c>
+      <c r="O4" s="4"/>
       <c r="P4" s="4"/>
       <c r="Q4" s="4"/>
       <c r="R4" s="4"/>
       <c r="S4" s="4"/>
       <c r="T4" s="4"/>
-      <c r="U4" s="4"/>
+      <c r="U4" s="3"/>
       <c r="V4" s="3"/>
       <c r="W4" s="3"/>
       <c r="X4" s="3"/>
@@ -1575,25 +1543,24 @@
       <c r="AG4" s="3"/>
       <c r="AH4" s="3"/>
       <c r="AI4" s="3"/>
-      <c r="AJ4" s="3"/>
-    </row>
-    <row r="5" spans="1:36">
+    </row>
+    <row r="5" spans="1:35">
       <c r="A5" s="3"/>
       <c r="B5" s="4" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="C5" s="2"/>
       <c r="D5" s="4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E5" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="H5" s="4" t="s">
         <v>18</v>
@@ -1606,15 +1573,13 @@
       <c r="N5" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O5" s="4" t="s">
-        <v>27</v>
-      </c>
+      <c r="O5" s="4"/>
       <c r="P5" s="4"/>
       <c r="Q5" s="4"/>
       <c r="R5" s="4"/>
       <c r="S5" s="4"/>
       <c r="T5" s="4"/>
-      <c r="U5" s="4"/>
+      <c r="U5" s="3"/>
       <c r="V5" s="3"/>
       <c r="W5" s="3"/>
       <c r="X5" s="3"/>
@@ -1629,25 +1594,24 @@
       <c r="AG5" s="3"/>
       <c r="AH5" s="3"/>
       <c r="AI5" s="3"/>
-      <c r="AJ5" s="3"/>
-    </row>
-    <row r="6" spans="1:36">
+    </row>
+    <row r="6" spans="1:35">
       <c r="A6" s="3"/>
       <c r="B6" s="4" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="C6" s="2"/>
       <c r="D6" s="4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E6" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="G6" s="4" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="H6" s="4" t="s">
         <v>18</v>
@@ -1660,15 +1624,13 @@
       <c r="N6" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O6" s="4" t="s">
-        <v>27</v>
-      </c>
+      <c r="O6" s="4"/>
       <c r="P6" s="4"/>
       <c r="Q6" s="4"/>
       <c r="R6" s="4"/>
       <c r="S6" s="4"/>
       <c r="T6" s="4"/>
-      <c r="U6" s="4"/>
+      <c r="U6" s="3"/>
       <c r="V6" s="3"/>
       <c r="W6" s="3"/>
       <c r="X6" s="3"/>
@@ -1683,25 +1645,24 @@
       <c r="AG6" s="3"/>
       <c r="AH6" s="3"/>
       <c r="AI6" s="3"/>
-      <c r="AJ6" s="3"/>
-    </row>
-    <row r="7" spans="1:36">
+    </row>
+    <row r="7" spans="1:35">
       <c r="A7" s="3"/>
       <c r="B7" s="4" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="C7" s="2"/>
       <c r="D7" s="4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E7" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="G7" s="4" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="H7" s="4" t="s">
         <v>18</v>
@@ -1714,15 +1675,13 @@
       <c r="N7" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O7" s="4" t="s">
-        <v>27</v>
-      </c>
+      <c r="O7" s="4"/>
       <c r="P7" s="4"/>
       <c r="Q7" s="4"/>
       <c r="R7" s="4"/>
       <c r="S7" s="4"/>
       <c r="T7" s="4"/>
-      <c r="U7" s="4"/>
+      <c r="U7" s="3"/>
       <c r="V7" s="3"/>
       <c r="W7" s="3"/>
       <c r="X7" s="3"/>
@@ -1737,30 +1696,29 @@
       <c r="AG7" s="3"/>
       <c r="AH7" s="3"/>
       <c r="AI7" s="3"/>
-      <c r="AJ7" s="3"/>
-    </row>
-    <row r="8" spans="1:36">
+    </row>
+    <row r="8" spans="1:35">
       <c r="A8" s="3"/>
       <c r="B8" s="4" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E8" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F8" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G8" s="4" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="H8" s="4" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="I8" s="4"/>
       <c r="J8" s="4"/>
@@ -1770,15 +1728,13 @@
       <c r="N8" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O8" s="4" t="s">
-        <v>27</v>
-      </c>
+      <c r="O8" s="4"/>
       <c r="P8" s="4"/>
       <c r="Q8" s="4"/>
       <c r="R8" s="4"/>
       <c r="S8" s="4"/>
       <c r="T8" s="4"/>
-      <c r="U8" s="4"/>
+      <c r="U8" s="3"/>
       <c r="V8" s="3"/>
       <c r="W8" s="3"/>
       <c r="X8" s="3"/>
@@ -1793,30 +1749,29 @@
       <c r="AG8" s="3"/>
       <c r="AH8" s="3"/>
       <c r="AI8" s="3"/>
-      <c r="AJ8" s="3"/>
-    </row>
-    <row r="9" spans="1:36">
+    </row>
+    <row r="9" spans="1:35">
       <c r="A9" s="3"/>
       <c r="B9" s="4" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E9" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F9" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G9" s="4" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="H9" s="4" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="I9" s="4"/>
       <c r="J9" s="4"/>
@@ -1826,15 +1781,13 @@
       <c r="N9" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O9" s="4" t="s">
-        <v>39</v>
-      </c>
+      <c r="O9" s="4"/>
       <c r="P9" s="4"/>
       <c r="Q9" s="4"/>
       <c r="R9" s="4"/>
       <c r="S9" s="4"/>
       <c r="T9" s="4"/>
-      <c r="U9" s="4"/>
+      <c r="U9" s="3"/>
       <c r="V9" s="3"/>
       <c r="W9" s="3"/>
       <c r="X9" s="3"/>
@@ -1849,48 +1802,45 @@
       <c r="AG9" s="3"/>
       <c r="AH9" s="3"/>
       <c r="AI9" s="3"/>
-      <c r="AJ9" s="3"/>
-    </row>
-    <row r="10" spans="1:36">
+    </row>
+    <row r="10" spans="1:35">
       <c r="A10" s="3"/>
       <c r="B10" s="4" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="C10" s="2"/>
       <c r="D10" s="4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E10" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F10" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G10" s="4" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="H10" s="4"/>
       <c r="I10" s="4"/>
       <c r="J10" s="4" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="K10" s="4" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="L10" s="4"/>
       <c r="M10" s="4"/>
       <c r="N10" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O10" s="4" t="s">
-        <v>44</v>
-      </c>
+      <c r="O10" s="4"/>
       <c r="P10" s="4"/>
       <c r="Q10" s="4"/>
       <c r="R10" s="4"/>
       <c r="S10" s="4"/>
       <c r="T10" s="4"/>
-      <c r="U10" s="4"/>
+      <c r="U10" s="3"/>
       <c r="V10" s="3"/>
       <c r="W10" s="3"/>
       <c r="X10" s="3"/>
@@ -1905,48 +1855,45 @@
       <c r="AG10" s="3"/>
       <c r="AH10" s="3"/>
       <c r="AI10" s="3"/>
-      <c r="AJ10" s="3"/>
-    </row>
-    <row r="11" spans="1:36">
+    </row>
+    <row r="11" spans="1:35">
       <c r="A11" s="3"/>
       <c r="B11" s="4" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="C11" s="2"/>
       <c r="D11" s="4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E11" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F11" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G11" s="4" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="H11" s="4"/>
       <c r="I11" s="4"/>
       <c r="J11" s="4" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="K11" s="4" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="L11" s="4"/>
       <c r="M11" s="4"/>
       <c r="N11" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O11" s="4" t="s">
-        <v>44</v>
-      </c>
+      <c r="O11" s="4"/>
       <c r="P11" s="4"/>
       <c r="Q11" s="4"/>
       <c r="R11" s="4"/>
       <c r="S11" s="4"/>
       <c r="T11" s="4"/>
-      <c r="U11" s="4"/>
+      <c r="U11" s="3"/>
       <c r="V11" s="3"/>
       <c r="W11" s="3"/>
       <c r="X11" s="3"/>
@@ -1961,48 +1908,45 @@
       <c r="AG11" s="3"/>
       <c r="AH11" s="3"/>
       <c r="AI11" s="3"/>
-      <c r="AJ11" s="3"/>
-    </row>
-    <row r="12" spans="1:36">
+    </row>
+    <row r="12" spans="1:35">
       <c r="A12" s="3"/>
       <c r="B12" s="4" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="C12" s="2"/>
       <c r="D12" s="4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E12" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F12" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G12" s="4" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="H12" s="4"/>
       <c r="I12" s="4"/>
       <c r="J12" s="4" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="K12" s="4" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="L12" s="4"/>
       <c r="M12" s="4"/>
       <c r="N12" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O12" s="4" t="s">
-        <v>44</v>
-      </c>
+      <c r="O12" s="4"/>
       <c r="P12" s="4"/>
       <c r="Q12" s="4"/>
       <c r="R12" s="4"/>
       <c r="S12" s="4"/>
       <c r="T12" s="4"/>
-      <c r="U12" s="4"/>
+      <c r="U12" s="3"/>
       <c r="V12" s="3"/>
       <c r="W12" s="3"/>
       <c r="X12" s="3"/>
@@ -2017,31 +1961,30 @@
       <c r="AG12" s="3"/>
       <c r="AH12" s="3"/>
       <c r="AI12" s="3"/>
-      <c r="AJ12" s="3"/>
-    </row>
-    <row r="13" spans="1:36">
+    </row>
+    <row r="13" spans="1:35">
       <c r="A13" s="3"/>
       <c r="B13" s="4" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="C13" s="2"/>
       <c r="D13" s="4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E13" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F13" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G13" s="4" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="H13" s="4" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="I13" s="4" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="J13" s="4"/>
       <c r="K13" s="4"/>
@@ -2050,15 +1993,13 @@
       <c r="N13" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O13" s="4" t="s">
-        <v>27</v>
-      </c>
+      <c r="O13" s="4"/>
       <c r="P13" s="4"/>
       <c r="Q13" s="4"/>
       <c r="R13" s="4"/>
       <c r="S13" s="4"/>
       <c r="T13" s="4"/>
-      <c r="U13" s="4"/>
+      <c r="U13" s="3"/>
       <c r="V13" s="3"/>
       <c r="W13" s="3"/>
       <c r="X13" s="3"/>
@@ -2073,31 +2014,30 @@
       <c r="AG13" s="3"/>
       <c r="AH13" s="3"/>
       <c r="AI13" s="3"/>
-      <c r="AJ13" s="3"/>
-    </row>
-    <row r="14" spans="1:36">
+    </row>
+    <row r="14" spans="1:35">
       <c r="A14" s="3"/>
       <c r="B14" s="4" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="C14" s="2"/>
       <c r="D14" s="4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E14" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F14" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G14" s="4" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="H14" s="4" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="I14" s="4" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="J14" s="4"/>
       <c r="K14" s="4"/>
@@ -2106,15 +2046,13 @@
       <c r="N14" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O14" s="4" t="s">
-        <v>27</v>
-      </c>
+      <c r="O14" s="4"/>
       <c r="P14" s="4"/>
       <c r="Q14" s="4"/>
       <c r="R14" s="4"/>
       <c r="S14" s="4"/>
       <c r="T14" s="4"/>
-      <c r="U14" s="4"/>
+      <c r="U14" s="3"/>
       <c r="V14" s="3"/>
       <c r="W14" s="3"/>
       <c r="X14" s="3"/>
@@ -2129,31 +2067,30 @@
       <c r="AG14" s="3"/>
       <c r="AH14" s="3"/>
       <c r="AI14" s="3"/>
-      <c r="AJ14" s="3"/>
-    </row>
-    <row r="15" spans="1:36">
+    </row>
+    <row r="15" spans="1:35">
       <c r="A15" s="3"/>
       <c r="B15" s="4" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="C15" s="2"/>
       <c r="D15" s="4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E15" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F15" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G15" s="4" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="H15" s="4" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="I15" s="4" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="J15" s="4"/>
       <c r="K15" s="4"/>
@@ -2162,15 +2099,13 @@
       <c r="N15" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O15" s="4" t="s">
-        <v>27</v>
-      </c>
+      <c r="O15" s="4"/>
       <c r="P15" s="4"/>
       <c r="Q15" s="4"/>
       <c r="R15" s="4"/>
       <c r="S15" s="4"/>
       <c r="T15" s="4"/>
-      <c r="U15" s="4"/>
+      <c r="U15" s="3"/>
       <c r="V15" s="3"/>
       <c r="W15" s="3"/>
       <c r="X15" s="3"/>
@@ -2185,31 +2120,30 @@
       <c r="AG15" s="3"/>
       <c r="AH15" s="3"/>
       <c r="AI15" s="3"/>
-      <c r="AJ15" s="3"/>
-    </row>
-    <row r="16" spans="1:36">
+    </row>
+    <row r="16" spans="1:35">
       <c r="A16" s="3"/>
       <c r="B16" s="4" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="C16" s="2"/>
       <c r="D16" s="4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E16" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F16" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G16" s="4" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="H16" s="4" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="I16" s="4" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="J16" s="4"/>
       <c r="K16" s="4"/>
@@ -2218,15 +2152,13 @@
       <c r="N16" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O16" s="4" t="s">
-        <v>27</v>
-      </c>
+      <c r="O16" s="4"/>
       <c r="P16" s="4"/>
       <c r="Q16" s="4"/>
       <c r="R16" s="4"/>
       <c r="S16" s="4"/>
       <c r="T16" s="4"/>
-      <c r="U16" s="4"/>
+      <c r="U16" s="3"/>
       <c r="V16" s="3"/>
       <c r="W16" s="3"/>
       <c r="X16" s="3"/>
@@ -2241,31 +2173,30 @@
       <c r="AG16" s="3"/>
       <c r="AH16" s="3"/>
       <c r="AI16" s="3"/>
-      <c r="AJ16" s="3"/>
-    </row>
-    <row r="17" spans="1:36">
+    </row>
+    <row r="17" spans="1:35">
       <c r="A17" s="3"/>
       <c r="B17" s="4" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="C17" s="2"/>
       <c r="D17" s="4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E17" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F17" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G17" s="4" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="H17" s="4" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="I17" s="4" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="J17" s="4"/>
       <c r="K17" s="4"/>
@@ -2274,15 +2205,13 @@
       <c r="N17" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O17" s="4" t="s">
-        <v>27</v>
-      </c>
+      <c r="O17" s="4"/>
       <c r="P17" s="4"/>
       <c r="Q17" s="4"/>
       <c r="R17" s="4"/>
       <c r="S17" s="4"/>
       <c r="T17" s="4"/>
-      <c r="U17" s="4"/>
+      <c r="U17" s="3"/>
       <c r="V17" s="3"/>
       <c r="W17" s="3"/>
       <c r="X17" s="3"/>
@@ -2297,46 +2226,43 @@
       <c r="AG17" s="3"/>
       <c r="AH17" s="3"/>
       <c r="AI17" s="3"/>
-      <c r="AJ17" s="3"/>
-    </row>
-    <row r="18" spans="1:36">
+    </row>
+    <row r="18" spans="1:35">
       <c r="A18" s="3"/>
       <c r="B18" s="4" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="C18" s="2"/>
       <c r="D18" s="4" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E18" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F18" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G18" s="4" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="H18" s="4"/>
       <c r="I18" s="4"/>
       <c r="J18" s="4"/>
       <c r="K18" s="4"/>
       <c r="L18" s="4" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="M18" s="4"/>
       <c r="N18" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O18" s="4" t="s">
-        <v>65</v>
-      </c>
+      <c r="O18" s="4"/>
       <c r="P18" s="4"/>
       <c r="Q18" s="4"/>
       <c r="R18" s="4"/>
       <c r="S18" s="4"/>
       <c r="T18" s="4"/>
-      <c r="U18" s="4"/>
+      <c r="U18" s="3"/>
       <c r="V18" s="3"/>
       <c r="W18" s="3"/>
       <c r="X18" s="3"/>
@@ -2351,46 +2277,43 @@
       <c r="AG18" s="3"/>
       <c r="AH18" s="3"/>
       <c r="AI18" s="3"/>
-      <c r="AJ18" s="3"/>
-    </row>
-    <row r="19" spans="1:36">
+    </row>
+    <row r="19" spans="1:35">
       <c r="A19" s="3"/>
       <c r="B19" s="4" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
       <c r="C19" s="2"/>
       <c r="D19" s="4" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E19" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F19" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G19" s="4" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="H19" s="4"/>
       <c r="I19" s="4"/>
       <c r="J19" s="4"/>
       <c r="K19" s="4"/>
       <c r="L19" s="4" t="s">
-        <v>67</v>
+        <v>62</v>
       </c>
       <c r="M19" s="4"/>
       <c r="N19" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O19" s="4" t="s">
-        <v>65</v>
-      </c>
+      <c r="O19" s="4"/>
       <c r="P19" s="4"/>
       <c r="Q19" s="4"/>
       <c r="R19" s="4"/>
       <c r="S19" s="4"/>
       <c r="T19" s="4"/>
-      <c r="U19" s="4"/>
+      <c r="U19" s="3"/>
       <c r="V19" s="3"/>
       <c r="W19" s="3"/>
       <c r="X19" s="3"/>
@@ -2405,46 +2328,43 @@
       <c r="AG19" s="3"/>
       <c r="AH19" s="3"/>
       <c r="AI19" s="3"/>
-      <c r="AJ19" s="3"/>
-    </row>
-    <row r="20" spans="1:36">
+    </row>
+    <row r="20" spans="1:35">
       <c r="A20" s="3"/>
       <c r="B20" s="4" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="C20" s="2"/>
       <c r="D20" s="4" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E20" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F20" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G20" s="4" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="H20" s="4"/>
       <c r="I20" s="4"/>
       <c r="J20" s="4"/>
       <c r="K20" s="4"/>
       <c r="L20" s="4" t="s">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="M20" s="4"/>
       <c r="N20" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O20" s="4" t="s">
-        <v>65</v>
-      </c>
+      <c r="O20" s="4"/>
       <c r="P20" s="4"/>
       <c r="Q20" s="4"/>
       <c r="R20" s="4"/>
       <c r="S20" s="4"/>
       <c r="T20" s="4"/>
-      <c r="U20" s="4"/>
+      <c r="U20" s="3"/>
       <c r="V20" s="3"/>
       <c r="W20" s="3"/>
       <c r="X20" s="3"/>
@@ -2459,46 +2379,43 @@
       <c r="AG20" s="3"/>
       <c r="AH20" s="3"/>
       <c r="AI20" s="3"/>
-      <c r="AJ20" s="3"/>
-    </row>
-    <row r="21" spans="1:36">
+    </row>
+    <row r="21" spans="1:35">
       <c r="A21" s="3"/>
       <c r="B21" s="4" t="s">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="C21" s="2"/>
       <c r="D21" s="4" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E21" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F21" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G21" s="4" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="H21" s="4"/>
       <c r="I21" s="4"/>
       <c r="J21" s="4"/>
       <c r="K21" s="4"/>
       <c r="L21" s="4" t="s">
-        <v>71</v>
+        <v>66</v>
       </c>
       <c r="M21" s="4"/>
       <c r="N21" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O21" s="4" t="s">
-        <v>65</v>
-      </c>
+      <c r="O21" s="4"/>
       <c r="P21" s="4"/>
       <c r="Q21" s="4"/>
       <c r="R21" s="4"/>
       <c r="S21" s="4"/>
       <c r="T21" s="4"/>
-      <c r="U21" s="4"/>
+      <c r="U21" s="3"/>
       <c r="V21" s="3"/>
       <c r="W21" s="3"/>
       <c r="X21" s="3"/>
@@ -2513,46 +2430,43 @@
       <c r="AG21" s="3"/>
       <c r="AH21" s="3"/>
       <c r="AI21" s="3"/>
-      <c r="AJ21" s="3"/>
-    </row>
-    <row r="22" spans="1:36">
+    </row>
+    <row r="22" spans="1:35">
       <c r="A22" s="3"/>
       <c r="B22" s="4" t="s">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="C22" s="2"/>
       <c r="D22" s="4" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E22" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F22" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G22" s="4" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="H22" s="4"/>
       <c r="I22" s="4"/>
       <c r="J22" s="4"/>
       <c r="K22" s="4"/>
       <c r="L22" s="4" t="s">
-        <v>73</v>
+        <v>68</v>
       </c>
       <c r="M22" s="4"/>
       <c r="N22" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O22" s="4" t="s">
-        <v>65</v>
-      </c>
+      <c r="O22" s="4"/>
       <c r="P22" s="4"/>
       <c r="Q22" s="4"/>
       <c r="R22" s="4"/>
       <c r="S22" s="4"/>
       <c r="T22" s="4"/>
-      <c r="U22" s="4"/>
+      <c r="U22" s="3"/>
       <c r="V22" s="3"/>
       <c r="W22" s="3"/>
       <c r="X22" s="3"/>
@@ -2567,46 +2481,43 @@
       <c r="AG22" s="3"/>
       <c r="AH22" s="3"/>
       <c r="AI22" s="3"/>
-      <c r="AJ22" s="3"/>
-    </row>
-    <row r="23" spans="1:36">
+    </row>
+    <row r="23" spans="1:35">
       <c r="A23" s="3"/>
       <c r="B23" s="4" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="C23" s="2"/>
       <c r="D23" s="4" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E23" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F23" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G23" s="4" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="H23" s="4"/>
       <c r="I23" s="4"/>
       <c r="J23" s="4"/>
       <c r="K23" s="4"/>
       <c r="L23" s="4" t="s">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="M23" s="4"/>
       <c r="N23" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O23" s="4" t="s">
-        <v>65</v>
-      </c>
+      <c r="O23" s="4"/>
       <c r="P23" s="4"/>
       <c r="Q23" s="4"/>
       <c r="R23" s="4"/>
       <c r="S23" s="4"/>
       <c r="T23" s="4"/>
-      <c r="U23" s="4"/>
+      <c r="U23" s="3"/>
       <c r="V23" s="3"/>
       <c r="W23" s="3"/>
       <c r="X23" s="3"/>
@@ -2621,25 +2532,24 @@
       <c r="AG23" s="3"/>
       <c r="AH23" s="3"/>
       <c r="AI23" s="3"/>
-      <c r="AJ23" s="3"/>
-    </row>
-    <row r="24" spans="1:36">
+    </row>
+    <row r="24" spans="1:35">
       <c r="A24" s="3"/>
       <c r="B24" s="4" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="C24" s="2"/>
       <c r="D24" s="4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E24" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F24" s="4" t="s">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="G24" s="4" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="H24" s="4" t="s">
         <v>18</v>
@@ -2652,15 +2562,13 @@
       <c r="N24" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O24" s="4" t="s">
-        <v>27</v>
-      </c>
+      <c r="O24" s="4"/>
       <c r="P24" s="4"/>
       <c r="Q24" s="4"/>
       <c r="R24" s="4"/>
       <c r="S24" s="4"/>
       <c r="T24" s="4"/>
-      <c r="U24" s="4"/>
+      <c r="U24" s="3"/>
       <c r="V24" s="3"/>
       <c r="W24" s="3"/>
       <c r="X24" s="3"/>
@@ -2675,25 +2583,24 @@
       <c r="AG24" s="3"/>
       <c r="AH24" s="3"/>
       <c r="AI24" s="3"/>
-      <c r="AJ24" s="3"/>
-    </row>
-    <row r="25" spans="1:36">
+    </row>
+    <row r="25" spans="1:35">
       <c r="A25" s="3"/>
       <c r="B25" s="4" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="C25" s="2"/>
       <c r="D25" s="4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E25" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F25" s="4" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="G25" s="4" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="H25" s="4" t="s">
         <v>18</v>
@@ -2706,15 +2613,13 @@
       <c r="N25" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O25" s="4" t="s">
-        <v>27</v>
-      </c>
+      <c r="O25" s="4"/>
       <c r="P25" s="4"/>
       <c r="Q25" s="4"/>
       <c r="R25" s="4"/>
       <c r="S25" s="4"/>
       <c r="T25" s="4"/>
-      <c r="U25" s="4"/>
+      <c r="U25" s="3"/>
       <c r="V25" s="3"/>
       <c r="W25" s="3"/>
       <c r="X25" s="3"/>
@@ -2729,22 +2634,21 @@
       <c r="AG25" s="3"/>
       <c r="AH25" s="3"/>
       <c r="AI25" s="3"/>
-      <c r="AJ25" s="3"/>
-    </row>
-    <row r="26" spans="1:36">
+    </row>
+    <row r="26" spans="1:35">
       <c r="A26" s="3"/>
       <c r="B26" s="4" t="s">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="C26" s="2"/>
       <c r="D26" s="4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E26" s="4" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="F26" s="4" t="s">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="G26" s="4"/>
       <c r="H26" s="4" t="s">
@@ -2758,15 +2662,13 @@
       <c r="N26" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O26" s="4" t="s">
-        <v>82</v>
-      </c>
+      <c r="O26" s="4"/>
       <c r="P26" s="4"/>
       <c r="Q26" s="4"/>
       <c r="R26" s="4"/>
       <c r="S26" s="4"/>
       <c r="T26" s="4"/>
-      <c r="U26" s="4"/>
+      <c r="U26" s="3"/>
       <c r="V26" s="3"/>
       <c r="W26" s="3"/>
       <c r="X26" s="3"/>
@@ -2781,22 +2683,21 @@
       <c r="AG26" s="3"/>
       <c r="AH26" s="3"/>
       <c r="AI26" s="3"/>
-      <c r="AJ26" s="3"/>
-    </row>
-    <row r="27" spans="1:36">
+    </row>
+    <row r="27" spans="1:35">
       <c r="A27" s="3"/>
       <c r="B27" s="4" t="s">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="C27" s="2"/>
       <c r="D27" s="4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E27" s="4" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="F27" s="4" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="G27" s="4"/>
       <c r="H27" s="4" t="s">
@@ -2810,15 +2711,13 @@
       <c r="N27" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O27" s="4" t="s">
-        <v>82</v>
-      </c>
+      <c r="O27" s="4"/>
       <c r="P27" s="4"/>
       <c r="Q27" s="4"/>
       <c r="R27" s="4"/>
       <c r="S27" s="4"/>
       <c r="T27" s="4"/>
-      <c r="U27" s="4"/>
+      <c r="U27" s="3"/>
       <c r="V27" s="3"/>
       <c r="W27" s="3"/>
       <c r="X27" s="3"/>
@@ -2833,25 +2732,24 @@
       <c r="AG27" s="3"/>
       <c r="AH27" s="3"/>
       <c r="AI27" s="3"/>
-      <c r="AJ27" s="3"/>
-    </row>
-    <row r="28" spans="1:36">
+    </row>
+    <row r="28" spans="1:35">
       <c r="A28" s="3"/>
       <c r="B28" s="4" t="s">
-        <v>84</v>
+        <v>78</v>
       </c>
       <c r="C28" s="2"/>
       <c r="D28" s="4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E28" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F28" s="4" t="s">
-        <v>85</v>
+        <v>79</v>
       </c>
       <c r="G28" s="4" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="H28" s="4" t="s">
         <v>18</v>
@@ -2864,15 +2762,13 @@
       <c r="N28" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O28" s="4" t="s">
-        <v>27</v>
-      </c>
+      <c r="O28" s="4"/>
       <c r="P28" s="4"/>
       <c r="Q28" s="4"/>
       <c r="R28" s="4"/>
       <c r="S28" s="4"/>
       <c r="T28" s="4"/>
-      <c r="U28" s="4"/>
+      <c r="U28" s="3"/>
       <c r="V28" s="3"/>
       <c r="W28" s="3"/>
       <c r="X28" s="3"/>
@@ -2887,22 +2783,21 @@
       <c r="AG28" s="3"/>
       <c r="AH28" s="3"/>
       <c r="AI28" s="3"/>
-      <c r="AJ28" s="3"/>
-    </row>
-    <row r="29" spans="1:36">
+    </row>
+    <row r="29" spans="1:35">
       <c r="A29" s="3"/>
       <c r="B29" s="4" t="s">
-        <v>86</v>
+        <v>80</v>
       </c>
       <c r="C29" s="2"/>
       <c r="D29" s="4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E29" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="F29" s="4" t="s">
         <v>81</v>
-      </c>
-      <c r="F29" s="4" t="s">
-        <v>87</v>
       </c>
       <c r="G29" s="4"/>
       <c r="H29" s="4" t="s">
@@ -2916,15 +2811,13 @@
       <c r="N29" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O29" s="4" t="s">
-        <v>82</v>
-      </c>
+      <c r="O29" s="4"/>
       <c r="P29" s="4"/>
       <c r="Q29" s="4"/>
       <c r="R29" s="4"/>
       <c r="S29" s="4"/>
       <c r="T29" s="4"/>
-      <c r="U29" s="4"/>
+      <c r="U29" s="3"/>
       <c r="V29" s="3"/>
       <c r="W29" s="3"/>
       <c r="X29" s="3"/>
@@ -2939,22 +2832,21 @@
       <c r="AG29" s="3"/>
       <c r="AH29" s="3"/>
       <c r="AI29" s="3"/>
-      <c r="AJ29" s="3"/>
-    </row>
-    <row r="30" spans="1:36">
+    </row>
+    <row r="30" spans="1:35">
       <c r="A30" s="3"/>
       <c r="B30" s="4" t="s">
-        <v>88</v>
+        <v>82</v>
       </c>
       <c r="C30" s="2"/>
       <c r="D30" s="4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E30" s="4" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="F30" s="4" t="s">
-        <v>89</v>
+        <v>83</v>
       </c>
       <c r="G30" s="4"/>
       <c r="H30" s="4" t="s">
@@ -2968,15 +2860,13 @@
       <c r="N30" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O30" s="4" t="s">
-        <v>82</v>
-      </c>
+      <c r="O30" s="4"/>
       <c r="P30" s="4"/>
       <c r="Q30" s="4"/>
       <c r="R30" s="4"/>
       <c r="S30" s="4"/>
       <c r="T30" s="4"/>
-      <c r="U30" s="4"/>
+      <c r="U30" s="3"/>
       <c r="V30" s="3"/>
       <c r="W30" s="3"/>
       <c r="X30" s="3"/>
@@ -2991,25 +2881,24 @@
       <c r="AG30" s="3"/>
       <c r="AH30" s="3"/>
       <c r="AI30" s="3"/>
-      <c r="AJ30" s="3"/>
-    </row>
-    <row r="31" spans="1:36">
+    </row>
+    <row r="31" spans="1:35">
       <c r="A31" s="3"/>
       <c r="B31" s="4" t="s">
-        <v>90</v>
+        <v>84</v>
       </c>
       <c r="C31" s="2"/>
       <c r="D31" s="4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E31" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F31" s="4" t="s">
-        <v>89</v>
+        <v>83</v>
       </c>
       <c r="G31" s="4" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="H31" s="4" t="s">
         <v>18</v>
@@ -3022,15 +2911,13 @@
       <c r="N31" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O31" s="4" t="s">
-        <v>27</v>
-      </c>
+      <c r="O31" s="4"/>
       <c r="P31" s="4"/>
       <c r="Q31" s="4"/>
       <c r="R31" s="4"/>
       <c r="S31" s="4"/>
       <c r="T31" s="4"/>
-      <c r="U31" s="4"/>
+      <c r="U31" s="3"/>
       <c r="V31" s="3"/>
       <c r="W31" s="3"/>
       <c r="X31" s="3"/>
@@ -3045,25 +2932,24 @@
       <c r="AG31" s="3"/>
       <c r="AH31" s="3"/>
       <c r="AI31" s="3"/>
-      <c r="AJ31" s="3"/>
-    </row>
-    <row r="32" spans="1:36">
+    </row>
+    <row r="32" spans="1:35">
       <c r="A32" s="3"/>
       <c r="B32" s="4" t="s">
-        <v>91</v>
+        <v>85</v>
       </c>
       <c r="C32" s="2"/>
       <c r="D32" s="4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E32" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F32" s="4" t="s">
-        <v>89</v>
+        <v>83</v>
       </c>
       <c r="G32" s="4" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="H32" s="4" t="s">
         <v>18</v>
@@ -3076,15 +2962,13 @@
       <c r="N32" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O32" s="4" t="s">
-        <v>27</v>
-      </c>
+      <c r="O32" s="4"/>
       <c r="P32" s="4"/>
       <c r="Q32" s="4"/>
       <c r="R32" s="4"/>
       <c r="S32" s="4"/>
       <c r="T32" s="4"/>
-      <c r="U32" s="4"/>
+      <c r="U32" s="3"/>
       <c r="V32" s="3"/>
       <c r="W32" s="3"/>
       <c r="X32" s="3"/>
@@ -3099,22 +2983,21 @@
       <c r="AG32" s="3"/>
       <c r="AH32" s="3"/>
       <c r="AI32" s="3"/>
-      <c r="AJ32" s="3"/>
-    </row>
-    <row r="33" spans="1:36">
+    </row>
+    <row r="33" spans="1:35">
       <c r="A33" s="3"/>
       <c r="B33" s="4" t="s">
-        <v>92</v>
+        <v>86</v>
       </c>
       <c r="C33" s="2"/>
       <c r="D33" s="4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E33" s="4" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="F33" s="4" t="s">
-        <v>85</v>
+        <v>79</v>
       </c>
       <c r="G33" s="4"/>
       <c r="H33" s="4" t="s">
@@ -3128,15 +3011,13 @@
       <c r="N33" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O33" s="4" t="s">
-        <v>82</v>
-      </c>
+      <c r="O33" s="4"/>
       <c r="P33" s="4"/>
       <c r="Q33" s="4"/>
       <c r="R33" s="4"/>
       <c r="S33" s="4"/>
       <c r="T33" s="4"/>
-      <c r="U33" s="4"/>
+      <c r="U33" s="3"/>
       <c r="V33" s="3"/>
       <c r="W33" s="3"/>
       <c r="X33" s="3"/>
@@ -3151,22 +3032,21 @@
       <c r="AG33" s="3"/>
       <c r="AH33" s="3"/>
       <c r="AI33" s="3"/>
-      <c r="AJ33" s="3"/>
-    </row>
-    <row r="34" spans="1:36">
+    </row>
+    <row r="34" spans="1:35">
       <c r="A34" s="3"/>
       <c r="B34" s="4" t="s">
-        <v>93</v>
+        <v>87</v>
       </c>
       <c r="C34" s="2"/>
       <c r="D34" s="4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E34" s="4" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="F34" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G34" s="4"/>
       <c r="H34" s="4" t="s">
@@ -3180,15 +3060,13 @@
       <c r="N34" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O34" s="4" t="s">
-        <v>82</v>
-      </c>
+      <c r="O34" s="4"/>
       <c r="P34" s="4"/>
       <c r="Q34" s="4"/>
       <c r="R34" s="4"/>
       <c r="S34" s="4"/>
       <c r="T34" s="4"/>
-      <c r="U34" s="4"/>
+      <c r="U34" s="3"/>
       <c r="V34" s="3"/>
       <c r="W34" s="3"/>
       <c r="X34" s="3"/>
@@ -3203,22 +3081,21 @@
       <c r="AG34" s="3"/>
       <c r="AH34" s="3"/>
       <c r="AI34" s="3"/>
-      <c r="AJ34" s="3"/>
-    </row>
-    <row r="35" spans="1:36">
+    </row>
+    <row r="35" spans="1:35">
       <c r="A35" s="3"/>
       <c r="B35" s="4" t="s">
-        <v>94</v>
+        <v>88</v>
       </c>
       <c r="C35" s="2"/>
       <c r="D35" s="4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E35" s="4" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="F35" s="4" t="s">
-        <v>95</v>
+        <v>89</v>
       </c>
       <c r="G35" s="4"/>
       <c r="H35" s="4" t="s">
@@ -3232,15 +3109,13 @@
       <c r="N35" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O35" s="4" t="s">
-        <v>82</v>
-      </c>
+      <c r="O35" s="4"/>
       <c r="P35" s="4"/>
       <c r="Q35" s="4"/>
       <c r="R35" s="4"/>
       <c r="S35" s="4"/>
       <c r="T35" s="4"/>
-      <c r="U35" s="4"/>
+      <c r="U35" s="3"/>
       <c r="V35" s="3"/>
       <c r="W35" s="3"/>
       <c r="X35" s="3"/>
@@ -3255,22 +3130,21 @@
       <c r="AG35" s="3"/>
       <c r="AH35" s="3"/>
       <c r="AI35" s="3"/>
-      <c r="AJ35" s="3"/>
-    </row>
-    <row r="36" spans="1:36">
+    </row>
+    <row r="36" spans="1:35">
       <c r="A36" s="3"/>
       <c r="B36" s="4" t="s">
-        <v>96</v>
+        <v>90</v>
       </c>
       <c r="C36" s="2"/>
       <c r="D36" s="4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E36" s="4" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="F36" s="4" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="G36" s="4"/>
       <c r="H36" s="4" t="s">
@@ -3284,15 +3158,13 @@
       <c r="N36" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O36" s="4" t="s">
-        <v>82</v>
-      </c>
+      <c r="O36" s="4"/>
       <c r="P36" s="4"/>
       <c r="Q36" s="4"/>
       <c r="R36" s="4"/>
       <c r="S36" s="4"/>
       <c r="T36" s="4"/>
-      <c r="U36" s="4"/>
+      <c r="U36" s="3"/>
       <c r="V36" s="3"/>
       <c r="W36" s="3"/>
       <c r="X36" s="3"/>
@@ -3307,22 +3179,21 @@
       <c r="AG36" s="3"/>
       <c r="AH36" s="3"/>
       <c r="AI36" s="3"/>
-      <c r="AJ36" s="3"/>
-    </row>
-    <row r="37" spans="1:36">
+    </row>
+    <row r="37" spans="1:35">
       <c r="A37" s="3"/>
       <c r="B37" s="4" t="s">
-        <v>97</v>
+        <v>91</v>
       </c>
       <c r="C37" s="2"/>
       <c r="D37" s="4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E37" s="4" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="F37" s="4" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="G37" s="4"/>
       <c r="H37" s="4" t="s">
@@ -3336,15 +3207,13 @@
       <c r="N37" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O37" s="4" t="s">
-        <v>82</v>
-      </c>
+      <c r="O37" s="4"/>
       <c r="P37" s="4"/>
       <c r="Q37" s="4"/>
       <c r="R37" s="4"/>
       <c r="S37" s="4"/>
       <c r="T37" s="4"/>
-      <c r="U37" s="4"/>
+      <c r="U37" s="3"/>
       <c r="V37" s="3"/>
       <c r="W37" s="3"/>
       <c r="X37" s="3"/>
@@ -3359,22 +3228,21 @@
       <c r="AG37" s="3"/>
       <c r="AH37" s="3"/>
       <c r="AI37" s="3"/>
-      <c r="AJ37" s="3"/>
-    </row>
-    <row r="38" spans="1:36">
+    </row>
+    <row r="38" spans="1:35">
       <c r="A38" s="3"/>
       <c r="B38" s="4" t="s">
-        <v>98</v>
+        <v>92</v>
       </c>
       <c r="C38" s="2"/>
       <c r="D38" s="4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E38" s="4" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="F38" s="4" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="G38" s="4"/>
       <c r="H38" s="4" t="s">
@@ -3388,15 +3256,13 @@
       <c r="N38" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O38" s="4" t="s">
-        <v>82</v>
-      </c>
+      <c r="O38" s="4"/>
       <c r="P38" s="4"/>
       <c r="Q38" s="4"/>
       <c r="R38" s="4"/>
       <c r="S38" s="4"/>
       <c r="T38" s="4"/>
-      <c r="U38" s="4"/>
+      <c r="U38" s="3"/>
       <c r="V38" s="3"/>
       <c r="W38" s="3"/>
       <c r="X38" s="3"/>
@@ -3411,46 +3277,43 @@
       <c r="AG38" s="3"/>
       <c r="AH38" s="3"/>
       <c r="AI38" s="3"/>
-      <c r="AJ38" s="3"/>
-    </row>
-    <row r="39" spans="1:36">
+    </row>
+    <row r="39" spans="1:35">
       <c r="A39" s="3"/>
       <c r="B39" s="4" t="s">
-        <v>99</v>
+        <v>93</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>100</v>
+        <v>94</v>
       </c>
       <c r="D39" s="4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E39" s="4" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="F39" s="4"/>
       <c r="G39" s="4"/>
       <c r="H39" s="4" t="s">
-        <v>101</v>
+        <v>95</v>
       </c>
       <c r="I39" s="4"/>
       <c r="J39" s="4"/>
       <c r="K39" s="4"/>
       <c r="L39" s="4"/>
       <c r="M39" s="4" t="s">
-        <v>102</v>
+        <v>96</v>
       </c>
       <c r="N39" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O39" s="4" t="s">
-        <v>82</v>
-      </c>
+      <c r="O39" s="4"/>
       <c r="P39" s="4"/>
       <c r="Q39" s="4"/>
       <c r="R39" s="4"/>
       <c r="S39" s="4"/>
       <c r="T39" s="4"/>
-      <c r="U39" s="4"/>
+      <c r="U39" s="3"/>
       <c r="V39" s="3"/>
       <c r="W39" s="3"/>
       <c r="X39" s="3"/>
@@ -3465,46 +3328,43 @@
       <c r="AG39" s="3"/>
       <c r="AH39" s="3"/>
       <c r="AI39" s="3"/>
-      <c r="AJ39" s="3"/>
-    </row>
-    <row r="40" spans="1:36">
+    </row>
+    <row r="40" spans="1:35">
       <c r="A40" s="3"/>
       <c r="B40" s="4" t="s">
-        <v>103</v>
+        <v>97</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>100</v>
+        <v>94</v>
       </c>
       <c r="D40" s="4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E40" s="4" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="F40" s="4"/>
       <c r="G40" s="4"/>
       <c r="H40" s="4" t="s">
-        <v>101</v>
+        <v>95</v>
       </c>
       <c r="I40" s="4"/>
       <c r="J40" s="4"/>
       <c r="K40" s="4"/>
       <c r="L40" s="4"/>
       <c r="M40" s="4" t="s">
-        <v>104</v>
+        <v>98</v>
       </c>
       <c r="N40" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O40" s="4" t="s">
-        <v>82</v>
-      </c>
+      <c r="O40" s="4"/>
       <c r="P40" s="4"/>
       <c r="Q40" s="4"/>
       <c r="R40" s="4"/>
       <c r="S40" s="4"/>
       <c r="T40" s="4"/>
-      <c r="U40" s="4"/>
+      <c r="U40" s="3"/>
       <c r="V40" s="3"/>
       <c r="W40" s="3"/>
       <c r="X40" s="3"/>
@@ -3519,42 +3379,39 @@
       <c r="AG40" s="3"/>
       <c r="AH40" s="3"/>
       <c r="AI40" s="3"/>
-      <c r="AJ40" s="3"/>
-    </row>
-    <row r="41" spans="1:36">
+    </row>
+    <row r="41" spans="1:35">
       <c r="A41" s="3"/>
       <c r="B41" s="4" t="s">
-        <v>105</v>
+        <v>99</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>106</v>
+        <v>100</v>
       </c>
       <c r="D41" s="4"/>
       <c r="E41" s="4"/>
       <c r="F41" s="4"/>
       <c r="G41" s="4"/>
       <c r="H41" s="4" t="s">
-        <v>101</v>
+        <v>95</v>
       </c>
       <c r="I41" s="4"/>
       <c r="J41" s="4"/>
       <c r="K41" s="4"/>
       <c r="L41" s="4"/>
       <c r="M41" s="4" t="s">
-        <v>107</v>
+        <v>101</v>
       </c>
       <c r="N41" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O41" s="4" t="s">
-        <v>108</v>
-      </c>
+      <c r="O41" s="4"/>
       <c r="P41" s="4"/>
       <c r="Q41" s="4"/>
       <c r="R41" s="4"/>
       <c r="S41" s="4"/>
       <c r="T41" s="4"/>
-      <c r="U41" s="4"/>
+      <c r="U41" s="3"/>
       <c r="V41" s="3"/>
       <c r="W41" s="3"/>
       <c r="X41" s="3"/>
@@ -3569,42 +3426,39 @@
       <c r="AG41" s="3"/>
       <c r="AH41" s="3"/>
       <c r="AI41" s="3"/>
-      <c r="AJ41" s="3"/>
-    </row>
-    <row r="42" spans="1:36">
+    </row>
+    <row r="42" spans="1:35">
       <c r="A42" s="3"/>
       <c r="B42" s="4" t="s">
-        <v>109</v>
+        <v>102</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>106</v>
+        <v>100</v>
       </c>
       <c r="D42" s="4"/>
       <c r="E42" s="4"/>
       <c r="F42" s="4"/>
       <c r="G42" s="4"/>
       <c r="H42" s="4" t="s">
-        <v>101</v>
+        <v>95</v>
       </c>
       <c r="I42" s="4"/>
       <c r="J42" s="4"/>
       <c r="K42" s="4"/>
       <c r="L42" s="4"/>
       <c r="M42" s="4" t="s">
-        <v>107</v>
+        <v>101</v>
       </c>
       <c r="N42" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O42" s="4" t="s">
-        <v>108</v>
-      </c>
+      <c r="O42" s="4"/>
       <c r="P42" s="4"/>
       <c r="Q42" s="4"/>
       <c r="R42" s="4"/>
       <c r="S42" s="4"/>
       <c r="T42" s="4"/>
-      <c r="U42" s="4"/>
+      <c r="U42" s="3"/>
       <c r="V42" s="3"/>
       <c r="W42" s="3"/>
       <c r="X42" s="3"/>
@@ -3619,11 +3473,10 @@
       <c r="AG42" s="3"/>
       <c r="AH42" s="3"/>
       <c r="AI42" s="3"/>
-      <c r="AJ42" s="3"/>
-    </row>
-    <row r="43" spans="2:36">
+    </row>
+    <row r="43" spans="2:35">
       <c r="B43" s="2" t="s">
-        <v>110</v>
+        <v>103</v>
       </c>
       <c r="C43" s="2"/>
       <c r="D43" s="2"/>
@@ -3639,15 +3492,13 @@
       <c r="N43" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="O43" s="2" t="s">
-        <v>27</v>
-      </c>
+      <c r="O43" s="2"/>
       <c r="P43" s="2"/>
       <c r="Q43" s="2"/>
       <c r="R43" s="2"/>
       <c r="S43" s="2"/>
       <c r="T43" s="2"/>
-      <c r="U43" s="2"/>
+      <c r="Y43" s="3"/>
       <c r="Z43" s="3"/>
       <c r="AA43" s="3"/>
       <c r="AB43" s="3"/>
@@ -3658,57 +3509,54 @@
       <c r="AG43" s="3"/>
       <c r="AH43" s="3"/>
       <c r="AI43" s="3"/>
-      <c r="AJ43" s="3"/>
-    </row>
-    <row r="44" spans="2:36">
+    </row>
+    <row r="44" spans="2:35">
       <c r="B44" s="2" t="s">
-        <v>111</v>
+        <v>104</v>
       </c>
       <c r="C44" s="2" t="s">
-        <v>100</v>
+        <v>94</v>
       </c>
       <c r="D44" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E44" s="2" t="s">
         <v>15</v>
       </c>
       <c r="F44" s="2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G44" s="2" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="H44" s="4" t="s">
-        <v>112</v>
+        <v>105</v>
       </c>
       <c r="I44" s="4" t="s">
-        <v>113</v>
+        <v>106</v>
       </c>
       <c r="J44" s="4" t="s">
-        <v>114</v>
+        <v>107</v>
       </c>
       <c r="K44" s="2" t="s">
-        <v>115</v>
+        <v>108</v>
       </c>
       <c r="L44" s="2" t="s">
-        <v>116</v>
+        <v>109</v>
       </c>
       <c r="M44" s="2" t="s">
-        <v>117</v>
+        <v>110</v>
       </c>
       <c r="N44" s="2" t="s">
-        <v>118</v>
-      </c>
-      <c r="O44" s="2" t="s">
-        <v>82</v>
-      </c>
+        <v>111</v>
+      </c>
+      <c r="O44" s="2"/>
       <c r="P44" s="2"/>
       <c r="Q44" s="2"/>
       <c r="R44" s="2"/>
       <c r="S44" s="2"/>
       <c r="T44" s="2"/>
-      <c r="U44" s="2"/>
+      <c r="Y44" s="3"/>
       <c r="Z44" s="3"/>
       <c r="AA44" s="3"/>
       <c r="AB44" s="3"/>
@@ -3719,9 +3567,8 @@
       <c r="AG44" s="3"/>
       <c r="AH44" s="3"/>
       <c r="AI44" s="3"/>
-      <c r="AJ44" s="3"/>
-    </row>
-    <row r="45" spans="1:36">
+    </row>
+    <row r="45" spans="1:35">
       <c r="A45" s="3"/>
       <c r="B45" s="4"/>
       <c r="C45" s="4"/>
@@ -3742,7 +3589,7 @@
       <c r="R45" s="4"/>
       <c r="S45" s="4"/>
       <c r="T45" s="4"/>
-      <c r="U45" s="4"/>
+      <c r="U45" s="3"/>
       <c r="V45" s="3"/>
       <c r="W45" s="3"/>
       <c r="X45" s="3"/>
@@ -3757,9 +3604,8 @@
       <c r="AG45" s="3"/>
       <c r="AH45" s="3"/>
       <c r="AI45" s="3"/>
-      <c r="AJ45" s="3"/>
-    </row>
-    <row r="46" s="1" customFormat="1" spans="1:36">
+    </row>
+    <row r="46" s="1" customFormat="1" spans="1:35">
       <c r="A46" s="3"/>
       <c r="B46" s="4"/>
       <c r="C46" s="4"/>
@@ -3780,7 +3626,7 @@
       <c r="R46" s="4"/>
       <c r="S46" s="4"/>
       <c r="T46" s="4"/>
-      <c r="U46" s="4"/>
+      <c r="U46" s="3"/>
       <c r="V46" s="3"/>
       <c r="W46" s="3"/>
       <c r="X46" s="3"/>
@@ -3795,9 +3641,8 @@
       <c r="AG46" s="3"/>
       <c r="AH46" s="3"/>
       <c r="AI46" s="3"/>
-      <c r="AJ46" s="3"/>
-    </row>
-    <row r="47" s="1" customFormat="1" spans="1:36">
+    </row>
+    <row r="47" s="1" customFormat="1" spans="1:35">
       <c r="A47" s="3"/>
       <c r="B47" s="4"/>
       <c r="C47" s="4"/>
@@ -3818,7 +3663,7 @@
       <c r="R47" s="4"/>
       <c r="S47" s="4"/>
       <c r="T47" s="4"/>
-      <c r="U47" s="4"/>
+      <c r="U47" s="3"/>
       <c r="V47" s="3"/>
       <c r="W47" s="3"/>
       <c r="X47" s="3"/>
@@ -3833,9 +3678,8 @@
       <c r="AG47" s="3"/>
       <c r="AH47" s="3"/>
       <c r="AI47" s="3"/>
-      <c r="AJ47" s="3"/>
-    </row>
-    <row r="48" spans="1:36">
+    </row>
+    <row r="48" spans="1:35">
       <c r="A48" s="3"/>
       <c r="B48" s="4"/>
       <c r="C48" s="4"/>
@@ -3856,7 +3700,7 @@
       <c r="R48" s="4"/>
       <c r="S48" s="4"/>
       <c r="T48" s="4"/>
-      <c r="U48" s="4"/>
+      <c r="U48" s="3"/>
       <c r="V48" s="3"/>
       <c r="W48" s="3"/>
       <c r="X48" s="3"/>
@@ -3871,9 +3715,8 @@
       <c r="AG48" s="3"/>
       <c r="AH48" s="3"/>
       <c r="AI48" s="3"/>
-      <c r="AJ48" s="3"/>
-    </row>
-    <row r="49" spans="1:36">
+    </row>
+    <row r="49" spans="1:35">
       <c r="A49" s="3"/>
       <c r="B49" s="4"/>
       <c r="C49" s="4"/>
@@ -3894,7 +3737,7 @@
       <c r="R49" s="4"/>
       <c r="S49" s="4"/>
       <c r="T49" s="4"/>
-      <c r="U49" s="4"/>
+      <c r="U49" s="3"/>
       <c r="V49" s="3"/>
       <c r="W49" s="3"/>
       <c r="X49" s="3"/>
@@ -3909,9 +3752,8 @@
       <c r="AG49" s="3"/>
       <c r="AH49" s="3"/>
       <c r="AI49" s="3"/>
-      <c r="AJ49" s="3"/>
-    </row>
-    <row r="50" spans="1:36">
+    </row>
+    <row r="50" spans="1:35">
       <c r="A50" s="3"/>
       <c r="B50" s="4"/>
       <c r="C50" s="4"/>
@@ -3932,7 +3774,7 @@
       <c r="R50" s="4"/>
       <c r="S50" s="4"/>
       <c r="T50" s="4"/>
-      <c r="U50" s="4"/>
+      <c r="U50" s="3"/>
       <c r="V50" s="3"/>
       <c r="W50" s="3"/>
       <c r="X50" s="3"/>
@@ -3947,9 +3789,8 @@
       <c r="AG50" s="3"/>
       <c r="AH50" s="3"/>
       <c r="AI50" s="3"/>
-      <c r="AJ50" s="3"/>
-    </row>
-    <row r="51" spans="1:36">
+    </row>
+    <row r="51" spans="1:35">
       <c r="A51" s="3"/>
       <c r="B51" s="4"/>
       <c r="C51" s="4"/>
@@ -3970,7 +3811,7 @@
       <c r="R51" s="4"/>
       <c r="S51" s="4"/>
       <c r="T51" s="4"/>
-      <c r="U51" s="4"/>
+      <c r="U51" s="3"/>
       <c r="V51" s="3"/>
       <c r="W51" s="3"/>
       <c r="X51" s="3"/>
@@ -3985,9 +3826,8 @@
       <c r="AG51" s="3"/>
       <c r="AH51" s="3"/>
       <c r="AI51" s="3"/>
-      <c r="AJ51" s="3"/>
-    </row>
-    <row r="52" spans="1:36">
+    </row>
+    <row r="52" spans="1:35">
       <c r="A52" s="3"/>
       <c r="B52" s="4"/>
       <c r="C52" s="4"/>
@@ -4008,7 +3848,7 @@
       <c r="R52" s="4"/>
       <c r="S52" s="4"/>
       <c r="T52" s="4"/>
-      <c r="U52" s="4"/>
+      <c r="U52" s="3"/>
       <c r="V52" s="3"/>
       <c r="W52" s="3"/>
       <c r="X52" s="3"/>
@@ -4023,9 +3863,8 @@
       <c r="AG52" s="3"/>
       <c r="AH52" s="3"/>
       <c r="AI52" s="3"/>
-      <c r="AJ52" s="3"/>
-    </row>
-    <row r="53" spans="1:36">
+    </row>
+    <row r="53" spans="1:35">
       <c r="A53" s="3"/>
       <c r="B53" s="4"/>
       <c r="C53" s="4"/>
@@ -4046,7 +3885,7 @@
       <c r="R53" s="4"/>
       <c r="S53" s="4"/>
       <c r="T53" s="4"/>
-      <c r="U53" s="4"/>
+      <c r="U53" s="3"/>
       <c r="V53" s="3"/>
       <c r="W53" s="3"/>
       <c r="X53" s="3"/>
@@ -4061,9 +3900,8 @@
       <c r="AG53" s="3"/>
       <c r="AH53" s="3"/>
       <c r="AI53" s="3"/>
-      <c r="AJ53" s="3"/>
-    </row>
-    <row r="54" spans="1:36">
+    </row>
+    <row r="54" spans="1:35">
       <c r="A54" s="3"/>
       <c r="B54" s="4"/>
       <c r="C54" s="4"/>
@@ -4084,7 +3922,7 @@
       <c r="R54" s="4"/>
       <c r="S54" s="4"/>
       <c r="T54" s="4"/>
-      <c r="U54" s="4"/>
+      <c r="U54" s="3"/>
       <c r="V54" s="3"/>
       <c r="W54" s="3"/>
       <c r="X54" s="3"/>
@@ -4099,9 +3937,8 @@
       <c r="AG54" s="3"/>
       <c r="AH54" s="3"/>
       <c r="AI54" s="3"/>
-      <c r="AJ54" s="3"/>
-    </row>
-    <row r="55" spans="1:36">
+    </row>
+    <row r="55" spans="1:35">
       <c r="A55" s="3"/>
       <c r="B55" s="4"/>
       <c r="C55" s="4"/>
@@ -4122,7 +3959,7 @@
       <c r="R55" s="4"/>
       <c r="S55" s="4"/>
       <c r="T55" s="4"/>
-      <c r="U55" s="4"/>
+      <c r="U55" s="3"/>
       <c r="V55" s="3"/>
       <c r="W55" s="3"/>
       <c r="X55" s="3"/>
@@ -4137,9 +3974,8 @@
       <c r="AG55" s="3"/>
       <c r="AH55" s="3"/>
       <c r="AI55" s="3"/>
-      <c r="AJ55" s="3"/>
-    </row>
-    <row r="56" spans="1:36">
+    </row>
+    <row r="56" spans="1:35">
       <c r="A56" s="3"/>
       <c r="B56" s="4"/>
       <c r="C56" s="4"/>
@@ -4160,7 +3996,7 @@
       <c r="R56" s="4"/>
       <c r="S56" s="4"/>
       <c r="T56" s="4"/>
-      <c r="U56" s="4"/>
+      <c r="U56" s="3"/>
       <c r="V56" s="3"/>
       <c r="W56" s="3"/>
       <c r="X56" s="3"/>
@@ -4175,9 +4011,8 @@
       <c r="AG56" s="3"/>
       <c r="AH56" s="3"/>
       <c r="AI56" s="3"/>
-      <c r="AJ56" s="3"/>
-    </row>
-    <row r="57" spans="1:36">
+    </row>
+    <row r="57" spans="1:35">
       <c r="A57" s="3"/>
       <c r="B57" s="4"/>
       <c r="C57" s="4"/>
@@ -4198,7 +4033,7 @@
       <c r="R57" s="4"/>
       <c r="S57" s="4"/>
       <c r="T57" s="4"/>
-      <c r="U57" s="4"/>
+      <c r="U57" s="3"/>
       <c r="V57" s="3"/>
       <c r="W57" s="3"/>
       <c r="X57" s="3"/>
@@ -4213,9 +4048,8 @@
       <c r="AG57" s="3"/>
       <c r="AH57" s="3"/>
       <c r="AI57" s="3"/>
-      <c r="AJ57" s="3"/>
-    </row>
-    <row r="58" spans="1:36">
+    </row>
+    <row r="58" spans="1:35">
       <c r="A58" s="3"/>
       <c r="B58" s="4"/>
       <c r="C58" s="4"/>
@@ -4236,7 +4070,7 @@
       <c r="R58" s="4"/>
       <c r="S58" s="4"/>
       <c r="T58" s="4"/>
-      <c r="U58" s="4"/>
+      <c r="U58" s="3"/>
       <c r="V58" s="3"/>
       <c r="W58" s="3"/>
       <c r="X58" s="3"/>
@@ -4251,9 +4085,8 @@
       <c r="AG58" s="3"/>
       <c r="AH58" s="3"/>
       <c r="AI58" s="3"/>
-      <c r="AJ58" s="3"/>
-    </row>
-    <row r="59" spans="1:36">
+    </row>
+    <row r="59" spans="1:35">
       <c r="A59" s="3"/>
       <c r="B59" s="4"/>
       <c r="C59" s="4"/>
@@ -4274,7 +4107,7 @@
       <c r="R59" s="4"/>
       <c r="S59" s="4"/>
       <c r="T59" s="4"/>
-      <c r="U59" s="4"/>
+      <c r="U59" s="3"/>
       <c r="V59" s="3"/>
       <c r="W59" s="3"/>
       <c r="X59" s="3"/>
@@ -4289,9 +4122,8 @@
       <c r="AG59" s="3"/>
       <c r="AH59" s="3"/>
       <c r="AI59" s="3"/>
-      <c r="AJ59" s="3"/>
-    </row>
-    <row r="60" spans="1:36">
+    </row>
+    <row r="60" spans="1:35">
       <c r="A60" s="3"/>
       <c r="B60" s="4"/>
       <c r="C60" s="4"/>
@@ -4312,7 +4144,7 @@
       <c r="R60" s="4"/>
       <c r="S60" s="4"/>
       <c r="T60" s="4"/>
-      <c r="U60" s="4"/>
+      <c r="U60" s="3"/>
       <c r="V60" s="3"/>
       <c r="W60" s="3"/>
       <c r="X60" s="3"/>
@@ -4327,9 +4159,8 @@
       <c r="AG60" s="3"/>
       <c r="AH60" s="3"/>
       <c r="AI60" s="3"/>
-      <c r="AJ60" s="3"/>
-    </row>
-    <row r="61" spans="1:36">
+    </row>
+    <row r="61" spans="1:35">
       <c r="A61" s="3"/>
       <c r="B61" s="4"/>
       <c r="C61" s="4"/>
@@ -4350,7 +4181,7 @@
       <c r="R61" s="4"/>
       <c r="S61" s="4"/>
       <c r="T61" s="4"/>
-      <c r="U61" s="4"/>
+      <c r="U61" s="3"/>
       <c r="V61" s="3"/>
       <c r="W61" s="3"/>
       <c r="X61" s="3"/>
@@ -4365,9 +4196,8 @@
       <c r="AG61" s="3"/>
       <c r="AH61" s="3"/>
       <c r="AI61" s="3"/>
-      <c r="AJ61" s="3"/>
-    </row>
-    <row r="62" spans="1:36">
+    </row>
+    <row r="62" spans="1:35">
       <c r="A62" s="3"/>
       <c r="B62" s="4"/>
       <c r="C62" s="4"/>
@@ -4388,7 +4218,7 @@
       <c r="R62" s="4"/>
       <c r="S62" s="4"/>
       <c r="T62" s="4"/>
-      <c r="U62" s="4"/>
+      <c r="U62" s="3"/>
       <c r="V62" s="3"/>
       <c r="W62" s="3"/>
       <c r="X62" s="3"/>
@@ -4403,9 +4233,8 @@
       <c r="AG62" s="3"/>
       <c r="AH62" s="3"/>
       <c r="AI62" s="3"/>
-      <c r="AJ62" s="3"/>
-    </row>
-    <row r="63" spans="1:36">
+    </row>
+    <row r="63" spans="1:35">
       <c r="A63" s="3"/>
       <c r="B63" s="4"/>
       <c r="C63" s="4"/>
@@ -4426,7 +4255,7 @@
       <c r="R63" s="4"/>
       <c r="S63" s="4"/>
       <c r="T63" s="4"/>
-      <c r="U63" s="4"/>
+      <c r="U63" s="3"/>
       <c r="V63" s="3"/>
       <c r="W63" s="3"/>
       <c r="X63" s="3"/>
@@ -4441,9 +4270,8 @@
       <c r="AG63" s="3"/>
       <c r="AH63" s="3"/>
       <c r="AI63" s="3"/>
-      <c r="AJ63" s="3"/>
-    </row>
-    <row r="64" spans="1:36">
+    </row>
+    <row r="64" spans="1:35">
       <c r="A64" s="3"/>
       <c r="B64" s="4"/>
       <c r="C64" s="4"/>
@@ -4464,7 +4292,7 @@
       <c r="R64" s="4"/>
       <c r="S64" s="4"/>
       <c r="T64" s="4"/>
-      <c r="U64" s="4"/>
+      <c r="U64" s="3"/>
       <c r="V64" s="3"/>
       <c r="W64" s="3"/>
       <c r="X64" s="3"/>
@@ -4479,9 +4307,8 @@
       <c r="AG64" s="3"/>
       <c r="AH64" s="3"/>
       <c r="AI64" s="3"/>
-      <c r="AJ64" s="3"/>
-    </row>
-    <row r="65" spans="1:36">
+    </row>
+    <row r="65" spans="1:35">
       <c r="A65" s="3"/>
       <c r="B65" s="4"/>
       <c r="C65" s="4"/>
@@ -4502,7 +4329,7 @@
       <c r="R65" s="4"/>
       <c r="S65" s="4"/>
       <c r="T65" s="4"/>
-      <c r="U65" s="4"/>
+      <c r="U65" s="3"/>
       <c r="V65" s="3"/>
       <c r="W65" s="3"/>
       <c r="X65" s="3"/>
@@ -4517,9 +4344,8 @@
       <c r="AG65" s="3"/>
       <c r="AH65" s="3"/>
       <c r="AI65" s="3"/>
-      <c r="AJ65" s="3"/>
-    </row>
-    <row r="66" spans="1:36">
+    </row>
+    <row r="66" spans="1:35">
       <c r="A66" s="3"/>
       <c r="B66" s="4"/>
       <c r="C66" s="4"/>
@@ -4540,7 +4366,7 @@
       <c r="R66" s="4"/>
       <c r="S66" s="4"/>
       <c r="T66" s="4"/>
-      <c r="U66" s="4"/>
+      <c r="U66" s="3"/>
       <c r="V66" s="3"/>
       <c r="W66" s="3"/>
       <c r="X66" s="3"/>
@@ -4555,9 +4381,8 @@
       <c r="AG66" s="3"/>
       <c r="AH66" s="3"/>
       <c r="AI66" s="3"/>
-      <c r="AJ66" s="3"/>
-    </row>
-    <row r="67" spans="1:36">
+    </row>
+    <row r="67" spans="1:35">
       <c r="A67" s="3"/>
       <c r="B67" s="4"/>
       <c r="C67" s="4"/>
@@ -4578,7 +4403,7 @@
       <c r="R67" s="4"/>
       <c r="S67" s="4"/>
       <c r="T67" s="4"/>
-      <c r="U67" s="4"/>
+      <c r="U67" s="3"/>
       <c r="V67" s="3"/>
       <c r="W67" s="3"/>
       <c r="X67" s="3"/>
@@ -4593,9 +4418,8 @@
       <c r="AG67" s="3"/>
       <c r="AH67" s="3"/>
       <c r="AI67" s="3"/>
-      <c r="AJ67" s="3"/>
-    </row>
-    <row r="68" spans="1:36">
+    </row>
+    <row r="68" spans="1:35">
       <c r="A68" s="3"/>
       <c r="B68" s="4"/>
       <c r="C68" s="4"/>
@@ -4616,7 +4440,7 @@
       <c r="R68" s="4"/>
       <c r="S68" s="4"/>
       <c r="T68" s="4"/>
-      <c r="U68" s="4"/>
+      <c r="U68" s="3"/>
       <c r="V68" s="3"/>
       <c r="W68" s="3"/>
       <c r="X68" s="3"/>
@@ -4631,9 +4455,8 @@
       <c r="AG68" s="3"/>
       <c r="AH68" s="3"/>
       <c r="AI68" s="3"/>
-      <c r="AJ68" s="3"/>
-    </row>
-    <row r="69" spans="1:36">
+    </row>
+    <row r="69" spans="1:35">
       <c r="A69" s="3"/>
       <c r="B69" s="4"/>
       <c r="C69" s="4"/>
@@ -4654,7 +4477,7 @@
       <c r="R69" s="4"/>
       <c r="S69" s="4"/>
       <c r="T69" s="4"/>
-      <c r="U69" s="4"/>
+      <c r="U69" s="3"/>
       <c r="V69" s="3"/>
       <c r="W69" s="3"/>
       <c r="X69" s="3"/>
@@ -4669,9 +4492,8 @@
       <c r="AG69" s="3"/>
       <c r="AH69" s="3"/>
       <c r="AI69" s="3"/>
-      <c r="AJ69" s="3"/>
-    </row>
-    <row r="70" spans="1:36">
+    </row>
+    <row r="70" spans="1:35">
       <c r="A70" s="3"/>
       <c r="B70" s="4"/>
       <c r="C70" s="4"/>
@@ -4692,7 +4514,7 @@
       <c r="R70" s="4"/>
       <c r="S70" s="4"/>
       <c r="T70" s="4"/>
-      <c r="U70" s="4"/>
+      <c r="U70" s="3"/>
       <c r="V70" s="3"/>
       <c r="W70" s="3"/>
       <c r="X70" s="3"/>
@@ -4707,9 +4529,8 @@
       <c r="AG70" s="3"/>
       <c r="AH70" s="3"/>
       <c r="AI70" s="3"/>
-      <c r="AJ70" s="3"/>
-    </row>
-    <row r="71" spans="1:36">
+    </row>
+    <row r="71" spans="1:35">
       <c r="A71" s="3"/>
       <c r="B71" s="4"/>
       <c r="C71" s="4"/>
@@ -4730,7 +4551,7 @@
       <c r="R71" s="4"/>
       <c r="S71" s="4"/>
       <c r="T71" s="4"/>
-      <c r="U71" s="4"/>
+      <c r="U71" s="3"/>
       <c r="V71" s="3"/>
       <c r="W71" s="3"/>
       <c r="X71" s="3"/>
@@ -4745,9 +4566,8 @@
       <c r="AG71" s="3"/>
       <c r="AH71" s="3"/>
       <c r="AI71" s="3"/>
-      <c r="AJ71" s="3"/>
-    </row>
-    <row r="72" spans="1:36">
+    </row>
+    <row r="72" spans="1:35">
       <c r="A72" s="3"/>
       <c r="B72" s="4"/>
       <c r="C72" s="4"/>
@@ -4768,7 +4588,7 @@
       <c r="R72" s="4"/>
       <c r="S72" s="4"/>
       <c r="T72" s="4"/>
-      <c r="U72" s="4"/>
+      <c r="U72" s="3"/>
       <c r="V72" s="3"/>
       <c r="W72" s="3"/>
       <c r="X72" s="3"/>
@@ -4783,9 +4603,8 @@
       <c r="AG72" s="3"/>
       <c r="AH72" s="3"/>
       <c r="AI72" s="3"/>
-      <c r="AJ72" s="3"/>
-    </row>
-    <row r="73" spans="1:36">
+    </row>
+    <row r="73" spans="1:35">
       <c r="A73" s="3"/>
       <c r="B73" s="4"/>
       <c r="C73" s="4"/>
@@ -4806,7 +4625,7 @@
       <c r="R73" s="4"/>
       <c r="S73" s="4"/>
       <c r="T73" s="4"/>
-      <c r="U73" s="4"/>
+      <c r="U73" s="3"/>
       <c r="V73" s="3"/>
       <c r="W73" s="3"/>
       <c r="X73" s="3"/>
@@ -4821,9 +4640,8 @@
       <c r="AG73" s="3"/>
       <c r="AH73" s="3"/>
       <c r="AI73" s="3"/>
-      <c r="AJ73" s="3"/>
-    </row>
-    <row r="74" spans="1:36">
+    </row>
+    <row r="74" spans="1:35">
       <c r="A74" s="3"/>
       <c r="B74" s="4"/>
       <c r="C74" s="4"/>
@@ -4844,7 +4662,7 @@
       <c r="R74" s="4"/>
       <c r="S74" s="4"/>
       <c r="T74" s="4"/>
-      <c r="U74" s="4"/>
+      <c r="U74" s="3"/>
       <c r="V74" s="3"/>
       <c r="W74" s="3"/>
       <c r="X74" s="3"/>
@@ -4859,9 +4677,8 @@
       <c r="AG74" s="3"/>
       <c r="AH74" s="3"/>
       <c r="AI74" s="3"/>
-      <c r="AJ74" s="3"/>
-    </row>
-    <row r="75" spans="1:36">
+    </row>
+    <row r="75" spans="1:35">
       <c r="A75" s="3"/>
       <c r="B75" s="4"/>
       <c r="C75" s="4"/>
@@ -4882,7 +4699,7 @@
       <c r="R75" s="4"/>
       <c r="S75" s="4"/>
       <c r="T75" s="4"/>
-      <c r="U75" s="4"/>
+      <c r="U75" s="3"/>
       <c r="V75" s="3"/>
       <c r="W75" s="3"/>
       <c r="X75" s="3"/>
@@ -4897,9 +4714,8 @@
       <c r="AG75" s="3"/>
       <c r="AH75" s="3"/>
       <c r="AI75" s="3"/>
-      <c r="AJ75" s="3"/>
-    </row>
-    <row r="76" spans="1:36">
+    </row>
+    <row r="76" spans="1:35">
       <c r="A76" s="3"/>
       <c r="B76" s="4"/>
       <c r="C76" s="4"/>
@@ -4920,7 +4736,7 @@
       <c r="R76" s="4"/>
       <c r="S76" s="4"/>
       <c r="T76" s="4"/>
-      <c r="U76" s="4"/>
+      <c r="U76" s="3"/>
       <c r="V76" s="3"/>
       <c r="W76" s="3"/>
       <c r="X76" s="3"/>
@@ -4935,9 +4751,8 @@
       <c r="AG76" s="3"/>
       <c r="AH76" s="3"/>
       <c r="AI76" s="3"/>
-      <c r="AJ76" s="3"/>
-    </row>
-    <row r="77" spans="1:36">
+    </row>
+    <row r="77" spans="1:35">
       <c r="A77" s="3"/>
       <c r="B77" s="4"/>
       <c r="C77" s="4"/>
@@ -4958,7 +4773,7 @@
       <c r="R77" s="4"/>
       <c r="S77" s="4"/>
       <c r="T77" s="4"/>
-      <c r="U77" s="4"/>
+      <c r="U77" s="3"/>
       <c r="V77" s="3"/>
       <c r="W77" s="3"/>
       <c r="X77" s="3"/>
@@ -4973,9 +4788,8 @@
       <c r="AG77" s="3"/>
       <c r="AH77" s="3"/>
       <c r="AI77" s="3"/>
-      <c r="AJ77" s="3"/>
-    </row>
-    <row r="78" spans="1:36">
+    </row>
+    <row r="78" spans="1:35">
       <c r="A78" s="3"/>
       <c r="B78" s="4"/>
       <c r="C78" s="4"/>
@@ -4996,7 +4810,7 @@
       <c r="R78" s="4"/>
       <c r="S78" s="4"/>
       <c r="T78" s="4"/>
-      <c r="U78" s="4"/>
+      <c r="U78" s="3"/>
       <c r="V78" s="3"/>
       <c r="W78" s="3"/>
       <c r="X78" s="3"/>
@@ -5011,195 +4825,194 @@
       <c r="AG78" s="3"/>
       <c r="AH78" s="3"/>
       <c r="AI78" s="3"/>
-      <c r="AJ78" s="3"/>
-    </row>
-    <row r="86" spans="1:25">
+    </row>
+    <row r="86" spans="1:24">
       <c r="A86" s="2"/>
       <c r="B86" s="2"/>
       <c r="C86" s="2"/>
       <c r="D86" s="2"/>
-      <c r="T86" s="2"/>
+      <c r="S86" s="2"/>
+      <c r="U86" s="2"/>
       <c r="V86" s="2"/>
       <c r="W86" s="2"/>
       <c r="X86" s="2"/>
-      <c r="Y86" s="2"/>
-    </row>
-    <row r="87" spans="1:25">
+    </row>
+    <row r="87" spans="1:24">
       <c r="A87" s="2"/>
       <c r="B87" s="2"/>
       <c r="C87" s="2"/>
       <c r="D87" s="2"/>
       <c r="E87" s="2"/>
+      <c r="S87" s="2"/>
       <c r="T87" s="2"/>
       <c r="U87" s="2"/>
       <c r="V87" s="2"/>
       <c r="W87" s="2"/>
       <c r="X87" s="2"/>
-      <c r="Y87" s="2"/>
-    </row>
-    <row r="88" spans="1:25">
+    </row>
+    <row r="88" spans="1:24">
       <c r="A88" s="2"/>
       <c r="B88" s="2"/>
       <c r="C88" s="2"/>
       <c r="D88" s="2"/>
+      <c r="S88" s="2"/>
       <c r="T88" s="2"/>
       <c r="U88" s="2"/>
       <c r="V88" s="2"/>
       <c r="W88" s="2"/>
       <c r="X88" s="2"/>
-      <c r="Y88" s="2"/>
-    </row>
-    <row r="89" spans="1:25">
+    </row>
+    <row r="89" spans="1:24">
       <c r="A89" s="2"/>
       <c r="B89" s="2"/>
       <c r="C89" s="2"/>
       <c r="D89" s="2"/>
+      <c r="S89" s="2"/>
       <c r="T89" s="2"/>
       <c r="U89" s="2"/>
       <c r="V89" s="2"/>
       <c r="W89" s="2"/>
       <c r="X89" s="2"/>
-      <c r="Y89" s="2"/>
-    </row>
-    <row r="90" spans="1:25">
+    </row>
+    <row r="90" spans="1:24">
       <c r="A90" s="2"/>
       <c r="B90" s="2"/>
       <c r="C90" s="2"/>
       <c r="D90" s="2"/>
+      <c r="S90" s="2"/>
       <c r="T90" s="2"/>
       <c r="U90" s="2"/>
       <c r="V90" s="2"/>
       <c r="W90" s="2"/>
       <c r="X90" s="2"/>
-      <c r="Y90" s="2"/>
-    </row>
-    <row r="91" spans="1:25">
+    </row>
+    <row r="91" spans="1:24">
       <c r="A91" s="2"/>
       <c r="B91" s="2"/>
       <c r="C91" s="2"/>
       <c r="D91" s="2"/>
+      <c r="S91" s="2"/>
       <c r="T91" s="2"/>
       <c r="U91" s="2"/>
       <c r="V91" s="2"/>
       <c r="W91" s="2"/>
       <c r="X91" s="2"/>
-      <c r="Y91" s="2"/>
-    </row>
-    <row r="92" spans="1:25">
+    </row>
+    <row r="92" spans="1:24">
       <c r="A92" s="2"/>
       <c r="B92" s="2"/>
       <c r="C92" s="2"/>
       <c r="D92" s="2"/>
+      <c r="S92" s="2"/>
       <c r="T92" s="2"/>
       <c r="U92" s="2"/>
       <c r="V92" s="2"/>
       <c r="W92" s="2"/>
       <c r="X92" s="2"/>
-      <c r="Y92" s="2"/>
-    </row>
-    <row r="93" spans="1:25">
+    </row>
+    <row r="93" spans="1:24">
       <c r="A93" s="2"/>
       <c r="B93" s="2"/>
       <c r="C93" s="2"/>
       <c r="D93" s="2"/>
+      <c r="S93" s="2"/>
       <c r="T93" s="2"/>
       <c r="U93" s="2"/>
       <c r="V93" s="2"/>
       <c r="W93" s="2"/>
       <c r="X93" s="2"/>
-      <c r="Y93" s="2"/>
-    </row>
-    <row r="94" spans="1:25">
+    </row>
+    <row r="94" spans="1:24">
       <c r="A94" s="2"/>
       <c r="B94" s="2"/>
       <c r="C94" s="2"/>
       <c r="D94" s="2"/>
+      <c r="S94" s="2"/>
       <c r="T94" s="2"/>
       <c r="U94" s="2"/>
       <c r="V94" s="2"/>
       <c r="W94" s="2"/>
       <c r="X94" s="2"/>
-      <c r="Y94" s="2"/>
-    </row>
-    <row r="95" spans="1:25">
+    </row>
+    <row r="95" spans="1:24">
       <c r="A95" s="2"/>
       <c r="B95" s="2"/>
       <c r="C95" s="2"/>
       <c r="D95" s="2"/>
+      <c r="S95" s="2"/>
       <c r="T95" s="2"/>
       <c r="U95" s="2"/>
       <c r="V95" s="2"/>
       <c r="W95" s="2"/>
       <c r="X95" s="2"/>
-      <c r="Y95" s="2"/>
-    </row>
-    <row r="96" spans="1:25">
+    </row>
+    <row r="96" spans="1:24">
       <c r="A96" s="2"/>
       <c r="B96" s="2"/>
       <c r="C96" s="2"/>
       <c r="D96" s="2"/>
+      <c r="S96" s="2"/>
       <c r="T96" s="2"/>
       <c r="U96" s="2"/>
       <c r="V96" s="2"/>
       <c r="W96" s="2"/>
       <c r="X96" s="2"/>
-      <c r="Y96" s="2"/>
-    </row>
-    <row r="97" spans="1:25">
+    </row>
+    <row r="97" spans="1:24">
       <c r="A97" s="2"/>
       <c r="B97" s="2"/>
       <c r="C97" s="2"/>
       <c r="D97" s="2"/>
+      <c r="S97" s="2"/>
       <c r="T97" s="2"/>
       <c r="U97" s="2"/>
       <c r="V97" s="2"/>
       <c r="W97" s="2"/>
       <c r="X97" s="2"/>
-      <c r="Y97" s="2"/>
-    </row>
-    <row r="98" spans="1:25">
+    </row>
+    <row r="98" spans="1:24">
       <c r="A98" s="2"/>
       <c r="B98" s="2"/>
       <c r="C98" s="2"/>
       <c r="D98" s="2"/>
+      <c r="S98" s="2"/>
       <c r="T98" s="2"/>
       <c r="U98" s="2"/>
       <c r="V98" s="2"/>
       <c r="W98" s="2"/>
       <c r="X98" s="2"/>
-      <c r="Y98" s="2"/>
-    </row>
-    <row r="99" spans="1:25">
+    </row>
+    <row r="99" spans="1:24">
       <c r="A99" s="2"/>
       <c r="B99" s="2"/>
       <c r="C99" s="2"/>
       <c r="D99" s="2"/>
+      <c r="S99" s="2"/>
       <c r="T99" s="2"/>
       <c r="U99" s="2"/>
       <c r="V99" s="2"/>
       <c r="W99" s="2"/>
       <c r="X99" s="2"/>
-      <c r="Y99" s="2"/>
     </row>
   </sheetData>
-  <dataValidations count="14">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="O2:O1048576">
-      <formula1>"R_TYPE,I_TYPE,S_TYPE,B_TYPE,U_TYPE,J_TYPE,ICSR_TYPE,FENCE_TYPE,N_TYPE"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="M29 M30 M31 M39 M40 M41 M42 M43 M2:M28 M32:M38 M44:M1048576">
-      <formula1>"CSR_W,CSR_S,CSR_C,CSR_P,CSR_XX"</formula1>
-    </dataValidation>
+  <dataValidations count="13">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H29 H30 H31 H40 H41 H42 H43 H10:H28 H32:H39 H44:H1048576">
       <formula1>"WB_ALU,WB_MEM,WB_PC4,WB_XX,WB_CSR"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F6 F15 F18 F19 F20 F21 F24 F25 F26 F27 F28 F29 F30 F31 F32 F33 F36 F37 F38 F39 F40 F41 F42 F43 F2:F5 F7:F14 F16:F17 F22:F23 F34:F35 F44:F1048576">
+      <formula1>"ALU_ADD,ALU_SUB,ALU_AND,ALU_OR,ALU_XOR,ALU_SLL,ALU_SRL,ALU_SLT,ALU_SLTU,ALU_COPY_A,ALU_COPY_B,ALU_SRA"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L5 L6 L7 L10 L11 L14 L15 L16 L17 L18 L19 L20 L21 L22 L23 L24 L25 L26 L27 L28 L29 L30 L31 L32 L33 L34 L35 L36 L37 L38 L39 L40 L41 L42 L43 L2:L4 L8:L9 L12:L13 L44:L1048576">
+      <formula1>"BR_EQ,BR_NE,BR_LTU,BR_GE,BR_GEU,BR_LT,BR_XX"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C29 C30 C31 C43 C2:C28 C32:C42 C44:C1048576">
       <formula1>"PC_4,PC_0,PC_ALU,PC_CSR"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E4 E5 E6 E7 E8 E9 E10 E11 E12 E13 E14 E15 E16 E17 E18 E19 E20 E21 E22 E23 E24 E25 E26 E27 E28 E29 E30 E31 E32 E33 E34 E35 E36 E37 E38 E39 E40 E41 E42 E43 E2:E3 E44:E1048576">
-      <formula1>"B_IMM,B_RS2"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="N4 N5 N6 N7 N8 N9 N10 N11 N12 N13 N14 N15 N16 N17 N18 N19 N20 N21 N22 N23 N24 N25 N26 N27 N28 N29 N30 N31 N32 N33 N34 N35 N36 N37 N38 N39 N40 N41 N42 N43 N2:N3 N44:N1048576">
+      <formula1>"INST_VALID,INST_INVALID"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G4 G5 G6 G7 G8 G9 G10 G11 G12 G13 G14 G15 G16 G17 G18 G19 G20 G21 G22 G23 G24 G25 G26 G27 G28 G29 G30 G31 G32 G33 G34 G35 G36 G37 G38 G39 G40 G41 G42 G43 G2:G3 G44:G1048576">
-      <formula1>"IMM_I,IMM_J,IMM_U,IMM_S,IMM_B"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D4 D5 D6 D7 D8 D9 D10 D11 D12 D13 D14 D15 D16 D17 D18 D19 D20 D21 D22 D23 D24 D25 D26 D27 D28 D29 D30 D31 D32 D33 D34 D35 D36 D37 D38 D39 D40 D41 D42 D43 D2:D3 D44:D1048576">
+      <formula1>"A_PC,A_RS1"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J5 J6 J7 J8 J9 J10 J11 J12 J13 J14 J15 J16 J17 J18 J19 J20 J21 J22 J23 J24 J25 J26 J27 J28 J29 J30 J31 J32 J33 J34 J35 J36 J37 J38 J39 J40 J41 J42 J43 J2:J4 J44:J1048576">
       <formula1>"ST_SW,ST_SH,ST_SB,ST_XX"</formula1>
@@ -5207,23 +5020,20 @@
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H5 H6 H7 H8 H9 H2:H4">
       <formula1>"WB_ALU,WB_MEM,WB_PC4,WB_XX"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L5 L6 L7 L10 L11 L14 L15 L16 L17 L18 L19 L20 L21 L22 L23 L24 L25 L26 L27 L28 L29 L30 L31 L32 L33 L34 L35 L36 L37 L38 L39 L40 L41 L42 L43 L2:L4 L8:L9 L12:L13 L44:L1048576">
-      <formula1>"BR_EQ,BR_NE,BR_LTU,BR_GE,BR_GEU,BR_LT,BR_XX"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K4 K5 K6 K7 K8 K9 K10 K11 K12 K13 K14 K15 K16 K17 K18 K19 K20 K21 K22 K23 K24 K25 K26 K27 K28 K29 K30 K31 K32 K33 K34 K35 K36 K37 K38 K39 K40 K41 K42 K43 K2:K3 K44:K1048576">
+      <formula1>"MASK_XX,MASK_B,MASK_H,MASK_W,MASK_D"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="N4 N5 N6 N7 N8 N9 N10 N11 N12 N13 N14 N15 N16 N17 N18 N19 N20 N21 N22 N23 N24 N25 N26 N27 N28 N29 N30 N31 N32 N33 N34 N35 N36 N37 N38 N39 N40 N41 N42 N43 N2:N3 N44:N1048576">
-      <formula1>"INST_VALID,INST_INVALID"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E4 E5 E6 E7 E8 E9 E10 E11 E12 E13 E14 E15 E16 E17 E18 E19 E20 E21 E22 E23 E24 E25 E26 E27 E28 E29 E30 E31 E32 E33 E34 E35 E36 E37 E38 E39 E40 E41 E42 E43 E2:E3 E44:E1048576">
+      <formula1>"B_IMM,B_RS2"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="M29 M30 M31 M39 M40 M41 M42 M43 M2:M28 M32:M38 M44:M1048576">
+      <formula1>"CSR_W,CSR_S,CSR_C,CSR_P,CSR_XX"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I4 I5 I6 I7 I8 I9 I10 I11 I12 I13 I14 I15 I16 I17 I18 I19 I20 I21 I22 I23 I24 I25 I26 I27 I28 I29 I30 I31 I32 I33 I34 I35 I36 I37 I38 I39 I40 I41 I42 I43 I2:I3 I44:I1048576">
       <formula1>"LD_LB,LD_LH,LD_LW,LD_LBU,LD_LHU,LD_XX"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F6 F15 F18 F19 F20 F21 F24 F25 F26 F27 F28 F29 F30 F31 F32 F33 F36 F37 F38 F39 F40 F41 F42 F43 F2:F5 F7:F14 F16:F17 F22:F23 F34:F35 F44:F1048576">
-      <formula1>"ALU_ADD,ALU_SUB,ALU_AND,ALU_OR,ALU_XOR,ALU_SLL,ALU_SRL,ALU_SLT,ALU_SLTU,ALU_COPY_A,ALU_COPY_B,ALU_SRA"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K4 K5 K6 K7 K8 K9 K10 K11 K12 K13 K14 K15 K16 K17 K18 K19 K20 K21 K22 K23 K24 K25 K26 K27 K28 K29 K30 K31 K32 K33 K34 K35 K36 K37 K38 K39 K40 K41 K42 K43 K2:K3 K44:K1048576">
-      <formula1>"MASK_XX,MASK_B,MASK_H,MASK_W,MASK_D"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D4 D5 D6 D7 D8 D9 D10 D11 D12 D13 D14 D15 D16 D17 D18 D19 D20 D21 D22 D23 D24 D25 D26 D27 D28 D29 D30 D31 D32 D33 D34 D35 D36 D37 D38 D39 D40 D41 D42 D43 D2:D3 D44:D1048576">
-      <formula1>"A_PC,A_RS1"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G4 G5 G6 G7 G8 G9 G10 G11 G12 G13 G14 G15 G16 G17 G18 G19 G20 G21 G22 G23 G24 G25 G26 G27 G28 G29 G30 G31 G32 G33 G34 G35 G36 G37 G38 G39 G40 G41 G42 G43 G2:G3 G44:G1048576">
+      <formula1>"IMM_I,IMM_J,IMM_U,IMM_S,IMM_B"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
> compile NEMU ysyx_23060246 韩炳晋 Linux archlinux 6.12.17-1-lts #1 SMP PREEMPT_DYNAMIC Thu, 27 Feb 2025 14:12:30 +0000 x86_64 GNU/Linux  14:07:30 up 17:57,  1 user,  load average: 0.43, 0.98, 2.64
</commit_message>
<xml_diff>
--- a/npc/tools/control_gen/control_table.xlsx
+++ b/npc/tools/control_gen/control_table.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="311" uniqueCount="112">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="355" uniqueCount="119">
   <si>
     <t>comment</t>
   </si>
@@ -76,6 +76,9 @@
     <t>INST_VALID</t>
   </si>
   <si>
+    <t>U_TYPE</t>
+  </si>
+  <si>
     <t>auipc</t>
   </si>
   <si>
@@ -94,6 +97,9 @@
     <t>IMM_I</t>
   </si>
   <si>
+    <t>I_TYPE</t>
+  </si>
+  <si>
     <t>andi</t>
   </si>
   <si>
@@ -127,6 +133,9 @@
     <t>IMM_J</t>
   </si>
   <si>
+    <t>J_TYPE</t>
+  </si>
+  <si>
     <t>sb</t>
   </si>
   <si>
@@ -139,6 +148,9 @@
     <t>MASK_B</t>
   </si>
   <si>
+    <t>S_TYPE</t>
+  </si>
+  <si>
     <t>sh</t>
   </si>
   <si>
@@ -199,6 +211,9 @@
     <t>BR_NE</t>
   </si>
   <si>
+    <t>B_TYPE</t>
+  </si>
+  <si>
     <t>beq</t>
   </si>
   <si>
@@ -247,6 +262,9 @@
     <t>B_RS2</t>
   </si>
   <si>
+    <t>R_TYPE</t>
+  </si>
+  <si>
     <t>sra</t>
   </si>
   <si>
@@ -320,6 +338,9 @@
   </si>
   <si>
     <t>CSR_P</t>
+  </si>
+  <si>
+    <t>N_TYPE</t>
   </si>
   <si>
     <t>mret</t>
@@ -358,9 +379,9 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="4">
     <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="42" formatCode="_ &quot;￥&quot;* #,##0_ ;_ &quot;￥&quot;* \-#,##0_ ;_ &quot;￥&quot;* &quot;-&quot;_ ;_ @_ "/>
     <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="41" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="42" formatCode="_ &quot;￥&quot;* #,##0_ ;_ &quot;￥&quot;* \-#,##0_ ;_ &quot;￥&quot;* &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
   <fonts count="22">
     <font>
@@ -378,21 +399,6 @@
     </font>
     <font>
       <sz val="10.8"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="3"/>
       <name val="宋体"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -419,6 +425,29 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF0000FF"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="3"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <b/>
       <sz val="18"/>
       <color theme="3"/>
@@ -432,22 +461,6 @@
       <color rgb="FF800080"/>
       <name val="宋体"/>
       <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="11"/>
-      <color rgb="FF7F7F7F"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="15"/>
-      <color theme="3"/>
-      <name val="宋体"/>
-      <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -476,14 +489,7 @@
     <font>
       <b/>
       <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF3F3F76"/>
+      <color theme="1"/>
       <name val="宋体"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -497,6 +503,21 @@
     </font>
     <font>
       <b/>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF006100"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="13"/>
       <color theme="3"/>
       <name val="宋体"/>
@@ -504,24 +525,24 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF0000FF"/>
+      <b/>
+      <sz val="15"/>
+      <color theme="3"/>
       <name val="宋体"/>
-      <charset val="0"/>
+      <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
+      <i/>
       <sz val="11"/>
-      <color theme="1"/>
+      <color rgb="FF7F7F7F"/>
       <name val="宋体"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FF006100"/>
+      <color rgb="FF3F3F76"/>
       <name val="宋体"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -536,7 +557,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.599993896298105"/>
+        <fgColor theme="4" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -554,19 +581,67 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="9"/>
+        <fgColor theme="5" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="7" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -584,25 +659,61 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor theme="4" tint="0.799981688894314"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.799981688894314"/>
+        <fgColor theme="6" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.799981688894314"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -614,37 +725,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.399975585192419"/>
+        <fgColor rgb="FFFFCC99"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -656,67 +737,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor theme="9" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -727,24 +748,6 @@
       <right/>
       <top/>
       <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="double">
-        <color rgb="FFFF8001"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4" tint="0.499984740745262"/>
-      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -766,8 +769,17 @@
       <left/>
       <right/>
       <top/>
+      <bottom style="double">
+        <color rgb="FFFF8001"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
       <bottom style="medium">
-        <color theme="4"/>
+        <color theme="4" tint="0.499984740745262"/>
       </bottom>
       <diagonal/>
     </border>
@@ -802,6 +814,17 @@
       <diagonal/>
     </border>
     <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="4"/>
+      </top>
+      <bottom style="double">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
       <left style="thin">
         <color rgb="FF7F7F7F"/>
       </left>
@@ -819,10 +842,8 @@
     <border>
       <left/>
       <right/>
-      <top style="thin">
-        <color theme="4"/>
-      </top>
-      <bottom style="double">
+      <top/>
+      <bottom style="medium">
         <color theme="4"/>
       </bottom>
       <diagonal/>
@@ -832,148 +853,148 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="10" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="4" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="30" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="4" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="7" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="8" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="7" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="15" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="17" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="15" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
@@ -1318,7 +1339,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:AI99"/>
+  <dimension ref="A1:AJ99"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
     <col min="1" max="1" width="13.1" customWidth="1"/>
@@ -1331,18 +1352,18 @@
     <col min="8" max="10" width="11.9833333333333" customWidth="1"/>
     <col min="11" max="11" width="15.075" customWidth="1"/>
     <col min="12" max="14" width="12.1083333333333" customWidth="1"/>
-    <col min="15" max="15" width="10.8583333333333" customWidth="1"/>
-    <col min="17" max="17" width="14.2166666666667" customWidth="1"/>
-    <col min="18" max="18" width="11.8083333333333" customWidth="1"/>
-    <col min="19" max="19" width="10.6" customWidth="1"/>
-    <col min="20" max="20" width="9.70833333333333" customWidth="1"/>
-    <col min="21" max="21" width="11.1666666666667" customWidth="1"/>
-    <col min="22" max="22" width="11.4083333333333" customWidth="1"/>
-    <col min="23" max="23" width="12.0583333333333" customWidth="1"/>
-    <col min="24" max="24" width="15.575" customWidth="1"/>
+    <col min="15" max="16" width="10.8583333333333" customWidth="1"/>
+    <col min="18" max="18" width="14.2166666666667" customWidth="1"/>
+    <col min="19" max="19" width="11.8083333333333" customWidth="1"/>
+    <col min="20" max="20" width="10.6" customWidth="1"/>
+    <col min="21" max="21" width="9.70833333333333" customWidth="1"/>
+    <col min="22" max="22" width="11.1666666666667" customWidth="1"/>
+    <col min="23" max="23" width="11.4083333333333" customWidth="1"/>
+    <col min="24" max="24" width="12.0583333333333" customWidth="1"/>
+    <col min="25" max="25" width="15.575" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="15" customHeight="1" spans="1:23">
+    <row r="1" ht="15" customHeight="1" spans="1:24">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1385,15 +1406,18 @@
       <c r="N1" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="2"/>
+      <c r="O1" s="2" t="s">
+        <v>1</v>
+      </c>
       <c r="P1" s="2"/>
       <c r="Q1" s="2"/>
       <c r="R1" s="2"/>
       <c r="S1" s="2"/>
       <c r="T1" s="2"/>
-      <c r="W1" s="6"/>
-    </row>
-    <row r="2" spans="1:35">
+      <c r="U1" s="2"/>
+      <c r="X1" s="6"/>
+    </row>
+    <row r="2" spans="1:36">
       <c r="A2" s="3"/>
       <c r="B2" s="4" t="s">
         <v>14</v>
@@ -1420,13 +1444,15 @@
       <c r="N2" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O2" s="4"/>
+      <c r="O2" s="4" t="s">
+        <v>20</v>
+      </c>
       <c r="P2" s="4"/>
       <c r="Q2" s="4"/>
       <c r="R2" s="4"/>
       <c r="S2" s="4"/>
       <c r="T2" s="4"/>
-      <c r="U2" s="3"/>
+      <c r="U2" s="4"/>
       <c r="V2" s="3"/>
       <c r="W2" s="3"/>
       <c r="X2" s="3"/>
@@ -1441,21 +1467,22 @@
       <c r="AG2" s="3"/>
       <c r="AH2" s="3"/>
       <c r="AI2" s="3"/>
-    </row>
-    <row r="3" spans="1:35">
+      <c r="AJ2" s="3"/>
+    </row>
+    <row r="3" spans="1:36">
       <c r="A3" s="3"/>
       <c r="B3" s="4" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C3" s="2"/>
       <c r="D3" s="4" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E3" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="G3" s="4" t="s">
         <v>17</v>
@@ -1471,13 +1498,15 @@
       <c r="N3" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O3" s="4"/>
+      <c r="O3" s="4" t="s">
+        <v>20</v>
+      </c>
       <c r="P3" s="4"/>
       <c r="Q3" s="4"/>
       <c r="R3" s="4"/>
       <c r="S3" s="4"/>
       <c r="T3" s="4"/>
-      <c r="U3" s="3"/>
+      <c r="U3" s="4"/>
       <c r="V3" s="3"/>
       <c r="W3" s="3"/>
       <c r="X3" s="3"/>
@@ -1492,24 +1521,25 @@
       <c r="AG3" s="3"/>
       <c r="AH3" s="3"/>
       <c r="AI3" s="3"/>
-    </row>
-    <row r="4" spans="1:35">
+      <c r="AJ3" s="3"/>
+    </row>
+    <row r="4" spans="1:36">
       <c r="A4" s="3"/>
       <c r="B4" s="4" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C4" s="2"/>
       <c r="D4" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E4" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="H4" s="4" t="s">
         <v>18</v>
@@ -1522,13 +1552,15 @@
       <c r="N4" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O4" s="4"/>
+      <c r="O4" s="4" t="s">
+        <v>27</v>
+      </c>
       <c r="P4" s="4"/>
       <c r="Q4" s="4"/>
       <c r="R4" s="4"/>
       <c r="S4" s="4"/>
       <c r="T4" s="4"/>
-      <c r="U4" s="3"/>
+      <c r="U4" s="4"/>
       <c r="V4" s="3"/>
       <c r="W4" s="3"/>
       <c r="X4" s="3"/>
@@ -1543,24 +1575,25 @@
       <c r="AG4" s="3"/>
       <c r="AH4" s="3"/>
       <c r="AI4" s="3"/>
-    </row>
-    <row r="5" spans="1:35">
+      <c r="AJ4" s="3"/>
+    </row>
+    <row r="5" spans="1:36">
       <c r="A5" s="3"/>
       <c r="B5" s="4" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="C5" s="2"/>
       <c r="D5" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E5" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="H5" s="4" t="s">
         <v>18</v>
@@ -1573,13 +1606,15 @@
       <c r="N5" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O5" s="4"/>
+      <c r="O5" s="4" t="s">
+        <v>27</v>
+      </c>
       <c r="P5" s="4"/>
       <c r="Q5" s="4"/>
       <c r="R5" s="4"/>
       <c r="S5" s="4"/>
       <c r="T5" s="4"/>
-      <c r="U5" s="3"/>
+      <c r="U5" s="4"/>
       <c r="V5" s="3"/>
       <c r="W5" s="3"/>
       <c r="X5" s="3"/>
@@ -1594,24 +1629,25 @@
       <c r="AG5" s="3"/>
       <c r="AH5" s="3"/>
       <c r="AI5" s="3"/>
-    </row>
-    <row r="6" spans="1:35">
+      <c r="AJ5" s="3"/>
+    </row>
+    <row r="6" spans="1:36">
       <c r="A6" s="3"/>
       <c r="B6" s="4" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="C6" s="2"/>
       <c r="D6" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E6" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="G6" s="4" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="H6" s="4" t="s">
         <v>18</v>
@@ -1624,13 +1660,15 @@
       <c r="N6" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O6" s="4"/>
+      <c r="O6" s="4" t="s">
+        <v>27</v>
+      </c>
       <c r="P6" s="4"/>
       <c r="Q6" s="4"/>
       <c r="R6" s="4"/>
       <c r="S6" s="4"/>
       <c r="T6" s="4"/>
-      <c r="U6" s="3"/>
+      <c r="U6" s="4"/>
       <c r="V6" s="3"/>
       <c r="W6" s="3"/>
       <c r="X6" s="3"/>
@@ -1645,24 +1683,25 @@
       <c r="AG6" s="3"/>
       <c r="AH6" s="3"/>
       <c r="AI6" s="3"/>
-    </row>
-    <row r="7" spans="1:35">
+      <c r="AJ6" s="3"/>
+    </row>
+    <row r="7" spans="1:36">
       <c r="A7" s="3"/>
       <c r="B7" s="4" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="C7" s="2"/>
       <c r="D7" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E7" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="G7" s="4" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="H7" s="4" t="s">
         <v>18</v>
@@ -1675,13 +1714,15 @@
       <c r="N7" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O7" s="4"/>
+      <c r="O7" s="4" t="s">
+        <v>27</v>
+      </c>
       <c r="P7" s="4"/>
       <c r="Q7" s="4"/>
       <c r="R7" s="4"/>
       <c r="S7" s="4"/>
       <c r="T7" s="4"/>
-      <c r="U7" s="3"/>
+      <c r="U7" s="4"/>
       <c r="V7" s="3"/>
       <c r="W7" s="3"/>
       <c r="X7" s="3"/>
@@ -1696,29 +1737,30 @@
       <c r="AG7" s="3"/>
       <c r="AH7" s="3"/>
       <c r="AI7" s="3"/>
-    </row>
-    <row r="8" spans="1:35">
+      <c r="AJ7" s="3"/>
+    </row>
+    <row r="8" spans="1:36">
       <c r="A8" s="3"/>
       <c r="B8" s="4" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E8" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F8" s="4" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="G8" s="4" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="H8" s="4" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="I8" s="4"/>
       <c r="J8" s="4"/>
@@ -1728,13 +1770,15 @@
       <c r="N8" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O8" s="4"/>
+      <c r="O8" s="4" t="s">
+        <v>27</v>
+      </c>
       <c r="P8" s="4"/>
       <c r="Q8" s="4"/>
       <c r="R8" s="4"/>
       <c r="S8" s="4"/>
       <c r="T8" s="4"/>
-      <c r="U8" s="3"/>
+      <c r="U8" s="4"/>
       <c r="V8" s="3"/>
       <c r="W8" s="3"/>
       <c r="X8" s="3"/>
@@ -1749,29 +1793,30 @@
       <c r="AG8" s="3"/>
       <c r="AH8" s="3"/>
       <c r="AI8" s="3"/>
-    </row>
-    <row r="9" spans="1:35">
+      <c r="AJ8" s="3"/>
+    </row>
+    <row r="9" spans="1:36">
       <c r="A9" s="3"/>
       <c r="B9" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="C9" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="C9" s="2" t="s">
-        <v>33</v>
-      </c>
       <c r="D9" s="4" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E9" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F9" s="4" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="G9" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="H9" s="4" t="s">
         <v>36</v>
-      </c>
-      <c r="H9" s="4" t="s">
-        <v>34</v>
       </c>
       <c r="I9" s="4"/>
       <c r="J9" s="4"/>
@@ -1781,13 +1826,15 @@
       <c r="N9" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O9" s="4"/>
+      <c r="O9" s="4" t="s">
+        <v>39</v>
+      </c>
       <c r="P9" s="4"/>
       <c r="Q9" s="4"/>
       <c r="R9" s="4"/>
       <c r="S9" s="4"/>
       <c r="T9" s="4"/>
-      <c r="U9" s="3"/>
+      <c r="U9" s="4"/>
       <c r="V9" s="3"/>
       <c r="W9" s="3"/>
       <c r="X9" s="3"/>
@@ -1802,45 +1849,48 @@
       <c r="AG9" s="3"/>
       <c r="AH9" s="3"/>
       <c r="AI9" s="3"/>
-    </row>
-    <row r="10" spans="1:35">
+      <c r="AJ9" s="3"/>
+    </row>
+    <row r="10" spans="1:36">
       <c r="A10" s="3"/>
       <c r="B10" s="4" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="C10" s="2"/>
       <c r="D10" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E10" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F10" s="4" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="G10" s="4" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="H10" s="4"/>
       <c r="I10" s="4"/>
       <c r="J10" s="4" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="K10" s="4" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="L10" s="4"/>
       <c r="M10" s="4"/>
       <c r="N10" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O10" s="4"/>
+      <c r="O10" s="4" t="s">
+        <v>44</v>
+      </c>
       <c r="P10" s="4"/>
       <c r="Q10" s="4"/>
       <c r="R10" s="4"/>
       <c r="S10" s="4"/>
       <c r="T10" s="4"/>
-      <c r="U10" s="3"/>
+      <c r="U10" s="4"/>
       <c r="V10" s="3"/>
       <c r="W10" s="3"/>
       <c r="X10" s="3"/>
@@ -1855,45 +1905,48 @@
       <c r="AG10" s="3"/>
       <c r="AH10" s="3"/>
       <c r="AI10" s="3"/>
-    </row>
-    <row r="11" spans="1:35">
+      <c r="AJ10" s="3"/>
+    </row>
+    <row r="11" spans="1:36">
       <c r="A11" s="3"/>
       <c r="B11" s="4" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="C11" s="2"/>
       <c r="D11" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E11" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F11" s="4" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="G11" s="4" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="H11" s="4"/>
       <c r="I11" s="4"/>
       <c r="J11" s="4" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="K11" s="4" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="L11" s="4"/>
       <c r="M11" s="4"/>
       <c r="N11" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O11" s="4"/>
+      <c r="O11" s="4" t="s">
+        <v>44</v>
+      </c>
       <c r="P11" s="4"/>
       <c r="Q11" s="4"/>
       <c r="R11" s="4"/>
       <c r="S11" s="4"/>
       <c r="T11" s="4"/>
-      <c r="U11" s="3"/>
+      <c r="U11" s="4"/>
       <c r="V11" s="3"/>
       <c r="W11" s="3"/>
       <c r="X11" s="3"/>
@@ -1908,45 +1961,48 @@
       <c r="AG11" s="3"/>
       <c r="AH11" s="3"/>
       <c r="AI11" s="3"/>
-    </row>
-    <row r="12" spans="1:35">
+      <c r="AJ11" s="3"/>
+    </row>
+    <row r="12" spans="1:36">
       <c r="A12" s="3"/>
       <c r="B12" s="4" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="C12" s="2"/>
       <c r="D12" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E12" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F12" s="4" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="G12" s="4" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="H12" s="4"/>
       <c r="I12" s="4"/>
       <c r="J12" s="4" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="K12" s="4" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="L12" s="4"/>
       <c r="M12" s="4"/>
       <c r="N12" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O12" s="4"/>
+      <c r="O12" s="4" t="s">
+        <v>44</v>
+      </c>
       <c r="P12" s="4"/>
       <c r="Q12" s="4"/>
       <c r="R12" s="4"/>
       <c r="S12" s="4"/>
       <c r="T12" s="4"/>
-      <c r="U12" s="3"/>
+      <c r="U12" s="4"/>
       <c r="V12" s="3"/>
       <c r="W12" s="3"/>
       <c r="X12" s="3"/>
@@ -1961,30 +2017,31 @@
       <c r="AG12" s="3"/>
       <c r="AH12" s="3"/>
       <c r="AI12" s="3"/>
-    </row>
-    <row r="13" spans="1:35">
+      <c r="AJ12" s="3"/>
+    </row>
+    <row r="13" spans="1:36">
       <c r="A13" s="3"/>
       <c r="B13" s="4" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="C13" s="2"/>
       <c r="D13" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E13" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F13" s="4" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="G13" s="4" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="H13" s="4" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="I13" s="4" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="J13" s="4"/>
       <c r="K13" s="4"/>
@@ -1993,13 +2050,15 @@
       <c r="N13" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O13" s="4"/>
+      <c r="O13" s="4" t="s">
+        <v>27</v>
+      </c>
       <c r="P13" s="4"/>
       <c r="Q13" s="4"/>
       <c r="R13" s="4"/>
       <c r="S13" s="4"/>
       <c r="T13" s="4"/>
-      <c r="U13" s="3"/>
+      <c r="U13" s="4"/>
       <c r="V13" s="3"/>
       <c r="W13" s="3"/>
       <c r="X13" s="3"/>
@@ -2014,30 +2073,31 @@
       <c r="AG13" s="3"/>
       <c r="AH13" s="3"/>
       <c r="AI13" s="3"/>
-    </row>
-    <row r="14" spans="1:35">
+      <c r="AJ13" s="3"/>
+    </row>
+    <row r="14" spans="1:36">
       <c r="A14" s="3"/>
       <c r="B14" s="4" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="C14" s="2"/>
       <c r="D14" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E14" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F14" s="4" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="G14" s="4" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="H14" s="4" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="I14" s="4" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="J14" s="4"/>
       <c r="K14" s="4"/>
@@ -2046,13 +2106,15 @@
       <c r="N14" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O14" s="4"/>
+      <c r="O14" s="4" t="s">
+        <v>27</v>
+      </c>
       <c r="P14" s="4"/>
       <c r="Q14" s="4"/>
       <c r="R14" s="4"/>
       <c r="S14" s="4"/>
       <c r="T14" s="4"/>
-      <c r="U14" s="3"/>
+      <c r="U14" s="4"/>
       <c r="V14" s="3"/>
       <c r="W14" s="3"/>
       <c r="X14" s="3"/>
@@ -2067,30 +2129,31 @@
       <c r="AG14" s="3"/>
       <c r="AH14" s="3"/>
       <c r="AI14" s="3"/>
-    </row>
-    <row r="15" spans="1:35">
+      <c r="AJ14" s="3"/>
+    </row>
+    <row r="15" spans="1:36">
       <c r="A15" s="3"/>
       <c r="B15" s="4" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="C15" s="2"/>
       <c r="D15" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E15" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F15" s="4" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="G15" s="4" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="H15" s="4" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="I15" s="4" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="J15" s="4"/>
       <c r="K15" s="4"/>
@@ -2099,13 +2162,15 @@
       <c r="N15" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O15" s="4"/>
+      <c r="O15" s="4" t="s">
+        <v>27</v>
+      </c>
       <c r="P15" s="4"/>
       <c r="Q15" s="4"/>
       <c r="R15" s="4"/>
       <c r="S15" s="4"/>
       <c r="T15" s="4"/>
-      <c r="U15" s="3"/>
+      <c r="U15" s="4"/>
       <c r="V15" s="3"/>
       <c r="W15" s="3"/>
       <c r="X15" s="3"/>
@@ -2120,30 +2185,31 @@
       <c r="AG15" s="3"/>
       <c r="AH15" s="3"/>
       <c r="AI15" s="3"/>
-    </row>
-    <row r="16" spans="1:35">
+      <c r="AJ15" s="3"/>
+    </row>
+    <row r="16" spans="1:36">
       <c r="A16" s="3"/>
       <c r="B16" s="4" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="C16" s="2"/>
       <c r="D16" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E16" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F16" s="4" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="G16" s="4" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="H16" s="4" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="I16" s="4" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="J16" s="4"/>
       <c r="K16" s="4"/>
@@ -2152,13 +2218,15 @@
       <c r="N16" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O16" s="4"/>
+      <c r="O16" s="4" t="s">
+        <v>27</v>
+      </c>
       <c r="P16" s="4"/>
       <c r="Q16" s="4"/>
       <c r="R16" s="4"/>
       <c r="S16" s="4"/>
       <c r="T16" s="4"/>
-      <c r="U16" s="3"/>
+      <c r="U16" s="4"/>
       <c r="V16" s="3"/>
       <c r="W16" s="3"/>
       <c r="X16" s="3"/>
@@ -2173,30 +2241,31 @@
       <c r="AG16" s="3"/>
       <c r="AH16" s="3"/>
       <c r="AI16" s="3"/>
-    </row>
-    <row r="17" spans="1:35">
+      <c r="AJ16" s="3"/>
+    </row>
+    <row r="17" spans="1:36">
       <c r="A17" s="3"/>
       <c r="B17" s="4" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="C17" s="2"/>
       <c r="D17" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E17" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F17" s="4" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="G17" s="4" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="H17" s="4" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="I17" s="4" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="J17" s="4"/>
       <c r="K17" s="4"/>
@@ -2205,13 +2274,15 @@
       <c r="N17" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O17" s="4"/>
+      <c r="O17" s="4" t="s">
+        <v>27</v>
+      </c>
       <c r="P17" s="4"/>
       <c r="Q17" s="4"/>
       <c r="R17" s="4"/>
       <c r="S17" s="4"/>
       <c r="T17" s="4"/>
-      <c r="U17" s="3"/>
+      <c r="U17" s="4"/>
       <c r="V17" s="3"/>
       <c r="W17" s="3"/>
       <c r="X17" s="3"/>
@@ -2226,43 +2297,46 @@
       <c r="AG17" s="3"/>
       <c r="AH17" s="3"/>
       <c r="AI17" s="3"/>
-    </row>
-    <row r="18" spans="1:35">
+      <c r="AJ17" s="3"/>
+    </row>
+    <row r="18" spans="1:36">
       <c r="A18" s="3"/>
       <c r="B18" s="4" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="C18" s="2"/>
       <c r="D18" s="4" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E18" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F18" s="4" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="G18" s="4" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="H18" s="4"/>
       <c r="I18" s="4"/>
       <c r="J18" s="4"/>
       <c r="K18" s="4"/>
       <c r="L18" s="4" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="M18" s="4"/>
       <c r="N18" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O18" s="4"/>
+      <c r="O18" s="4" t="s">
+        <v>65</v>
+      </c>
       <c r="P18" s="4"/>
       <c r="Q18" s="4"/>
       <c r="R18" s="4"/>
       <c r="S18" s="4"/>
       <c r="T18" s="4"/>
-      <c r="U18" s="3"/>
+      <c r="U18" s="4"/>
       <c r="V18" s="3"/>
       <c r="W18" s="3"/>
       <c r="X18" s="3"/>
@@ -2277,43 +2351,46 @@
       <c r="AG18" s="3"/>
       <c r="AH18" s="3"/>
       <c r="AI18" s="3"/>
-    </row>
-    <row r="19" spans="1:35">
+      <c r="AJ18" s="3"/>
+    </row>
+    <row r="19" spans="1:36">
       <c r="A19" s="3"/>
       <c r="B19" s="4" t="s">
-        <v>61</v>
+        <v>66</v>
       </c>
       <c r="C19" s="2"/>
       <c r="D19" s="4" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E19" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F19" s="4" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="G19" s="4" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="H19" s="4"/>
       <c r="I19" s="4"/>
       <c r="J19" s="4"/>
       <c r="K19" s="4"/>
       <c r="L19" s="4" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="M19" s="4"/>
       <c r="N19" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O19" s="4"/>
+      <c r="O19" s="4" t="s">
+        <v>65</v>
+      </c>
       <c r="P19" s="4"/>
       <c r="Q19" s="4"/>
       <c r="R19" s="4"/>
       <c r="S19" s="4"/>
       <c r="T19" s="4"/>
-      <c r="U19" s="3"/>
+      <c r="U19" s="4"/>
       <c r="V19" s="3"/>
       <c r="W19" s="3"/>
       <c r="X19" s="3"/>
@@ -2328,43 +2405,46 @@
       <c r="AG19" s="3"/>
       <c r="AH19" s="3"/>
       <c r="AI19" s="3"/>
-    </row>
-    <row r="20" spans="1:35">
+      <c r="AJ19" s="3"/>
+    </row>
+    <row r="20" spans="1:36">
       <c r="A20" s="3"/>
       <c r="B20" s="4" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="C20" s="2"/>
       <c r="D20" s="4" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E20" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F20" s="4" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="G20" s="4" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="H20" s="4"/>
       <c r="I20" s="4"/>
       <c r="J20" s="4"/>
       <c r="K20" s="4"/>
       <c r="L20" s="4" t="s">
-        <v>64</v>
+        <v>69</v>
       </c>
       <c r="M20" s="4"/>
       <c r="N20" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O20" s="4"/>
+      <c r="O20" s="4" t="s">
+        <v>65</v>
+      </c>
       <c r="P20" s="4"/>
       <c r="Q20" s="4"/>
       <c r="R20" s="4"/>
       <c r="S20" s="4"/>
       <c r="T20" s="4"/>
-      <c r="U20" s="3"/>
+      <c r="U20" s="4"/>
       <c r="V20" s="3"/>
       <c r="W20" s="3"/>
       <c r="X20" s="3"/>
@@ -2379,43 +2459,46 @@
       <c r="AG20" s="3"/>
       <c r="AH20" s="3"/>
       <c r="AI20" s="3"/>
-    </row>
-    <row r="21" spans="1:35">
+      <c r="AJ20" s="3"/>
+    </row>
+    <row r="21" spans="1:36">
       <c r="A21" s="3"/>
       <c r="B21" s="4" t="s">
-        <v>65</v>
+        <v>70</v>
       </c>
       <c r="C21" s="2"/>
       <c r="D21" s="4" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E21" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F21" s="4" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="G21" s="4" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="H21" s="4"/>
       <c r="I21" s="4"/>
       <c r="J21" s="4"/>
       <c r="K21" s="4"/>
       <c r="L21" s="4" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="M21" s="4"/>
       <c r="N21" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O21" s="4"/>
+      <c r="O21" s="4" t="s">
+        <v>65</v>
+      </c>
       <c r="P21" s="4"/>
       <c r="Q21" s="4"/>
       <c r="R21" s="4"/>
       <c r="S21" s="4"/>
       <c r="T21" s="4"/>
-      <c r="U21" s="3"/>
+      <c r="U21" s="4"/>
       <c r="V21" s="3"/>
       <c r="W21" s="3"/>
       <c r="X21" s="3"/>
@@ -2430,43 +2513,46 @@
       <c r="AG21" s="3"/>
       <c r="AH21" s="3"/>
       <c r="AI21" s="3"/>
-    </row>
-    <row r="22" spans="1:35">
+      <c r="AJ21" s="3"/>
+    </row>
+    <row r="22" spans="1:36">
       <c r="A22" s="3"/>
       <c r="B22" s="4" t="s">
-        <v>67</v>
+        <v>72</v>
       </c>
       <c r="C22" s="2"/>
       <c r="D22" s="4" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E22" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F22" s="4" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="G22" s="4" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="H22" s="4"/>
       <c r="I22" s="4"/>
       <c r="J22" s="4"/>
       <c r="K22" s="4"/>
       <c r="L22" s="4" t="s">
-        <v>68</v>
+        <v>73</v>
       </c>
       <c r="M22" s="4"/>
       <c r="N22" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O22" s="4"/>
+      <c r="O22" s="4" t="s">
+        <v>65</v>
+      </c>
       <c r="P22" s="4"/>
       <c r="Q22" s="4"/>
       <c r="R22" s="4"/>
       <c r="S22" s="4"/>
       <c r="T22" s="4"/>
-      <c r="U22" s="3"/>
+      <c r="U22" s="4"/>
       <c r="V22" s="3"/>
       <c r="W22" s="3"/>
       <c r="X22" s="3"/>
@@ -2481,43 +2567,46 @@
       <c r="AG22" s="3"/>
       <c r="AH22" s="3"/>
       <c r="AI22" s="3"/>
-    </row>
-    <row r="23" spans="1:35">
+      <c r="AJ22" s="3"/>
+    </row>
+    <row r="23" spans="1:36">
       <c r="A23" s="3"/>
       <c r="B23" s="4" t="s">
-        <v>69</v>
+        <v>74</v>
       </c>
       <c r="C23" s="2"/>
       <c r="D23" s="4" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E23" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F23" s="4" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="G23" s="4" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="H23" s="4"/>
       <c r="I23" s="4"/>
       <c r="J23" s="4"/>
       <c r="K23" s="4"/>
       <c r="L23" s="4" t="s">
-        <v>70</v>
+        <v>75</v>
       </c>
       <c r="M23" s="4"/>
       <c r="N23" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O23" s="4"/>
+      <c r="O23" s="4" t="s">
+        <v>65</v>
+      </c>
       <c r="P23" s="4"/>
       <c r="Q23" s="4"/>
       <c r="R23" s="4"/>
       <c r="S23" s="4"/>
       <c r="T23" s="4"/>
-      <c r="U23" s="3"/>
+      <c r="U23" s="4"/>
       <c r="V23" s="3"/>
       <c r="W23" s="3"/>
       <c r="X23" s="3"/>
@@ -2532,24 +2621,25 @@
       <c r="AG23" s="3"/>
       <c r="AH23" s="3"/>
       <c r="AI23" s="3"/>
-    </row>
-    <row r="24" spans="1:35">
+      <c r="AJ23" s="3"/>
+    </row>
+    <row r="24" spans="1:36">
       <c r="A24" s="3"/>
       <c r="B24" s="4" t="s">
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="C24" s="2"/>
       <c r="D24" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E24" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F24" s="4" t="s">
-        <v>72</v>
+        <v>77</v>
       </c>
       <c r="G24" s="4" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="H24" s="4" t="s">
         <v>18</v>
@@ -2562,13 +2652,15 @@
       <c r="N24" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O24" s="4"/>
+      <c r="O24" s="4" t="s">
+        <v>27</v>
+      </c>
       <c r="P24" s="4"/>
       <c r="Q24" s="4"/>
       <c r="R24" s="4"/>
       <c r="S24" s="4"/>
       <c r="T24" s="4"/>
-      <c r="U24" s="3"/>
+      <c r="U24" s="4"/>
       <c r="V24" s="3"/>
       <c r="W24" s="3"/>
       <c r="X24" s="3"/>
@@ -2583,24 +2675,25 @@
       <c r="AG24" s="3"/>
       <c r="AH24" s="3"/>
       <c r="AI24" s="3"/>
-    </row>
-    <row r="25" spans="1:35">
+      <c r="AJ24" s="3"/>
+    </row>
+    <row r="25" spans="1:36">
       <c r="A25" s="3"/>
       <c r="B25" s="4" t="s">
-        <v>73</v>
+        <v>78</v>
       </c>
       <c r="C25" s="2"/>
       <c r="D25" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E25" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F25" s="4" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="G25" s="4" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="H25" s="4" t="s">
         <v>18</v>
@@ -2613,13 +2706,15 @@
       <c r="N25" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O25" s="4"/>
+      <c r="O25" s="4" t="s">
+        <v>27</v>
+      </c>
       <c r="P25" s="4"/>
       <c r="Q25" s="4"/>
       <c r="R25" s="4"/>
       <c r="S25" s="4"/>
       <c r="T25" s="4"/>
-      <c r="U25" s="3"/>
+      <c r="U25" s="4"/>
       <c r="V25" s="3"/>
       <c r="W25" s="3"/>
       <c r="X25" s="3"/>
@@ -2634,21 +2729,22 @@
       <c r="AG25" s="3"/>
       <c r="AH25" s="3"/>
       <c r="AI25" s="3"/>
-    </row>
-    <row r="26" spans="1:35">
+      <c r="AJ25" s="3"/>
+    </row>
+    <row r="26" spans="1:36">
       <c r="A26" s="3"/>
       <c r="B26" s="4" t="s">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="C26" s="2"/>
       <c r="D26" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E26" s="4" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="F26" s="4" t="s">
-        <v>72</v>
+        <v>77</v>
       </c>
       <c r="G26" s="4"/>
       <c r="H26" s="4" t="s">
@@ -2662,13 +2758,15 @@
       <c r="N26" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O26" s="4"/>
+      <c r="O26" s="4" t="s">
+        <v>82</v>
+      </c>
       <c r="P26" s="4"/>
       <c r="Q26" s="4"/>
       <c r="R26" s="4"/>
       <c r="S26" s="4"/>
       <c r="T26" s="4"/>
-      <c r="U26" s="3"/>
+      <c r="U26" s="4"/>
       <c r="V26" s="3"/>
       <c r="W26" s="3"/>
       <c r="X26" s="3"/>
@@ -2683,21 +2781,22 @@
       <c r="AG26" s="3"/>
       <c r="AH26" s="3"/>
       <c r="AI26" s="3"/>
-    </row>
-    <row r="27" spans="1:35">
+      <c r="AJ26" s="3"/>
+    </row>
+    <row r="27" spans="1:36">
       <c r="A27" s="3"/>
       <c r="B27" s="4" t="s">
-        <v>77</v>
+        <v>83</v>
       </c>
       <c r="C27" s="2"/>
       <c r="D27" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E27" s="4" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="F27" s="4" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="G27" s="4"/>
       <c r="H27" s="4" t="s">
@@ -2711,13 +2810,15 @@
       <c r="N27" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O27" s="4"/>
+      <c r="O27" s="4" t="s">
+        <v>82</v>
+      </c>
       <c r="P27" s="4"/>
       <c r="Q27" s="4"/>
       <c r="R27" s="4"/>
       <c r="S27" s="4"/>
       <c r="T27" s="4"/>
-      <c r="U27" s="3"/>
+      <c r="U27" s="4"/>
       <c r="V27" s="3"/>
       <c r="W27" s="3"/>
       <c r="X27" s="3"/>
@@ -2732,24 +2833,25 @@
       <c r="AG27" s="3"/>
       <c r="AH27" s="3"/>
       <c r="AI27" s="3"/>
-    </row>
-    <row r="28" spans="1:35">
+      <c r="AJ27" s="3"/>
+    </row>
+    <row r="28" spans="1:36">
       <c r="A28" s="3"/>
       <c r="B28" s="4" t="s">
-        <v>78</v>
+        <v>84</v>
       </c>
       <c r="C28" s="2"/>
       <c r="D28" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E28" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F28" s="4" t="s">
-        <v>79</v>
+        <v>85</v>
       </c>
       <c r="G28" s="4" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="H28" s="4" t="s">
         <v>18</v>
@@ -2762,13 +2864,15 @@
       <c r="N28" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O28" s="4"/>
+      <c r="O28" s="4" t="s">
+        <v>27</v>
+      </c>
       <c r="P28" s="4"/>
       <c r="Q28" s="4"/>
       <c r="R28" s="4"/>
       <c r="S28" s="4"/>
       <c r="T28" s="4"/>
-      <c r="U28" s="3"/>
+      <c r="U28" s="4"/>
       <c r="V28" s="3"/>
       <c r="W28" s="3"/>
       <c r="X28" s="3"/>
@@ -2783,21 +2887,22 @@
       <c r="AG28" s="3"/>
       <c r="AH28" s="3"/>
       <c r="AI28" s="3"/>
-    </row>
-    <row r="29" spans="1:35">
+      <c r="AJ28" s="3"/>
+    </row>
+    <row r="29" spans="1:36">
       <c r="A29" s="3"/>
       <c r="B29" s="4" t="s">
-        <v>80</v>
+        <v>86</v>
       </c>
       <c r="C29" s="2"/>
       <c r="D29" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E29" s="4" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="F29" s="4" t="s">
-        <v>81</v>
+        <v>87</v>
       </c>
       <c r="G29" s="4"/>
       <c r="H29" s="4" t="s">
@@ -2811,13 +2916,15 @@
       <c r="N29" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O29" s="4"/>
+      <c r="O29" s="4" t="s">
+        <v>82</v>
+      </c>
       <c r="P29" s="4"/>
       <c r="Q29" s="4"/>
       <c r="R29" s="4"/>
       <c r="S29" s="4"/>
       <c r="T29" s="4"/>
-      <c r="U29" s="3"/>
+      <c r="U29" s="4"/>
       <c r="V29" s="3"/>
       <c r="W29" s="3"/>
       <c r="X29" s="3"/>
@@ -2832,21 +2939,22 @@
       <c r="AG29" s="3"/>
       <c r="AH29" s="3"/>
       <c r="AI29" s="3"/>
-    </row>
-    <row r="30" spans="1:35">
+      <c r="AJ29" s="3"/>
+    </row>
+    <row r="30" spans="1:36">
       <c r="A30" s="3"/>
       <c r="B30" s="4" t="s">
-        <v>82</v>
+        <v>88</v>
       </c>
       <c r="C30" s="2"/>
       <c r="D30" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E30" s="4" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="F30" s="4" t="s">
-        <v>83</v>
+        <v>89</v>
       </c>
       <c r="G30" s="4"/>
       <c r="H30" s="4" t="s">
@@ -2860,13 +2968,15 @@
       <c r="N30" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O30" s="4"/>
+      <c r="O30" s="4" t="s">
+        <v>82</v>
+      </c>
       <c r="P30" s="4"/>
       <c r="Q30" s="4"/>
       <c r="R30" s="4"/>
       <c r="S30" s="4"/>
       <c r="T30" s="4"/>
-      <c r="U30" s="3"/>
+      <c r="U30" s="4"/>
       <c r="V30" s="3"/>
       <c r="W30" s="3"/>
       <c r="X30" s="3"/>
@@ -2881,24 +2991,25 @@
       <c r="AG30" s="3"/>
       <c r="AH30" s="3"/>
       <c r="AI30" s="3"/>
-    </row>
-    <row r="31" spans="1:35">
+      <c r="AJ30" s="3"/>
+    </row>
+    <row r="31" spans="1:36">
       <c r="A31" s="3"/>
       <c r="B31" s="4" t="s">
-        <v>84</v>
+        <v>90</v>
       </c>
       <c r="C31" s="2"/>
       <c r="D31" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E31" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F31" s="4" t="s">
-        <v>83</v>
+        <v>89</v>
       </c>
       <c r="G31" s="4" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="H31" s="4" t="s">
         <v>18</v>
@@ -2911,13 +3022,15 @@
       <c r="N31" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O31" s="4"/>
+      <c r="O31" s="4" t="s">
+        <v>27</v>
+      </c>
       <c r="P31" s="4"/>
       <c r="Q31" s="4"/>
       <c r="R31" s="4"/>
       <c r="S31" s="4"/>
       <c r="T31" s="4"/>
-      <c r="U31" s="3"/>
+      <c r="U31" s="4"/>
       <c r="V31" s="3"/>
       <c r="W31" s="3"/>
       <c r="X31" s="3"/>
@@ -2932,24 +3045,25 @@
       <c r="AG31" s="3"/>
       <c r="AH31" s="3"/>
       <c r="AI31" s="3"/>
-    </row>
-    <row r="32" spans="1:35">
+      <c r="AJ31" s="3"/>
+    </row>
+    <row r="32" spans="1:36">
       <c r="A32" s="3"/>
       <c r="B32" s="4" t="s">
-        <v>85</v>
+        <v>91</v>
       </c>
       <c r="C32" s="2"/>
       <c r="D32" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E32" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F32" s="4" t="s">
-        <v>83</v>
+        <v>89</v>
       </c>
       <c r="G32" s="4" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="H32" s="4" t="s">
         <v>18</v>
@@ -2962,13 +3076,15 @@
       <c r="N32" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O32" s="4"/>
+      <c r="O32" s="4" t="s">
+        <v>27</v>
+      </c>
       <c r="P32" s="4"/>
       <c r="Q32" s="4"/>
       <c r="R32" s="4"/>
       <c r="S32" s="4"/>
       <c r="T32" s="4"/>
-      <c r="U32" s="3"/>
+      <c r="U32" s="4"/>
       <c r="V32" s="3"/>
       <c r="W32" s="3"/>
       <c r="X32" s="3"/>
@@ -2983,21 +3099,22 @@
       <c r="AG32" s="3"/>
       <c r="AH32" s="3"/>
       <c r="AI32" s="3"/>
-    </row>
-    <row r="33" spans="1:35">
+      <c r="AJ32" s="3"/>
+    </row>
+    <row r="33" spans="1:36">
       <c r="A33" s="3"/>
       <c r="B33" s="4" t="s">
-        <v>86</v>
+        <v>92</v>
       </c>
       <c r="C33" s="2"/>
       <c r="D33" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E33" s="4" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="F33" s="4" t="s">
-        <v>79</v>
+        <v>85</v>
       </c>
       <c r="G33" s="4"/>
       <c r="H33" s="4" t="s">
@@ -3011,13 +3128,15 @@
       <c r="N33" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O33" s="4"/>
+      <c r="O33" s="4" t="s">
+        <v>82</v>
+      </c>
       <c r="P33" s="4"/>
       <c r="Q33" s="4"/>
       <c r="R33" s="4"/>
       <c r="S33" s="4"/>
       <c r="T33" s="4"/>
-      <c r="U33" s="3"/>
+      <c r="U33" s="4"/>
       <c r="V33" s="3"/>
       <c r="W33" s="3"/>
       <c r="X33" s="3"/>
@@ -3032,21 +3151,22 @@
       <c r="AG33" s="3"/>
       <c r="AH33" s="3"/>
       <c r="AI33" s="3"/>
-    </row>
-    <row r="34" spans="1:35">
+      <c r="AJ33" s="3"/>
+    </row>
+    <row r="34" spans="1:36">
       <c r="A34" s="3"/>
       <c r="B34" s="4" t="s">
-        <v>87</v>
+        <v>93</v>
       </c>
       <c r="C34" s="2"/>
       <c r="D34" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E34" s="4" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="F34" s="4" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="G34" s="4"/>
       <c r="H34" s="4" t="s">
@@ -3060,13 +3180,15 @@
       <c r="N34" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O34" s="4"/>
+      <c r="O34" s="4" t="s">
+        <v>82</v>
+      </c>
       <c r="P34" s="4"/>
       <c r="Q34" s="4"/>
       <c r="R34" s="4"/>
       <c r="S34" s="4"/>
       <c r="T34" s="4"/>
-      <c r="U34" s="3"/>
+      <c r="U34" s="4"/>
       <c r="V34" s="3"/>
       <c r="W34" s="3"/>
       <c r="X34" s="3"/>
@@ -3081,21 +3203,22 @@
       <c r="AG34" s="3"/>
       <c r="AH34" s="3"/>
       <c r="AI34" s="3"/>
-    </row>
-    <row r="35" spans="1:35">
+      <c r="AJ34" s="3"/>
+    </row>
+    <row r="35" spans="1:36">
       <c r="A35" s="3"/>
       <c r="B35" s="4" t="s">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="C35" s="2"/>
       <c r="D35" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E35" s="4" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="F35" s="4" t="s">
-        <v>89</v>
+        <v>95</v>
       </c>
       <c r="G35" s="4"/>
       <c r="H35" s="4" t="s">
@@ -3109,13 +3232,15 @@
       <c r="N35" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O35" s="4"/>
+      <c r="O35" s="4" t="s">
+        <v>82</v>
+      </c>
       <c r="P35" s="4"/>
       <c r="Q35" s="4"/>
       <c r="R35" s="4"/>
       <c r="S35" s="4"/>
       <c r="T35" s="4"/>
-      <c r="U35" s="3"/>
+      <c r="U35" s="4"/>
       <c r="V35" s="3"/>
       <c r="W35" s="3"/>
       <c r="X35" s="3"/>
@@ -3130,21 +3255,22 @@
       <c r="AG35" s="3"/>
       <c r="AH35" s="3"/>
       <c r="AI35" s="3"/>
-    </row>
-    <row r="36" spans="1:35">
+      <c r="AJ35" s="3"/>
+    </row>
+    <row r="36" spans="1:36">
       <c r="A36" s="3"/>
       <c r="B36" s="4" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="C36" s="2"/>
       <c r="D36" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E36" s="4" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="F36" s="4" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="G36" s="4"/>
       <c r="H36" s="4" t="s">
@@ -3158,13 +3284,15 @@
       <c r="N36" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O36" s="4"/>
+      <c r="O36" s="4" t="s">
+        <v>82</v>
+      </c>
       <c r="P36" s="4"/>
       <c r="Q36" s="4"/>
       <c r="R36" s="4"/>
       <c r="S36" s="4"/>
       <c r="T36" s="4"/>
-      <c r="U36" s="3"/>
+      <c r="U36" s="4"/>
       <c r="V36" s="3"/>
       <c r="W36" s="3"/>
       <c r="X36" s="3"/>
@@ -3179,21 +3307,22 @@
       <c r="AG36" s="3"/>
       <c r="AH36" s="3"/>
       <c r="AI36" s="3"/>
-    </row>
-    <row r="37" spans="1:35">
+      <c r="AJ36" s="3"/>
+    </row>
+    <row r="37" spans="1:36">
       <c r="A37" s="3"/>
       <c r="B37" s="4" t="s">
-        <v>91</v>
+        <v>97</v>
       </c>
       <c r="C37" s="2"/>
       <c r="D37" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E37" s="4" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="F37" s="4" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="G37" s="4"/>
       <c r="H37" s="4" t="s">
@@ -3207,13 +3336,15 @@
       <c r="N37" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O37" s="4"/>
+      <c r="O37" s="4" t="s">
+        <v>82</v>
+      </c>
       <c r="P37" s="4"/>
       <c r="Q37" s="4"/>
       <c r="R37" s="4"/>
       <c r="S37" s="4"/>
       <c r="T37" s="4"/>
-      <c r="U37" s="3"/>
+      <c r="U37" s="4"/>
       <c r="V37" s="3"/>
       <c r="W37" s="3"/>
       <c r="X37" s="3"/>
@@ -3228,21 +3359,22 @@
       <c r="AG37" s="3"/>
       <c r="AH37" s="3"/>
       <c r="AI37" s="3"/>
-    </row>
-    <row r="38" spans="1:35">
+      <c r="AJ37" s="3"/>
+    </row>
+    <row r="38" spans="1:36">
       <c r="A38" s="3"/>
       <c r="B38" s="4" t="s">
-        <v>92</v>
+        <v>98</v>
       </c>
       <c r="C38" s="2"/>
       <c r="D38" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E38" s="4" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="F38" s="4" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="G38" s="4"/>
       <c r="H38" s="4" t="s">
@@ -3256,13 +3388,15 @@
       <c r="N38" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O38" s="4"/>
+      <c r="O38" s="4" t="s">
+        <v>82</v>
+      </c>
       <c r="P38" s="4"/>
       <c r="Q38" s="4"/>
       <c r="R38" s="4"/>
       <c r="S38" s="4"/>
       <c r="T38" s="4"/>
-      <c r="U38" s="3"/>
+      <c r="U38" s="4"/>
       <c r="V38" s="3"/>
       <c r="W38" s="3"/>
       <c r="X38" s="3"/>
@@ -3277,43 +3411,46 @@
       <c r="AG38" s="3"/>
       <c r="AH38" s="3"/>
       <c r="AI38" s="3"/>
-    </row>
-    <row r="39" spans="1:35">
+      <c r="AJ38" s="3"/>
+    </row>
+    <row r="39" spans="1:36">
       <c r="A39" s="3"/>
       <c r="B39" s="4" t="s">
-        <v>93</v>
+        <v>99</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="D39" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E39" s="4" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="F39" s="4"/>
       <c r="G39" s="4"/>
       <c r="H39" s="4" t="s">
-        <v>95</v>
+        <v>101</v>
       </c>
       <c r="I39" s="4"/>
       <c r="J39" s="4"/>
       <c r="K39" s="4"/>
       <c r="L39" s="4"/>
       <c r="M39" s="4" t="s">
-        <v>96</v>
+        <v>102</v>
       </c>
       <c r="N39" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O39" s="4"/>
+      <c r="O39" s="4" t="s">
+        <v>82</v>
+      </c>
       <c r="P39" s="4"/>
       <c r="Q39" s="4"/>
       <c r="R39" s="4"/>
       <c r="S39" s="4"/>
       <c r="T39" s="4"/>
-      <c r="U39" s="3"/>
+      <c r="U39" s="4"/>
       <c r="V39" s="3"/>
       <c r="W39" s="3"/>
       <c r="X39" s="3"/>
@@ -3328,43 +3465,46 @@
       <c r="AG39" s="3"/>
       <c r="AH39" s="3"/>
       <c r="AI39" s="3"/>
-    </row>
-    <row r="40" spans="1:35">
+      <c r="AJ39" s="3"/>
+    </row>
+    <row r="40" spans="1:36">
       <c r="A40" s="3"/>
       <c r="B40" s="4" t="s">
-        <v>97</v>
+        <v>103</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="D40" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E40" s="4" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="F40" s="4"/>
       <c r="G40" s="4"/>
       <c r="H40" s="4" t="s">
-        <v>95</v>
+        <v>101</v>
       </c>
       <c r="I40" s="4"/>
       <c r="J40" s="4"/>
       <c r="K40" s="4"/>
       <c r="L40" s="4"/>
       <c r="M40" s="4" t="s">
-        <v>98</v>
+        <v>104</v>
       </c>
       <c r="N40" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O40" s="4"/>
+      <c r="O40" s="4" t="s">
+        <v>82</v>
+      </c>
       <c r="P40" s="4"/>
       <c r="Q40" s="4"/>
       <c r="R40" s="4"/>
       <c r="S40" s="4"/>
       <c r="T40" s="4"/>
-      <c r="U40" s="3"/>
+      <c r="U40" s="4"/>
       <c r="V40" s="3"/>
       <c r="W40" s="3"/>
       <c r="X40" s="3"/>
@@ -3379,39 +3519,42 @@
       <c r="AG40" s="3"/>
       <c r="AH40" s="3"/>
       <c r="AI40" s="3"/>
-    </row>
-    <row r="41" spans="1:35">
+      <c r="AJ40" s="3"/>
+    </row>
+    <row r="41" spans="1:36">
       <c r="A41" s="3"/>
       <c r="B41" s="4" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="D41" s="4"/>
       <c r="E41" s="4"/>
       <c r="F41" s="4"/>
       <c r="G41" s="4"/>
       <c r="H41" s="4" t="s">
-        <v>95</v>
+        <v>101</v>
       </c>
       <c r="I41" s="4"/>
       <c r="J41" s="4"/>
       <c r="K41" s="4"/>
       <c r="L41" s="4"/>
       <c r="M41" s="4" t="s">
-        <v>101</v>
+        <v>107</v>
       </c>
       <c r="N41" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O41" s="4"/>
+      <c r="O41" s="4" t="s">
+        <v>108</v>
+      </c>
       <c r="P41" s="4"/>
       <c r="Q41" s="4"/>
       <c r="R41" s="4"/>
       <c r="S41" s="4"/>
       <c r="T41" s="4"/>
-      <c r="U41" s="3"/>
+      <c r="U41" s="4"/>
       <c r="V41" s="3"/>
       <c r="W41" s="3"/>
       <c r="X41" s="3"/>
@@ -3426,39 +3569,42 @@
       <c r="AG41" s="3"/>
       <c r="AH41" s="3"/>
       <c r="AI41" s="3"/>
-    </row>
-    <row r="42" spans="1:35">
+      <c r="AJ41" s="3"/>
+    </row>
+    <row r="42" spans="1:36">
       <c r="A42" s="3"/>
       <c r="B42" s="4" t="s">
-        <v>102</v>
+        <v>109</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="D42" s="4"/>
       <c r="E42" s="4"/>
       <c r="F42" s="4"/>
       <c r="G42" s="4"/>
       <c r="H42" s="4" t="s">
-        <v>95</v>
+        <v>101</v>
       </c>
       <c r="I42" s="4"/>
       <c r="J42" s="4"/>
       <c r="K42" s="4"/>
       <c r="L42" s="4"/>
       <c r="M42" s="4" t="s">
-        <v>101</v>
+        <v>107</v>
       </c>
       <c r="N42" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O42" s="4"/>
+      <c r="O42" s="4" t="s">
+        <v>108</v>
+      </c>
       <c r="P42" s="4"/>
       <c r="Q42" s="4"/>
       <c r="R42" s="4"/>
       <c r="S42" s="4"/>
       <c r="T42" s="4"/>
-      <c r="U42" s="3"/>
+      <c r="U42" s="4"/>
       <c r="V42" s="3"/>
       <c r="W42" s="3"/>
       <c r="X42" s="3"/>
@@ -3473,10 +3619,11 @@
       <c r="AG42" s="3"/>
       <c r="AH42" s="3"/>
       <c r="AI42" s="3"/>
-    </row>
-    <row r="43" spans="2:35">
+      <c r="AJ42" s="3"/>
+    </row>
+    <row r="43" spans="2:36">
       <c r="B43" s="2" t="s">
-        <v>103</v>
+        <v>110</v>
       </c>
       <c r="C43" s="2"/>
       <c r="D43" s="2"/>
@@ -3492,13 +3639,15 @@
       <c r="N43" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="O43" s="2"/>
+      <c r="O43" s="2" t="s">
+        <v>27</v>
+      </c>
       <c r="P43" s="2"/>
       <c r="Q43" s="2"/>
       <c r="R43" s="2"/>
       <c r="S43" s="2"/>
       <c r="T43" s="2"/>
-      <c r="Y43" s="3"/>
+      <c r="U43" s="2"/>
       <c r="Z43" s="3"/>
       <c r="AA43" s="3"/>
       <c r="AB43" s="3"/>
@@ -3509,54 +3658,57 @@
       <c r="AG43" s="3"/>
       <c r="AH43" s="3"/>
       <c r="AI43" s="3"/>
-    </row>
-    <row r="44" spans="2:35">
+      <c r="AJ43" s="3"/>
+    </row>
+    <row r="44" spans="2:36">
       <c r="B44" s="2" t="s">
-        <v>104</v>
+        <v>111</v>
       </c>
       <c r="C44" s="2" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="D44" s="2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E44" s="2" t="s">
         <v>15</v>
       </c>
       <c r="F44" s="2" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="G44" s="2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="H44" s="4" t="s">
-        <v>105</v>
+        <v>112</v>
       </c>
       <c r="I44" s="4" t="s">
-        <v>106</v>
+        <v>113</v>
       </c>
       <c r="J44" s="4" t="s">
-        <v>107</v>
+        <v>114</v>
       </c>
       <c r="K44" s="2" t="s">
-        <v>108</v>
+        <v>115</v>
       </c>
       <c r="L44" s="2" t="s">
-        <v>109</v>
+        <v>116</v>
       </c>
       <c r="M44" s="2" t="s">
-        <v>110</v>
+        <v>117</v>
       </c>
       <c r="N44" s="2" t="s">
-        <v>111</v>
-      </c>
-      <c r="O44" s="2"/>
+        <v>118</v>
+      </c>
+      <c r="O44" s="2" t="s">
+        <v>82</v>
+      </c>
       <c r="P44" s="2"/>
       <c r="Q44" s="2"/>
       <c r="R44" s="2"/>
       <c r="S44" s="2"/>
       <c r="T44" s="2"/>
-      <c r="Y44" s="3"/>
+      <c r="U44" s="2"/>
       <c r="Z44" s="3"/>
       <c r="AA44" s="3"/>
       <c r="AB44" s="3"/>
@@ -3567,8 +3719,9 @@
       <c r="AG44" s="3"/>
       <c r="AH44" s="3"/>
       <c r="AI44" s="3"/>
-    </row>
-    <row r="45" spans="1:35">
+      <c r="AJ44" s="3"/>
+    </row>
+    <row r="45" spans="1:36">
       <c r="A45" s="3"/>
       <c r="B45" s="4"/>
       <c r="C45" s="4"/>
@@ -3589,7 +3742,7 @@
       <c r="R45" s="4"/>
       <c r="S45" s="4"/>
       <c r="T45" s="4"/>
-      <c r="U45" s="3"/>
+      <c r="U45" s="4"/>
       <c r="V45" s="3"/>
       <c r="W45" s="3"/>
       <c r="X45" s="3"/>
@@ -3604,8 +3757,9 @@
       <c r="AG45" s="3"/>
       <c r="AH45" s="3"/>
       <c r="AI45" s="3"/>
-    </row>
-    <row r="46" s="1" customFormat="1" spans="1:35">
+      <c r="AJ45" s="3"/>
+    </row>
+    <row r="46" s="1" customFormat="1" spans="1:36">
       <c r="A46" s="3"/>
       <c r="B46" s="4"/>
       <c r="C46" s="4"/>
@@ -3626,7 +3780,7 @@
       <c r="R46" s="4"/>
       <c r="S46" s="4"/>
       <c r="T46" s="4"/>
-      <c r="U46" s="3"/>
+      <c r="U46" s="4"/>
       <c r="V46" s="3"/>
       <c r="W46" s="3"/>
       <c r="X46" s="3"/>
@@ -3641,8 +3795,9 @@
       <c r="AG46" s="3"/>
       <c r="AH46" s="3"/>
       <c r="AI46" s="3"/>
-    </row>
-    <row r="47" s="1" customFormat="1" spans="1:35">
+      <c r="AJ46" s="3"/>
+    </row>
+    <row r="47" s="1" customFormat="1" spans="1:36">
       <c r="A47" s="3"/>
       <c r="B47" s="4"/>
       <c r="C47" s="4"/>
@@ -3663,7 +3818,7 @@
       <c r="R47" s="4"/>
       <c r="S47" s="4"/>
       <c r="T47" s="4"/>
-      <c r="U47" s="3"/>
+      <c r="U47" s="4"/>
       <c r="V47" s="3"/>
       <c r="W47" s="3"/>
       <c r="X47" s="3"/>
@@ -3678,8 +3833,9 @@
       <c r="AG47" s="3"/>
       <c r="AH47" s="3"/>
       <c r="AI47" s="3"/>
-    </row>
-    <row r="48" spans="1:35">
+      <c r="AJ47" s="3"/>
+    </row>
+    <row r="48" spans="1:36">
       <c r="A48" s="3"/>
       <c r="B48" s="4"/>
       <c r="C48" s="4"/>
@@ -3700,7 +3856,7 @@
       <c r="R48" s="4"/>
       <c r="S48" s="4"/>
       <c r="T48" s="4"/>
-      <c r="U48" s="3"/>
+      <c r="U48" s="4"/>
       <c r="V48" s="3"/>
       <c r="W48" s="3"/>
       <c r="X48" s="3"/>
@@ -3715,8 +3871,9 @@
       <c r="AG48" s="3"/>
       <c r="AH48" s="3"/>
       <c r="AI48" s="3"/>
-    </row>
-    <row r="49" spans="1:35">
+      <c r="AJ48" s="3"/>
+    </row>
+    <row r="49" spans="1:36">
       <c r="A49" s="3"/>
       <c r="B49" s="4"/>
       <c r="C49" s="4"/>
@@ -3737,7 +3894,7 @@
       <c r="R49" s="4"/>
       <c r="S49" s="4"/>
       <c r="T49" s="4"/>
-      <c r="U49" s="3"/>
+      <c r="U49" s="4"/>
       <c r="V49" s="3"/>
       <c r="W49" s="3"/>
       <c r="X49" s="3"/>
@@ -3752,8 +3909,9 @@
       <c r="AG49" s="3"/>
       <c r="AH49" s="3"/>
       <c r="AI49" s="3"/>
-    </row>
-    <row r="50" spans="1:35">
+      <c r="AJ49" s="3"/>
+    </row>
+    <row r="50" spans="1:36">
       <c r="A50" s="3"/>
       <c r="B50" s="4"/>
       <c r="C50" s="4"/>
@@ -3774,7 +3932,7 @@
       <c r="R50" s="4"/>
       <c r="S50" s="4"/>
       <c r="T50" s="4"/>
-      <c r="U50" s="3"/>
+      <c r="U50" s="4"/>
       <c r="V50" s="3"/>
       <c r="W50" s="3"/>
       <c r="X50" s="3"/>
@@ -3789,8 +3947,9 @@
       <c r="AG50" s="3"/>
       <c r="AH50" s="3"/>
       <c r="AI50" s="3"/>
-    </row>
-    <row r="51" spans="1:35">
+      <c r="AJ50" s="3"/>
+    </row>
+    <row r="51" spans="1:36">
       <c r="A51" s="3"/>
       <c r="B51" s="4"/>
       <c r="C51" s="4"/>
@@ -3811,7 +3970,7 @@
       <c r="R51" s="4"/>
       <c r="S51" s="4"/>
       <c r="T51" s="4"/>
-      <c r="U51" s="3"/>
+      <c r="U51" s="4"/>
       <c r="V51" s="3"/>
       <c r="W51" s="3"/>
       <c r="X51" s="3"/>
@@ -3826,8 +3985,9 @@
       <c r="AG51" s="3"/>
       <c r="AH51" s="3"/>
       <c r="AI51" s="3"/>
-    </row>
-    <row r="52" spans="1:35">
+      <c r="AJ51" s="3"/>
+    </row>
+    <row r="52" spans="1:36">
       <c r="A52" s="3"/>
       <c r="B52" s="4"/>
       <c r="C52" s="4"/>
@@ -3848,7 +4008,7 @@
       <c r="R52" s="4"/>
       <c r="S52" s="4"/>
       <c r="T52" s="4"/>
-      <c r="U52" s="3"/>
+      <c r="U52" s="4"/>
       <c r="V52" s="3"/>
       <c r="W52" s="3"/>
       <c r="X52" s="3"/>
@@ -3863,8 +4023,9 @@
       <c r="AG52" s="3"/>
       <c r="AH52" s="3"/>
       <c r="AI52" s="3"/>
-    </row>
-    <row r="53" spans="1:35">
+      <c r="AJ52" s="3"/>
+    </row>
+    <row r="53" spans="1:36">
       <c r="A53" s="3"/>
       <c r="B53" s="4"/>
       <c r="C53" s="4"/>
@@ -3885,7 +4046,7 @@
       <c r="R53" s="4"/>
       <c r="S53" s="4"/>
       <c r="T53" s="4"/>
-      <c r="U53" s="3"/>
+      <c r="U53" s="4"/>
       <c r="V53" s="3"/>
       <c r="W53" s="3"/>
       <c r="X53" s="3"/>
@@ -3900,8 +4061,9 @@
       <c r="AG53" s="3"/>
       <c r="AH53" s="3"/>
       <c r="AI53" s="3"/>
-    </row>
-    <row r="54" spans="1:35">
+      <c r="AJ53" s="3"/>
+    </row>
+    <row r="54" spans="1:36">
       <c r="A54" s="3"/>
       <c r="B54" s="4"/>
       <c r="C54" s="4"/>
@@ -3922,7 +4084,7 @@
       <c r="R54" s="4"/>
       <c r="S54" s="4"/>
       <c r="T54" s="4"/>
-      <c r="U54" s="3"/>
+      <c r="U54" s="4"/>
       <c r="V54" s="3"/>
       <c r="W54" s="3"/>
       <c r="X54" s="3"/>
@@ -3937,8 +4099,9 @@
       <c r="AG54" s="3"/>
       <c r="AH54" s="3"/>
       <c r="AI54" s="3"/>
-    </row>
-    <row r="55" spans="1:35">
+      <c r="AJ54" s="3"/>
+    </row>
+    <row r="55" spans="1:36">
       <c r="A55" s="3"/>
       <c r="B55" s="4"/>
       <c r="C55" s="4"/>
@@ -3959,7 +4122,7 @@
       <c r="R55" s="4"/>
       <c r="S55" s="4"/>
       <c r="T55" s="4"/>
-      <c r="U55" s="3"/>
+      <c r="U55" s="4"/>
       <c r="V55" s="3"/>
       <c r="W55" s="3"/>
       <c r="X55" s="3"/>
@@ -3974,8 +4137,9 @@
       <c r="AG55" s="3"/>
       <c r="AH55" s="3"/>
       <c r="AI55" s="3"/>
-    </row>
-    <row r="56" spans="1:35">
+      <c r="AJ55" s="3"/>
+    </row>
+    <row r="56" spans="1:36">
       <c r="A56" s="3"/>
       <c r="B56" s="4"/>
       <c r="C56" s="4"/>
@@ -3996,7 +4160,7 @@
       <c r="R56" s="4"/>
       <c r="S56" s="4"/>
       <c r="T56" s="4"/>
-      <c r="U56" s="3"/>
+      <c r="U56" s="4"/>
       <c r="V56" s="3"/>
       <c r="W56" s="3"/>
       <c r="X56" s="3"/>
@@ -4011,8 +4175,9 @@
       <c r="AG56" s="3"/>
       <c r="AH56" s="3"/>
       <c r="AI56" s="3"/>
-    </row>
-    <row r="57" spans="1:35">
+      <c r="AJ56" s="3"/>
+    </row>
+    <row r="57" spans="1:36">
       <c r="A57" s="3"/>
       <c r="B57" s="4"/>
       <c r="C57" s="4"/>
@@ -4033,7 +4198,7 @@
       <c r="R57" s="4"/>
       <c r="S57" s="4"/>
       <c r="T57" s="4"/>
-      <c r="U57" s="3"/>
+      <c r="U57" s="4"/>
       <c r="V57" s="3"/>
       <c r="W57" s="3"/>
       <c r="X57" s="3"/>
@@ -4048,8 +4213,9 @@
       <c r="AG57" s="3"/>
       <c r="AH57" s="3"/>
       <c r="AI57" s="3"/>
-    </row>
-    <row r="58" spans="1:35">
+      <c r="AJ57" s="3"/>
+    </row>
+    <row r="58" spans="1:36">
       <c r="A58" s="3"/>
       <c r="B58" s="4"/>
       <c r="C58" s="4"/>
@@ -4070,7 +4236,7 @@
       <c r="R58" s="4"/>
       <c r="S58" s="4"/>
       <c r="T58" s="4"/>
-      <c r="U58" s="3"/>
+      <c r="U58" s="4"/>
       <c r="V58" s="3"/>
       <c r="W58" s="3"/>
       <c r="X58" s="3"/>
@@ -4085,8 +4251,9 @@
       <c r="AG58" s="3"/>
       <c r="AH58" s="3"/>
       <c r="AI58" s="3"/>
-    </row>
-    <row r="59" spans="1:35">
+      <c r="AJ58" s="3"/>
+    </row>
+    <row r="59" spans="1:36">
       <c r="A59" s="3"/>
       <c r="B59" s="4"/>
       <c r="C59" s="4"/>
@@ -4107,7 +4274,7 @@
       <c r="R59" s="4"/>
       <c r="S59" s="4"/>
       <c r="T59" s="4"/>
-      <c r="U59" s="3"/>
+      <c r="U59" s="4"/>
       <c r="V59" s="3"/>
       <c r="W59" s="3"/>
       <c r="X59" s="3"/>
@@ -4122,8 +4289,9 @@
       <c r="AG59" s="3"/>
       <c r="AH59" s="3"/>
       <c r="AI59" s="3"/>
-    </row>
-    <row r="60" spans="1:35">
+      <c r="AJ59" s="3"/>
+    </row>
+    <row r="60" spans="1:36">
       <c r="A60" s="3"/>
       <c r="B60" s="4"/>
       <c r="C60" s="4"/>
@@ -4144,7 +4312,7 @@
       <c r="R60" s="4"/>
       <c r="S60" s="4"/>
       <c r="T60" s="4"/>
-      <c r="U60" s="3"/>
+      <c r="U60" s="4"/>
       <c r="V60" s="3"/>
       <c r="W60" s="3"/>
       <c r="X60" s="3"/>
@@ -4159,8 +4327,9 @@
       <c r="AG60" s="3"/>
       <c r="AH60" s="3"/>
       <c r="AI60" s="3"/>
-    </row>
-    <row r="61" spans="1:35">
+      <c r="AJ60" s="3"/>
+    </row>
+    <row r="61" spans="1:36">
       <c r="A61" s="3"/>
       <c r="B61" s="4"/>
       <c r="C61" s="4"/>
@@ -4181,7 +4350,7 @@
       <c r="R61" s="4"/>
       <c r="S61" s="4"/>
       <c r="T61" s="4"/>
-      <c r="U61" s="3"/>
+      <c r="U61" s="4"/>
       <c r="V61" s="3"/>
       <c r="W61" s="3"/>
       <c r="X61" s="3"/>
@@ -4196,8 +4365,9 @@
       <c r="AG61" s="3"/>
       <c r="AH61" s="3"/>
       <c r="AI61" s="3"/>
-    </row>
-    <row r="62" spans="1:35">
+      <c r="AJ61" s="3"/>
+    </row>
+    <row r="62" spans="1:36">
       <c r="A62" s="3"/>
       <c r="B62" s="4"/>
       <c r="C62" s="4"/>
@@ -4218,7 +4388,7 @@
       <c r="R62" s="4"/>
       <c r="S62" s="4"/>
       <c r="T62" s="4"/>
-      <c r="U62" s="3"/>
+      <c r="U62" s="4"/>
       <c r="V62" s="3"/>
       <c r="W62" s="3"/>
       <c r="X62" s="3"/>
@@ -4233,8 +4403,9 @@
       <c r="AG62" s="3"/>
       <c r="AH62" s="3"/>
       <c r="AI62" s="3"/>
-    </row>
-    <row r="63" spans="1:35">
+      <c r="AJ62" s="3"/>
+    </row>
+    <row r="63" spans="1:36">
       <c r="A63" s="3"/>
       <c r="B63" s="4"/>
       <c r="C63" s="4"/>
@@ -4255,7 +4426,7 @@
       <c r="R63" s="4"/>
       <c r="S63" s="4"/>
       <c r="T63" s="4"/>
-      <c r="U63" s="3"/>
+      <c r="U63" s="4"/>
       <c r="V63" s="3"/>
       <c r="W63" s="3"/>
       <c r="X63" s="3"/>
@@ -4270,8 +4441,9 @@
       <c r="AG63" s="3"/>
       <c r="AH63" s="3"/>
       <c r="AI63" s="3"/>
-    </row>
-    <row r="64" spans="1:35">
+      <c r="AJ63" s="3"/>
+    </row>
+    <row r="64" spans="1:36">
       <c r="A64" s="3"/>
       <c r="B64" s="4"/>
       <c r="C64" s="4"/>
@@ -4292,7 +4464,7 @@
       <c r="R64" s="4"/>
       <c r="S64" s="4"/>
       <c r="T64" s="4"/>
-      <c r="U64" s="3"/>
+      <c r="U64" s="4"/>
       <c r="V64" s="3"/>
       <c r="W64" s="3"/>
       <c r="X64" s="3"/>
@@ -4307,8 +4479,9 @@
       <c r="AG64" s="3"/>
       <c r="AH64" s="3"/>
       <c r="AI64" s="3"/>
-    </row>
-    <row r="65" spans="1:35">
+      <c r="AJ64" s="3"/>
+    </row>
+    <row r="65" spans="1:36">
       <c r="A65" s="3"/>
       <c r="B65" s="4"/>
       <c r="C65" s="4"/>
@@ -4329,7 +4502,7 @@
       <c r="R65" s="4"/>
       <c r="S65" s="4"/>
       <c r="T65" s="4"/>
-      <c r="U65" s="3"/>
+      <c r="U65" s="4"/>
       <c r="V65" s="3"/>
       <c r="W65" s="3"/>
       <c r="X65" s="3"/>
@@ -4344,8 +4517,9 @@
       <c r="AG65" s="3"/>
       <c r="AH65" s="3"/>
       <c r="AI65" s="3"/>
-    </row>
-    <row r="66" spans="1:35">
+      <c r="AJ65" s="3"/>
+    </row>
+    <row r="66" spans="1:36">
       <c r="A66" s="3"/>
       <c r="B66" s="4"/>
       <c r="C66" s="4"/>
@@ -4366,7 +4540,7 @@
       <c r="R66" s="4"/>
       <c r="S66" s="4"/>
       <c r="T66" s="4"/>
-      <c r="U66" s="3"/>
+      <c r="U66" s="4"/>
       <c r="V66" s="3"/>
       <c r="W66" s="3"/>
       <c r="X66" s="3"/>
@@ -4381,8 +4555,9 @@
       <c r="AG66" s="3"/>
       <c r="AH66" s="3"/>
       <c r="AI66" s="3"/>
-    </row>
-    <row r="67" spans="1:35">
+      <c r="AJ66" s="3"/>
+    </row>
+    <row r="67" spans="1:36">
       <c r="A67" s="3"/>
       <c r="B67" s="4"/>
       <c r="C67" s="4"/>
@@ -4403,7 +4578,7 @@
       <c r="R67" s="4"/>
       <c r="S67" s="4"/>
       <c r="T67" s="4"/>
-      <c r="U67" s="3"/>
+      <c r="U67" s="4"/>
       <c r="V67" s="3"/>
       <c r="W67" s="3"/>
       <c r="X67" s="3"/>
@@ -4418,8 +4593,9 @@
       <c r="AG67" s="3"/>
       <c r="AH67" s="3"/>
       <c r="AI67" s="3"/>
-    </row>
-    <row r="68" spans="1:35">
+      <c r="AJ67" s="3"/>
+    </row>
+    <row r="68" spans="1:36">
       <c r="A68" s="3"/>
       <c r="B68" s="4"/>
       <c r="C68" s="4"/>
@@ -4440,7 +4616,7 @@
       <c r="R68" s="4"/>
       <c r="S68" s="4"/>
       <c r="T68" s="4"/>
-      <c r="U68" s="3"/>
+      <c r="U68" s="4"/>
       <c r="V68" s="3"/>
       <c r="W68" s="3"/>
       <c r="X68" s="3"/>
@@ -4455,8 +4631,9 @@
       <c r="AG68" s="3"/>
       <c r="AH68" s="3"/>
       <c r="AI68" s="3"/>
-    </row>
-    <row r="69" spans="1:35">
+      <c r="AJ68" s="3"/>
+    </row>
+    <row r="69" spans="1:36">
       <c r="A69" s="3"/>
       <c r="B69" s="4"/>
       <c r="C69" s="4"/>
@@ -4477,7 +4654,7 @@
       <c r="R69" s="4"/>
       <c r="S69" s="4"/>
       <c r="T69" s="4"/>
-      <c r="U69" s="3"/>
+      <c r="U69" s="4"/>
       <c r="V69" s="3"/>
       <c r="W69" s="3"/>
       <c r="X69" s="3"/>
@@ -4492,8 +4669,9 @@
       <c r="AG69" s="3"/>
       <c r="AH69" s="3"/>
       <c r="AI69" s="3"/>
-    </row>
-    <row r="70" spans="1:35">
+      <c r="AJ69" s="3"/>
+    </row>
+    <row r="70" spans="1:36">
       <c r="A70" s="3"/>
       <c r="B70" s="4"/>
       <c r="C70" s="4"/>
@@ -4514,7 +4692,7 @@
       <c r="R70" s="4"/>
       <c r="S70" s="4"/>
       <c r="T70" s="4"/>
-      <c r="U70" s="3"/>
+      <c r="U70" s="4"/>
       <c r="V70" s="3"/>
       <c r="W70" s="3"/>
       <c r="X70" s="3"/>
@@ -4529,8 +4707,9 @@
       <c r="AG70" s="3"/>
       <c r="AH70" s="3"/>
       <c r="AI70" s="3"/>
-    </row>
-    <row r="71" spans="1:35">
+      <c r="AJ70" s="3"/>
+    </row>
+    <row r="71" spans="1:36">
       <c r="A71" s="3"/>
       <c r="B71" s="4"/>
       <c r="C71" s="4"/>
@@ -4551,7 +4730,7 @@
       <c r="R71" s="4"/>
       <c r="S71" s="4"/>
       <c r="T71" s="4"/>
-      <c r="U71" s="3"/>
+      <c r="U71" s="4"/>
       <c r="V71" s="3"/>
       <c r="W71" s="3"/>
       <c r="X71" s="3"/>
@@ -4566,8 +4745,9 @@
       <c r="AG71" s="3"/>
       <c r="AH71" s="3"/>
       <c r="AI71" s="3"/>
-    </row>
-    <row r="72" spans="1:35">
+      <c r="AJ71" s="3"/>
+    </row>
+    <row r="72" spans="1:36">
       <c r="A72" s="3"/>
       <c r="B72" s="4"/>
       <c r="C72" s="4"/>
@@ -4588,7 +4768,7 @@
       <c r="R72" s="4"/>
       <c r="S72" s="4"/>
       <c r="T72" s="4"/>
-      <c r="U72" s="3"/>
+      <c r="U72" s="4"/>
       <c r="V72" s="3"/>
       <c r="W72" s="3"/>
       <c r="X72" s="3"/>
@@ -4603,8 +4783,9 @@
       <c r="AG72" s="3"/>
       <c r="AH72" s="3"/>
       <c r="AI72" s="3"/>
-    </row>
-    <row r="73" spans="1:35">
+      <c r="AJ72" s="3"/>
+    </row>
+    <row r="73" spans="1:36">
       <c r="A73" s="3"/>
       <c r="B73" s="4"/>
       <c r="C73" s="4"/>
@@ -4625,7 +4806,7 @@
       <c r="R73" s="4"/>
       <c r="S73" s="4"/>
       <c r="T73" s="4"/>
-      <c r="U73" s="3"/>
+      <c r="U73" s="4"/>
       <c r="V73" s="3"/>
       <c r="W73" s="3"/>
       <c r="X73" s="3"/>
@@ -4640,8 +4821,9 @@
       <c r="AG73" s="3"/>
       <c r="AH73" s="3"/>
       <c r="AI73" s="3"/>
-    </row>
-    <row r="74" spans="1:35">
+      <c r="AJ73" s="3"/>
+    </row>
+    <row r="74" spans="1:36">
       <c r="A74" s="3"/>
       <c r="B74" s="4"/>
       <c r="C74" s="4"/>
@@ -4662,7 +4844,7 @@
       <c r="R74" s="4"/>
       <c r="S74" s="4"/>
       <c r="T74" s="4"/>
-      <c r="U74" s="3"/>
+      <c r="U74" s="4"/>
       <c r="V74" s="3"/>
       <c r="W74" s="3"/>
       <c r="X74" s="3"/>
@@ -4677,8 +4859,9 @@
       <c r="AG74" s="3"/>
       <c r="AH74" s="3"/>
       <c r="AI74" s="3"/>
-    </row>
-    <row r="75" spans="1:35">
+      <c r="AJ74" s="3"/>
+    </row>
+    <row r="75" spans="1:36">
       <c r="A75" s="3"/>
       <c r="B75" s="4"/>
       <c r="C75" s="4"/>
@@ -4699,7 +4882,7 @@
       <c r="R75" s="4"/>
       <c r="S75" s="4"/>
       <c r="T75" s="4"/>
-      <c r="U75" s="3"/>
+      <c r="U75" s="4"/>
       <c r="V75" s="3"/>
       <c r="W75" s="3"/>
       <c r="X75" s="3"/>
@@ -4714,8 +4897,9 @@
       <c r="AG75" s="3"/>
       <c r="AH75" s="3"/>
       <c r="AI75" s="3"/>
-    </row>
-    <row r="76" spans="1:35">
+      <c r="AJ75" s="3"/>
+    </row>
+    <row r="76" spans="1:36">
       <c r="A76" s="3"/>
       <c r="B76" s="4"/>
       <c r="C76" s="4"/>
@@ -4736,7 +4920,7 @@
       <c r="R76" s="4"/>
       <c r="S76" s="4"/>
       <c r="T76" s="4"/>
-      <c r="U76" s="3"/>
+      <c r="U76" s="4"/>
       <c r="V76" s="3"/>
       <c r="W76" s="3"/>
       <c r="X76" s="3"/>
@@ -4751,8 +4935,9 @@
       <c r="AG76" s="3"/>
       <c r="AH76" s="3"/>
       <c r="AI76" s="3"/>
-    </row>
-    <row r="77" spans="1:35">
+      <c r="AJ76" s="3"/>
+    </row>
+    <row r="77" spans="1:36">
       <c r="A77" s="3"/>
       <c r="B77" s="4"/>
       <c r="C77" s="4"/>
@@ -4773,7 +4958,7 @@
       <c r="R77" s="4"/>
       <c r="S77" s="4"/>
       <c r="T77" s="4"/>
-      <c r="U77" s="3"/>
+      <c r="U77" s="4"/>
       <c r="V77" s="3"/>
       <c r="W77" s="3"/>
       <c r="X77" s="3"/>
@@ -4788,8 +4973,9 @@
       <c r="AG77" s="3"/>
       <c r="AH77" s="3"/>
       <c r="AI77" s="3"/>
-    </row>
-    <row r="78" spans="1:35">
+      <c r="AJ77" s="3"/>
+    </row>
+    <row r="78" spans="1:36">
       <c r="A78" s="3"/>
       <c r="B78" s="4"/>
       <c r="C78" s="4"/>
@@ -4810,7 +4996,7 @@
       <c r="R78" s="4"/>
       <c r="S78" s="4"/>
       <c r="T78" s="4"/>
-      <c r="U78" s="3"/>
+      <c r="U78" s="4"/>
       <c r="V78" s="3"/>
       <c r="W78" s="3"/>
       <c r="X78" s="3"/>
@@ -4825,194 +5011,195 @@
       <c r="AG78" s="3"/>
       <c r="AH78" s="3"/>
       <c r="AI78" s="3"/>
-    </row>
-    <row r="86" spans="1:24">
+      <c r="AJ78" s="3"/>
+    </row>
+    <row r="86" spans="1:25">
       <c r="A86" s="2"/>
       <c r="B86" s="2"/>
       <c r="C86" s="2"/>
       <c r="D86" s="2"/>
-      <c r="S86" s="2"/>
-      <c r="U86" s="2"/>
+      <c r="T86" s="2"/>
       <c r="V86" s="2"/>
       <c r="W86" s="2"/>
       <c r="X86" s="2"/>
-    </row>
-    <row r="87" spans="1:24">
+      <c r="Y86" s="2"/>
+    </row>
+    <row r="87" spans="1:25">
       <c r="A87" s="2"/>
       <c r="B87" s="2"/>
       <c r="C87" s="2"/>
       <c r="D87" s="2"/>
       <c r="E87" s="2"/>
-      <c r="S87" s="2"/>
       <c r="T87" s="2"/>
       <c r="U87" s="2"/>
       <c r="V87" s="2"/>
       <c r="W87" s="2"/>
       <c r="X87" s="2"/>
-    </row>
-    <row r="88" spans="1:24">
+      <c r="Y87" s="2"/>
+    </row>
+    <row r="88" spans="1:25">
       <c r="A88" s="2"/>
       <c r="B88" s="2"/>
       <c r="C88" s="2"/>
       <c r="D88" s="2"/>
-      <c r="S88" s="2"/>
       <c r="T88" s="2"/>
       <c r="U88" s="2"/>
       <c r="V88" s="2"/>
       <c r="W88" s="2"/>
       <c r="X88" s="2"/>
-    </row>
-    <row r="89" spans="1:24">
+      <c r="Y88" s="2"/>
+    </row>
+    <row r="89" spans="1:25">
       <c r="A89" s="2"/>
       <c r="B89" s="2"/>
       <c r="C89" s="2"/>
       <c r="D89" s="2"/>
-      <c r="S89" s="2"/>
       <c r="T89" s="2"/>
       <c r="U89" s="2"/>
       <c r="V89" s="2"/>
       <c r="W89" s="2"/>
       <c r="X89" s="2"/>
-    </row>
-    <row r="90" spans="1:24">
+      <c r="Y89" s="2"/>
+    </row>
+    <row r="90" spans="1:25">
       <c r="A90" s="2"/>
       <c r="B90" s="2"/>
       <c r="C90" s="2"/>
       <c r="D90" s="2"/>
-      <c r="S90" s="2"/>
       <c r="T90" s="2"/>
       <c r="U90" s="2"/>
       <c r="V90" s="2"/>
       <c r="W90" s="2"/>
       <c r="X90" s="2"/>
-    </row>
-    <row r="91" spans="1:24">
+      <c r="Y90" s="2"/>
+    </row>
+    <row r="91" spans="1:25">
       <c r="A91" s="2"/>
       <c r="B91" s="2"/>
       <c r="C91" s="2"/>
       <c r="D91" s="2"/>
-      <c r="S91" s="2"/>
       <c r="T91" s="2"/>
       <c r="U91" s="2"/>
       <c r="V91" s="2"/>
       <c r="W91" s="2"/>
       <c r="X91" s="2"/>
-    </row>
-    <row r="92" spans="1:24">
+      <c r="Y91" s="2"/>
+    </row>
+    <row r="92" spans="1:25">
       <c r="A92" s="2"/>
       <c r="B92" s="2"/>
       <c r="C92" s="2"/>
       <c r="D92" s="2"/>
-      <c r="S92" s="2"/>
       <c r="T92" s="2"/>
       <c r="U92" s="2"/>
       <c r="V92" s="2"/>
       <c r="W92" s="2"/>
       <c r="X92" s="2"/>
-    </row>
-    <row r="93" spans="1:24">
+      <c r="Y92" s="2"/>
+    </row>
+    <row r="93" spans="1:25">
       <c r="A93" s="2"/>
       <c r="B93" s="2"/>
       <c r="C93" s="2"/>
       <c r="D93" s="2"/>
-      <c r="S93" s="2"/>
       <c r="T93" s="2"/>
       <c r="U93" s="2"/>
       <c r="V93" s="2"/>
       <c r="W93" s="2"/>
       <c r="X93" s="2"/>
-    </row>
-    <row r="94" spans="1:24">
+      <c r="Y93" s="2"/>
+    </row>
+    <row r="94" spans="1:25">
       <c r="A94" s="2"/>
       <c r="B94" s="2"/>
       <c r="C94" s="2"/>
       <c r="D94" s="2"/>
-      <c r="S94" s="2"/>
       <c r="T94" s="2"/>
       <c r="U94" s="2"/>
       <c r="V94" s="2"/>
       <c r="W94" s="2"/>
       <c r="X94" s="2"/>
-    </row>
-    <row r="95" spans="1:24">
+      <c r="Y94" s="2"/>
+    </row>
+    <row r="95" spans="1:25">
       <c r="A95" s="2"/>
       <c r="B95" s="2"/>
       <c r="C95" s="2"/>
       <c r="D95" s="2"/>
-      <c r="S95" s="2"/>
       <c r="T95" s="2"/>
       <c r="U95" s="2"/>
       <c r="V95" s="2"/>
       <c r="W95" s="2"/>
       <c r="X95" s="2"/>
-    </row>
-    <row r="96" spans="1:24">
+      <c r="Y95" s="2"/>
+    </row>
+    <row r="96" spans="1:25">
       <c r="A96" s="2"/>
       <c r="B96" s="2"/>
       <c r="C96" s="2"/>
       <c r="D96" s="2"/>
-      <c r="S96" s="2"/>
       <c r="T96" s="2"/>
       <c r="U96" s="2"/>
       <c r="V96" s="2"/>
       <c r="W96" s="2"/>
       <c r="X96" s="2"/>
-    </row>
-    <row r="97" spans="1:24">
+      <c r="Y96" s="2"/>
+    </row>
+    <row r="97" spans="1:25">
       <c r="A97" s="2"/>
       <c r="B97" s="2"/>
       <c r="C97" s="2"/>
       <c r="D97" s="2"/>
-      <c r="S97" s="2"/>
       <c r="T97" s="2"/>
       <c r="U97" s="2"/>
       <c r="V97" s="2"/>
       <c r="W97" s="2"/>
       <c r="X97" s="2"/>
-    </row>
-    <row r="98" spans="1:24">
+      <c r="Y97" s="2"/>
+    </row>
+    <row r="98" spans="1:25">
       <c r="A98" s="2"/>
       <c r="B98" s="2"/>
       <c r="C98" s="2"/>
       <c r="D98" s="2"/>
-      <c r="S98" s="2"/>
       <c r="T98" s="2"/>
       <c r="U98" s="2"/>
       <c r="V98" s="2"/>
       <c r="W98" s="2"/>
       <c r="X98" s="2"/>
-    </row>
-    <row r="99" spans="1:24">
+      <c r="Y98" s="2"/>
+    </row>
+    <row r="99" spans="1:25">
       <c r="A99" s="2"/>
       <c r="B99" s="2"/>
       <c r="C99" s="2"/>
       <c r="D99" s="2"/>
-      <c r="S99" s="2"/>
       <c r="T99" s="2"/>
       <c r="U99" s="2"/>
       <c r="V99" s="2"/>
       <c r="W99" s="2"/>
       <c r="X99" s="2"/>
+      <c r="Y99" s="2"/>
     </row>
   </sheetData>
-  <dataValidations count="13">
+  <dataValidations count="14">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="O2:O1048576">
+      <formula1>"R_TYPE,I_TYPE,S_TYPE,B_TYPE,U_TYPE,J_TYPE,ICSR_TYPE,FENCE_TYPE,N_TYPE"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="M29 M30 M31 M39 M40 M41 M42 M43 M2:M28 M32:M38 M44:M1048576">
+      <formula1>"CSR_W,CSR_S,CSR_C,CSR_P,CSR_XX"</formula1>
+    </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H29 H30 H31 H40 H41 H42 H43 H10:H28 H32:H39 H44:H1048576">
       <formula1>"WB_ALU,WB_MEM,WB_PC4,WB_XX,WB_CSR"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F6 F15 F18 F19 F20 F21 F24 F25 F26 F27 F28 F29 F30 F31 F32 F33 F36 F37 F38 F39 F40 F41 F42 F43 F2:F5 F7:F14 F16:F17 F22:F23 F34:F35 F44:F1048576">
-      <formula1>"ALU_ADD,ALU_SUB,ALU_AND,ALU_OR,ALU_XOR,ALU_SLL,ALU_SRL,ALU_SLT,ALU_SLTU,ALU_COPY_A,ALU_COPY_B,ALU_SRA"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L5 L6 L7 L10 L11 L14 L15 L16 L17 L18 L19 L20 L21 L22 L23 L24 L25 L26 L27 L28 L29 L30 L31 L32 L33 L34 L35 L36 L37 L38 L39 L40 L41 L42 L43 L2:L4 L8:L9 L12:L13 L44:L1048576">
-      <formula1>"BR_EQ,BR_NE,BR_LTU,BR_GE,BR_GEU,BR_LT,BR_XX"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C29 C30 C31 C43 C2:C28 C32:C42 C44:C1048576">
       <formula1>"PC_4,PC_0,PC_ALU,PC_CSR"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="N4 N5 N6 N7 N8 N9 N10 N11 N12 N13 N14 N15 N16 N17 N18 N19 N20 N21 N22 N23 N24 N25 N26 N27 N28 N29 N30 N31 N32 N33 N34 N35 N36 N37 N38 N39 N40 N41 N42 N43 N2:N3 N44:N1048576">
-      <formula1>"INST_VALID,INST_INVALID"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E4 E5 E6 E7 E8 E9 E10 E11 E12 E13 E14 E15 E16 E17 E18 E19 E20 E21 E22 E23 E24 E25 E26 E27 E28 E29 E30 E31 E32 E33 E34 E35 E36 E37 E38 E39 E40 E41 E42 E43 E2:E3 E44:E1048576">
+      <formula1>"B_IMM,B_RS2"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D4 D5 D6 D7 D8 D9 D10 D11 D12 D13 D14 D15 D16 D17 D18 D19 D20 D21 D22 D23 D24 D25 D26 D27 D28 D29 D30 D31 D32 D33 D34 D35 D36 D37 D38 D39 D40 D41 D42 D43 D2:D3 D44:D1048576">
-      <formula1>"A_PC,A_RS1"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G4 G5 G6 G7 G8 G9 G10 G11 G12 G13 G14 G15 G16 G17 G18 G19 G20 G21 G22 G23 G24 G25 G26 G27 G28 G29 G30 G31 G32 G33 G34 G35 G36 G37 G38 G39 G40 G41 G42 G43 G2:G3 G44:G1048576">
+      <formula1>"IMM_I,IMM_J,IMM_U,IMM_S,IMM_B"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J5 J6 J7 J8 J9 J10 J11 J12 J13 J14 J15 J16 J17 J18 J19 J20 J21 J22 J23 J24 J25 J26 J27 J28 J29 J30 J31 J32 J33 J34 J35 J36 J37 J38 J39 J40 J41 J42 J43 J2:J4 J44:J1048576">
       <formula1>"ST_SW,ST_SH,ST_SB,ST_XX"</formula1>
@@ -5020,20 +5207,23 @@
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H5 H6 H7 H8 H9 H2:H4">
       <formula1>"WB_ALU,WB_MEM,WB_PC4,WB_XX"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K4 K5 K6 K7 K8 K9 K10 K11 K12 K13 K14 K15 K16 K17 K18 K19 K20 K21 K22 K23 K24 K25 K26 K27 K28 K29 K30 K31 K32 K33 K34 K35 K36 K37 K38 K39 K40 K41 K42 K43 K2:K3 K44:K1048576">
-      <formula1>"MASK_XX,MASK_B,MASK_H,MASK_W,MASK_D"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L5 L6 L7 L10 L11 L14 L15 L16 L17 L18 L19 L20 L21 L22 L23 L24 L25 L26 L27 L28 L29 L30 L31 L32 L33 L34 L35 L36 L37 L38 L39 L40 L41 L42 L43 L2:L4 L8:L9 L12:L13 L44:L1048576">
+      <formula1>"BR_EQ,BR_NE,BR_LTU,BR_GE,BR_GEU,BR_LT,BR_XX"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E4 E5 E6 E7 E8 E9 E10 E11 E12 E13 E14 E15 E16 E17 E18 E19 E20 E21 E22 E23 E24 E25 E26 E27 E28 E29 E30 E31 E32 E33 E34 E35 E36 E37 E38 E39 E40 E41 E42 E43 E2:E3 E44:E1048576">
-      <formula1>"B_IMM,B_RS2"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="M29 M30 M31 M39 M40 M41 M42 M43 M2:M28 M32:M38 M44:M1048576">
-      <formula1>"CSR_W,CSR_S,CSR_C,CSR_P,CSR_XX"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="N4 N5 N6 N7 N8 N9 N10 N11 N12 N13 N14 N15 N16 N17 N18 N19 N20 N21 N22 N23 N24 N25 N26 N27 N28 N29 N30 N31 N32 N33 N34 N35 N36 N37 N38 N39 N40 N41 N42 N43 N2:N3 N44:N1048576">
+      <formula1>"INST_VALID,INST_INVALID"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I4 I5 I6 I7 I8 I9 I10 I11 I12 I13 I14 I15 I16 I17 I18 I19 I20 I21 I22 I23 I24 I25 I26 I27 I28 I29 I30 I31 I32 I33 I34 I35 I36 I37 I38 I39 I40 I41 I42 I43 I2:I3 I44:I1048576">
       <formula1>"LD_LB,LD_LH,LD_LW,LD_LBU,LD_LHU,LD_XX"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G4 G5 G6 G7 G8 G9 G10 G11 G12 G13 G14 G15 G16 G17 G18 G19 G20 G21 G22 G23 G24 G25 G26 G27 G28 G29 G30 G31 G32 G33 G34 G35 G36 G37 G38 G39 G40 G41 G42 G43 G2:G3 G44:G1048576">
-      <formula1>"IMM_I,IMM_J,IMM_U,IMM_S,IMM_B"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F6 F15 F18 F19 F20 F21 F24 F25 F26 F27 F28 F29 F30 F31 F32 F33 F36 F37 F38 F39 F40 F41 F42 F43 F2:F5 F7:F14 F16:F17 F22:F23 F34:F35 F44:F1048576">
+      <formula1>"ALU_ADD,ALU_SUB,ALU_AND,ALU_OR,ALU_XOR,ALU_SLL,ALU_SRL,ALU_SLT,ALU_SLTU,ALU_COPY_A,ALU_COPY_B,ALU_SRA"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K4 K5 K6 K7 K8 K9 K10 K11 K12 K13 K14 K15 K16 K17 K18 K19 K20 K21 K22 K23 K24 K25 K26 K27 K28 K29 K30 K31 K32 K33 K34 K35 K36 K37 K38 K39 K40 K41 K42 K43 K2:K3 K44:K1048576">
+      <formula1>"MASK_XX,MASK_B,MASK_H,MASK_W,MASK_D"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D4 D5 D6 D7 D8 D9 D10 D11 D12 D13 D14 D15 D16 D17 D18 D19 D20 D21 D22 D23 D24 D25 D26 D27 D28 D29 D30 D31 D32 D33 D34 D35 D36 D37 D38 D39 D40 D41 D42 D43 D2:D3 D44:D1048576">
+      <formula1>"A_PC,A_RS1"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
> compile NEMU ysyx_23060246 韩炳晋 Linux archlinux 6.12.17-1-lts #1 SMP PREEMPT_DYNAMIC Thu, 27 Feb 2025 14:12:30 +0000 x86_64 GNU/Linux  14:21:42 up 18:12,  1 user,  load average: 0.92, 2.10, 2.56
</commit_message>
<xml_diff>
--- a/npc/tools/control_gen/control_table.xlsx
+++ b/npc/tools/control_gen/control_table.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="355" uniqueCount="119">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="311" uniqueCount="112">
   <si>
     <t>comment</t>
   </si>
@@ -76,9 +76,6 @@
     <t>INST_VALID</t>
   </si>
   <si>
-    <t>U_TYPE</t>
-  </si>
-  <si>
     <t>auipc</t>
   </si>
   <si>
@@ -97,9 +94,6 @@
     <t>IMM_I</t>
   </si>
   <si>
-    <t>I_TYPE</t>
-  </si>
-  <si>
     <t>andi</t>
   </si>
   <si>
@@ -133,9 +127,6 @@
     <t>IMM_J</t>
   </si>
   <si>
-    <t>J_TYPE</t>
-  </si>
-  <si>
     <t>sb</t>
   </si>
   <si>
@@ -148,9 +139,6 @@
     <t>MASK_B</t>
   </si>
   <si>
-    <t>S_TYPE</t>
-  </si>
-  <si>
     <t>sh</t>
   </si>
   <si>
@@ -211,9 +199,6 @@
     <t>BR_NE</t>
   </si>
   <si>
-    <t>B_TYPE</t>
-  </si>
-  <si>
     <t>beq</t>
   </si>
   <si>
@@ -262,9 +247,6 @@
     <t>B_RS2</t>
   </si>
   <si>
-    <t>R_TYPE</t>
-  </si>
-  <si>
     <t>sra</t>
   </si>
   <si>
@@ -338,9 +320,6 @@
   </si>
   <si>
     <t>CSR_P</t>
-  </si>
-  <si>
-    <t>N_TYPE</t>
   </si>
   <si>
     <t>mret</t>
@@ -379,9 +358,9 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="4">
     <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="42" formatCode="_ &quot;￥&quot;* #,##0_ ;_ &quot;￥&quot;* \-#,##0_ ;_ &quot;￥&quot;* &quot;-&quot;_ ;_ @_ "/>
     <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="41" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
+    <numFmt numFmtId="42" formatCode="_ &quot;￥&quot;* #,##0_ ;_ &quot;￥&quot;* \-#,##0_ ;_ &quot;￥&quot;* &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
   <fonts count="22">
     <font>
@@ -399,6 +378,21 @@
     </font>
     <font>
       <sz val="10.8"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="3"/>
       <name val="宋体"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -425,29 +419,6 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF0000FF"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="3"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <b/>
       <sz val="18"/>
       <color theme="3"/>
@@ -461,6 +432,22 @@
       <color rgb="FF800080"/>
       <name val="宋体"/>
       <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color rgb="FF7F7F7F"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="15"/>
+      <color theme="3"/>
+      <name val="宋体"/>
+      <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -489,7 +476,14 @@
     <font>
       <b/>
       <sz val="11"/>
-      <color theme="1"/>
+      <color rgb="FFFA7D00"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF3F3F76"/>
       <name val="宋体"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -503,8 +497,24 @@
     </font>
     <font>
       <b/>
+      <sz val="13"/>
+      <color theme="3"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
       <sz val="11"/>
-      <color rgb="FFFA7D00"/>
+      <color rgb="FF0000FF"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="宋体"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -512,37 +522,6 @@
     <font>
       <sz val="11"/>
       <color rgb="FF006100"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="13"/>
-      <color theme="3"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="15"/>
-      <color theme="3"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="11"/>
-      <color rgb="FF7F7F7F"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF3F3F76"/>
       <name val="宋体"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -557,13 +536,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9"/>
+        <fgColor theme="8" tint="0.599993896298105"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -581,67 +554,19 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.599993896298105"/>
+        <fgColor theme="9"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.399975585192419"/>
+        <fgColor theme="7" tint="0.599993896298105"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFF2F2F2"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.599993896298105"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -659,7 +584,61 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FFFFCC99"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor theme="4" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.399975585192419"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -671,19 +650,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.799981688894314"/>
+        <fgColor theme="8" tint="0.799981688894314"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
+        <fgColor theme="7" tint="0.399975585192419"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -695,19 +668,25 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor theme="8" tint="0.399975585192419"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="4"/>
+        <fgColor theme="6" tint="0.799981688894314"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5"/>
+        <fgColor theme="9" tint="0.399975585192419"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -719,25 +698,25 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="6"/>
+        <fgColor theme="7"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
+        <fgColor theme="5" tint="0.599993896298105"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.799981688894314"/>
+        <fgColor theme="6" tint="0.599993896298105"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.399975585192419"/>
+        <fgColor rgb="FFC6EFCE"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -748,6 +727,24 @@
       <right/>
       <top/>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="double">
+        <color rgb="FFFF8001"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4" tint="0.499984740745262"/>
+      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -769,17 +766,8 @@
       <left/>
       <right/>
       <top/>
-      <bottom style="double">
-        <color rgb="FFFF8001"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
       <bottom style="medium">
-        <color theme="4" tint="0.499984740745262"/>
+        <color theme="4"/>
       </bottom>
       <diagonal/>
     </border>
@@ -814,17 +802,6 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color theme="4"/>
-      </top>
-      <bottom style="double">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
       <left style="thin">
         <color rgb="FF7F7F7F"/>
       </left>
@@ -842,8 +819,10 @@
     <border>
       <left/>
       <right/>
-      <top/>
-      <bottom style="medium">
+      <top style="thin">
+        <color theme="4"/>
+      </top>
+      <bottom style="double">
         <color theme="4"/>
       </bottom>
       <diagonal/>
@@ -853,148 +832,148 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="30" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="6" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="10" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="6" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="15" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="17" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="15" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="6" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="7" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="8" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="7" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="5" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
@@ -1339,7 +1318,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:AJ99"/>
+  <dimension ref="A1:AI99"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
     <col min="1" max="1" width="13.1" customWidth="1"/>
@@ -1352,18 +1331,18 @@
     <col min="8" max="10" width="11.9833333333333" customWidth="1"/>
     <col min="11" max="11" width="15.075" customWidth="1"/>
     <col min="12" max="14" width="12.1083333333333" customWidth="1"/>
-    <col min="15" max="16" width="10.8583333333333" customWidth="1"/>
-    <col min="18" max="18" width="14.2166666666667" customWidth="1"/>
-    <col min="19" max="19" width="11.8083333333333" customWidth="1"/>
-    <col min="20" max="20" width="10.6" customWidth="1"/>
-    <col min="21" max="21" width="9.70833333333333" customWidth="1"/>
-    <col min="22" max="22" width="11.1666666666667" customWidth="1"/>
-    <col min="23" max="23" width="11.4083333333333" customWidth="1"/>
-    <col min="24" max="24" width="12.0583333333333" customWidth="1"/>
-    <col min="25" max="25" width="15.575" customWidth="1"/>
+    <col min="15" max="15" width="10.8583333333333" customWidth="1"/>
+    <col min="17" max="17" width="14.2166666666667" customWidth="1"/>
+    <col min="18" max="18" width="11.8083333333333" customWidth="1"/>
+    <col min="19" max="19" width="10.6" customWidth="1"/>
+    <col min="20" max="20" width="9.70833333333333" customWidth="1"/>
+    <col min="21" max="21" width="11.1666666666667" customWidth="1"/>
+    <col min="22" max="22" width="11.4083333333333" customWidth="1"/>
+    <col min="23" max="23" width="12.0583333333333" customWidth="1"/>
+    <col min="24" max="24" width="15.575" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="15" customHeight="1" spans="1:24">
+    <row r="1" ht="15" customHeight="1" spans="1:23">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1406,18 +1385,15 @@
       <c r="N1" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="2" t="s">
-        <v>1</v>
-      </c>
+      <c r="O1" s="2"/>
       <c r="P1" s="2"/>
       <c r="Q1" s="2"/>
       <c r="R1" s="2"/>
       <c r="S1" s="2"/>
       <c r="T1" s="2"/>
-      <c r="U1" s="2"/>
-      <c r="X1" s="6"/>
-    </row>
-    <row r="2" spans="1:36">
+      <c r="W1" s="6"/>
+    </row>
+    <row r="2" spans="1:35">
       <c r="A2" s="3"/>
       <c r="B2" s="4" t="s">
         <v>14</v>
@@ -1444,15 +1420,13 @@
       <c r="N2" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O2" s="4" t="s">
-        <v>20</v>
-      </c>
+      <c r="O2" s="4"/>
       <c r="P2" s="4"/>
       <c r="Q2" s="4"/>
       <c r="R2" s="4"/>
       <c r="S2" s="4"/>
       <c r="T2" s="4"/>
-      <c r="U2" s="4"/>
+      <c r="U2" s="3"/>
       <c r="V2" s="3"/>
       <c r="W2" s="3"/>
       <c r="X2" s="3"/>
@@ -1467,22 +1441,21 @@
       <c r="AG2" s="3"/>
       <c r="AH2" s="3"/>
       <c r="AI2" s="3"/>
-      <c r="AJ2" s="3"/>
-    </row>
-    <row r="3" spans="1:36">
+    </row>
+    <row r="3" spans="1:35">
       <c r="A3" s="3"/>
       <c r="B3" s="4" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C3" s="2"/>
       <c r="D3" s="4" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E3" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G3" s="4" t="s">
         <v>17</v>
@@ -1498,15 +1471,13 @@
       <c r="N3" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O3" s="4" t="s">
-        <v>20</v>
-      </c>
+      <c r="O3" s="4"/>
       <c r="P3" s="4"/>
       <c r="Q3" s="4"/>
       <c r="R3" s="4"/>
       <c r="S3" s="4"/>
       <c r="T3" s="4"/>
-      <c r="U3" s="4"/>
+      <c r="U3" s="3"/>
       <c r="V3" s="3"/>
       <c r="W3" s="3"/>
       <c r="X3" s="3"/>
@@ -1521,25 +1492,24 @@
       <c r="AG3" s="3"/>
       <c r="AH3" s="3"/>
       <c r="AI3" s="3"/>
-      <c r="AJ3" s="3"/>
-    </row>
-    <row r="4" spans="1:36">
+    </row>
+    <row r="4" spans="1:35">
       <c r="A4" s="3"/>
       <c r="B4" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C4" s="2"/>
       <c r="D4" s="4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E4" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="H4" s="4" t="s">
         <v>18</v>
@@ -1552,15 +1522,13 @@
       <c r="N4" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O4" s="4" t="s">
-        <v>27</v>
-      </c>
+      <c r="O4" s="4"/>
       <c r="P4" s="4"/>
       <c r="Q4" s="4"/>
       <c r="R4" s="4"/>
       <c r="S4" s="4"/>
       <c r="T4" s="4"/>
-      <c r="U4" s="4"/>
+      <c r="U4" s="3"/>
       <c r="V4" s="3"/>
       <c r="W4" s="3"/>
       <c r="X4" s="3"/>
@@ -1575,25 +1543,24 @@
       <c r="AG4" s="3"/>
       <c r="AH4" s="3"/>
       <c r="AI4" s="3"/>
-      <c r="AJ4" s="3"/>
-    </row>
-    <row r="5" spans="1:36">
+    </row>
+    <row r="5" spans="1:35">
       <c r="A5" s="3"/>
       <c r="B5" s="4" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="C5" s="2"/>
       <c r="D5" s="4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E5" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="H5" s="4" t="s">
         <v>18</v>
@@ -1606,15 +1573,13 @@
       <c r="N5" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O5" s="4" t="s">
-        <v>27</v>
-      </c>
+      <c r="O5" s="4"/>
       <c r="P5" s="4"/>
       <c r="Q5" s="4"/>
       <c r="R5" s="4"/>
       <c r="S5" s="4"/>
       <c r="T5" s="4"/>
-      <c r="U5" s="4"/>
+      <c r="U5" s="3"/>
       <c r="V5" s="3"/>
       <c r="W5" s="3"/>
       <c r="X5" s="3"/>
@@ -1629,25 +1594,24 @@
       <c r="AG5" s="3"/>
       <c r="AH5" s="3"/>
       <c r="AI5" s="3"/>
-      <c r="AJ5" s="3"/>
-    </row>
-    <row r="6" spans="1:36">
+    </row>
+    <row r="6" spans="1:35">
       <c r="A6" s="3"/>
       <c r="B6" s="4" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="C6" s="2"/>
       <c r="D6" s="4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E6" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="G6" s="4" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="H6" s="4" t="s">
         <v>18</v>
@@ -1660,15 +1624,13 @@
       <c r="N6" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O6" s="4" t="s">
-        <v>27</v>
-      </c>
+      <c r="O6" s="4"/>
       <c r="P6" s="4"/>
       <c r="Q6" s="4"/>
       <c r="R6" s="4"/>
       <c r="S6" s="4"/>
       <c r="T6" s="4"/>
-      <c r="U6" s="4"/>
+      <c r="U6" s="3"/>
       <c r="V6" s="3"/>
       <c r="W6" s="3"/>
       <c r="X6" s="3"/>
@@ -1683,25 +1645,24 @@
       <c r="AG6" s="3"/>
       <c r="AH6" s="3"/>
       <c r="AI6" s="3"/>
-      <c r="AJ6" s="3"/>
-    </row>
-    <row r="7" spans="1:36">
+    </row>
+    <row r="7" spans="1:35">
       <c r="A7" s="3"/>
       <c r="B7" s="4" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="C7" s="2"/>
       <c r="D7" s="4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E7" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="G7" s="4" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="H7" s="4" t="s">
         <v>18</v>
@@ -1714,15 +1675,13 @@
       <c r="N7" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O7" s="4" t="s">
-        <v>27</v>
-      </c>
+      <c r="O7" s="4"/>
       <c r="P7" s="4"/>
       <c r="Q7" s="4"/>
       <c r="R7" s="4"/>
       <c r="S7" s="4"/>
       <c r="T7" s="4"/>
-      <c r="U7" s="4"/>
+      <c r="U7" s="3"/>
       <c r="V7" s="3"/>
       <c r="W7" s="3"/>
       <c r="X7" s="3"/>
@@ -1737,30 +1696,29 @@
       <c r="AG7" s="3"/>
       <c r="AH7" s="3"/>
       <c r="AI7" s="3"/>
-      <c r="AJ7" s="3"/>
-    </row>
-    <row r="8" spans="1:36">
+    </row>
+    <row r="8" spans="1:35">
       <c r="A8" s="3"/>
       <c r="B8" s="4" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E8" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F8" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G8" s="4" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="H8" s="4" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="I8" s="4"/>
       <c r="J8" s="4"/>
@@ -1770,15 +1728,13 @@
       <c r="N8" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O8" s="4" t="s">
-        <v>27</v>
-      </c>
+      <c r="O8" s="4"/>
       <c r="P8" s="4"/>
       <c r="Q8" s="4"/>
       <c r="R8" s="4"/>
       <c r="S8" s="4"/>
       <c r="T8" s="4"/>
-      <c r="U8" s="4"/>
+      <c r="U8" s="3"/>
       <c r="V8" s="3"/>
       <c r="W8" s="3"/>
       <c r="X8" s="3"/>
@@ -1793,30 +1749,29 @@
       <c r="AG8" s="3"/>
       <c r="AH8" s="3"/>
       <c r="AI8" s="3"/>
-      <c r="AJ8" s="3"/>
-    </row>
-    <row r="9" spans="1:36">
+    </row>
+    <row r="9" spans="1:35">
       <c r="A9" s="3"/>
       <c r="B9" s="4" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E9" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F9" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G9" s="4" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="H9" s="4" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="I9" s="4"/>
       <c r="J9" s="4"/>
@@ -1826,15 +1781,13 @@
       <c r="N9" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O9" s="4" t="s">
-        <v>39</v>
-      </c>
+      <c r="O9" s="4"/>
       <c r="P9" s="4"/>
       <c r="Q9" s="4"/>
       <c r="R9" s="4"/>
       <c r="S9" s="4"/>
       <c r="T9" s="4"/>
-      <c r="U9" s="4"/>
+      <c r="U9" s="3"/>
       <c r="V9" s="3"/>
       <c r="W9" s="3"/>
       <c r="X9" s="3"/>
@@ -1849,48 +1802,45 @@
       <c r="AG9" s="3"/>
       <c r="AH9" s="3"/>
       <c r="AI9" s="3"/>
-      <c r="AJ9" s="3"/>
-    </row>
-    <row r="10" spans="1:36">
+    </row>
+    <row r="10" spans="1:35">
       <c r="A10" s="3"/>
       <c r="B10" s="4" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="C10" s="2"/>
       <c r="D10" s="4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E10" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F10" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G10" s="4" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="H10" s="4"/>
       <c r="I10" s="4"/>
       <c r="J10" s="4" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="K10" s="4" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="L10" s="4"/>
       <c r="M10" s="4"/>
       <c r="N10" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O10" s="4" t="s">
-        <v>44</v>
-      </c>
+      <c r="O10" s="4"/>
       <c r="P10" s="4"/>
       <c r="Q10" s="4"/>
       <c r="R10" s="4"/>
       <c r="S10" s="4"/>
       <c r="T10" s="4"/>
-      <c r="U10" s="4"/>
+      <c r="U10" s="3"/>
       <c r="V10" s="3"/>
       <c r="W10" s="3"/>
       <c r="X10" s="3"/>
@@ -1905,48 +1855,45 @@
       <c r="AG10" s="3"/>
       <c r="AH10" s="3"/>
       <c r="AI10" s="3"/>
-      <c r="AJ10" s="3"/>
-    </row>
-    <row r="11" spans="1:36">
+    </row>
+    <row r="11" spans="1:35">
       <c r="A11" s="3"/>
       <c r="B11" s="4" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="C11" s="2"/>
       <c r="D11" s="4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E11" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F11" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G11" s="4" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="H11" s="4"/>
       <c r="I11" s="4"/>
       <c r="J11" s="4" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="K11" s="4" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="L11" s="4"/>
       <c r="M11" s="4"/>
       <c r="N11" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O11" s="4" t="s">
-        <v>44</v>
-      </c>
+      <c r="O11" s="4"/>
       <c r="P11" s="4"/>
       <c r="Q11" s="4"/>
       <c r="R11" s="4"/>
       <c r="S11" s="4"/>
       <c r="T11" s="4"/>
-      <c r="U11" s="4"/>
+      <c r="U11" s="3"/>
       <c r="V11" s="3"/>
       <c r="W11" s="3"/>
       <c r="X11" s="3"/>
@@ -1961,48 +1908,45 @@
       <c r="AG11" s="3"/>
       <c r="AH11" s="3"/>
       <c r="AI11" s="3"/>
-      <c r="AJ11" s="3"/>
-    </row>
-    <row r="12" spans="1:36">
+    </row>
+    <row r="12" spans="1:35">
       <c r="A12" s="3"/>
       <c r="B12" s="4" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="C12" s="2"/>
       <c r="D12" s="4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E12" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F12" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G12" s="4" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="H12" s="4"/>
       <c r="I12" s="4"/>
       <c r="J12" s="4" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="K12" s="4" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="L12" s="4"/>
       <c r="M12" s="4"/>
       <c r="N12" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O12" s="4" t="s">
-        <v>44</v>
-      </c>
+      <c r="O12" s="4"/>
       <c r="P12" s="4"/>
       <c r="Q12" s="4"/>
       <c r="R12" s="4"/>
       <c r="S12" s="4"/>
       <c r="T12" s="4"/>
-      <c r="U12" s="4"/>
+      <c r="U12" s="3"/>
       <c r="V12" s="3"/>
       <c r="W12" s="3"/>
       <c r="X12" s="3"/>
@@ -2017,31 +1961,30 @@
       <c r="AG12" s="3"/>
       <c r="AH12" s="3"/>
       <c r="AI12" s="3"/>
-      <c r="AJ12" s="3"/>
-    </row>
-    <row r="13" spans="1:36">
+    </row>
+    <row r="13" spans="1:35">
       <c r="A13" s="3"/>
       <c r="B13" s="4" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="C13" s="2"/>
       <c r="D13" s="4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E13" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F13" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G13" s="4" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="H13" s="4" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="I13" s="4" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="J13" s="4"/>
       <c r="K13" s="4"/>
@@ -2050,15 +1993,13 @@
       <c r="N13" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O13" s="4" t="s">
-        <v>27</v>
-      </c>
+      <c r="O13" s="4"/>
       <c r="P13" s="4"/>
       <c r="Q13" s="4"/>
       <c r="R13" s="4"/>
       <c r="S13" s="4"/>
       <c r="T13" s="4"/>
-      <c r="U13" s="4"/>
+      <c r="U13" s="3"/>
       <c r="V13" s="3"/>
       <c r="W13" s="3"/>
       <c r="X13" s="3"/>
@@ -2073,31 +2014,30 @@
       <c r="AG13" s="3"/>
       <c r="AH13" s="3"/>
       <c r="AI13" s="3"/>
-      <c r="AJ13" s="3"/>
-    </row>
-    <row r="14" spans="1:36">
+    </row>
+    <row r="14" spans="1:35">
       <c r="A14" s="3"/>
       <c r="B14" s="4" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="C14" s="2"/>
       <c r="D14" s="4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E14" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F14" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G14" s="4" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="H14" s="4" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="I14" s="4" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="J14" s="4"/>
       <c r="K14" s="4"/>
@@ -2106,15 +2046,13 @@
       <c r="N14" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O14" s="4" t="s">
-        <v>27</v>
-      </c>
+      <c r="O14" s="4"/>
       <c r="P14" s="4"/>
       <c r="Q14" s="4"/>
       <c r="R14" s="4"/>
       <c r="S14" s="4"/>
       <c r="T14" s="4"/>
-      <c r="U14" s="4"/>
+      <c r="U14" s="3"/>
       <c r="V14" s="3"/>
       <c r="W14" s="3"/>
       <c r="X14" s="3"/>
@@ -2129,31 +2067,30 @@
       <c r="AG14" s="3"/>
       <c r="AH14" s="3"/>
       <c r="AI14" s="3"/>
-      <c r="AJ14" s="3"/>
-    </row>
-    <row r="15" spans="1:36">
+    </row>
+    <row r="15" spans="1:35">
       <c r="A15" s="3"/>
       <c r="B15" s="4" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="C15" s="2"/>
       <c r="D15" s="4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E15" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F15" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G15" s="4" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="H15" s="4" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="I15" s="4" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="J15" s="4"/>
       <c r="K15" s="4"/>
@@ -2162,15 +2099,13 @@
       <c r="N15" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O15" s="4" t="s">
-        <v>27</v>
-      </c>
+      <c r="O15" s="4"/>
       <c r="P15" s="4"/>
       <c r="Q15" s="4"/>
       <c r="R15" s="4"/>
       <c r="S15" s="4"/>
       <c r="T15" s="4"/>
-      <c r="U15" s="4"/>
+      <c r="U15" s="3"/>
       <c r="V15" s="3"/>
       <c r="W15" s="3"/>
       <c r="X15" s="3"/>
@@ -2185,31 +2120,30 @@
       <c r="AG15" s="3"/>
       <c r="AH15" s="3"/>
       <c r="AI15" s="3"/>
-      <c r="AJ15" s="3"/>
-    </row>
-    <row r="16" spans="1:36">
+    </row>
+    <row r="16" spans="1:35">
       <c r="A16" s="3"/>
       <c r="B16" s="4" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="C16" s="2"/>
       <c r="D16" s="4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E16" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F16" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G16" s="4" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="H16" s="4" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="I16" s="4" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="J16" s="4"/>
       <c r="K16" s="4"/>
@@ -2218,15 +2152,13 @@
       <c r="N16" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O16" s="4" t="s">
-        <v>27</v>
-      </c>
+      <c r="O16" s="4"/>
       <c r="P16" s="4"/>
       <c r="Q16" s="4"/>
       <c r="R16" s="4"/>
       <c r="S16" s="4"/>
       <c r="T16" s="4"/>
-      <c r="U16" s="4"/>
+      <c r="U16" s="3"/>
       <c r="V16" s="3"/>
       <c r="W16" s="3"/>
       <c r="X16" s="3"/>
@@ -2241,31 +2173,30 @@
       <c r="AG16" s="3"/>
       <c r="AH16" s="3"/>
       <c r="AI16" s="3"/>
-      <c r="AJ16" s="3"/>
-    </row>
-    <row r="17" spans="1:36">
+    </row>
+    <row r="17" spans="1:35">
       <c r="A17" s="3"/>
       <c r="B17" s="4" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="C17" s="2"/>
       <c r="D17" s="4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E17" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F17" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G17" s="4" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="H17" s="4" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="I17" s="4" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="J17" s="4"/>
       <c r="K17" s="4"/>
@@ -2274,15 +2205,13 @@
       <c r="N17" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O17" s="4" t="s">
-        <v>27</v>
-      </c>
+      <c r="O17" s="4"/>
       <c r="P17" s="4"/>
       <c r="Q17" s="4"/>
       <c r="R17" s="4"/>
       <c r="S17" s="4"/>
       <c r="T17" s="4"/>
-      <c r="U17" s="4"/>
+      <c r="U17" s="3"/>
       <c r="V17" s="3"/>
       <c r="W17" s="3"/>
       <c r="X17" s="3"/>
@@ -2297,46 +2226,43 @@
       <c r="AG17" s="3"/>
       <c r="AH17" s="3"/>
       <c r="AI17" s="3"/>
-      <c r="AJ17" s="3"/>
-    </row>
-    <row r="18" spans="1:36">
+    </row>
+    <row r="18" spans="1:35">
       <c r="A18" s="3"/>
       <c r="B18" s="4" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="C18" s="2"/>
       <c r="D18" s="4" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E18" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F18" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G18" s="4" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="H18" s="4"/>
       <c r="I18" s="4"/>
       <c r="J18" s="4"/>
       <c r="K18" s="4"/>
       <c r="L18" s="4" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="M18" s="4"/>
       <c r="N18" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O18" s="4" t="s">
-        <v>65</v>
-      </c>
+      <c r="O18" s="4"/>
       <c r="P18" s="4"/>
       <c r="Q18" s="4"/>
       <c r="R18" s="4"/>
       <c r="S18" s="4"/>
       <c r="T18" s="4"/>
-      <c r="U18" s="4"/>
+      <c r="U18" s="3"/>
       <c r="V18" s="3"/>
       <c r="W18" s="3"/>
       <c r="X18" s="3"/>
@@ -2351,46 +2277,43 @@
       <c r="AG18" s="3"/>
       <c r="AH18" s="3"/>
       <c r="AI18" s="3"/>
-      <c r="AJ18" s="3"/>
-    </row>
-    <row r="19" spans="1:36">
+    </row>
+    <row r="19" spans="1:35">
       <c r="A19" s="3"/>
       <c r="B19" s="4" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
       <c r="C19" s="2"/>
       <c r="D19" s="4" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E19" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F19" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G19" s="4" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="H19" s="4"/>
       <c r="I19" s="4"/>
       <c r="J19" s="4"/>
       <c r="K19" s="4"/>
       <c r="L19" s="4" t="s">
-        <v>67</v>
+        <v>62</v>
       </c>
       <c r="M19" s="4"/>
       <c r="N19" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O19" s="4" t="s">
-        <v>65</v>
-      </c>
+      <c r="O19" s="4"/>
       <c r="P19" s="4"/>
       <c r="Q19" s="4"/>
       <c r="R19" s="4"/>
       <c r="S19" s="4"/>
       <c r="T19" s="4"/>
-      <c r="U19" s="4"/>
+      <c r="U19" s="3"/>
       <c r="V19" s="3"/>
       <c r="W19" s="3"/>
       <c r="X19" s="3"/>
@@ -2405,46 +2328,43 @@
       <c r="AG19" s="3"/>
       <c r="AH19" s="3"/>
       <c r="AI19" s="3"/>
-      <c r="AJ19" s="3"/>
-    </row>
-    <row r="20" spans="1:36">
+    </row>
+    <row r="20" spans="1:35">
       <c r="A20" s="3"/>
       <c r="B20" s="4" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="C20" s="2"/>
       <c r="D20" s="4" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E20" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F20" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G20" s="4" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="H20" s="4"/>
       <c r="I20" s="4"/>
       <c r="J20" s="4"/>
       <c r="K20" s="4"/>
       <c r="L20" s="4" t="s">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="M20" s="4"/>
       <c r="N20" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O20" s="4" t="s">
-        <v>65</v>
-      </c>
+      <c r="O20" s="4"/>
       <c r="P20" s="4"/>
       <c r="Q20" s="4"/>
       <c r="R20" s="4"/>
       <c r="S20" s="4"/>
       <c r="T20" s="4"/>
-      <c r="U20" s="4"/>
+      <c r="U20" s="3"/>
       <c r="V20" s="3"/>
       <c r="W20" s="3"/>
       <c r="X20" s="3"/>
@@ -2459,46 +2379,43 @@
       <c r="AG20" s="3"/>
       <c r="AH20" s="3"/>
       <c r="AI20" s="3"/>
-      <c r="AJ20" s="3"/>
-    </row>
-    <row r="21" spans="1:36">
+    </row>
+    <row r="21" spans="1:35">
       <c r="A21" s="3"/>
       <c r="B21" s="4" t="s">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="C21" s="2"/>
       <c r="D21" s="4" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E21" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F21" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G21" s="4" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="H21" s="4"/>
       <c r="I21" s="4"/>
       <c r="J21" s="4"/>
       <c r="K21" s="4"/>
       <c r="L21" s="4" t="s">
-        <v>71</v>
+        <v>66</v>
       </c>
       <c r="M21" s="4"/>
       <c r="N21" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O21" s="4" t="s">
-        <v>65</v>
-      </c>
+      <c r="O21" s="4"/>
       <c r="P21" s="4"/>
       <c r="Q21" s="4"/>
       <c r="R21" s="4"/>
       <c r="S21" s="4"/>
       <c r="T21" s="4"/>
-      <c r="U21" s="4"/>
+      <c r="U21" s="3"/>
       <c r="V21" s="3"/>
       <c r="W21" s="3"/>
       <c r="X21" s="3"/>
@@ -2513,46 +2430,43 @@
       <c r="AG21" s="3"/>
       <c r="AH21" s="3"/>
       <c r="AI21" s="3"/>
-      <c r="AJ21" s="3"/>
-    </row>
-    <row r="22" spans="1:36">
+    </row>
+    <row r="22" spans="1:35">
       <c r="A22" s="3"/>
       <c r="B22" s="4" t="s">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="C22" s="2"/>
       <c r="D22" s="4" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E22" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F22" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G22" s="4" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="H22" s="4"/>
       <c r="I22" s="4"/>
       <c r="J22" s="4"/>
       <c r="K22" s="4"/>
       <c r="L22" s="4" t="s">
-        <v>73</v>
+        <v>68</v>
       </c>
       <c r="M22" s="4"/>
       <c r="N22" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O22" s="4" t="s">
-        <v>65</v>
-      </c>
+      <c r="O22" s="4"/>
       <c r="P22" s="4"/>
       <c r="Q22" s="4"/>
       <c r="R22" s="4"/>
       <c r="S22" s="4"/>
       <c r="T22" s="4"/>
-      <c r="U22" s="4"/>
+      <c r="U22" s="3"/>
       <c r="V22" s="3"/>
       <c r="W22" s="3"/>
       <c r="X22" s="3"/>
@@ -2567,46 +2481,43 @@
       <c r="AG22" s="3"/>
       <c r="AH22" s="3"/>
       <c r="AI22" s="3"/>
-      <c r="AJ22" s="3"/>
-    </row>
-    <row r="23" spans="1:36">
+    </row>
+    <row r="23" spans="1:35">
       <c r="A23" s="3"/>
       <c r="B23" s="4" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="C23" s="2"/>
       <c r="D23" s="4" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E23" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F23" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G23" s="4" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="H23" s="4"/>
       <c r="I23" s="4"/>
       <c r="J23" s="4"/>
       <c r="K23" s="4"/>
       <c r="L23" s="4" t="s">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="M23" s="4"/>
       <c r="N23" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O23" s="4" t="s">
-        <v>65</v>
-      </c>
+      <c r="O23" s="4"/>
       <c r="P23" s="4"/>
       <c r="Q23" s="4"/>
       <c r="R23" s="4"/>
       <c r="S23" s="4"/>
       <c r="T23" s="4"/>
-      <c r="U23" s="4"/>
+      <c r="U23" s="3"/>
       <c r="V23" s="3"/>
       <c r="W23" s="3"/>
       <c r="X23" s="3"/>
@@ -2621,25 +2532,24 @@
       <c r="AG23" s="3"/>
       <c r="AH23" s="3"/>
       <c r="AI23" s="3"/>
-      <c r="AJ23" s="3"/>
-    </row>
-    <row r="24" spans="1:36">
+    </row>
+    <row r="24" spans="1:35">
       <c r="A24" s="3"/>
       <c r="B24" s="4" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="C24" s="2"/>
       <c r="D24" s="4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E24" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F24" s="4" t="s">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="G24" s="4" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="H24" s="4" t="s">
         <v>18</v>
@@ -2652,15 +2562,13 @@
       <c r="N24" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O24" s="4" t="s">
-        <v>27</v>
-      </c>
+      <c r="O24" s="4"/>
       <c r="P24" s="4"/>
       <c r="Q24" s="4"/>
       <c r="R24" s="4"/>
       <c r="S24" s="4"/>
       <c r="T24" s="4"/>
-      <c r="U24" s="4"/>
+      <c r="U24" s="3"/>
       <c r="V24" s="3"/>
       <c r="W24" s="3"/>
       <c r="X24" s="3"/>
@@ -2675,25 +2583,24 @@
       <c r="AG24" s="3"/>
       <c r="AH24" s="3"/>
       <c r="AI24" s="3"/>
-      <c r="AJ24" s="3"/>
-    </row>
-    <row r="25" spans="1:36">
+    </row>
+    <row r="25" spans="1:35">
       <c r="A25" s="3"/>
       <c r="B25" s="4" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="C25" s="2"/>
       <c r="D25" s="4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E25" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F25" s="4" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="G25" s="4" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="H25" s="4" t="s">
         <v>18</v>
@@ -2706,15 +2613,13 @@
       <c r="N25" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O25" s="4" t="s">
-        <v>27</v>
-      </c>
+      <c r="O25" s="4"/>
       <c r="P25" s="4"/>
       <c r="Q25" s="4"/>
       <c r="R25" s="4"/>
       <c r="S25" s="4"/>
       <c r="T25" s="4"/>
-      <c r="U25" s="4"/>
+      <c r="U25" s="3"/>
       <c r="V25" s="3"/>
       <c r="W25" s="3"/>
       <c r="X25" s="3"/>
@@ -2729,22 +2634,21 @@
       <c r="AG25" s="3"/>
       <c r="AH25" s="3"/>
       <c r="AI25" s="3"/>
-      <c r="AJ25" s="3"/>
-    </row>
-    <row r="26" spans="1:36">
+    </row>
+    <row r="26" spans="1:35">
       <c r="A26" s="3"/>
       <c r="B26" s="4" t="s">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="C26" s="2"/>
       <c r="D26" s="4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E26" s="4" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="F26" s="4" t="s">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="G26" s="4"/>
       <c r="H26" s="4" t="s">
@@ -2758,15 +2662,13 @@
       <c r="N26" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O26" s="4" t="s">
-        <v>82</v>
-      </c>
+      <c r="O26" s="4"/>
       <c r="P26" s="4"/>
       <c r="Q26" s="4"/>
       <c r="R26" s="4"/>
       <c r="S26" s="4"/>
       <c r="T26" s="4"/>
-      <c r="U26" s="4"/>
+      <c r="U26" s="3"/>
       <c r="V26" s="3"/>
       <c r="W26" s="3"/>
       <c r="X26" s="3"/>
@@ -2781,22 +2683,21 @@
       <c r="AG26" s="3"/>
       <c r="AH26" s="3"/>
       <c r="AI26" s="3"/>
-      <c r="AJ26" s="3"/>
-    </row>
-    <row r="27" spans="1:36">
+    </row>
+    <row r="27" spans="1:35">
       <c r="A27" s="3"/>
       <c r="B27" s="4" t="s">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="C27" s="2"/>
       <c r="D27" s="4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E27" s="4" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="F27" s="4" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="G27" s="4"/>
       <c r="H27" s="4" t="s">
@@ -2810,15 +2711,13 @@
       <c r="N27" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O27" s="4" t="s">
-        <v>82</v>
-      </c>
+      <c r="O27" s="4"/>
       <c r="P27" s="4"/>
       <c r="Q27" s="4"/>
       <c r="R27" s="4"/>
       <c r="S27" s="4"/>
       <c r="T27" s="4"/>
-      <c r="U27" s="4"/>
+      <c r="U27" s="3"/>
       <c r="V27" s="3"/>
       <c r="W27" s="3"/>
       <c r="X27" s="3"/>
@@ -2833,25 +2732,24 @@
       <c r="AG27" s="3"/>
       <c r="AH27" s="3"/>
       <c r="AI27" s="3"/>
-      <c r="AJ27" s="3"/>
-    </row>
-    <row r="28" spans="1:36">
+    </row>
+    <row r="28" spans="1:35">
       <c r="A28" s="3"/>
       <c r="B28" s="4" t="s">
-        <v>84</v>
+        <v>78</v>
       </c>
       <c r="C28" s="2"/>
       <c r="D28" s="4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E28" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F28" s="4" t="s">
-        <v>85</v>
+        <v>79</v>
       </c>
       <c r="G28" s="4" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="H28" s="4" t="s">
         <v>18</v>
@@ -2864,15 +2762,13 @@
       <c r="N28" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O28" s="4" t="s">
-        <v>27</v>
-      </c>
+      <c r="O28" s="4"/>
       <c r="P28" s="4"/>
       <c r="Q28" s="4"/>
       <c r="R28" s="4"/>
       <c r="S28" s="4"/>
       <c r="T28" s="4"/>
-      <c r="U28" s="4"/>
+      <c r="U28" s="3"/>
       <c r="V28" s="3"/>
       <c r="W28" s="3"/>
       <c r="X28" s="3"/>
@@ -2887,22 +2783,21 @@
       <c r="AG28" s="3"/>
       <c r="AH28" s="3"/>
       <c r="AI28" s="3"/>
-      <c r="AJ28" s="3"/>
-    </row>
-    <row r="29" spans="1:36">
+    </row>
+    <row r="29" spans="1:35">
       <c r="A29" s="3"/>
       <c r="B29" s="4" t="s">
-        <v>86</v>
+        <v>80</v>
       </c>
       <c r="C29" s="2"/>
       <c r="D29" s="4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E29" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="F29" s="4" t="s">
         <v>81</v>
-      </c>
-      <c r="F29" s="4" t="s">
-        <v>87</v>
       </c>
       <c r="G29" s="4"/>
       <c r="H29" s="4" t="s">
@@ -2916,15 +2811,13 @@
       <c r="N29" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O29" s="4" t="s">
-        <v>82</v>
-      </c>
+      <c r="O29" s="4"/>
       <c r="P29" s="4"/>
       <c r="Q29" s="4"/>
       <c r="R29" s="4"/>
       <c r="S29" s="4"/>
       <c r="T29" s="4"/>
-      <c r="U29" s="4"/>
+      <c r="U29" s="3"/>
       <c r="V29" s="3"/>
       <c r="W29" s="3"/>
       <c r="X29" s="3"/>
@@ -2939,22 +2832,21 @@
       <c r="AG29" s="3"/>
       <c r="AH29" s="3"/>
       <c r="AI29" s="3"/>
-      <c r="AJ29" s="3"/>
-    </row>
-    <row r="30" spans="1:36">
+    </row>
+    <row r="30" spans="1:35">
       <c r="A30" s="3"/>
       <c r="B30" s="4" t="s">
-        <v>88</v>
+        <v>82</v>
       </c>
       <c r="C30" s="2"/>
       <c r="D30" s="4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E30" s="4" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="F30" s="4" t="s">
-        <v>89</v>
+        <v>83</v>
       </c>
       <c r="G30" s="4"/>
       <c r="H30" s="4" t="s">
@@ -2968,15 +2860,13 @@
       <c r="N30" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O30" s="4" t="s">
-        <v>82</v>
-      </c>
+      <c r="O30" s="4"/>
       <c r="P30" s="4"/>
       <c r="Q30" s="4"/>
       <c r="R30" s="4"/>
       <c r="S30" s="4"/>
       <c r="T30" s="4"/>
-      <c r="U30" s="4"/>
+      <c r="U30" s="3"/>
       <c r="V30" s="3"/>
       <c r="W30" s="3"/>
       <c r="X30" s="3"/>
@@ -2991,25 +2881,24 @@
       <c r="AG30" s="3"/>
       <c r="AH30" s="3"/>
       <c r="AI30" s="3"/>
-      <c r="AJ30" s="3"/>
-    </row>
-    <row r="31" spans="1:36">
+    </row>
+    <row r="31" spans="1:35">
       <c r="A31" s="3"/>
       <c r="B31" s="4" t="s">
-        <v>90</v>
+        <v>84</v>
       </c>
       <c r="C31" s="2"/>
       <c r="D31" s="4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E31" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F31" s="4" t="s">
-        <v>89</v>
+        <v>83</v>
       </c>
       <c r="G31" s="4" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="H31" s="4" t="s">
         <v>18</v>
@@ -3022,15 +2911,13 @@
       <c r="N31" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O31" s="4" t="s">
-        <v>27</v>
-      </c>
+      <c r="O31" s="4"/>
       <c r="P31" s="4"/>
       <c r="Q31" s="4"/>
       <c r="R31" s="4"/>
       <c r="S31" s="4"/>
       <c r="T31" s="4"/>
-      <c r="U31" s="4"/>
+      <c r="U31" s="3"/>
       <c r="V31" s="3"/>
       <c r="W31" s="3"/>
       <c r="X31" s="3"/>
@@ -3045,25 +2932,24 @@
       <c r="AG31" s="3"/>
       <c r="AH31" s="3"/>
       <c r="AI31" s="3"/>
-      <c r="AJ31" s="3"/>
-    </row>
-    <row r="32" spans="1:36">
+    </row>
+    <row r="32" spans="1:35">
       <c r="A32" s="3"/>
       <c r="B32" s="4" t="s">
-        <v>91</v>
+        <v>85</v>
       </c>
       <c r="C32" s="2"/>
       <c r="D32" s="4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E32" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F32" s="4" t="s">
-        <v>89</v>
+        <v>83</v>
       </c>
       <c r="G32" s="4" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="H32" s="4" t="s">
         <v>18</v>
@@ -3076,15 +2962,13 @@
       <c r="N32" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O32" s="4" t="s">
-        <v>27</v>
-      </c>
+      <c r="O32" s="4"/>
       <c r="P32" s="4"/>
       <c r="Q32" s="4"/>
       <c r="R32" s="4"/>
       <c r="S32" s="4"/>
       <c r="T32" s="4"/>
-      <c r="U32" s="4"/>
+      <c r="U32" s="3"/>
       <c r="V32" s="3"/>
       <c r="W32" s="3"/>
       <c r="X32" s="3"/>
@@ -3099,22 +2983,21 @@
       <c r="AG32" s="3"/>
       <c r="AH32" s="3"/>
       <c r="AI32" s="3"/>
-      <c r="AJ32" s="3"/>
-    </row>
-    <row r="33" spans="1:36">
+    </row>
+    <row r="33" spans="1:35">
       <c r="A33" s="3"/>
       <c r="B33" s="4" t="s">
-        <v>92</v>
+        <v>86</v>
       </c>
       <c r="C33" s="2"/>
       <c r="D33" s="4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E33" s="4" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="F33" s="4" t="s">
-        <v>85</v>
+        <v>79</v>
       </c>
       <c r="G33" s="4"/>
       <c r="H33" s="4" t="s">
@@ -3128,15 +3011,13 @@
       <c r="N33" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O33" s="4" t="s">
-        <v>82</v>
-      </c>
+      <c r="O33" s="4"/>
       <c r="P33" s="4"/>
       <c r="Q33" s="4"/>
       <c r="R33" s="4"/>
       <c r="S33" s="4"/>
       <c r="T33" s="4"/>
-      <c r="U33" s="4"/>
+      <c r="U33" s="3"/>
       <c r="V33" s="3"/>
       <c r="W33" s="3"/>
       <c r="X33" s="3"/>
@@ -3151,22 +3032,21 @@
       <c r="AG33" s="3"/>
       <c r="AH33" s="3"/>
       <c r="AI33" s="3"/>
-      <c r="AJ33" s="3"/>
-    </row>
-    <row r="34" spans="1:36">
+    </row>
+    <row r="34" spans="1:35">
       <c r="A34" s="3"/>
       <c r="B34" s="4" t="s">
-        <v>93</v>
+        <v>87</v>
       </c>
       <c r="C34" s="2"/>
       <c r="D34" s="4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E34" s="4" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="F34" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G34" s="4"/>
       <c r="H34" s="4" t="s">
@@ -3180,15 +3060,13 @@
       <c r="N34" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O34" s="4" t="s">
-        <v>82</v>
-      </c>
+      <c r="O34" s="4"/>
       <c r="P34" s="4"/>
       <c r="Q34" s="4"/>
       <c r="R34" s="4"/>
       <c r="S34" s="4"/>
       <c r="T34" s="4"/>
-      <c r="U34" s="4"/>
+      <c r="U34" s="3"/>
       <c r="V34" s="3"/>
       <c r="W34" s="3"/>
       <c r="X34" s="3"/>
@@ -3203,22 +3081,21 @@
       <c r="AG34" s="3"/>
       <c r="AH34" s="3"/>
       <c r="AI34" s="3"/>
-      <c r="AJ34" s="3"/>
-    </row>
-    <row r="35" spans="1:36">
+    </row>
+    <row r="35" spans="1:35">
       <c r="A35" s="3"/>
       <c r="B35" s="4" t="s">
-        <v>94</v>
+        <v>88</v>
       </c>
       <c r="C35" s="2"/>
       <c r="D35" s="4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E35" s="4" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="F35" s="4" t="s">
-        <v>95</v>
+        <v>89</v>
       </c>
       <c r="G35" s="4"/>
       <c r="H35" s="4" t="s">
@@ -3232,15 +3109,13 @@
       <c r="N35" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O35" s="4" t="s">
-        <v>82</v>
-      </c>
+      <c r="O35" s="4"/>
       <c r="P35" s="4"/>
       <c r="Q35" s="4"/>
       <c r="R35" s="4"/>
       <c r="S35" s="4"/>
       <c r="T35" s="4"/>
-      <c r="U35" s="4"/>
+      <c r="U35" s="3"/>
       <c r="V35" s="3"/>
       <c r="W35" s="3"/>
       <c r="X35" s="3"/>
@@ -3255,22 +3130,21 @@
       <c r="AG35" s="3"/>
       <c r="AH35" s="3"/>
       <c r="AI35" s="3"/>
-      <c r="AJ35" s="3"/>
-    </row>
-    <row r="36" spans="1:36">
+    </row>
+    <row r="36" spans="1:35">
       <c r="A36" s="3"/>
       <c r="B36" s="4" t="s">
-        <v>96</v>
+        <v>90</v>
       </c>
       <c r="C36" s="2"/>
       <c r="D36" s="4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E36" s="4" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="F36" s="4" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="G36" s="4"/>
       <c r="H36" s="4" t="s">
@@ -3284,15 +3158,13 @@
       <c r="N36" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O36" s="4" t="s">
-        <v>82</v>
-      </c>
+      <c r="O36" s="4"/>
       <c r="P36" s="4"/>
       <c r="Q36" s="4"/>
       <c r="R36" s="4"/>
       <c r="S36" s="4"/>
       <c r="T36" s="4"/>
-      <c r="U36" s="4"/>
+      <c r="U36" s="3"/>
       <c r="V36" s="3"/>
       <c r="W36" s="3"/>
       <c r="X36" s="3"/>
@@ -3307,22 +3179,21 @@
       <c r="AG36" s="3"/>
       <c r="AH36" s="3"/>
       <c r="AI36" s="3"/>
-      <c r="AJ36" s="3"/>
-    </row>
-    <row r="37" spans="1:36">
+    </row>
+    <row r="37" spans="1:35">
       <c r="A37" s="3"/>
       <c r="B37" s="4" t="s">
-        <v>97</v>
+        <v>91</v>
       </c>
       <c r="C37" s="2"/>
       <c r="D37" s="4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E37" s="4" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="F37" s="4" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="G37" s="4"/>
       <c r="H37" s="4" t="s">
@@ -3336,15 +3207,13 @@
       <c r="N37" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O37" s="4" t="s">
-        <v>82</v>
-      </c>
+      <c r="O37" s="4"/>
       <c r="P37" s="4"/>
       <c r="Q37" s="4"/>
       <c r="R37" s="4"/>
       <c r="S37" s="4"/>
       <c r="T37" s="4"/>
-      <c r="U37" s="4"/>
+      <c r="U37" s="3"/>
       <c r="V37" s="3"/>
       <c r="W37" s="3"/>
       <c r="X37" s="3"/>
@@ -3359,22 +3228,21 @@
       <c r="AG37" s="3"/>
       <c r="AH37" s="3"/>
       <c r="AI37" s="3"/>
-      <c r="AJ37" s="3"/>
-    </row>
-    <row r="38" spans="1:36">
+    </row>
+    <row r="38" spans="1:35">
       <c r="A38" s="3"/>
       <c r="B38" s="4" t="s">
-        <v>98</v>
+        <v>92</v>
       </c>
       <c r="C38" s="2"/>
       <c r="D38" s="4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E38" s="4" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="F38" s="4" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="G38" s="4"/>
       <c r="H38" s="4" t="s">
@@ -3388,15 +3256,13 @@
       <c r="N38" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O38" s="4" t="s">
-        <v>82</v>
-      </c>
+      <c r="O38" s="4"/>
       <c r="P38" s="4"/>
       <c r="Q38" s="4"/>
       <c r="R38" s="4"/>
       <c r="S38" s="4"/>
       <c r="T38" s="4"/>
-      <c r="U38" s="4"/>
+      <c r="U38" s="3"/>
       <c r="V38" s="3"/>
       <c r="W38" s="3"/>
       <c r="X38" s="3"/>
@@ -3411,46 +3277,43 @@
       <c r="AG38" s="3"/>
       <c r="AH38" s="3"/>
       <c r="AI38" s="3"/>
-      <c r="AJ38" s="3"/>
-    </row>
-    <row r="39" spans="1:36">
+    </row>
+    <row r="39" spans="1:35">
       <c r="A39" s="3"/>
       <c r="B39" s="4" t="s">
-        <v>99</v>
+        <v>93</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>100</v>
+        <v>94</v>
       </c>
       <c r="D39" s="4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E39" s="4" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="F39" s="4"/>
       <c r="G39" s="4"/>
       <c r="H39" s="4" t="s">
-        <v>101</v>
+        <v>95</v>
       </c>
       <c r="I39" s="4"/>
       <c r="J39" s="4"/>
       <c r="K39" s="4"/>
       <c r="L39" s="4"/>
       <c r="M39" s="4" t="s">
-        <v>102</v>
+        <v>96</v>
       </c>
       <c r="N39" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O39" s="4" t="s">
-        <v>82</v>
-      </c>
+      <c r="O39" s="4"/>
       <c r="P39" s="4"/>
       <c r="Q39" s="4"/>
       <c r="R39" s="4"/>
       <c r="S39" s="4"/>
       <c r="T39" s="4"/>
-      <c r="U39" s="4"/>
+      <c r="U39" s="3"/>
       <c r="V39" s="3"/>
       <c r="W39" s="3"/>
       <c r="X39" s="3"/>
@@ -3465,46 +3328,43 @@
       <c r="AG39" s="3"/>
       <c r="AH39" s="3"/>
       <c r="AI39" s="3"/>
-      <c r="AJ39" s="3"/>
-    </row>
-    <row r="40" spans="1:36">
+    </row>
+    <row r="40" spans="1:35">
       <c r="A40" s="3"/>
       <c r="B40" s="4" t="s">
-        <v>103</v>
+        <v>97</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>100</v>
+        <v>94</v>
       </c>
       <c r="D40" s="4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E40" s="4" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="F40" s="4"/>
       <c r="G40" s="4"/>
       <c r="H40" s="4" t="s">
-        <v>101</v>
+        <v>95</v>
       </c>
       <c r="I40" s="4"/>
       <c r="J40" s="4"/>
       <c r="K40" s="4"/>
       <c r="L40" s="4"/>
       <c r="M40" s="4" t="s">
-        <v>104</v>
+        <v>98</v>
       </c>
       <c r="N40" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O40" s="4" t="s">
-        <v>82</v>
-      </c>
+      <c r="O40" s="4"/>
       <c r="P40" s="4"/>
       <c r="Q40" s="4"/>
       <c r="R40" s="4"/>
       <c r="S40" s="4"/>
       <c r="T40" s="4"/>
-      <c r="U40" s="4"/>
+      <c r="U40" s="3"/>
       <c r="V40" s="3"/>
       <c r="W40" s="3"/>
       <c r="X40" s="3"/>
@@ -3519,42 +3379,39 @@
       <c r="AG40" s="3"/>
       <c r="AH40" s="3"/>
       <c r="AI40" s="3"/>
-      <c r="AJ40" s="3"/>
-    </row>
-    <row r="41" spans="1:36">
+    </row>
+    <row r="41" spans="1:35">
       <c r="A41" s="3"/>
       <c r="B41" s="4" t="s">
-        <v>105</v>
+        <v>99</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>106</v>
+        <v>100</v>
       </c>
       <c r="D41" s="4"/>
       <c r="E41" s="4"/>
       <c r="F41" s="4"/>
       <c r="G41" s="4"/>
       <c r="H41" s="4" t="s">
-        <v>101</v>
+        <v>95</v>
       </c>
       <c r="I41" s="4"/>
       <c r="J41" s="4"/>
       <c r="K41" s="4"/>
       <c r="L41" s="4"/>
       <c r="M41" s="4" t="s">
-        <v>107</v>
+        <v>101</v>
       </c>
       <c r="N41" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O41" s="4" t="s">
-        <v>108</v>
-      </c>
+      <c r="O41" s="4"/>
       <c r="P41" s="4"/>
       <c r="Q41" s="4"/>
       <c r="R41" s="4"/>
       <c r="S41" s="4"/>
       <c r="T41" s="4"/>
-      <c r="U41" s="4"/>
+      <c r="U41" s="3"/>
       <c r="V41" s="3"/>
       <c r="W41" s="3"/>
       <c r="X41" s="3"/>
@@ -3569,42 +3426,39 @@
       <c r="AG41" s="3"/>
       <c r="AH41" s="3"/>
       <c r="AI41" s="3"/>
-      <c r="AJ41" s="3"/>
-    </row>
-    <row r="42" spans="1:36">
+    </row>
+    <row r="42" spans="1:35">
       <c r="A42" s="3"/>
       <c r="B42" s="4" t="s">
-        <v>109</v>
+        <v>102</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>106</v>
+        <v>100</v>
       </c>
       <c r="D42" s="4"/>
       <c r="E42" s="4"/>
       <c r="F42" s="4"/>
       <c r="G42" s="4"/>
       <c r="H42" s="4" t="s">
-        <v>101</v>
+        <v>95</v>
       </c>
       <c r="I42" s="4"/>
       <c r="J42" s="4"/>
       <c r="K42" s="4"/>
       <c r="L42" s="4"/>
       <c r="M42" s="4" t="s">
-        <v>107</v>
+        <v>101</v>
       </c>
       <c r="N42" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O42" s="4" t="s">
-        <v>108</v>
-      </c>
+      <c r="O42" s="4"/>
       <c r="P42" s="4"/>
       <c r="Q42" s="4"/>
       <c r="R42" s="4"/>
       <c r="S42" s="4"/>
       <c r="T42" s="4"/>
-      <c r="U42" s="4"/>
+      <c r="U42" s="3"/>
       <c r="V42" s="3"/>
       <c r="W42" s="3"/>
       <c r="X42" s="3"/>
@@ -3619,11 +3473,10 @@
       <c r="AG42" s="3"/>
       <c r="AH42" s="3"/>
       <c r="AI42" s="3"/>
-      <c r="AJ42" s="3"/>
-    </row>
-    <row r="43" spans="2:36">
+    </row>
+    <row r="43" spans="2:35">
       <c r="B43" s="2" t="s">
-        <v>110</v>
+        <v>103</v>
       </c>
       <c r="C43" s="2"/>
       <c r="D43" s="2"/>
@@ -3639,15 +3492,13 @@
       <c r="N43" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="O43" s="2" t="s">
-        <v>27</v>
-      </c>
+      <c r="O43" s="2"/>
       <c r="P43" s="2"/>
       <c r="Q43" s="2"/>
       <c r="R43" s="2"/>
       <c r="S43" s="2"/>
       <c r="T43" s="2"/>
-      <c r="U43" s="2"/>
+      <c r="Y43" s="3"/>
       <c r="Z43" s="3"/>
       <c r="AA43" s="3"/>
       <c r="AB43" s="3"/>
@@ -3658,57 +3509,54 @@
       <c r="AG43" s="3"/>
       <c r="AH43" s="3"/>
       <c r="AI43" s="3"/>
-      <c r="AJ43" s="3"/>
-    </row>
-    <row r="44" spans="2:36">
+    </row>
+    <row r="44" spans="2:35">
       <c r="B44" s="2" t="s">
-        <v>111</v>
+        <v>104</v>
       </c>
       <c r="C44" s="2" t="s">
-        <v>100</v>
+        <v>94</v>
       </c>
       <c r="D44" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E44" s="2" t="s">
         <v>15</v>
       </c>
       <c r="F44" s="2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G44" s="2" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="H44" s="4" t="s">
-        <v>112</v>
+        <v>105</v>
       </c>
       <c r="I44" s="4" t="s">
-        <v>113</v>
+        <v>106</v>
       </c>
       <c r="J44" s="4" t="s">
-        <v>114</v>
+        <v>107</v>
       </c>
       <c r="K44" s="2" t="s">
-        <v>115</v>
+        <v>108</v>
       </c>
       <c r="L44" s="2" t="s">
-        <v>116</v>
+        <v>109</v>
       </c>
       <c r="M44" s="2" t="s">
-        <v>117</v>
+        <v>110</v>
       </c>
       <c r="N44" s="2" t="s">
-        <v>118</v>
-      </c>
-      <c r="O44" s="2" t="s">
-        <v>82</v>
-      </c>
+        <v>111</v>
+      </c>
+      <c r="O44" s="2"/>
       <c r="P44" s="2"/>
       <c r="Q44" s="2"/>
       <c r="R44" s="2"/>
       <c r="S44" s="2"/>
       <c r="T44" s="2"/>
-      <c r="U44" s="2"/>
+      <c r="Y44" s="3"/>
       <c r="Z44" s="3"/>
       <c r="AA44" s="3"/>
       <c r="AB44" s="3"/>
@@ -3719,9 +3567,8 @@
       <c r="AG44" s="3"/>
       <c r="AH44" s="3"/>
       <c r="AI44" s="3"/>
-      <c r="AJ44" s="3"/>
-    </row>
-    <row r="45" spans="1:36">
+    </row>
+    <row r="45" spans="1:35">
       <c r="A45" s="3"/>
       <c r="B45" s="4"/>
       <c r="C45" s="4"/>
@@ -3742,7 +3589,7 @@
       <c r="R45" s="4"/>
       <c r="S45" s="4"/>
       <c r="T45" s="4"/>
-      <c r="U45" s="4"/>
+      <c r="U45" s="3"/>
       <c r="V45" s="3"/>
       <c r="W45" s="3"/>
       <c r="X45" s="3"/>
@@ -3757,9 +3604,8 @@
       <c r="AG45" s="3"/>
       <c r="AH45" s="3"/>
       <c r="AI45" s="3"/>
-      <c r="AJ45" s="3"/>
-    </row>
-    <row r="46" s="1" customFormat="1" spans="1:36">
+    </row>
+    <row r="46" s="1" customFormat="1" spans="1:35">
       <c r="A46" s="3"/>
       <c r="B46" s="4"/>
       <c r="C46" s="4"/>
@@ -3780,7 +3626,7 @@
       <c r="R46" s="4"/>
       <c r="S46" s="4"/>
       <c r="T46" s="4"/>
-      <c r="U46" s="4"/>
+      <c r="U46" s="3"/>
       <c r="V46" s="3"/>
       <c r="W46" s="3"/>
       <c r="X46" s="3"/>
@@ -3795,9 +3641,8 @@
       <c r="AG46" s="3"/>
       <c r="AH46" s="3"/>
       <c r="AI46" s="3"/>
-      <c r="AJ46" s="3"/>
-    </row>
-    <row r="47" s="1" customFormat="1" spans="1:36">
+    </row>
+    <row r="47" s="1" customFormat="1" spans="1:35">
       <c r="A47" s="3"/>
       <c r="B47" s="4"/>
       <c r="C47" s="4"/>
@@ -3818,7 +3663,7 @@
       <c r="R47" s="4"/>
       <c r="S47" s="4"/>
       <c r="T47" s="4"/>
-      <c r="U47" s="4"/>
+      <c r="U47" s="3"/>
       <c r="V47" s="3"/>
       <c r="W47" s="3"/>
       <c r="X47" s="3"/>
@@ -3833,9 +3678,8 @@
       <c r="AG47" s="3"/>
       <c r="AH47" s="3"/>
       <c r="AI47" s="3"/>
-      <c r="AJ47" s="3"/>
-    </row>
-    <row r="48" spans="1:36">
+    </row>
+    <row r="48" spans="1:35">
       <c r="A48" s="3"/>
       <c r="B48" s="4"/>
       <c r="C48" s="4"/>
@@ -3856,7 +3700,7 @@
       <c r="R48" s="4"/>
       <c r="S48" s="4"/>
       <c r="T48" s="4"/>
-      <c r="U48" s="4"/>
+      <c r="U48" s="3"/>
       <c r="V48" s="3"/>
       <c r="W48" s="3"/>
       <c r="X48" s="3"/>
@@ -3871,9 +3715,8 @@
       <c r="AG48" s="3"/>
       <c r="AH48" s="3"/>
       <c r="AI48" s="3"/>
-      <c r="AJ48" s="3"/>
-    </row>
-    <row r="49" spans="1:36">
+    </row>
+    <row r="49" spans="1:35">
       <c r="A49" s="3"/>
       <c r="B49" s="4"/>
       <c r="C49" s="4"/>
@@ -3894,7 +3737,7 @@
       <c r="R49" s="4"/>
       <c r="S49" s="4"/>
       <c r="T49" s="4"/>
-      <c r="U49" s="4"/>
+      <c r="U49" s="3"/>
       <c r="V49" s="3"/>
       <c r="W49" s="3"/>
       <c r="X49" s="3"/>
@@ -3909,9 +3752,8 @@
       <c r="AG49" s="3"/>
       <c r="AH49" s="3"/>
       <c r="AI49" s="3"/>
-      <c r="AJ49" s="3"/>
-    </row>
-    <row r="50" spans="1:36">
+    </row>
+    <row r="50" spans="1:35">
       <c r="A50" s="3"/>
       <c r="B50" s="4"/>
       <c r="C50" s="4"/>
@@ -3932,7 +3774,7 @@
       <c r="R50" s="4"/>
       <c r="S50" s="4"/>
       <c r="T50" s="4"/>
-      <c r="U50" s="4"/>
+      <c r="U50" s="3"/>
       <c r="V50" s="3"/>
       <c r="W50" s="3"/>
       <c r="X50" s="3"/>
@@ -3947,9 +3789,8 @@
       <c r="AG50" s="3"/>
       <c r="AH50" s="3"/>
       <c r="AI50" s="3"/>
-      <c r="AJ50" s="3"/>
-    </row>
-    <row r="51" spans="1:36">
+    </row>
+    <row r="51" spans="1:35">
       <c r="A51" s="3"/>
       <c r="B51" s="4"/>
       <c r="C51" s="4"/>
@@ -3970,7 +3811,7 @@
       <c r="R51" s="4"/>
       <c r="S51" s="4"/>
       <c r="T51" s="4"/>
-      <c r="U51" s="4"/>
+      <c r="U51" s="3"/>
       <c r="V51" s="3"/>
       <c r="W51" s="3"/>
       <c r="X51" s="3"/>
@@ -3985,9 +3826,8 @@
       <c r="AG51" s="3"/>
       <c r="AH51" s="3"/>
       <c r="AI51" s="3"/>
-      <c r="AJ51" s="3"/>
-    </row>
-    <row r="52" spans="1:36">
+    </row>
+    <row r="52" spans="1:35">
       <c r="A52" s="3"/>
       <c r="B52" s="4"/>
       <c r="C52" s="4"/>
@@ -4008,7 +3848,7 @@
       <c r="R52" s="4"/>
       <c r="S52" s="4"/>
       <c r="T52" s="4"/>
-      <c r="U52" s="4"/>
+      <c r="U52" s="3"/>
       <c r="V52" s="3"/>
       <c r="W52" s="3"/>
       <c r="X52" s="3"/>
@@ -4023,9 +3863,8 @@
       <c r="AG52" s="3"/>
       <c r="AH52" s="3"/>
       <c r="AI52" s="3"/>
-      <c r="AJ52" s="3"/>
-    </row>
-    <row r="53" spans="1:36">
+    </row>
+    <row r="53" spans="1:35">
       <c r="A53" s="3"/>
       <c r="B53" s="4"/>
       <c r="C53" s="4"/>
@@ -4046,7 +3885,7 @@
       <c r="R53" s="4"/>
       <c r="S53" s="4"/>
       <c r="T53" s="4"/>
-      <c r="U53" s="4"/>
+      <c r="U53" s="3"/>
       <c r="V53" s="3"/>
       <c r="W53" s="3"/>
       <c r="X53" s="3"/>
@@ -4061,9 +3900,8 @@
       <c r="AG53" s="3"/>
       <c r="AH53" s="3"/>
       <c r="AI53" s="3"/>
-      <c r="AJ53" s="3"/>
-    </row>
-    <row r="54" spans="1:36">
+    </row>
+    <row r="54" spans="1:35">
       <c r="A54" s="3"/>
       <c r="B54" s="4"/>
       <c r="C54" s="4"/>
@@ -4084,7 +3922,7 @@
       <c r="R54" s="4"/>
       <c r="S54" s="4"/>
       <c r="T54" s="4"/>
-      <c r="U54" s="4"/>
+      <c r="U54" s="3"/>
       <c r="V54" s="3"/>
       <c r="W54" s="3"/>
       <c r="X54" s="3"/>
@@ -4099,9 +3937,8 @@
       <c r="AG54" s="3"/>
       <c r="AH54" s="3"/>
       <c r="AI54" s="3"/>
-      <c r="AJ54" s="3"/>
-    </row>
-    <row r="55" spans="1:36">
+    </row>
+    <row r="55" spans="1:35">
       <c r="A55" s="3"/>
       <c r="B55" s="4"/>
       <c r="C55" s="4"/>
@@ -4122,7 +3959,7 @@
       <c r="R55" s="4"/>
       <c r="S55" s="4"/>
       <c r="T55" s="4"/>
-      <c r="U55" s="4"/>
+      <c r="U55" s="3"/>
       <c r="V55" s="3"/>
       <c r="W55" s="3"/>
       <c r="X55" s="3"/>
@@ -4137,9 +3974,8 @@
       <c r="AG55" s="3"/>
       <c r="AH55" s="3"/>
       <c r="AI55" s="3"/>
-      <c r="AJ55" s="3"/>
-    </row>
-    <row r="56" spans="1:36">
+    </row>
+    <row r="56" spans="1:35">
       <c r="A56" s="3"/>
       <c r="B56" s="4"/>
       <c r="C56" s="4"/>
@@ -4160,7 +3996,7 @@
       <c r="R56" s="4"/>
       <c r="S56" s="4"/>
       <c r="T56" s="4"/>
-      <c r="U56" s="4"/>
+      <c r="U56" s="3"/>
       <c r="V56" s="3"/>
       <c r="W56" s="3"/>
       <c r="X56" s="3"/>
@@ -4175,9 +4011,8 @@
       <c r="AG56" s="3"/>
       <c r="AH56" s="3"/>
       <c r="AI56" s="3"/>
-      <c r="AJ56" s="3"/>
-    </row>
-    <row r="57" spans="1:36">
+    </row>
+    <row r="57" spans="1:35">
       <c r="A57" s="3"/>
       <c r="B57" s="4"/>
       <c r="C57" s="4"/>
@@ -4198,7 +4033,7 @@
       <c r="R57" s="4"/>
       <c r="S57" s="4"/>
       <c r="T57" s="4"/>
-      <c r="U57" s="4"/>
+      <c r="U57" s="3"/>
       <c r="V57" s="3"/>
       <c r="W57" s="3"/>
       <c r="X57" s="3"/>
@@ -4213,9 +4048,8 @@
       <c r="AG57" s="3"/>
       <c r="AH57" s="3"/>
       <c r="AI57" s="3"/>
-      <c r="AJ57" s="3"/>
-    </row>
-    <row r="58" spans="1:36">
+    </row>
+    <row r="58" spans="1:35">
       <c r="A58" s="3"/>
       <c r="B58" s="4"/>
       <c r="C58" s="4"/>
@@ -4236,7 +4070,7 @@
       <c r="R58" s="4"/>
       <c r="S58" s="4"/>
       <c r="T58" s="4"/>
-      <c r="U58" s="4"/>
+      <c r="U58" s="3"/>
       <c r="V58" s="3"/>
       <c r="W58" s="3"/>
       <c r="X58" s="3"/>
@@ -4251,9 +4085,8 @@
       <c r="AG58" s="3"/>
       <c r="AH58" s="3"/>
       <c r="AI58" s="3"/>
-      <c r="AJ58" s="3"/>
-    </row>
-    <row r="59" spans="1:36">
+    </row>
+    <row r="59" spans="1:35">
       <c r="A59" s="3"/>
       <c r="B59" s="4"/>
       <c r="C59" s="4"/>
@@ -4274,7 +4107,7 @@
       <c r="R59" s="4"/>
       <c r="S59" s="4"/>
       <c r="T59" s="4"/>
-      <c r="U59" s="4"/>
+      <c r="U59" s="3"/>
       <c r="V59" s="3"/>
       <c r="W59" s="3"/>
       <c r="X59" s="3"/>
@@ -4289,9 +4122,8 @@
       <c r="AG59" s="3"/>
       <c r="AH59" s="3"/>
       <c r="AI59" s="3"/>
-      <c r="AJ59" s="3"/>
-    </row>
-    <row r="60" spans="1:36">
+    </row>
+    <row r="60" spans="1:35">
       <c r="A60" s="3"/>
       <c r="B60" s="4"/>
       <c r="C60" s="4"/>
@@ -4312,7 +4144,7 @@
       <c r="R60" s="4"/>
       <c r="S60" s="4"/>
       <c r="T60" s="4"/>
-      <c r="U60" s="4"/>
+      <c r="U60" s="3"/>
       <c r="V60" s="3"/>
       <c r="W60" s="3"/>
       <c r="X60" s="3"/>
@@ -4327,9 +4159,8 @@
       <c r="AG60" s="3"/>
       <c r="AH60" s="3"/>
       <c r="AI60" s="3"/>
-      <c r="AJ60" s="3"/>
-    </row>
-    <row r="61" spans="1:36">
+    </row>
+    <row r="61" spans="1:35">
       <c r="A61" s="3"/>
       <c r="B61" s="4"/>
       <c r="C61" s="4"/>
@@ -4350,7 +4181,7 @@
       <c r="R61" s="4"/>
       <c r="S61" s="4"/>
       <c r="T61" s="4"/>
-      <c r="U61" s="4"/>
+      <c r="U61" s="3"/>
       <c r="V61" s="3"/>
       <c r="W61" s="3"/>
       <c r="X61" s="3"/>
@@ -4365,9 +4196,8 @@
       <c r="AG61" s="3"/>
       <c r="AH61" s="3"/>
       <c r="AI61" s="3"/>
-      <c r="AJ61" s="3"/>
-    </row>
-    <row r="62" spans="1:36">
+    </row>
+    <row r="62" spans="1:35">
       <c r="A62" s="3"/>
       <c r="B62" s="4"/>
       <c r="C62" s="4"/>
@@ -4388,7 +4218,7 @@
       <c r="R62" s="4"/>
       <c r="S62" s="4"/>
       <c r="T62" s="4"/>
-      <c r="U62" s="4"/>
+      <c r="U62" s="3"/>
       <c r="V62" s="3"/>
       <c r="W62" s="3"/>
       <c r="X62" s="3"/>
@@ -4403,9 +4233,8 @@
       <c r="AG62" s="3"/>
       <c r="AH62" s="3"/>
       <c r="AI62" s="3"/>
-      <c r="AJ62" s="3"/>
-    </row>
-    <row r="63" spans="1:36">
+    </row>
+    <row r="63" spans="1:35">
       <c r="A63" s="3"/>
       <c r="B63" s="4"/>
       <c r="C63" s="4"/>
@@ -4426,7 +4255,7 @@
       <c r="R63" s="4"/>
       <c r="S63" s="4"/>
       <c r="T63" s="4"/>
-      <c r="U63" s="4"/>
+      <c r="U63" s="3"/>
       <c r="V63" s="3"/>
       <c r="W63" s="3"/>
       <c r="X63" s="3"/>
@@ -4441,9 +4270,8 @@
       <c r="AG63" s="3"/>
       <c r="AH63" s="3"/>
       <c r="AI63" s="3"/>
-      <c r="AJ63" s="3"/>
-    </row>
-    <row r="64" spans="1:36">
+    </row>
+    <row r="64" spans="1:35">
       <c r="A64" s="3"/>
       <c r="B64" s="4"/>
       <c r="C64" s="4"/>
@@ -4464,7 +4292,7 @@
       <c r="R64" s="4"/>
       <c r="S64" s="4"/>
       <c r="T64" s="4"/>
-      <c r="U64" s="4"/>
+      <c r="U64" s="3"/>
       <c r="V64" s="3"/>
       <c r="W64" s="3"/>
       <c r="X64" s="3"/>
@@ -4479,9 +4307,8 @@
       <c r="AG64" s="3"/>
       <c r="AH64" s="3"/>
       <c r="AI64" s="3"/>
-      <c r="AJ64" s="3"/>
-    </row>
-    <row r="65" spans="1:36">
+    </row>
+    <row r="65" spans="1:35">
       <c r="A65" s="3"/>
       <c r="B65" s="4"/>
       <c r="C65" s="4"/>
@@ -4502,7 +4329,7 @@
       <c r="R65" s="4"/>
       <c r="S65" s="4"/>
       <c r="T65" s="4"/>
-      <c r="U65" s="4"/>
+      <c r="U65" s="3"/>
       <c r="V65" s="3"/>
       <c r="W65" s="3"/>
       <c r="X65" s="3"/>
@@ -4517,9 +4344,8 @@
       <c r="AG65" s="3"/>
       <c r="AH65" s="3"/>
       <c r="AI65" s="3"/>
-      <c r="AJ65" s="3"/>
-    </row>
-    <row r="66" spans="1:36">
+    </row>
+    <row r="66" spans="1:35">
       <c r="A66" s="3"/>
       <c r="B66" s="4"/>
       <c r="C66" s="4"/>
@@ -4540,7 +4366,7 @@
       <c r="R66" s="4"/>
       <c r="S66" s="4"/>
       <c r="T66" s="4"/>
-      <c r="U66" s="4"/>
+      <c r="U66" s="3"/>
       <c r="V66" s="3"/>
       <c r="W66" s="3"/>
       <c r="X66" s="3"/>
@@ -4555,9 +4381,8 @@
       <c r="AG66" s="3"/>
       <c r="AH66" s="3"/>
       <c r="AI66" s="3"/>
-      <c r="AJ66" s="3"/>
-    </row>
-    <row r="67" spans="1:36">
+    </row>
+    <row r="67" spans="1:35">
       <c r="A67" s="3"/>
       <c r="B67" s="4"/>
       <c r="C67" s="4"/>
@@ -4578,7 +4403,7 @@
       <c r="R67" s="4"/>
       <c r="S67" s="4"/>
       <c r="T67" s="4"/>
-      <c r="U67" s="4"/>
+      <c r="U67" s="3"/>
       <c r="V67" s="3"/>
       <c r="W67" s="3"/>
       <c r="X67" s="3"/>
@@ -4593,9 +4418,8 @@
       <c r="AG67" s="3"/>
       <c r="AH67" s="3"/>
       <c r="AI67" s="3"/>
-      <c r="AJ67" s="3"/>
-    </row>
-    <row r="68" spans="1:36">
+    </row>
+    <row r="68" spans="1:35">
       <c r="A68" s="3"/>
       <c r="B68" s="4"/>
       <c r="C68" s="4"/>
@@ -4616,7 +4440,7 @@
       <c r="R68" s="4"/>
       <c r="S68" s="4"/>
       <c r="T68" s="4"/>
-      <c r="U68" s="4"/>
+      <c r="U68" s="3"/>
       <c r="V68" s="3"/>
       <c r="W68" s="3"/>
       <c r="X68" s="3"/>
@@ -4631,9 +4455,8 @@
       <c r="AG68" s="3"/>
       <c r="AH68" s="3"/>
       <c r="AI68" s="3"/>
-      <c r="AJ68" s="3"/>
-    </row>
-    <row r="69" spans="1:36">
+    </row>
+    <row r="69" spans="1:35">
       <c r="A69" s="3"/>
       <c r="B69" s="4"/>
       <c r="C69" s="4"/>
@@ -4654,7 +4477,7 @@
       <c r="R69" s="4"/>
       <c r="S69" s="4"/>
       <c r="T69" s="4"/>
-      <c r="U69" s="4"/>
+      <c r="U69" s="3"/>
       <c r="V69" s="3"/>
       <c r="W69" s="3"/>
       <c r="X69" s="3"/>
@@ -4669,9 +4492,8 @@
       <c r="AG69" s="3"/>
       <c r="AH69" s="3"/>
       <c r="AI69" s="3"/>
-      <c r="AJ69" s="3"/>
-    </row>
-    <row r="70" spans="1:36">
+    </row>
+    <row r="70" spans="1:35">
       <c r="A70" s="3"/>
       <c r="B70" s="4"/>
       <c r="C70" s="4"/>
@@ -4692,7 +4514,7 @@
       <c r="R70" s="4"/>
       <c r="S70" s="4"/>
       <c r="T70" s="4"/>
-      <c r="U70" s="4"/>
+      <c r="U70" s="3"/>
       <c r="V70" s="3"/>
       <c r="W70" s="3"/>
       <c r="X70" s="3"/>
@@ -4707,9 +4529,8 @@
       <c r="AG70" s="3"/>
       <c r="AH70" s="3"/>
       <c r="AI70" s="3"/>
-      <c r="AJ70" s="3"/>
-    </row>
-    <row r="71" spans="1:36">
+    </row>
+    <row r="71" spans="1:35">
       <c r="A71" s="3"/>
       <c r="B71" s="4"/>
       <c r="C71" s="4"/>
@@ -4730,7 +4551,7 @@
       <c r="R71" s="4"/>
       <c r="S71" s="4"/>
       <c r="T71" s="4"/>
-      <c r="U71" s="4"/>
+      <c r="U71" s="3"/>
       <c r="V71" s="3"/>
       <c r="W71" s="3"/>
       <c r="X71" s="3"/>
@@ -4745,9 +4566,8 @@
       <c r="AG71" s="3"/>
       <c r="AH71" s="3"/>
       <c r="AI71" s="3"/>
-      <c r="AJ71" s="3"/>
-    </row>
-    <row r="72" spans="1:36">
+    </row>
+    <row r="72" spans="1:35">
       <c r="A72" s="3"/>
       <c r="B72" s="4"/>
       <c r="C72" s="4"/>
@@ -4768,7 +4588,7 @@
       <c r="R72" s="4"/>
       <c r="S72" s="4"/>
       <c r="T72" s="4"/>
-      <c r="U72" s="4"/>
+      <c r="U72" s="3"/>
       <c r="V72" s="3"/>
       <c r="W72" s="3"/>
       <c r="X72" s="3"/>
@@ -4783,9 +4603,8 @@
       <c r="AG72" s="3"/>
       <c r="AH72" s="3"/>
       <c r="AI72" s="3"/>
-      <c r="AJ72" s="3"/>
-    </row>
-    <row r="73" spans="1:36">
+    </row>
+    <row r="73" spans="1:35">
       <c r="A73" s="3"/>
       <c r="B73" s="4"/>
       <c r="C73" s="4"/>
@@ -4806,7 +4625,7 @@
       <c r="R73" s="4"/>
       <c r="S73" s="4"/>
       <c r="T73" s="4"/>
-      <c r="U73" s="4"/>
+      <c r="U73" s="3"/>
       <c r="V73" s="3"/>
       <c r="W73" s="3"/>
       <c r="X73" s="3"/>
@@ -4821,9 +4640,8 @@
       <c r="AG73" s="3"/>
       <c r="AH73" s="3"/>
       <c r="AI73" s="3"/>
-      <c r="AJ73" s="3"/>
-    </row>
-    <row r="74" spans="1:36">
+    </row>
+    <row r="74" spans="1:35">
       <c r="A74" s="3"/>
       <c r="B74" s="4"/>
       <c r="C74" s="4"/>
@@ -4844,7 +4662,7 @@
       <c r="R74" s="4"/>
       <c r="S74" s="4"/>
       <c r="T74" s="4"/>
-      <c r="U74" s="4"/>
+      <c r="U74" s="3"/>
       <c r="V74" s="3"/>
       <c r="W74" s="3"/>
       <c r="X74" s="3"/>
@@ -4859,9 +4677,8 @@
       <c r="AG74" s="3"/>
       <c r="AH74" s="3"/>
       <c r="AI74" s="3"/>
-      <c r="AJ74" s="3"/>
-    </row>
-    <row r="75" spans="1:36">
+    </row>
+    <row r="75" spans="1:35">
       <c r="A75" s="3"/>
       <c r="B75" s="4"/>
       <c r="C75" s="4"/>
@@ -4882,7 +4699,7 @@
       <c r="R75" s="4"/>
       <c r="S75" s="4"/>
       <c r="T75" s="4"/>
-      <c r="U75" s="4"/>
+      <c r="U75" s="3"/>
       <c r="V75" s="3"/>
       <c r="W75" s="3"/>
       <c r="X75" s="3"/>
@@ -4897,9 +4714,8 @@
       <c r="AG75" s="3"/>
       <c r="AH75" s="3"/>
       <c r="AI75" s="3"/>
-      <c r="AJ75" s="3"/>
-    </row>
-    <row r="76" spans="1:36">
+    </row>
+    <row r="76" spans="1:35">
       <c r="A76" s="3"/>
       <c r="B76" s="4"/>
       <c r="C76" s="4"/>
@@ -4920,7 +4736,7 @@
       <c r="R76" s="4"/>
       <c r="S76" s="4"/>
       <c r="T76" s="4"/>
-      <c r="U76" s="4"/>
+      <c r="U76" s="3"/>
       <c r="V76" s="3"/>
       <c r="W76" s="3"/>
       <c r="X76" s="3"/>
@@ -4935,9 +4751,8 @@
       <c r="AG76" s="3"/>
       <c r="AH76" s="3"/>
       <c r="AI76" s="3"/>
-      <c r="AJ76" s="3"/>
-    </row>
-    <row r="77" spans="1:36">
+    </row>
+    <row r="77" spans="1:35">
       <c r="A77" s="3"/>
       <c r="B77" s="4"/>
       <c r="C77" s="4"/>
@@ -4958,7 +4773,7 @@
       <c r="R77" s="4"/>
       <c r="S77" s="4"/>
       <c r="T77" s="4"/>
-      <c r="U77" s="4"/>
+      <c r="U77" s="3"/>
       <c r="V77" s="3"/>
       <c r="W77" s="3"/>
       <c r="X77" s="3"/>
@@ -4973,9 +4788,8 @@
       <c r="AG77" s="3"/>
       <c r="AH77" s="3"/>
       <c r="AI77" s="3"/>
-      <c r="AJ77" s="3"/>
-    </row>
-    <row r="78" spans="1:36">
+    </row>
+    <row r="78" spans="1:35">
       <c r="A78" s="3"/>
       <c r="B78" s="4"/>
       <c r="C78" s="4"/>
@@ -4996,7 +4810,7 @@
       <c r="R78" s="4"/>
       <c r="S78" s="4"/>
       <c r="T78" s="4"/>
-      <c r="U78" s="4"/>
+      <c r="U78" s="3"/>
       <c r="V78" s="3"/>
       <c r="W78" s="3"/>
       <c r="X78" s="3"/>
@@ -5011,195 +4825,194 @@
       <c r="AG78" s="3"/>
       <c r="AH78" s="3"/>
       <c r="AI78" s="3"/>
-      <c r="AJ78" s="3"/>
-    </row>
-    <row r="86" spans="1:25">
+    </row>
+    <row r="86" spans="1:24">
       <c r="A86" s="2"/>
       <c r="B86" s="2"/>
       <c r="C86" s="2"/>
       <c r="D86" s="2"/>
-      <c r="T86" s="2"/>
+      <c r="S86" s="2"/>
+      <c r="U86" s="2"/>
       <c r="V86" s="2"/>
       <c r="W86" s="2"/>
       <c r="X86" s="2"/>
-      <c r="Y86" s="2"/>
-    </row>
-    <row r="87" spans="1:25">
+    </row>
+    <row r="87" spans="1:24">
       <c r="A87" s="2"/>
       <c r="B87" s="2"/>
       <c r="C87" s="2"/>
       <c r="D87" s="2"/>
       <c r="E87" s="2"/>
+      <c r="S87" s="2"/>
       <c r="T87" s="2"/>
       <c r="U87" s="2"/>
       <c r="V87" s="2"/>
       <c r="W87" s="2"/>
       <c r="X87" s="2"/>
-      <c r="Y87" s="2"/>
-    </row>
-    <row r="88" spans="1:25">
+    </row>
+    <row r="88" spans="1:24">
       <c r="A88" s="2"/>
       <c r="B88" s="2"/>
       <c r="C88" s="2"/>
       <c r="D88" s="2"/>
+      <c r="S88" s="2"/>
       <c r="T88" s="2"/>
       <c r="U88" s="2"/>
       <c r="V88" s="2"/>
       <c r="W88" s="2"/>
       <c r="X88" s="2"/>
-      <c r="Y88" s="2"/>
-    </row>
-    <row r="89" spans="1:25">
+    </row>
+    <row r="89" spans="1:24">
       <c r="A89" s="2"/>
       <c r="B89" s="2"/>
       <c r="C89" s="2"/>
       <c r="D89" s="2"/>
+      <c r="S89" s="2"/>
       <c r="T89" s="2"/>
       <c r="U89" s="2"/>
       <c r="V89" s="2"/>
       <c r="W89" s="2"/>
       <c r="X89" s="2"/>
-      <c r="Y89" s="2"/>
-    </row>
-    <row r="90" spans="1:25">
+    </row>
+    <row r="90" spans="1:24">
       <c r="A90" s="2"/>
       <c r="B90" s="2"/>
       <c r="C90" s="2"/>
       <c r="D90" s="2"/>
+      <c r="S90" s="2"/>
       <c r="T90" s="2"/>
       <c r="U90" s="2"/>
       <c r="V90" s="2"/>
       <c r="W90" s="2"/>
       <c r="X90" s="2"/>
-      <c r="Y90" s="2"/>
-    </row>
-    <row r="91" spans="1:25">
+    </row>
+    <row r="91" spans="1:24">
       <c r="A91" s="2"/>
       <c r="B91" s="2"/>
       <c r="C91" s="2"/>
       <c r="D91" s="2"/>
+      <c r="S91" s="2"/>
       <c r="T91" s="2"/>
       <c r="U91" s="2"/>
       <c r="V91" s="2"/>
       <c r="W91" s="2"/>
       <c r="X91" s="2"/>
-      <c r="Y91" s="2"/>
-    </row>
-    <row r="92" spans="1:25">
+    </row>
+    <row r="92" spans="1:24">
       <c r="A92" s="2"/>
       <c r="B92" s="2"/>
       <c r="C92" s="2"/>
       <c r="D92" s="2"/>
+      <c r="S92" s="2"/>
       <c r="T92" s="2"/>
       <c r="U92" s="2"/>
       <c r="V92" s="2"/>
       <c r="W92" s="2"/>
       <c r="X92" s="2"/>
-      <c r="Y92" s="2"/>
-    </row>
-    <row r="93" spans="1:25">
+    </row>
+    <row r="93" spans="1:24">
       <c r="A93" s="2"/>
       <c r="B93" s="2"/>
       <c r="C93" s="2"/>
       <c r="D93" s="2"/>
+      <c r="S93" s="2"/>
       <c r="T93" s="2"/>
       <c r="U93" s="2"/>
       <c r="V93" s="2"/>
       <c r="W93" s="2"/>
       <c r="X93" s="2"/>
-      <c r="Y93" s="2"/>
-    </row>
-    <row r="94" spans="1:25">
+    </row>
+    <row r="94" spans="1:24">
       <c r="A94" s="2"/>
       <c r="B94" s="2"/>
       <c r="C94" s="2"/>
       <c r="D94" s="2"/>
+      <c r="S94" s="2"/>
       <c r="T94" s="2"/>
       <c r="U94" s="2"/>
       <c r="V94" s="2"/>
       <c r="W94" s="2"/>
       <c r="X94" s="2"/>
-      <c r="Y94" s="2"/>
-    </row>
-    <row r="95" spans="1:25">
+    </row>
+    <row r="95" spans="1:24">
       <c r="A95" s="2"/>
       <c r="B95" s="2"/>
       <c r="C95" s="2"/>
       <c r="D95" s="2"/>
+      <c r="S95" s="2"/>
       <c r="T95" s="2"/>
       <c r="U95" s="2"/>
       <c r="V95" s="2"/>
       <c r="W95" s="2"/>
       <c r="X95" s="2"/>
-      <c r="Y95" s="2"/>
-    </row>
-    <row r="96" spans="1:25">
+    </row>
+    <row r="96" spans="1:24">
       <c r="A96" s="2"/>
       <c r="B96" s="2"/>
       <c r="C96" s="2"/>
       <c r="D96" s="2"/>
+      <c r="S96" s="2"/>
       <c r="T96" s="2"/>
       <c r="U96" s="2"/>
       <c r="V96" s="2"/>
       <c r="W96" s="2"/>
       <c r="X96" s="2"/>
-      <c r="Y96" s="2"/>
-    </row>
-    <row r="97" spans="1:25">
+    </row>
+    <row r="97" spans="1:24">
       <c r="A97" s="2"/>
       <c r="B97" s="2"/>
       <c r="C97" s="2"/>
       <c r="D97" s="2"/>
+      <c r="S97" s="2"/>
       <c r="T97" s="2"/>
       <c r="U97" s="2"/>
       <c r="V97" s="2"/>
       <c r="W97" s="2"/>
       <c r="X97" s="2"/>
-      <c r="Y97" s="2"/>
-    </row>
-    <row r="98" spans="1:25">
+    </row>
+    <row r="98" spans="1:24">
       <c r="A98" s="2"/>
       <c r="B98" s="2"/>
       <c r="C98" s="2"/>
       <c r="D98" s="2"/>
+      <c r="S98" s="2"/>
       <c r="T98" s="2"/>
       <c r="U98" s="2"/>
       <c r="V98" s="2"/>
       <c r="W98" s="2"/>
       <c r="X98" s="2"/>
-      <c r="Y98" s="2"/>
-    </row>
-    <row r="99" spans="1:25">
+    </row>
+    <row r="99" spans="1:24">
       <c r="A99" s="2"/>
       <c r="B99" s="2"/>
       <c r="C99" s="2"/>
       <c r="D99" s="2"/>
+      <c r="S99" s="2"/>
       <c r="T99" s="2"/>
       <c r="U99" s="2"/>
       <c r="V99" s="2"/>
       <c r="W99" s="2"/>
       <c r="X99" s="2"/>
-      <c r="Y99" s="2"/>
     </row>
   </sheetData>
-  <dataValidations count="14">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="O2:O1048576">
-      <formula1>"R_TYPE,I_TYPE,S_TYPE,B_TYPE,U_TYPE,J_TYPE,ICSR_TYPE,FENCE_TYPE,N_TYPE"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="M29 M30 M31 M39 M40 M41 M42 M43 M2:M28 M32:M38 M44:M1048576">
-      <formula1>"CSR_W,CSR_S,CSR_C,CSR_P,CSR_XX"</formula1>
-    </dataValidation>
+  <dataValidations count="13">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H29 H30 H31 H40 H41 H42 H43 H10:H28 H32:H39 H44:H1048576">
       <formula1>"WB_ALU,WB_MEM,WB_PC4,WB_XX,WB_CSR"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F6 F15 F18 F19 F20 F21 F24 F25 F26 F27 F28 F29 F30 F31 F32 F33 F36 F37 F38 F39 F40 F41 F42 F43 F2:F5 F7:F14 F16:F17 F22:F23 F34:F35 F44:F1048576">
+      <formula1>"ALU_ADD,ALU_SUB,ALU_AND,ALU_OR,ALU_XOR,ALU_SLL,ALU_SRL,ALU_SLT,ALU_SLTU,ALU_COPY_A,ALU_COPY_B,ALU_SRA"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L5 L6 L7 L10 L11 L14 L15 L16 L17 L18 L19 L20 L21 L22 L23 L24 L25 L26 L27 L28 L29 L30 L31 L32 L33 L34 L35 L36 L37 L38 L39 L40 L41 L42 L43 L2:L4 L8:L9 L12:L13 L44:L1048576">
+      <formula1>"BR_EQ,BR_NE,BR_LTU,BR_GE,BR_GEU,BR_LT,BR_XX"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C29 C30 C31 C43 C2:C28 C32:C42 C44:C1048576">
       <formula1>"PC_4,PC_0,PC_ALU,PC_CSR"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E4 E5 E6 E7 E8 E9 E10 E11 E12 E13 E14 E15 E16 E17 E18 E19 E20 E21 E22 E23 E24 E25 E26 E27 E28 E29 E30 E31 E32 E33 E34 E35 E36 E37 E38 E39 E40 E41 E42 E43 E2:E3 E44:E1048576">
-      <formula1>"B_IMM,B_RS2"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="N4 N5 N6 N7 N8 N9 N10 N11 N12 N13 N14 N15 N16 N17 N18 N19 N20 N21 N22 N23 N24 N25 N26 N27 N28 N29 N30 N31 N32 N33 N34 N35 N36 N37 N38 N39 N40 N41 N42 N43 N2:N3 N44:N1048576">
+      <formula1>"INST_VALID,INST_INVALID"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G4 G5 G6 G7 G8 G9 G10 G11 G12 G13 G14 G15 G16 G17 G18 G19 G20 G21 G22 G23 G24 G25 G26 G27 G28 G29 G30 G31 G32 G33 G34 G35 G36 G37 G38 G39 G40 G41 G42 G43 G2:G3 G44:G1048576">
-      <formula1>"IMM_I,IMM_J,IMM_U,IMM_S,IMM_B"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D4 D5 D6 D7 D8 D9 D10 D11 D12 D13 D14 D15 D16 D17 D18 D19 D20 D21 D22 D23 D24 D25 D26 D27 D28 D29 D30 D31 D32 D33 D34 D35 D36 D37 D38 D39 D40 D41 D42 D43 D2:D3 D44:D1048576">
+      <formula1>"A_PC,A_RS1"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J5 J6 J7 J8 J9 J10 J11 J12 J13 J14 J15 J16 J17 J18 J19 J20 J21 J22 J23 J24 J25 J26 J27 J28 J29 J30 J31 J32 J33 J34 J35 J36 J37 J38 J39 J40 J41 J42 J43 J2:J4 J44:J1048576">
       <formula1>"ST_SW,ST_SH,ST_SB,ST_XX"</formula1>
@@ -5207,23 +5020,20 @@
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H5 H6 H7 H8 H9 H2:H4">
       <formula1>"WB_ALU,WB_MEM,WB_PC4,WB_XX"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L5 L6 L7 L10 L11 L14 L15 L16 L17 L18 L19 L20 L21 L22 L23 L24 L25 L26 L27 L28 L29 L30 L31 L32 L33 L34 L35 L36 L37 L38 L39 L40 L41 L42 L43 L2:L4 L8:L9 L12:L13 L44:L1048576">
-      <formula1>"BR_EQ,BR_NE,BR_LTU,BR_GE,BR_GEU,BR_LT,BR_XX"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K4 K5 K6 K7 K8 K9 K10 K11 K12 K13 K14 K15 K16 K17 K18 K19 K20 K21 K22 K23 K24 K25 K26 K27 K28 K29 K30 K31 K32 K33 K34 K35 K36 K37 K38 K39 K40 K41 K42 K43 K2:K3 K44:K1048576">
+      <formula1>"MASK_XX,MASK_B,MASK_H,MASK_W,MASK_D"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="N4 N5 N6 N7 N8 N9 N10 N11 N12 N13 N14 N15 N16 N17 N18 N19 N20 N21 N22 N23 N24 N25 N26 N27 N28 N29 N30 N31 N32 N33 N34 N35 N36 N37 N38 N39 N40 N41 N42 N43 N2:N3 N44:N1048576">
-      <formula1>"INST_VALID,INST_INVALID"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E4 E5 E6 E7 E8 E9 E10 E11 E12 E13 E14 E15 E16 E17 E18 E19 E20 E21 E22 E23 E24 E25 E26 E27 E28 E29 E30 E31 E32 E33 E34 E35 E36 E37 E38 E39 E40 E41 E42 E43 E2:E3 E44:E1048576">
+      <formula1>"B_IMM,B_RS2"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="M29 M30 M31 M39 M40 M41 M42 M43 M2:M28 M32:M38 M44:M1048576">
+      <formula1>"CSR_W,CSR_S,CSR_C,CSR_P,CSR_XX"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I4 I5 I6 I7 I8 I9 I10 I11 I12 I13 I14 I15 I16 I17 I18 I19 I20 I21 I22 I23 I24 I25 I26 I27 I28 I29 I30 I31 I32 I33 I34 I35 I36 I37 I38 I39 I40 I41 I42 I43 I2:I3 I44:I1048576">
       <formula1>"LD_LB,LD_LH,LD_LW,LD_LBU,LD_LHU,LD_XX"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F6 F15 F18 F19 F20 F21 F24 F25 F26 F27 F28 F29 F30 F31 F32 F33 F36 F37 F38 F39 F40 F41 F42 F43 F2:F5 F7:F14 F16:F17 F22:F23 F34:F35 F44:F1048576">
-      <formula1>"ALU_ADD,ALU_SUB,ALU_AND,ALU_OR,ALU_XOR,ALU_SLL,ALU_SRL,ALU_SLT,ALU_SLTU,ALU_COPY_A,ALU_COPY_B,ALU_SRA"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K4 K5 K6 K7 K8 K9 K10 K11 K12 K13 K14 K15 K16 K17 K18 K19 K20 K21 K22 K23 K24 K25 K26 K27 K28 K29 K30 K31 K32 K33 K34 K35 K36 K37 K38 K39 K40 K41 K42 K43 K2:K3 K44:K1048576">
-      <formula1>"MASK_XX,MASK_B,MASK_H,MASK_W,MASK_D"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D4 D5 D6 D7 D8 D9 D10 D11 D12 D13 D14 D15 D16 D17 D18 D19 D20 D21 D22 D23 D24 D25 D26 D27 D28 D29 D30 D31 D32 D33 D34 D35 D36 D37 D38 D39 D40 D41 D42 D43 D2:D3 D44:D1048576">
-      <formula1>"A_PC,A_RS1"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G4 G5 G6 G7 G8 G9 G10 G11 G12 G13 G14 G15 G16 G17 G18 G19 G20 G21 G22 G23 G24 G25 G26 G27 G28 G29 G30 G31 G32 G33 G34 G35 G36 G37 G38 G39 G40 G41 G42 G43 G2:G3 G44:G1048576">
+      <formula1>"IMM_I,IMM_J,IMM_U,IMM_S,IMM_B"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
> compile NEMU ysyx_23060246 韩炳晋 Linux archlinux 6.12.17-1-lts #1 SMP PREEMPT_DYNAMIC Thu, 27 Feb 2025 14:12:30 +0000 x86_64 GNU/Linux  14:24:18 up 18:14,  1 user,  load average: 0.41, 1.45, 2.24
</commit_message>
<xml_diff>
--- a/npc/tools/control_gen/control_table.xlsx
+++ b/npc/tools/control_gen/control_table.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="311" uniqueCount="112">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="355" uniqueCount="119">
   <si>
     <t>comment</t>
   </si>
@@ -76,6 +76,9 @@
     <t>INST_VALID</t>
   </si>
   <si>
+    <t>U_TYPE</t>
+  </si>
+  <si>
     <t>auipc</t>
   </si>
   <si>
@@ -94,6 +97,9 @@
     <t>IMM_I</t>
   </si>
   <si>
+    <t>I_TYPE</t>
+  </si>
+  <si>
     <t>andi</t>
   </si>
   <si>
@@ -127,6 +133,9 @@
     <t>IMM_J</t>
   </si>
   <si>
+    <t>J_TYPE</t>
+  </si>
+  <si>
     <t>sb</t>
   </si>
   <si>
@@ -139,6 +148,9 @@
     <t>MASK_B</t>
   </si>
   <si>
+    <t>S_TYPE</t>
+  </si>
+  <si>
     <t>sh</t>
   </si>
   <si>
@@ -199,6 +211,9 @@
     <t>BR_NE</t>
   </si>
   <si>
+    <t>B_TYPE</t>
+  </si>
+  <si>
     <t>beq</t>
   </si>
   <si>
@@ -247,6 +262,9 @@
     <t>B_RS2</t>
   </si>
   <si>
+    <t>R_TYPE</t>
+  </si>
+  <si>
     <t>sra</t>
   </si>
   <si>
@@ -320,6 +338,9 @@
   </si>
   <si>
     <t>CSR_P</t>
+  </si>
+  <si>
+    <t>N_TYPE</t>
   </si>
   <si>
     <t>mret</t>
@@ -358,9 +379,9 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="4">
     <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="42" formatCode="_ &quot;￥&quot;* #,##0_ ;_ &quot;￥&quot;* \-#,##0_ ;_ &quot;￥&quot;* &quot;-&quot;_ ;_ @_ "/>
     <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="41" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="42" formatCode="_ &quot;￥&quot;* #,##0_ ;_ &quot;￥&quot;* \-#,##0_ ;_ &quot;￥&quot;* &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
   <fonts count="22">
     <font>
@@ -378,21 +399,6 @@
     </font>
     <font>
       <sz val="10.8"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="3"/>
       <name val="宋体"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -419,6 +425,29 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF0000FF"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="3"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <b/>
       <sz val="18"/>
       <color theme="3"/>
@@ -432,22 +461,6 @@
       <color rgb="FF800080"/>
       <name val="宋体"/>
       <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="11"/>
-      <color rgb="FF7F7F7F"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="15"/>
-      <color theme="3"/>
-      <name val="宋体"/>
-      <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -476,14 +489,7 @@
     <font>
       <b/>
       <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF3F3F76"/>
+      <color theme="1"/>
       <name val="宋体"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -497,6 +503,21 @@
     </font>
     <font>
       <b/>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF006100"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="13"/>
       <color theme="3"/>
       <name val="宋体"/>
@@ -504,24 +525,24 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF0000FF"/>
+      <b/>
+      <sz val="15"/>
+      <color theme="3"/>
       <name val="宋体"/>
-      <charset val="0"/>
+      <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
+      <i/>
       <sz val="11"/>
-      <color theme="1"/>
+      <color rgb="FF7F7F7F"/>
       <name val="宋体"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FF006100"/>
+      <color rgb="FF3F3F76"/>
       <name val="宋体"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -536,7 +557,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.599993896298105"/>
+        <fgColor theme="4" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -554,19 +581,67 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="9"/>
+        <fgColor theme="5" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="7" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -584,25 +659,61 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor theme="4" tint="0.799981688894314"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.799981688894314"/>
+        <fgColor theme="6" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.799981688894314"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -614,37 +725,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.399975585192419"/>
+        <fgColor rgb="FFFFCC99"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -656,67 +737,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor theme="9" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -727,24 +748,6 @@
       <right/>
       <top/>
       <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="double">
-        <color rgb="FFFF8001"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4" tint="0.499984740745262"/>
-      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -766,8 +769,17 @@
       <left/>
       <right/>
       <top/>
+      <bottom style="double">
+        <color rgb="FFFF8001"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
       <bottom style="medium">
-        <color theme="4"/>
+        <color theme="4" tint="0.499984740745262"/>
       </bottom>
       <diagonal/>
     </border>
@@ -802,6 +814,17 @@
       <diagonal/>
     </border>
     <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="4"/>
+      </top>
+      <bottom style="double">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
       <left style="thin">
         <color rgb="FF7F7F7F"/>
       </left>
@@ -819,10 +842,8 @@
     <border>
       <left/>
       <right/>
-      <top style="thin">
-        <color theme="4"/>
-      </top>
-      <bottom style="double">
+      <top/>
+      <bottom style="medium">
         <color theme="4"/>
       </bottom>
       <diagonal/>
@@ -832,148 +853,148 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="10" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="4" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="30" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="4" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="7" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="8" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="7" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="15" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="17" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="15" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
@@ -1318,7 +1339,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:AI99"/>
+  <dimension ref="A1:AJ99"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
     <col min="1" max="1" width="13.1" customWidth="1"/>
@@ -1331,18 +1352,18 @@
     <col min="8" max="10" width="11.9833333333333" customWidth="1"/>
     <col min="11" max="11" width="15.075" customWidth="1"/>
     <col min="12" max="14" width="12.1083333333333" customWidth="1"/>
-    <col min="15" max="15" width="10.8583333333333" customWidth="1"/>
-    <col min="17" max="17" width="14.2166666666667" customWidth="1"/>
-    <col min="18" max="18" width="11.8083333333333" customWidth="1"/>
-    <col min="19" max="19" width="10.6" customWidth="1"/>
-    <col min="20" max="20" width="9.70833333333333" customWidth="1"/>
-    <col min="21" max="21" width="11.1666666666667" customWidth="1"/>
-    <col min="22" max="22" width="11.4083333333333" customWidth="1"/>
-    <col min="23" max="23" width="12.0583333333333" customWidth="1"/>
-    <col min="24" max="24" width="15.575" customWidth="1"/>
+    <col min="15" max="16" width="10.8583333333333" customWidth="1"/>
+    <col min="18" max="18" width="14.2166666666667" customWidth="1"/>
+    <col min="19" max="19" width="11.8083333333333" customWidth="1"/>
+    <col min="20" max="20" width="10.6" customWidth="1"/>
+    <col min="21" max="21" width="9.70833333333333" customWidth="1"/>
+    <col min="22" max="22" width="11.1666666666667" customWidth="1"/>
+    <col min="23" max="23" width="11.4083333333333" customWidth="1"/>
+    <col min="24" max="24" width="12.0583333333333" customWidth="1"/>
+    <col min="25" max="25" width="15.575" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="15" customHeight="1" spans="1:23">
+    <row r="1" ht="15" customHeight="1" spans="1:24">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1385,15 +1406,18 @@
       <c r="N1" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="2"/>
+      <c r="O1" s="2" t="s">
+        <v>1</v>
+      </c>
       <c r="P1" s="2"/>
       <c r="Q1" s="2"/>
       <c r="R1" s="2"/>
       <c r="S1" s="2"/>
       <c r="T1" s="2"/>
-      <c r="W1" s="6"/>
-    </row>
-    <row r="2" spans="1:35">
+      <c r="U1" s="2"/>
+      <c r="X1" s="6"/>
+    </row>
+    <row r="2" spans="1:36">
       <c r="A2" s="3"/>
       <c r="B2" s="4" t="s">
         <v>14</v>
@@ -1420,13 +1444,15 @@
       <c r="N2" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O2" s="4"/>
+      <c r="O2" s="4" t="s">
+        <v>20</v>
+      </c>
       <c r="P2" s="4"/>
       <c r="Q2" s="4"/>
       <c r="R2" s="4"/>
       <c r="S2" s="4"/>
       <c r="T2" s="4"/>
-      <c r="U2" s="3"/>
+      <c r="U2" s="4"/>
       <c r="V2" s="3"/>
       <c r="W2" s="3"/>
       <c r="X2" s="3"/>
@@ -1441,21 +1467,22 @@
       <c r="AG2" s="3"/>
       <c r="AH2" s="3"/>
       <c r="AI2" s="3"/>
-    </row>
-    <row r="3" spans="1:35">
+      <c r="AJ2" s="3"/>
+    </row>
+    <row r="3" spans="1:36">
       <c r="A3" s="3"/>
       <c r="B3" s="4" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C3" s="2"/>
       <c r="D3" s="4" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E3" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="G3" s="4" t="s">
         <v>17</v>
@@ -1471,13 +1498,15 @@
       <c r="N3" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O3" s="4"/>
+      <c r="O3" s="4" t="s">
+        <v>20</v>
+      </c>
       <c r="P3" s="4"/>
       <c r="Q3" s="4"/>
       <c r="R3" s="4"/>
       <c r="S3" s="4"/>
       <c r="T3" s="4"/>
-      <c r="U3" s="3"/>
+      <c r="U3" s="4"/>
       <c r="V3" s="3"/>
       <c r="W3" s="3"/>
       <c r="X3" s="3"/>
@@ -1492,24 +1521,25 @@
       <c r="AG3" s="3"/>
       <c r="AH3" s="3"/>
       <c r="AI3" s="3"/>
-    </row>
-    <row r="4" spans="1:35">
+      <c r="AJ3" s="3"/>
+    </row>
+    <row r="4" spans="1:36">
       <c r="A4" s="3"/>
       <c r="B4" s="4" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C4" s="2"/>
       <c r="D4" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E4" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="H4" s="4" t="s">
         <v>18</v>
@@ -1522,13 +1552,15 @@
       <c r="N4" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O4" s="4"/>
+      <c r="O4" s="4" t="s">
+        <v>27</v>
+      </c>
       <c r="P4" s="4"/>
       <c r="Q4" s="4"/>
       <c r="R4" s="4"/>
       <c r="S4" s="4"/>
       <c r="T4" s="4"/>
-      <c r="U4" s="3"/>
+      <c r="U4" s="4"/>
       <c r="V4" s="3"/>
       <c r="W4" s="3"/>
       <c r="X4" s="3"/>
@@ -1543,24 +1575,25 @@
       <c r="AG4" s="3"/>
       <c r="AH4" s="3"/>
       <c r="AI4" s="3"/>
-    </row>
-    <row r="5" spans="1:35">
+      <c r="AJ4" s="3"/>
+    </row>
+    <row r="5" spans="1:36">
       <c r="A5" s="3"/>
       <c r="B5" s="4" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="C5" s="2"/>
       <c r="D5" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E5" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="H5" s="4" t="s">
         <v>18</v>
@@ -1573,13 +1606,15 @@
       <c r="N5" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O5" s="4"/>
+      <c r="O5" s="4" t="s">
+        <v>27</v>
+      </c>
       <c r="P5" s="4"/>
       <c r="Q5" s="4"/>
       <c r="R5" s="4"/>
       <c r="S5" s="4"/>
       <c r="T5" s="4"/>
-      <c r="U5" s="3"/>
+      <c r="U5" s="4"/>
       <c r="V5" s="3"/>
       <c r="W5" s="3"/>
       <c r="X5" s="3"/>
@@ -1594,24 +1629,25 @@
       <c r="AG5" s="3"/>
       <c r="AH5" s="3"/>
       <c r="AI5" s="3"/>
-    </row>
-    <row r="6" spans="1:35">
+      <c r="AJ5" s="3"/>
+    </row>
+    <row r="6" spans="1:36">
       <c r="A6" s="3"/>
       <c r="B6" s="4" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="C6" s="2"/>
       <c r="D6" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E6" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="G6" s="4" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="H6" s="4" t="s">
         <v>18</v>
@@ -1624,13 +1660,15 @@
       <c r="N6" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O6" s="4"/>
+      <c r="O6" s="4" t="s">
+        <v>27</v>
+      </c>
       <c r="P6" s="4"/>
       <c r="Q6" s="4"/>
       <c r="R6" s="4"/>
       <c r="S6" s="4"/>
       <c r="T6" s="4"/>
-      <c r="U6" s="3"/>
+      <c r="U6" s="4"/>
       <c r="V6" s="3"/>
       <c r="W6" s="3"/>
       <c r="X6" s="3"/>
@@ -1645,24 +1683,25 @@
       <c r="AG6" s="3"/>
       <c r="AH6" s="3"/>
       <c r="AI6" s="3"/>
-    </row>
-    <row r="7" spans="1:35">
+      <c r="AJ6" s="3"/>
+    </row>
+    <row r="7" spans="1:36">
       <c r="A7" s="3"/>
       <c r="B7" s="4" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="C7" s="2"/>
       <c r="D7" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E7" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="G7" s="4" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="H7" s="4" t="s">
         <v>18</v>
@@ -1675,13 +1714,15 @@
       <c r="N7" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O7" s="4"/>
+      <c r="O7" s="4" t="s">
+        <v>27</v>
+      </c>
       <c r="P7" s="4"/>
       <c r="Q7" s="4"/>
       <c r="R7" s="4"/>
       <c r="S7" s="4"/>
       <c r="T7" s="4"/>
-      <c r="U7" s="3"/>
+      <c r="U7" s="4"/>
       <c r="V7" s="3"/>
       <c r="W7" s="3"/>
       <c r="X7" s="3"/>
@@ -1696,29 +1737,30 @@
       <c r="AG7" s="3"/>
       <c r="AH7" s="3"/>
       <c r="AI7" s="3"/>
-    </row>
-    <row r="8" spans="1:35">
+      <c r="AJ7" s="3"/>
+    </row>
+    <row r="8" spans="1:36">
       <c r="A8" s="3"/>
       <c r="B8" s="4" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E8" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F8" s="4" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="G8" s="4" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="H8" s="4" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="I8" s="4"/>
       <c r="J8" s="4"/>
@@ -1728,13 +1770,15 @@
       <c r="N8" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O8" s="4"/>
+      <c r="O8" s="4" t="s">
+        <v>27</v>
+      </c>
       <c r="P8" s="4"/>
       <c r="Q8" s="4"/>
       <c r="R8" s="4"/>
       <c r="S8" s="4"/>
       <c r="T8" s="4"/>
-      <c r="U8" s="3"/>
+      <c r="U8" s="4"/>
       <c r="V8" s="3"/>
       <c r="W8" s="3"/>
       <c r="X8" s="3"/>
@@ -1749,29 +1793,30 @@
       <c r="AG8" s="3"/>
       <c r="AH8" s="3"/>
       <c r="AI8" s="3"/>
-    </row>
-    <row r="9" spans="1:35">
+      <c r="AJ8" s="3"/>
+    </row>
+    <row r="9" spans="1:36">
       <c r="A9" s="3"/>
       <c r="B9" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="C9" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="C9" s="2" t="s">
-        <v>33</v>
-      </c>
       <c r="D9" s="4" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E9" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F9" s="4" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="G9" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="H9" s="4" t="s">
         <v>36</v>
-      </c>
-      <c r="H9" s="4" t="s">
-        <v>34</v>
       </c>
       <c r="I9" s="4"/>
       <c r="J9" s="4"/>
@@ -1781,13 +1826,15 @@
       <c r="N9" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O9" s="4"/>
+      <c r="O9" s="4" t="s">
+        <v>39</v>
+      </c>
       <c r="P9" s="4"/>
       <c r="Q9" s="4"/>
       <c r="R9" s="4"/>
       <c r="S9" s="4"/>
       <c r="T9" s="4"/>
-      <c r="U9" s="3"/>
+      <c r="U9" s="4"/>
       <c r="V9" s="3"/>
       <c r="W9" s="3"/>
       <c r="X9" s="3"/>
@@ -1802,45 +1849,48 @@
       <c r="AG9" s="3"/>
       <c r="AH9" s="3"/>
       <c r="AI9" s="3"/>
-    </row>
-    <row r="10" spans="1:35">
+      <c r="AJ9" s="3"/>
+    </row>
+    <row r="10" spans="1:36">
       <c r="A10" s="3"/>
       <c r="B10" s="4" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="C10" s="2"/>
       <c r="D10" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E10" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F10" s="4" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="G10" s="4" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="H10" s="4"/>
       <c r="I10" s="4"/>
       <c r="J10" s="4" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="K10" s="4" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="L10" s="4"/>
       <c r="M10" s="4"/>
       <c r="N10" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O10" s="4"/>
+      <c r="O10" s="4" t="s">
+        <v>44</v>
+      </c>
       <c r="P10" s="4"/>
       <c r="Q10" s="4"/>
       <c r="R10" s="4"/>
       <c r="S10" s="4"/>
       <c r="T10" s="4"/>
-      <c r="U10" s="3"/>
+      <c r="U10" s="4"/>
       <c r="V10" s="3"/>
       <c r="W10" s="3"/>
       <c r="X10" s="3"/>
@@ -1855,45 +1905,48 @@
       <c r="AG10" s="3"/>
       <c r="AH10" s="3"/>
       <c r="AI10" s="3"/>
-    </row>
-    <row r="11" spans="1:35">
+      <c r="AJ10" s="3"/>
+    </row>
+    <row r="11" spans="1:36">
       <c r="A11" s="3"/>
       <c r="B11" s="4" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="C11" s="2"/>
       <c r="D11" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E11" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F11" s="4" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="G11" s="4" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="H11" s="4"/>
       <c r="I11" s="4"/>
       <c r="J11" s="4" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="K11" s="4" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="L11" s="4"/>
       <c r="M11" s="4"/>
       <c r="N11" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O11" s="4"/>
+      <c r="O11" s="4" t="s">
+        <v>44</v>
+      </c>
       <c r="P11" s="4"/>
       <c r="Q11" s="4"/>
       <c r="R11" s="4"/>
       <c r="S11" s="4"/>
       <c r="T11" s="4"/>
-      <c r="U11" s="3"/>
+      <c r="U11" s="4"/>
       <c r="V11" s="3"/>
       <c r="W11" s="3"/>
       <c r="X11" s="3"/>
@@ -1908,45 +1961,48 @@
       <c r="AG11" s="3"/>
       <c r="AH11" s="3"/>
       <c r="AI11" s="3"/>
-    </row>
-    <row r="12" spans="1:35">
+      <c r="AJ11" s="3"/>
+    </row>
+    <row r="12" spans="1:36">
       <c r="A12" s="3"/>
       <c r="B12" s="4" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="C12" s="2"/>
       <c r="D12" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E12" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F12" s="4" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="G12" s="4" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="H12" s="4"/>
       <c r="I12" s="4"/>
       <c r="J12" s="4" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="K12" s="4" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="L12" s="4"/>
       <c r="M12" s="4"/>
       <c r="N12" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O12" s="4"/>
+      <c r="O12" s="4" t="s">
+        <v>44</v>
+      </c>
       <c r="P12" s="4"/>
       <c r="Q12" s="4"/>
       <c r="R12" s="4"/>
       <c r="S12" s="4"/>
       <c r="T12" s="4"/>
-      <c r="U12" s="3"/>
+      <c r="U12" s="4"/>
       <c r="V12" s="3"/>
       <c r="W12" s="3"/>
       <c r="X12" s="3"/>
@@ -1961,30 +2017,31 @@
       <c r="AG12" s="3"/>
       <c r="AH12" s="3"/>
       <c r="AI12" s="3"/>
-    </row>
-    <row r="13" spans="1:35">
+      <c r="AJ12" s="3"/>
+    </row>
+    <row r="13" spans="1:36">
       <c r="A13" s="3"/>
       <c r="B13" s="4" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="C13" s="2"/>
       <c r="D13" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E13" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F13" s="4" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="G13" s="4" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="H13" s="4" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="I13" s="4" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="J13" s="4"/>
       <c r="K13" s="4"/>
@@ -1993,13 +2050,15 @@
       <c r="N13" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O13" s="4"/>
+      <c r="O13" s="4" t="s">
+        <v>27</v>
+      </c>
       <c r="P13" s="4"/>
       <c r="Q13" s="4"/>
       <c r="R13" s="4"/>
       <c r="S13" s="4"/>
       <c r="T13" s="4"/>
-      <c r="U13" s="3"/>
+      <c r="U13" s="4"/>
       <c r="V13" s="3"/>
       <c r="W13" s="3"/>
       <c r="X13" s="3"/>
@@ -2014,30 +2073,31 @@
       <c r="AG13" s="3"/>
       <c r="AH13" s="3"/>
       <c r="AI13" s="3"/>
-    </row>
-    <row r="14" spans="1:35">
+      <c r="AJ13" s="3"/>
+    </row>
+    <row r="14" spans="1:36">
       <c r="A14" s="3"/>
       <c r="B14" s="4" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="C14" s="2"/>
       <c r="D14" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E14" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F14" s="4" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="G14" s="4" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="H14" s="4" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="I14" s="4" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="J14" s="4"/>
       <c r="K14" s="4"/>
@@ -2046,13 +2106,15 @@
       <c r="N14" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O14" s="4"/>
+      <c r="O14" s="4" t="s">
+        <v>27</v>
+      </c>
       <c r="P14" s="4"/>
       <c r="Q14" s="4"/>
       <c r="R14" s="4"/>
       <c r="S14" s="4"/>
       <c r="T14" s="4"/>
-      <c r="U14" s="3"/>
+      <c r="U14" s="4"/>
       <c r="V14" s="3"/>
       <c r="W14" s="3"/>
       <c r="X14" s="3"/>
@@ -2067,30 +2129,31 @@
       <c r="AG14" s="3"/>
       <c r="AH14" s="3"/>
       <c r="AI14" s="3"/>
-    </row>
-    <row r="15" spans="1:35">
+      <c r="AJ14" s="3"/>
+    </row>
+    <row r="15" spans="1:36">
       <c r="A15" s="3"/>
       <c r="B15" s="4" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="C15" s="2"/>
       <c r="D15" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E15" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F15" s="4" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="G15" s="4" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="H15" s="4" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="I15" s="4" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="J15" s="4"/>
       <c r="K15" s="4"/>
@@ -2099,13 +2162,15 @@
       <c r="N15" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O15" s="4"/>
+      <c r="O15" s="4" t="s">
+        <v>27</v>
+      </c>
       <c r="P15" s="4"/>
       <c r="Q15" s="4"/>
       <c r="R15" s="4"/>
       <c r="S15" s="4"/>
       <c r="T15" s="4"/>
-      <c r="U15" s="3"/>
+      <c r="U15" s="4"/>
       <c r="V15" s="3"/>
       <c r="W15" s="3"/>
       <c r="X15" s="3"/>
@@ -2120,30 +2185,31 @@
       <c r="AG15" s="3"/>
       <c r="AH15" s="3"/>
       <c r="AI15" s="3"/>
-    </row>
-    <row r="16" spans="1:35">
+      <c r="AJ15" s="3"/>
+    </row>
+    <row r="16" spans="1:36">
       <c r="A16" s="3"/>
       <c r="B16" s="4" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="C16" s="2"/>
       <c r="D16" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E16" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F16" s="4" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="G16" s="4" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="H16" s="4" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="I16" s="4" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="J16" s="4"/>
       <c r="K16" s="4"/>
@@ -2152,13 +2218,15 @@
       <c r="N16" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O16" s="4"/>
+      <c r="O16" s="4" t="s">
+        <v>27</v>
+      </c>
       <c r="P16" s="4"/>
       <c r="Q16" s="4"/>
       <c r="R16" s="4"/>
       <c r="S16" s="4"/>
       <c r="T16" s="4"/>
-      <c r="U16" s="3"/>
+      <c r="U16" s="4"/>
       <c r="V16" s="3"/>
       <c r="W16" s="3"/>
       <c r="X16" s="3"/>
@@ -2173,30 +2241,31 @@
       <c r="AG16" s="3"/>
       <c r="AH16" s="3"/>
       <c r="AI16" s="3"/>
-    </row>
-    <row r="17" spans="1:35">
+      <c r="AJ16" s="3"/>
+    </row>
+    <row r="17" spans="1:36">
       <c r="A17" s="3"/>
       <c r="B17" s="4" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="C17" s="2"/>
       <c r="D17" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E17" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F17" s="4" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="G17" s="4" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="H17" s="4" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="I17" s="4" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="J17" s="4"/>
       <c r="K17" s="4"/>
@@ -2205,13 +2274,15 @@
       <c r="N17" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O17" s="4"/>
+      <c r="O17" s="4" t="s">
+        <v>27</v>
+      </c>
       <c r="P17" s="4"/>
       <c r="Q17" s="4"/>
       <c r="R17" s="4"/>
       <c r="S17" s="4"/>
       <c r="T17" s="4"/>
-      <c r="U17" s="3"/>
+      <c r="U17" s="4"/>
       <c r="V17" s="3"/>
       <c r="W17" s="3"/>
       <c r="X17" s="3"/>
@@ -2226,43 +2297,46 @@
       <c r="AG17" s="3"/>
       <c r="AH17" s="3"/>
       <c r="AI17" s="3"/>
-    </row>
-    <row r="18" spans="1:35">
+      <c r="AJ17" s="3"/>
+    </row>
+    <row r="18" spans="1:36">
       <c r="A18" s="3"/>
       <c r="B18" s="4" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="C18" s="2"/>
       <c r="D18" s="4" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E18" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F18" s="4" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="G18" s="4" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="H18" s="4"/>
       <c r="I18" s="4"/>
       <c r="J18" s="4"/>
       <c r="K18" s="4"/>
       <c r="L18" s="4" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="M18" s="4"/>
       <c r="N18" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O18" s="4"/>
+      <c r="O18" s="4" t="s">
+        <v>65</v>
+      </c>
       <c r="P18" s="4"/>
       <c r="Q18" s="4"/>
       <c r="R18" s="4"/>
       <c r="S18" s="4"/>
       <c r="T18" s="4"/>
-      <c r="U18" s="3"/>
+      <c r="U18" s="4"/>
       <c r="V18" s="3"/>
       <c r="W18" s="3"/>
       <c r="X18" s="3"/>
@@ -2277,43 +2351,46 @@
       <c r="AG18" s="3"/>
       <c r="AH18" s="3"/>
       <c r="AI18" s="3"/>
-    </row>
-    <row r="19" spans="1:35">
+      <c r="AJ18" s="3"/>
+    </row>
+    <row r="19" spans="1:36">
       <c r="A19" s="3"/>
       <c r="B19" s="4" t="s">
-        <v>61</v>
+        <v>66</v>
       </c>
       <c r="C19" s="2"/>
       <c r="D19" s="4" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E19" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F19" s="4" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="G19" s="4" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="H19" s="4"/>
       <c r="I19" s="4"/>
       <c r="J19" s="4"/>
       <c r="K19" s="4"/>
       <c r="L19" s="4" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="M19" s="4"/>
       <c r="N19" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O19" s="4"/>
+      <c r="O19" s="4" t="s">
+        <v>65</v>
+      </c>
       <c r="P19" s="4"/>
       <c r="Q19" s="4"/>
       <c r="R19" s="4"/>
       <c r="S19" s="4"/>
       <c r="T19" s="4"/>
-      <c r="U19" s="3"/>
+      <c r="U19" s="4"/>
       <c r="V19" s="3"/>
       <c r="W19" s="3"/>
       <c r="X19" s="3"/>
@@ -2328,43 +2405,46 @@
       <c r="AG19" s="3"/>
       <c r="AH19" s="3"/>
       <c r="AI19" s="3"/>
-    </row>
-    <row r="20" spans="1:35">
+      <c r="AJ19" s="3"/>
+    </row>
+    <row r="20" spans="1:36">
       <c r="A20" s="3"/>
       <c r="B20" s="4" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="C20" s="2"/>
       <c r="D20" s="4" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E20" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F20" s="4" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="G20" s="4" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="H20" s="4"/>
       <c r="I20" s="4"/>
       <c r="J20" s="4"/>
       <c r="K20" s="4"/>
       <c r="L20" s="4" t="s">
-        <v>64</v>
+        <v>69</v>
       </c>
       <c r="M20" s="4"/>
       <c r="N20" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O20" s="4"/>
+      <c r="O20" s="4" t="s">
+        <v>65</v>
+      </c>
       <c r="P20" s="4"/>
       <c r="Q20" s="4"/>
       <c r="R20" s="4"/>
       <c r="S20" s="4"/>
       <c r="T20" s="4"/>
-      <c r="U20" s="3"/>
+      <c r="U20" s="4"/>
       <c r="V20" s="3"/>
       <c r="W20" s="3"/>
       <c r="X20" s="3"/>
@@ -2379,43 +2459,46 @@
       <c r="AG20" s="3"/>
       <c r="AH20" s="3"/>
       <c r="AI20" s="3"/>
-    </row>
-    <row r="21" spans="1:35">
+      <c r="AJ20" s="3"/>
+    </row>
+    <row r="21" spans="1:36">
       <c r="A21" s="3"/>
       <c r="B21" s="4" t="s">
-        <v>65</v>
+        <v>70</v>
       </c>
       <c r="C21" s="2"/>
       <c r="D21" s="4" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E21" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F21" s="4" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="G21" s="4" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="H21" s="4"/>
       <c r="I21" s="4"/>
       <c r="J21" s="4"/>
       <c r="K21" s="4"/>
       <c r="L21" s="4" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="M21" s="4"/>
       <c r="N21" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O21" s="4"/>
+      <c r="O21" s="4" t="s">
+        <v>65</v>
+      </c>
       <c r="P21" s="4"/>
       <c r="Q21" s="4"/>
       <c r="R21" s="4"/>
       <c r="S21" s="4"/>
       <c r="T21" s="4"/>
-      <c r="U21" s="3"/>
+      <c r="U21" s="4"/>
       <c r="V21" s="3"/>
       <c r="W21" s="3"/>
       <c r="X21" s="3"/>
@@ -2430,43 +2513,46 @@
       <c r="AG21" s="3"/>
       <c r="AH21" s="3"/>
       <c r="AI21" s="3"/>
-    </row>
-    <row r="22" spans="1:35">
+      <c r="AJ21" s="3"/>
+    </row>
+    <row r="22" spans="1:36">
       <c r="A22" s="3"/>
       <c r="B22" s="4" t="s">
-        <v>67</v>
+        <v>72</v>
       </c>
       <c r="C22" s="2"/>
       <c r="D22" s="4" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E22" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F22" s="4" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="G22" s="4" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="H22" s="4"/>
       <c r="I22" s="4"/>
       <c r="J22" s="4"/>
       <c r="K22" s="4"/>
       <c r="L22" s="4" t="s">
-        <v>68</v>
+        <v>73</v>
       </c>
       <c r="M22" s="4"/>
       <c r="N22" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O22" s="4"/>
+      <c r="O22" s="4" t="s">
+        <v>65</v>
+      </c>
       <c r="P22" s="4"/>
       <c r="Q22" s="4"/>
       <c r="R22" s="4"/>
       <c r="S22" s="4"/>
       <c r="T22" s="4"/>
-      <c r="U22" s="3"/>
+      <c r="U22" s="4"/>
       <c r="V22" s="3"/>
       <c r="W22" s="3"/>
       <c r="X22" s="3"/>
@@ -2481,43 +2567,46 @@
       <c r="AG22" s="3"/>
       <c r="AH22" s="3"/>
       <c r="AI22" s="3"/>
-    </row>
-    <row r="23" spans="1:35">
+      <c r="AJ22" s="3"/>
+    </row>
+    <row r="23" spans="1:36">
       <c r="A23" s="3"/>
       <c r="B23" s="4" t="s">
-        <v>69</v>
+        <v>74</v>
       </c>
       <c r="C23" s="2"/>
       <c r="D23" s="4" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E23" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F23" s="4" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="G23" s="4" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="H23" s="4"/>
       <c r="I23" s="4"/>
       <c r="J23" s="4"/>
       <c r="K23" s="4"/>
       <c r="L23" s="4" t="s">
-        <v>70</v>
+        <v>75</v>
       </c>
       <c r="M23" s="4"/>
       <c r="N23" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O23" s="4"/>
+      <c r="O23" s="4" t="s">
+        <v>65</v>
+      </c>
       <c r="P23" s="4"/>
       <c r="Q23" s="4"/>
       <c r="R23" s="4"/>
       <c r="S23" s="4"/>
       <c r="T23" s="4"/>
-      <c r="U23" s="3"/>
+      <c r="U23" s="4"/>
       <c r="V23" s="3"/>
       <c r="W23" s="3"/>
       <c r="X23" s="3"/>
@@ -2532,24 +2621,25 @@
       <c r="AG23" s="3"/>
       <c r="AH23" s="3"/>
       <c r="AI23" s="3"/>
-    </row>
-    <row r="24" spans="1:35">
+      <c r="AJ23" s="3"/>
+    </row>
+    <row r="24" spans="1:36">
       <c r="A24" s="3"/>
       <c r="B24" s="4" t="s">
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="C24" s="2"/>
       <c r="D24" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E24" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F24" s="4" t="s">
-        <v>72</v>
+        <v>77</v>
       </c>
       <c r="G24" s="4" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="H24" s="4" t="s">
         <v>18</v>
@@ -2562,13 +2652,15 @@
       <c r="N24" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O24" s="4"/>
+      <c r="O24" s="4" t="s">
+        <v>27</v>
+      </c>
       <c r="P24" s="4"/>
       <c r="Q24" s="4"/>
       <c r="R24" s="4"/>
       <c r="S24" s="4"/>
       <c r="T24" s="4"/>
-      <c r="U24" s="3"/>
+      <c r="U24" s="4"/>
       <c r="V24" s="3"/>
       <c r="W24" s="3"/>
       <c r="X24" s="3"/>
@@ -2583,24 +2675,25 @@
       <c r="AG24" s="3"/>
       <c r="AH24" s="3"/>
       <c r="AI24" s="3"/>
-    </row>
-    <row r="25" spans="1:35">
+      <c r="AJ24" s="3"/>
+    </row>
+    <row r="25" spans="1:36">
       <c r="A25" s="3"/>
       <c r="B25" s="4" t="s">
-        <v>73</v>
+        <v>78</v>
       </c>
       <c r="C25" s="2"/>
       <c r="D25" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E25" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F25" s="4" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="G25" s="4" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="H25" s="4" t="s">
         <v>18</v>
@@ -2613,13 +2706,15 @@
       <c r="N25" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O25" s="4"/>
+      <c r="O25" s="4" t="s">
+        <v>27</v>
+      </c>
       <c r="P25" s="4"/>
       <c r="Q25" s="4"/>
       <c r="R25" s="4"/>
       <c r="S25" s="4"/>
       <c r="T25" s="4"/>
-      <c r="U25" s="3"/>
+      <c r="U25" s="4"/>
       <c r="V25" s="3"/>
       <c r="W25" s="3"/>
       <c r="X25" s="3"/>
@@ -2634,21 +2729,22 @@
       <c r="AG25" s="3"/>
       <c r="AH25" s="3"/>
       <c r="AI25" s="3"/>
-    </row>
-    <row r="26" spans="1:35">
+      <c r="AJ25" s="3"/>
+    </row>
+    <row r="26" spans="1:36">
       <c r="A26" s="3"/>
       <c r="B26" s="4" t="s">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="C26" s="2"/>
       <c r="D26" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E26" s="4" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="F26" s="4" t="s">
-        <v>72</v>
+        <v>77</v>
       </c>
       <c r="G26" s="4"/>
       <c r="H26" s="4" t="s">
@@ -2662,13 +2758,15 @@
       <c r="N26" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O26" s="4"/>
+      <c r="O26" s="4" t="s">
+        <v>82</v>
+      </c>
       <c r="P26" s="4"/>
       <c r="Q26" s="4"/>
       <c r="R26" s="4"/>
       <c r="S26" s="4"/>
       <c r="T26" s="4"/>
-      <c r="U26" s="3"/>
+      <c r="U26" s="4"/>
       <c r="V26" s="3"/>
       <c r="W26" s="3"/>
       <c r="X26" s="3"/>
@@ -2683,21 +2781,22 @@
       <c r="AG26" s="3"/>
       <c r="AH26" s="3"/>
       <c r="AI26" s="3"/>
-    </row>
-    <row r="27" spans="1:35">
+      <c r="AJ26" s="3"/>
+    </row>
+    <row r="27" spans="1:36">
       <c r="A27" s="3"/>
       <c r="B27" s="4" t="s">
-        <v>77</v>
+        <v>83</v>
       </c>
       <c r="C27" s="2"/>
       <c r="D27" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E27" s="4" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="F27" s="4" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="G27" s="4"/>
       <c r="H27" s="4" t="s">
@@ -2711,13 +2810,15 @@
       <c r="N27" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O27" s="4"/>
+      <c r="O27" s="4" t="s">
+        <v>82</v>
+      </c>
       <c r="P27" s="4"/>
       <c r="Q27" s="4"/>
       <c r="R27" s="4"/>
       <c r="S27" s="4"/>
       <c r="T27" s="4"/>
-      <c r="U27" s="3"/>
+      <c r="U27" s="4"/>
       <c r="V27" s="3"/>
       <c r="W27" s="3"/>
       <c r="X27" s="3"/>
@@ -2732,24 +2833,25 @@
       <c r="AG27" s="3"/>
       <c r="AH27" s="3"/>
       <c r="AI27" s="3"/>
-    </row>
-    <row r="28" spans="1:35">
+      <c r="AJ27" s="3"/>
+    </row>
+    <row r="28" spans="1:36">
       <c r="A28" s="3"/>
       <c r="B28" s="4" t="s">
-        <v>78</v>
+        <v>84</v>
       </c>
       <c r="C28" s="2"/>
       <c r="D28" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E28" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F28" s="4" t="s">
-        <v>79</v>
+        <v>85</v>
       </c>
       <c r="G28" s="4" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="H28" s="4" t="s">
         <v>18</v>
@@ -2762,13 +2864,15 @@
       <c r="N28" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O28" s="4"/>
+      <c r="O28" s="4" t="s">
+        <v>27</v>
+      </c>
       <c r="P28" s="4"/>
       <c r="Q28" s="4"/>
       <c r="R28" s="4"/>
       <c r="S28" s="4"/>
       <c r="T28" s="4"/>
-      <c r="U28" s="3"/>
+      <c r="U28" s="4"/>
       <c r="V28" s="3"/>
       <c r="W28" s="3"/>
       <c r="X28" s="3"/>
@@ -2783,21 +2887,22 @@
       <c r="AG28" s="3"/>
       <c r="AH28" s="3"/>
       <c r="AI28" s="3"/>
-    </row>
-    <row r="29" spans="1:35">
+      <c r="AJ28" s="3"/>
+    </row>
+    <row r="29" spans="1:36">
       <c r="A29" s="3"/>
       <c r="B29" s="4" t="s">
-        <v>80</v>
+        <v>86</v>
       </c>
       <c r="C29" s="2"/>
       <c r="D29" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E29" s="4" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="F29" s="4" t="s">
-        <v>81</v>
+        <v>87</v>
       </c>
       <c r="G29" s="4"/>
       <c r="H29" s="4" t="s">
@@ -2811,13 +2916,15 @@
       <c r="N29" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O29" s="4"/>
+      <c r="O29" s="4" t="s">
+        <v>82</v>
+      </c>
       <c r="P29" s="4"/>
       <c r="Q29" s="4"/>
       <c r="R29" s="4"/>
       <c r="S29" s="4"/>
       <c r="T29" s="4"/>
-      <c r="U29" s="3"/>
+      <c r="U29" s="4"/>
       <c r="V29" s="3"/>
       <c r="W29" s="3"/>
       <c r="X29" s="3"/>
@@ -2832,21 +2939,22 @@
       <c r="AG29" s="3"/>
       <c r="AH29" s="3"/>
       <c r="AI29" s="3"/>
-    </row>
-    <row r="30" spans="1:35">
+      <c r="AJ29" s="3"/>
+    </row>
+    <row r="30" spans="1:36">
       <c r="A30" s="3"/>
       <c r="B30" s="4" t="s">
-        <v>82</v>
+        <v>88</v>
       </c>
       <c r="C30" s="2"/>
       <c r="D30" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E30" s="4" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="F30" s="4" t="s">
-        <v>83</v>
+        <v>89</v>
       </c>
       <c r="G30" s="4"/>
       <c r="H30" s="4" t="s">
@@ -2860,13 +2968,15 @@
       <c r="N30" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O30" s="4"/>
+      <c r="O30" s="4" t="s">
+        <v>82</v>
+      </c>
       <c r="P30" s="4"/>
       <c r="Q30" s="4"/>
       <c r="R30" s="4"/>
       <c r="S30" s="4"/>
       <c r="T30" s="4"/>
-      <c r="U30" s="3"/>
+      <c r="U30" s="4"/>
       <c r="V30" s="3"/>
       <c r="W30" s="3"/>
       <c r="X30" s="3"/>
@@ -2881,24 +2991,25 @@
       <c r="AG30" s="3"/>
       <c r="AH30" s="3"/>
       <c r="AI30" s="3"/>
-    </row>
-    <row r="31" spans="1:35">
+      <c r="AJ30" s="3"/>
+    </row>
+    <row r="31" spans="1:36">
       <c r="A31" s="3"/>
       <c r="B31" s="4" t="s">
-        <v>84</v>
+        <v>90</v>
       </c>
       <c r="C31" s="2"/>
       <c r="D31" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E31" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F31" s="4" t="s">
-        <v>83</v>
+        <v>89</v>
       </c>
       <c r="G31" s="4" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="H31" s="4" t="s">
         <v>18</v>
@@ -2911,13 +3022,15 @@
       <c r="N31" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O31" s="4"/>
+      <c r="O31" s="4" t="s">
+        <v>27</v>
+      </c>
       <c r="P31" s="4"/>
       <c r="Q31" s="4"/>
       <c r="R31" s="4"/>
       <c r="S31" s="4"/>
       <c r="T31" s="4"/>
-      <c r="U31" s="3"/>
+      <c r="U31" s="4"/>
       <c r="V31" s="3"/>
       <c r="W31" s="3"/>
       <c r="X31" s="3"/>
@@ -2932,24 +3045,25 @@
       <c r="AG31" s="3"/>
       <c r="AH31" s="3"/>
       <c r="AI31" s="3"/>
-    </row>
-    <row r="32" spans="1:35">
+      <c r="AJ31" s="3"/>
+    </row>
+    <row r="32" spans="1:36">
       <c r="A32" s="3"/>
       <c r="B32" s="4" t="s">
-        <v>85</v>
+        <v>91</v>
       </c>
       <c r="C32" s="2"/>
       <c r="D32" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E32" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F32" s="4" t="s">
-        <v>83</v>
+        <v>89</v>
       </c>
       <c r="G32" s="4" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="H32" s="4" t="s">
         <v>18</v>
@@ -2962,13 +3076,15 @@
       <c r="N32" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O32" s="4"/>
+      <c r="O32" s="4" t="s">
+        <v>27</v>
+      </c>
       <c r="P32" s="4"/>
       <c r="Q32" s="4"/>
       <c r="R32" s="4"/>
       <c r="S32" s="4"/>
       <c r="T32" s="4"/>
-      <c r="U32" s="3"/>
+      <c r="U32" s="4"/>
       <c r="V32" s="3"/>
       <c r="W32" s="3"/>
       <c r="X32" s="3"/>
@@ -2983,21 +3099,22 @@
       <c r="AG32" s="3"/>
       <c r="AH32" s="3"/>
       <c r="AI32" s="3"/>
-    </row>
-    <row r="33" spans="1:35">
+      <c r="AJ32" s="3"/>
+    </row>
+    <row r="33" spans="1:36">
       <c r="A33" s="3"/>
       <c r="B33" s="4" t="s">
-        <v>86</v>
+        <v>92</v>
       </c>
       <c r="C33" s="2"/>
       <c r="D33" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E33" s="4" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="F33" s="4" t="s">
-        <v>79</v>
+        <v>85</v>
       </c>
       <c r="G33" s="4"/>
       <c r="H33" s="4" t="s">
@@ -3011,13 +3128,15 @@
       <c r="N33" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O33" s="4"/>
+      <c r="O33" s="4" t="s">
+        <v>82</v>
+      </c>
       <c r="P33" s="4"/>
       <c r="Q33" s="4"/>
       <c r="R33" s="4"/>
       <c r="S33" s="4"/>
       <c r="T33" s="4"/>
-      <c r="U33" s="3"/>
+      <c r="U33" s="4"/>
       <c r="V33" s="3"/>
       <c r="W33" s="3"/>
       <c r="X33" s="3"/>
@@ -3032,21 +3151,22 @@
       <c r="AG33" s="3"/>
       <c r="AH33" s="3"/>
       <c r="AI33" s="3"/>
-    </row>
-    <row r="34" spans="1:35">
+      <c r="AJ33" s="3"/>
+    </row>
+    <row r="34" spans="1:36">
       <c r="A34" s="3"/>
       <c r="B34" s="4" t="s">
-        <v>87</v>
+        <v>93</v>
       </c>
       <c r="C34" s="2"/>
       <c r="D34" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E34" s="4" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="F34" s="4" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="G34" s="4"/>
       <c r="H34" s="4" t="s">
@@ -3060,13 +3180,15 @@
       <c r="N34" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O34" s="4"/>
+      <c r="O34" s="4" t="s">
+        <v>82</v>
+      </c>
       <c r="P34" s="4"/>
       <c r="Q34" s="4"/>
       <c r="R34" s="4"/>
       <c r="S34" s="4"/>
       <c r="T34" s="4"/>
-      <c r="U34" s="3"/>
+      <c r="U34" s="4"/>
       <c r="V34" s="3"/>
       <c r="W34" s="3"/>
       <c r="X34" s="3"/>
@@ -3081,21 +3203,22 @@
       <c r="AG34" s="3"/>
       <c r="AH34" s="3"/>
       <c r="AI34" s="3"/>
-    </row>
-    <row r="35" spans="1:35">
+      <c r="AJ34" s="3"/>
+    </row>
+    <row r="35" spans="1:36">
       <c r="A35" s="3"/>
       <c r="B35" s="4" t="s">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="C35" s="2"/>
       <c r="D35" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E35" s="4" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="F35" s="4" t="s">
-        <v>89</v>
+        <v>95</v>
       </c>
       <c r="G35" s="4"/>
       <c r="H35" s="4" t="s">
@@ -3109,13 +3232,15 @@
       <c r="N35" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O35" s="4"/>
+      <c r="O35" s="4" t="s">
+        <v>82</v>
+      </c>
       <c r="P35" s="4"/>
       <c r="Q35" s="4"/>
       <c r="R35" s="4"/>
       <c r="S35" s="4"/>
       <c r="T35" s="4"/>
-      <c r="U35" s="3"/>
+      <c r="U35" s="4"/>
       <c r="V35" s="3"/>
       <c r="W35" s="3"/>
       <c r="X35" s="3"/>
@@ -3130,21 +3255,22 @@
       <c r="AG35" s="3"/>
       <c r="AH35" s="3"/>
       <c r="AI35" s="3"/>
-    </row>
-    <row r="36" spans="1:35">
+      <c r="AJ35" s="3"/>
+    </row>
+    <row r="36" spans="1:36">
       <c r="A36" s="3"/>
       <c r="B36" s="4" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="C36" s="2"/>
       <c r="D36" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E36" s="4" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="F36" s="4" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="G36" s="4"/>
       <c r="H36" s="4" t="s">
@@ -3158,13 +3284,15 @@
       <c r="N36" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O36" s="4"/>
+      <c r="O36" s="4" t="s">
+        <v>82</v>
+      </c>
       <c r="P36" s="4"/>
       <c r="Q36" s="4"/>
       <c r="R36" s="4"/>
       <c r="S36" s="4"/>
       <c r="T36" s="4"/>
-      <c r="U36" s="3"/>
+      <c r="U36" s="4"/>
       <c r="V36" s="3"/>
       <c r="W36" s="3"/>
       <c r="X36" s="3"/>
@@ -3179,21 +3307,22 @@
       <c r="AG36" s="3"/>
       <c r="AH36" s="3"/>
       <c r="AI36" s="3"/>
-    </row>
-    <row r="37" spans="1:35">
+      <c r="AJ36" s="3"/>
+    </row>
+    <row r="37" spans="1:36">
       <c r="A37" s="3"/>
       <c r="B37" s="4" t="s">
-        <v>91</v>
+        <v>97</v>
       </c>
       <c r="C37" s="2"/>
       <c r="D37" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E37" s="4" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="F37" s="4" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="G37" s="4"/>
       <c r="H37" s="4" t="s">
@@ -3207,13 +3336,15 @@
       <c r="N37" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O37" s="4"/>
+      <c r="O37" s="4" t="s">
+        <v>82</v>
+      </c>
       <c r="P37" s="4"/>
       <c r="Q37" s="4"/>
       <c r="R37" s="4"/>
       <c r="S37" s="4"/>
       <c r="T37" s="4"/>
-      <c r="U37" s="3"/>
+      <c r="U37" s="4"/>
       <c r="V37" s="3"/>
       <c r="W37" s="3"/>
       <c r="X37" s="3"/>
@@ -3228,21 +3359,22 @@
       <c r="AG37" s="3"/>
       <c r="AH37" s="3"/>
       <c r="AI37" s="3"/>
-    </row>
-    <row r="38" spans="1:35">
+      <c r="AJ37" s="3"/>
+    </row>
+    <row r="38" spans="1:36">
       <c r="A38" s="3"/>
       <c r="B38" s="4" t="s">
-        <v>92</v>
+        <v>98</v>
       </c>
       <c r="C38" s="2"/>
       <c r="D38" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E38" s="4" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="F38" s="4" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="G38" s="4"/>
       <c r="H38" s="4" t="s">
@@ -3256,13 +3388,15 @@
       <c r="N38" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O38" s="4"/>
+      <c r="O38" s="4" t="s">
+        <v>82</v>
+      </c>
       <c r="P38" s="4"/>
       <c r="Q38" s="4"/>
       <c r="R38" s="4"/>
       <c r="S38" s="4"/>
       <c r="T38" s="4"/>
-      <c r="U38" s="3"/>
+      <c r="U38" s="4"/>
       <c r="V38" s="3"/>
       <c r="W38" s="3"/>
       <c r="X38" s="3"/>
@@ -3277,43 +3411,46 @@
       <c r="AG38" s="3"/>
       <c r="AH38" s="3"/>
       <c r="AI38" s="3"/>
-    </row>
-    <row r="39" spans="1:35">
+      <c r="AJ38" s="3"/>
+    </row>
+    <row r="39" spans="1:36">
       <c r="A39" s="3"/>
       <c r="B39" s="4" t="s">
-        <v>93</v>
+        <v>99</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="D39" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E39" s="4" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="F39" s="4"/>
       <c r="G39" s="4"/>
       <c r="H39" s="4" t="s">
-        <v>95</v>
+        <v>101</v>
       </c>
       <c r="I39" s="4"/>
       <c r="J39" s="4"/>
       <c r="K39" s="4"/>
       <c r="L39" s="4"/>
       <c r="M39" s="4" t="s">
-        <v>96</v>
+        <v>102</v>
       </c>
       <c r="N39" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O39" s="4"/>
+      <c r="O39" s="4" t="s">
+        <v>82</v>
+      </c>
       <c r="P39" s="4"/>
       <c r="Q39" s="4"/>
       <c r="R39" s="4"/>
       <c r="S39" s="4"/>
       <c r="T39" s="4"/>
-      <c r="U39" s="3"/>
+      <c r="U39" s="4"/>
       <c r="V39" s="3"/>
       <c r="W39" s="3"/>
       <c r="X39" s="3"/>
@@ -3328,43 +3465,46 @@
       <c r="AG39" s="3"/>
       <c r="AH39" s="3"/>
       <c r="AI39" s="3"/>
-    </row>
-    <row r="40" spans="1:35">
+      <c r="AJ39" s="3"/>
+    </row>
+    <row r="40" spans="1:36">
       <c r="A40" s="3"/>
       <c r="B40" s="4" t="s">
-        <v>97</v>
+        <v>103</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="D40" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E40" s="4" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="F40" s="4"/>
       <c r="G40" s="4"/>
       <c r="H40" s="4" t="s">
-        <v>95</v>
+        <v>101</v>
       </c>
       <c r="I40" s="4"/>
       <c r="J40" s="4"/>
       <c r="K40" s="4"/>
       <c r="L40" s="4"/>
       <c r="M40" s="4" t="s">
-        <v>98</v>
+        <v>104</v>
       </c>
       <c r="N40" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O40" s="4"/>
+      <c r="O40" s="4" t="s">
+        <v>82</v>
+      </c>
       <c r="P40" s="4"/>
       <c r="Q40" s="4"/>
       <c r="R40" s="4"/>
       <c r="S40" s="4"/>
       <c r="T40" s="4"/>
-      <c r="U40" s="3"/>
+      <c r="U40" s="4"/>
       <c r="V40" s="3"/>
       <c r="W40" s="3"/>
       <c r="X40" s="3"/>
@@ -3379,39 +3519,42 @@
       <c r="AG40" s="3"/>
       <c r="AH40" s="3"/>
       <c r="AI40" s="3"/>
-    </row>
-    <row r="41" spans="1:35">
+      <c r="AJ40" s="3"/>
+    </row>
+    <row r="41" spans="1:36">
       <c r="A41" s="3"/>
       <c r="B41" s="4" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="D41" s="4"/>
       <c r="E41" s="4"/>
       <c r="F41" s="4"/>
       <c r="G41" s="4"/>
       <c r="H41" s="4" t="s">
-        <v>95</v>
+        <v>101</v>
       </c>
       <c r="I41" s="4"/>
       <c r="J41" s="4"/>
       <c r="K41" s="4"/>
       <c r="L41" s="4"/>
       <c r="M41" s="4" t="s">
-        <v>101</v>
+        <v>107</v>
       </c>
       <c r="N41" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O41" s="4"/>
+      <c r="O41" s="4" t="s">
+        <v>108</v>
+      </c>
       <c r="P41" s="4"/>
       <c r="Q41" s="4"/>
       <c r="R41" s="4"/>
       <c r="S41" s="4"/>
       <c r="T41" s="4"/>
-      <c r="U41" s="3"/>
+      <c r="U41" s="4"/>
       <c r="V41" s="3"/>
       <c r="W41" s="3"/>
       <c r="X41" s="3"/>
@@ -3426,39 +3569,42 @@
       <c r="AG41" s="3"/>
       <c r="AH41" s="3"/>
       <c r="AI41" s="3"/>
-    </row>
-    <row r="42" spans="1:35">
+      <c r="AJ41" s="3"/>
+    </row>
+    <row r="42" spans="1:36">
       <c r="A42" s="3"/>
       <c r="B42" s="4" t="s">
-        <v>102</v>
+        <v>109</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="D42" s="4"/>
       <c r="E42" s="4"/>
       <c r="F42" s="4"/>
       <c r="G42" s="4"/>
       <c r="H42" s="4" t="s">
-        <v>95</v>
+        <v>101</v>
       </c>
       <c r="I42" s="4"/>
       <c r="J42" s="4"/>
       <c r="K42" s="4"/>
       <c r="L42" s="4"/>
       <c r="M42" s="4" t="s">
-        <v>101</v>
+        <v>107</v>
       </c>
       <c r="N42" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O42" s="4"/>
+      <c r="O42" s="4" t="s">
+        <v>108</v>
+      </c>
       <c r="P42" s="4"/>
       <c r="Q42" s="4"/>
       <c r="R42" s="4"/>
       <c r="S42" s="4"/>
       <c r="T42" s="4"/>
-      <c r="U42" s="3"/>
+      <c r="U42" s="4"/>
       <c r="V42" s="3"/>
       <c r="W42" s="3"/>
       <c r="X42" s="3"/>
@@ -3473,10 +3619,11 @@
       <c r="AG42" s="3"/>
       <c r="AH42" s="3"/>
       <c r="AI42" s="3"/>
-    </row>
-    <row r="43" spans="2:35">
+      <c r="AJ42" s="3"/>
+    </row>
+    <row r="43" spans="2:36">
       <c r="B43" s="2" t="s">
-        <v>103</v>
+        <v>110</v>
       </c>
       <c r="C43" s="2"/>
       <c r="D43" s="2"/>
@@ -3492,13 +3639,15 @@
       <c r="N43" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="O43" s="2"/>
+      <c r="O43" s="2" t="s">
+        <v>27</v>
+      </c>
       <c r="P43" s="2"/>
       <c r="Q43" s="2"/>
       <c r="R43" s="2"/>
       <c r="S43" s="2"/>
       <c r="T43" s="2"/>
-      <c r="Y43" s="3"/>
+      <c r="U43" s="2"/>
       <c r="Z43" s="3"/>
       <c r="AA43" s="3"/>
       <c r="AB43" s="3"/>
@@ -3509,54 +3658,57 @@
       <c r="AG43" s="3"/>
       <c r="AH43" s="3"/>
       <c r="AI43" s="3"/>
-    </row>
-    <row r="44" spans="2:35">
+      <c r="AJ43" s="3"/>
+    </row>
+    <row r="44" spans="2:36">
       <c r="B44" s="2" t="s">
-        <v>104</v>
+        <v>111</v>
       </c>
       <c r="C44" s="2" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="D44" s="2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E44" s="2" t="s">
         <v>15</v>
       </c>
       <c r="F44" s="2" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="G44" s="2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="H44" s="4" t="s">
-        <v>105</v>
+        <v>112</v>
       </c>
       <c r="I44" s="4" t="s">
-        <v>106</v>
+        <v>113</v>
       </c>
       <c r="J44" s="4" t="s">
-        <v>107</v>
+        <v>114</v>
       </c>
       <c r="K44" s="2" t="s">
-        <v>108</v>
+        <v>115</v>
       </c>
       <c r="L44" s="2" t="s">
-        <v>109</v>
+        <v>116</v>
       </c>
       <c r="M44" s="2" t="s">
-        <v>110</v>
+        <v>117</v>
       </c>
       <c r="N44" s="2" t="s">
-        <v>111</v>
-      </c>
-      <c r="O44" s="2"/>
+        <v>118</v>
+      </c>
+      <c r="O44" s="2" t="s">
+        <v>82</v>
+      </c>
       <c r="P44" s="2"/>
       <c r="Q44" s="2"/>
       <c r="R44" s="2"/>
       <c r="S44" s="2"/>
       <c r="T44" s="2"/>
-      <c r="Y44" s="3"/>
+      <c r="U44" s="2"/>
       <c r="Z44" s="3"/>
       <c r="AA44" s="3"/>
       <c r="AB44" s="3"/>
@@ -3567,8 +3719,9 @@
       <c r="AG44" s="3"/>
       <c r="AH44" s="3"/>
       <c r="AI44" s="3"/>
-    </row>
-    <row r="45" spans="1:35">
+      <c r="AJ44" s="3"/>
+    </row>
+    <row r="45" spans="1:36">
       <c r="A45" s="3"/>
       <c r="B45" s="4"/>
       <c r="C45" s="4"/>
@@ -3589,7 +3742,7 @@
       <c r="R45" s="4"/>
       <c r="S45" s="4"/>
       <c r="T45" s="4"/>
-      <c r="U45" s="3"/>
+      <c r="U45" s="4"/>
       <c r="V45" s="3"/>
       <c r="W45" s="3"/>
       <c r="X45" s="3"/>
@@ -3604,8 +3757,9 @@
       <c r="AG45" s="3"/>
       <c r="AH45" s="3"/>
       <c r="AI45" s="3"/>
-    </row>
-    <row r="46" s="1" customFormat="1" spans="1:35">
+      <c r="AJ45" s="3"/>
+    </row>
+    <row r="46" s="1" customFormat="1" spans="1:36">
       <c r="A46" s="3"/>
       <c r="B46" s="4"/>
       <c r="C46" s="4"/>
@@ -3626,7 +3780,7 @@
       <c r="R46" s="4"/>
       <c r="S46" s="4"/>
       <c r="T46" s="4"/>
-      <c r="U46" s="3"/>
+      <c r="U46" s="4"/>
       <c r="V46" s="3"/>
       <c r="W46" s="3"/>
       <c r="X46" s="3"/>
@@ -3641,8 +3795,9 @@
       <c r="AG46" s="3"/>
       <c r="AH46" s="3"/>
       <c r="AI46" s="3"/>
-    </row>
-    <row r="47" s="1" customFormat="1" spans="1:35">
+      <c r="AJ46" s="3"/>
+    </row>
+    <row r="47" s="1" customFormat="1" spans="1:36">
       <c r="A47" s="3"/>
       <c r="B47" s="4"/>
       <c r="C47" s="4"/>
@@ -3663,7 +3818,7 @@
       <c r="R47" s="4"/>
       <c r="S47" s="4"/>
       <c r="T47" s="4"/>
-      <c r="U47" s="3"/>
+      <c r="U47" s="4"/>
       <c r="V47" s="3"/>
       <c r="W47" s="3"/>
       <c r="X47" s="3"/>
@@ -3678,8 +3833,9 @@
       <c r="AG47" s="3"/>
       <c r="AH47" s="3"/>
       <c r="AI47" s="3"/>
-    </row>
-    <row r="48" spans="1:35">
+      <c r="AJ47" s="3"/>
+    </row>
+    <row r="48" spans="1:36">
       <c r="A48" s="3"/>
       <c r="B48" s="4"/>
       <c r="C48" s="4"/>
@@ -3700,7 +3856,7 @@
       <c r="R48" s="4"/>
       <c r="S48" s="4"/>
       <c r="T48" s="4"/>
-      <c r="U48" s="3"/>
+      <c r="U48" s="4"/>
       <c r="V48" s="3"/>
       <c r="W48" s="3"/>
       <c r="X48" s="3"/>
@@ -3715,8 +3871,9 @@
       <c r="AG48" s="3"/>
       <c r="AH48" s="3"/>
       <c r="AI48" s="3"/>
-    </row>
-    <row r="49" spans="1:35">
+      <c r="AJ48" s="3"/>
+    </row>
+    <row r="49" spans="1:36">
       <c r="A49" s="3"/>
       <c r="B49" s="4"/>
       <c r="C49" s="4"/>
@@ -3737,7 +3894,7 @@
       <c r="R49" s="4"/>
       <c r="S49" s="4"/>
       <c r="T49" s="4"/>
-      <c r="U49" s="3"/>
+      <c r="U49" s="4"/>
       <c r="V49" s="3"/>
       <c r="W49" s="3"/>
       <c r="X49" s="3"/>
@@ -3752,8 +3909,9 @@
       <c r="AG49" s="3"/>
       <c r="AH49" s="3"/>
       <c r="AI49" s="3"/>
-    </row>
-    <row r="50" spans="1:35">
+      <c r="AJ49" s="3"/>
+    </row>
+    <row r="50" spans="1:36">
       <c r="A50" s="3"/>
       <c r="B50" s="4"/>
       <c r="C50" s="4"/>
@@ -3774,7 +3932,7 @@
       <c r="R50" s="4"/>
       <c r="S50" s="4"/>
       <c r="T50" s="4"/>
-      <c r="U50" s="3"/>
+      <c r="U50" s="4"/>
       <c r="V50" s="3"/>
       <c r="W50" s="3"/>
       <c r="X50" s="3"/>
@@ -3789,8 +3947,9 @@
       <c r="AG50" s="3"/>
       <c r="AH50" s="3"/>
       <c r="AI50" s="3"/>
-    </row>
-    <row r="51" spans="1:35">
+      <c r="AJ50" s="3"/>
+    </row>
+    <row r="51" spans="1:36">
       <c r="A51" s="3"/>
       <c r="B51" s="4"/>
       <c r="C51" s="4"/>
@@ -3811,7 +3970,7 @@
       <c r="R51" s="4"/>
       <c r="S51" s="4"/>
       <c r="T51" s="4"/>
-      <c r="U51" s="3"/>
+      <c r="U51" s="4"/>
       <c r="V51" s="3"/>
       <c r="W51" s="3"/>
       <c r="X51" s="3"/>
@@ -3826,8 +3985,9 @@
       <c r="AG51" s="3"/>
       <c r="AH51" s="3"/>
       <c r="AI51" s="3"/>
-    </row>
-    <row r="52" spans="1:35">
+      <c r="AJ51" s="3"/>
+    </row>
+    <row r="52" spans="1:36">
       <c r="A52" s="3"/>
       <c r="B52" s="4"/>
       <c r="C52" s="4"/>
@@ -3848,7 +4008,7 @@
       <c r="R52" s="4"/>
       <c r="S52" s="4"/>
       <c r="T52" s="4"/>
-      <c r="U52" s="3"/>
+      <c r="U52" s="4"/>
       <c r="V52" s="3"/>
       <c r="W52" s="3"/>
       <c r="X52" s="3"/>
@@ -3863,8 +4023,9 @@
       <c r="AG52" s="3"/>
       <c r="AH52" s="3"/>
       <c r="AI52" s="3"/>
-    </row>
-    <row r="53" spans="1:35">
+      <c r="AJ52" s="3"/>
+    </row>
+    <row r="53" spans="1:36">
       <c r="A53" s="3"/>
       <c r="B53" s="4"/>
       <c r="C53" s="4"/>
@@ -3885,7 +4046,7 @@
       <c r="R53" s="4"/>
       <c r="S53" s="4"/>
       <c r="T53" s="4"/>
-      <c r="U53" s="3"/>
+      <c r="U53" s="4"/>
       <c r="V53" s="3"/>
       <c r="W53" s="3"/>
       <c r="X53" s="3"/>
@@ -3900,8 +4061,9 @@
       <c r="AG53" s="3"/>
       <c r="AH53" s="3"/>
       <c r="AI53" s="3"/>
-    </row>
-    <row r="54" spans="1:35">
+      <c r="AJ53" s="3"/>
+    </row>
+    <row r="54" spans="1:36">
       <c r="A54" s="3"/>
       <c r="B54" s="4"/>
       <c r="C54" s="4"/>
@@ -3922,7 +4084,7 @@
       <c r="R54" s="4"/>
       <c r="S54" s="4"/>
       <c r="T54" s="4"/>
-      <c r="U54" s="3"/>
+      <c r="U54" s="4"/>
       <c r="V54" s="3"/>
       <c r="W54" s="3"/>
       <c r="X54" s="3"/>
@@ -3937,8 +4099,9 @@
       <c r="AG54" s="3"/>
       <c r="AH54" s="3"/>
       <c r="AI54" s="3"/>
-    </row>
-    <row r="55" spans="1:35">
+      <c r="AJ54" s="3"/>
+    </row>
+    <row r="55" spans="1:36">
       <c r="A55" s="3"/>
       <c r="B55" s="4"/>
       <c r="C55" s="4"/>
@@ -3959,7 +4122,7 @@
       <c r="R55" s="4"/>
       <c r="S55" s="4"/>
       <c r="T55" s="4"/>
-      <c r="U55" s="3"/>
+      <c r="U55" s="4"/>
       <c r="V55" s="3"/>
       <c r="W55" s="3"/>
       <c r="X55" s="3"/>
@@ -3974,8 +4137,9 @@
       <c r="AG55" s="3"/>
       <c r="AH55" s="3"/>
       <c r="AI55" s="3"/>
-    </row>
-    <row r="56" spans="1:35">
+      <c r="AJ55" s="3"/>
+    </row>
+    <row r="56" spans="1:36">
       <c r="A56" s="3"/>
       <c r="B56" s="4"/>
       <c r="C56" s="4"/>
@@ -3996,7 +4160,7 @@
       <c r="R56" s="4"/>
       <c r="S56" s="4"/>
       <c r="T56" s="4"/>
-      <c r="U56" s="3"/>
+      <c r="U56" s="4"/>
       <c r="V56" s="3"/>
       <c r="W56" s="3"/>
       <c r="X56" s="3"/>
@@ -4011,8 +4175,9 @@
       <c r="AG56" s="3"/>
       <c r="AH56" s="3"/>
       <c r="AI56" s="3"/>
-    </row>
-    <row r="57" spans="1:35">
+      <c r="AJ56" s="3"/>
+    </row>
+    <row r="57" spans="1:36">
       <c r="A57" s="3"/>
       <c r="B57" s="4"/>
       <c r="C57" s="4"/>
@@ -4033,7 +4198,7 @@
       <c r="R57" s="4"/>
       <c r="S57" s="4"/>
       <c r="T57" s="4"/>
-      <c r="U57" s="3"/>
+      <c r="U57" s="4"/>
       <c r="V57" s="3"/>
       <c r="W57" s="3"/>
       <c r="X57" s="3"/>
@@ -4048,8 +4213,9 @@
       <c r="AG57" s="3"/>
       <c r="AH57" s="3"/>
       <c r="AI57" s="3"/>
-    </row>
-    <row r="58" spans="1:35">
+      <c r="AJ57" s="3"/>
+    </row>
+    <row r="58" spans="1:36">
       <c r="A58" s="3"/>
       <c r="B58" s="4"/>
       <c r="C58" s="4"/>
@@ -4070,7 +4236,7 @@
       <c r="R58" s="4"/>
       <c r="S58" s="4"/>
       <c r="T58" s="4"/>
-      <c r="U58" s="3"/>
+      <c r="U58" s="4"/>
       <c r="V58" s="3"/>
       <c r="W58" s="3"/>
       <c r="X58" s="3"/>
@@ -4085,8 +4251,9 @@
       <c r="AG58" s="3"/>
       <c r="AH58" s="3"/>
       <c r="AI58" s="3"/>
-    </row>
-    <row r="59" spans="1:35">
+      <c r="AJ58" s="3"/>
+    </row>
+    <row r="59" spans="1:36">
       <c r="A59" s="3"/>
       <c r="B59" s="4"/>
       <c r="C59" s="4"/>
@@ -4107,7 +4274,7 @@
       <c r="R59" s="4"/>
       <c r="S59" s="4"/>
       <c r="T59" s="4"/>
-      <c r="U59" s="3"/>
+      <c r="U59" s="4"/>
       <c r="V59" s="3"/>
       <c r="W59" s="3"/>
       <c r="X59" s="3"/>
@@ -4122,8 +4289,9 @@
       <c r="AG59" s="3"/>
       <c r="AH59" s="3"/>
       <c r="AI59" s="3"/>
-    </row>
-    <row r="60" spans="1:35">
+      <c r="AJ59" s="3"/>
+    </row>
+    <row r="60" spans="1:36">
       <c r="A60" s="3"/>
       <c r="B60" s="4"/>
       <c r="C60" s="4"/>
@@ -4144,7 +4312,7 @@
       <c r="R60" s="4"/>
       <c r="S60" s="4"/>
       <c r="T60" s="4"/>
-      <c r="U60" s="3"/>
+      <c r="U60" s="4"/>
       <c r="V60" s="3"/>
       <c r="W60" s="3"/>
       <c r="X60" s="3"/>
@@ -4159,8 +4327,9 @@
       <c r="AG60" s="3"/>
       <c r="AH60" s="3"/>
       <c r="AI60" s="3"/>
-    </row>
-    <row r="61" spans="1:35">
+      <c r="AJ60" s="3"/>
+    </row>
+    <row r="61" spans="1:36">
       <c r="A61" s="3"/>
       <c r="B61" s="4"/>
       <c r="C61" s="4"/>
@@ -4181,7 +4350,7 @@
       <c r="R61" s="4"/>
       <c r="S61" s="4"/>
       <c r="T61" s="4"/>
-      <c r="U61" s="3"/>
+      <c r="U61" s="4"/>
       <c r="V61" s="3"/>
       <c r="W61" s="3"/>
       <c r="X61" s="3"/>
@@ -4196,8 +4365,9 @@
       <c r="AG61" s="3"/>
       <c r="AH61" s="3"/>
       <c r="AI61" s="3"/>
-    </row>
-    <row r="62" spans="1:35">
+      <c r="AJ61" s="3"/>
+    </row>
+    <row r="62" spans="1:36">
       <c r="A62" s="3"/>
       <c r="B62" s="4"/>
       <c r="C62" s="4"/>
@@ -4218,7 +4388,7 @@
       <c r="R62" s="4"/>
       <c r="S62" s="4"/>
       <c r="T62" s="4"/>
-      <c r="U62" s="3"/>
+      <c r="U62" s="4"/>
       <c r="V62" s="3"/>
       <c r="W62" s="3"/>
       <c r="X62" s="3"/>
@@ -4233,8 +4403,9 @@
       <c r="AG62" s="3"/>
       <c r="AH62" s="3"/>
       <c r="AI62" s="3"/>
-    </row>
-    <row r="63" spans="1:35">
+      <c r="AJ62" s="3"/>
+    </row>
+    <row r="63" spans="1:36">
       <c r="A63" s="3"/>
       <c r="B63" s="4"/>
       <c r="C63" s="4"/>
@@ -4255,7 +4426,7 @@
       <c r="R63" s="4"/>
       <c r="S63" s="4"/>
       <c r="T63" s="4"/>
-      <c r="U63" s="3"/>
+      <c r="U63" s="4"/>
       <c r="V63" s="3"/>
       <c r="W63" s="3"/>
       <c r="X63" s="3"/>
@@ -4270,8 +4441,9 @@
       <c r="AG63" s="3"/>
       <c r="AH63" s="3"/>
       <c r="AI63" s="3"/>
-    </row>
-    <row r="64" spans="1:35">
+      <c r="AJ63" s="3"/>
+    </row>
+    <row r="64" spans="1:36">
       <c r="A64" s="3"/>
       <c r="B64" s="4"/>
       <c r="C64" s="4"/>
@@ -4292,7 +4464,7 @@
       <c r="R64" s="4"/>
       <c r="S64" s="4"/>
       <c r="T64" s="4"/>
-      <c r="U64" s="3"/>
+      <c r="U64" s="4"/>
       <c r="V64" s="3"/>
       <c r="W64" s="3"/>
       <c r="X64" s="3"/>
@@ -4307,8 +4479,9 @@
       <c r="AG64" s="3"/>
       <c r="AH64" s="3"/>
       <c r="AI64" s="3"/>
-    </row>
-    <row r="65" spans="1:35">
+      <c r="AJ64" s="3"/>
+    </row>
+    <row r="65" spans="1:36">
       <c r="A65" s="3"/>
       <c r="B65" s="4"/>
       <c r="C65" s="4"/>
@@ -4329,7 +4502,7 @@
       <c r="R65" s="4"/>
       <c r="S65" s="4"/>
       <c r="T65" s="4"/>
-      <c r="U65" s="3"/>
+      <c r="U65" s="4"/>
       <c r="V65" s="3"/>
       <c r="W65" s="3"/>
       <c r="X65" s="3"/>
@@ -4344,8 +4517,9 @@
       <c r="AG65" s="3"/>
       <c r="AH65" s="3"/>
       <c r="AI65" s="3"/>
-    </row>
-    <row r="66" spans="1:35">
+      <c r="AJ65" s="3"/>
+    </row>
+    <row r="66" spans="1:36">
       <c r="A66" s="3"/>
       <c r="B66" s="4"/>
       <c r="C66" s="4"/>
@@ -4366,7 +4540,7 @@
       <c r="R66" s="4"/>
       <c r="S66" s="4"/>
       <c r="T66" s="4"/>
-      <c r="U66" s="3"/>
+      <c r="U66" s="4"/>
       <c r="V66" s="3"/>
       <c r="W66" s="3"/>
       <c r="X66" s="3"/>
@@ -4381,8 +4555,9 @@
       <c r="AG66" s="3"/>
       <c r="AH66" s="3"/>
       <c r="AI66" s="3"/>
-    </row>
-    <row r="67" spans="1:35">
+      <c r="AJ66" s="3"/>
+    </row>
+    <row r="67" spans="1:36">
       <c r="A67" s="3"/>
       <c r="B67" s="4"/>
       <c r="C67" s="4"/>
@@ -4403,7 +4578,7 @@
       <c r="R67" s="4"/>
       <c r="S67" s="4"/>
       <c r="T67" s="4"/>
-      <c r="U67" s="3"/>
+      <c r="U67" s="4"/>
       <c r="V67" s="3"/>
       <c r="W67" s="3"/>
       <c r="X67" s="3"/>
@@ -4418,8 +4593,9 @@
       <c r="AG67" s="3"/>
       <c r="AH67" s="3"/>
       <c r="AI67" s="3"/>
-    </row>
-    <row r="68" spans="1:35">
+      <c r="AJ67" s="3"/>
+    </row>
+    <row r="68" spans="1:36">
       <c r="A68" s="3"/>
       <c r="B68" s="4"/>
       <c r="C68" s="4"/>
@@ -4440,7 +4616,7 @@
       <c r="R68" s="4"/>
       <c r="S68" s="4"/>
       <c r="T68" s="4"/>
-      <c r="U68" s="3"/>
+      <c r="U68" s="4"/>
       <c r="V68" s="3"/>
       <c r="W68" s="3"/>
       <c r="X68" s="3"/>
@@ -4455,8 +4631,9 @@
       <c r="AG68" s="3"/>
       <c r="AH68" s="3"/>
       <c r="AI68" s="3"/>
-    </row>
-    <row r="69" spans="1:35">
+      <c r="AJ68" s="3"/>
+    </row>
+    <row r="69" spans="1:36">
       <c r="A69" s="3"/>
       <c r="B69" s="4"/>
       <c r="C69" s="4"/>
@@ -4477,7 +4654,7 @@
       <c r="R69" s="4"/>
       <c r="S69" s="4"/>
       <c r="T69" s="4"/>
-      <c r="U69" s="3"/>
+      <c r="U69" s="4"/>
       <c r="V69" s="3"/>
       <c r="W69" s="3"/>
       <c r="X69" s="3"/>
@@ -4492,8 +4669,9 @@
       <c r="AG69" s="3"/>
       <c r="AH69" s="3"/>
       <c r="AI69" s="3"/>
-    </row>
-    <row r="70" spans="1:35">
+      <c r="AJ69" s="3"/>
+    </row>
+    <row r="70" spans="1:36">
       <c r="A70" s="3"/>
       <c r="B70" s="4"/>
       <c r="C70" s="4"/>
@@ -4514,7 +4692,7 @@
       <c r="R70" s="4"/>
       <c r="S70" s="4"/>
       <c r="T70" s="4"/>
-      <c r="U70" s="3"/>
+      <c r="U70" s="4"/>
       <c r="V70" s="3"/>
       <c r="W70" s="3"/>
       <c r="X70" s="3"/>
@@ -4529,8 +4707,9 @@
       <c r="AG70" s="3"/>
       <c r="AH70" s="3"/>
       <c r="AI70" s="3"/>
-    </row>
-    <row r="71" spans="1:35">
+      <c r="AJ70" s="3"/>
+    </row>
+    <row r="71" spans="1:36">
       <c r="A71" s="3"/>
       <c r="B71" s="4"/>
       <c r="C71" s="4"/>
@@ -4551,7 +4730,7 @@
       <c r="R71" s="4"/>
       <c r="S71" s="4"/>
       <c r="T71" s="4"/>
-      <c r="U71" s="3"/>
+      <c r="U71" s="4"/>
       <c r="V71" s="3"/>
       <c r="W71" s="3"/>
       <c r="X71" s="3"/>
@@ -4566,8 +4745,9 @@
       <c r="AG71" s="3"/>
       <c r="AH71" s="3"/>
       <c r="AI71" s="3"/>
-    </row>
-    <row r="72" spans="1:35">
+      <c r="AJ71" s="3"/>
+    </row>
+    <row r="72" spans="1:36">
       <c r="A72" s="3"/>
       <c r="B72" s="4"/>
       <c r="C72" s="4"/>
@@ -4588,7 +4768,7 @@
       <c r="R72" s="4"/>
       <c r="S72" s="4"/>
       <c r="T72" s="4"/>
-      <c r="U72" s="3"/>
+      <c r="U72" s="4"/>
       <c r="V72" s="3"/>
       <c r="W72" s="3"/>
       <c r="X72" s="3"/>
@@ -4603,8 +4783,9 @@
       <c r="AG72" s="3"/>
       <c r="AH72" s="3"/>
       <c r="AI72" s="3"/>
-    </row>
-    <row r="73" spans="1:35">
+      <c r="AJ72" s="3"/>
+    </row>
+    <row r="73" spans="1:36">
       <c r="A73" s="3"/>
       <c r="B73" s="4"/>
       <c r="C73" s="4"/>
@@ -4625,7 +4806,7 @@
       <c r="R73" s="4"/>
       <c r="S73" s="4"/>
       <c r="T73" s="4"/>
-      <c r="U73" s="3"/>
+      <c r="U73" s="4"/>
       <c r="V73" s="3"/>
       <c r="W73" s="3"/>
       <c r="X73" s="3"/>
@@ -4640,8 +4821,9 @@
       <c r="AG73" s="3"/>
       <c r="AH73" s="3"/>
       <c r="AI73" s="3"/>
-    </row>
-    <row r="74" spans="1:35">
+      <c r="AJ73" s="3"/>
+    </row>
+    <row r="74" spans="1:36">
       <c r="A74" s="3"/>
       <c r="B74" s="4"/>
       <c r="C74" s="4"/>
@@ -4662,7 +4844,7 @@
       <c r="R74" s="4"/>
       <c r="S74" s="4"/>
       <c r="T74" s="4"/>
-      <c r="U74" s="3"/>
+      <c r="U74" s="4"/>
       <c r="V74" s="3"/>
       <c r="W74" s="3"/>
       <c r="X74" s="3"/>
@@ -4677,8 +4859,9 @@
       <c r="AG74" s="3"/>
       <c r="AH74" s="3"/>
       <c r="AI74" s="3"/>
-    </row>
-    <row r="75" spans="1:35">
+      <c r="AJ74" s="3"/>
+    </row>
+    <row r="75" spans="1:36">
       <c r="A75" s="3"/>
       <c r="B75" s="4"/>
       <c r="C75" s="4"/>
@@ -4699,7 +4882,7 @@
       <c r="R75" s="4"/>
       <c r="S75" s="4"/>
       <c r="T75" s="4"/>
-      <c r="U75" s="3"/>
+      <c r="U75" s="4"/>
       <c r="V75" s="3"/>
       <c r="W75" s="3"/>
       <c r="X75" s="3"/>
@@ -4714,8 +4897,9 @@
       <c r="AG75" s="3"/>
       <c r="AH75" s="3"/>
       <c r="AI75" s="3"/>
-    </row>
-    <row r="76" spans="1:35">
+      <c r="AJ75" s="3"/>
+    </row>
+    <row r="76" spans="1:36">
       <c r="A76" s="3"/>
       <c r="B76" s="4"/>
       <c r="C76" s="4"/>
@@ -4736,7 +4920,7 @@
       <c r="R76" s="4"/>
       <c r="S76" s="4"/>
       <c r="T76" s="4"/>
-      <c r="U76" s="3"/>
+      <c r="U76" s="4"/>
       <c r="V76" s="3"/>
       <c r="W76" s="3"/>
       <c r="X76" s="3"/>
@@ -4751,8 +4935,9 @@
       <c r="AG76" s="3"/>
       <c r="AH76" s="3"/>
       <c r="AI76" s="3"/>
-    </row>
-    <row r="77" spans="1:35">
+      <c r="AJ76" s="3"/>
+    </row>
+    <row r="77" spans="1:36">
       <c r="A77" s="3"/>
       <c r="B77" s="4"/>
       <c r="C77" s="4"/>
@@ -4773,7 +4958,7 @@
       <c r="R77" s="4"/>
       <c r="S77" s="4"/>
       <c r="T77" s="4"/>
-      <c r="U77" s="3"/>
+      <c r="U77" s="4"/>
       <c r="V77" s="3"/>
       <c r="W77" s="3"/>
       <c r="X77" s="3"/>
@@ -4788,8 +4973,9 @@
       <c r="AG77" s="3"/>
       <c r="AH77" s="3"/>
       <c r="AI77" s="3"/>
-    </row>
-    <row r="78" spans="1:35">
+      <c r="AJ77" s="3"/>
+    </row>
+    <row r="78" spans="1:36">
       <c r="A78" s="3"/>
       <c r="B78" s="4"/>
       <c r="C78" s="4"/>
@@ -4810,7 +4996,7 @@
       <c r="R78" s="4"/>
       <c r="S78" s="4"/>
       <c r="T78" s="4"/>
-      <c r="U78" s="3"/>
+      <c r="U78" s="4"/>
       <c r="V78" s="3"/>
       <c r="W78" s="3"/>
       <c r="X78" s="3"/>
@@ -4825,194 +5011,195 @@
       <c r="AG78" s="3"/>
       <c r="AH78" s="3"/>
       <c r="AI78" s="3"/>
-    </row>
-    <row r="86" spans="1:24">
+      <c r="AJ78" s="3"/>
+    </row>
+    <row r="86" spans="1:25">
       <c r="A86" s="2"/>
       <c r="B86" s="2"/>
       <c r="C86" s="2"/>
       <c r="D86" s="2"/>
-      <c r="S86" s="2"/>
-      <c r="U86" s="2"/>
+      <c r="T86" s="2"/>
       <c r="V86" s="2"/>
       <c r="W86" s="2"/>
       <c r="X86" s="2"/>
-    </row>
-    <row r="87" spans="1:24">
+      <c r="Y86" s="2"/>
+    </row>
+    <row r="87" spans="1:25">
       <c r="A87" s="2"/>
       <c r="B87" s="2"/>
       <c r="C87" s="2"/>
       <c r="D87" s="2"/>
       <c r="E87" s="2"/>
-      <c r="S87" s="2"/>
       <c r="T87" s="2"/>
       <c r="U87" s="2"/>
       <c r="V87" s="2"/>
       <c r="W87" s="2"/>
       <c r="X87" s="2"/>
-    </row>
-    <row r="88" spans="1:24">
+      <c r="Y87" s="2"/>
+    </row>
+    <row r="88" spans="1:25">
       <c r="A88" s="2"/>
       <c r="B88" s="2"/>
       <c r="C88" s="2"/>
       <c r="D88" s="2"/>
-      <c r="S88" s="2"/>
       <c r="T88" s="2"/>
       <c r="U88" s="2"/>
       <c r="V88" s="2"/>
       <c r="W88" s="2"/>
       <c r="X88" s="2"/>
-    </row>
-    <row r="89" spans="1:24">
+      <c r="Y88" s="2"/>
+    </row>
+    <row r="89" spans="1:25">
       <c r="A89" s="2"/>
       <c r="B89" s="2"/>
       <c r="C89" s="2"/>
       <c r="D89" s="2"/>
-      <c r="S89" s="2"/>
       <c r="T89" s="2"/>
       <c r="U89" s="2"/>
       <c r="V89" s="2"/>
       <c r="W89" s="2"/>
       <c r="X89" s="2"/>
-    </row>
-    <row r="90" spans="1:24">
+      <c r="Y89" s="2"/>
+    </row>
+    <row r="90" spans="1:25">
       <c r="A90" s="2"/>
       <c r="B90" s="2"/>
       <c r="C90" s="2"/>
       <c r="D90" s="2"/>
-      <c r="S90" s="2"/>
       <c r="T90" s="2"/>
       <c r="U90" s="2"/>
       <c r="V90" s="2"/>
       <c r="W90" s="2"/>
       <c r="X90" s="2"/>
-    </row>
-    <row r="91" spans="1:24">
+      <c r="Y90" s="2"/>
+    </row>
+    <row r="91" spans="1:25">
       <c r="A91" s="2"/>
       <c r="B91" s="2"/>
       <c r="C91" s="2"/>
       <c r="D91" s="2"/>
-      <c r="S91" s="2"/>
       <c r="T91" s="2"/>
       <c r="U91" s="2"/>
       <c r="V91" s="2"/>
       <c r="W91" s="2"/>
       <c r="X91" s="2"/>
-    </row>
-    <row r="92" spans="1:24">
+      <c r="Y91" s="2"/>
+    </row>
+    <row r="92" spans="1:25">
       <c r="A92" s="2"/>
       <c r="B92" s="2"/>
       <c r="C92" s="2"/>
       <c r="D92" s="2"/>
-      <c r="S92" s="2"/>
       <c r="T92" s="2"/>
       <c r="U92" s="2"/>
       <c r="V92" s="2"/>
       <c r="W92" s="2"/>
       <c r="X92" s="2"/>
-    </row>
-    <row r="93" spans="1:24">
+      <c r="Y92" s="2"/>
+    </row>
+    <row r="93" spans="1:25">
       <c r="A93" s="2"/>
       <c r="B93" s="2"/>
       <c r="C93" s="2"/>
       <c r="D93" s="2"/>
-      <c r="S93" s="2"/>
       <c r="T93" s="2"/>
       <c r="U93" s="2"/>
       <c r="V93" s="2"/>
       <c r="W93" s="2"/>
       <c r="X93" s="2"/>
-    </row>
-    <row r="94" spans="1:24">
+      <c r="Y93" s="2"/>
+    </row>
+    <row r="94" spans="1:25">
       <c r="A94" s="2"/>
       <c r="B94" s="2"/>
       <c r="C94" s="2"/>
       <c r="D94" s="2"/>
-      <c r="S94" s="2"/>
       <c r="T94" s="2"/>
       <c r="U94" s="2"/>
       <c r="V94" s="2"/>
       <c r="W94" s="2"/>
       <c r="X94" s="2"/>
-    </row>
-    <row r="95" spans="1:24">
+      <c r="Y94" s="2"/>
+    </row>
+    <row r="95" spans="1:25">
       <c r="A95" s="2"/>
       <c r="B95" s="2"/>
       <c r="C95" s="2"/>
       <c r="D95" s="2"/>
-      <c r="S95" s="2"/>
       <c r="T95" s="2"/>
       <c r="U95" s="2"/>
       <c r="V95" s="2"/>
       <c r="W95" s="2"/>
       <c r="X95" s="2"/>
-    </row>
-    <row r="96" spans="1:24">
+      <c r="Y95" s="2"/>
+    </row>
+    <row r="96" spans="1:25">
       <c r="A96" s="2"/>
       <c r="B96" s="2"/>
       <c r="C96" s="2"/>
       <c r="D96" s="2"/>
-      <c r="S96" s="2"/>
       <c r="T96" s="2"/>
       <c r="U96" s="2"/>
       <c r="V96" s="2"/>
       <c r="W96" s="2"/>
       <c r="X96" s="2"/>
-    </row>
-    <row r="97" spans="1:24">
+      <c r="Y96" s="2"/>
+    </row>
+    <row r="97" spans="1:25">
       <c r="A97" s="2"/>
       <c r="B97" s="2"/>
       <c r="C97" s="2"/>
       <c r="D97" s="2"/>
-      <c r="S97" s="2"/>
       <c r="T97" s="2"/>
       <c r="U97" s="2"/>
       <c r="V97" s="2"/>
       <c r="W97" s="2"/>
       <c r="X97" s="2"/>
-    </row>
-    <row r="98" spans="1:24">
+      <c r="Y97" s="2"/>
+    </row>
+    <row r="98" spans="1:25">
       <c r="A98" s="2"/>
       <c r="B98" s="2"/>
       <c r="C98" s="2"/>
       <c r="D98" s="2"/>
-      <c r="S98" s="2"/>
       <c r="T98" s="2"/>
       <c r="U98" s="2"/>
       <c r="V98" s="2"/>
       <c r="W98" s="2"/>
       <c r="X98" s="2"/>
-    </row>
-    <row r="99" spans="1:24">
+      <c r="Y98" s="2"/>
+    </row>
+    <row r="99" spans="1:25">
       <c r="A99" s="2"/>
       <c r="B99" s="2"/>
       <c r="C99" s="2"/>
       <c r="D99" s="2"/>
-      <c r="S99" s="2"/>
       <c r="T99" s="2"/>
       <c r="U99" s="2"/>
       <c r="V99" s="2"/>
       <c r="W99" s="2"/>
       <c r="X99" s="2"/>
+      <c r="Y99" s="2"/>
     </row>
   </sheetData>
-  <dataValidations count="13">
+  <dataValidations count="14">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="O2:O1048576">
+      <formula1>"R_TYPE,I_TYPE,S_TYPE,B_TYPE,U_TYPE,J_TYPE,ICSR_TYPE,FENCE_TYPE,N_TYPE"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="M29 M30 M31 M39 M40 M41 M42 M43 M2:M28 M32:M38 M44:M1048576">
+      <formula1>"CSR_W,CSR_S,CSR_C,CSR_P,CSR_XX"</formula1>
+    </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H29 H30 H31 H40 H41 H42 H43 H10:H28 H32:H39 H44:H1048576">
       <formula1>"WB_ALU,WB_MEM,WB_PC4,WB_XX,WB_CSR"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F6 F15 F18 F19 F20 F21 F24 F25 F26 F27 F28 F29 F30 F31 F32 F33 F36 F37 F38 F39 F40 F41 F42 F43 F2:F5 F7:F14 F16:F17 F22:F23 F34:F35 F44:F1048576">
-      <formula1>"ALU_ADD,ALU_SUB,ALU_AND,ALU_OR,ALU_XOR,ALU_SLL,ALU_SRL,ALU_SLT,ALU_SLTU,ALU_COPY_A,ALU_COPY_B,ALU_SRA"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L5 L6 L7 L10 L11 L14 L15 L16 L17 L18 L19 L20 L21 L22 L23 L24 L25 L26 L27 L28 L29 L30 L31 L32 L33 L34 L35 L36 L37 L38 L39 L40 L41 L42 L43 L2:L4 L8:L9 L12:L13 L44:L1048576">
-      <formula1>"BR_EQ,BR_NE,BR_LTU,BR_GE,BR_GEU,BR_LT,BR_XX"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C29 C30 C31 C43 C2:C28 C32:C42 C44:C1048576">
       <formula1>"PC_4,PC_0,PC_ALU,PC_CSR"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="N4 N5 N6 N7 N8 N9 N10 N11 N12 N13 N14 N15 N16 N17 N18 N19 N20 N21 N22 N23 N24 N25 N26 N27 N28 N29 N30 N31 N32 N33 N34 N35 N36 N37 N38 N39 N40 N41 N42 N43 N2:N3 N44:N1048576">
-      <formula1>"INST_VALID,INST_INVALID"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E4 E5 E6 E7 E8 E9 E10 E11 E12 E13 E14 E15 E16 E17 E18 E19 E20 E21 E22 E23 E24 E25 E26 E27 E28 E29 E30 E31 E32 E33 E34 E35 E36 E37 E38 E39 E40 E41 E42 E43 E2:E3 E44:E1048576">
+      <formula1>"B_IMM,B_RS2"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D4 D5 D6 D7 D8 D9 D10 D11 D12 D13 D14 D15 D16 D17 D18 D19 D20 D21 D22 D23 D24 D25 D26 D27 D28 D29 D30 D31 D32 D33 D34 D35 D36 D37 D38 D39 D40 D41 D42 D43 D2:D3 D44:D1048576">
-      <formula1>"A_PC,A_RS1"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G4 G5 G6 G7 G8 G9 G10 G11 G12 G13 G14 G15 G16 G17 G18 G19 G20 G21 G22 G23 G24 G25 G26 G27 G28 G29 G30 G31 G32 G33 G34 G35 G36 G37 G38 G39 G40 G41 G42 G43 G2:G3 G44:G1048576">
+      <formula1>"IMM_I,IMM_J,IMM_U,IMM_S,IMM_B"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J5 J6 J7 J8 J9 J10 J11 J12 J13 J14 J15 J16 J17 J18 J19 J20 J21 J22 J23 J24 J25 J26 J27 J28 J29 J30 J31 J32 J33 J34 J35 J36 J37 J38 J39 J40 J41 J42 J43 J2:J4 J44:J1048576">
       <formula1>"ST_SW,ST_SH,ST_SB,ST_XX"</formula1>
@@ -5020,20 +5207,23 @@
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H5 H6 H7 H8 H9 H2:H4">
       <formula1>"WB_ALU,WB_MEM,WB_PC4,WB_XX"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K4 K5 K6 K7 K8 K9 K10 K11 K12 K13 K14 K15 K16 K17 K18 K19 K20 K21 K22 K23 K24 K25 K26 K27 K28 K29 K30 K31 K32 K33 K34 K35 K36 K37 K38 K39 K40 K41 K42 K43 K2:K3 K44:K1048576">
-      <formula1>"MASK_XX,MASK_B,MASK_H,MASK_W,MASK_D"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L5 L6 L7 L10 L11 L14 L15 L16 L17 L18 L19 L20 L21 L22 L23 L24 L25 L26 L27 L28 L29 L30 L31 L32 L33 L34 L35 L36 L37 L38 L39 L40 L41 L42 L43 L2:L4 L8:L9 L12:L13 L44:L1048576">
+      <formula1>"BR_EQ,BR_NE,BR_LTU,BR_GE,BR_GEU,BR_LT,BR_XX"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E4 E5 E6 E7 E8 E9 E10 E11 E12 E13 E14 E15 E16 E17 E18 E19 E20 E21 E22 E23 E24 E25 E26 E27 E28 E29 E30 E31 E32 E33 E34 E35 E36 E37 E38 E39 E40 E41 E42 E43 E2:E3 E44:E1048576">
-      <formula1>"B_IMM,B_RS2"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="M29 M30 M31 M39 M40 M41 M42 M43 M2:M28 M32:M38 M44:M1048576">
-      <formula1>"CSR_W,CSR_S,CSR_C,CSR_P,CSR_XX"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="N4 N5 N6 N7 N8 N9 N10 N11 N12 N13 N14 N15 N16 N17 N18 N19 N20 N21 N22 N23 N24 N25 N26 N27 N28 N29 N30 N31 N32 N33 N34 N35 N36 N37 N38 N39 N40 N41 N42 N43 N2:N3 N44:N1048576">
+      <formula1>"INST_VALID,INST_INVALID"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I4 I5 I6 I7 I8 I9 I10 I11 I12 I13 I14 I15 I16 I17 I18 I19 I20 I21 I22 I23 I24 I25 I26 I27 I28 I29 I30 I31 I32 I33 I34 I35 I36 I37 I38 I39 I40 I41 I42 I43 I2:I3 I44:I1048576">
       <formula1>"LD_LB,LD_LH,LD_LW,LD_LBU,LD_LHU,LD_XX"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G4 G5 G6 G7 G8 G9 G10 G11 G12 G13 G14 G15 G16 G17 G18 G19 G20 G21 G22 G23 G24 G25 G26 G27 G28 G29 G30 G31 G32 G33 G34 G35 G36 G37 G38 G39 G40 G41 G42 G43 G2:G3 G44:G1048576">
-      <formula1>"IMM_I,IMM_J,IMM_U,IMM_S,IMM_B"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F6 F15 F18 F19 F20 F21 F24 F25 F26 F27 F28 F29 F30 F31 F32 F33 F36 F37 F38 F39 F40 F41 F42 F43 F2:F5 F7:F14 F16:F17 F22:F23 F34:F35 F44:F1048576">
+      <formula1>"ALU_ADD,ALU_SUB,ALU_AND,ALU_OR,ALU_XOR,ALU_SLL,ALU_SRL,ALU_SLT,ALU_SLTU,ALU_COPY_A,ALU_COPY_B,ALU_SRA"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K4 K5 K6 K7 K8 K9 K10 K11 K12 K13 K14 K15 K16 K17 K18 K19 K20 K21 K22 K23 K24 K25 K26 K27 K28 K29 K30 K31 K32 K33 K34 K35 K36 K37 K38 K39 K40 K41 K42 K43 K2:K3 K44:K1048576">
+      <formula1>"MASK_XX,MASK_B,MASK_H,MASK_W,MASK_D"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D4 D5 D6 D7 D8 D9 D10 D11 D12 D13 D14 D15 D16 D17 D18 D19 D20 D21 D22 D23 D24 D25 D26 D27 D28 D29 D30 D31 D32 D33 D34 D35 D36 D37 D38 D39 D40 D41 D42 D43 D2:D3 D44:D1048576">
+      <formula1>"A_PC,A_RS1"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
> sim RTL ysyx_23060246 韩炳晋 Linux archlinux 6.12.17-1-lts #1 SMP PREEMPT_DYNAMIC Thu, 27 Feb 2025 14:12:30 +0000 x86_64 GNU/Linux  17:58:59 up 21:49,  1 user,  load average: 1.93, 1.56, 1.49
</commit_message>
<xml_diff>
--- a/npc/tools/control_gen/control_table.xlsx
+++ b/npc/tools/control_gen/control_table.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="23370" windowHeight="12150"/>
+    <workbookView windowHeight="17510"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="355" uniqueCount="119">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="358" uniqueCount="120">
   <si>
     <t>comment</t>
   </si>
@@ -349,10 +349,13 @@
     <t>fencei</t>
   </si>
   <si>
+    <t>ebreak</t>
+  </si>
+  <si>
+    <t>WB_XX</t>
+  </si>
+  <si>
     <t>default</t>
-  </si>
-  <si>
-    <t>WB_XX</t>
   </si>
   <si>
     <t>LD_XX</t>
@@ -379,9 +382,9 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="4">
     <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="42" formatCode="_ &quot;￥&quot;* #,##0_ ;_ &quot;￥&quot;* \-#,##0_ ;_ &quot;￥&quot;* &quot;-&quot;_ ;_ @_ "/>
     <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="41" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
+    <numFmt numFmtId="42" formatCode="_ &quot;￥&quot;* #,##0_ ;_ &quot;￥&quot;* \-#,##0_ ;_ &quot;￥&quot;* &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
   <fonts count="22">
     <font>
@@ -405,7 +408,37 @@
     </font>
     <font>
       <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
       <color theme="1"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="3"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="13"/>
+      <color theme="3"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C0006"/>
       <name val="宋体"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -418,33 +451,11 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <u/>
       <sz val="11"/>
       <color rgb="FF0000FF"/>
       <name val="宋体"/>
       <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="3"/>
-      <name val="宋体"/>
-      <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -466,7 +477,7 @@
     <font>
       <b/>
       <sz val="11"/>
-      <color rgb="FF3F3F3F"/>
+      <color theme="1"/>
       <name val="宋体"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -480,16 +491,9 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color rgb="FF9C0006"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <b/>
       <sz val="11"/>
-      <color theme="1"/>
+      <color rgb="FF3F3F3F"/>
       <name val="宋体"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -497,6 +501,13 @@
     <font>
       <sz val="11"/>
       <color rgb="FF9C6500"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
       <name val="宋体"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -511,17 +522,17 @@
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FF006100"/>
+      <color rgb="FF3F3F76"/>
       <name val="宋体"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <sz val="13"/>
-      <color theme="3"/>
+      <i/>
+      <sz val="11"/>
+      <color rgb="FF7F7F7F"/>
       <name val="宋体"/>
-      <charset val="134"/>
+      <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -533,16 +544,8 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <i/>
       <sz val="11"/>
-      <color rgb="FF7F7F7F"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF3F3F76"/>
+      <color rgb="FF006100"/>
       <name val="宋体"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -563,54 +566,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="9"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor theme="8" tint="0.599993896298105"/>
         <bgColor indexed="64"/>
       </patternFill>
@@ -623,7 +578,97 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor theme="9" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFA5A5A5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.799981688894314"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -635,37 +680,25 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
+        <fgColor theme="6"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.599993896298105"/>
+        <fgColor theme="5" tint="0.399975585192419"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFA5A5A5"/>
+        <fgColor theme="8" tint="0.799981688894314"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.399975585192419"/>
+        <fgColor theme="4" tint="0.399975585192419"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -677,7 +710,19 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
+        <fgColor theme="6" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFCC99"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -689,55 +734,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.399975585192419"/>
+        <fgColor theme="7"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.399975585192419"/>
+        <fgColor theme="8"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -748,21 +751,6 @@
       <right/>
       <top/>
       <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFB2B2B2"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFB2B2B2"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFB2B2B2"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFB2B2B2"/>
-      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -784,17 +772,22 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF3F3F3F"/>
-      </right>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
       <top style="thin">
-        <color rgb="FF3F3F3F"/>
+        <color theme="4"/>
       </top>
-      <bottom style="thin">
-        <color rgb="FF3F3F3F"/>
+      <bottom style="double">
+        <color theme="4"/>
       </bottom>
       <diagonal/>
     </border>
@@ -814,13 +807,17 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right/>
+      <left style="thin">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF3F3F3F"/>
+      </right>
       <top style="thin">
-        <color theme="4"/>
+        <color rgb="FF3F3F3F"/>
       </top>
-      <bottom style="double">
-        <color theme="4"/>
+      <bottom style="thin">
+        <color rgb="FF3F3F3F"/>
       </bottom>
       <diagonal/>
     </border>
@@ -840,11 +837,17 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4"/>
+      <left style="thin">
+        <color rgb="FFB2B2B2"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFB2B2B2"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFB2B2B2"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFB2B2B2"/>
       </bottom>
       <diagonal/>
     </border>
@@ -853,148 +856,148 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="8" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="28" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="16" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="14" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="16" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="30" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="15" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="17" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="15" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="29" borderId="8" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
@@ -1339,28 +1342,28 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:AJ99"/>
+  <dimension ref="A1:AJ100"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
     <col min="1" max="1" width="13.1" customWidth="1"/>
-    <col min="2" max="2" width="17.7583333333333" customWidth="1"/>
-    <col min="3" max="3" width="10.1416666666667" customWidth="1"/>
-    <col min="4" max="4" width="7.75" customWidth="1"/>
-    <col min="5" max="5" width="11.7166666666667" customWidth="1"/>
-    <col min="6" max="6" width="11.1166666666667" customWidth="1"/>
-    <col min="7" max="7" width="10.9416666666667" customWidth="1"/>
-    <col min="8" max="10" width="11.9833333333333" customWidth="1"/>
-    <col min="11" max="11" width="15.075" customWidth="1"/>
-    <col min="12" max="14" width="12.1083333333333" customWidth="1"/>
-    <col min="15" max="16" width="10.8583333333333" customWidth="1"/>
-    <col min="18" max="18" width="14.2166666666667" customWidth="1"/>
-    <col min="19" max="19" width="11.8083333333333" customWidth="1"/>
+    <col min="2" max="2" width="17.7545454545455" customWidth="1"/>
+    <col min="3" max="3" width="10.1454545454545" customWidth="1"/>
+    <col min="4" max="4" width="7.75454545454545" customWidth="1"/>
+    <col min="5" max="5" width="11.7181818181818" customWidth="1"/>
+    <col min="6" max="6" width="11.1181818181818" customWidth="1"/>
+    <col min="7" max="7" width="10.9454545454545" customWidth="1"/>
+    <col min="8" max="10" width="11.9818181818182" customWidth="1"/>
+    <col min="11" max="11" width="15.0727272727273" customWidth="1"/>
+    <col min="12" max="14" width="12.1090909090909" customWidth="1"/>
+    <col min="15" max="16" width="10.8545454545455" customWidth="1"/>
+    <col min="18" max="18" width="14.2181818181818" customWidth="1"/>
+    <col min="19" max="19" width="11.8090909090909" customWidth="1"/>
     <col min="20" max="20" width="10.6" customWidth="1"/>
-    <col min="21" max="21" width="9.70833333333333" customWidth="1"/>
-    <col min="22" max="22" width="11.1666666666667" customWidth="1"/>
-    <col min="23" max="23" width="11.4083333333333" customWidth="1"/>
-    <col min="24" max="24" width="12.0583333333333" customWidth="1"/>
-    <col min="25" max="25" width="15.575" customWidth="1"/>
+    <col min="21" max="21" width="9.70909090909091" customWidth="1"/>
+    <col min="22" max="22" width="11.1636363636364" customWidth="1"/>
+    <col min="23" max="23" width="11.4090909090909" customWidth="1"/>
+    <col min="24" max="24" width="12.0545454545455" customWidth="1"/>
+    <col min="25" max="25" width="15.5727272727273" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1" spans="1:24">
@@ -3664,45 +3667,23 @@
       <c r="B44" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="C44" s="2" t="s">
-        <v>100</v>
-      </c>
-      <c r="D44" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="E44" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="F44" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="G44" s="2" t="s">
-        <v>26</v>
-      </c>
+      <c r="C44" s="2"/>
+      <c r="D44" s="2"/>
+      <c r="E44" s="2"/>
+      <c r="F44" s="2"/>
+      <c r="G44" s="2"/>
       <c r="H44" s="4" t="s">
         <v>112</v>
       </c>
-      <c r="I44" s="4" t="s">
-        <v>113</v>
-      </c>
-      <c r="J44" s="4" t="s">
-        <v>114</v>
-      </c>
-      <c r="K44" s="2" t="s">
-        <v>115</v>
-      </c>
-      <c r="L44" s="2" t="s">
-        <v>116</v>
-      </c>
-      <c r="M44" s="2" t="s">
-        <v>117</v>
-      </c>
+      <c r="I44" s="4"/>
+      <c r="J44" s="4"/>
+      <c r="K44" s="2"/>
+      <c r="L44" s="2"/>
+      <c r="M44" s="2"/>
       <c r="N44" s="2" t="s">
-        <v>118</v>
-      </c>
-      <c r="O44" s="2" t="s">
-        <v>82</v>
-      </c>
+        <v>19</v>
+      </c>
+      <c r="O44" s="2"/>
       <c r="P44" s="2"/>
       <c r="Q44" s="2"/>
       <c r="R44" s="2"/>
@@ -3721,32 +3702,55 @@
       <c r="AI44" s="3"/>
       <c r="AJ44" s="3"/>
     </row>
-    <row r="45" spans="1:36">
-      <c r="A45" s="3"/>
-      <c r="B45" s="4"/>
-      <c r="C45" s="4"/>
-      <c r="D45" s="4"/>
-      <c r="E45" s="4"/>
-      <c r="F45" s="4"/>
-      <c r="G45" s="4"/>
-      <c r="H45" s="4"/>
-      <c r="I45" s="4"/>
-      <c r="J45" s="4"/>
-      <c r="K45" s="4"/>
-      <c r="L45" s="4"/>
-      <c r="M45" s="4"/>
-      <c r="N45" s="4"/>
-      <c r="O45" s="4"/>
-      <c r="P45" s="4"/>
-      <c r="Q45" s="4"/>
-      <c r="R45" s="4"/>
-      <c r="S45" s="4"/>
-      <c r="T45" s="4"/>
-      <c r="U45" s="4"/>
-      <c r="V45" s="3"/>
-      <c r="W45" s="3"/>
-      <c r="X45" s="3"/>
-      <c r="Y45" s="3"/>
+    <row r="45" spans="2:36">
+      <c r="B45" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="C45" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="D45" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="E45" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="F45" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="G45" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="H45" s="4" t="s">
+        <v>112</v>
+      </c>
+      <c r="I45" s="4" t="s">
+        <v>114</v>
+      </c>
+      <c r="J45" s="4" t="s">
+        <v>115</v>
+      </c>
+      <c r="K45" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="L45" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="M45" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="N45" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="O45" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="P45" s="2"/>
+      <c r="Q45" s="2"/>
+      <c r="R45" s="2"/>
+      <c r="S45" s="2"/>
+      <c r="T45" s="2"/>
+      <c r="U45" s="2"/>
       <c r="Z45" s="3"/>
       <c r="AA45" s="3"/>
       <c r="AB45" s="3"/>
@@ -3759,7 +3763,7 @@
       <c r="AI45" s="3"/>
       <c r="AJ45" s="3"/>
     </row>
-    <row r="46" s="1" customFormat="1" spans="1:36">
+    <row r="46" spans="1:36">
       <c r="A46" s="3"/>
       <c r="B46" s="4"/>
       <c r="C46" s="4"/>
@@ -3835,7 +3839,7 @@
       <c r="AI47" s="3"/>
       <c r="AJ47" s="3"/>
     </row>
-    <row r="48" spans="1:36">
+    <row r="48" s="1" customFormat="1" spans="1:36">
       <c r="A48" s="3"/>
       <c r="B48" s="4"/>
       <c r="C48" s="4"/>
@@ -4410,7 +4414,7 @@
       <c r="B63" s="4"/>
       <c r="C63" s="4"/>
       <c r="D63" s="4"/>
-      <c r="E63" s="5"/>
+      <c r="E63" s="4"/>
       <c r="F63" s="4"/>
       <c r="G63" s="4"/>
       <c r="H63" s="4"/>
@@ -4524,7 +4528,7 @@
       <c r="B66" s="4"/>
       <c r="C66" s="4"/>
       <c r="D66" s="4"/>
-      <c r="E66" s="4"/>
+      <c r="E66" s="5"/>
       <c r="F66" s="4"/>
       <c r="G66" s="4"/>
       <c r="H66" s="4"/>
@@ -4676,7 +4680,7 @@
       <c r="B70" s="4"/>
       <c r="C70" s="4"/>
       <c r="D70" s="4"/>
-      <c r="E70" s="5"/>
+      <c r="E70" s="4"/>
       <c r="F70" s="4"/>
       <c r="G70" s="4"/>
       <c r="H70" s="4"/>
@@ -4714,7 +4718,7 @@
       <c r="B71" s="4"/>
       <c r="C71" s="4"/>
       <c r="D71" s="4"/>
-      <c r="E71" s="4"/>
+      <c r="E71" s="5"/>
       <c r="F71" s="4"/>
       <c r="G71" s="4"/>
       <c r="H71" s="4"/>
@@ -5013,25 +5017,50 @@
       <c r="AI78" s="3"/>
       <c r="AJ78" s="3"/>
     </row>
-    <row r="86" spans="1:25">
-      <c r="A86" s="2"/>
-      <c r="B86" s="2"/>
-      <c r="C86" s="2"/>
-      <c r="D86" s="2"/>
-      <c r="T86" s="2"/>
-      <c r="V86" s="2"/>
-      <c r="W86" s="2"/>
-      <c r="X86" s="2"/>
-      <c r="Y86" s="2"/>
+    <row r="79" spans="1:36">
+      <c r="A79" s="3"/>
+      <c r="B79" s="4"/>
+      <c r="C79" s="4"/>
+      <c r="D79" s="4"/>
+      <c r="E79" s="4"/>
+      <c r="F79" s="4"/>
+      <c r="G79" s="4"/>
+      <c r="H79" s="4"/>
+      <c r="I79" s="4"/>
+      <c r="J79" s="4"/>
+      <c r="K79" s="4"/>
+      <c r="L79" s="4"/>
+      <c r="M79" s="4"/>
+      <c r="N79" s="4"/>
+      <c r="O79" s="4"/>
+      <c r="P79" s="4"/>
+      <c r="Q79" s="4"/>
+      <c r="R79" s="4"/>
+      <c r="S79" s="4"/>
+      <c r="T79" s="4"/>
+      <c r="U79" s="4"/>
+      <c r="V79" s="3"/>
+      <c r="W79" s="3"/>
+      <c r="X79" s="3"/>
+      <c r="Y79" s="3"/>
+      <c r="Z79" s="3"/>
+      <c r="AA79" s="3"/>
+      <c r="AB79" s="3"/>
+      <c r="AC79" s="3"/>
+      <c r="AD79" s="3"/>
+      <c r="AE79" s="3"/>
+      <c r="AF79" s="3"/>
+      <c r="AG79" s="3"/>
+      <c r="AH79" s="3"/>
+      <c r="AI79" s="3"/>
+      <c r="AJ79" s="3"/>
     </row>
     <row r="87" spans="1:25">
       <c r="A87" s="2"/>
       <c r="B87" s="2"/>
       <c r="C87" s="2"/>
       <c r="D87" s="2"/>
-      <c r="E87" s="2"/>
       <c r="T87" s="2"/>
-      <c r="U87" s="2"/>
       <c r="V87" s="2"/>
       <c r="W87" s="2"/>
       <c r="X87" s="2"/>
@@ -5042,6 +5071,7 @@
       <c r="B88" s="2"/>
       <c r="C88" s="2"/>
       <c r="D88" s="2"/>
+      <c r="E88" s="2"/>
       <c r="T88" s="2"/>
       <c r="U88" s="2"/>
       <c r="V88" s="2"/>
@@ -5181,48 +5211,60 @@
       <c r="X99" s="2"/>
       <c r="Y99" s="2"/>
     </row>
+    <row r="100" spans="1:25">
+      <c r="A100" s="2"/>
+      <c r="B100" s="2"/>
+      <c r="C100" s="2"/>
+      <c r="D100" s="2"/>
+      <c r="T100" s="2"/>
+      <c r="U100" s="2"/>
+      <c r="V100" s="2"/>
+      <c r="W100" s="2"/>
+      <c r="X100" s="2"/>
+      <c r="Y100" s="2"/>
+    </row>
   </sheetData>
   <dataValidations count="14">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="O2:O1048576">
-      <formula1>"R_TYPE,I_TYPE,S_TYPE,B_TYPE,U_TYPE,J_TYPE,ICSR_TYPE,FENCE_TYPE,N_TYPE"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="M29 M30 M31 M39 M40 M41 M42 M43 M2:M28 M32:M38 M44:M1048576">
-      <formula1>"CSR_W,CSR_S,CSR_C,CSR_P,CSR_XX"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H29 H30 H31 H40 H41 H42 H43 H10:H28 H32:H39 H44:H1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H29 H30 H31 H40 H41 H42 H43 H44 H10:H28 H32:H39 H45:H1048576">
       <formula1>"WB_ALU,WB_MEM,WB_PC4,WB_XX,WB_CSR"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C29 C30 C31 C43 C2:C28 C32:C42 C44:C1048576">
-      <formula1>"PC_4,PC_0,PC_ALU,PC_CSR"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E4 E5 E6 E7 E8 E9 E10 E11 E12 E13 E14 E15 E16 E17 E18 E19 E20 E21 E22 E23 E24 E25 E26 E27 E28 E29 E30 E31 E32 E33 E34 E35 E36 E37 E38 E39 E40 E41 E42 E43 E2:E3 E44:E1048576">
-      <formula1>"B_IMM,B_RS2"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G4 G5 G6 G7 G8 G9 G10 G11 G12 G13 G14 G15 G16 G17 G18 G19 G20 G21 G22 G23 G24 G25 G26 G27 G28 G29 G30 G31 G32 G33 G34 G35 G36 G37 G38 G39 G40 G41 G42 G43 G2:G3 G44:G1048576">
-      <formula1>"IMM_I,IMM_J,IMM_U,IMM_S,IMM_B"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J5 J6 J7 J8 J9 J10 J11 J12 J13 J14 J15 J16 J17 J18 J19 J20 J21 J22 J23 J24 J25 J26 J27 J28 J29 J30 J31 J32 J33 J34 J35 J36 J37 J38 J39 J40 J41 J42 J43 J2:J4 J44:J1048576">
-      <formula1>"ST_SW,ST_SH,ST_SB,ST_XX"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L5 L6 L7 L10 L11 L14 L15 L16 L17 L18 L19 L20 L21 L22 L23 L24 L25 L26 L27 L28 L29 L30 L31 L32 L33 L34 L35 L36 L37 L38 L39 L40 L41 L42 L43 L44 L2:L4 L8:L9 L12:L13 L45:L1048576">
+      <formula1>"BR_EQ,BR_NE,BR_LTU,BR_GE,BR_GEU,BR_LT,BR_XX"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H5 H6 H7 H8 H9 H2:H4">
       <formula1>"WB_ALU,WB_MEM,WB_PC4,WB_XX"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L5 L6 L7 L10 L11 L14 L15 L16 L17 L18 L19 L20 L21 L22 L23 L24 L25 L26 L27 L28 L29 L30 L31 L32 L33 L34 L35 L36 L37 L38 L39 L40 L41 L42 L43 L2:L4 L8:L9 L12:L13 L44:L1048576">
-      <formula1>"BR_EQ,BR_NE,BR_LTU,BR_GE,BR_GEU,BR_LT,BR_XX"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="M29 M30 M31 M39 M40 M41 M42 M43 M44 M2:M28 M32:M38 M45:M1048576">
+      <formula1>"CSR_W,CSR_S,CSR_C,CSR_P,CSR_XX"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="N4 N5 N6 N7 N8 N9 N10 N11 N12 N13 N14 N15 N16 N17 N18 N19 N20 N21 N22 N23 N24 N25 N26 N27 N28 N29 N30 N31 N32 N33 N34 N35 N36 N37 N38 N39 N40 N41 N42 N43 N2:N3 N44:N1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E4 E5 E6 E7 E8 E9 E10 E11 E12 E13 E14 E15 E16 E17 E18 E19 E20 E21 E22 E23 E24 E25 E26 E27 E28 E29 E30 E31 E32 E33 E34 E35 E36 E37 E38 E39 E40 E41 E42 E43 E44 E2:E3 E45:E1048576">
+      <formula1>"B_IMM,B_RS2"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C29 C30 C31 C43 C44 C2:C28 C32:C42 C45:C1048576">
+      <formula1>"PC_4,PC_0,PC_ALU,PC_CSR"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="N4 N5 N6 N7 N8 N9 N10 N11 N12 N13 N14 N15 N16 N17 N18 N19 N20 N21 N22 N23 N24 N25 N26 N27 N28 N29 N30 N31 N32 N33 N34 N35 N36 N37 N38 N39 N40 N41 N42 N43 N44 N2:N3 N45:N1048576">
       <formula1>"INST_VALID,INST_INVALID"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I4 I5 I6 I7 I8 I9 I10 I11 I12 I13 I14 I15 I16 I17 I18 I19 I20 I21 I22 I23 I24 I25 I26 I27 I28 I29 I30 I31 I32 I33 I34 I35 I36 I37 I38 I39 I40 I41 I42 I43 I2:I3 I44:I1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I4 I5 I6 I7 I8 I9 I10 I11 I12 I13 I14 I15 I16 I17 I18 I19 I20 I21 I22 I23 I24 I25 I26 I27 I28 I29 I30 I31 I32 I33 I34 I35 I36 I37 I38 I39 I40 I41 I42 I43 I44 I2:I3 I45:I1048576">
       <formula1>"LD_LB,LD_LH,LD_LW,LD_LBU,LD_LHU,LD_XX"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F6 F15 F18 F19 F20 F21 F24 F25 F26 F27 F28 F29 F30 F31 F32 F33 F36 F37 F38 F39 F40 F41 F42 F43 F2:F5 F7:F14 F16:F17 F22:F23 F34:F35 F44:F1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="O44 O2:O43 O45:O1048576">
+      <formula1>"R_TYPE,I_TYPE,S_TYPE,B_TYPE,U_TYPE,J_TYPE,ICSR_TYPE,FENCE_TYPE,N_TYPE"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J5 J6 J7 J8 J9 J10 J11 J12 J13 J14 J15 J16 J17 J18 J19 J20 J21 J22 J23 J24 J25 J26 J27 J28 J29 J30 J31 J32 J33 J34 J35 J36 J37 J38 J39 J40 J41 J42 J43 J44 J2:J4 J45:J1048576">
+      <formula1>"ST_SW,ST_SH,ST_SB,ST_XX"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G4 G5 G6 G7 G8 G9 G10 G11 G12 G13 G14 G15 G16 G17 G18 G19 G20 G21 G22 G23 G24 G25 G26 G27 G28 G29 G30 G31 G32 G33 G34 G35 G36 G37 G38 G39 G40 G41 G42 G43 G44 G2:G3 G45:G1048576">
+      <formula1>"IMM_I,IMM_J,IMM_U,IMM_S,IMM_B"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K4 K5 K6 K7 K8 K9 K10 K11 K12 K13 K14 K15 K16 K17 K18 K19 K20 K21 K22 K23 K24 K25 K26 K27 K28 K29 K30 K31 K32 K33 K34 K35 K36 K37 K38 K39 K40 K41 K42 K43 K44 K2:K3 K45:K1048576">
+      <formula1>"MASK_XX,MASK_B,MASK_H,MASK_W,MASK_D"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F6 F15 F18 F19 F20 F21 F24 F25 F26 F27 F28 F29 F30 F31 F32 F33 F36 F37 F38 F39 F40 F41 F42 F43 F44 F2:F5 F7:F14 F16:F17 F22:F23 F34:F35 F45:F1048576">
       <formula1>"ALU_ADD,ALU_SUB,ALU_AND,ALU_OR,ALU_XOR,ALU_SLL,ALU_SRL,ALU_SLT,ALU_SLTU,ALU_COPY_A,ALU_COPY_B,ALU_SRA"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K4 K5 K6 K7 K8 K9 K10 K11 K12 K13 K14 K15 K16 K17 K18 K19 K20 K21 K22 K23 K24 K25 K26 K27 K28 K29 K30 K31 K32 K33 K34 K35 K36 K37 K38 K39 K40 K41 K42 K43 K2:K3 K44:K1048576">
-      <formula1>"MASK_XX,MASK_B,MASK_H,MASK_W,MASK_D"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D4 D5 D6 D7 D8 D9 D10 D11 D12 D13 D14 D15 D16 D17 D18 D19 D20 D21 D22 D23 D24 D25 D26 D27 D28 D29 D30 D31 D32 D33 D34 D35 D36 D37 D38 D39 D40 D41 D42 D43 D2:D3 D44:D1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D4 D5 D6 D7 D8 D9 D10 D11 D12 D13 D14 D15 D16 D17 D18 D19 D20 D21 D22 D23 D24 D25 D26 D27 D28 D29 D30 D31 D32 D33 D34 D35 D36 D37 D38 D39 D40 D41 D42 D43 D44 D2:D3 D45:D1048576">
       <formula1>"A_PC,A_RS1"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
> sim RTL ysyx_23060246 韩炳晋 Linux archlinux 6.12.17-1-lts #1 SMP PREEMPT_DYNAMIC Thu, 27 Feb 2025 14:12:30 +0000 x86_64 GNU/Linux  18:03:06 up 21:53,  1 user,  load average: 2.02, 1.81, 1.61
</commit_message>
<xml_diff>
--- a/npc/tools/control_gen/control_table.xlsx
+++ b/npc/tools/control_gen/control_table.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowHeight="17510"/>
+    <workbookView windowWidth="23370" windowHeight="12150"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="358" uniqueCount="120">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="355" uniqueCount="119">
   <si>
     <t>comment</t>
   </si>
@@ -349,13 +349,10 @@
     <t>fencei</t>
   </si>
   <si>
-    <t>ebreak</t>
+    <t>default</t>
   </si>
   <si>
     <t>WB_XX</t>
-  </si>
-  <si>
-    <t>default</t>
   </si>
   <si>
     <t>LD_XX</t>
@@ -382,9 +379,9 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="4">
     <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="42" formatCode="_ &quot;￥&quot;* #,##0_ ;_ &quot;￥&quot;* \-#,##0_ ;_ &quot;￥&quot;* &quot;-&quot;_ ;_ @_ "/>
     <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="41" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="42" formatCode="_ &quot;￥&quot;* #,##0_ ;_ &quot;￥&quot;* \-#,##0_ ;_ &quot;￥&quot;* &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
   <fonts count="22">
     <font>
@@ -408,37 +405,7 @@
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
       <color theme="1"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="3"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="13"/>
-      <color theme="3"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C0006"/>
       <name val="宋体"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -451,11 +418,33 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <u/>
       <sz val="11"/>
       <color rgb="FF0000FF"/>
       <name val="宋体"/>
       <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="3"/>
+      <name val="宋体"/>
+      <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -477,7 +466,7 @@
     <font>
       <b/>
       <sz val="11"/>
-      <color theme="1"/>
+      <color rgb="FF3F3F3F"/>
       <name val="宋体"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -491,9 +480,16 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="11"/>
+      <color rgb="FF9C0006"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <b/>
       <sz val="11"/>
-      <color rgb="FF3F3F3F"/>
+      <color theme="1"/>
       <name val="宋体"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -501,13 +497,6 @@
     <font>
       <sz val="11"/>
       <color rgb="FF9C6500"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
       <name val="宋体"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -522,9 +511,25 @@
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FF3F3F76"/>
+      <color rgb="FF006100"/>
       <name val="宋体"/>
       <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="13"/>
+      <color theme="3"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="15"/>
+      <color theme="3"/>
+      <name val="宋体"/>
+      <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -536,16 +541,8 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <sz val="15"/>
-      <color theme="3"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <sz val="11"/>
-      <color rgb="FF006100"/>
+      <color rgb="FF3F3F76"/>
       <name val="宋体"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -566,6 +563,54 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor theme="8" tint="0.599993896298105"/>
         <bgColor indexed="64"/>
       </patternFill>
@@ -578,7 +623,73 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFA5A5A5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="FFFFC7CE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.399975585192419"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -590,25 +701,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor theme="4"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.599993896298105"/>
+        <fgColor theme="5"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -620,73 +719,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="9"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFA5A5A5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor theme="6"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.399975585192419"/>
+        <fgColor rgb="FFFFCC99"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -698,49 +737,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8"/>
+        <fgColor theme="9" tint="0.399975585192419"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -751,6 +748,21 @@
       <right/>
       <top/>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFB2B2B2"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFB2B2B2"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFB2B2B2"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFB2B2B2"/>
+      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -772,22 +784,17 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
+      <left style="thin">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF3F3F3F"/>
+      </right>
       <top style="thin">
-        <color theme="4"/>
+        <color rgb="FF3F3F3F"/>
       </top>
-      <bottom style="double">
-        <color theme="4"/>
+      <bottom style="thin">
+        <color rgb="FF3F3F3F"/>
       </bottom>
       <diagonal/>
     </border>
@@ -807,17 +814,13 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF3F3F3F"/>
-      </right>
+      <left/>
+      <right/>
       <top style="thin">
-        <color rgb="FF3F3F3F"/>
+        <color theme="4"/>
       </top>
-      <bottom style="thin">
-        <color rgb="FF3F3F3F"/>
+      <bottom style="double">
+        <color theme="4"/>
       </bottom>
       <diagonal/>
     </border>
@@ -837,17 +840,11 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color rgb="FFB2B2B2"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFB2B2B2"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFB2B2B2"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFB2B2B2"/>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4"/>
       </bottom>
       <diagonal/>
     </border>
@@ -856,148 +853,148 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="28" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="4" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="30" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="15" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="16" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="15" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="17" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="15" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="14" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="16" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="29" borderId="8" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="3" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
@@ -1342,28 +1339,28 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:AJ100"/>
+  <dimension ref="A1:AJ99"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
     <col min="1" max="1" width="13.1" customWidth="1"/>
-    <col min="2" max="2" width="17.7545454545455" customWidth="1"/>
-    <col min="3" max="3" width="10.1454545454545" customWidth="1"/>
-    <col min="4" max="4" width="7.75454545454545" customWidth="1"/>
-    <col min="5" max="5" width="11.7181818181818" customWidth="1"/>
-    <col min="6" max="6" width="11.1181818181818" customWidth="1"/>
-    <col min="7" max="7" width="10.9454545454545" customWidth="1"/>
-    <col min="8" max="10" width="11.9818181818182" customWidth="1"/>
-    <col min="11" max="11" width="15.0727272727273" customWidth="1"/>
-    <col min="12" max="14" width="12.1090909090909" customWidth="1"/>
-    <col min="15" max="16" width="10.8545454545455" customWidth="1"/>
-    <col min="18" max="18" width="14.2181818181818" customWidth="1"/>
-    <col min="19" max="19" width="11.8090909090909" customWidth="1"/>
+    <col min="2" max="2" width="17.7583333333333" customWidth="1"/>
+    <col min="3" max="3" width="10.1416666666667" customWidth="1"/>
+    <col min="4" max="4" width="7.75" customWidth="1"/>
+    <col min="5" max="5" width="11.7166666666667" customWidth="1"/>
+    <col min="6" max="6" width="11.1166666666667" customWidth="1"/>
+    <col min="7" max="7" width="10.9416666666667" customWidth="1"/>
+    <col min="8" max="10" width="11.9833333333333" customWidth="1"/>
+    <col min="11" max="11" width="15.075" customWidth="1"/>
+    <col min="12" max="14" width="12.1083333333333" customWidth="1"/>
+    <col min="15" max="16" width="10.8583333333333" customWidth="1"/>
+    <col min="18" max="18" width="14.2166666666667" customWidth="1"/>
+    <col min="19" max="19" width="11.8083333333333" customWidth="1"/>
     <col min="20" max="20" width="10.6" customWidth="1"/>
-    <col min="21" max="21" width="9.70909090909091" customWidth="1"/>
-    <col min="22" max="22" width="11.1636363636364" customWidth="1"/>
-    <col min="23" max="23" width="11.4090909090909" customWidth="1"/>
-    <col min="24" max="24" width="12.0545454545455" customWidth="1"/>
-    <col min="25" max="25" width="15.5727272727273" customWidth="1"/>
+    <col min="21" max="21" width="9.70833333333333" customWidth="1"/>
+    <col min="22" max="22" width="11.1666666666667" customWidth="1"/>
+    <col min="23" max="23" width="11.4083333333333" customWidth="1"/>
+    <col min="24" max="24" width="12.0583333333333" customWidth="1"/>
+    <col min="25" max="25" width="15.575" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1" spans="1:24">
@@ -3667,23 +3664,45 @@
       <c r="B44" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="C44" s="2"/>
-      <c r="D44" s="2"/>
-      <c r="E44" s="2"/>
-      <c r="F44" s="2"/>
-      <c r="G44" s="2"/>
+      <c r="C44" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="D44" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="E44" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="F44" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="G44" s="2" t="s">
+        <v>26</v>
+      </c>
       <c r="H44" s="4" t="s">
         <v>112</v>
       </c>
-      <c r="I44" s="4"/>
-      <c r="J44" s="4"/>
-      <c r="K44" s="2"/>
-      <c r="L44" s="2"/>
-      <c r="M44" s="2"/>
+      <c r="I44" s="4" t="s">
+        <v>113</v>
+      </c>
+      <c r="J44" s="4" t="s">
+        <v>114</v>
+      </c>
+      <c r="K44" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="L44" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="M44" s="2" t="s">
+        <v>117</v>
+      </c>
       <c r="N44" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="O44" s="2"/>
+        <v>118</v>
+      </c>
+      <c r="O44" s="2" t="s">
+        <v>82</v>
+      </c>
       <c r="P44" s="2"/>
       <c r="Q44" s="2"/>
       <c r="R44" s="2"/>
@@ -3702,55 +3721,32 @@
       <c r="AI44" s="3"/>
       <c r="AJ44" s="3"/>
     </row>
-    <row r="45" spans="2:36">
-      <c r="B45" s="2" t="s">
-        <v>113</v>
-      </c>
-      <c r="C45" s="2" t="s">
-        <v>100</v>
-      </c>
-      <c r="D45" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="E45" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="F45" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="G45" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="H45" s="4" t="s">
-        <v>112</v>
-      </c>
-      <c r="I45" s="4" t="s">
-        <v>114</v>
-      </c>
-      <c r="J45" s="4" t="s">
-        <v>115</v>
-      </c>
-      <c r="K45" s="2" t="s">
-        <v>116</v>
-      </c>
-      <c r="L45" s="2" t="s">
-        <v>117</v>
-      </c>
-      <c r="M45" s="2" t="s">
-        <v>118</v>
-      </c>
-      <c r="N45" s="2" t="s">
-        <v>119</v>
-      </c>
-      <c r="O45" s="2" t="s">
-        <v>82</v>
-      </c>
-      <c r="P45" s="2"/>
-      <c r="Q45" s="2"/>
-      <c r="R45" s="2"/>
-      <c r="S45" s="2"/>
-      <c r="T45" s="2"/>
-      <c r="U45" s="2"/>
+    <row r="45" spans="1:36">
+      <c r="A45" s="3"/>
+      <c r="B45" s="4"/>
+      <c r="C45" s="4"/>
+      <c r="D45" s="4"/>
+      <c r="E45" s="4"/>
+      <c r="F45" s="4"/>
+      <c r="G45" s="4"/>
+      <c r="H45" s="4"/>
+      <c r="I45" s="4"/>
+      <c r="J45" s="4"/>
+      <c r="K45" s="4"/>
+      <c r="L45" s="4"/>
+      <c r="M45" s="4"/>
+      <c r="N45" s="4"/>
+      <c r="O45" s="4"/>
+      <c r="P45" s="4"/>
+      <c r="Q45" s="4"/>
+      <c r="R45" s="4"/>
+      <c r="S45" s="4"/>
+      <c r="T45" s="4"/>
+      <c r="U45" s="4"/>
+      <c r="V45" s="3"/>
+      <c r="W45" s="3"/>
+      <c r="X45" s="3"/>
+      <c r="Y45" s="3"/>
       <c r="Z45" s="3"/>
       <c r="AA45" s="3"/>
       <c r="AB45" s="3"/>
@@ -3763,7 +3759,7 @@
       <c r="AI45" s="3"/>
       <c r="AJ45" s="3"/>
     </row>
-    <row r="46" spans="1:36">
+    <row r="46" s="1" customFormat="1" spans="1:36">
       <c r="A46" s="3"/>
       <c r="B46" s="4"/>
       <c r="C46" s="4"/>
@@ -3839,7 +3835,7 @@
       <c r="AI47" s="3"/>
       <c r="AJ47" s="3"/>
     </row>
-    <row r="48" s="1" customFormat="1" spans="1:36">
+    <row r="48" spans="1:36">
       <c r="A48" s="3"/>
       <c r="B48" s="4"/>
       <c r="C48" s="4"/>
@@ -4414,7 +4410,7 @@
       <c r="B63" s="4"/>
       <c r="C63" s="4"/>
       <c r="D63" s="4"/>
-      <c r="E63" s="4"/>
+      <c r="E63" s="5"/>
       <c r="F63" s="4"/>
       <c r="G63" s="4"/>
       <c r="H63" s="4"/>
@@ -4528,7 +4524,7 @@
       <c r="B66" s="4"/>
       <c r="C66" s="4"/>
       <c r="D66" s="4"/>
-      <c r="E66" s="5"/>
+      <c r="E66" s="4"/>
       <c r="F66" s="4"/>
       <c r="G66" s="4"/>
       <c r="H66" s="4"/>
@@ -4680,7 +4676,7 @@
       <c r="B70" s="4"/>
       <c r="C70" s="4"/>
       <c r="D70" s="4"/>
-      <c r="E70" s="4"/>
+      <c r="E70" s="5"/>
       <c r="F70" s="4"/>
       <c r="G70" s="4"/>
       <c r="H70" s="4"/>
@@ -4718,7 +4714,7 @@
       <c r="B71" s="4"/>
       <c r="C71" s="4"/>
       <c r="D71" s="4"/>
-      <c r="E71" s="5"/>
+      <c r="E71" s="4"/>
       <c r="F71" s="4"/>
       <c r="G71" s="4"/>
       <c r="H71" s="4"/>
@@ -5017,50 +5013,25 @@
       <c r="AI78" s="3"/>
       <c r="AJ78" s="3"/>
     </row>
-    <row r="79" spans="1:36">
-      <c r="A79" s="3"/>
-      <c r="B79" s="4"/>
-      <c r="C79" s="4"/>
-      <c r="D79" s="4"/>
-      <c r="E79" s="4"/>
-      <c r="F79" s="4"/>
-      <c r="G79" s="4"/>
-      <c r="H79" s="4"/>
-      <c r="I79" s="4"/>
-      <c r="J79" s="4"/>
-      <c r="K79" s="4"/>
-      <c r="L79" s="4"/>
-      <c r="M79" s="4"/>
-      <c r="N79" s="4"/>
-      <c r="O79" s="4"/>
-      <c r="P79" s="4"/>
-      <c r="Q79" s="4"/>
-      <c r="R79" s="4"/>
-      <c r="S79" s="4"/>
-      <c r="T79" s="4"/>
-      <c r="U79" s="4"/>
-      <c r="V79" s="3"/>
-      <c r="W79" s="3"/>
-      <c r="X79" s="3"/>
-      <c r="Y79" s="3"/>
-      <c r="Z79" s="3"/>
-      <c r="AA79" s="3"/>
-      <c r="AB79" s="3"/>
-      <c r="AC79" s="3"/>
-      <c r="AD79" s="3"/>
-      <c r="AE79" s="3"/>
-      <c r="AF79" s="3"/>
-      <c r="AG79" s="3"/>
-      <c r="AH79" s="3"/>
-      <c r="AI79" s="3"/>
-      <c r="AJ79" s="3"/>
+    <row r="86" spans="1:25">
+      <c r="A86" s="2"/>
+      <c r="B86" s="2"/>
+      <c r="C86" s="2"/>
+      <c r="D86" s="2"/>
+      <c r="T86" s="2"/>
+      <c r="V86" s="2"/>
+      <c r="W86" s="2"/>
+      <c r="X86" s="2"/>
+      <c r="Y86" s="2"/>
     </row>
     <row r="87" spans="1:25">
       <c r="A87" s="2"/>
       <c r="B87" s="2"/>
       <c r="C87" s="2"/>
       <c r="D87" s="2"/>
+      <c r="E87" s="2"/>
       <c r="T87" s="2"/>
+      <c r="U87" s="2"/>
       <c r="V87" s="2"/>
       <c r="W87" s="2"/>
       <c r="X87" s="2"/>
@@ -5071,7 +5042,6 @@
       <c r="B88" s="2"/>
       <c r="C88" s="2"/>
       <c r="D88" s="2"/>
-      <c r="E88" s="2"/>
       <c r="T88" s="2"/>
       <c r="U88" s="2"/>
       <c r="V88" s="2"/>
@@ -5211,60 +5181,48 @@
       <c r="X99" s="2"/>
       <c r="Y99" s="2"/>
     </row>
-    <row r="100" spans="1:25">
-      <c r="A100" s="2"/>
-      <c r="B100" s="2"/>
-      <c r="C100" s="2"/>
-      <c r="D100" s="2"/>
-      <c r="T100" s="2"/>
-      <c r="U100" s="2"/>
-      <c r="V100" s="2"/>
-      <c r="W100" s="2"/>
-      <c r="X100" s="2"/>
-      <c r="Y100" s="2"/>
-    </row>
   </sheetData>
   <dataValidations count="14">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H29 H30 H31 H40 H41 H42 H43 H44 H10:H28 H32:H39 H45:H1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="O2:O1048576">
+      <formula1>"R_TYPE,I_TYPE,S_TYPE,B_TYPE,U_TYPE,J_TYPE,ICSR_TYPE,FENCE_TYPE,N_TYPE"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="M29 M30 M31 M39 M40 M41 M42 M43 M2:M28 M32:M38 M44:M1048576">
+      <formula1>"CSR_W,CSR_S,CSR_C,CSR_P,CSR_XX"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H29 H30 H31 H40 H41 H42 H43 H10:H28 H32:H39 H44:H1048576">
       <formula1>"WB_ALU,WB_MEM,WB_PC4,WB_XX,WB_CSR"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L5 L6 L7 L10 L11 L14 L15 L16 L17 L18 L19 L20 L21 L22 L23 L24 L25 L26 L27 L28 L29 L30 L31 L32 L33 L34 L35 L36 L37 L38 L39 L40 L41 L42 L43 L44 L2:L4 L8:L9 L12:L13 L45:L1048576">
-      <formula1>"BR_EQ,BR_NE,BR_LTU,BR_GE,BR_GEU,BR_LT,BR_XX"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C29 C30 C31 C43 C2:C28 C32:C42 C44:C1048576">
+      <formula1>"PC_4,PC_0,PC_ALU,PC_CSR"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E4 E5 E6 E7 E8 E9 E10 E11 E12 E13 E14 E15 E16 E17 E18 E19 E20 E21 E22 E23 E24 E25 E26 E27 E28 E29 E30 E31 E32 E33 E34 E35 E36 E37 E38 E39 E40 E41 E42 E43 E2:E3 E44:E1048576">
+      <formula1>"B_IMM,B_RS2"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G4 G5 G6 G7 G8 G9 G10 G11 G12 G13 G14 G15 G16 G17 G18 G19 G20 G21 G22 G23 G24 G25 G26 G27 G28 G29 G30 G31 G32 G33 G34 G35 G36 G37 G38 G39 G40 G41 G42 G43 G2:G3 G44:G1048576">
+      <formula1>"IMM_I,IMM_J,IMM_U,IMM_S,IMM_B"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J5 J6 J7 J8 J9 J10 J11 J12 J13 J14 J15 J16 J17 J18 J19 J20 J21 J22 J23 J24 J25 J26 J27 J28 J29 J30 J31 J32 J33 J34 J35 J36 J37 J38 J39 J40 J41 J42 J43 J2:J4 J44:J1048576">
+      <formula1>"ST_SW,ST_SH,ST_SB,ST_XX"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H5 H6 H7 H8 H9 H2:H4">
       <formula1>"WB_ALU,WB_MEM,WB_PC4,WB_XX"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="M29 M30 M31 M39 M40 M41 M42 M43 M44 M2:M28 M32:M38 M45:M1048576">
-      <formula1>"CSR_W,CSR_S,CSR_C,CSR_P,CSR_XX"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L5 L6 L7 L10 L11 L14 L15 L16 L17 L18 L19 L20 L21 L22 L23 L24 L25 L26 L27 L28 L29 L30 L31 L32 L33 L34 L35 L36 L37 L38 L39 L40 L41 L42 L43 L2:L4 L8:L9 L12:L13 L44:L1048576">
+      <formula1>"BR_EQ,BR_NE,BR_LTU,BR_GE,BR_GEU,BR_LT,BR_XX"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E4 E5 E6 E7 E8 E9 E10 E11 E12 E13 E14 E15 E16 E17 E18 E19 E20 E21 E22 E23 E24 E25 E26 E27 E28 E29 E30 E31 E32 E33 E34 E35 E36 E37 E38 E39 E40 E41 E42 E43 E44 E2:E3 E45:E1048576">
-      <formula1>"B_IMM,B_RS2"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C29 C30 C31 C43 C44 C2:C28 C32:C42 C45:C1048576">
-      <formula1>"PC_4,PC_0,PC_ALU,PC_CSR"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="N4 N5 N6 N7 N8 N9 N10 N11 N12 N13 N14 N15 N16 N17 N18 N19 N20 N21 N22 N23 N24 N25 N26 N27 N28 N29 N30 N31 N32 N33 N34 N35 N36 N37 N38 N39 N40 N41 N42 N43 N44 N2:N3 N45:N1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="N4 N5 N6 N7 N8 N9 N10 N11 N12 N13 N14 N15 N16 N17 N18 N19 N20 N21 N22 N23 N24 N25 N26 N27 N28 N29 N30 N31 N32 N33 N34 N35 N36 N37 N38 N39 N40 N41 N42 N43 N2:N3 N44:N1048576">
       <formula1>"INST_VALID,INST_INVALID"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I4 I5 I6 I7 I8 I9 I10 I11 I12 I13 I14 I15 I16 I17 I18 I19 I20 I21 I22 I23 I24 I25 I26 I27 I28 I29 I30 I31 I32 I33 I34 I35 I36 I37 I38 I39 I40 I41 I42 I43 I44 I2:I3 I45:I1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I4 I5 I6 I7 I8 I9 I10 I11 I12 I13 I14 I15 I16 I17 I18 I19 I20 I21 I22 I23 I24 I25 I26 I27 I28 I29 I30 I31 I32 I33 I34 I35 I36 I37 I38 I39 I40 I41 I42 I43 I2:I3 I44:I1048576">
       <formula1>"LD_LB,LD_LH,LD_LW,LD_LBU,LD_LHU,LD_XX"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="O44 O2:O43 O45:O1048576">
-      <formula1>"R_TYPE,I_TYPE,S_TYPE,B_TYPE,U_TYPE,J_TYPE,ICSR_TYPE,FENCE_TYPE,N_TYPE"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F6 F15 F18 F19 F20 F21 F24 F25 F26 F27 F28 F29 F30 F31 F32 F33 F36 F37 F38 F39 F40 F41 F42 F43 F2:F5 F7:F14 F16:F17 F22:F23 F34:F35 F44:F1048576">
+      <formula1>"ALU_ADD,ALU_SUB,ALU_AND,ALU_OR,ALU_XOR,ALU_SLL,ALU_SRL,ALU_SLT,ALU_SLTU,ALU_COPY_A,ALU_COPY_B,ALU_SRA"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J5 J6 J7 J8 J9 J10 J11 J12 J13 J14 J15 J16 J17 J18 J19 J20 J21 J22 J23 J24 J25 J26 J27 J28 J29 J30 J31 J32 J33 J34 J35 J36 J37 J38 J39 J40 J41 J42 J43 J44 J2:J4 J45:J1048576">
-      <formula1>"ST_SW,ST_SH,ST_SB,ST_XX"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G4 G5 G6 G7 G8 G9 G10 G11 G12 G13 G14 G15 G16 G17 G18 G19 G20 G21 G22 G23 G24 G25 G26 G27 G28 G29 G30 G31 G32 G33 G34 G35 G36 G37 G38 G39 G40 G41 G42 G43 G44 G2:G3 G45:G1048576">
-      <formula1>"IMM_I,IMM_J,IMM_U,IMM_S,IMM_B"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K4 K5 K6 K7 K8 K9 K10 K11 K12 K13 K14 K15 K16 K17 K18 K19 K20 K21 K22 K23 K24 K25 K26 K27 K28 K29 K30 K31 K32 K33 K34 K35 K36 K37 K38 K39 K40 K41 K42 K43 K44 K2:K3 K45:K1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K4 K5 K6 K7 K8 K9 K10 K11 K12 K13 K14 K15 K16 K17 K18 K19 K20 K21 K22 K23 K24 K25 K26 K27 K28 K29 K30 K31 K32 K33 K34 K35 K36 K37 K38 K39 K40 K41 K42 K43 K2:K3 K44:K1048576">
       <formula1>"MASK_XX,MASK_B,MASK_H,MASK_W,MASK_D"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F6 F15 F18 F19 F20 F21 F24 F25 F26 F27 F28 F29 F30 F31 F32 F33 F36 F37 F38 F39 F40 F41 F42 F43 F44 F2:F5 F7:F14 F16:F17 F22:F23 F34:F35 F45:F1048576">
-      <formula1>"ALU_ADD,ALU_SUB,ALU_AND,ALU_OR,ALU_XOR,ALU_SLL,ALU_SRL,ALU_SLT,ALU_SLTU,ALU_COPY_A,ALU_COPY_B,ALU_SRA"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D4 D5 D6 D7 D8 D9 D10 D11 D12 D13 D14 D15 D16 D17 D18 D19 D20 D21 D22 D23 D24 D25 D26 D27 D28 D29 D30 D31 D32 D33 D34 D35 D36 D37 D38 D39 D40 D41 D42 D43 D44 D2:D3 D45:D1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D4 D5 D6 D7 D8 D9 D10 D11 D12 D13 D14 D15 D16 D17 D18 D19 D20 D21 D22 D23 D24 D25 D26 D27 D28 D29 D30 D31 D32 D33 D34 D35 D36 D37 D38 D39 D40 D41 D42 D43 D2:D3 D44:D1048576">
       <formula1>"A_PC,A_RS1"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
> sim RTL ysyx_23060246 韩炳晋 Linux archlinux 6.12.17-1-lts #1 SMP PREEMPT_DYNAMIC Thu, 27 Feb 2025 14:12:30 +0000 x86_64 GNU/Linux  18:04:20 up 21:54,  1 user,  load average: 2.17, 1.83, 1.63
</commit_message>
<xml_diff>
--- a/npc/tools/control_gen/control_table.xlsx
+++ b/npc/tools/control_gen/control_table.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="23370" windowHeight="12150"/>
+    <workbookView windowWidth="18200" windowHeight="7440"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="355" uniqueCount="119">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="356" uniqueCount="120">
   <si>
     <t>comment</t>
   </si>
@@ -347,6 +347,9 @@
   </si>
   <si>
     <t>fencei</t>
+  </si>
+  <si>
+    <t>ebreak</t>
   </si>
   <si>
     <t>default</t>
@@ -378,10 +381,10 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="4">
+    <numFmt numFmtId="42" formatCode="_ &quot;￥&quot;* #,##0_ ;_ &quot;￥&quot;* \-#,##0_ ;_ &quot;￥&quot;* &quot;-&quot;_ ;_ @_ "/>
+    <numFmt numFmtId="41" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
     <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="42" formatCode="_ &quot;￥&quot;* #,##0_ ;_ &quot;￥&quot;* \-#,##0_ ;_ &quot;￥&quot;* &quot;-&quot;_ ;_ @_ "/>
     <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="41" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
   <fonts count="22">
     <font>
@@ -405,6 +408,13 @@
     </font>
     <font>
       <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
       <color theme="1"/>
       <name val="宋体"/>
       <charset val="0"/>
@@ -413,28 +423,6 @@
     <font>
       <sz val="11"/>
       <color theme="0"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF0000FF"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
       <name val="宋体"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -449,16 +437,32 @@
     </font>
     <font>
       <b/>
-      <sz val="18"/>
+      <sz val="13"/>
       <color theme="3"/>
       <name val="宋体"/>
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <u/>
       <sz val="11"/>
-      <color rgb="FF800080"/>
+      <color rgb="FF0000FF"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color rgb="FF7F7F7F"/>
       <name val="宋体"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -474,7 +478,14 @@
     <font>
       <b/>
       <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
+      <color theme="1"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF3F3F76"/>
       <name val="宋体"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -487,18 +498,26 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
       <sz val="11"/>
-      <color theme="1"/>
+      <color rgb="FFFF0000"/>
       <name val="宋体"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color rgb="FF9C6500"/>
+      <b/>
+      <sz val="18"/>
+      <color theme="3"/>
       <name val="宋体"/>
-      <charset val="0"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="15"/>
+      <color theme="3"/>
+      <name val="宋体"/>
+      <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -517,32 +536,16 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <sz val="13"/>
-      <color theme="3"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="15"/>
-      <color theme="3"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <i/>
       <sz val="11"/>
-      <color rgb="FF7F7F7F"/>
+      <color rgb="FF9C6500"/>
       <name val="宋体"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <u/>
       <sz val="11"/>
-      <color rgb="FF3F3F76"/>
+      <color rgb="FF800080"/>
       <name val="宋体"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -569,7 +572,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="8"/>
+        <fgColor theme="8" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.599993896298105"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -581,37 +590,25 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FFA5A5A5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor theme="5" tint="0.599993896298105"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.599993896298105"/>
+        <fgColor theme="7" tint="0.599993896298105"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -623,73 +620,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.599993896298105"/>
+        <fgColor rgb="FFF2F2F2"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="7" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFA5A5A5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.399975585192419"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -707,7 +644,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5"/>
+        <fgColor theme="4" tint="0.799981688894314"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -719,19 +656,85 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FFFFCC99"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor theme="6"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
+        <fgColor theme="6" tint="0.599993896298105"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.799981688894314"/>
+        <fgColor theme="7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -748,21 +751,6 @@
       <right/>
       <top/>
       <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFB2B2B2"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFB2B2B2"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFB2B2B2"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFB2B2B2"/>
-      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -784,17 +772,26 @@
       <diagonal/>
     </border>
     <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
       <left style="thin">
-        <color rgb="FF3F3F3F"/>
+        <color rgb="FFB2B2B2"/>
       </left>
       <right style="thin">
-        <color rgb="FF3F3F3F"/>
+        <color rgb="FFB2B2B2"/>
       </right>
       <top style="thin">
-        <color rgb="FF3F3F3F"/>
+        <color rgb="FFB2B2B2"/>
       </top>
       <bottom style="thin">
-        <color rgb="FF3F3F3F"/>
+        <color rgb="FFB2B2B2"/>
       </bottom>
       <diagonal/>
     </border>
@@ -809,6 +806,21 @@
         <color rgb="FF3F3F3F"/>
       </top>
       <bottom style="double">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="thin">
         <color rgb="FF3F3F3F"/>
       </bottom>
       <diagonal/>
@@ -839,162 +851,153 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="5" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="18" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="12" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="12" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="30" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="15" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="17" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="15" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="4" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
@@ -1339,28 +1342,28 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:AJ99"/>
+  <dimension ref="A1:AJ100"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
     <col min="1" max="1" width="13.1" customWidth="1"/>
-    <col min="2" max="2" width="17.7583333333333" customWidth="1"/>
-    <col min="3" max="3" width="10.1416666666667" customWidth="1"/>
-    <col min="4" max="4" width="7.75" customWidth="1"/>
-    <col min="5" max="5" width="11.7166666666667" customWidth="1"/>
-    <col min="6" max="6" width="11.1166666666667" customWidth="1"/>
-    <col min="7" max="7" width="10.9416666666667" customWidth="1"/>
-    <col min="8" max="10" width="11.9833333333333" customWidth="1"/>
-    <col min="11" max="11" width="15.075" customWidth="1"/>
-    <col min="12" max="14" width="12.1083333333333" customWidth="1"/>
-    <col min="15" max="16" width="10.8583333333333" customWidth="1"/>
-    <col min="18" max="18" width="14.2166666666667" customWidth="1"/>
-    <col min="19" max="19" width="11.8083333333333" customWidth="1"/>
+    <col min="2" max="2" width="17.7545454545455" customWidth="1"/>
+    <col min="3" max="3" width="10.1454545454545" customWidth="1"/>
+    <col min="4" max="4" width="7.75454545454545" customWidth="1"/>
+    <col min="5" max="5" width="11.7181818181818" customWidth="1"/>
+    <col min="6" max="6" width="11.1181818181818" customWidth="1"/>
+    <col min="7" max="7" width="10.9454545454545" customWidth="1"/>
+    <col min="8" max="10" width="11.9818181818182" customWidth="1"/>
+    <col min="11" max="11" width="15.0727272727273" customWidth="1"/>
+    <col min="12" max="14" width="12.1090909090909" customWidth="1"/>
+    <col min="15" max="16" width="10.8545454545455" customWidth="1"/>
+    <col min="18" max="18" width="14.2181818181818" customWidth="1"/>
+    <col min="19" max="19" width="11.8090909090909" customWidth="1"/>
     <col min="20" max="20" width="10.6" customWidth="1"/>
-    <col min="21" max="21" width="9.70833333333333" customWidth="1"/>
-    <col min="22" max="22" width="11.1666666666667" customWidth="1"/>
-    <col min="23" max="23" width="11.4083333333333" customWidth="1"/>
-    <col min="24" max="24" width="12.0583333333333" customWidth="1"/>
-    <col min="25" max="25" width="15.575" customWidth="1"/>
+    <col min="21" max="21" width="9.70909090909091" customWidth="1"/>
+    <col min="22" max="22" width="11.1636363636364" customWidth="1"/>
+    <col min="23" max="23" width="11.4090909090909" customWidth="1"/>
+    <col min="24" max="24" width="12.0545454545455" customWidth="1"/>
+    <col min="25" max="25" width="15.5727272727273" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1" spans="1:24">
@@ -3664,45 +3667,19 @@
       <c r="B44" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="C44" s="2" t="s">
-        <v>100</v>
-      </c>
-      <c r="D44" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="E44" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="F44" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="G44" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="H44" s="4" t="s">
-        <v>112</v>
-      </c>
-      <c r="I44" s="4" t="s">
-        <v>113</v>
-      </c>
-      <c r="J44" s="4" t="s">
-        <v>114</v>
-      </c>
-      <c r="K44" s="2" t="s">
-        <v>115</v>
-      </c>
-      <c r="L44" s="2" t="s">
-        <v>116</v>
-      </c>
-      <c r="M44" s="2" t="s">
-        <v>117</v>
-      </c>
-      <c r="N44" s="2" t="s">
-        <v>118</v>
-      </c>
-      <c r="O44" s="2" t="s">
-        <v>82</v>
-      </c>
+      <c r="C44" s="2"/>
+      <c r="D44" s="2"/>
+      <c r="E44" s="2"/>
+      <c r="F44" s="2"/>
+      <c r="G44" s="2"/>
+      <c r="H44" s="4"/>
+      <c r="I44" s="4"/>
+      <c r="J44" s="4"/>
+      <c r="K44" s="2"/>
+      <c r="L44" s="2"/>
+      <c r="M44" s="2"/>
+      <c r="N44" s="2"/>
+      <c r="O44" s="2"/>
       <c r="P44" s="2"/>
       <c r="Q44" s="2"/>
       <c r="R44" s="2"/>
@@ -3721,32 +3698,55 @@
       <c r="AI44" s="3"/>
       <c r="AJ44" s="3"/>
     </row>
-    <row r="45" spans="1:36">
-      <c r="A45" s="3"/>
-      <c r="B45" s="4"/>
-      <c r="C45" s="4"/>
-      <c r="D45" s="4"/>
-      <c r="E45" s="4"/>
-      <c r="F45" s="4"/>
-      <c r="G45" s="4"/>
-      <c r="H45" s="4"/>
-      <c r="I45" s="4"/>
-      <c r="J45" s="4"/>
-      <c r="K45" s="4"/>
-      <c r="L45" s="4"/>
-      <c r="M45" s="4"/>
-      <c r="N45" s="4"/>
-      <c r="O45" s="4"/>
-      <c r="P45" s="4"/>
-      <c r="Q45" s="4"/>
-      <c r="R45" s="4"/>
-      <c r="S45" s="4"/>
-      <c r="T45" s="4"/>
-      <c r="U45" s="4"/>
-      <c r="V45" s="3"/>
-      <c r="W45" s="3"/>
-      <c r="X45" s="3"/>
-      <c r="Y45" s="3"/>
+    <row r="45" spans="2:36">
+      <c r="B45" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="C45" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="D45" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="E45" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="F45" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="G45" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="H45" s="4" t="s">
+        <v>113</v>
+      </c>
+      <c r="I45" s="4" t="s">
+        <v>114</v>
+      </c>
+      <c r="J45" s="4" t="s">
+        <v>115</v>
+      </c>
+      <c r="K45" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="L45" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="M45" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="N45" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="O45" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="P45" s="2"/>
+      <c r="Q45" s="2"/>
+      <c r="R45" s="2"/>
+      <c r="S45" s="2"/>
+      <c r="T45" s="2"/>
+      <c r="U45" s="2"/>
       <c r="Z45" s="3"/>
       <c r="AA45" s="3"/>
       <c r="AB45" s="3"/>
@@ -3759,7 +3759,7 @@
       <c r="AI45" s="3"/>
       <c r="AJ45" s="3"/>
     </row>
-    <row r="46" s="1" customFormat="1" spans="1:36">
+    <row r="46" spans="1:36">
       <c r="A46" s="3"/>
       <c r="B46" s="4"/>
       <c r="C46" s="4"/>
@@ -3835,7 +3835,7 @@
       <c r="AI47" s="3"/>
       <c r="AJ47" s="3"/>
     </row>
-    <row r="48" spans="1:36">
+    <row r="48" s="1" customFormat="1" spans="1:36">
       <c r="A48" s="3"/>
       <c r="B48" s="4"/>
       <c r="C48" s="4"/>
@@ -4410,7 +4410,7 @@
       <c r="B63" s="4"/>
       <c r="C63" s="4"/>
       <c r="D63" s="4"/>
-      <c r="E63" s="5"/>
+      <c r="E63" s="4"/>
       <c r="F63" s="4"/>
       <c r="G63" s="4"/>
       <c r="H63" s="4"/>
@@ -4524,7 +4524,7 @@
       <c r="B66" s="4"/>
       <c r="C66" s="4"/>
       <c r="D66" s="4"/>
-      <c r="E66" s="4"/>
+      <c r="E66" s="5"/>
       <c r="F66" s="4"/>
       <c r="G66" s="4"/>
       <c r="H66" s="4"/>
@@ -4676,7 +4676,7 @@
       <c r="B70" s="4"/>
       <c r="C70" s="4"/>
       <c r="D70" s="4"/>
-      <c r="E70" s="5"/>
+      <c r="E70" s="4"/>
       <c r="F70" s="4"/>
       <c r="G70" s="4"/>
       <c r="H70" s="4"/>
@@ -4714,7 +4714,7 @@
       <c r="B71" s="4"/>
       <c r="C71" s="4"/>
       <c r="D71" s="4"/>
-      <c r="E71" s="4"/>
+      <c r="E71" s="5"/>
       <c r="F71" s="4"/>
       <c r="G71" s="4"/>
       <c r="H71" s="4"/>
@@ -5013,25 +5013,50 @@
       <c r="AI78" s="3"/>
       <c r="AJ78" s="3"/>
     </row>
-    <row r="86" spans="1:25">
-      <c r="A86" s="2"/>
-      <c r="B86" s="2"/>
-      <c r="C86" s="2"/>
-      <c r="D86" s="2"/>
-      <c r="T86" s="2"/>
-      <c r="V86" s="2"/>
-      <c r="W86" s="2"/>
-      <c r="X86" s="2"/>
-      <c r="Y86" s="2"/>
+    <row r="79" spans="1:36">
+      <c r="A79" s="3"/>
+      <c r="B79" s="4"/>
+      <c r="C79" s="4"/>
+      <c r="D79" s="4"/>
+      <c r="E79" s="4"/>
+      <c r="F79" s="4"/>
+      <c r="G79" s="4"/>
+      <c r="H79" s="4"/>
+      <c r="I79" s="4"/>
+      <c r="J79" s="4"/>
+      <c r="K79" s="4"/>
+      <c r="L79" s="4"/>
+      <c r="M79" s="4"/>
+      <c r="N79" s="4"/>
+      <c r="O79" s="4"/>
+      <c r="P79" s="4"/>
+      <c r="Q79" s="4"/>
+      <c r="R79" s="4"/>
+      <c r="S79" s="4"/>
+      <c r="T79" s="4"/>
+      <c r="U79" s="4"/>
+      <c r="V79" s="3"/>
+      <c r="W79" s="3"/>
+      <c r="X79" s="3"/>
+      <c r="Y79" s="3"/>
+      <c r="Z79" s="3"/>
+      <c r="AA79" s="3"/>
+      <c r="AB79" s="3"/>
+      <c r="AC79" s="3"/>
+      <c r="AD79" s="3"/>
+      <c r="AE79" s="3"/>
+      <c r="AF79" s="3"/>
+      <c r="AG79" s="3"/>
+      <c r="AH79" s="3"/>
+      <c r="AI79" s="3"/>
+      <c r="AJ79" s="3"/>
     </row>
     <row r="87" spans="1:25">
       <c r="A87" s="2"/>
       <c r="B87" s="2"/>
       <c r="C87" s="2"/>
       <c r="D87" s="2"/>
-      <c r="E87" s="2"/>
       <c r="T87" s="2"/>
-      <c r="U87" s="2"/>
       <c r="V87" s="2"/>
       <c r="W87" s="2"/>
       <c r="X87" s="2"/>
@@ -5042,6 +5067,7 @@
       <c r="B88" s="2"/>
       <c r="C88" s="2"/>
       <c r="D88" s="2"/>
+      <c r="E88" s="2"/>
       <c r="T88" s="2"/>
       <c r="U88" s="2"/>
       <c r="V88" s="2"/>
@@ -5181,48 +5207,60 @@
       <c r="X99" s="2"/>
       <c r="Y99" s="2"/>
     </row>
+    <row r="100" spans="1:25">
+      <c r="A100" s="2"/>
+      <c r="B100" s="2"/>
+      <c r="C100" s="2"/>
+      <c r="D100" s="2"/>
+      <c r="T100" s="2"/>
+      <c r="U100" s="2"/>
+      <c r="V100" s="2"/>
+      <c r="W100" s="2"/>
+      <c r="X100" s="2"/>
+      <c r="Y100" s="2"/>
+    </row>
   </sheetData>
   <dataValidations count="14">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="O2:O1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F6 F15 F18 F19 F20 F21 F24 F25 F26 F27 F28 F29 F30 F31 F32 F33 F36 F37 F38 F39 F40 F41 F42 F43 F44 F2:F5 F7:F14 F16:F17 F22:F23 F34:F35 F45:F1048576">
+      <formula1>"ALU_ADD,ALU_SUB,ALU_AND,ALU_OR,ALU_XOR,ALU_SLL,ALU_SRL,ALU_SLT,ALU_SLTU,ALU_COPY_A,ALU_COPY_B,ALU_SRA"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J5 J6 J7 J8 J9 J10 J11 J12 J13 J14 J15 J16 J17 J18 J19 J20 J21 J22 J23 J24 J25 J26 J27 J28 J29 J30 J31 J32 J33 J34 J35 J36 J37 J38 J39 J40 J41 J42 J43 J44 J2:J4 J45:J1048576">
+      <formula1>"ST_SW,ST_SH,ST_SB,ST_XX"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C29 C30 C31 C43 C44 C2:C28 C32:C42 C45:C1048576">
+      <formula1>"PC_4,PC_0,PC_ALU,PC_CSR"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="N4 N5 N6 N7 N8 N9 N10 N11 N12 N13 N14 N15 N16 N17 N18 N19 N20 N21 N22 N23 N24 N25 N26 N27 N28 N29 N30 N31 N32 N33 N34 N35 N36 N37 N38 N39 N40 N41 N42 N43 N44 N2:N3 N45:N1048576">
+      <formula1>"INST_VALID,INST_INVALID"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="M29 M30 M31 M39 M40 M41 M42 M43 M44 M2:M28 M32:M38 M45:M1048576">
+      <formula1>"CSR_W,CSR_S,CSR_C,CSR_P,CSR_XX"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G4 G5 G6 G7 G8 G9 G10 G11 G12 G13 G14 G15 G16 G17 G18 G19 G20 G21 G22 G23 G24 G25 G26 G27 G28 G29 G30 G31 G32 G33 G34 G35 G36 G37 G38 G39 G40 G41 G42 G43 G44 G2:G3 G45:G1048576">
+      <formula1>"IMM_I,IMM_J,IMM_U,IMM_S,IMM_B"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E4 E5 E6 E7 E8 E9 E10 E11 E12 E13 E14 E15 E16 E17 E18 E19 E20 E21 E22 E23 E24 E25 E26 E27 E28 E29 E30 E31 E32 E33 E34 E35 E36 E37 E38 E39 E40 E41 E42 E43 E44 E2:E3 E45:E1048576">
+      <formula1>"B_IMM,B_RS2"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="O44 O2:O43 O45:O1048576">
       <formula1>"R_TYPE,I_TYPE,S_TYPE,B_TYPE,U_TYPE,J_TYPE,ICSR_TYPE,FENCE_TYPE,N_TYPE"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="M29 M30 M31 M39 M40 M41 M42 M43 M2:M28 M32:M38 M44:M1048576">
-      <formula1>"CSR_W,CSR_S,CSR_C,CSR_P,CSR_XX"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K4 K5 K6 K7 K8 K9 K10 K11 K12 K13 K14 K15 K16 K17 K18 K19 K20 K21 K22 K23 K24 K25 K26 K27 K28 K29 K30 K31 K32 K33 K34 K35 K36 K37 K38 K39 K40 K41 K42 K43 K44 K2:K3 K45:K1048576">
+      <formula1>"MASK_XX,MASK_B,MASK_H,MASK_W,MASK_D"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H29 H30 H31 H40 H41 H42 H43 H10:H28 H32:H39 H44:H1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L5 L6 L7 L10 L11 L14 L15 L16 L17 L18 L19 L20 L21 L22 L23 L24 L25 L26 L27 L28 L29 L30 L31 L32 L33 L34 L35 L36 L37 L38 L39 L40 L41 L42 L43 L44 L2:L4 L8:L9 L12:L13 L45:L1048576">
+      <formula1>"BR_EQ,BR_NE,BR_LTU,BR_GE,BR_GEU,BR_LT,BR_XX"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I4 I5 I6 I7 I8 I9 I10 I11 I12 I13 I14 I15 I16 I17 I18 I19 I20 I21 I22 I23 I24 I25 I26 I27 I28 I29 I30 I31 I32 I33 I34 I35 I36 I37 I38 I39 I40 I41 I42 I43 I44 I2:I3 I45:I1048576">
+      <formula1>"LD_LB,LD_LH,LD_LW,LD_LBU,LD_LHU,LD_XX"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H29 H30 H31 H40 H41 H42 H43 H44 H10:H28 H32:H39 H45:H1048576">
       <formula1>"WB_ALU,WB_MEM,WB_PC4,WB_XX,WB_CSR"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C29 C30 C31 C43 C2:C28 C32:C42 C44:C1048576">
-      <formula1>"PC_4,PC_0,PC_ALU,PC_CSR"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E4 E5 E6 E7 E8 E9 E10 E11 E12 E13 E14 E15 E16 E17 E18 E19 E20 E21 E22 E23 E24 E25 E26 E27 E28 E29 E30 E31 E32 E33 E34 E35 E36 E37 E38 E39 E40 E41 E42 E43 E2:E3 E44:E1048576">
-      <formula1>"B_IMM,B_RS2"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G4 G5 G6 G7 G8 G9 G10 G11 G12 G13 G14 G15 G16 G17 G18 G19 G20 G21 G22 G23 G24 G25 G26 G27 G28 G29 G30 G31 G32 G33 G34 G35 G36 G37 G38 G39 G40 G41 G42 G43 G2:G3 G44:G1048576">
-      <formula1>"IMM_I,IMM_J,IMM_U,IMM_S,IMM_B"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J5 J6 J7 J8 J9 J10 J11 J12 J13 J14 J15 J16 J17 J18 J19 J20 J21 J22 J23 J24 J25 J26 J27 J28 J29 J30 J31 J32 J33 J34 J35 J36 J37 J38 J39 J40 J41 J42 J43 J2:J4 J44:J1048576">
-      <formula1>"ST_SW,ST_SH,ST_SB,ST_XX"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H5 H6 H7 H8 H9 H2:H4">
       <formula1>"WB_ALU,WB_MEM,WB_PC4,WB_XX"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L5 L6 L7 L10 L11 L14 L15 L16 L17 L18 L19 L20 L21 L22 L23 L24 L25 L26 L27 L28 L29 L30 L31 L32 L33 L34 L35 L36 L37 L38 L39 L40 L41 L42 L43 L2:L4 L8:L9 L12:L13 L44:L1048576">
-      <formula1>"BR_EQ,BR_NE,BR_LTU,BR_GE,BR_GEU,BR_LT,BR_XX"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="N4 N5 N6 N7 N8 N9 N10 N11 N12 N13 N14 N15 N16 N17 N18 N19 N20 N21 N22 N23 N24 N25 N26 N27 N28 N29 N30 N31 N32 N33 N34 N35 N36 N37 N38 N39 N40 N41 N42 N43 N2:N3 N44:N1048576">
-      <formula1>"INST_VALID,INST_INVALID"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I4 I5 I6 I7 I8 I9 I10 I11 I12 I13 I14 I15 I16 I17 I18 I19 I20 I21 I22 I23 I24 I25 I26 I27 I28 I29 I30 I31 I32 I33 I34 I35 I36 I37 I38 I39 I40 I41 I42 I43 I2:I3 I44:I1048576">
-      <formula1>"LD_LB,LD_LH,LD_LW,LD_LBU,LD_LHU,LD_XX"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F6 F15 F18 F19 F20 F21 F24 F25 F26 F27 F28 F29 F30 F31 F32 F33 F36 F37 F38 F39 F40 F41 F42 F43 F2:F5 F7:F14 F16:F17 F22:F23 F34:F35 F44:F1048576">
-      <formula1>"ALU_ADD,ALU_SUB,ALU_AND,ALU_OR,ALU_XOR,ALU_SLL,ALU_SRL,ALU_SLT,ALU_SLTU,ALU_COPY_A,ALU_COPY_B,ALU_SRA"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K4 K5 K6 K7 K8 K9 K10 K11 K12 K13 K14 K15 K16 K17 K18 K19 K20 K21 K22 K23 K24 K25 K26 K27 K28 K29 K30 K31 K32 K33 K34 K35 K36 K37 K38 K39 K40 K41 K42 K43 K2:K3 K44:K1048576">
-      <formula1>"MASK_XX,MASK_B,MASK_H,MASK_W,MASK_D"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D4 D5 D6 D7 D8 D9 D10 D11 D12 D13 D14 D15 D16 D17 D18 D19 D20 D21 D22 D23 D24 D25 D26 D27 D28 D29 D30 D31 D32 D33 D34 D35 D36 D37 D38 D39 D40 D41 D42 D43 D2:D3 D44:D1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D4 D5 D6 D7 D8 D9 D10 D11 D12 D13 D14 D15 D16 D17 D18 D19 D20 D21 D22 D23 D24 D25 D26 D27 D28 D29 D30 D31 D32 D33 D34 D35 D36 D37 D38 D39 D40 D41 D42 D43 D44 D2:D3 D45:D1048576">
       <formula1>"A_PC,A_RS1"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
> sim RTL ysyx_23060246 韩炳晋 Linux archlinux 6.12.17-1-lts #1 SMP PREEMPT_DYNAMIC Thu, 27 Feb 2025 14:12:30 +0000 x86_64 GNU/Linux  18:05:21 up 21:55,  1 user,  load average: 2.20, 1.84, 1.65
</commit_message>
<xml_diff>
--- a/npc/tools/control_gen/control_table.xlsx
+++ b/npc/tools/control_gen/control_table.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="356" uniqueCount="120">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="357" uniqueCount="120">
   <si>
     <t>comment</t>
   </si>
@@ -381,9 +381,9 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="4">
+    <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="41" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
     <numFmt numFmtId="42" formatCode="_ &quot;￥&quot;* #,##0_ ;_ &quot;￥&quot;* \-#,##0_ ;_ &quot;￥&quot;* &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="41" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
   </numFmts>
   <fonts count="22">
@@ -408,61 +408,7 @@
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
       <color theme="1"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="0"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="3"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="13"/>
-      <color theme="3"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF0000FF"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="11"/>
-      <color rgb="FF7F7F7F"/>
       <name val="宋体"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -476,23 +422,8 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
       <sz val="11"/>
-      <color theme="1"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF3F3F76"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C0006"/>
+      <color theme="0"/>
       <name val="宋体"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -505,8 +436,16 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF800080"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <b/>
-      <sz val="18"/>
+      <sz val="11"/>
       <color theme="3"/>
       <name val="宋体"/>
       <charset val="134"/>
@@ -530,7 +469,44 @@
     </font>
     <font>
       <sz val="11"/>
+      <color rgb="FF9C0006"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
       <color rgb="FF006100"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="13"/>
+      <color theme="3"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF3F3F76"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
       <name val="宋体"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -543,9 +519,33 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <i/>
+      <sz val="11"/>
+      <color rgb="FF7F7F7F"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="18"/>
+      <color theme="3"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <u/>
       <sz val="11"/>
-      <color rgb="FF800080"/>
+      <color rgb="FF0000FF"/>
       <name val="宋体"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -566,6 +566,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor theme="9"/>
         <bgColor indexed="64"/>
       </patternFill>
@@ -578,7 +584,19 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor theme="9" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -590,7 +608,49 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFA5A5A5"/>
+        <fgColor theme="5" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.799981688894314"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -602,7 +662,73 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FFFFCC99"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor theme="5" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFA5A5A5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.399975585192419"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -614,133 +740,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor theme="7" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.399975585192419"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -751,63 +751,6 @@
       <right/>
       <top/>
       <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="double">
-        <color rgb="FFFF8001"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4" tint="0.499984740745262"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFB2B2B2"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFB2B2B2"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFB2B2B2"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFB2B2B2"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="double">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="double">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="double">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="double">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -828,10 +771,32 @@
     <border>
       <left/>
       <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4" tint="0.499984740745262"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFB2B2B2"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFB2B2B2"/>
+      </right>
       <top style="thin">
-        <color theme="4"/>
+        <color rgb="FFB2B2B2"/>
       </top>
-      <bottom style="double">
+      <bottom style="thin">
+        <color rgb="FFB2B2B2"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
         <color theme="4"/>
       </bottom>
       <diagonal/>
@@ -851,153 +816,188 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="4"/>
+      </top>
+      <bottom style="double">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="double">
+        <color rgb="FFFF8001"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="double">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="double">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="double">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="double">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="5" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="19" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="18" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="5" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="12" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="7" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="12" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="17" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="26" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="5" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="4" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
@@ -3678,7 +3678,9 @@
       <c r="K44" s="2"/>
       <c r="L44" s="2"/>
       <c r="M44" s="2"/>
-      <c r="N44" s="2"/>
+      <c r="N44" s="2" t="s">
+        <v>19</v>
+      </c>
       <c r="O44" s="2"/>
       <c r="P44" s="2"/>
       <c r="Q44" s="2"/>
@@ -5221,44 +5223,44 @@
     </row>
   </sheetData>
   <dataValidations count="14">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="M29 M30 M31 M39 M40 M41 M42 M43 M44 M2:M28 M32:M38 M45:M1048576">
+      <formula1>"CSR_W,CSR_S,CSR_C,CSR_P,CSR_XX"</formula1>
+    </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F6 F15 F18 F19 F20 F21 F24 F25 F26 F27 F28 F29 F30 F31 F32 F33 F36 F37 F38 F39 F40 F41 F42 F43 F44 F2:F5 F7:F14 F16:F17 F22:F23 F34:F35 F45:F1048576">
       <formula1>"ALU_ADD,ALU_SUB,ALU_AND,ALU_OR,ALU_XOR,ALU_SLL,ALU_SRL,ALU_SLT,ALU_SLTU,ALU_COPY_A,ALU_COPY_B,ALU_SRA"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L5 L6 L7 L10 L11 L14 L15 L16 L17 L18 L19 L20 L21 L22 L23 L24 L25 L26 L27 L28 L29 L30 L31 L32 L33 L34 L35 L36 L37 L38 L39 L40 L41 L42 L43 L44 L2:L4 L8:L9 L12:L13 L45:L1048576">
+      <formula1>"BR_EQ,BR_NE,BR_LTU,BR_GE,BR_GEU,BR_LT,BR_XX"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="O44 O2:O43 O45:O1048576">
+      <formula1>"R_TYPE,I_TYPE,S_TYPE,B_TYPE,U_TYPE,J_TYPE,ICSR_TYPE,FENCE_TYPE,N_TYPE"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J5 J6 J7 J8 J9 J10 J11 J12 J13 J14 J15 J16 J17 J18 J19 J20 J21 J22 J23 J24 J25 J26 J27 J28 J29 J30 J31 J32 J33 J34 J35 J36 J37 J38 J39 J40 J41 J42 J43 J44 J2:J4 J45:J1048576">
       <formula1>"ST_SW,ST_SH,ST_SB,ST_XX"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C29 C30 C31 C43 C44 C2:C28 C32:C42 C45:C1048576">
-      <formula1>"PC_4,PC_0,PC_ALU,PC_CSR"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K4 K5 K6 K7 K8 K9 K10 K11 K12 K13 K14 K15 K16 K17 K18 K19 K20 K21 K22 K23 K24 K25 K26 K27 K28 K29 K30 K31 K32 K33 K34 K35 K36 K37 K38 K39 K40 K41 K42 K43 K44 K2:K3 K45:K1048576">
+      <formula1>"MASK_XX,MASK_B,MASK_H,MASK_W,MASK_D"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G4 G5 G6 G7 G8 G9 G10 G11 G12 G13 G14 G15 G16 G17 G18 G19 G20 G21 G22 G23 G24 G25 G26 G27 G28 G29 G30 G31 G32 G33 G34 G35 G36 G37 G38 G39 G40 G41 G42 G43 G44 G2:G3 G45:G1048576">
+      <formula1>"IMM_I,IMM_J,IMM_U,IMM_S,IMM_B"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="N4 N5 N6 N7 N8 N9 N10 N11 N12 N13 N14 N15 N16 N17 N18 N19 N20 N21 N22 N23 N24 N25 N26 N27 N28 N29 N30 N31 N32 N33 N34 N35 N36 N37 N38 N39 N40 N41 N42 N43 N44 N2:N3 N45:N1048576">
       <formula1>"INST_VALID,INST_INVALID"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="M29 M30 M31 M39 M40 M41 M42 M43 M44 M2:M28 M32:M38 M45:M1048576">
-      <formula1>"CSR_W,CSR_S,CSR_C,CSR_P,CSR_XX"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G4 G5 G6 G7 G8 G9 G10 G11 G12 G13 G14 G15 G16 G17 G18 G19 G20 G21 G22 G23 G24 G25 G26 G27 G28 G29 G30 G31 G32 G33 G34 G35 G36 G37 G38 G39 G40 G41 G42 G43 G44 G2:G3 G45:G1048576">
-      <formula1>"IMM_I,IMM_J,IMM_U,IMM_S,IMM_B"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H29 H30 H31 H40 H41 H42 H43 H44 H10:H28 H32:H39 H45:H1048576">
+      <formula1>"WB_ALU,WB_MEM,WB_PC4,WB_XX,WB_CSR"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E4 E5 E6 E7 E8 E9 E10 E11 E12 E13 E14 E15 E16 E17 E18 E19 E20 E21 E22 E23 E24 E25 E26 E27 E28 E29 E30 E31 E32 E33 E34 E35 E36 E37 E38 E39 E40 E41 E42 E43 E44 E2:E3 E45:E1048576">
       <formula1>"B_IMM,B_RS2"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="O44 O2:O43 O45:O1048576">
-      <formula1>"R_TYPE,I_TYPE,S_TYPE,B_TYPE,U_TYPE,J_TYPE,ICSR_TYPE,FENCE_TYPE,N_TYPE"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K4 K5 K6 K7 K8 K9 K10 K11 K12 K13 K14 K15 K16 K17 K18 K19 K20 K21 K22 K23 K24 K25 K26 K27 K28 K29 K30 K31 K32 K33 K34 K35 K36 K37 K38 K39 K40 K41 K42 K43 K44 K2:K3 K45:K1048576">
-      <formula1>"MASK_XX,MASK_B,MASK_H,MASK_W,MASK_D"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L5 L6 L7 L10 L11 L14 L15 L16 L17 L18 L19 L20 L21 L22 L23 L24 L25 L26 L27 L28 L29 L30 L31 L32 L33 L34 L35 L36 L37 L38 L39 L40 L41 L42 L43 L44 L2:L4 L8:L9 L12:L13 L45:L1048576">
-      <formula1>"BR_EQ,BR_NE,BR_LTU,BR_GE,BR_GEU,BR_LT,BR_XX"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H5 H6 H7 H8 H9 H2:H4">
+      <formula1>"WB_ALU,WB_MEM,WB_PC4,WB_XX"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I4 I5 I6 I7 I8 I9 I10 I11 I12 I13 I14 I15 I16 I17 I18 I19 I20 I21 I22 I23 I24 I25 I26 I27 I28 I29 I30 I31 I32 I33 I34 I35 I36 I37 I38 I39 I40 I41 I42 I43 I44 I2:I3 I45:I1048576">
       <formula1>"LD_LB,LD_LH,LD_LW,LD_LBU,LD_LHU,LD_XX"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H29 H30 H31 H40 H41 H42 H43 H44 H10:H28 H32:H39 H45:H1048576">
-      <formula1>"WB_ALU,WB_MEM,WB_PC4,WB_XX,WB_CSR"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H5 H6 H7 H8 H9 H2:H4">
-      <formula1>"WB_ALU,WB_MEM,WB_PC4,WB_XX"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C29 C30 C31 C43 C44 C2:C28 C32:C42 C45:C1048576">
+      <formula1>"PC_4,PC_0,PC_ALU,PC_CSR"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D4 D5 D6 D7 D8 D9 D10 D11 D12 D13 D14 D15 D16 D17 D18 D19 D20 D21 D22 D23 D24 D25 D26 D27 D28 D29 D30 D31 D32 D33 D34 D35 D36 D37 D38 D39 D40 D41 D42 D43 D44 D2:D3 D45:D1048576">
       <formula1>"A_PC,A_RS1"</formula1>

</xml_diff>

<commit_message>
move ebreak to wbu stage
</commit_message>
<xml_diff>
--- a/npc/tools/control_gen/control_table.xlsx
+++ b/npc/tools/control_gen/control_table.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="23370" windowHeight="12150"/>
+    <workbookView windowWidth="18200" windowHeight="7440"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="355" uniqueCount="119">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="357" uniqueCount="120">
   <si>
     <t>comment</t>
   </si>
@@ -347,6 +347,9 @@
   </si>
   <si>
     <t>fencei</t>
+  </si>
+  <si>
+    <t>ebreak</t>
   </si>
   <si>
     <t>default</t>
@@ -379,9 +382,9 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="4">
     <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="41" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
     <numFmt numFmtId="42" formatCode="_ &quot;￥&quot;* #,##0_ ;_ &quot;￥&quot;* \-#,##0_ ;_ &quot;￥&quot;* &quot;-&quot;_ ;_ @_ "/>
     <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="41" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
   <fonts count="22">
     <font>
@@ -411,6 +414,14 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF3F3F3F"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <sz val="11"/>
       <color theme="0"/>
       <name val="宋体"/>
@@ -427,14 +438,7 @@
     <font>
       <u/>
       <sz val="11"/>
-      <color rgb="FF0000FF"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
+      <color rgb="FF800080"/>
       <name val="宋体"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -449,32 +453,16 @@
     </font>
     <font>
       <b/>
-      <sz val="18"/>
+      <sz val="15"/>
       <color theme="3"/>
       <name val="宋体"/>
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF800080"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <b/>
       <sz val="11"/>
-      <color rgb="FF3F3F3F"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
+      <color rgb="FFFA7D00"/>
       <name val="宋体"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -482,6 +470,13 @@
     <font>
       <sz val="11"/>
       <color rgb="FF9C0006"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF006100"/>
       <name val="宋体"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -495,14 +490,21 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <b/>
+      <sz val="13"/>
+      <color theme="3"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <sz val="11"/>
-      <color rgb="FF9C6500"/>
+      <color rgb="FF3F3F76"/>
       <name val="宋体"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
       <sz val="11"/>
       <color rgb="FFFA7D00"/>
       <name val="宋体"/>
@@ -511,25 +513,9 @@
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FF006100"/>
+      <color rgb="FF9C6500"/>
       <name val="宋体"/>
       <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="13"/>
-      <color theme="3"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="15"/>
-      <color theme="3"/>
-      <name val="宋体"/>
-      <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -541,8 +527,25 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <b/>
+      <sz val="18"/>
+      <color theme="3"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
-      <color rgb="FF3F3F76"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF0000FF"/>
       <name val="宋体"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -563,7 +566,31 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.599993896298105"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -581,49 +608,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor theme="5" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.599993896298105"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -635,25 +620,31 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
+        <fgColor rgb="FFFFC7CE"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.599993896298105"/>
+        <fgColor theme="4" tint="0.399975585192419"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFA5A5A5"/>
+        <fgColor rgb="FFC6EFCE"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
+        <fgColor theme="8" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.599993896298105"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -671,6 +662,18 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FFFFCC99"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor theme="6" tint="0.799981688894314"/>
         <bgColor indexed="64"/>
       </patternFill>
@@ -683,19 +686,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.399975585192419"/>
+        <fgColor theme="5" tint="0.599993896298105"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -707,13 +698,19 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5"/>
+        <fgColor theme="7"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.799981688894314"/>
+        <fgColor rgb="FFA5A5A5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.799981688894314"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -725,19 +722,25 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.799981688894314"/>
+        <fgColor theme="5" tint="0.399975585192419"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="9" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.799981688894314"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -748,6 +751,30 @@
       <right/>
       <top/>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4" tint="0.499984740745262"/>
+      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -769,57 +796,7 @@
       <left/>
       <right/>
       <top/>
-      <bottom style="double">
-        <color rgb="FFFF8001"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
       <bottom style="medium">
-        <color theme="4" tint="0.499984740745262"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="double">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="double">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="double">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="double">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color theme="4"/>
-      </top>
-      <bottom style="double">
         <color theme="4"/>
       </bottom>
       <diagonal/>
@@ -842,9 +819,35 @@
     <border>
       <left/>
       <right/>
+      <top style="thin">
+        <color theme="4"/>
+      </top>
+      <bottom style="double">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
       <top/>
-      <bottom style="medium">
-        <color theme="4"/>
+      <bottom style="double">
+        <color rgb="FFFF8001"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="double">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="double">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="double">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="double">
+        <color rgb="FF3F3F3F"/>
       </bottom>
       <diagonal/>
     </border>
@@ -853,148 +856,148 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="30" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="5" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="19" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="26" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="15" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="17" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="15" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
@@ -1339,28 +1342,28 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:AJ99"/>
+  <dimension ref="A1:AJ100"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
     <col min="1" max="1" width="13.1" customWidth="1"/>
-    <col min="2" max="2" width="17.7583333333333" customWidth="1"/>
-    <col min="3" max="3" width="10.1416666666667" customWidth="1"/>
-    <col min="4" max="4" width="7.75" customWidth="1"/>
-    <col min="5" max="5" width="11.7166666666667" customWidth="1"/>
-    <col min="6" max="6" width="11.1166666666667" customWidth="1"/>
-    <col min="7" max="7" width="10.9416666666667" customWidth="1"/>
-    <col min="8" max="10" width="11.9833333333333" customWidth="1"/>
-    <col min="11" max="11" width="15.075" customWidth="1"/>
-    <col min="12" max="14" width="12.1083333333333" customWidth="1"/>
-    <col min="15" max="16" width="10.8583333333333" customWidth="1"/>
-    <col min="18" max="18" width="14.2166666666667" customWidth="1"/>
-    <col min="19" max="19" width="11.8083333333333" customWidth="1"/>
+    <col min="2" max="2" width="17.7545454545455" customWidth="1"/>
+    <col min="3" max="3" width="10.1454545454545" customWidth="1"/>
+    <col min="4" max="4" width="7.75454545454545" customWidth="1"/>
+    <col min="5" max="5" width="11.7181818181818" customWidth="1"/>
+    <col min="6" max="6" width="11.1181818181818" customWidth="1"/>
+    <col min="7" max="7" width="10.9454545454545" customWidth="1"/>
+    <col min="8" max="10" width="11.9818181818182" customWidth="1"/>
+    <col min="11" max="11" width="15.0727272727273" customWidth="1"/>
+    <col min="12" max="14" width="12.1090909090909" customWidth="1"/>
+    <col min="15" max="16" width="10.8545454545455" customWidth="1"/>
+    <col min="18" max="18" width="14.2181818181818" customWidth="1"/>
+    <col min="19" max="19" width="11.8090909090909" customWidth="1"/>
     <col min="20" max="20" width="10.6" customWidth="1"/>
-    <col min="21" max="21" width="9.70833333333333" customWidth="1"/>
-    <col min="22" max="22" width="11.1666666666667" customWidth="1"/>
-    <col min="23" max="23" width="11.4083333333333" customWidth="1"/>
-    <col min="24" max="24" width="12.0583333333333" customWidth="1"/>
-    <col min="25" max="25" width="15.575" customWidth="1"/>
+    <col min="21" max="21" width="9.70909090909091" customWidth="1"/>
+    <col min="22" max="22" width="11.1636363636364" customWidth="1"/>
+    <col min="23" max="23" width="11.4090909090909" customWidth="1"/>
+    <col min="24" max="24" width="12.0545454545455" customWidth="1"/>
+    <col min="25" max="25" width="15.5727272727273" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1" spans="1:24">
@@ -3664,45 +3667,21 @@
       <c r="B44" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="C44" s="2" t="s">
-        <v>100</v>
-      </c>
-      <c r="D44" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="E44" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="F44" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="G44" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="H44" s="4" t="s">
-        <v>112</v>
-      </c>
-      <c r="I44" s="4" t="s">
-        <v>113</v>
-      </c>
-      <c r="J44" s="4" t="s">
-        <v>114</v>
-      </c>
-      <c r="K44" s="2" t="s">
-        <v>115</v>
-      </c>
-      <c r="L44" s="2" t="s">
-        <v>116</v>
-      </c>
-      <c r="M44" s="2" t="s">
-        <v>117</v>
-      </c>
+      <c r="C44" s="2"/>
+      <c r="D44" s="2"/>
+      <c r="E44" s="2"/>
+      <c r="F44" s="2"/>
+      <c r="G44" s="2"/>
+      <c r="H44" s="4"/>
+      <c r="I44" s="4"/>
+      <c r="J44" s="4"/>
+      <c r="K44" s="2"/>
+      <c r="L44" s="2"/>
+      <c r="M44" s="2"/>
       <c r="N44" s="2" t="s">
-        <v>118</v>
-      </c>
-      <c r="O44" s="2" t="s">
-        <v>82</v>
-      </c>
+        <v>19</v>
+      </c>
+      <c r="O44" s="2"/>
       <c r="P44" s="2"/>
       <c r="Q44" s="2"/>
       <c r="R44" s="2"/>
@@ -3721,32 +3700,55 @@
       <c r="AI44" s="3"/>
       <c r="AJ44" s="3"/>
     </row>
-    <row r="45" spans="1:36">
-      <c r="A45" s="3"/>
-      <c r="B45" s="4"/>
-      <c r="C45" s="4"/>
-      <c r="D45" s="4"/>
-      <c r="E45" s="4"/>
-      <c r="F45" s="4"/>
-      <c r="G45" s="4"/>
-      <c r="H45" s="4"/>
-      <c r="I45" s="4"/>
-      <c r="J45" s="4"/>
-      <c r="K45" s="4"/>
-      <c r="L45" s="4"/>
-      <c r="M45" s="4"/>
-      <c r="N45" s="4"/>
-      <c r="O45" s="4"/>
-      <c r="P45" s="4"/>
-      <c r="Q45" s="4"/>
-      <c r="R45" s="4"/>
-      <c r="S45" s="4"/>
-      <c r="T45" s="4"/>
-      <c r="U45" s="4"/>
-      <c r="V45" s="3"/>
-      <c r="W45" s="3"/>
-      <c r="X45" s="3"/>
-      <c r="Y45" s="3"/>
+    <row r="45" spans="2:36">
+      <c r="B45" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="C45" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="D45" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="E45" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="F45" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="G45" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="H45" s="4" t="s">
+        <v>113</v>
+      </c>
+      <c r="I45" s="4" t="s">
+        <v>114</v>
+      </c>
+      <c r="J45" s="4" t="s">
+        <v>115</v>
+      </c>
+      <c r="K45" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="L45" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="M45" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="N45" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="O45" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="P45" s="2"/>
+      <c r="Q45" s="2"/>
+      <c r="R45" s="2"/>
+      <c r="S45" s="2"/>
+      <c r="T45" s="2"/>
+      <c r="U45" s="2"/>
       <c r="Z45" s="3"/>
       <c r="AA45" s="3"/>
       <c r="AB45" s="3"/>
@@ -3759,7 +3761,7 @@
       <c r="AI45" s="3"/>
       <c r="AJ45" s="3"/>
     </row>
-    <row r="46" s="1" customFormat="1" spans="1:36">
+    <row r="46" spans="1:36">
       <c r="A46" s="3"/>
       <c r="B46" s="4"/>
       <c r="C46" s="4"/>
@@ -3835,7 +3837,7 @@
       <c r="AI47" s="3"/>
       <c r="AJ47" s="3"/>
     </row>
-    <row r="48" spans="1:36">
+    <row r="48" s="1" customFormat="1" spans="1:36">
       <c r="A48" s="3"/>
       <c r="B48" s="4"/>
       <c r="C48" s="4"/>
@@ -4410,7 +4412,7 @@
       <c r="B63" s="4"/>
       <c r="C63" s="4"/>
       <c r="D63" s="4"/>
-      <c r="E63" s="5"/>
+      <c r="E63" s="4"/>
       <c r="F63" s="4"/>
       <c r="G63" s="4"/>
       <c r="H63" s="4"/>
@@ -4524,7 +4526,7 @@
       <c r="B66" s="4"/>
       <c r="C66" s="4"/>
       <c r="D66" s="4"/>
-      <c r="E66" s="4"/>
+      <c r="E66" s="5"/>
       <c r="F66" s="4"/>
       <c r="G66" s="4"/>
       <c r="H66" s="4"/>
@@ -4676,7 +4678,7 @@
       <c r="B70" s="4"/>
       <c r="C70" s="4"/>
       <c r="D70" s="4"/>
-      <c r="E70" s="5"/>
+      <c r="E70" s="4"/>
       <c r="F70" s="4"/>
       <c r="G70" s="4"/>
       <c r="H70" s="4"/>
@@ -4714,7 +4716,7 @@
       <c r="B71" s="4"/>
       <c r="C71" s="4"/>
       <c r="D71" s="4"/>
-      <c r="E71" s="4"/>
+      <c r="E71" s="5"/>
       <c r="F71" s="4"/>
       <c r="G71" s="4"/>
       <c r="H71" s="4"/>
@@ -5013,25 +5015,50 @@
       <c r="AI78" s="3"/>
       <c r="AJ78" s="3"/>
     </row>
-    <row r="86" spans="1:25">
-      <c r="A86" s="2"/>
-      <c r="B86" s="2"/>
-      <c r="C86" s="2"/>
-      <c r="D86" s="2"/>
-      <c r="T86" s="2"/>
-      <c r="V86" s="2"/>
-      <c r="W86" s="2"/>
-      <c r="X86" s="2"/>
-      <c r="Y86" s="2"/>
+    <row r="79" spans="1:36">
+      <c r="A79" s="3"/>
+      <c r="B79" s="4"/>
+      <c r="C79" s="4"/>
+      <c r="D79" s="4"/>
+      <c r="E79" s="4"/>
+      <c r="F79" s="4"/>
+      <c r="G79" s="4"/>
+      <c r="H79" s="4"/>
+      <c r="I79" s="4"/>
+      <c r="J79" s="4"/>
+      <c r="K79" s="4"/>
+      <c r="L79" s="4"/>
+      <c r="M79" s="4"/>
+      <c r="N79" s="4"/>
+      <c r="O79" s="4"/>
+      <c r="P79" s="4"/>
+      <c r="Q79" s="4"/>
+      <c r="R79" s="4"/>
+      <c r="S79" s="4"/>
+      <c r="T79" s="4"/>
+      <c r="U79" s="4"/>
+      <c r="V79" s="3"/>
+      <c r="W79" s="3"/>
+      <c r="X79" s="3"/>
+      <c r="Y79" s="3"/>
+      <c r="Z79" s="3"/>
+      <c r="AA79" s="3"/>
+      <c r="AB79" s="3"/>
+      <c r="AC79" s="3"/>
+      <c r="AD79" s="3"/>
+      <c r="AE79" s="3"/>
+      <c r="AF79" s="3"/>
+      <c r="AG79" s="3"/>
+      <c r="AH79" s="3"/>
+      <c r="AI79" s="3"/>
+      <c r="AJ79" s="3"/>
     </row>
     <row r="87" spans="1:25">
       <c r="A87" s="2"/>
       <c r="B87" s="2"/>
       <c r="C87" s="2"/>
       <c r="D87" s="2"/>
-      <c r="E87" s="2"/>
       <c r="T87" s="2"/>
-      <c r="U87" s="2"/>
       <c r="V87" s="2"/>
       <c r="W87" s="2"/>
       <c r="X87" s="2"/>
@@ -5042,6 +5069,7 @@
       <c r="B88" s="2"/>
       <c r="C88" s="2"/>
       <c r="D88" s="2"/>
+      <c r="E88" s="2"/>
       <c r="T88" s="2"/>
       <c r="U88" s="2"/>
       <c r="V88" s="2"/>
@@ -5181,48 +5209,60 @@
       <c r="X99" s="2"/>
       <c r="Y99" s="2"/>
     </row>
+    <row r="100" spans="1:25">
+      <c r="A100" s="2"/>
+      <c r="B100" s="2"/>
+      <c r="C100" s="2"/>
+      <c r="D100" s="2"/>
+      <c r="T100" s="2"/>
+      <c r="U100" s="2"/>
+      <c r="V100" s="2"/>
+      <c r="W100" s="2"/>
+      <c r="X100" s="2"/>
+      <c r="Y100" s="2"/>
+    </row>
   </sheetData>
   <dataValidations count="14">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="O2:O1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="M29 M30 M31 M39 M40 M41 M42 M43 M44 M2:M28 M32:M38 M45:M1048576">
+      <formula1>"CSR_W,CSR_S,CSR_C,CSR_P,CSR_XX"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F6 F15 F18 F19 F20 F21 F24 F25 F26 F27 F28 F29 F30 F31 F32 F33 F36 F37 F38 F39 F40 F41 F42 F43 F44 F2:F5 F7:F14 F16:F17 F22:F23 F34:F35 F45:F1048576">
+      <formula1>"ALU_ADD,ALU_SUB,ALU_AND,ALU_OR,ALU_XOR,ALU_SLL,ALU_SRL,ALU_SLT,ALU_SLTU,ALU_COPY_A,ALU_COPY_B,ALU_SRA"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L5 L6 L7 L10 L11 L14 L15 L16 L17 L18 L19 L20 L21 L22 L23 L24 L25 L26 L27 L28 L29 L30 L31 L32 L33 L34 L35 L36 L37 L38 L39 L40 L41 L42 L43 L44 L2:L4 L8:L9 L12:L13 L45:L1048576">
+      <formula1>"BR_EQ,BR_NE,BR_LTU,BR_GE,BR_GEU,BR_LT,BR_XX"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="O44 O2:O43 O45:O1048576">
       <formula1>"R_TYPE,I_TYPE,S_TYPE,B_TYPE,U_TYPE,J_TYPE,ICSR_TYPE,FENCE_TYPE,N_TYPE"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="M29 M30 M31 M39 M40 M41 M42 M43 M2:M28 M32:M38 M44:M1048576">
-      <formula1>"CSR_W,CSR_S,CSR_C,CSR_P,CSR_XX"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J5 J6 J7 J8 J9 J10 J11 J12 J13 J14 J15 J16 J17 J18 J19 J20 J21 J22 J23 J24 J25 J26 J27 J28 J29 J30 J31 J32 J33 J34 J35 J36 J37 J38 J39 J40 J41 J42 J43 J44 J2:J4 J45:J1048576">
+      <formula1>"ST_SW,ST_SH,ST_SB,ST_XX"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H29 H30 H31 H40 H41 H42 H43 H10:H28 H32:H39 H44:H1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K4 K5 K6 K7 K8 K9 K10 K11 K12 K13 K14 K15 K16 K17 K18 K19 K20 K21 K22 K23 K24 K25 K26 K27 K28 K29 K30 K31 K32 K33 K34 K35 K36 K37 K38 K39 K40 K41 K42 K43 K44 K2:K3 K45:K1048576">
+      <formula1>"MASK_XX,MASK_B,MASK_H,MASK_W,MASK_D"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G4 G5 G6 G7 G8 G9 G10 G11 G12 G13 G14 G15 G16 G17 G18 G19 G20 G21 G22 G23 G24 G25 G26 G27 G28 G29 G30 G31 G32 G33 G34 G35 G36 G37 G38 G39 G40 G41 G42 G43 G44 G2:G3 G45:G1048576">
+      <formula1>"IMM_I,IMM_J,IMM_U,IMM_S,IMM_B"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="N4 N5 N6 N7 N8 N9 N10 N11 N12 N13 N14 N15 N16 N17 N18 N19 N20 N21 N22 N23 N24 N25 N26 N27 N28 N29 N30 N31 N32 N33 N34 N35 N36 N37 N38 N39 N40 N41 N42 N43 N44 N2:N3 N45:N1048576">
+      <formula1>"INST_VALID,INST_INVALID"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H29 H30 H31 H40 H41 H42 H43 H44 H10:H28 H32:H39 H45:H1048576">
       <formula1>"WB_ALU,WB_MEM,WB_PC4,WB_XX,WB_CSR"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C29 C30 C31 C43 C2:C28 C32:C42 C44:C1048576">
-      <formula1>"PC_4,PC_0,PC_ALU,PC_CSR"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E4 E5 E6 E7 E8 E9 E10 E11 E12 E13 E14 E15 E16 E17 E18 E19 E20 E21 E22 E23 E24 E25 E26 E27 E28 E29 E30 E31 E32 E33 E34 E35 E36 E37 E38 E39 E40 E41 E42 E43 E2:E3 E44:E1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E4 E5 E6 E7 E8 E9 E10 E11 E12 E13 E14 E15 E16 E17 E18 E19 E20 E21 E22 E23 E24 E25 E26 E27 E28 E29 E30 E31 E32 E33 E34 E35 E36 E37 E38 E39 E40 E41 E42 E43 E44 E2:E3 E45:E1048576">
       <formula1>"B_IMM,B_RS2"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G4 G5 G6 G7 G8 G9 G10 G11 G12 G13 G14 G15 G16 G17 G18 G19 G20 G21 G22 G23 G24 G25 G26 G27 G28 G29 G30 G31 G32 G33 G34 G35 G36 G37 G38 G39 G40 G41 G42 G43 G2:G3 G44:G1048576">
-      <formula1>"IMM_I,IMM_J,IMM_U,IMM_S,IMM_B"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J5 J6 J7 J8 J9 J10 J11 J12 J13 J14 J15 J16 J17 J18 J19 J20 J21 J22 J23 J24 J25 J26 J27 J28 J29 J30 J31 J32 J33 J34 J35 J36 J37 J38 J39 J40 J41 J42 J43 J2:J4 J44:J1048576">
-      <formula1>"ST_SW,ST_SH,ST_SB,ST_XX"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H5 H6 H7 H8 H9 H2:H4">
       <formula1>"WB_ALU,WB_MEM,WB_PC4,WB_XX"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L5 L6 L7 L10 L11 L14 L15 L16 L17 L18 L19 L20 L21 L22 L23 L24 L25 L26 L27 L28 L29 L30 L31 L32 L33 L34 L35 L36 L37 L38 L39 L40 L41 L42 L43 L2:L4 L8:L9 L12:L13 L44:L1048576">
-      <formula1>"BR_EQ,BR_NE,BR_LTU,BR_GE,BR_GEU,BR_LT,BR_XX"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="N4 N5 N6 N7 N8 N9 N10 N11 N12 N13 N14 N15 N16 N17 N18 N19 N20 N21 N22 N23 N24 N25 N26 N27 N28 N29 N30 N31 N32 N33 N34 N35 N36 N37 N38 N39 N40 N41 N42 N43 N2:N3 N44:N1048576">
-      <formula1>"INST_VALID,INST_INVALID"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I4 I5 I6 I7 I8 I9 I10 I11 I12 I13 I14 I15 I16 I17 I18 I19 I20 I21 I22 I23 I24 I25 I26 I27 I28 I29 I30 I31 I32 I33 I34 I35 I36 I37 I38 I39 I40 I41 I42 I43 I2:I3 I44:I1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I4 I5 I6 I7 I8 I9 I10 I11 I12 I13 I14 I15 I16 I17 I18 I19 I20 I21 I22 I23 I24 I25 I26 I27 I28 I29 I30 I31 I32 I33 I34 I35 I36 I37 I38 I39 I40 I41 I42 I43 I44 I2:I3 I45:I1048576">
       <formula1>"LD_LB,LD_LH,LD_LW,LD_LBU,LD_LHU,LD_XX"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F6 F15 F18 F19 F20 F21 F24 F25 F26 F27 F28 F29 F30 F31 F32 F33 F36 F37 F38 F39 F40 F41 F42 F43 F2:F5 F7:F14 F16:F17 F22:F23 F34:F35 F44:F1048576">
-      <formula1>"ALU_ADD,ALU_SUB,ALU_AND,ALU_OR,ALU_XOR,ALU_SLL,ALU_SRL,ALU_SLT,ALU_SLTU,ALU_COPY_A,ALU_COPY_B,ALU_SRA"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C29 C30 C31 C43 C44 C2:C28 C32:C42 C45:C1048576">
+      <formula1>"PC_4,PC_0,PC_ALU,PC_CSR"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K4 K5 K6 K7 K8 K9 K10 K11 K12 K13 K14 K15 K16 K17 K18 K19 K20 K21 K22 K23 K24 K25 K26 K27 K28 K29 K30 K31 K32 K33 K34 K35 K36 K37 K38 K39 K40 K41 K42 K43 K2:K3 K44:K1048576">
-      <formula1>"MASK_XX,MASK_B,MASK_H,MASK_W,MASK_D"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D4 D5 D6 D7 D8 D9 D10 D11 D12 D13 D14 D15 D16 D17 D18 D19 D20 D21 D22 D23 D24 D25 D26 D27 D28 D29 D30 D31 D32 D33 D34 D35 D36 D37 D38 D39 D40 D41 D42 D43 D2:D3 D44:D1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D4 D5 D6 D7 D8 D9 D10 D11 D12 D13 D14 D15 D16 D17 D18 D19 D20 D21 D22 D23 D24 D25 D26 D27 D28 D29 D30 D31 D32 D33 D34 D35 D36 D37 D38 D39 D40 D41 D42 D43 D44 D2:D3 D45:D1048576">
       <formula1>"A_PC,A_RS1"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
> sim RTL ysyx_23060246 韩炳晋 Linux archlinux 6.12.43-1-lts #1 SMP PREEMPT_DYNAMIC Wed, 20 Aug 2025 17:50:11 +0000 x86_64 GNU/Linux  18:20:23 up 3 days,  4:29,  1 user,  load average: 1.42, 1.30, 1.92
</commit_message>
<xml_diff>
--- a/npc/tools/control_gen/control_table.xlsx
+++ b/npc/tools/control_gen/control_table.xlsx
@@ -4,12 +4,25 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="18200" windowHeight="7440"/>
+    <workbookView windowHeight="17715"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="144525"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -379,12 +392,12 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
   <numFmts count="4">
-    <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="41" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
     <numFmt numFmtId="42" formatCode="_ &quot;￥&quot;* #,##0_ ;_ &quot;￥&quot;* \-#,##0_ ;_ &quot;￥&quot;* &quot;-&quot;_ ;_ @_ "/>
     <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
   </numFmts>
   <fonts count="22">
     <font>
@@ -407,8 +420,71 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <u/>
       <sz val="11"/>
-      <color theme="1"/>
+      <color rgb="FF0000FF"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF800080"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="18"/>
+      <color theme="3"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color rgb="FF7F7F7F"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="15"/>
+      <color theme="3"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="13"/>
+      <color theme="3"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="3"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF3F3F76"/>
       <name val="宋体"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -422,23 +498,9 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <b/>
       <sz val="11"/>
-      <color theme="0"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF800080"/>
+      <color rgb="FFFA7D00"/>
       <name val="宋体"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -446,23 +508,29 @@
     <font>
       <b/>
       <sz val="11"/>
-      <color theme="3"/>
+      <color rgb="FFFFFFFF"/>
       <name val="宋体"/>
-      <charset val="134"/>
+      <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <sz val="15"/>
-      <color theme="3"/>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
       <name val="宋体"/>
-      <charset val="134"/>
+      <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
-      <color rgb="FFFA7D00"/>
+      <color theme="1"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF006100"/>
       <name val="宋体"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -476,76 +544,21 @@
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FF006100"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="13"/>
-      <color theme="3"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF3F3F76"/>
+      <color rgb="FF9C6500"/>
       <name val="宋体"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FFFA7D00"/>
+      <color theme="0"/>
       <name val="宋体"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FF9C6500"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="11"/>
-      <color rgb="FF7F7F7F"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="18"/>
-      <color theme="3"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF0000FF"/>
+      <color theme="1"/>
       <name val="宋体"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -560,7 +573,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.599993896298105"/>
+        <fgColor rgb="FFFFFFCC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFCC99"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -572,7 +591,133 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="9"/>
+        <fgColor rgb="FFA5A5A5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.799981688894314"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -584,7 +729,19 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.799981688894314"/>
+        <fgColor theme="8" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.799981688894314"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -596,151 +753,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="8"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFA5A5A5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor theme="9" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.799981688894314"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -751,30 +764,6 @@
       <right/>
       <top/>
       <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4" tint="0.499984740745262"/>
-      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -802,6 +791,15 @@
       <diagonal/>
     </border>
     <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4" tint="0.499984740745262"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
       <left style="thin">
         <color rgb="FF7F7F7F"/>
       </left>
@@ -817,22 +815,17 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right/>
+      <left style="thin">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF3F3F3F"/>
+      </right>
       <top style="thin">
-        <color theme="4"/>
+        <color rgb="FF3F3F3F"/>
       </top>
-      <bottom style="double">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="double">
-        <color rgb="FFFF8001"/>
+      <bottom style="thin">
+        <color rgb="FF3F3F3F"/>
       </bottom>
       <diagonal/>
     </border>
@@ -851,153 +844,173 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="double">
+        <color rgb="FFFF8001"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="4"/>
+      </top>
+      <bottom style="double">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="19" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="26" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
@@ -1026,54 +1039,54 @@
   </cellXfs>
   <cellStyles count="49">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
-    <cellStyle name="60% - 强调文字颜色 6" xfId="1" builtinId="52"/>
-    <cellStyle name="20% - 强调文字颜色 4" xfId="2" builtinId="42"/>
-    <cellStyle name="强调文字颜色 4" xfId="3" builtinId="41"/>
-    <cellStyle name="输入" xfId="4" builtinId="20"/>
-    <cellStyle name="40% - 强调文字颜色 3" xfId="5" builtinId="39"/>
-    <cellStyle name="20% - 强调文字颜色 3" xfId="6" builtinId="38"/>
-    <cellStyle name="货币" xfId="7" builtinId="4"/>
-    <cellStyle name="强调文字颜色 3" xfId="8" builtinId="37"/>
-    <cellStyle name="百分比" xfId="9" builtinId="5"/>
-    <cellStyle name="60% - 强调文字颜色 2" xfId="10" builtinId="36"/>
-    <cellStyle name="60% - 强调文字颜色 5" xfId="11" builtinId="48"/>
-    <cellStyle name="强调文字颜色 2" xfId="12" builtinId="33"/>
-    <cellStyle name="60% - 强调文字颜色 1" xfId="13" builtinId="32"/>
-    <cellStyle name="60% - 强调文字颜色 4" xfId="14" builtinId="44"/>
-    <cellStyle name="计算" xfId="15" builtinId="22"/>
-    <cellStyle name="强调文字颜色 1" xfId="16" builtinId="29"/>
-    <cellStyle name="适中" xfId="17" builtinId="28"/>
-    <cellStyle name="20% - 强调文字颜色 5" xfId="18" builtinId="46"/>
-    <cellStyle name="好" xfId="19" builtinId="26"/>
-    <cellStyle name="20% - 强调文字颜色 1" xfId="20" builtinId="30"/>
+    <cellStyle name="千位分隔" xfId="1" builtinId="3"/>
+    <cellStyle name="货币" xfId="2" builtinId="4"/>
+    <cellStyle name="百分比" xfId="3" builtinId="5"/>
+    <cellStyle name="千位分隔[0]" xfId="4" builtinId="6"/>
+    <cellStyle name="货币[0]" xfId="5" builtinId="7"/>
+    <cellStyle name="超链接" xfId="6" builtinId="8"/>
+    <cellStyle name="已访问的超链接" xfId="7" builtinId="9"/>
+    <cellStyle name="注释" xfId="8" builtinId="10"/>
+    <cellStyle name="警告文本" xfId="9" builtinId="11"/>
+    <cellStyle name="标题" xfId="10" builtinId="15"/>
+    <cellStyle name="解释性文本" xfId="11" builtinId="53"/>
+    <cellStyle name="标题 1" xfId="12" builtinId="16"/>
+    <cellStyle name="标题 2" xfId="13" builtinId="17"/>
+    <cellStyle name="标题 3" xfId="14" builtinId="18"/>
+    <cellStyle name="标题 4" xfId="15" builtinId="19"/>
+    <cellStyle name="输入" xfId="16" builtinId="20"/>
+    <cellStyle name="输出" xfId="17" builtinId="21"/>
+    <cellStyle name="计算" xfId="18" builtinId="22"/>
+    <cellStyle name="检查单元格" xfId="19" builtinId="23"/>
+    <cellStyle name="链接单元格" xfId="20" builtinId="24"/>
     <cellStyle name="汇总" xfId="21" builtinId="25"/>
-    <cellStyle name="差" xfId="22" builtinId="27"/>
-    <cellStyle name="检查单元格" xfId="23" builtinId="23"/>
-    <cellStyle name="输出" xfId="24" builtinId="21"/>
-    <cellStyle name="标题 1" xfId="25" builtinId="16"/>
-    <cellStyle name="解释性文本" xfId="26" builtinId="53"/>
-    <cellStyle name="20% - 强调文字颜色 2" xfId="27" builtinId="34"/>
-    <cellStyle name="标题 4" xfId="28" builtinId="19"/>
-    <cellStyle name="货币[0]" xfId="29" builtinId="7"/>
-    <cellStyle name="40% - 强调文字颜色 4" xfId="30" builtinId="43"/>
-    <cellStyle name="千位分隔" xfId="31" builtinId="3"/>
-    <cellStyle name="已访问的超链接" xfId="32" builtinId="9"/>
-    <cellStyle name="标题" xfId="33" builtinId="15"/>
-    <cellStyle name="40% - 强调文字颜色 2" xfId="34" builtinId="35"/>
-    <cellStyle name="警告文本" xfId="35" builtinId="11"/>
+    <cellStyle name="好" xfId="22" builtinId="26"/>
+    <cellStyle name="差" xfId="23" builtinId="27"/>
+    <cellStyle name="适中" xfId="24" builtinId="28"/>
+    <cellStyle name="强调文字颜色 1" xfId="25" builtinId="29"/>
+    <cellStyle name="20% - 强调文字颜色 1" xfId="26" builtinId="30"/>
+    <cellStyle name="40% - 强调文字颜色 1" xfId="27" builtinId="31"/>
+    <cellStyle name="60% - 强调文字颜色 1" xfId="28" builtinId="32"/>
+    <cellStyle name="强调文字颜色 2" xfId="29" builtinId="33"/>
+    <cellStyle name="20% - 强调文字颜色 2" xfId="30" builtinId="34"/>
+    <cellStyle name="40% - 强调文字颜色 2" xfId="31" builtinId="35"/>
+    <cellStyle name="60% - 强调文字颜色 2" xfId="32" builtinId="36"/>
+    <cellStyle name="强调文字颜色 3" xfId="33" builtinId="37"/>
+    <cellStyle name="20% - 强调文字颜色 3" xfId="34" builtinId="38"/>
+    <cellStyle name="40% - 强调文字颜色 3" xfId="35" builtinId="39"/>
     <cellStyle name="60% - 强调文字颜色 3" xfId="36" builtinId="40"/>
-    <cellStyle name="注释" xfId="37" builtinId="10"/>
-    <cellStyle name="20% - 强调文字颜色 6" xfId="38" builtinId="50"/>
-    <cellStyle name="强调文字颜色 5" xfId="39" builtinId="45"/>
-    <cellStyle name="40% - 强调文字颜色 6" xfId="40" builtinId="51"/>
-    <cellStyle name="超链接" xfId="41" builtinId="8"/>
-    <cellStyle name="千位分隔[0]" xfId="42" builtinId="6"/>
-    <cellStyle name="标题 2" xfId="43" builtinId="17"/>
-    <cellStyle name="40% - 强调文字颜色 5" xfId="44" builtinId="47"/>
-    <cellStyle name="标题 3" xfId="45" builtinId="18"/>
-    <cellStyle name="强调文字颜色 6" xfId="46" builtinId="49"/>
-    <cellStyle name="40% - 强调文字颜色 1" xfId="47" builtinId="31"/>
-    <cellStyle name="链接单元格" xfId="48" builtinId="24"/>
+    <cellStyle name="强调文字颜色 4" xfId="37" builtinId="41"/>
+    <cellStyle name="20% - 强调文字颜色 4" xfId="38" builtinId="42"/>
+    <cellStyle name="40% - 强调文字颜色 4" xfId="39" builtinId="43"/>
+    <cellStyle name="60% - 强调文字颜色 4" xfId="40" builtinId="44"/>
+    <cellStyle name="强调文字颜色 5" xfId="41" builtinId="45"/>
+    <cellStyle name="20% - 强调文字颜色 5" xfId="42" builtinId="46"/>
+    <cellStyle name="40% - 强调文字颜色 5" xfId="43" builtinId="47"/>
+    <cellStyle name="60% - 强调文字颜色 5" xfId="44" builtinId="48"/>
+    <cellStyle name="强调文字颜色 6" xfId="45" builtinId="49"/>
+    <cellStyle name="20% - 强调文字颜色 6" xfId="46" builtinId="50"/>
+    <cellStyle name="40% - 强调文字颜色 6" xfId="47" builtinId="51"/>
+    <cellStyle name="60% - 强调文字颜色 6" xfId="48" builtinId="52"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -1346,24 +1359,24 @@
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
     <col min="1" max="1" width="13.1" customWidth="1"/>
-    <col min="2" max="2" width="17.7545454545455" customWidth="1"/>
-    <col min="3" max="3" width="10.1454545454545" customWidth="1"/>
-    <col min="4" max="4" width="7.75454545454545" customWidth="1"/>
-    <col min="5" max="5" width="11.7181818181818" customWidth="1"/>
-    <col min="6" max="6" width="11.1181818181818" customWidth="1"/>
-    <col min="7" max="7" width="10.9454545454545" customWidth="1"/>
-    <col min="8" max="10" width="11.9818181818182" customWidth="1"/>
-    <col min="11" max="11" width="15.0727272727273" customWidth="1"/>
-    <col min="12" max="14" width="12.1090909090909" customWidth="1"/>
-    <col min="15" max="16" width="10.8545454545455" customWidth="1"/>
-    <col min="18" max="18" width="14.2181818181818" customWidth="1"/>
-    <col min="19" max="19" width="11.8090909090909" customWidth="1"/>
+    <col min="2" max="2" width="17.7583333333333" customWidth="1"/>
+    <col min="3" max="3" width="10.1416666666667" customWidth="1"/>
+    <col min="4" max="4" width="7.75833333333333" customWidth="1"/>
+    <col min="5" max="5" width="11.7166666666667" customWidth="1"/>
+    <col min="6" max="6" width="11.1166666666667" customWidth="1"/>
+    <col min="7" max="7" width="10.9416666666667" customWidth="1"/>
+    <col min="8" max="10" width="11.9833333333333" customWidth="1"/>
+    <col min="11" max="11" width="15.075" customWidth="1"/>
+    <col min="12" max="14" width="12.1083333333333" customWidth="1"/>
+    <col min="15" max="16" width="10.8583333333333" customWidth="1"/>
+    <col min="18" max="18" width="14.2166666666667" customWidth="1"/>
+    <col min="19" max="19" width="11.8083333333333" customWidth="1"/>
     <col min="20" max="20" width="10.6" customWidth="1"/>
-    <col min="21" max="21" width="9.70909090909091" customWidth="1"/>
-    <col min="22" max="22" width="11.1636363636364" customWidth="1"/>
-    <col min="23" max="23" width="11.4090909090909" customWidth="1"/>
-    <col min="24" max="24" width="12.0545454545455" customWidth="1"/>
-    <col min="25" max="25" width="15.5727272727273" customWidth="1"/>
+    <col min="21" max="21" width="9.70833333333333" customWidth="1"/>
+    <col min="22" max="22" width="11.1666666666667" customWidth="1"/>
+    <col min="23" max="23" width="11.4083333333333" customWidth="1"/>
+    <col min="24" max="24" width="12.0583333333333" customWidth="1"/>
+    <col min="25" max="25" width="15.575" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1" spans="1:24">
@@ -3009,7 +3022,7 @@
         <v>15</v>
       </c>
       <c r="F31" s="4" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="G31" s="4" t="s">
         <v>26</v>
@@ -5223,47 +5236,47 @@
     </row>
   </sheetData>
   <dataValidations count="14">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="M29 M30 M31 M39 M40 M41 M42 M43 M44 M2:M28 M32:M38 M45:M1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C2:C1048576">
+      <formula1>"PC_4,PC_0,PC_ALU,PC_CSR"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D2:D1048576">
+      <formula1>"A_PC,A_RS1"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E2:E1048576">
+      <formula1>"B_IMM,B_RS2"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F2:F1048576">
+      <formula1>"ALU_ADD,ALU_SUB,ALU_AND,ALU_OR,ALU_XOR,ALU_SLL,ALU_SRL,ALU_SLT,ALU_SLTU,ALU_COPY_A,ALU_COPY_B,ALU_SRA"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G2:G1048576">
+      <formula1>"IMM_I,IMM_J,IMM_U,IMM_S,IMM_B"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H2:H9">
+      <formula1>"WB_ALU,WB_MEM,WB_PC4,WB_XX"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H10:H1048576">
+      <formula1>"WB_ALU,WB_MEM,WB_PC4,WB_XX,WB_CSR"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I2:I1048576">
+      <formula1>"LD_LB,LD_LH,LD_LW,LD_LBU,LD_LHU,LD_XX"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J2:J1048576">
+      <formula1>"ST_SW,ST_SH,ST_SB,ST_XX"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K2:K1048576">
+      <formula1>"MASK_XX,MASK_B,MASK_H,MASK_W,MASK_D"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L2:L1048576">
+      <formula1>"BR_EQ,BR_NE,BR_LTU,BR_GE,BR_GEU,BR_LT,BR_XX"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="M2:M1048576">
       <formula1>"CSR_W,CSR_S,CSR_C,CSR_P,CSR_XX"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F6 F15 F18 F19 F20 F21 F24 F25 F26 F27 F28 F29 F30 F31 F32 F33 F36 F37 F38 F39 F40 F41 F42 F43 F44 F2:F5 F7:F14 F16:F17 F22:F23 F34:F35 F45:F1048576">
-      <formula1>"ALU_ADD,ALU_SUB,ALU_AND,ALU_OR,ALU_XOR,ALU_SLL,ALU_SRL,ALU_SLT,ALU_SLTU,ALU_COPY_A,ALU_COPY_B,ALU_SRA"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L5 L6 L7 L10 L11 L14 L15 L16 L17 L18 L19 L20 L21 L22 L23 L24 L25 L26 L27 L28 L29 L30 L31 L32 L33 L34 L35 L36 L37 L38 L39 L40 L41 L42 L43 L44 L2:L4 L8:L9 L12:L13 L45:L1048576">
-      <formula1>"BR_EQ,BR_NE,BR_LTU,BR_GE,BR_GEU,BR_LT,BR_XX"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="O44 O2:O43 O45:O1048576">
-      <formula1>"R_TYPE,I_TYPE,S_TYPE,B_TYPE,U_TYPE,J_TYPE,ICSR_TYPE,FENCE_TYPE,N_TYPE"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J5 J6 J7 J8 J9 J10 J11 J12 J13 J14 J15 J16 J17 J18 J19 J20 J21 J22 J23 J24 J25 J26 J27 J28 J29 J30 J31 J32 J33 J34 J35 J36 J37 J38 J39 J40 J41 J42 J43 J44 J2:J4 J45:J1048576">
-      <formula1>"ST_SW,ST_SH,ST_SB,ST_XX"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K4 K5 K6 K7 K8 K9 K10 K11 K12 K13 K14 K15 K16 K17 K18 K19 K20 K21 K22 K23 K24 K25 K26 K27 K28 K29 K30 K31 K32 K33 K34 K35 K36 K37 K38 K39 K40 K41 K42 K43 K44 K2:K3 K45:K1048576">
-      <formula1>"MASK_XX,MASK_B,MASK_H,MASK_W,MASK_D"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G4 G5 G6 G7 G8 G9 G10 G11 G12 G13 G14 G15 G16 G17 G18 G19 G20 G21 G22 G23 G24 G25 G26 G27 G28 G29 G30 G31 G32 G33 G34 G35 G36 G37 G38 G39 G40 G41 G42 G43 G44 G2:G3 G45:G1048576">
-      <formula1>"IMM_I,IMM_J,IMM_U,IMM_S,IMM_B"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="N4 N5 N6 N7 N8 N9 N10 N11 N12 N13 N14 N15 N16 N17 N18 N19 N20 N21 N22 N23 N24 N25 N26 N27 N28 N29 N30 N31 N32 N33 N34 N35 N36 N37 N38 N39 N40 N41 N42 N43 N44 N2:N3 N45:N1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="N2:N1048576">
       <formula1>"INST_VALID,INST_INVALID"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H29 H30 H31 H40 H41 H42 H43 H44 H10:H28 H32:H39 H45:H1048576">
-      <formula1>"WB_ALU,WB_MEM,WB_PC4,WB_XX,WB_CSR"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E4 E5 E6 E7 E8 E9 E10 E11 E12 E13 E14 E15 E16 E17 E18 E19 E20 E21 E22 E23 E24 E25 E26 E27 E28 E29 E30 E31 E32 E33 E34 E35 E36 E37 E38 E39 E40 E41 E42 E43 E44 E2:E3 E45:E1048576">
-      <formula1>"B_IMM,B_RS2"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H5 H6 H7 H8 H9 H2:H4">
-      <formula1>"WB_ALU,WB_MEM,WB_PC4,WB_XX"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I4 I5 I6 I7 I8 I9 I10 I11 I12 I13 I14 I15 I16 I17 I18 I19 I20 I21 I22 I23 I24 I25 I26 I27 I28 I29 I30 I31 I32 I33 I34 I35 I36 I37 I38 I39 I40 I41 I42 I43 I44 I2:I3 I45:I1048576">
-      <formula1>"LD_LB,LD_LH,LD_LW,LD_LBU,LD_LHU,LD_XX"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C29 C30 C31 C43 C44 C2:C28 C32:C42 C45:C1048576">
-      <formula1>"PC_4,PC_0,PC_ALU,PC_CSR"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D4 D5 D6 D7 D8 D9 D10 D11 D12 D13 D14 D15 D16 D17 D18 D19 D20 D21 D22 D23 D24 D25 D26 D27 D28 D29 D30 D31 D32 D33 D34 D35 D36 D37 D38 D39 D40 D41 D42 D43 D44 D2:D3 D45:D1048576">
-      <formula1>"A_PC,A_RS1"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="O2:O1048576">
+      <formula1>"R_TYPE,I_TYPE,S_TYPE,B_TYPE,U_TYPE,J_TYPE,ICSR_TYPE,FENCE_TYPE,N_TYPE"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
fixed bug for slti
</commit_message>
<xml_diff>
--- a/npc/tools/control_gen/control_table.xlsx
+++ b/npc/tools/control_gen/control_table.xlsx
@@ -4,12 +4,25 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="18200" windowHeight="7440"/>
+    <workbookView windowHeight="17715"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="144525"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -379,12 +392,12 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
   <numFmts count="4">
-    <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="41" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
     <numFmt numFmtId="42" formatCode="_ &quot;￥&quot;* #,##0_ ;_ &quot;￥&quot;* \-#,##0_ ;_ &quot;￥&quot;* &quot;-&quot;_ ;_ @_ "/>
     <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
   </numFmts>
   <fonts count="22">
     <font>
@@ -407,8 +420,71 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <u/>
       <sz val="11"/>
-      <color theme="1"/>
+      <color rgb="FF0000FF"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF800080"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="18"/>
+      <color theme="3"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color rgb="FF7F7F7F"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="15"/>
+      <color theme="3"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="13"/>
+      <color theme="3"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="3"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF3F3F76"/>
       <name val="宋体"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -422,23 +498,9 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <b/>
       <sz val="11"/>
-      <color theme="0"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF800080"/>
+      <color rgb="FFFA7D00"/>
       <name val="宋体"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -446,23 +508,29 @@
     <font>
       <b/>
       <sz val="11"/>
-      <color theme="3"/>
+      <color rgb="FFFFFFFF"/>
       <name val="宋体"/>
-      <charset val="134"/>
+      <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <sz val="15"/>
-      <color theme="3"/>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
       <name val="宋体"/>
-      <charset val="134"/>
+      <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
-      <color rgb="FFFA7D00"/>
+      <color theme="1"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF006100"/>
       <name val="宋体"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -476,76 +544,21 @@
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FF006100"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="13"/>
-      <color theme="3"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF3F3F76"/>
+      <color rgb="FF9C6500"/>
       <name val="宋体"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FFFA7D00"/>
+      <color theme="0"/>
       <name val="宋体"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FF9C6500"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="11"/>
-      <color rgb="FF7F7F7F"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="18"/>
-      <color theme="3"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF0000FF"/>
+      <color theme="1"/>
       <name val="宋体"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -560,7 +573,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.599993896298105"/>
+        <fgColor rgb="FFFFFFCC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFCC99"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -572,7 +591,133 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="9"/>
+        <fgColor rgb="FFA5A5A5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.799981688894314"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -584,7 +729,19 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.799981688894314"/>
+        <fgColor theme="8" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.799981688894314"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -596,151 +753,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="8"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFA5A5A5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor theme="9" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.799981688894314"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -751,30 +764,6 @@
       <right/>
       <top/>
       <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4" tint="0.499984740745262"/>
-      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -802,6 +791,15 @@
       <diagonal/>
     </border>
     <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4" tint="0.499984740745262"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
       <left style="thin">
         <color rgb="FF7F7F7F"/>
       </left>
@@ -817,22 +815,17 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right/>
+      <left style="thin">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF3F3F3F"/>
+      </right>
       <top style="thin">
-        <color theme="4"/>
+        <color rgb="FF3F3F3F"/>
       </top>
-      <bottom style="double">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="double">
-        <color rgb="FFFF8001"/>
+      <bottom style="thin">
+        <color rgb="FF3F3F3F"/>
       </bottom>
       <diagonal/>
     </border>
@@ -851,153 +844,173 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="double">
+        <color rgb="FFFF8001"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="4"/>
+      </top>
+      <bottom style="double">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="19" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="26" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
@@ -1026,54 +1039,54 @@
   </cellXfs>
   <cellStyles count="49">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
-    <cellStyle name="60% - 强调文字颜色 6" xfId="1" builtinId="52"/>
-    <cellStyle name="20% - 强调文字颜色 4" xfId="2" builtinId="42"/>
-    <cellStyle name="强调文字颜色 4" xfId="3" builtinId="41"/>
-    <cellStyle name="输入" xfId="4" builtinId="20"/>
-    <cellStyle name="40% - 强调文字颜色 3" xfId="5" builtinId="39"/>
-    <cellStyle name="20% - 强调文字颜色 3" xfId="6" builtinId="38"/>
-    <cellStyle name="货币" xfId="7" builtinId="4"/>
-    <cellStyle name="强调文字颜色 3" xfId="8" builtinId="37"/>
-    <cellStyle name="百分比" xfId="9" builtinId="5"/>
-    <cellStyle name="60% - 强调文字颜色 2" xfId="10" builtinId="36"/>
-    <cellStyle name="60% - 强调文字颜色 5" xfId="11" builtinId="48"/>
-    <cellStyle name="强调文字颜色 2" xfId="12" builtinId="33"/>
-    <cellStyle name="60% - 强调文字颜色 1" xfId="13" builtinId="32"/>
-    <cellStyle name="60% - 强调文字颜色 4" xfId="14" builtinId="44"/>
-    <cellStyle name="计算" xfId="15" builtinId="22"/>
-    <cellStyle name="强调文字颜色 1" xfId="16" builtinId="29"/>
-    <cellStyle name="适中" xfId="17" builtinId="28"/>
-    <cellStyle name="20% - 强调文字颜色 5" xfId="18" builtinId="46"/>
-    <cellStyle name="好" xfId="19" builtinId="26"/>
-    <cellStyle name="20% - 强调文字颜色 1" xfId="20" builtinId="30"/>
+    <cellStyle name="千位分隔" xfId="1" builtinId="3"/>
+    <cellStyle name="货币" xfId="2" builtinId="4"/>
+    <cellStyle name="百分比" xfId="3" builtinId="5"/>
+    <cellStyle name="千位分隔[0]" xfId="4" builtinId="6"/>
+    <cellStyle name="货币[0]" xfId="5" builtinId="7"/>
+    <cellStyle name="超链接" xfId="6" builtinId="8"/>
+    <cellStyle name="已访问的超链接" xfId="7" builtinId="9"/>
+    <cellStyle name="注释" xfId="8" builtinId="10"/>
+    <cellStyle name="警告文本" xfId="9" builtinId="11"/>
+    <cellStyle name="标题" xfId="10" builtinId="15"/>
+    <cellStyle name="解释性文本" xfId="11" builtinId="53"/>
+    <cellStyle name="标题 1" xfId="12" builtinId="16"/>
+    <cellStyle name="标题 2" xfId="13" builtinId="17"/>
+    <cellStyle name="标题 3" xfId="14" builtinId="18"/>
+    <cellStyle name="标题 4" xfId="15" builtinId="19"/>
+    <cellStyle name="输入" xfId="16" builtinId="20"/>
+    <cellStyle name="输出" xfId="17" builtinId="21"/>
+    <cellStyle name="计算" xfId="18" builtinId="22"/>
+    <cellStyle name="检查单元格" xfId="19" builtinId="23"/>
+    <cellStyle name="链接单元格" xfId="20" builtinId="24"/>
     <cellStyle name="汇总" xfId="21" builtinId="25"/>
-    <cellStyle name="差" xfId="22" builtinId="27"/>
-    <cellStyle name="检查单元格" xfId="23" builtinId="23"/>
-    <cellStyle name="输出" xfId="24" builtinId="21"/>
-    <cellStyle name="标题 1" xfId="25" builtinId="16"/>
-    <cellStyle name="解释性文本" xfId="26" builtinId="53"/>
-    <cellStyle name="20% - 强调文字颜色 2" xfId="27" builtinId="34"/>
-    <cellStyle name="标题 4" xfId="28" builtinId="19"/>
-    <cellStyle name="货币[0]" xfId="29" builtinId="7"/>
-    <cellStyle name="40% - 强调文字颜色 4" xfId="30" builtinId="43"/>
-    <cellStyle name="千位分隔" xfId="31" builtinId="3"/>
-    <cellStyle name="已访问的超链接" xfId="32" builtinId="9"/>
-    <cellStyle name="标题" xfId="33" builtinId="15"/>
-    <cellStyle name="40% - 强调文字颜色 2" xfId="34" builtinId="35"/>
-    <cellStyle name="警告文本" xfId="35" builtinId="11"/>
+    <cellStyle name="好" xfId="22" builtinId="26"/>
+    <cellStyle name="差" xfId="23" builtinId="27"/>
+    <cellStyle name="适中" xfId="24" builtinId="28"/>
+    <cellStyle name="强调文字颜色 1" xfId="25" builtinId="29"/>
+    <cellStyle name="20% - 强调文字颜色 1" xfId="26" builtinId="30"/>
+    <cellStyle name="40% - 强调文字颜色 1" xfId="27" builtinId="31"/>
+    <cellStyle name="60% - 强调文字颜色 1" xfId="28" builtinId="32"/>
+    <cellStyle name="强调文字颜色 2" xfId="29" builtinId="33"/>
+    <cellStyle name="20% - 强调文字颜色 2" xfId="30" builtinId="34"/>
+    <cellStyle name="40% - 强调文字颜色 2" xfId="31" builtinId="35"/>
+    <cellStyle name="60% - 强调文字颜色 2" xfId="32" builtinId="36"/>
+    <cellStyle name="强调文字颜色 3" xfId="33" builtinId="37"/>
+    <cellStyle name="20% - 强调文字颜色 3" xfId="34" builtinId="38"/>
+    <cellStyle name="40% - 强调文字颜色 3" xfId="35" builtinId="39"/>
     <cellStyle name="60% - 强调文字颜色 3" xfId="36" builtinId="40"/>
-    <cellStyle name="注释" xfId="37" builtinId="10"/>
-    <cellStyle name="20% - 强调文字颜色 6" xfId="38" builtinId="50"/>
-    <cellStyle name="强调文字颜色 5" xfId="39" builtinId="45"/>
-    <cellStyle name="40% - 强调文字颜色 6" xfId="40" builtinId="51"/>
-    <cellStyle name="超链接" xfId="41" builtinId="8"/>
-    <cellStyle name="千位分隔[0]" xfId="42" builtinId="6"/>
-    <cellStyle name="标题 2" xfId="43" builtinId="17"/>
-    <cellStyle name="40% - 强调文字颜色 5" xfId="44" builtinId="47"/>
-    <cellStyle name="标题 3" xfId="45" builtinId="18"/>
-    <cellStyle name="强调文字颜色 6" xfId="46" builtinId="49"/>
-    <cellStyle name="40% - 强调文字颜色 1" xfId="47" builtinId="31"/>
-    <cellStyle name="链接单元格" xfId="48" builtinId="24"/>
+    <cellStyle name="强调文字颜色 4" xfId="37" builtinId="41"/>
+    <cellStyle name="20% - 强调文字颜色 4" xfId="38" builtinId="42"/>
+    <cellStyle name="40% - 强调文字颜色 4" xfId="39" builtinId="43"/>
+    <cellStyle name="60% - 强调文字颜色 4" xfId="40" builtinId="44"/>
+    <cellStyle name="强调文字颜色 5" xfId="41" builtinId="45"/>
+    <cellStyle name="20% - 强调文字颜色 5" xfId="42" builtinId="46"/>
+    <cellStyle name="40% - 强调文字颜色 5" xfId="43" builtinId="47"/>
+    <cellStyle name="60% - 强调文字颜色 5" xfId="44" builtinId="48"/>
+    <cellStyle name="强调文字颜色 6" xfId="45" builtinId="49"/>
+    <cellStyle name="20% - 强调文字颜色 6" xfId="46" builtinId="50"/>
+    <cellStyle name="40% - 强调文字颜色 6" xfId="47" builtinId="51"/>
+    <cellStyle name="60% - 强调文字颜色 6" xfId="48" builtinId="52"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -1346,24 +1359,24 @@
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
     <col min="1" max="1" width="13.1" customWidth="1"/>
-    <col min="2" max="2" width="17.7545454545455" customWidth="1"/>
-    <col min="3" max="3" width="10.1454545454545" customWidth="1"/>
-    <col min="4" max="4" width="7.75454545454545" customWidth="1"/>
-    <col min="5" max="5" width="11.7181818181818" customWidth="1"/>
-    <col min="6" max="6" width="11.1181818181818" customWidth="1"/>
-    <col min="7" max="7" width="10.9454545454545" customWidth="1"/>
-    <col min="8" max="10" width="11.9818181818182" customWidth="1"/>
-    <col min="11" max="11" width="15.0727272727273" customWidth="1"/>
-    <col min="12" max="14" width="12.1090909090909" customWidth="1"/>
-    <col min="15" max="16" width="10.8545454545455" customWidth="1"/>
-    <col min="18" max="18" width="14.2181818181818" customWidth="1"/>
-    <col min="19" max="19" width="11.8090909090909" customWidth="1"/>
+    <col min="2" max="2" width="17.7583333333333" customWidth="1"/>
+    <col min="3" max="3" width="10.1416666666667" customWidth="1"/>
+    <col min="4" max="4" width="7.75833333333333" customWidth="1"/>
+    <col min="5" max="5" width="11.7166666666667" customWidth="1"/>
+    <col min="6" max="6" width="11.1166666666667" customWidth="1"/>
+    <col min="7" max="7" width="10.9416666666667" customWidth="1"/>
+    <col min="8" max="10" width="11.9833333333333" customWidth="1"/>
+    <col min="11" max="11" width="15.075" customWidth="1"/>
+    <col min="12" max="14" width="12.1083333333333" customWidth="1"/>
+    <col min="15" max="16" width="10.8583333333333" customWidth="1"/>
+    <col min="18" max="18" width="14.2166666666667" customWidth="1"/>
+    <col min="19" max="19" width="11.8083333333333" customWidth="1"/>
     <col min="20" max="20" width="10.6" customWidth="1"/>
-    <col min="21" max="21" width="9.70909090909091" customWidth="1"/>
-    <col min="22" max="22" width="11.1636363636364" customWidth="1"/>
-    <col min="23" max="23" width="11.4090909090909" customWidth="1"/>
-    <col min="24" max="24" width="12.0545454545455" customWidth="1"/>
-    <col min="25" max="25" width="15.5727272727273" customWidth="1"/>
+    <col min="21" max="21" width="9.70833333333333" customWidth="1"/>
+    <col min="22" max="22" width="11.1666666666667" customWidth="1"/>
+    <col min="23" max="23" width="11.4083333333333" customWidth="1"/>
+    <col min="24" max="24" width="12.0583333333333" customWidth="1"/>
+    <col min="25" max="25" width="15.575" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1" spans="1:24">
@@ -3009,7 +3022,7 @@
         <v>15</v>
       </c>
       <c r="F31" s="4" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="G31" s="4" t="s">
         <v>26</v>
@@ -5223,47 +5236,47 @@
     </row>
   </sheetData>
   <dataValidations count="14">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="M29 M30 M31 M39 M40 M41 M42 M43 M44 M2:M28 M32:M38 M45:M1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C2:C1048576">
+      <formula1>"PC_4,PC_0,PC_ALU,PC_CSR"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D2:D1048576">
+      <formula1>"A_PC,A_RS1"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E2:E1048576">
+      <formula1>"B_IMM,B_RS2"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F2:F1048576">
+      <formula1>"ALU_ADD,ALU_SUB,ALU_AND,ALU_OR,ALU_XOR,ALU_SLL,ALU_SRL,ALU_SLT,ALU_SLTU,ALU_COPY_A,ALU_COPY_B,ALU_SRA"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G2:G1048576">
+      <formula1>"IMM_I,IMM_J,IMM_U,IMM_S,IMM_B"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H2:H9">
+      <formula1>"WB_ALU,WB_MEM,WB_PC4,WB_XX"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H10:H1048576">
+      <formula1>"WB_ALU,WB_MEM,WB_PC4,WB_XX,WB_CSR"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I2:I1048576">
+      <formula1>"LD_LB,LD_LH,LD_LW,LD_LBU,LD_LHU,LD_XX"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J2:J1048576">
+      <formula1>"ST_SW,ST_SH,ST_SB,ST_XX"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K2:K1048576">
+      <formula1>"MASK_XX,MASK_B,MASK_H,MASK_W,MASK_D"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L2:L1048576">
+      <formula1>"BR_EQ,BR_NE,BR_LTU,BR_GE,BR_GEU,BR_LT,BR_XX"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="M2:M1048576">
       <formula1>"CSR_W,CSR_S,CSR_C,CSR_P,CSR_XX"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F6 F15 F18 F19 F20 F21 F24 F25 F26 F27 F28 F29 F30 F31 F32 F33 F36 F37 F38 F39 F40 F41 F42 F43 F44 F2:F5 F7:F14 F16:F17 F22:F23 F34:F35 F45:F1048576">
-      <formula1>"ALU_ADD,ALU_SUB,ALU_AND,ALU_OR,ALU_XOR,ALU_SLL,ALU_SRL,ALU_SLT,ALU_SLTU,ALU_COPY_A,ALU_COPY_B,ALU_SRA"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L5 L6 L7 L10 L11 L14 L15 L16 L17 L18 L19 L20 L21 L22 L23 L24 L25 L26 L27 L28 L29 L30 L31 L32 L33 L34 L35 L36 L37 L38 L39 L40 L41 L42 L43 L44 L2:L4 L8:L9 L12:L13 L45:L1048576">
-      <formula1>"BR_EQ,BR_NE,BR_LTU,BR_GE,BR_GEU,BR_LT,BR_XX"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="O44 O2:O43 O45:O1048576">
-      <formula1>"R_TYPE,I_TYPE,S_TYPE,B_TYPE,U_TYPE,J_TYPE,ICSR_TYPE,FENCE_TYPE,N_TYPE"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J5 J6 J7 J8 J9 J10 J11 J12 J13 J14 J15 J16 J17 J18 J19 J20 J21 J22 J23 J24 J25 J26 J27 J28 J29 J30 J31 J32 J33 J34 J35 J36 J37 J38 J39 J40 J41 J42 J43 J44 J2:J4 J45:J1048576">
-      <formula1>"ST_SW,ST_SH,ST_SB,ST_XX"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K4 K5 K6 K7 K8 K9 K10 K11 K12 K13 K14 K15 K16 K17 K18 K19 K20 K21 K22 K23 K24 K25 K26 K27 K28 K29 K30 K31 K32 K33 K34 K35 K36 K37 K38 K39 K40 K41 K42 K43 K44 K2:K3 K45:K1048576">
-      <formula1>"MASK_XX,MASK_B,MASK_H,MASK_W,MASK_D"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G4 G5 G6 G7 G8 G9 G10 G11 G12 G13 G14 G15 G16 G17 G18 G19 G20 G21 G22 G23 G24 G25 G26 G27 G28 G29 G30 G31 G32 G33 G34 G35 G36 G37 G38 G39 G40 G41 G42 G43 G44 G2:G3 G45:G1048576">
-      <formula1>"IMM_I,IMM_J,IMM_U,IMM_S,IMM_B"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="N4 N5 N6 N7 N8 N9 N10 N11 N12 N13 N14 N15 N16 N17 N18 N19 N20 N21 N22 N23 N24 N25 N26 N27 N28 N29 N30 N31 N32 N33 N34 N35 N36 N37 N38 N39 N40 N41 N42 N43 N44 N2:N3 N45:N1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="N2:N1048576">
       <formula1>"INST_VALID,INST_INVALID"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H29 H30 H31 H40 H41 H42 H43 H44 H10:H28 H32:H39 H45:H1048576">
-      <formula1>"WB_ALU,WB_MEM,WB_PC4,WB_XX,WB_CSR"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E4 E5 E6 E7 E8 E9 E10 E11 E12 E13 E14 E15 E16 E17 E18 E19 E20 E21 E22 E23 E24 E25 E26 E27 E28 E29 E30 E31 E32 E33 E34 E35 E36 E37 E38 E39 E40 E41 E42 E43 E44 E2:E3 E45:E1048576">
-      <formula1>"B_IMM,B_RS2"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H5 H6 H7 H8 H9 H2:H4">
-      <formula1>"WB_ALU,WB_MEM,WB_PC4,WB_XX"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I4 I5 I6 I7 I8 I9 I10 I11 I12 I13 I14 I15 I16 I17 I18 I19 I20 I21 I22 I23 I24 I25 I26 I27 I28 I29 I30 I31 I32 I33 I34 I35 I36 I37 I38 I39 I40 I41 I42 I43 I44 I2:I3 I45:I1048576">
-      <formula1>"LD_LB,LD_LH,LD_LW,LD_LBU,LD_LHU,LD_XX"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C29 C30 C31 C43 C44 C2:C28 C32:C42 C45:C1048576">
-      <formula1>"PC_4,PC_0,PC_ALU,PC_CSR"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D4 D5 D6 D7 D8 D9 D10 D11 D12 D13 D14 D15 D16 D17 D18 D19 D20 D21 D22 D23 D24 D25 D26 D27 D28 D29 D30 D31 D32 D33 D34 D35 D36 D37 D38 D39 D40 D41 D42 D43 D44 D2:D3 D45:D1048576">
-      <formula1>"A_PC,A_RS1"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="O2:O1048576">
+      <formula1>"R_TYPE,I_TYPE,S_TYPE,B_TYPE,U_TYPE,J_TYPE,ICSR_TYPE,FENCE_TYPE,N_TYPE"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>